<commit_message>
chore: update coding-agents leaderboard (2026-09-20)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agentic Models" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Agentic Models" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z31"/>
+  <dimension ref="A1:Z32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -591,10 +591,10 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>53.3737509623252</v>
+        <v>53.3549259623252</v>
       </c>
       <c r="K2" t="n">
-        <v>14.89500026855587</v>
+        <v>14.72537055077972</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.087069</v>
       </c>
       <c r="Q2" t="n">
-        <v>215</v>
+        <v>217.4</v>
       </c>
       <c r="R2" t="n">
         <v>23039.4</v>
@@ -623,19 +623,19 @@
       </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="n">
-        <v>44.35223936254697</v>
+        <v>44.3365962628782</v>
       </c>
       <c r="W2" t="n">
-        <v>0.2482500044759312</v>
+        <v>0.2454228425129954</v>
       </c>
       <c r="X2" t="n">
-        <v>0.02254677586459017</v>
+        <v>0.022554730951173</v>
       </c>
       <c r="Y2" t="n">
-        <v>107.16</v>
+        <v>105.9770009199632</v>
       </c>
       <c r="Z2" t="n">
-        <v>2.316629381074385</v>
+        <v>2.315812302504631</v>
       </c>
     </row>
     <row r="3">
@@ -681,10 +681,10 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>53.1840337538944</v>
+        <v>53.2032587538944</v>
       </c>
       <c r="K3" t="n">
-        <v>30.18961234847364</v>
+        <v>28.02629960696808</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>0.452635</v>
       </c>
       <c r="Q3" t="n">
-        <v>105.7</v>
+        <v>113.9</v>
       </c>
       <c r="R3" t="n">
         <v>10176.4</v>
@@ -713,19 +713,19 @@
       </c>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="n">
-        <v>95.48677641467778</v>
+        <v>95.52129303831462</v>
       </c>
       <c r="W3" t="n">
-        <v>0.503160205807894</v>
+        <v>0.4671049934494679</v>
       </c>
       <c r="X3" t="n">
-        <v>0.0104726543040601</v>
+        <v>0.01046887000994521</v>
       </c>
       <c r="Y3" t="n">
-        <v>96.27625354777672</v>
+        <v>89.34503950834065</v>
       </c>
       <c r="Z3" t="n">
-        <v>5.226212978449589</v>
+        <v>5.228102153403404</v>
       </c>
     </row>
     <row r="4">
@@ -771,10 +771,10 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>52.814069395513</v>
+        <v>52.673669395513</v>
       </c>
       <c r="K4" t="n">
-        <v>34.036994239858</v>
+        <v>33.58576156993391</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.25811</v>
       </c>
       <c r="Q4" t="n">
-        <v>93.09999999999999</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="R4" t="n">
         <v>5609.9</v>
@@ -803,19 +803,19 @@
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="n">
-        <v>174.0683213984806</v>
+        <v>173.6055812119343</v>
       </c>
       <c r="W4" t="n">
-        <v>0.5672832373309667</v>
+        <v>0.5597626928322317</v>
       </c>
       <c r="X4" t="n">
-        <v>0.005744870703445117</v>
+        <v>0.005760183474627001</v>
       </c>
       <c r="Y4" t="n">
-        <v>60.25671321160043</v>
+        <v>59.6163655685441</v>
       </c>
       <c r="Z4" t="n">
-        <v>9.414440434858555</v>
+        <v>9.389413250773277</v>
       </c>
     </row>
     <row r="5">
@@ -861,10 +861,10 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>52.5059027108782</v>
+        <v>52.3863277108782</v>
       </c>
       <c r="K5" t="n">
-        <v>53.76030994287871</v>
+        <v>56.83869191053692</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -880,7 +880,7 @@
         <v>0.126814</v>
       </c>
       <c r="Q5" t="n">
-        <v>58.6</v>
+        <v>55.3</v>
       </c>
       <c r="R5" t="n">
         <v>2987.7</v>
@@ -893,19 +893,19 @@
       </c>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="n">
-        <v>304.4597039875574</v>
+        <v>303.7663387233741</v>
       </c>
       <c r="W5" t="n">
-        <v>0.8960051657146451</v>
+        <v>0.9473115318422821</v>
       </c>
       <c r="X5" t="n">
-        <v>0.00328450690486406</v>
+        <v>0.003292003992946215</v>
       </c>
       <c r="Y5" t="n">
-        <v>50.98464163822525</v>
+        <v>54.02712477396022</v>
       </c>
       <c r="Z5" t="n">
-        <v>17.5740210566249</v>
+        <v>17.53399863134793</v>
       </c>
     </row>
     <row r="6">
@@ -951,10 +951,10 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>51.2094958852237</v>
+        <v>51.1515708852237</v>
       </c>
       <c r="K6" t="n">
-        <v>75.67905795845867</v>
+        <v>77.89579322622899</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -970,7 +970,7 @@
         <v>0.123</v>
       </c>
       <c r="Q6" t="n">
-        <v>40.6</v>
+        <v>39.4</v>
       </c>
       <c r="R6" t="n">
         <v>3396.5</v>
@@ -983,19 +983,19 @@
       </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="n">
-        <v>238.6421166483697</v>
+        <v>238.3721795133149</v>
       </c>
       <c r="W6" t="n">
-        <v>1.261317632640978</v>
+        <v>1.29826322043715</v>
       </c>
       <c r="X6" t="n">
-        <v>0.004190375169498949</v>
+        <v>0.004195120429077348</v>
       </c>
       <c r="Y6" t="n">
-        <v>83.6576354679803</v>
+        <v>86.20558375634518</v>
       </c>
       <c r="Z6" t="n">
-        <v>15.077137019056</v>
+        <v>15.06008269843183</v>
       </c>
     </row>
     <row r="7">
@@ -1041,10 +1041,10 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>51.0480721636152</v>
+        <v>50.9191471636152</v>
       </c>
       <c r="K7" t="n">
-        <v>98.80272031667458</v>
+        <v>101.4999611234854</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1060,7 +1060,7 @@
         <v>0.057183</v>
       </c>
       <c r="Q7" t="n">
-        <v>31</v>
+        <v>30.1</v>
       </c>
       <c r="R7" t="n">
         <v>1583.7</v>
@@ -1073,19 +1073,19 @@
       </c>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="n">
-        <v>501.2378948550253</v>
+        <v>499.9719881742194</v>
       </c>
       <c r="W7" t="n">
-        <v>1.64671200527791</v>
+        <v>1.691666018724757</v>
       </c>
       <c r="X7" t="n">
-        <v>0.001995060649373354</v>
+        <v>0.002000112053580773</v>
       </c>
       <c r="Y7" t="n">
-        <v>51.08709677419355</v>
+        <v>52.61461794019934</v>
       </c>
       <c r="Z7" t="n">
-        <v>32.23342310009168</v>
+        <v>32.15201563655692</v>
       </c>
     </row>
     <row r="8">
@@ -1131,10 +1131,10 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>50.7001865797629</v>
+        <v>50.7771115797629</v>
       </c>
       <c r="K8" t="n">
-        <v>27.83175841524039</v>
+        <v>26.79530954077198</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1150,7 +1150,7 @@
         <v>0.20946</v>
       </c>
       <c r="Q8" t="n">
-        <v>109.3</v>
+        <v>113.7</v>
       </c>
       <c r="R8" t="n">
         <v>9435.6</v>
@@ -1163,35 +1163,35 @@
       </c>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="n">
-        <v>198.4693511984956</v>
+        <v>198.7704793771252</v>
       </c>
       <c r="W8" t="n">
-        <v>0.4638626402540064</v>
+        <v>0.4465884923461997</v>
       </c>
       <c r="X8" t="n">
-        <v>0.00503856133937712</v>
+        <v>0.005030928149560429</v>
       </c>
       <c r="Y8" t="n">
-        <v>86.32753888380604</v>
+        <v>82.9868073878628</v>
       </c>
       <c r="Z8" t="n">
-        <v>5.373286974836035</v>
+        <v>5.381439609538651</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>claude-fable-5</t>
+          <t>claude-opus-5-xhigh</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Claude Fable 5 (Adaptive Reasoning, Max Effort, Opus 4.8 Fallback)</t>
+          <t>Claude Opus 5 (Adaptive Reasoning, Xhigh Effort)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Claude Fable 5 (with fallback)</t>
+          <t>Claude Opus 5 (xhigh)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1221,82 +1221,82 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>49.6994452733378</v>
+        <v>49.6773552926939</v>
       </c>
       <c r="K9" t="n">
-        <v>31.92683850535618</v>
+        <v>39.37438992815897</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
-        <v>0.520062</v>
+        <v>0.177537</v>
       </c>
       <c r="N9" t="n">
-        <v>0.036048</v>
+        <v>0.018451</v>
       </c>
       <c r="O9" t="n">
-        <v>0.046389</v>
+        <v>0.022483</v>
       </c>
       <c r="P9" t="n">
-        <v>0.437625</v>
+        <v>0.136603</v>
       </c>
       <c r="Q9" t="n">
-        <v>93.40000000000001</v>
+        <v>75.7</v>
       </c>
       <c r="R9" t="n">
-        <v>9680.299999999999</v>
+        <v>6363.5</v>
       </c>
       <c r="S9" t="n">
-        <v>927.8</v>
+        <v>899.3</v>
       </c>
       <c r="T9" t="n">
-        <v>8752.5</v>
+        <v>5464.1</v>
       </c>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="n">
-        <v>95.56446207055659</v>
+        <v>279.8140967386736</v>
       </c>
       <c r="W9" t="n">
-        <v>0.5321139750892698</v>
+        <v>0.6562398321359828</v>
       </c>
       <c r="X9" t="n">
-        <v>0.01046414094040195</v>
+        <v>0.003573801361887527</v>
       </c>
       <c r="Y9" t="n">
-        <v>103.6434689507495</v>
+        <v>84.06208718626155</v>
       </c>
       <c r="Z9" t="n">
-        <v>5.134081100104109</v>
+        <v>7.806608830469695</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>gpt-6-astra-medium</t>
+          <t>claude-fable-5</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (medium)</t>
+          <t>Claude Fable 5 (Adaptive Reasoning, Max Effort, Opus 4.8 Fallback)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (medium)</t>
+          <t>Claude Fable 5 (with fallback)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1311,51 +1311,51 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>49.6685363034369</v>
+        <v>49.6258202733378</v>
       </c>
       <c r="K10" t="n">
-        <v>157.6778930267838</v>
+        <v>30.10666548433031</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
-        <v>0.070427</v>
+        <v>0.520062</v>
       </c>
       <c r="N10" t="n">
-        <v>0.022736</v>
+        <v>0.036048</v>
       </c>
       <c r="O10" t="n">
-        <v>0.022007</v>
+        <v>0.046389</v>
       </c>
       <c r="P10" t="n">
-        <v>0.025683</v>
+        <v>0.437625</v>
       </c>
       <c r="Q10" t="n">
-        <v>18.9</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="R10" t="n">
-        <v>953.8</v>
+        <v>9680.299999999999</v>
       </c>
       <c r="S10" t="n">
-        <v>440.1</v>
+        <v>927.8</v>
       </c>
       <c r="T10" t="n">
-        <v>513.7</v>
+        <v>8752.5</v>
       </c>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="n">
-        <v>705.2485027537294</v>
+        <v>95.42289241155439</v>
       </c>
       <c r="W10" t="n">
-        <v>2.62796488377973</v>
+        <v>0.5017777580721718</v>
       </c>
       <c r="X10" t="n">
-        <v>0.00141793991209535</v>
+        <v>0.01047966556795457</v>
       </c>
       <c r="Y10" t="n">
-        <v>50.46560846560847</v>
+        <v>97.87967644084932</v>
       </c>
       <c r="Z10" t="n">
-        <v>52.07437230387598</v>
+        <v>5.126475447386735</v>
       </c>
     </row>
     <row r="11">
@@ -1401,10 +1401,10 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>48.1690107719685</v>
+        <v>48.0923107719685</v>
       </c>
       <c r="K11" t="n">
-        <v>38.58665749423378</v>
+        <v>31.09416644739343</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1420,7 +1420,7 @@
         <v>0.07542500000000001</v>
       </c>
       <c r="Q11" t="n">
-        <v>74.90000000000001</v>
+        <v>92.8</v>
       </c>
       <c r="R11" t="n">
         <v>18553.6</v>
@@ -1433,19 +1433,19 @@
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>579.4001488160184</v>
+        <v>578.4775641354948</v>
       </c>
       <c r="W11" t="n">
-        <v>0.6431109582372296</v>
+        <v>0.5182361074565571</v>
       </c>
       <c r="X11" t="n">
-        <v>0.001725922925707667</v>
+        <v>0.001728675513102135</v>
       </c>
       <c r="Y11" t="n">
-        <v>247.7116154873164</v>
+        <v>199.9310344827586</v>
       </c>
       <c r="Z11" t="n">
-        <v>2.596208324636109</v>
+        <v>2.592074356026243</v>
       </c>
     </row>
     <row r="12">
@@ -1491,10 +1491,10 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>47.0613568915036</v>
+        <v>46.9727068915036</v>
       </c>
       <c r="K12" t="n">
-        <v>29.35219764542844</v>
+        <v>29.17559434254882</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1510,7 +1510,7 @@
         <v>0.111119</v>
       </c>
       <c r="Q12" t="n">
-        <v>96.2</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="R12" t="n">
         <v>5952.7</v>
@@ -1523,50 +1523,50 @@
       </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="n">
-        <v>371.4744639705702</v>
+        <v>370.7747134022449</v>
       </c>
       <c r="W12" t="n">
-        <v>0.489203294090474</v>
+        <v>0.486259905709147</v>
       </c>
       <c r="X12" t="n">
-        <v>0.002691975080363059</v>
+        <v>0.002697055553826625</v>
       </c>
       <c r="Y12" t="n">
-        <v>61.87837837837837</v>
+        <v>61.62215320910973</v>
       </c>
       <c r="Z12" t="n">
-        <v>7.905884202379357</v>
+        <v>7.890991800612092</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>glm-5-3</t>
+          <t>qwen3-8-max</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1578,85 +1578,85 @@
         <v>1</v>
       </c>
       <c r="I13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>44.855717385614</v>
+        <v>45.4152084980521</v>
       </c>
       <c r="K13" t="n">
-        <v>6.611012142315991</v>
+        <v>4.919502635643846</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
-        <v>0.15892</v>
+        <v>0.156468</v>
       </c>
       <c r="N13" t="n">
-        <v>0.006115</v>
+        <v>0.007406</v>
       </c>
       <c r="O13" t="n">
-        <v>0.004153</v>
+        <v>0.007526</v>
       </c>
       <c r="P13" t="n">
-        <v>0.148652</v>
+        <v>0.141536</v>
       </c>
       <c r="Q13" t="n">
-        <v>407.1</v>
+        <v>553.9</v>
       </c>
       <c r="R13" t="n">
-        <v>34728.3</v>
+        <v>24843.6</v>
       </c>
       <c r="S13" t="n">
-        <v>943.8</v>
+        <v>1254.3</v>
       </c>
       <c r="T13" t="n">
-        <v>33784.5</v>
+        <v>23589.3</v>
       </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="n">
-        <v>282.253444409854</v>
+        <v>290.2523742749451</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1101835357052665</v>
+        <v>0.0819917105940641</v>
       </c>
       <c r="X13" t="n">
-        <v>0.003542915134626035</v>
+        <v>0.003445277588161046</v>
       </c>
       <c r="Y13" t="n">
-        <v>85.30655858511423</v>
+        <v>44.85213937533851</v>
       </c>
       <c r="Z13" t="n">
-        <v>1.291618575790177</v>
+        <v>1.828044586857464</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>grok-4-6</t>
+          <t>glm-5-3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Grok 4.6 (high)</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Grok 4.6 (high)</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>SpaceXAI</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>xai</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1668,85 +1668,85 @@
         <v>1</v>
       </c>
       <c r="I14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
-        <v>44.4050073012592</v>
+        <v>44.777392385614</v>
       </c>
       <c r="K14" t="n">
-        <v>15.31207148319283</v>
+        <v>6.351403175264397</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>0.066873</v>
+        <v>0.15892</v>
       </c>
       <c r="N14" t="n">
-        <v>0.005686</v>
+        <v>0.006115</v>
       </c>
       <c r="O14" t="n">
-        <v>0.003091</v>
+        <v>0.004153</v>
       </c>
       <c r="P14" t="n">
-        <v>0.058096</v>
+        <v>0.148652</v>
       </c>
       <c r="Q14" t="n">
-        <v>174</v>
+        <v>423</v>
       </c>
       <c r="R14" t="n">
-        <v>10197.8</v>
+        <v>34728.3</v>
       </c>
       <c r="S14" t="n">
-        <v>515.2</v>
+        <v>943.8</v>
       </c>
       <c r="T14" t="n">
-        <v>9682.6</v>
+        <v>33784.5</v>
       </c>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="n">
-        <v>664.0199677187983</v>
+        <v>281.760586368072</v>
       </c>
       <c r="W14" t="n">
-        <v>0.2552011913865471</v>
+        <v>0.10585671958774</v>
       </c>
       <c r="X14" t="n">
-        <v>0.001505978808793117</v>
+        <v>0.003549112432260739</v>
       </c>
       <c r="Y14" t="n">
-        <v>58.60804597701149</v>
+        <v>82.10000000000001</v>
       </c>
       <c r="Z14" t="n">
-        <v>4.354371266475043</v>
+        <v>1.289363210569305</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>kimi-k3</t>
+          <t>grok-4-6</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Kimi K3 (max)</t>
+          <t>Grok 4.6 (high)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Kimi K3 (max)</t>
+          <t>Grok 4.6 (high)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Kimi</t>
+          <t>SpaceXAI</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>kimi</t>
+          <t>xai</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1758,85 +1758,85 @@
         <v>1</v>
       </c>
       <c r="I15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>43.7841729518782</v>
+        <v>44.3113073012592</v>
       </c>
       <c r="K15" t="n">
-        <v>9.898456582941568</v>
+        <v>15.23597958782551</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>0.163338</v>
+        <v>0.066873</v>
       </c>
       <c r="N15" t="n">
-        <v>0.007471</v>
+        <v>0.005686</v>
       </c>
       <c r="O15" t="n">
-        <v>0.007591</v>
+        <v>0.003091</v>
       </c>
       <c r="P15" t="n">
-        <v>0.148276</v>
+        <v>0.058096</v>
       </c>
       <c r="Q15" t="n">
-        <v>265.4</v>
+        <v>174.5</v>
       </c>
       <c r="R15" t="n">
-        <v>10391.2</v>
+        <v>10197.8</v>
       </c>
       <c r="S15" t="n">
-        <v>506.1</v>
+        <v>515.2</v>
       </c>
       <c r="T15" t="n">
-        <v>9885.1</v>
+        <v>9682.6</v>
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="n">
-        <v>268.0587061913222</v>
+        <v>662.6188043195191</v>
       </c>
       <c r="W15" t="n">
-        <v>0.1649742763823595</v>
+        <v>0.2539329931304252</v>
       </c>
       <c r="X15" t="n">
-        <v>0.003730526100824598</v>
+        <v>0.001509163328117374</v>
       </c>
       <c r="Y15" t="n">
-        <v>39.15297663903542</v>
+        <v>58.44011461318051</v>
       </c>
       <c r="Z15" t="n">
-        <v>4.213581968577084</v>
+        <v>4.345183010184472</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>gpt-5-6-terra</t>
+          <t>step-5</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GPT-5.6 Terra (max)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>GPT-5.6 Terra (max)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>StepFun</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>stepfun</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1851,82 +1851,82 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>42.2514998239494</v>
+        <v>43.7343049141614</v>
       </c>
       <c r="K16" t="n">
-        <v>23.13038311530077</v>
+        <v>14.84195868127649</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
-        <v>0.14583</v>
+        <v>0.044989</v>
       </c>
       <c r="N16" t="n">
-        <v>0.004243</v>
+        <v>0.003221</v>
       </c>
       <c r="O16" t="n">
-        <v>0.004487</v>
+        <v>0.002192</v>
       </c>
       <c r="P16" t="n">
-        <v>0.137101</v>
+        <v>0.039576</v>
       </c>
       <c r="Q16" t="n">
-        <v>109.6</v>
+        <v>176.8</v>
       </c>
       <c r="R16" t="n">
-        <v>11799</v>
+        <v>15469.6</v>
       </c>
       <c r="S16" t="n">
-        <v>373.9</v>
+        <v>811.7</v>
       </c>
       <c r="T16" t="n">
-        <v>11425.1</v>
+        <v>14657.8</v>
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="n">
-        <v>289.7311926486279</v>
+        <v>972.1110696872879</v>
       </c>
       <c r="W16" t="n">
-        <v>0.3855063852550128</v>
+        <v>0.2473659780212749</v>
       </c>
       <c r="X16" t="n">
-        <v>0.003451475109940102</v>
+        <v>0.001028689036862509</v>
       </c>
       <c r="Y16" t="n">
-        <v>107.6551094890511</v>
+        <v>87.49773755656108</v>
       </c>
       <c r="Z16" t="n">
-        <v>3.58093904771162</v>
+        <v>2.827112848047875</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>glm-5-3-flash</t>
+          <t>kimi-k3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Kimi K3 (max)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Kimi K3 (max)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>Kimi</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>kimi</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1941,82 +1941,82 @@
         <v>1</v>
       </c>
       <c r="J17" t="n">
-        <v>41.907366113455</v>
+        <v>43.5938229518782</v>
       </c>
       <c r="K17" t="n">
-        <v>7.508038121252016</v>
+        <v>10.75063451341016</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
-        <v>0.022786</v>
+        <v>0.163338</v>
       </c>
       <c r="N17" t="n">
-        <v>0.000576</v>
+        <v>0.007471</v>
       </c>
       <c r="O17" t="n">
-        <v>0.000417</v>
+        <v>0.007591</v>
       </c>
       <c r="P17" t="n">
-        <v>0.021793</v>
+        <v>0.148276</v>
       </c>
       <c r="Q17" t="n">
-        <v>334.9</v>
+        <v>243.3</v>
       </c>
       <c r="R17" t="n">
-        <v>44420.3</v>
+        <v>10391.2</v>
       </c>
       <c r="S17" t="n">
-        <v>834.1</v>
+        <v>506.1</v>
       </c>
       <c r="T17" t="n">
-        <v>43586.3</v>
+        <v>9885.1</v>
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="n">
-        <v>1839.171689346748</v>
+        <v>266.8933313244817</v>
       </c>
       <c r="W17" t="n">
-        <v>0.1251339686875336</v>
+        <v>0.1791772418901693</v>
       </c>
       <c r="X17" t="n">
-        <v>0.0005437230280307263</v>
+        <v>0.0037468152352755</v>
       </c>
       <c r="Y17" t="n">
-        <v>132.6375037324575</v>
+        <v>42.70941224825319</v>
       </c>
       <c r="Z17" t="n">
-        <v>0.9434282549522401</v>
+        <v>4.195263583789957</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>gemini-3-8-flash</t>
+          <t>gpt-5-6-terra</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>GPT-5.6 Terra (max)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>GPT-5.6 Terra (max)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2031,82 +2031,82 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>41.1863571765904</v>
+        <v>42.0829248239494</v>
       </c>
       <c r="K18" t="n">
-        <v>30.28408615925765</v>
+        <v>20.08731495176582</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
-        <v>0.093127</v>
+        <v>0.14583</v>
       </c>
       <c r="N18" t="n">
-        <v>0.001995</v>
+        <v>0.004243</v>
       </c>
       <c r="O18" t="n">
-        <v>0.002368</v>
+        <v>0.004487</v>
       </c>
       <c r="P18" t="n">
-        <v>0.088764</v>
+        <v>0.137101</v>
       </c>
       <c r="Q18" t="n">
-        <v>81.59999999999999</v>
+        <v>125.7</v>
       </c>
       <c r="R18" t="n">
-        <v>24301.8</v>
+        <v>11799</v>
       </c>
       <c r="S18" t="n">
-        <v>631.5</v>
+        <v>373.9</v>
       </c>
       <c r="T18" t="n">
-        <v>23670.3</v>
+        <v>11425.1</v>
       </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="n">
-        <v>442.2601090617157</v>
+        <v>288.57522336933</v>
       </c>
       <c r="W18" t="n">
-        <v>0.5047347693209608</v>
+        <v>0.3347885825294304</v>
       </c>
       <c r="X18" t="n">
-        <v>0.00226111281463202</v>
+        <v>0.003465300964941679</v>
       </c>
       <c r="Y18" t="n">
-        <v>297.8161764705882</v>
+        <v>93.86634844868735</v>
       </c>
       <c r="Z18" t="n">
-        <v>1.694786278242369</v>
+        <v>3.566651819980456</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>qwen3-8-2-4t-a95b</t>
+          <t>glm-5-3-flash</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Qwen3.8 2.4T A95B</t>
+          <t>GLM 5.3 Flash</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Qwen3.8 2.4T A95B</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2121,82 +2121,82 @@
         <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>40.0445723105325</v>
+        <v>41.807466113455</v>
       </c>
       <c r="K19" t="n">
-        <v>3.888451753733533</v>
+        <v>6.855556072170812</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
-        <v>0.178757</v>
+        <v>0.022786</v>
       </c>
       <c r="N19" t="n">
-        <v>0.009473000000000001</v>
+        <v>0.000576</v>
       </c>
       <c r="O19" t="n">
-        <v>0.009109000000000001</v>
+        <v>0.000417</v>
       </c>
       <c r="P19" t="n">
-        <v>0.160175</v>
+        <v>0.021793</v>
       </c>
       <c r="Q19" t="n">
-        <v>617.9</v>
+        <v>365.9</v>
       </c>
       <c r="R19" t="n">
-        <v>28213.9</v>
+        <v>44420.3</v>
       </c>
       <c r="S19" t="n">
-        <v>1518.1</v>
+        <v>834.1</v>
       </c>
       <c r="T19" t="n">
-        <v>26695.8</v>
+        <v>43586.3</v>
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="n">
-        <v>224.0168066734869</v>
+        <v>1834.787418303125</v>
       </c>
       <c r="W19" t="n">
-        <v>0.06480752922889223</v>
+        <v>0.1142592678695135</v>
       </c>
       <c r="X19" t="n">
-        <v>0.004463950784985246</v>
+        <v>0.0005450222679883181</v>
       </c>
       <c r="Y19" t="n">
-        <v>45.66094837352323</v>
+        <v>121.4001093194862</v>
       </c>
       <c r="Z19" t="n">
-        <v>1.419320700453766</v>
+        <v>0.9411792831983349</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>deepseek-v4-1-flash</t>
+          <t>gemini-3-8-flash</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (Reasoning, Max Effort)</t>
+          <t>Gemini 3.8 Flash (high)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (max)</t>
+          <t>Gemini 3.8 Flash (high)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>DeepSeek</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>deepseek</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2208,270 +2208,270 @@
         <v>1</v>
       </c>
       <c r="I20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>39.545442472527</v>
+        <v>40.9262321765904</v>
       </c>
       <c r="K20" t="n">
-        <v>30.5763730457683</v>
+        <v>31.72576137720186</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
-        <v>0.027666</v>
+        <v>0.093127</v>
       </c>
       <c r="N20" t="n">
-        <v>0.000862</v>
+        <v>0.001995</v>
       </c>
       <c r="O20" t="n">
-        <v>0.000595</v>
+        <v>0.002368</v>
       </c>
       <c r="P20" t="n">
-        <v>0.02621</v>
+        <v>0.088764</v>
       </c>
       <c r="Q20" t="n">
-        <v>77.59999999999999</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="R20" t="n">
-        <v>22336.9</v>
+        <v>24301.8</v>
       </c>
       <c r="S20" t="n">
-        <v>495.4</v>
+        <v>631.5</v>
       </c>
       <c r="T20" t="n">
-        <v>21841.5</v>
+        <v>23670.3</v>
       </c>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="n">
-        <v>1429.387785459662</v>
+        <v>439.4668804599139</v>
       </c>
       <c r="W20" t="n">
-        <v>0.5096062174294717</v>
+        <v>0.528762689620031</v>
       </c>
       <c r="X20" t="n">
-        <v>0.0006996002135826427</v>
+        <v>0.002275484329907804</v>
       </c>
       <c r="Y20" t="n">
-        <v>287.8466494845361</v>
+        <v>313.9767441860465</v>
       </c>
       <c r="Z20" t="n">
-        <v>1.770408717079228</v>
+        <v>1.684082338616498</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>gpt-5-6-luna</t>
+          <t>deepseek-v4-1-flash</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>GPT-5.6 Luna (max)</t>
+          <t>DeepSeek V4.1 Flash (Reasoning, Max Effort)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GPT-5.6 Luna (max)</t>
+          <t>DeepSeek V4.1 Flash (max)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>DeepSeek</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>deepseek</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H21" t="b">
         <v>1</v>
       </c>
       <c r="I21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" t="n">
-        <v>37.5048489690841</v>
+        <v>39.456167472527</v>
       </c>
       <c r="K21" t="n">
-        <v>20.00258611684485</v>
+        <v>28.97637758080318</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
-        <v>0.016448</v>
+        <v>0.027666</v>
       </c>
       <c r="N21" t="n">
-        <v>0.000637</v>
+        <v>0.000862</v>
       </c>
       <c r="O21" t="n">
-        <v>0.000541</v>
+        <v>0.000595</v>
       </c>
       <c r="P21" t="n">
-        <v>0.015269</v>
+        <v>0.02621</v>
       </c>
       <c r="Q21" t="n">
-        <v>112.5</v>
+        <v>81.7</v>
       </c>
       <c r="R21" t="n">
-        <v>13175.4</v>
+        <v>22336.9</v>
       </c>
       <c r="S21" t="n">
-        <v>451.2</v>
+        <v>495.4</v>
       </c>
       <c r="T21" t="n">
-        <v>12724.3</v>
+        <v>21841.5</v>
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="n">
-        <v>2280.207257361631</v>
+        <v>1426.160900474481</v>
       </c>
       <c r="W21" t="n">
-        <v>0.3333764352807476</v>
+        <v>0.4829396263467197</v>
       </c>
       <c r="X21" t="n">
-        <v>0.0004385566253995149</v>
+        <v>0.0007011831551876802</v>
       </c>
       <c r="Y21" t="n">
-        <v>117.1146666666667</v>
+        <v>273.4014687882497</v>
       </c>
       <c r="Z21" t="n">
-        <v>2.846581429716297</v>
+        <v>1.76641196730643</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>deepseek-v4-pro</t>
+          <t>gpt-5-6-luna</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DeepSeek V4 Pro 0813 (Reasoning, Max Effort)</t>
+          <t>GPT-5.6 Luna (max)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DeepSeek V4 Pro 0813 (max)</t>
+          <t>GPT-5.6 Luna (max)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>DeepSeek</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>deepseek</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H22" t="b">
         <v>1</v>
       </c>
       <c r="I22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>36.2828791278402</v>
+        <v>37.3244239690841</v>
       </c>
       <c r="K22" t="n">
-        <v>7.717024982879871</v>
+        <v>27.64772145858081</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
-        <v>0.101663</v>
+        <v>0.016448</v>
       </c>
       <c r="N22" t="n">
-        <v>0.003745</v>
+        <v>0.000637</v>
       </c>
       <c r="O22" t="n">
-        <v>0.001918</v>
+        <v>0.000541</v>
       </c>
       <c r="P22" t="n">
-        <v>0.096</v>
+        <v>0.015269</v>
       </c>
       <c r="Q22" t="n">
-        <v>282.1</v>
+        <v>81</v>
       </c>
       <c r="R22" t="n">
-        <v>24726.8</v>
+        <v>13175.4</v>
       </c>
       <c r="S22" t="n">
-        <v>484.3</v>
+        <v>451.2</v>
       </c>
       <c r="T22" t="n">
-        <v>24242.5</v>
+        <v>12724.3</v>
       </c>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="n">
-        <v>356.8936498808829</v>
+        <v>2269.237838587312</v>
       </c>
       <c r="W22" t="n">
-        <v>0.1286170830479978</v>
+        <v>0.4607953576430136</v>
       </c>
       <c r="X22" t="n">
-        <v>0.002801955149198538</v>
+        <v>0.0004406765932576458</v>
       </c>
       <c r="Y22" t="n">
-        <v>87.65260545905706</v>
+        <v>162.6592592592592</v>
       </c>
       <c r="Z22" t="n">
-        <v>1.467350369956492</v>
+        <v>2.832887348322184</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>qwen3-8-27b</t>
+          <t>deepseek-v4-pro</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (xhigh)</t>
+          <t>DeepSeek V4 Pro 0813 (Reasoning, Max Effort)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (xhigh)</t>
+          <t>DeepSeek V4 Pro 0813 (max)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>DeepSeek</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>deepseek</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H23" t="b">
@@ -2481,87 +2481,87 @@
         <v>1</v>
       </c>
       <c r="J23" t="n">
-        <v>33.9015108057476</v>
+        <v>35.9967791278402</v>
       </c>
       <c r="K23" t="n">
-        <v>3.628417139395034</v>
+        <v>9.269556856954559</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
-        <v>0.09057999999999999</v>
+        <v>0.101663</v>
       </c>
       <c r="N23" t="n">
-        <v>0.001883</v>
+        <v>0.003745</v>
       </c>
       <c r="O23" t="n">
-        <v>0.003858</v>
+        <v>0.001918</v>
       </c>
       <c r="P23" t="n">
-        <v>0.084838</v>
+        <v>0.096</v>
       </c>
       <c r="Q23" t="n">
-        <v>560.6</v>
+        <v>233</v>
       </c>
       <c r="R23" t="n">
-        <v>29565.5</v>
+        <v>24726.8</v>
       </c>
       <c r="S23" t="n">
-        <v>1286.1</v>
+        <v>484.3</v>
       </c>
       <c r="T23" t="n">
-        <v>28279.4</v>
+        <v>24242.5</v>
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="n">
-        <v>374.2714816267123</v>
+        <v>354.0794500244946</v>
       </c>
       <c r="W23" t="n">
-        <v>0.06047361898991722</v>
+        <v>0.154492614282576</v>
       </c>
       <c r="X23" t="n">
-        <v>0.00267185732574028</v>
+        <v>0.002824224901871096</v>
       </c>
       <c r="Y23" t="n">
-        <v>52.73902961113093</v>
+        <v>106.1236051502146</v>
       </c>
       <c r="Z23" t="n">
-        <v>1.146657787142027</v>
+        <v>1.455779928168635</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>k2-horizon-375b-a23b</t>
+          <t>qwen3-8-27b</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Qwen3.8 27B (xhigh)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Qwen3.8 27B (xhigh)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MBZUAI Institute of Foundation Models</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>mbzuai</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H24" t="b">
@@ -2571,54 +2571,82 @@
         <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>30.7949302696723</v>
-      </c>
-      <c r="K24" t="inlineStr"/>
+        <v>33.6962858057476</v>
+      </c>
+      <c r="K24" t="n">
+        <v>3.459577598126037</v>
+      </c>
       <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
+      <c r="M24" t="n">
+        <v>0.09057999999999999</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0.001883</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0.003858</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.084838</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>584.4</v>
+      </c>
+      <c r="R24" t="n">
+        <v>29565.5</v>
+      </c>
+      <c r="S24" t="n">
+        <v>1286.1</v>
+      </c>
+      <c r="T24" t="n">
+        <v>28279.4</v>
+      </c>
       <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="inlineStr"/>
+      <c r="V24" t="n">
+        <v>372.0058048768779</v>
+      </c>
+      <c r="W24" t="n">
+        <v>0.05765962663543395</v>
+      </c>
+      <c r="X24" t="n">
+        <v>0.002688130096063873</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>50.59120465434634</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>1.139716419669804</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>minimax-m3</t>
+          <t>k2-horizon-375b-a23b</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>Institute of Foundation Models</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>minimax</t>
+          <t>ifm</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2633,82 +2661,54 @@
         <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>29.6125932236316</v>
-      </c>
-      <c r="K25" t="n">
-        <v>9.051225641456423</v>
-      </c>
+        <v>30.5015302696723</v>
+      </c>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
-      <c r="M25" t="n">
-        <v>0.026465</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0.004611</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0.00061</v>
-      </c>
-      <c r="P25" t="n">
-        <v>0.021244</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>196.3</v>
-      </c>
-      <c r="R25" t="n">
-        <v>18211.1</v>
-      </c>
-      <c r="S25" t="n">
-        <v>508</v>
-      </c>
-      <c r="T25" t="n">
-        <v>17703.1</v>
-      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
-      <c r="V25" t="n">
-        <v>1118.934185665279</v>
-      </c>
-      <c r="W25" t="n">
-        <v>0.1508537606909404</v>
-      </c>
-      <c r="X25" t="n">
-        <v>0.0008937076128435877</v>
-      </c>
-      <c r="Y25" t="n">
-        <v>92.77177789098317</v>
-      </c>
-      <c r="Z25" t="n">
-        <v>1.626073835387846</v>
-      </c>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>inkling</t>
+          <t>minimax-m3</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Inkling (xhigh)</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Inkling</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Thinking Machines</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>thinking-machines</t>
+          <t>minimax</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2723,82 +2723,82 @@
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>25.5423060999384</v>
+        <v>29.2202932236316</v>
       </c>
       <c r="K26" t="n">
-        <v>6.026497703485269</v>
+        <v>18.77106631068411</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
-        <v>0.09468799999999999</v>
+        <v>0.026465</v>
       </c>
       <c r="N26" t="n">
-        <v>0.002374</v>
+        <v>0.004611</v>
       </c>
       <c r="O26" t="n">
-        <v>0.001895</v>
+        <v>0.00061</v>
       </c>
       <c r="P26" t="n">
-        <v>0.09042</v>
+        <v>0.021244</v>
       </c>
       <c r="Q26" t="n">
-        <v>254.3</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="R26" t="n">
-        <v>22793.6</v>
+        <v>18211.1</v>
       </c>
       <c r="S26" t="n">
-        <v>467.8</v>
+        <v>508</v>
       </c>
       <c r="T26" t="n">
-        <v>22325.9</v>
+        <v>17703.1</v>
       </c>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="n">
-        <v>269.7523033535232</v>
+        <v>1104.110834068831</v>
       </c>
       <c r="W26" t="n">
-        <v>0.1004416283914212</v>
+        <v>0.3128511051780685</v>
       </c>
       <c r="X26" t="n">
-        <v>0.003707104582864127</v>
+        <v>0.0009057061747277989</v>
       </c>
       <c r="Y26" t="n">
-        <v>89.63271726307509</v>
+        <v>194.9796573875803</v>
       </c>
       <c r="Z26" t="n">
-        <v>1.12059113522824</v>
+        <v>1.604532028467891</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
+          <t>inkling</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
+          <t>Inkling (xhigh)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra</t>
+          <t>Inkling</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Thinking Machines</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>thinking-machines</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2813,267 +2813,267 @@
         <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>23.4145123422858</v>
+        <v>24.9847810999384</v>
       </c>
       <c r="K27" t="n">
-        <v>21.6466986215277</v>
+        <v>5.449243424195943</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
-        <v>0.034269</v>
+        <v>0.09468799999999999</v>
       </c>
       <c r="N27" t="n">
-        <v>0.001525</v>
+        <v>0.002374</v>
       </c>
       <c r="O27" t="n">
-        <v>0.002978</v>
+        <v>0.001895</v>
       </c>
       <c r="P27" t="n">
-        <v>0.029765</v>
+        <v>0.09042</v>
       </c>
       <c r="Q27" t="n">
-        <v>64.90000000000001</v>
+        <v>275.1</v>
       </c>
       <c r="R27" t="n">
-        <v>12593.6</v>
+        <v>22793.6</v>
       </c>
       <c r="S27" t="n">
-        <v>1145.5</v>
+        <v>467.8</v>
       </c>
       <c r="T27" t="n">
-        <v>11448.1</v>
+        <v>22325.9</v>
       </c>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="n">
-        <v>683.2563641275146</v>
+        <v>263.8642816401065</v>
       </c>
       <c r="W27" t="n">
-        <v>0.360778310358795</v>
+        <v>0.09082072373659904</v>
       </c>
       <c r="X27" t="n">
-        <v>0.00146357948861106</v>
+        <v>0.00378982707998324</v>
       </c>
       <c r="Y27" t="n">
-        <v>194.0462249614792</v>
+        <v>82.85568884042165</v>
       </c>
       <c r="Z27" t="n">
-        <v>1.859239005708122</v>
+        <v>1.096131418465639</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>gemini-3-5-flash-lite</t>
+          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash-Lite</t>
+          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash-Lite</t>
+          <t>Nemotron 3 Ultra</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>nvidia</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H28" t="b">
         <v>1</v>
       </c>
       <c r="I28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>22.6606674839812</v>
+        <v>22.9279123422858</v>
       </c>
       <c r="K28" t="n">
-        <v>68.32362055471718</v>
+        <v>18.59019919644794</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
-        <v>0.019232</v>
+        <v>0.03175</v>
       </c>
       <c r="N28" t="n">
-        <v>0.000782</v>
+        <v>0.001525</v>
       </c>
       <c r="O28" t="n">
-        <v>0.001426</v>
+        <v>0.002749</v>
       </c>
       <c r="P28" t="n">
-        <v>0.017024</v>
+        <v>0.027475</v>
       </c>
       <c r="Q28" t="n">
-        <v>19.9</v>
+        <v>74</v>
       </c>
       <c r="R28" t="n">
-        <v>7379.9</v>
+        <v>12593.6</v>
       </c>
       <c r="S28" t="n">
-        <v>570.5</v>
+        <v>1145.5</v>
       </c>
       <c r="T28" t="n">
-        <v>6809.5</v>
+        <v>11448.1</v>
       </c>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="n">
-        <v>1178.279299291868</v>
+        <v>722.1389714105763</v>
       </c>
       <c r="W28" t="n">
-        <v>1.138727009245287</v>
+        <v>0.3098366532741325</v>
       </c>
       <c r="X28" t="n">
-        <v>0.000848695212248054</v>
+        <v>0.001384775008121593</v>
       </c>
       <c r="Y28" t="n">
-        <v>370.8492462311558</v>
+        <v>170.1837837837838</v>
       </c>
       <c r="Z28" t="n">
-        <v>3.070592756538869</v>
+        <v>1.820600332096128</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>muse-glimmer</t>
+          <t>gemini-3-5-flash-lite</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Muse Glimmer (high)</t>
+          <t>Gemini 3.5 Flash-Lite</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Muse Glimmer (high)</t>
+          <t>Gemini 3.5 Flash-Lite</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H29" t="b">
         <v>1</v>
       </c>
       <c r="I29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>18.0678176089465</v>
+        <v>22.1685424839812</v>
       </c>
       <c r="K29" t="n">
-        <v>12.62012871404878</v>
+        <v>68.21089995071138</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
-        <v>0.012326</v>
+        <v>0.019232</v>
       </c>
       <c r="N29" t="n">
-        <v>0.00072</v>
+        <v>0.000782</v>
       </c>
       <c r="O29" t="n">
-        <v>0.00067</v>
+        <v>0.001426</v>
       </c>
       <c r="P29" t="n">
-        <v>0.010936</v>
+        <v>0.017024</v>
       </c>
       <c r="Q29" t="n">
-        <v>85.90000000000001</v>
+        <v>19.5</v>
       </c>
       <c r="R29" t="n">
-        <v>7737.1</v>
+        <v>7379.9</v>
       </c>
       <c r="S29" t="n">
-        <v>446.4</v>
+        <v>570.5</v>
       </c>
       <c r="T29" t="n">
-        <v>7290.7</v>
+        <v>6809.5</v>
       </c>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="n">
-        <v>1465.829758960449</v>
+        <v>1152.690436979056</v>
       </c>
       <c r="W29" t="n">
-        <v>0.2103354785674796</v>
+        <v>1.136848332511856</v>
       </c>
       <c r="X29" t="n">
-        <v>0.0006822074622834709</v>
+        <v>0.0008675356087977764</v>
       </c>
       <c r="Y29" t="n">
-        <v>90.0710128055879</v>
+        <v>378.4564102564103</v>
       </c>
       <c r="Z29" t="n">
-        <v>2.335218312926871</v>
+        <v>3.003908248618708</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>mistral-medium-3-5</t>
+          <t>muse-glimmer</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Mistral Medium 3.5</t>
+          <t>Muse Glimmer (high)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Mistral Medium 3.5</t>
+          <t>Muse Glimmer (high)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Mistral</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>mistral</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H30" t="b">
@@ -3083,82 +3083,82 @@
         <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>14.8946727802691</v>
+        <v>17.4754176089465</v>
       </c>
       <c r="K30" t="n">
-        <v>10.62640150792088</v>
+        <v>12.36468227048101</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
-        <v>0.108206</v>
+        <v>0.012326</v>
       </c>
       <c r="N30" t="n">
-        <v>0.002141</v>
+        <v>0.00072</v>
       </c>
       <c r="O30" t="n">
-        <v>0.058389</v>
+        <v>0.00067</v>
       </c>
       <c r="P30" t="n">
-        <v>0.047676</v>
+        <v>0.010936</v>
       </c>
       <c r="Q30" t="n">
-        <v>84.09999999999999</v>
+        <v>84.8</v>
       </c>
       <c r="R30" t="n">
-        <v>14142</v>
+        <v>7737.1</v>
       </c>
       <c r="S30" t="n">
-        <v>7785.3</v>
+        <v>446.4</v>
       </c>
       <c r="T30" t="n">
-        <v>6356.8</v>
+        <v>7290.7</v>
       </c>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="n">
-        <v>137.6510801644003</v>
+        <v>1417.768749711707</v>
       </c>
       <c r="W30" t="n">
-        <v>0.1771066917986814</v>
+        <v>0.2060780378413503</v>
       </c>
       <c r="X30" t="n">
-        <v>0.007264745026378824</v>
+        <v>0.0007053336449991176</v>
       </c>
       <c r="Y30" t="n">
-        <v>168.1569560047563</v>
+        <v>91.23938679245283</v>
       </c>
       <c r="Z30" t="n">
-        <v>1.053222513100629</v>
+        <v>2.258652157649054</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>gpt-oss-120b</t>
+          <t>mistral-medium-3-5</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>gpt-oss-120b (high)</t>
+          <t>Mistral Medium 3.5</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>gpt-oss-120b (high)</t>
+          <t>Mistral Medium 3.5</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Mistral</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>mistral</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2025-08-05</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3173,51 +3173,141 @@
         <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>12.3483931512592</v>
+        <v>14.1889227802691</v>
       </c>
       <c r="K31" t="n">
-        <v>13.02115270783044</v>
+        <v>9.114939687539035</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
-        <v>0.007271</v>
+        <v>0.108206</v>
       </c>
       <c r="N31" t="n">
-        <v>0.000449</v>
+        <v>0.002141</v>
       </c>
       <c r="O31" t="n">
-        <v>0.000691</v>
+        <v>0.058389</v>
       </c>
       <c r="P31" t="n">
-        <v>0.006131</v>
+        <v>0.047676</v>
       </c>
       <c r="Q31" t="n">
-        <v>56.9</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="R31" t="n">
-        <v>11465.4</v>
+        <v>14142</v>
       </c>
       <c r="S31" t="n">
-        <v>1161.3</v>
+        <v>7785.3</v>
       </c>
       <c r="T31" t="n">
-        <v>10304</v>
+        <v>6356.8</v>
       </c>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="n">
-        <v>1698.307406307138</v>
+        <v>131.1287985903656</v>
       </c>
       <c r="W31" t="n">
-        <v>0.217019211797174</v>
+        <v>0.1519156614589839</v>
       </c>
       <c r="X31" t="n">
-        <v>0.000588821550377877</v>
+        <v>0.007626089850208333</v>
       </c>
       <c r="Y31" t="n">
-        <v>201.5008787346221</v>
+        <v>151.4132762312634</v>
       </c>
       <c r="Z31" t="n">
-        <v>1.077013724009559</v>
+        <v>1.003317973431558</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>gpt-oss-120b</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>gpt-oss-120b (high)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>gpt-oss-120b (high)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2025-08-05</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H32" t="b">
+        <v>1</v>
+      </c>
+      <c r="I32" t="b">
+        <v>1</v>
+      </c>
+      <c r="J32" t="n">
+        <v>11.6028431512592</v>
+      </c>
+      <c r="K32" t="n">
+        <v>11.62221350710437</v>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="n">
+        <v>0.007271</v>
+      </c>
+      <c r="N32" t="n">
+        <v>0.000449</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0.000691</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0.006131</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="R32" t="n">
+        <v>11465.4</v>
+      </c>
+      <c r="S32" t="n">
+        <v>1161.3</v>
+      </c>
+      <c r="T32" t="n">
+        <v>10304</v>
+      </c>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="n">
+        <v>1595.769928656196</v>
+      </c>
+      <c r="W32" t="n">
+        <v>0.1937035584517396</v>
+      </c>
+      <c r="X32" t="n">
+        <v>0.0006266567517299338</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>191.4090150250417</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>1.011987645547404</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-09-23)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z32"/>
+  <dimension ref="A1:Z33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,17 +551,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>claude-fable-5-1</t>
+          <t>claude-opus-5-5</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (Adaptive Reasoning, Max Effort, Default Fallback)</t>
+          <t>Claude Opus 5.5 (Adaptive Reasoning, Max Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (max with fallback)</t>
+          <t>Claude Opus 5.5 (max with fallback)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -576,7 +576,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -591,67 +591,59 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>53.3549259623252</v>
-      </c>
-      <c r="K2" t="n">
-        <v>14.72537055077972</v>
-      </c>
+        <v>57.6223698102963</v>
+      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
-        <v>1.203406</v>
+        <v>0.770958</v>
       </c>
       <c r="N2" t="n">
-        <v>0.051436</v>
+        <v>0.02173</v>
       </c>
       <c r="O2" t="n">
-        <v>0.064901</v>
+        <v>0.0373</v>
       </c>
       <c r="P2" t="n">
-        <v>1.087069</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>217.4</v>
-      </c>
+        <v>0.711927</v>
+      </c>
+      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="n">
-        <v>23039.4</v>
+        <v>37461.4</v>
       </c>
       <c r="S2" t="n">
-        <v>1298</v>
+        <v>1865</v>
       </c>
       <c r="T2" t="n">
-        <v>21741.4</v>
+        <v>35596.4</v>
       </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="n">
-        <v>44.3365962628782</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0.2454228425129954</v>
-      </c>
+        <v>74.74125673551127</v>
+      </c>
+      <c r="W2" t="inlineStr"/>
       <c r="X2" t="n">
-        <v>0.022554730951173</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>105.9770009199632</v>
-      </c>
+        <v>0.0133794913770145</v>
+      </c>
+      <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="n">
-        <v>2.315812302504631</v>
+        <v>1.538179828044235</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>claude-fable-5-1-xhigh</t>
+          <t>claude-opus-5-5-xhigh</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (Adaptive Reasoning, Xhigh Effort, Default Fallback)</t>
+          <t>Claude Opus 5.5 (Adaptive Reasoning, Xhigh Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (xhigh with fallback)</t>
+          <t>Claude Opus 5.5 (xhigh with fallback)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -666,7 +658,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -681,82 +673,82 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>53.2032587538944</v>
+        <v>55.9873505840139</v>
       </c>
       <c r="K3" t="n">
-        <v>28.02629960696808</v>
+        <v>77.58062436583914</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
-        <v>0.556978</v>
+        <v>0.145854</v>
       </c>
       <c r="N3" t="n">
-        <v>0.048158</v>
+        <v>0.018785</v>
       </c>
       <c r="O3" t="n">
-        <v>0.056185</v>
+        <v>0.030496</v>
       </c>
       <c r="P3" t="n">
-        <v>0.452635</v>
+        <v>0.09657399999999999</v>
       </c>
       <c r="Q3" t="n">
-        <v>113.9</v>
+        <v>43.3</v>
       </c>
       <c r="R3" t="n">
-        <v>10176.4</v>
+        <v>6353.5</v>
       </c>
       <c r="S3" t="n">
-        <v>1123.7</v>
+        <v>1524.8</v>
       </c>
       <c r="T3" t="n">
-        <v>9052.700000000001</v>
+        <v>4828.7</v>
       </c>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="n">
-        <v>95.52129303831462</v>
+        <v>383.8588628629582</v>
       </c>
       <c r="W3" t="n">
-        <v>0.4671049934494679</v>
+        <v>1.293010406097319</v>
       </c>
       <c r="X3" t="n">
-        <v>0.01046887000994521</v>
+        <v>0.002605124166058427</v>
       </c>
       <c r="Y3" t="n">
-        <v>89.34503950834065</v>
+        <v>146.7321016166282</v>
       </c>
       <c r="Z3" t="n">
-        <v>5.228102153403404</v>
+        <v>8.81204856913731</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>gpt-6-astra</t>
+          <t>claude-opus-5-5-high</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (max)</t>
+          <t>Claude Opus 5.5 (Adaptive Reasoning, High Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (max)</t>
+          <t>Claude Opus 5.5 (high with fallback)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -771,82 +763,82 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>52.673669395513</v>
+        <v>53.5831959822067</v>
       </c>
       <c r="K4" t="n">
-        <v>33.58576156993391</v>
+        <v>144.8194486005587</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
-        <v>0.30341</v>
+        <v>0.078086</v>
       </c>
       <c r="N4" t="n">
-        <v>0.022917</v>
+        <v>0.018005</v>
       </c>
       <c r="O4" t="n">
-        <v>0.022384</v>
+        <v>0.027341</v>
       </c>
       <c r="P4" t="n">
-        <v>0.25811</v>
+        <v>0.03274</v>
       </c>
       <c r="Q4" t="n">
-        <v>94.09999999999999</v>
+        <v>22.2</v>
       </c>
       <c r="R4" t="n">
-        <v>5609.9</v>
+        <v>3004</v>
       </c>
       <c r="S4" t="n">
-        <v>447.7</v>
+        <v>1367.1</v>
       </c>
       <c r="T4" t="n">
-        <v>5162.2</v>
+        <v>1637</v>
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="n">
-        <v>173.6055812119343</v>
+        <v>686.2074633379441</v>
       </c>
       <c r="W4" t="n">
-        <v>0.5597626928322317</v>
+        <v>2.413657476675978</v>
       </c>
       <c r="X4" t="n">
-        <v>0.005760183474627001</v>
+        <v>0.001457285228487116</v>
       </c>
       <c r="Y4" t="n">
-        <v>59.6163655685441</v>
+        <v>135.3153153153153</v>
       </c>
       <c r="Z4" t="n">
-        <v>9.389413250773277</v>
+        <v>17.83728228435643</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>gpt-6-astra-xhigh</t>
+          <t>claude-fable-5-1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (xhigh)</t>
+          <t>Claude Fable 5.1 (Adaptive Reasoning, Max Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (xhigh)</t>
+          <t>Claude Fable 5.1 (max with fallback)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -861,67 +853,67 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>52.3863277108782</v>
+        <v>53.3549259623252</v>
       </c>
       <c r="K5" t="n">
-        <v>56.83869191053692</v>
+        <v>15.00138499409331</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
-        <v>0.172456</v>
+        <v>1.203406</v>
       </c>
       <c r="N5" t="n">
-        <v>0.023073</v>
+        <v>0.051436</v>
       </c>
       <c r="O5" t="n">
-        <v>0.02257</v>
+        <v>0.064901</v>
       </c>
       <c r="P5" t="n">
-        <v>0.126814</v>
+        <v>1.087069</v>
       </c>
       <c r="Q5" t="n">
-        <v>55.3</v>
+        <v>213.4</v>
       </c>
       <c r="R5" t="n">
-        <v>2987.7</v>
+        <v>23039.4</v>
       </c>
       <c r="S5" t="n">
-        <v>451.4</v>
+        <v>1298</v>
       </c>
       <c r="T5" t="n">
-        <v>2536.3</v>
+        <v>21741.4</v>
       </c>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="n">
-        <v>303.7663387233741</v>
+        <v>44.3365962628782</v>
       </c>
       <c r="W5" t="n">
-        <v>0.9473115318422821</v>
+        <v>0.2500230832348885</v>
       </c>
       <c r="X5" t="n">
-        <v>0.003292003992946215</v>
+        <v>0.022554730951173</v>
       </c>
       <c r="Y5" t="n">
-        <v>54.02712477396022</v>
+        <v>107.9634489222118</v>
       </c>
       <c r="Z5" t="n">
-        <v>17.53399863134793</v>
+        <v>2.315812302504631</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>claude-fable-5-1-high</t>
+          <t>claude-fable-5-1-xhigh</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (Adaptive Reasoning, High Effort, Default Fallback)</t>
+          <t>Claude Fable 5.1 (Adaptive Reasoning, Xhigh Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (high with fallback)</t>
+          <t>Claude Fable 5.1 (xhigh with fallback)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -951,67 +943,67 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>51.1515708852237</v>
+        <v>53.2032587538944</v>
       </c>
       <c r="K6" t="n">
-        <v>77.89579322622899</v>
+        <v>30.72372979050687</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
-        <v>0.214587</v>
+        <v>0.556978</v>
       </c>
       <c r="N6" t="n">
-        <v>0.044761</v>
+        <v>0.048158</v>
       </c>
       <c r="O6" t="n">
-        <v>0.046826</v>
+        <v>0.056185</v>
       </c>
       <c r="P6" t="n">
-        <v>0.123</v>
+        <v>0.452635</v>
       </c>
       <c r="Q6" t="n">
-        <v>39.4</v>
+        <v>103.9</v>
       </c>
       <c r="R6" t="n">
-        <v>3396.5</v>
+        <v>10176.4</v>
       </c>
       <c r="S6" t="n">
-        <v>936.5</v>
+        <v>1123.7</v>
       </c>
       <c r="T6" t="n">
-        <v>2460</v>
+        <v>9052.700000000001</v>
       </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="n">
-        <v>238.3721795133149</v>
+        <v>95.52129303831462</v>
       </c>
       <c r="W6" t="n">
-        <v>1.29826322043715</v>
+        <v>0.5120621631751145</v>
       </c>
       <c r="X6" t="n">
-        <v>0.004195120429077348</v>
+        <v>0.01046887000994521</v>
       </c>
       <c r="Y6" t="n">
-        <v>86.20558375634518</v>
+        <v>97.94417709335899</v>
       </c>
       <c r="Z6" t="n">
-        <v>15.06008269843183</v>
+        <v>5.228102153403404</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>gpt-6-astra-high</t>
+          <t>gpt-6-astra</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (high)</t>
+          <t>GPT-6 Astra (max)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (high)</t>
+          <t>GPT-6 Astra (max)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1041,82 +1033,82 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>50.9191471636152</v>
+        <v>52.673669395513</v>
       </c>
       <c r="K7" t="n">
-        <v>101.4999611234854</v>
+        <v>29.18208830776344</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
-        <v>0.101844</v>
+        <v>0.30341</v>
       </c>
       <c r="N7" t="n">
-        <v>0.022658</v>
+        <v>0.022917</v>
       </c>
       <c r="O7" t="n">
-        <v>0.022004</v>
+        <v>0.022384</v>
       </c>
       <c r="P7" t="n">
-        <v>0.057183</v>
+        <v>0.25811</v>
       </c>
       <c r="Q7" t="n">
-        <v>30.1</v>
+        <v>108.3</v>
       </c>
       <c r="R7" t="n">
-        <v>1583.7</v>
+        <v>5609.9</v>
       </c>
       <c r="S7" t="n">
-        <v>440.1</v>
+        <v>447.7</v>
       </c>
       <c r="T7" t="n">
-        <v>1143.7</v>
+        <v>5162.2</v>
       </c>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="n">
-        <v>499.9719881742194</v>
+        <v>173.6055812119343</v>
       </c>
       <c r="W7" t="n">
-        <v>1.691666018724757</v>
+        <v>0.486368138462724</v>
       </c>
       <c r="X7" t="n">
-        <v>0.002000112053580773</v>
+        <v>0.005760183474627001</v>
       </c>
       <c r="Y7" t="n">
-        <v>52.61461794019934</v>
+        <v>51.79963065558633</v>
       </c>
       <c r="Z7" t="n">
-        <v>32.15201563655692</v>
+        <v>9.389413250773277</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>claude-opus-5</t>
+          <t>gpt-6-astra-xhigh</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Claude Opus 5 (Adaptive Reasoning, Max Effort)</t>
+          <t>GPT-6 Astra (xhigh)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Claude Opus 5 (max)</t>
+          <t>GPT-6 Astra (xhigh)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1131,67 +1123,67 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>50.7771115797629</v>
+        <v>52.3863277108782</v>
       </c>
       <c r="K8" t="n">
-        <v>26.79530954077198</v>
+        <v>53.91388786711308</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
-        <v>0.255456</v>
+        <v>0.172456</v>
       </c>
       <c r="N8" t="n">
-        <v>0.019565</v>
+        <v>0.023073</v>
       </c>
       <c r="O8" t="n">
-        <v>0.02643</v>
+        <v>0.02257</v>
       </c>
       <c r="P8" t="n">
-        <v>0.20946</v>
+        <v>0.126814</v>
       </c>
       <c r="Q8" t="n">
-        <v>113.7</v>
+        <v>58.3</v>
       </c>
       <c r="R8" t="n">
-        <v>9435.6</v>
+        <v>2987.7</v>
       </c>
       <c r="S8" t="n">
-        <v>1057.2</v>
+        <v>451.4</v>
       </c>
       <c r="T8" t="n">
-        <v>8378.4</v>
+        <v>2536.3</v>
       </c>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="n">
-        <v>198.7704793771252</v>
+        <v>303.7663387233741</v>
       </c>
       <c r="W8" t="n">
-        <v>0.4465884923461997</v>
+        <v>0.8985647977852178</v>
       </c>
       <c r="X8" t="n">
-        <v>0.005030928149560429</v>
+        <v>0.003292003992946215</v>
       </c>
       <c r="Y8" t="n">
-        <v>82.9868073878628</v>
+        <v>51.24699828473413</v>
       </c>
       <c r="Z8" t="n">
-        <v>5.381439609538651</v>
+        <v>17.53399863134793</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>claude-opus-5-xhigh</t>
+          <t>claude-opus-5-5-medium</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Claude Opus 5 (Adaptive Reasoning, Xhigh Effort)</t>
+          <t>Claude Opus 5.5 (Adaptive Reasoning, Medium Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Claude Opus 5 (xhigh)</t>
+          <t>Claude Opus 5.5 (medium with fallback)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1206,7 +1198,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1221,67 +1213,67 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>49.6773552926939</v>
+        <v>51.2434931792768</v>
       </c>
       <c r="K9" t="n">
-        <v>39.37438992815897</v>
+        <v>170.8116439309227</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
-        <v>0.177537</v>
+        <v>0.062154</v>
       </c>
       <c r="N9" t="n">
-        <v>0.018451</v>
+        <v>0.017457</v>
       </c>
       <c r="O9" t="n">
-        <v>0.022483</v>
+        <v>0.025716</v>
       </c>
       <c r="P9" t="n">
-        <v>0.136603</v>
+        <v>0.01898</v>
       </c>
       <c r="Q9" t="n">
-        <v>75.7</v>
+        <v>18</v>
       </c>
       <c r="R9" t="n">
-        <v>6363.5</v>
+        <v>2234.8</v>
       </c>
       <c r="S9" t="n">
-        <v>899.3</v>
+        <v>1285.8</v>
       </c>
       <c r="T9" t="n">
-        <v>5464.1</v>
+        <v>949</v>
       </c>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="n">
-        <v>279.8140967386736</v>
+        <v>824.4601019930624</v>
       </c>
       <c r="W9" t="n">
-        <v>0.6562398321359828</v>
+        <v>2.846860732182044</v>
       </c>
       <c r="X9" t="n">
-        <v>0.003573801361887527</v>
+        <v>0.001212914970151478</v>
       </c>
       <c r="Y9" t="n">
-        <v>84.06208718626155</v>
+        <v>124.1555555555556</v>
       </c>
       <c r="Z9" t="n">
-        <v>7.806608830469695</v>
+        <v>22.92978932310578</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>claude-fable-5</t>
+          <t>claude-opus-5</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Claude Fable 5 (Adaptive Reasoning, Max Effort, Opus 4.8 Fallback)</t>
+          <t>Claude Opus 5 (Adaptive Reasoning, Max Effort)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Claude Fable 5 (with fallback)</t>
+          <t>Claude Opus 5 (max)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1296,7 +1288,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1311,51 +1303,51 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>49.6258202733378</v>
+        <v>50.7771115797629</v>
       </c>
       <c r="K10" t="n">
-        <v>30.10666548433031</v>
+        <v>28.63370953746028</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
-        <v>0.520062</v>
+        <v>0.255456</v>
       </c>
       <c r="N10" t="n">
-        <v>0.036048</v>
+        <v>0.019565</v>
       </c>
       <c r="O10" t="n">
-        <v>0.046389</v>
+        <v>0.02643</v>
       </c>
       <c r="P10" t="n">
-        <v>0.437625</v>
+        <v>0.20946</v>
       </c>
       <c r="Q10" t="n">
-        <v>98.90000000000001</v>
+        <v>106.4</v>
       </c>
       <c r="R10" t="n">
-        <v>9680.299999999999</v>
+        <v>9435.6</v>
       </c>
       <c r="S10" t="n">
-        <v>927.8</v>
+        <v>1057.2</v>
       </c>
       <c r="T10" t="n">
-        <v>8752.5</v>
+        <v>8378.4</v>
       </c>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="n">
-        <v>95.42289241155439</v>
+        <v>198.7704793771252</v>
       </c>
       <c r="W10" t="n">
-        <v>0.5017777580721718</v>
+        <v>0.4772284922910047</v>
       </c>
       <c r="X10" t="n">
-        <v>0.01047966556795457</v>
+        <v>0.005030928149560429</v>
       </c>
       <c r="Y10" t="n">
-        <v>97.87967644084932</v>
+        <v>88.68045112781955</v>
       </c>
       <c r="Z10" t="n">
-        <v>5.126475447386735</v>
+        <v>5.381439609538651</v>
       </c>
     </row>
     <row r="11">
@@ -1404,7 +1396,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K11" t="n">
-        <v>31.09416644739343</v>
+        <v>36.06923307897637</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1420,7 +1412,7 @@
         <v>0.07542500000000001</v>
       </c>
       <c r="Q11" t="n">
-        <v>92.8</v>
+        <v>80</v>
       </c>
       <c r="R11" t="n">
         <v>18553.6</v>
@@ -1436,13 +1428,13 @@
         <v>578.4775641354948</v>
       </c>
       <c r="W11" t="n">
-        <v>0.5182361074565571</v>
+        <v>0.6011538846496063</v>
       </c>
       <c r="X11" t="n">
         <v>0.001728675513102135</v>
       </c>
       <c r="Y11" t="n">
-        <v>199.9310344827586</v>
+        <v>231.92</v>
       </c>
       <c r="Z11" t="n">
         <v>2.592074356026243</v>
@@ -1451,17 +1443,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>gpt-5-6-sol</t>
+          <t>gpt-6-sol</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>GPT-5.6 Sol (max)</t>
+          <t>GPT-6 Sol (max)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GPT-5.6 Sol (max)</t>
+          <t>GPT-6 Sol (max)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1476,7 +1468,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1491,82 +1483,82 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>46.9727068915036</v>
+        <v>47.5276426437724</v>
       </c>
       <c r="K12" t="n">
-        <v>29.17559434254882</v>
+        <v>41.1494741504523</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
-        <v>0.126688</v>
+        <v>0.08570700000000001</v>
       </c>
       <c r="N12" t="n">
-        <v>0.007634</v>
+        <v>0.00525</v>
       </c>
       <c r="O12" t="n">
-        <v>0.007934999999999999</v>
+        <v>0.003693</v>
       </c>
       <c r="P12" t="n">
-        <v>0.111119</v>
+        <v>0.076765</v>
       </c>
       <c r="Q12" t="n">
-        <v>96.59999999999999</v>
+        <v>69.3</v>
       </c>
       <c r="R12" t="n">
-        <v>5952.7</v>
+        <v>8045.8</v>
       </c>
       <c r="S12" t="n">
-        <v>396.7</v>
+        <v>369.3</v>
       </c>
       <c r="T12" t="n">
-        <v>5555.9</v>
+        <v>7676.5</v>
       </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="n">
-        <v>370.7747134022449</v>
+        <v>554.5362997628245</v>
       </c>
       <c r="W12" t="n">
-        <v>0.486259905709147</v>
+        <v>0.685824569174205</v>
       </c>
       <c r="X12" t="n">
-        <v>0.002697055553826625</v>
+        <v>0.001803308458666638</v>
       </c>
       <c r="Y12" t="n">
-        <v>61.62215320910973</v>
+        <v>116.1010101010101</v>
       </c>
       <c r="Z12" t="n">
-        <v>7.890991800612092</v>
+        <v>5.907136971310796</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>qwen3-8-max</t>
+          <t>gpt-5-6-sol</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>GPT-5.6 Sol (max)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>GPT-5.6 Sol (max)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1581,82 +1573,82 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>45.4152084980521</v>
+        <v>46.9727068915036</v>
       </c>
       <c r="K13" t="n">
-        <v>4.919502635643846</v>
+        <v>34.79459769741007</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
-        <v>0.156468</v>
+        <v>0.126688</v>
       </c>
       <c r="N13" t="n">
-        <v>0.007406</v>
+        <v>0.007634</v>
       </c>
       <c r="O13" t="n">
-        <v>0.007526</v>
+        <v>0.007934999999999999</v>
       </c>
       <c r="P13" t="n">
-        <v>0.141536</v>
+        <v>0.111119</v>
       </c>
       <c r="Q13" t="n">
-        <v>553.9</v>
+        <v>81</v>
       </c>
       <c r="R13" t="n">
-        <v>24843.6</v>
+        <v>5952.7</v>
       </c>
       <c r="S13" t="n">
-        <v>1254.3</v>
+        <v>396.7</v>
       </c>
       <c r="T13" t="n">
-        <v>23589.3</v>
+        <v>5555.9</v>
       </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="n">
-        <v>290.2523742749451</v>
+        <v>370.7747134022449</v>
       </c>
       <c r="W13" t="n">
-        <v>0.0819917105940641</v>
+        <v>0.5799099616235012</v>
       </c>
       <c r="X13" t="n">
-        <v>0.003445277588161046</v>
+        <v>0.002697055553826625</v>
       </c>
       <c r="Y13" t="n">
-        <v>44.85213937533851</v>
+        <v>73.49012345679012</v>
       </c>
       <c r="Z13" t="n">
-        <v>1.828044586857464</v>
+        <v>7.890991800612092</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>glm-5-3</t>
+          <t>grok-4-7</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>Grok 4.7 (xhigh)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>Grok 4.7 (xhigh)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>SpaceXAI</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>xai</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1668,85 +1660,85 @@
         <v>1</v>
       </c>
       <c r="I14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>44.777392385614</v>
+        <v>46.4465506302286</v>
       </c>
       <c r="K14" t="n">
-        <v>6.351403175264397</v>
+        <v>3.525800908165126</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>0.15892</v>
+        <v>0.350873</v>
       </c>
       <c r="N14" t="n">
-        <v>0.006115</v>
+        <v>0.008541999999999999</v>
       </c>
       <c r="O14" t="n">
-        <v>0.004153</v>
+        <v>0.004758</v>
       </c>
       <c r="P14" t="n">
-        <v>0.148652</v>
+        <v>0.337573</v>
       </c>
       <c r="Q14" t="n">
-        <v>423</v>
+        <v>790.4</v>
       </c>
       <c r="R14" t="n">
-        <v>34728.3</v>
+        <v>57055.2</v>
       </c>
       <c r="S14" t="n">
-        <v>943.8</v>
+        <v>793</v>
       </c>
       <c r="T14" t="n">
-        <v>33784.5</v>
+        <v>56262.1</v>
       </c>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="n">
-        <v>281.760586368072</v>
+        <v>132.374251168453</v>
       </c>
       <c r="W14" t="n">
-        <v>0.10585671958774</v>
+        <v>0.05876334846941877</v>
       </c>
       <c r="X14" t="n">
-        <v>0.003549112432260739</v>
+        <v>0.007554339240245816</v>
       </c>
       <c r="Y14" t="n">
-        <v>82.10000000000001</v>
+        <v>72.18522267206478</v>
       </c>
       <c r="Z14" t="n">
-        <v>1.289363210569305</v>
+        <v>0.814063409298865</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>grok-4-6</t>
+          <t>mimo-v2-6-pro</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Grok 4.6 (high)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Grok 4.6 (high)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>SpaceXAI</t>
+          <t>Xiaomi</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>xai</t>
+          <t>xiaomi</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1758,85 +1750,85 @@
         <v>1</v>
       </c>
       <c r="I15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" t="n">
-        <v>44.3113073012592</v>
+        <v>46.3242065310383</v>
       </c>
       <c r="K15" t="n">
-        <v>15.23597958782551</v>
+        <v>7.829443357358586</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>0.066873</v>
+        <v>0.021122</v>
       </c>
       <c r="N15" t="n">
-        <v>0.005686</v>
+        <v>0.003029</v>
       </c>
       <c r="O15" t="n">
-        <v>0.003091</v>
+        <v>0.002893</v>
       </c>
       <c r="P15" t="n">
-        <v>0.058096</v>
+        <v>0.0152</v>
       </c>
       <c r="Q15" t="n">
-        <v>174.5</v>
+        <v>355</v>
       </c>
       <c r="R15" t="n">
-        <v>10197.8</v>
+        <v>20796.5</v>
       </c>
       <c r="S15" t="n">
-        <v>515.2</v>
+        <v>3325.3</v>
       </c>
       <c r="T15" t="n">
-        <v>9682.6</v>
+        <v>17471.2</v>
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="n">
-        <v>662.6188043195191</v>
+        <v>2193.173304187023</v>
       </c>
       <c r="W15" t="n">
-        <v>0.2539329931304252</v>
+        <v>0.1304907226226431</v>
       </c>
       <c r="X15" t="n">
-        <v>0.001509163328117374</v>
+        <v>0.0004559603192738502</v>
       </c>
       <c r="Y15" t="n">
-        <v>58.44011461318051</v>
+        <v>58.58169014084507</v>
       </c>
       <c r="Z15" t="n">
-        <v>4.345183010184472</v>
+        <v>2.227500133726266</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>step-5</t>
+          <t>qwen3-8-max</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>StepFun</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>stepfun</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1851,82 +1843,82 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>43.7343049141614</v>
+        <v>45.4152084980521</v>
       </c>
       <c r="K16" t="n">
-        <v>14.84195868127649</v>
+        <v>5.831184485091218</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
-        <v>0.044989</v>
+        <v>0.156468</v>
       </c>
       <c r="N16" t="n">
-        <v>0.003221</v>
+        <v>0.007406</v>
       </c>
       <c r="O16" t="n">
-        <v>0.002192</v>
+        <v>0.007526</v>
       </c>
       <c r="P16" t="n">
-        <v>0.039576</v>
+        <v>0.141536</v>
       </c>
       <c r="Q16" t="n">
-        <v>176.8</v>
+        <v>467.3</v>
       </c>
       <c r="R16" t="n">
-        <v>15469.6</v>
+        <v>24843.6</v>
       </c>
       <c r="S16" t="n">
-        <v>811.7</v>
+        <v>1254.3</v>
       </c>
       <c r="T16" t="n">
-        <v>14657.8</v>
+        <v>23589.3</v>
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="n">
-        <v>972.1110696872879</v>
+        <v>290.2523742749451</v>
       </c>
       <c r="W16" t="n">
-        <v>0.2473659780212749</v>
+        <v>0.09718640808485363</v>
       </c>
       <c r="X16" t="n">
-        <v>0.001028689036862509</v>
+        <v>0.003445277588161046</v>
       </c>
       <c r="Y16" t="n">
-        <v>87.49773755656108</v>
+        <v>53.16413438904344</v>
       </c>
       <c r="Z16" t="n">
-        <v>2.827112848047875</v>
+        <v>1.828044586857464</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>kimi-k3</t>
+          <t>glm-5-3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Kimi K3 (max)</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Kimi K3 (max)</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Kimi</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>kimi</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1941,82 +1933,82 @@
         <v>1</v>
       </c>
       <c r="J17" t="n">
-        <v>43.5938229518782</v>
+        <v>44.777392385614</v>
       </c>
       <c r="K17" t="n">
-        <v>10.75063451341016</v>
+        <v>5.704126418549555</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
-        <v>0.163338</v>
+        <v>0.15892</v>
       </c>
       <c r="N17" t="n">
-        <v>0.007471</v>
+        <v>0.006115</v>
       </c>
       <c r="O17" t="n">
-        <v>0.007591</v>
+        <v>0.004153</v>
       </c>
       <c r="P17" t="n">
-        <v>0.148276</v>
+        <v>0.148652</v>
       </c>
       <c r="Q17" t="n">
-        <v>243.3</v>
+        <v>471</v>
       </c>
       <c r="R17" t="n">
-        <v>10391.2</v>
+        <v>34728.3</v>
       </c>
       <c r="S17" t="n">
-        <v>506.1</v>
+        <v>943.8</v>
       </c>
       <c r="T17" t="n">
-        <v>9885.1</v>
+        <v>33784.5</v>
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="n">
-        <v>266.8933313244817</v>
+        <v>281.760586368072</v>
       </c>
       <c r="W17" t="n">
-        <v>0.1791772418901693</v>
+        <v>0.09506877364249257</v>
       </c>
       <c r="X17" t="n">
-        <v>0.0037468152352755</v>
+        <v>0.003549112432260739</v>
       </c>
       <c r="Y17" t="n">
-        <v>42.70941224825319</v>
+        <v>73.73312101910828</v>
       </c>
       <c r="Z17" t="n">
-        <v>4.195263583789957</v>
+        <v>1.289363210569305</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>gpt-5-6-terra</t>
+          <t>grok-4-6</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>GPT-5.6 Terra (max)</t>
+          <t>Grok 4.6 (high)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GPT-5.6 Terra (max)</t>
+          <t>Grok 4.6 (high)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>SpaceXAI</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>xai</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2031,82 +2023,82 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>42.0829248239494</v>
+        <v>44.3113073012592</v>
       </c>
       <c r="K18" t="n">
-        <v>20.08731495176582</v>
+        <v>15.85377720975284</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
-        <v>0.14583</v>
+        <v>0.066873</v>
       </c>
       <c r="N18" t="n">
-        <v>0.004243</v>
+        <v>0.005686</v>
       </c>
       <c r="O18" t="n">
-        <v>0.004487</v>
+        <v>0.003091</v>
       </c>
       <c r="P18" t="n">
-        <v>0.137101</v>
+        <v>0.058096</v>
       </c>
       <c r="Q18" t="n">
-        <v>125.7</v>
+        <v>167.7</v>
       </c>
       <c r="R18" t="n">
-        <v>11799</v>
+        <v>10197.8</v>
       </c>
       <c r="S18" t="n">
-        <v>373.9</v>
+        <v>515.2</v>
       </c>
       <c r="T18" t="n">
-        <v>11425.1</v>
+        <v>9682.6</v>
       </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="n">
-        <v>288.57522336933</v>
+        <v>662.6188043195191</v>
       </c>
       <c r="W18" t="n">
-        <v>0.3347885825294304</v>
+        <v>0.2642296201625474</v>
       </c>
       <c r="X18" t="n">
-        <v>0.003465300964941679</v>
+        <v>0.001509163328117374</v>
       </c>
       <c r="Y18" t="n">
-        <v>93.86634844868735</v>
+        <v>60.8097793679189</v>
       </c>
       <c r="Z18" t="n">
-        <v>3.566651819980456</v>
+        <v>4.345183010184472</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>glm-5-3-flash</t>
+          <t>step-5</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>GLM 5.3 Flash</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>StepFun</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>stepfun</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2118,85 +2110,85 @@
         <v>1</v>
       </c>
       <c r="I19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>41.807466113455</v>
+        <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>6.855556072170812</v>
+        <v>15.98086659469966</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
-        <v>0.022786</v>
+        <v>0.044989</v>
       </c>
       <c r="N19" t="n">
-        <v>0.000576</v>
+        <v>0.003221</v>
       </c>
       <c r="O19" t="n">
-        <v>0.000417</v>
+        <v>0.002192</v>
       </c>
       <c r="P19" t="n">
-        <v>0.021793</v>
+        <v>0.039576</v>
       </c>
       <c r="Q19" t="n">
-        <v>365.9</v>
+        <v>164.2</v>
       </c>
       <c r="R19" t="n">
-        <v>44420.3</v>
+        <v>15469.6</v>
       </c>
       <c r="S19" t="n">
-        <v>834.1</v>
+        <v>811.7</v>
       </c>
       <c r="T19" t="n">
-        <v>43586.3</v>
+        <v>14657.8</v>
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="n">
-        <v>1834.787418303125</v>
+        <v>972.1110696872879</v>
       </c>
       <c r="W19" t="n">
-        <v>0.1142592678695135</v>
+        <v>0.2663477765783276</v>
       </c>
       <c r="X19" t="n">
-        <v>0.0005450222679883181</v>
+        <v>0.001028689036862509</v>
       </c>
       <c r="Y19" t="n">
-        <v>121.4001093194862</v>
+        <v>94.21193666260659</v>
       </c>
       <c r="Z19" t="n">
-        <v>0.9411792831983349</v>
+        <v>2.827112848047875</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>gemini-3-8-flash</t>
+          <t>kimi-k3</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>Kimi K3 (max)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>Kimi K3 (max)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Kimi</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>kimi</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2208,85 +2200,85 @@
         <v>1</v>
       </c>
       <c r="I20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20" t="n">
-        <v>40.9262321765904</v>
+        <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>31.72576137720186</v>
+        <v>9.859138247692016</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
-        <v>0.093127</v>
+        <v>0.163338</v>
       </c>
       <c r="N20" t="n">
-        <v>0.001995</v>
+        <v>0.007471</v>
       </c>
       <c r="O20" t="n">
-        <v>0.002368</v>
+        <v>0.007591</v>
       </c>
       <c r="P20" t="n">
-        <v>0.088764</v>
+        <v>0.148276</v>
       </c>
       <c r="Q20" t="n">
-        <v>77.40000000000001</v>
+        <v>265.3</v>
       </c>
       <c r="R20" t="n">
-        <v>24301.8</v>
+        <v>10391.2</v>
       </c>
       <c r="S20" t="n">
-        <v>631.5</v>
+        <v>506.1</v>
       </c>
       <c r="T20" t="n">
-        <v>23670.3</v>
+        <v>9885.1</v>
       </c>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="n">
-        <v>439.4668804599139</v>
+        <v>266.8933313244817</v>
       </c>
       <c r="W20" t="n">
-        <v>0.528762689620031</v>
+        <v>0.164318970794867</v>
       </c>
       <c r="X20" t="n">
-        <v>0.002275484329907804</v>
+        <v>0.0037468152352755</v>
       </c>
       <c r="Y20" t="n">
-        <v>313.9767441860465</v>
+        <v>39.16773464003015</v>
       </c>
       <c r="Z20" t="n">
-        <v>1.684082338616498</v>
+        <v>4.195263583789957</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>deepseek-v4-1-flash</t>
+          <t>glm-5-3-flash</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (Reasoning, Max Effort)</t>
+          <t>GLM 5.3 Flash</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (max)</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>DeepSeek</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>deepseek</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2301,87 +2293,87 @@
         <v>1</v>
       </c>
       <c r="J21" t="n">
-        <v>39.456167472527</v>
+        <v>41.807466113455</v>
       </c>
       <c r="K21" t="n">
-        <v>28.97637758080318</v>
+        <v>3.906022994094207</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
-        <v>0.027666</v>
+        <v>0.022786</v>
       </c>
       <c r="N21" t="n">
-        <v>0.000862</v>
+        <v>0.000576</v>
       </c>
       <c r="O21" t="n">
-        <v>0.000595</v>
+        <v>0.000417</v>
       </c>
       <c r="P21" t="n">
-        <v>0.02621</v>
+        <v>0.021793</v>
       </c>
       <c r="Q21" t="n">
-        <v>81.7</v>
+        <v>642.2</v>
       </c>
       <c r="R21" t="n">
-        <v>22336.9</v>
+        <v>44420.3</v>
       </c>
       <c r="S21" t="n">
-        <v>495.4</v>
+        <v>834.1</v>
       </c>
       <c r="T21" t="n">
-        <v>21841.5</v>
+        <v>43586.3</v>
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="n">
-        <v>1426.160900474481</v>
+        <v>1834.787418303125</v>
       </c>
       <c r="W21" t="n">
-        <v>0.4829396263467197</v>
+        <v>0.06510038323490346</v>
       </c>
       <c r="X21" t="n">
-        <v>0.0007011831551876802</v>
+        <v>0.0005450222679883181</v>
       </c>
       <c r="Y21" t="n">
-        <v>273.4014687882497</v>
+        <v>69.16895048271566</v>
       </c>
       <c r="Z21" t="n">
-        <v>1.76641196730643</v>
+        <v>0.9411792831983349</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>gpt-5-6-luna</t>
+          <t>gemini-3-8-flash</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GPT-5.6 Luna (max)</t>
+          <t>Gemini 3.8 Flash (high)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GPT-5.6 Luna (max)</t>
+          <t>Gemini 3.8 Flash (high)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H22" t="b">
@@ -2391,67 +2383,67 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>37.3244239690841</v>
+        <v>40.9262321765904</v>
       </c>
       <c r="K22" t="n">
-        <v>27.64772145858081</v>
+        <v>29.94602354384664</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
-        <v>0.016448</v>
+        <v>0.093127</v>
       </c>
       <c r="N22" t="n">
-        <v>0.000637</v>
+        <v>0.001995</v>
       </c>
       <c r="O22" t="n">
-        <v>0.000541</v>
+        <v>0.002368</v>
       </c>
       <c r="P22" t="n">
-        <v>0.015269</v>
+        <v>0.088764</v>
       </c>
       <c r="Q22" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="R22" t="n">
-        <v>13175.4</v>
+        <v>24301.8</v>
       </c>
       <c r="S22" t="n">
-        <v>451.2</v>
+        <v>631.5</v>
       </c>
       <c r="T22" t="n">
-        <v>12724.3</v>
+        <v>23670.3</v>
       </c>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="n">
-        <v>2269.237838587312</v>
+        <v>439.4668804599139</v>
       </c>
       <c r="W22" t="n">
-        <v>0.4607953576430136</v>
+        <v>0.499100392397444</v>
       </c>
       <c r="X22" t="n">
-        <v>0.0004406765932576458</v>
+        <v>0.002275484329907804</v>
       </c>
       <c r="Y22" t="n">
-        <v>162.6592592592592</v>
+        <v>296.3634146341464</v>
       </c>
       <c r="Z22" t="n">
-        <v>2.832887348322184</v>
+        <v>1.684082338616498</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>deepseek-v4-pro</t>
+          <t>deepseek-v4-1-flash</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DeepSeek V4 Pro 0813 (Reasoning, Max Effort)</t>
+          <t>DeepSeek V4.1 Flash (Reasoning, Max Effort)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DeepSeek V4 Pro 0813 (max)</t>
+          <t>DeepSeek V4.1 Flash (max)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2466,7 +2458,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2481,239 +2473,267 @@
         <v>1</v>
       </c>
       <c r="J23" t="n">
-        <v>35.9967791278402</v>
+        <v>39.456167472527</v>
       </c>
       <c r="K23" t="n">
-        <v>9.269556856954559</v>
+        <v>33.24957933078117</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
-        <v>0.101663</v>
+        <v>0.027666</v>
       </c>
       <c r="N23" t="n">
-        <v>0.003745</v>
+        <v>0.000862</v>
       </c>
       <c r="O23" t="n">
-        <v>0.001918</v>
+        <v>0.000595</v>
       </c>
       <c r="P23" t="n">
-        <v>0.096</v>
+        <v>0.02621</v>
       </c>
       <c r="Q23" t="n">
-        <v>233</v>
+        <v>71.2</v>
       </c>
       <c r="R23" t="n">
-        <v>24726.8</v>
+        <v>22336.9</v>
       </c>
       <c r="S23" t="n">
-        <v>484.3</v>
+        <v>495.4</v>
       </c>
       <c r="T23" t="n">
-        <v>24242.5</v>
+        <v>21841.5</v>
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="n">
-        <v>354.0794500244946</v>
+        <v>1426.160900474481</v>
       </c>
       <c r="W23" t="n">
-        <v>0.154492614282576</v>
+        <v>0.5541596555130196</v>
       </c>
       <c r="X23" t="n">
-        <v>0.002824224901871096</v>
+        <v>0.0007011831551876802</v>
       </c>
       <c r="Y23" t="n">
-        <v>106.1236051502146</v>
+        <v>313.7205056179776</v>
       </c>
       <c r="Z23" t="n">
-        <v>1.455779928168635</v>
+        <v>1.76641196730643</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>qwen3-8-27b</t>
+          <t>gpt-5-6-luna</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (xhigh)</t>
+          <t>GPT-5.6 Luna (max)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (xhigh)</t>
+          <t>GPT-5.6 Luna (max)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H24" t="b">
         <v>1</v>
       </c>
       <c r="I24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>33.6962858057476</v>
+        <v>37.3244239690841</v>
       </c>
       <c r="K24" t="n">
-        <v>3.459577598126037</v>
+        <v>23.49911267728275</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>0.09057999999999999</v>
+        <v>0.016448</v>
       </c>
       <c r="N24" t="n">
-        <v>0.001883</v>
+        <v>0.000637</v>
       </c>
       <c r="O24" t="n">
-        <v>0.003858</v>
+        <v>0.000541</v>
       </c>
       <c r="P24" t="n">
-        <v>0.084838</v>
+        <v>0.015269</v>
       </c>
       <c r="Q24" t="n">
-        <v>584.4</v>
+        <v>95.3</v>
       </c>
       <c r="R24" t="n">
-        <v>29565.5</v>
+        <v>13175.4</v>
       </c>
       <c r="S24" t="n">
-        <v>1286.1</v>
+        <v>451.2</v>
       </c>
       <c r="T24" t="n">
-        <v>28279.4</v>
+        <v>12724.3</v>
       </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="n">
-        <v>372.0058048768779</v>
+        <v>2269.237838587312</v>
       </c>
       <c r="W24" t="n">
-        <v>0.05765962663543395</v>
+        <v>0.3916518779547125</v>
       </c>
       <c r="X24" t="n">
-        <v>0.002688130096063873</v>
+        <v>0.0004406765932576458</v>
       </c>
       <c r="Y24" t="n">
-        <v>50.59120465434634</v>
+        <v>138.2518363064008</v>
       </c>
       <c r="Z24" t="n">
-        <v>1.139716419669804</v>
+        <v>2.832887348322184</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>k2-horizon-375b-a23b</t>
+          <t>gpt-6-luna</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>GPT-6 Luna (max)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>GPT-6 Luna (max)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Institute of Foundation Models</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ifm</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H25" t="b">
         <v>1</v>
       </c>
       <c r="I25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>30.5015302696723</v>
-      </c>
-      <c r="K25" t="inlineStr"/>
+        <v>37.2559686869738</v>
+      </c>
+      <c r="K25" t="n">
+        <v>20.28455645388773</v>
+      </c>
       <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
+      <c r="M25" t="n">
+        <v>0.008175999999999999</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0.000295</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0.000254</v>
+      </c>
+      <c r="P25" t="n">
+        <v>0.007626</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>110.2</v>
+      </c>
+      <c r="R25" t="n">
+        <v>15761.3</v>
+      </c>
+      <c r="S25" t="n">
+        <v>508.9</v>
+      </c>
+      <c r="T25" t="n">
+        <v>15252.5</v>
+      </c>
       <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
-      <c r="Z25" t="inlineStr"/>
+      <c r="V25" t="n">
+        <v>4556.747637839262</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0.3380759408981289</v>
+      </c>
+      <c r="X25" t="n">
+        <v>0.0002194547689444097</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>143.024500907441</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>2.363762423592839</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>minimax-m3</t>
+          <t>qwen3-8-27b</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>Qwen3.8 27B (xhigh)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>Qwen3.8 27B (xhigh)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>minimax</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H26" t="b">
@@ -2723,82 +2743,82 @@
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>29.2202932236316</v>
+        <v>33.6962858057476</v>
       </c>
       <c r="K26" t="n">
-        <v>18.77106631068411</v>
+        <v>3.45602931341001</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
-        <v>0.026465</v>
+        <v>0.09057999999999999</v>
       </c>
       <c r="N26" t="n">
-        <v>0.004611</v>
+        <v>0.001883</v>
       </c>
       <c r="O26" t="n">
-        <v>0.00061</v>
+        <v>0.003858</v>
       </c>
       <c r="P26" t="n">
-        <v>0.021244</v>
+        <v>0.084838</v>
       </c>
       <c r="Q26" t="n">
-        <v>93.40000000000001</v>
+        <v>585</v>
       </c>
       <c r="R26" t="n">
-        <v>18211.1</v>
+        <v>29565.5</v>
       </c>
       <c r="S26" t="n">
-        <v>508</v>
+        <v>1286.1</v>
       </c>
       <c r="T26" t="n">
-        <v>17703.1</v>
+        <v>28279.4</v>
       </c>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="n">
-        <v>1104.110834068831</v>
+        <v>372.0058048768779</v>
       </c>
       <c r="W26" t="n">
-        <v>0.3128511051780685</v>
+        <v>0.0576004885568335</v>
       </c>
       <c r="X26" t="n">
-        <v>0.0009057061747277989</v>
+        <v>0.002688130096063873</v>
       </c>
       <c r="Y26" t="n">
-        <v>194.9796573875803</v>
+        <v>50.53931623931624</v>
       </c>
       <c r="Z26" t="n">
-        <v>1.604532028467891</v>
+        <v>1.139716419669804</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>inkling</t>
+          <t>k2-horizon-375b-a23b</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Inkling (xhigh)</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Inkling</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Thinking Machines</t>
+          <t>Institute of Foundation Models</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>thinking-machines</t>
+          <t>ifm</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2813,82 +2833,54 @@
         <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>24.9847810999384</v>
-      </c>
-      <c r="K27" t="n">
-        <v>5.449243424195943</v>
-      </c>
+        <v>30.5015302696723</v>
+      </c>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
-      <c r="M27" t="n">
-        <v>0.09468799999999999</v>
-      </c>
-      <c r="N27" t="n">
-        <v>0.002374</v>
-      </c>
-      <c r="O27" t="n">
-        <v>0.001895</v>
-      </c>
-      <c r="P27" t="n">
-        <v>0.09042</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>275.1</v>
-      </c>
-      <c r="R27" t="n">
-        <v>22793.6</v>
-      </c>
-      <c r="S27" t="n">
-        <v>467.8</v>
-      </c>
-      <c r="T27" t="n">
-        <v>22325.9</v>
-      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
-      <c r="V27" t="n">
-        <v>263.8642816401065</v>
-      </c>
-      <c r="W27" t="n">
-        <v>0.09082072373659904</v>
-      </c>
-      <c r="X27" t="n">
-        <v>0.00378982707998324</v>
-      </c>
-      <c r="Y27" t="n">
-        <v>82.85568884042165</v>
-      </c>
-      <c r="Z27" t="n">
-        <v>1.096131418465639</v>
-      </c>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
+          <t>minimax-m3</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>minimax</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2903,177 +2895,177 @@
         <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>22.9279123422858</v>
+        <v>29.2202932236316</v>
       </c>
       <c r="K28" t="n">
-        <v>18.59019919644794</v>
+        <v>10.81565449363292</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
-        <v>0.03175</v>
+        <v>0.026465</v>
       </c>
       <c r="N28" t="n">
-        <v>0.001525</v>
+        <v>0.004611</v>
       </c>
       <c r="O28" t="n">
-        <v>0.002749</v>
+        <v>0.00061</v>
       </c>
       <c r="P28" t="n">
-        <v>0.027475</v>
+        <v>0.021244</v>
       </c>
       <c r="Q28" t="n">
-        <v>74</v>
+        <v>162.1</v>
       </c>
       <c r="R28" t="n">
-        <v>12593.6</v>
+        <v>18211.1</v>
       </c>
       <c r="S28" t="n">
-        <v>1145.5</v>
+        <v>508</v>
       </c>
       <c r="T28" t="n">
-        <v>11448.1</v>
+        <v>17703.1</v>
       </c>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="n">
-        <v>722.1389714105763</v>
+        <v>1104.110834068831</v>
       </c>
       <c r="W28" t="n">
-        <v>0.3098366532741325</v>
+        <v>0.1802609082272153</v>
       </c>
       <c r="X28" t="n">
-        <v>0.001384775008121593</v>
+        <v>0.0009057061747277989</v>
       </c>
       <c r="Y28" t="n">
-        <v>170.1837837837838</v>
+        <v>112.3448488587292</v>
       </c>
       <c r="Z28" t="n">
-        <v>1.820600332096128</v>
+        <v>1.604532028467891</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>gemini-3-5-flash-lite</t>
+          <t>inkling</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash-Lite</t>
+          <t>Inkling (xhigh)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash-Lite</t>
+          <t>Inkling</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Thinking Machines</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>thinking-machines</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H29" t="b">
         <v>1</v>
       </c>
       <c r="I29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J29" t="n">
-        <v>22.1685424839812</v>
+        <v>24.9847810999384</v>
       </c>
       <c r="K29" t="n">
-        <v>68.21089995071138</v>
+        <v>8.536941150320636</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
-        <v>0.019232</v>
+        <v>0.09468799999999999</v>
       </c>
       <c r="N29" t="n">
-        <v>0.000782</v>
+        <v>0.002374</v>
       </c>
       <c r="O29" t="n">
-        <v>0.001426</v>
+        <v>0.001895</v>
       </c>
       <c r="P29" t="n">
-        <v>0.017024</v>
+        <v>0.09042</v>
       </c>
       <c r="Q29" t="n">
-        <v>19.5</v>
+        <v>175.6</v>
       </c>
       <c r="R29" t="n">
-        <v>7379.9</v>
+        <v>22793.6</v>
       </c>
       <c r="S29" t="n">
-        <v>570.5</v>
+        <v>467.8</v>
       </c>
       <c r="T29" t="n">
-        <v>6809.5</v>
+        <v>22325.9</v>
       </c>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="n">
-        <v>1152.690436979056</v>
+        <v>263.8642816401065</v>
       </c>
       <c r="W29" t="n">
-        <v>1.136848332511856</v>
+        <v>0.142282352505344</v>
       </c>
       <c r="X29" t="n">
-        <v>0.0008675356087977764</v>
+        <v>0.00378982707998324</v>
       </c>
       <c r="Y29" t="n">
-        <v>378.4564102564103</v>
+        <v>129.8041002277904</v>
       </c>
       <c r="Z29" t="n">
-        <v>3.003908248618708</v>
+        <v>1.096131418465639</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>muse-glimmer</t>
+          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Muse Glimmer (high)</t>
+          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Muse Glimmer (high)</t>
+          <t>Nemotron 3 Ultra</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>nvidia</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H30" t="b">
@@ -3083,82 +3075,82 @@
         <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>17.4754176089465</v>
+        <v>22.9279123422858</v>
       </c>
       <c r="K30" t="n">
-        <v>12.36468227048101</v>
+        <v>16.6546578757524</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
-        <v>0.012326</v>
+        <v>0.033009</v>
       </c>
       <c r="N30" t="n">
-        <v>0.00072</v>
+        <v>0.001525</v>
       </c>
       <c r="O30" t="n">
-        <v>0.00067</v>
+        <v>0.002864</v>
       </c>
       <c r="P30" t="n">
-        <v>0.010936</v>
+        <v>0.02862</v>
       </c>
       <c r="Q30" t="n">
-        <v>84.8</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="R30" t="n">
-        <v>7737.1</v>
+        <v>12593.6</v>
       </c>
       <c r="S30" t="n">
-        <v>446.4</v>
+        <v>1145.5</v>
       </c>
       <c r="T30" t="n">
-        <v>7290.7</v>
+        <v>11448.1</v>
       </c>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="n">
-        <v>1417.768749711707</v>
+        <v>694.5957872787968</v>
       </c>
       <c r="W30" t="n">
-        <v>0.2060780378413503</v>
+        <v>0.27757763126254</v>
       </c>
       <c r="X30" t="n">
-        <v>0.0007053336449991176</v>
+        <v>0.001439686243876714</v>
       </c>
       <c r="Y30" t="n">
-        <v>91.23938679245283</v>
+        <v>152.4648910411622</v>
       </c>
       <c r="Z30" t="n">
-        <v>2.258652157649054</v>
+        <v>1.820600332096128</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>mistral-medium-3-5</t>
+          <t>gemini-3-5-flash-lite</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mistral Medium 3.5</t>
+          <t>Gemini 3.5 Flash-Lite</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Mistral Medium 3.5</t>
+          <t>Gemini 3.5 Flash-Lite</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Mistral</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>mistral</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3170,90 +3162,90 @@
         <v>1</v>
       </c>
       <c r="I31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>14.1889227802691</v>
+        <v>22.1685424839812</v>
       </c>
       <c r="K31" t="n">
-        <v>9.114939687539035</v>
+        <v>65.20159554112118</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
-        <v>0.108206</v>
+        <v>0.019232</v>
       </c>
       <c r="N31" t="n">
-        <v>0.002141</v>
+        <v>0.000782</v>
       </c>
       <c r="O31" t="n">
-        <v>0.058389</v>
+        <v>0.001426</v>
       </c>
       <c r="P31" t="n">
-        <v>0.047676</v>
+        <v>0.017024</v>
       </c>
       <c r="Q31" t="n">
-        <v>93.40000000000001</v>
+        <v>20.4</v>
       </c>
       <c r="R31" t="n">
-        <v>14142</v>
+        <v>7379.9</v>
       </c>
       <c r="S31" t="n">
-        <v>7785.3</v>
+        <v>570.5</v>
       </c>
       <c r="T31" t="n">
-        <v>6356.8</v>
+        <v>6809.5</v>
       </c>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="n">
-        <v>131.1287985903656</v>
+        <v>1152.690436979056</v>
       </c>
       <c r="W31" t="n">
-        <v>0.1519156614589839</v>
+        <v>1.086693259018686</v>
       </c>
       <c r="X31" t="n">
-        <v>0.007626089850208333</v>
+        <v>0.0008675356087977764</v>
       </c>
       <c r="Y31" t="n">
-        <v>151.4132762312634</v>
+        <v>361.7598039215686</v>
       </c>
       <c r="Z31" t="n">
-        <v>1.003317973431558</v>
+        <v>3.003908248618708</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>gpt-oss-120b</t>
+          <t>muse-glimmer</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>gpt-oss-120b (high)</t>
+          <t>Muse Glimmer (high)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>gpt-oss-120b (high)</t>
+          <t>Muse Glimmer (high)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2025-08-05</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H32" t="b">
@@ -3263,51 +3255,141 @@
         <v>1</v>
       </c>
       <c r="J32" t="n">
-        <v>11.6028431512592</v>
+        <v>17.4754176089465</v>
       </c>
       <c r="K32" t="n">
-        <v>11.62221350710437</v>
+        <v>12.45279164533005</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
-        <v>0.007271</v>
+        <v>0.012326</v>
       </c>
       <c r="N32" t="n">
-        <v>0.000449</v>
+        <v>0.00072</v>
       </c>
       <c r="O32" t="n">
-        <v>0.000691</v>
+        <v>0.00067</v>
       </c>
       <c r="P32" t="n">
-        <v>0.006131</v>
+        <v>0.010936</v>
       </c>
       <c r="Q32" t="n">
-        <v>59.9</v>
+        <v>84.2</v>
       </c>
       <c r="R32" t="n">
-        <v>11465.4</v>
+        <v>7737.1</v>
       </c>
       <c r="S32" t="n">
-        <v>1161.3</v>
+        <v>446.4</v>
       </c>
       <c r="T32" t="n">
-        <v>10304</v>
+        <v>7290.7</v>
       </c>
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="n">
-        <v>1595.769928656196</v>
+        <v>1417.768749711707</v>
       </c>
       <c r="W32" t="n">
-        <v>0.1937035584517396</v>
+        <v>0.2075465274221674</v>
       </c>
       <c r="X32" t="n">
-        <v>0.0006266567517299338</v>
+        <v>0.0007053336449991176</v>
       </c>
       <c r="Y32" t="n">
-        <v>191.4090150250417</v>
+        <v>91.8895486935867</v>
       </c>
       <c r="Z32" t="n">
-        <v>1.011987645547404</v>
+        <v>2.258652157649054</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>mistral-medium-3-5</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Mistral Medium 3.5</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Mistral Medium 3.5</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Mistral</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>mistral</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H33" t="b">
+        <v>1</v>
+      </c>
+      <c r="I33" t="b">
+        <v>1</v>
+      </c>
+      <c r="J33" t="n">
+        <v>14.1889227802691</v>
+      </c>
+      <c r="K33" t="n">
+        <v>9.36562559753736</v>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="n">
+        <v>0.108206</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0.002141</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0.058389</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0.047676</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>90.90000000000001</v>
+      </c>
+      <c r="R33" t="n">
+        <v>14142</v>
+      </c>
+      <c r="S33" t="n">
+        <v>7785.3</v>
+      </c>
+      <c r="T33" t="n">
+        <v>6356.8</v>
+      </c>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="n">
+        <v>131.1287985903656</v>
+      </c>
+      <c r="W33" t="n">
+        <v>0.156093759958956</v>
+      </c>
+      <c r="X33" t="n">
+        <v>0.007626089850208333</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>155.5775577557756</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>1.003317973431558</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-09-24)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -676,7 +676,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K3" t="n">
-        <v>77.58062436583914</v>
+        <v>76.69500080001905</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -692,7 +692,7 @@
         <v>0.09657399999999999</v>
       </c>
       <c r="Q3" t="n">
-        <v>43.3</v>
+        <v>43.8</v>
       </c>
       <c r="R3" t="n">
         <v>6353.5</v>
@@ -708,13 +708,13 @@
         <v>383.8588628629582</v>
       </c>
       <c r="W3" t="n">
-        <v>1.293010406097319</v>
+        <v>1.278250013333651</v>
       </c>
       <c r="X3" t="n">
         <v>0.002605124166058427</v>
       </c>
       <c r="Y3" t="n">
-        <v>146.7321016166282</v>
+        <v>145.0570776255708</v>
       </c>
       <c r="Z3" t="n">
         <v>8.81204856913731</v>
@@ -766,7 +766,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K4" t="n">
-        <v>144.8194486005587</v>
+        <v>146.1359890423819</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -782,7 +782,7 @@
         <v>0.03274</v>
       </c>
       <c r="Q4" t="n">
-        <v>22.2</v>
+        <v>22</v>
       </c>
       <c r="R4" t="n">
         <v>3004</v>
@@ -798,13 +798,13 @@
         <v>686.2074633379441</v>
       </c>
       <c r="W4" t="n">
-        <v>2.413657476675978</v>
+        <v>2.435599817373032</v>
       </c>
       <c r="X4" t="n">
         <v>0.001457285228487116</v>
       </c>
       <c r="Y4" t="n">
-        <v>135.3153153153153</v>
+        <v>136.5454545454545</v>
       </c>
       <c r="Z4" t="n">
         <v>17.83728228435643</v>
@@ -946,7 +946,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K6" t="n">
-        <v>30.72372979050687</v>
+        <v>30.43084390117887</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -962,7 +962,7 @@
         <v>0.452635</v>
       </c>
       <c r="Q6" t="n">
-        <v>103.9</v>
+        <v>104.9</v>
       </c>
       <c r="R6" t="n">
         <v>10176.4</v>
@@ -978,13 +978,13 @@
         <v>95.52129303831462</v>
       </c>
       <c r="W6" t="n">
-        <v>0.5120621631751145</v>
+        <v>0.5071807316863146</v>
       </c>
       <c r="X6" t="n">
         <v>0.01046887000994521</v>
       </c>
       <c r="Y6" t="n">
-        <v>97.94417709335899</v>
+        <v>97.01048617731172</v>
       </c>
       <c r="Z6" t="n">
         <v>5.228102153403404</v>
@@ -1126,7 +1126,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K8" t="n">
-        <v>53.91388786711308</v>
+        <v>54.09947784255924</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1142,7 +1142,7 @@
         <v>0.126814</v>
       </c>
       <c r="Q8" t="n">
-        <v>58.3</v>
+        <v>58.1</v>
       </c>
       <c r="R8" t="n">
         <v>2987.7</v>
@@ -1158,13 +1158,13 @@
         <v>303.7663387233741</v>
       </c>
       <c r="W8" t="n">
-        <v>0.8985647977852178</v>
+        <v>0.901657964042654</v>
       </c>
       <c r="X8" t="n">
         <v>0.003292003992946215</v>
       </c>
       <c r="Y8" t="n">
-        <v>51.24699828473413</v>
+        <v>51.42340791738382</v>
       </c>
       <c r="Z8" t="n">
         <v>17.53399863134793</v>
@@ -1216,7 +1216,7 @@
         <v>51.2434931792768</v>
       </c>
       <c r="K9" t="n">
-        <v>170.8116439309227</v>
+        <v>177.7230977315958</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1232,7 +1232,7 @@
         <v>0.01898</v>
       </c>
       <c r="Q9" t="n">
-        <v>18</v>
+        <v>17.3</v>
       </c>
       <c r="R9" t="n">
         <v>2234.8</v>
@@ -1248,13 +1248,13 @@
         <v>824.4601019930624</v>
       </c>
       <c r="W9" t="n">
-        <v>2.846860732182044</v>
+        <v>2.96205162885993</v>
       </c>
       <c r="X9" t="n">
         <v>0.001212914970151478</v>
       </c>
       <c r="Y9" t="n">
-        <v>124.1555555555556</v>
+        <v>129.1791907514451</v>
       </c>
       <c r="Z9" t="n">
         <v>22.92978932310578</v>
@@ -1306,7 +1306,7 @@
         <v>50.7771115797629</v>
       </c>
       <c r="K10" t="n">
-        <v>28.63370953746028</v>
+        <v>28.36710144120832</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1322,7 @@
         <v>0.20946</v>
       </c>
       <c r="Q10" t="n">
-        <v>106.4</v>
+        <v>107.4</v>
       </c>
       <c r="R10" t="n">
         <v>9435.6</v>
@@ -1338,13 +1338,13 @@
         <v>198.7704793771252</v>
       </c>
       <c r="W10" t="n">
-        <v>0.4772284922910047</v>
+        <v>0.4727850240201387</v>
       </c>
       <c r="X10" t="n">
         <v>0.005030928149560429</v>
       </c>
       <c r="Y10" t="n">
-        <v>88.68045112781955</v>
+        <v>87.85474860335195</v>
       </c>
       <c r="Z10" t="n">
         <v>5.381439609538651</v>
@@ -1396,7 +1396,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K11" t="n">
-        <v>36.06923307897637</v>
+        <v>34.27005518192529</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1412,7 +1412,7 @@
         <v>0.07542500000000001</v>
       </c>
       <c r="Q11" t="n">
-        <v>80</v>
+        <v>84.2</v>
       </c>
       <c r="R11" t="n">
         <v>18553.6</v>
@@ -1428,13 +1428,13 @@
         <v>578.4775641354948</v>
       </c>
       <c r="W11" t="n">
-        <v>0.6011538846496063</v>
+        <v>0.5711675863654216</v>
       </c>
       <c r="X11" t="n">
         <v>0.001728675513102135</v>
       </c>
       <c r="Y11" t="n">
-        <v>231.92</v>
+        <v>220.3515439429929</v>
       </c>
       <c r="Z11" t="n">
         <v>2.592074356026243</v>
@@ -1486,7 +1486,7 @@
         <v>47.5276426437724</v>
       </c>
       <c r="K12" t="n">
-        <v>41.1494741504523</v>
+        <v>39.88333648428453</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1502,7 +1502,7 @@
         <v>0.076765</v>
       </c>
       <c r="Q12" t="n">
-        <v>69.3</v>
+        <v>71.5</v>
       </c>
       <c r="R12" t="n">
         <v>8045.8</v>
@@ -1518,13 +1518,13 @@
         <v>554.5362997628245</v>
       </c>
       <c r="W12" t="n">
-        <v>0.685824569174205</v>
+        <v>0.6647222747380755</v>
       </c>
       <c r="X12" t="n">
         <v>0.001803308458666638</v>
       </c>
       <c r="Y12" t="n">
-        <v>116.1010101010101</v>
+        <v>112.5286713286713</v>
       </c>
       <c r="Z12" t="n">
         <v>5.907136971310796</v>
@@ -1576,7 +1576,7 @@
         <v>46.9727068915036</v>
       </c>
       <c r="K13" t="n">
-        <v>34.79459769741007</v>
+        <v>35.2295301686277</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1592,7 +1592,7 @@
         <v>0.111119</v>
       </c>
       <c r="Q13" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="R13" t="n">
         <v>5952.7</v>
@@ -1608,13 +1608,13 @@
         <v>370.7747134022449</v>
       </c>
       <c r="W13" t="n">
-        <v>0.5799099616235012</v>
+        <v>0.5871588361437949</v>
       </c>
       <c r="X13" t="n">
         <v>0.002697055553826625</v>
       </c>
       <c r="Y13" t="n">
-        <v>73.49012345679012</v>
+        <v>74.40875</v>
       </c>
       <c r="Z13" t="n">
         <v>7.890991800612092</v>
@@ -1666,7 +1666,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K14" t="n">
-        <v>3.525800908165126</v>
+        <v>3.709294606433803</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1682,7 @@
         <v>0.337573</v>
       </c>
       <c r="Q14" t="n">
-        <v>790.4</v>
+        <v>751.3</v>
       </c>
       <c r="R14" t="n">
         <v>57055.2</v>
@@ -1698,13 +1698,13 @@
         <v>132.374251168453</v>
       </c>
       <c r="W14" t="n">
-        <v>0.05876334846941877</v>
+        <v>0.06182157677389671</v>
       </c>
       <c r="X14" t="n">
         <v>0.007554339240245816</v>
       </c>
       <c r="Y14" t="n">
-        <v>72.18522267206478</v>
+        <v>75.94196725675496</v>
       </c>
       <c r="Z14" t="n">
         <v>0.814063409298865</v>
@@ -1756,7 +1756,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K15" t="n">
-        <v>7.829443357358586</v>
+        <v>7.766002771339195</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1772,7 +1772,7 @@
         <v>0.0152</v>
       </c>
       <c r="Q15" t="n">
-        <v>355</v>
+        <v>357.9</v>
       </c>
       <c r="R15" t="n">
         <v>20796.5</v>
@@ -1788,13 +1788,13 @@
         <v>2193.173304187023</v>
       </c>
       <c r="W15" t="n">
-        <v>0.1304907226226431</v>
+        <v>0.1294333795223199</v>
       </c>
       <c r="X15" t="n">
         <v>0.0004559603192738502</v>
       </c>
       <c r="Y15" t="n">
-        <v>58.58169014084507</v>
+        <v>58.10701313215983</v>
       </c>
       <c r="Z15" t="n">
         <v>2.227500133726266</v>
@@ -1846,7 +1846,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K16" t="n">
-        <v>5.831184485091218</v>
+        <v>5.675718620877163</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1862,7 @@
         <v>0.141536</v>
       </c>
       <c r="Q16" t="n">
-        <v>467.3</v>
+        <v>480.1</v>
       </c>
       <c r="R16" t="n">
         <v>24843.6</v>
@@ -1878,13 +1878,13 @@
         <v>290.2523742749451</v>
       </c>
       <c r="W16" t="n">
-        <v>0.09718640808485363</v>
+        <v>0.09459531034795272</v>
       </c>
       <c r="X16" t="n">
         <v>0.003445277588161046</v>
       </c>
       <c r="Y16" t="n">
-        <v>53.16413438904344</v>
+        <v>51.74671943345136</v>
       </c>
       <c r="Z16" t="n">
         <v>1.828044586857464</v>
@@ -1936,7 +1936,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K17" t="n">
-        <v>5.704126418549555</v>
+        <v>5.681208591957793</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1952,7 @@
         <v>0.148652</v>
       </c>
       <c r="Q17" t="n">
-        <v>471</v>
+        <v>472.9</v>
       </c>
       <c r="R17" t="n">
         <v>34728.3</v>
@@ -1968,13 +1968,13 @@
         <v>281.760586368072</v>
       </c>
       <c r="W17" t="n">
-        <v>0.09506877364249257</v>
+        <v>0.09468680986596321</v>
       </c>
       <c r="X17" t="n">
         <v>0.003549112432260739</v>
       </c>
       <c r="Y17" t="n">
-        <v>73.73312101910828</v>
+        <v>73.43687883273421</v>
       </c>
       <c r="Z17" t="n">
         <v>1.289363210569305</v>
@@ -2116,7 +2116,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>15.98086659469966</v>
+        <v>16.82088650544669</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2132,7 @@
         <v>0.039576</v>
       </c>
       <c r="Q19" t="n">
-        <v>164.2</v>
+        <v>156</v>
       </c>
       <c r="R19" t="n">
         <v>15469.6</v>
@@ -2148,13 +2148,13 @@
         <v>972.1110696872879</v>
       </c>
       <c r="W19" t="n">
-        <v>0.2663477765783276</v>
+        <v>0.2803481084241115</v>
       </c>
       <c r="X19" t="n">
         <v>0.001028689036862509</v>
       </c>
       <c r="Y19" t="n">
-        <v>94.21193666260659</v>
+        <v>99.16410256410256</v>
       </c>
       <c r="Z19" t="n">
         <v>2.827112848047875</v>
@@ -2206,7 +2206,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>9.859138247692016</v>
+        <v>9.712697278546944</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2222,7 +2222,7 @@
         <v>0.148276</v>
       </c>
       <c r="Q20" t="n">
-        <v>265.3</v>
+        <v>269.3</v>
       </c>
       <c r="R20" t="n">
         <v>10391.2</v>
@@ -2238,13 +2238,13 @@
         <v>266.8933313244817</v>
       </c>
       <c r="W20" t="n">
-        <v>0.164318970794867</v>
+        <v>0.1618782879757824</v>
       </c>
       <c r="X20" t="n">
         <v>0.0037468152352755</v>
       </c>
       <c r="Y20" t="n">
-        <v>39.16773464003015</v>
+        <v>38.58596360935759</v>
       </c>
       <c r="Z20" t="n">
         <v>4.195263583789957</v>
@@ -2296,7 +2296,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K21" t="n">
-        <v>3.906022994094207</v>
+        <v>3.23170312652319</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.021793</v>
       </c>
       <c r="Q21" t="n">
-        <v>642.2</v>
+        <v>776.2</v>
       </c>
       <c r="R21" t="n">
         <v>44420.3</v>
@@ -2328,13 +2328,13 @@
         <v>1834.787418303125</v>
       </c>
       <c r="W21" t="n">
-        <v>0.06510038323490346</v>
+        <v>0.05386171877538649</v>
       </c>
       <c r="X21" t="n">
         <v>0.0005450222679883181</v>
       </c>
       <c r="Y21" t="n">
-        <v>69.16895048271566</v>
+        <v>57.22790517907756</v>
       </c>
       <c r="Z21" t="n">
         <v>0.9411792831983349</v>
@@ -2386,7 +2386,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K22" t="n">
-        <v>29.94602354384664</v>
+        <v>30.54196431088836</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.088764</v>
       </c>
       <c r="Q22" t="n">
-        <v>82</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="R22" t="n">
         <v>24301.8</v>
@@ -2418,13 +2418,13 @@
         <v>439.4668804599139</v>
       </c>
       <c r="W22" t="n">
-        <v>0.499100392397444</v>
+        <v>0.509032738514806</v>
       </c>
       <c r="X22" t="n">
         <v>0.002275484329907804</v>
       </c>
       <c r="Y22" t="n">
-        <v>296.3634146341464</v>
+        <v>302.2611940298507</v>
       </c>
       <c r="Z22" t="n">
         <v>1.684082338616498</v>
@@ -2566,7 +2566,7 @@
         <v>37.3244239690841</v>
       </c>
       <c r="K24" t="n">
-        <v>23.49911267728275</v>
+        <v>21.72129425940879</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2582,7 +2582,7 @@
         <v>0.015269</v>
       </c>
       <c r="Q24" t="n">
-        <v>95.3</v>
+        <v>103.1</v>
       </c>
       <c r="R24" t="n">
         <v>13175.4</v>
@@ -2598,13 +2598,13 @@
         <v>2269.237838587312</v>
       </c>
       <c r="W24" t="n">
-        <v>0.3916518779547125</v>
+        <v>0.3620215709901465</v>
       </c>
       <c r="X24" t="n">
         <v>0.0004406765932576458</v>
       </c>
       <c r="Y24" t="n">
-        <v>138.2518363064008</v>
+        <v>127.7924345295829</v>
       </c>
       <c r="Z24" t="n">
         <v>2.832887348322184</v>
@@ -2656,7 +2656,7 @@
         <v>37.2559686869738</v>
       </c>
       <c r="K25" t="n">
-        <v>20.28455645388773</v>
+        <v>20.87169114116179</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2672,7 +2672,7 @@
         <v>0.007626</v>
       </c>
       <c r="Q25" t="n">
-        <v>110.2</v>
+        <v>107.1</v>
       </c>
       <c r="R25" t="n">
         <v>15761.3</v>
@@ -2688,13 +2688,13 @@
         <v>4556.747637839262</v>
       </c>
       <c r="W25" t="n">
-        <v>0.3380759408981289</v>
+        <v>0.3478615190193632</v>
       </c>
       <c r="X25" t="n">
         <v>0.0002194547689444097</v>
       </c>
       <c r="Y25" t="n">
-        <v>143.024500907441</v>
+        <v>147.1643323996265</v>
       </c>
       <c r="Z25" t="n">
         <v>2.363762423592839</v>
@@ -2746,7 +2746,7 @@
         <v>33.6962858057476</v>
       </c>
       <c r="K26" t="n">
-        <v>3.45602931341001</v>
+        <v>3.47205417885086</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2762,7 +2762,7 @@
         <v>0.084838</v>
       </c>
       <c r="Q26" t="n">
-        <v>585</v>
+        <v>582.3</v>
       </c>
       <c r="R26" t="n">
         <v>29565.5</v>
@@ -2778,13 +2778,13 @@
         <v>372.0058048768779</v>
       </c>
       <c r="W26" t="n">
-        <v>0.0576004885568335</v>
+        <v>0.05786756964751434</v>
       </c>
       <c r="X26" t="n">
         <v>0.002688130096063873</v>
       </c>
       <c r="Y26" t="n">
-        <v>50.53931623931624</v>
+        <v>50.77365619096686</v>
       </c>
       <c r="Z26" t="n">
         <v>1.139716419669804</v>
@@ -2898,7 +2898,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K28" t="n">
-        <v>10.81565449363292</v>
+        <v>12.64035755888894</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2914,7 +2914,7 @@
         <v>0.021244</v>
       </c>
       <c r="Q28" t="n">
-        <v>162.1</v>
+        <v>138.7</v>
       </c>
       <c r="R28" t="n">
         <v>18211.1</v>
@@ -2930,13 +2930,13 @@
         <v>1104.110834068831</v>
       </c>
       <c r="W28" t="n">
-        <v>0.1802609082272153</v>
+        <v>0.2106726259814823</v>
       </c>
       <c r="X28" t="n">
         <v>0.0009057061747277989</v>
       </c>
       <c r="Y28" t="n">
-        <v>112.3448488587292</v>
+        <v>131.2984859408796</v>
       </c>
       <c r="Z28" t="n">
         <v>1.604532028467891</v>
@@ -2988,7 +2988,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K29" t="n">
-        <v>8.536941150320636</v>
+        <v>10.25367213403765</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -3004,7 +3004,7 @@
         <v>0.09042</v>
       </c>
       <c r="Q29" t="n">
-        <v>175.6</v>
+        <v>146.2</v>
       </c>
       <c r="R29" t="n">
         <v>22793.6</v>
@@ -3020,13 +3020,13 @@
         <v>263.8642816401065</v>
       </c>
       <c r="W29" t="n">
-        <v>0.142282352505344</v>
+        <v>0.1708945355672941</v>
       </c>
       <c r="X29" t="n">
         <v>0.00378982707998324</v>
       </c>
       <c r="Y29" t="n">
-        <v>129.8041002277904</v>
+        <v>155.906976744186</v>
       </c>
       <c r="Z29" t="n">
         <v>1.096131418465639</v>
@@ -3078,7 +3078,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K30" t="n">
-        <v>16.6546578757524</v>
+        <v>14.61928523418861</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3094,7 +3094,7 @@
         <v>0.02862</v>
       </c>
       <c r="Q30" t="n">
-        <v>82.59999999999999</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="R30" t="n">
         <v>12593.6</v>
@@ -3110,13 +3110,13 @@
         <v>694.5957872787968</v>
       </c>
       <c r="W30" t="n">
-        <v>0.27757763126254</v>
+        <v>0.2436547539031435</v>
       </c>
       <c r="X30" t="n">
         <v>0.001439686243876714</v>
       </c>
       <c r="Y30" t="n">
-        <v>152.4648910411622</v>
+        <v>133.8320935175346</v>
       </c>
       <c r="Z30" t="n">
         <v>1.820600332096128</v>
@@ -3168,7 +3168,7 @@
         <v>22.1685424839812</v>
       </c>
       <c r="K31" t="n">
-        <v>65.20159554112118</v>
+        <v>63.03850943312189</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3184,7 +3184,7 @@
         <v>0.017024</v>
       </c>
       <c r="Q31" t="n">
-        <v>20.4</v>
+        <v>21.1</v>
       </c>
       <c r="R31" t="n">
         <v>7379.9</v>
@@ -3200,13 +3200,13 @@
         <v>1152.690436979056</v>
       </c>
       <c r="W31" t="n">
-        <v>1.086693259018686</v>
+        <v>1.050641823885365</v>
       </c>
       <c r="X31" t="n">
         <v>0.0008675356087977764</v>
       </c>
       <c r="Y31" t="n">
-        <v>361.7598039215686</v>
+        <v>349.7582938388625</v>
       </c>
       <c r="Z31" t="n">
         <v>3.003908248618708</v>
@@ -3258,7 +3258,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K32" t="n">
-        <v>12.45279164533005</v>
+        <v>12.32109349631951</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3274,7 +3274,7 @@
         <v>0.010936</v>
       </c>
       <c r="Q32" t="n">
-        <v>84.2</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="R32" t="n">
         <v>7737.1</v>
@@ -3290,13 +3290,13 @@
         <v>1417.768749711707</v>
       </c>
       <c r="W32" t="n">
-        <v>0.2075465274221674</v>
+        <v>0.2053515582719918</v>
       </c>
       <c r="X32" t="n">
         <v>0.0007053336449991176</v>
       </c>
       <c r="Y32" t="n">
-        <v>91.8895486935867</v>
+        <v>90.91774383078732</v>
       </c>
       <c r="Z32" t="n">
         <v>2.258652157649054</v>
@@ -3348,7 +3348,7 @@
         <v>14.1889227802691</v>
       </c>
       <c r="K33" t="n">
-        <v>9.36562559753736</v>
+        <v>9.144311136585888</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -3364,7 +3364,7 @@
         <v>0.047676</v>
       </c>
       <c r="Q33" t="n">
-        <v>90.90000000000001</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="R33" t="n">
         <v>14142</v>
@@ -3380,13 +3380,13 @@
         <v>131.1287985903656</v>
       </c>
       <c r="W33" t="n">
-        <v>0.156093759958956</v>
+        <v>0.1524051856097648</v>
       </c>
       <c r="X33" t="n">
         <v>0.007626089850208333</v>
       </c>
       <c r="Y33" t="n">
-        <v>155.5775577557756</v>
+        <v>151.9011815252417</v>
       </c>
       <c r="Z33" t="n">
         <v>1.003317973431558</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-09-25)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -676,7 +676,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K3" t="n">
-        <v>76.69500080001905</v>
+        <v>75.31930571840435</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -692,7 +692,7 @@
         <v>0.09657399999999999</v>
       </c>
       <c r="Q3" t="n">
-        <v>43.8</v>
+        <v>44.6</v>
       </c>
       <c r="R3" t="n">
         <v>6353.5</v>
@@ -708,13 +708,13 @@
         <v>383.8588628629582</v>
       </c>
       <c r="W3" t="n">
-        <v>1.278250013333651</v>
+        <v>1.255321761973406</v>
       </c>
       <c r="X3" t="n">
         <v>0.002605124166058427</v>
       </c>
       <c r="Y3" t="n">
-        <v>145.0570776255708</v>
+        <v>142.4551569506726</v>
       </c>
       <c r="Z3" t="n">
         <v>8.81204856913731</v>
@@ -766,7 +766,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K4" t="n">
-        <v>146.1359890423819</v>
+        <v>144.8194486005587</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -782,7 +782,7 @@
         <v>0.03274</v>
       </c>
       <c r="Q4" t="n">
-        <v>22</v>
+        <v>22.2</v>
       </c>
       <c r="R4" t="n">
         <v>3004</v>
@@ -798,13 +798,13 @@
         <v>686.2074633379441</v>
       </c>
       <c r="W4" t="n">
-        <v>2.435599817373032</v>
+        <v>2.413657476675978</v>
       </c>
       <c r="X4" t="n">
         <v>0.001457285228487116</v>
       </c>
       <c r="Y4" t="n">
-        <v>136.5454545454545</v>
+        <v>135.3153153153153</v>
       </c>
       <c r="Z4" t="n">
         <v>17.83728228435643</v>
@@ -856,7 +856,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K5" t="n">
-        <v>15.00138499409331</v>
+        <v>15.0154575878964</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -872,7 +872,7 @@
         <v>1.087069</v>
       </c>
       <c r="Q5" t="n">
-        <v>213.4</v>
+        <v>213.2</v>
       </c>
       <c r="R5" t="n">
         <v>23039.4</v>
@@ -888,13 +888,13 @@
         <v>44.3365962628782</v>
       </c>
       <c r="W5" t="n">
-        <v>0.2500230832348885</v>
+        <v>0.25025762646494</v>
       </c>
       <c r="X5" t="n">
         <v>0.022554730951173</v>
       </c>
       <c r="Y5" t="n">
-        <v>107.9634489222118</v>
+        <v>108.0647279549719</v>
       </c>
       <c r="Z5" t="n">
         <v>2.315812302504631</v>
@@ -946,7 +946,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K6" t="n">
-        <v>30.43084390117887</v>
+        <v>29.259354035139</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -962,7 +962,7 @@
         <v>0.452635</v>
       </c>
       <c r="Q6" t="n">
-        <v>104.9</v>
+        <v>109.1</v>
       </c>
       <c r="R6" t="n">
         <v>10176.4</v>
@@ -978,13 +978,13 @@
         <v>95.52129303831462</v>
       </c>
       <c r="W6" t="n">
-        <v>0.5071807316863146</v>
+        <v>0.4876559005856499</v>
       </c>
       <c r="X6" t="n">
         <v>0.01046887000994521</v>
       </c>
       <c r="Y6" t="n">
-        <v>97.01048617731172</v>
+        <v>93.27589367552704</v>
       </c>
       <c r="Z6" t="n">
         <v>5.228102153403404</v>
@@ -1036,7 +1036,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K7" t="n">
-        <v>29.18208830776344</v>
+        <v>30.74338680671965</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1052,7 +1052,7 @@
         <v>0.25811</v>
       </c>
       <c r="Q7" t="n">
-        <v>108.3</v>
+        <v>102.8</v>
       </c>
       <c r="R7" t="n">
         <v>5609.9</v>
@@ -1068,13 +1068,13 @@
         <v>173.6055812119343</v>
       </c>
       <c r="W7" t="n">
-        <v>0.486368138462724</v>
+        <v>0.5123897801119942</v>
       </c>
       <c r="X7" t="n">
         <v>0.005760183474627001</v>
       </c>
       <c r="Y7" t="n">
-        <v>51.79963065558633</v>
+        <v>54.57101167315175</v>
       </c>
       <c r="Z7" t="n">
         <v>9.389413250773277</v>
@@ -1126,7 +1126,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K8" t="n">
-        <v>54.09947784255924</v>
+        <v>55.24041586384344</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1142,7 +1142,7 @@
         <v>0.126814</v>
       </c>
       <c r="Q8" t="n">
-        <v>58.1</v>
+        <v>56.9</v>
       </c>
       <c r="R8" t="n">
         <v>2987.7</v>
@@ -1158,13 +1158,13 @@
         <v>303.7663387233741</v>
       </c>
       <c r="W8" t="n">
-        <v>0.901657964042654</v>
+        <v>0.9206735977307241</v>
       </c>
       <c r="X8" t="n">
         <v>0.003292003992946215</v>
       </c>
       <c r="Y8" t="n">
-        <v>51.42340791738382</v>
+        <v>52.5079086115993</v>
       </c>
       <c r="Z8" t="n">
         <v>17.53399863134793</v>
@@ -1216,7 +1216,7 @@
         <v>51.2434931792768</v>
       </c>
       <c r="K9" t="n">
-        <v>177.7230977315958</v>
+        <v>174.6937267475345</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1232,7 +1232,7 @@
         <v>0.01898</v>
       </c>
       <c r="Q9" t="n">
-        <v>17.3</v>
+        <v>17.6</v>
       </c>
       <c r="R9" t="n">
         <v>2234.8</v>
@@ -1248,13 +1248,13 @@
         <v>824.4601019930624</v>
       </c>
       <c r="W9" t="n">
-        <v>2.96205162885993</v>
+        <v>2.911562112458909</v>
       </c>
       <c r="X9" t="n">
         <v>0.001212914970151478</v>
       </c>
       <c r="Y9" t="n">
-        <v>129.1791907514451</v>
+        <v>126.9772727272727</v>
       </c>
       <c r="Z9" t="n">
         <v>22.92978932310578</v>
@@ -1306,7 +1306,7 @@
         <v>50.7771115797629</v>
       </c>
       <c r="K10" t="n">
-        <v>28.36710144120832</v>
+        <v>28.79609352349503</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1322,7 @@
         <v>0.20946</v>
       </c>
       <c r="Q10" t="n">
-        <v>107.4</v>
+        <v>105.8</v>
       </c>
       <c r="R10" t="n">
         <v>9435.6</v>
@@ -1338,13 +1338,13 @@
         <v>198.7704793771252</v>
       </c>
       <c r="W10" t="n">
-        <v>0.4727850240201387</v>
+        <v>0.4799348920582505</v>
       </c>
       <c r="X10" t="n">
         <v>0.005030928149560429</v>
       </c>
       <c r="Y10" t="n">
-        <v>87.85474860335195</v>
+        <v>89.18336483931948</v>
       </c>
       <c r="Z10" t="n">
         <v>5.381439609538651</v>
@@ -1396,7 +1396,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K11" t="n">
-        <v>34.27005518192529</v>
+        <v>33.16711087721966</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1412,7 +1412,7 @@
         <v>0.07542500000000001</v>
       </c>
       <c r="Q11" t="n">
-        <v>84.2</v>
+        <v>87</v>
       </c>
       <c r="R11" t="n">
         <v>18553.6</v>
@@ -1428,13 +1428,13 @@
         <v>578.4775641354948</v>
       </c>
       <c r="W11" t="n">
-        <v>0.5711675863654216</v>
+        <v>0.5527851812869943</v>
       </c>
       <c r="X11" t="n">
         <v>0.001728675513102135</v>
       </c>
       <c r="Y11" t="n">
-        <v>220.3515439429929</v>
+        <v>213.2597701149425</v>
       </c>
       <c r="Z11" t="n">
         <v>2.592074356026243</v>
@@ -1486,7 +1486,7 @@
         <v>47.5276426437724</v>
       </c>
       <c r="K12" t="n">
-        <v>39.88333648428453</v>
+        <v>32.47902686362578</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1502,7 +1502,7 @@
         <v>0.076765</v>
       </c>
       <c r="Q12" t="n">
-        <v>71.5</v>
+        <v>87.8</v>
       </c>
       <c r="R12" t="n">
         <v>8045.8</v>
@@ -1518,13 +1518,13 @@
         <v>554.5362997628245</v>
       </c>
       <c r="W12" t="n">
-        <v>0.6647222747380755</v>
+        <v>0.5413171143937632</v>
       </c>
       <c r="X12" t="n">
         <v>0.001803308458666638</v>
       </c>
       <c r="Y12" t="n">
-        <v>112.5286713286713</v>
+        <v>91.63781321184511</v>
       </c>
       <c r="Z12" t="n">
         <v>5.907136971310796</v>
@@ -1666,7 +1666,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K14" t="n">
-        <v>3.709294606433803</v>
+        <v>4.065343600020008</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1682,7 @@
         <v>0.337573</v>
       </c>
       <c r="Q14" t="n">
-        <v>751.3</v>
+        <v>685.5</v>
       </c>
       <c r="R14" t="n">
         <v>57055.2</v>
@@ -1698,13 +1698,13 @@
         <v>132.374251168453</v>
       </c>
       <c r="W14" t="n">
-        <v>0.06182157677389671</v>
+        <v>0.06775572666700015</v>
       </c>
       <c r="X14" t="n">
         <v>0.007554339240245816</v>
       </c>
       <c r="Y14" t="n">
-        <v>75.94196725675496</v>
+        <v>83.23150984682712</v>
       </c>
       <c r="Z14" t="n">
         <v>0.814063409298865</v>
@@ -1756,7 +1756,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K15" t="n">
-        <v>7.766002771339195</v>
+        <v>5.867537242690095</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1772,7 +1772,7 @@
         <v>0.0152</v>
       </c>
       <c r="Q15" t="n">
-        <v>357.9</v>
+        <v>473.7</v>
       </c>
       <c r="R15" t="n">
         <v>20796.5</v>
@@ -1788,13 +1788,13 @@
         <v>2193.173304187023</v>
       </c>
       <c r="W15" t="n">
-        <v>0.1294333795223199</v>
+        <v>0.09779228737816825</v>
       </c>
       <c r="X15" t="n">
         <v>0.0004559603192738502</v>
       </c>
       <c r="Y15" t="n">
-        <v>58.10701313215983</v>
+        <v>43.9022588135951</v>
       </c>
       <c r="Z15" t="n">
         <v>2.227500133726266</v>
@@ -1846,7 +1846,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K16" t="n">
-        <v>5.675718620877163</v>
+        <v>5.590710935336738</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1862,7 @@
         <v>0.141536</v>
       </c>
       <c r="Q16" t="n">
-        <v>480.1</v>
+        <v>487.4</v>
       </c>
       <c r="R16" t="n">
         <v>24843.6</v>
@@ -1878,13 +1878,13 @@
         <v>290.2523742749451</v>
       </c>
       <c r="W16" t="n">
-        <v>0.09459531034795272</v>
+        <v>0.09317851558894565</v>
       </c>
       <c r="X16" t="n">
         <v>0.003445277588161046</v>
       </c>
       <c r="Y16" t="n">
-        <v>51.74671943345136</v>
+        <v>50.97168649979483</v>
       </c>
       <c r="Z16" t="n">
         <v>1.828044586857464</v>
@@ -1936,7 +1936,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K17" t="n">
-        <v>5.681208591957793</v>
+        <v>6.699859209817556</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1952,7 @@
         <v>0.148652</v>
       </c>
       <c r="Q17" t="n">
-        <v>472.9</v>
+        <v>401</v>
       </c>
       <c r="R17" t="n">
         <v>34728.3</v>
@@ -1968,13 +1968,13 @@
         <v>281.760586368072</v>
       </c>
       <c r="W17" t="n">
-        <v>0.09468680986596321</v>
+        <v>0.1116643201636259</v>
       </c>
       <c r="X17" t="n">
         <v>0.003549112432260739</v>
       </c>
       <c r="Y17" t="n">
-        <v>73.43687883273421</v>
+        <v>86.60423940149627</v>
       </c>
       <c r="Z17" t="n">
         <v>1.289363210569305</v>
@@ -2026,7 +2026,7 @@
         <v>44.3113073012592</v>
       </c>
       <c r="K18" t="n">
-        <v>15.85377720975284</v>
+        <v>16.54435866879622</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2042,7 +2042,7 @@
         <v>0.058096</v>
       </c>
       <c r="Q18" t="n">
-        <v>167.7</v>
+        <v>160.7</v>
       </c>
       <c r="R18" t="n">
         <v>10197.8</v>
@@ -2058,13 +2058,13 @@
         <v>662.6188043195191</v>
       </c>
       <c r="W18" t="n">
-        <v>0.2642296201625474</v>
+        <v>0.2757393111466036</v>
       </c>
       <c r="X18" t="n">
         <v>0.001509163328117374</v>
       </c>
       <c r="Y18" t="n">
-        <v>60.8097793679189</v>
+        <v>63.45861854387056</v>
       </c>
       <c r="Z18" t="n">
         <v>4.345183010184472</v>
@@ -2116,7 +2116,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>16.82088650544669</v>
+        <v>14.18409889107937</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2132,7 @@
         <v>0.039576</v>
       </c>
       <c r="Q19" t="n">
-        <v>156</v>
+        <v>185</v>
       </c>
       <c r="R19" t="n">
         <v>15469.6</v>
@@ -2148,13 +2148,13 @@
         <v>972.1110696872879</v>
       </c>
       <c r="W19" t="n">
-        <v>0.2803481084241115</v>
+        <v>0.2364016481846562</v>
       </c>
       <c r="X19" t="n">
         <v>0.001028689036862509</v>
       </c>
       <c r="Y19" t="n">
-        <v>99.16410256410256</v>
+        <v>83.61945945945946</v>
       </c>
       <c r="Z19" t="n">
         <v>2.827112848047875</v>
@@ -2206,7 +2206,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>9.712697278546944</v>
+        <v>9.655331772287532</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2222,7 +2222,7 @@
         <v>0.148276</v>
       </c>
       <c r="Q20" t="n">
-        <v>269.3</v>
+        <v>270.9</v>
       </c>
       <c r="R20" t="n">
         <v>10391.2</v>
@@ -2238,13 +2238,13 @@
         <v>266.8933313244817</v>
       </c>
       <c r="W20" t="n">
-        <v>0.1618782879757824</v>
+        <v>0.1609221962047922</v>
       </c>
       <c r="X20" t="n">
         <v>0.0037468152352755</v>
       </c>
       <c r="Y20" t="n">
-        <v>38.58596360935759</v>
+        <v>38.35806570690292</v>
       </c>
       <c r="Z20" t="n">
         <v>4.195263583789957</v>
@@ -2296,7 +2296,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K21" t="n">
-        <v>3.23170312652319</v>
+        <v>2.923599028912937</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.021793</v>
       </c>
       <c r="Q21" t="n">
-        <v>776.2</v>
+        <v>858</v>
       </c>
       <c r="R21" t="n">
         <v>44420.3</v>
@@ -2328,13 +2328,13 @@
         <v>1834.787418303125</v>
       </c>
       <c r="W21" t="n">
-        <v>0.05386171877538649</v>
+        <v>0.04872665048188229</v>
       </c>
       <c r="X21" t="n">
         <v>0.0005450222679883181</v>
       </c>
       <c r="Y21" t="n">
-        <v>57.22790517907756</v>
+        <v>51.77191142191143</v>
       </c>
       <c r="Z21" t="n">
         <v>0.9411792831983349</v>
@@ -2386,7 +2386,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K22" t="n">
-        <v>30.54196431088836</v>
+        <v>30.39076646776515</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.088764</v>
       </c>
       <c r="Q22" t="n">
-        <v>80.40000000000001</v>
+        <v>80.8</v>
       </c>
       <c r="R22" t="n">
         <v>24301.8</v>
@@ -2418,13 +2418,13 @@
         <v>439.4668804599139</v>
       </c>
       <c r="W22" t="n">
-        <v>0.509032738514806</v>
+        <v>0.5065127744627526</v>
       </c>
       <c r="X22" t="n">
         <v>0.002275484329907804</v>
       </c>
       <c r="Y22" t="n">
-        <v>302.2611940298507</v>
+        <v>300.7648514851485</v>
       </c>
       <c r="Z22" t="n">
         <v>1.684082338616498</v>
@@ -2476,7 +2476,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K23" t="n">
-        <v>33.24957933078117</v>
+        <v>34.21054983167081</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2492,7 +2492,7 @@
         <v>0.02621</v>
       </c>
       <c r="Q23" t="n">
-        <v>71.2</v>
+        <v>69.2</v>
       </c>
       <c r="R23" t="n">
         <v>22336.9</v>
@@ -2508,13 +2508,13 @@
         <v>1426.160900474481</v>
       </c>
       <c r="W23" t="n">
-        <v>0.5541596555130196</v>
+        <v>0.5701758305278468</v>
       </c>
       <c r="X23" t="n">
         <v>0.0007011831551876802</v>
       </c>
       <c r="Y23" t="n">
-        <v>313.7205056179776</v>
+        <v>322.7875722543353</v>
       </c>
       <c r="Z23" t="n">
         <v>1.76641196730643</v>
@@ -2566,7 +2566,7 @@
         <v>37.3244239690841</v>
       </c>
       <c r="K24" t="n">
-        <v>21.72129425940879</v>
+        <v>21.70024649365355</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2582,7 +2582,7 @@
         <v>0.015269</v>
       </c>
       <c r="Q24" t="n">
-        <v>103.1</v>
+        <v>103.2</v>
       </c>
       <c r="R24" t="n">
         <v>13175.4</v>
@@ -2598,13 +2598,13 @@
         <v>2269.237838587312</v>
       </c>
       <c r="W24" t="n">
-        <v>0.3620215709901465</v>
+        <v>0.3616707748942258</v>
       </c>
       <c r="X24" t="n">
         <v>0.0004406765932576458</v>
       </c>
       <c r="Y24" t="n">
-        <v>127.7924345295829</v>
+        <v>127.6686046511628</v>
       </c>
       <c r="Z24" t="n">
         <v>2.832887348322184</v>
@@ -2656,7 +2656,7 @@
         <v>37.2559686869738</v>
       </c>
       <c r="K25" t="n">
-        <v>20.87169114116179</v>
+        <v>20.79402903459003</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2672,7 +2672,7 @@
         <v>0.007626</v>
       </c>
       <c r="Q25" t="n">
-        <v>107.1</v>
+        <v>107.5</v>
       </c>
       <c r="R25" t="n">
         <v>15761.3</v>
@@ -2688,13 +2688,13 @@
         <v>4556.747637839262</v>
       </c>
       <c r="W25" t="n">
-        <v>0.3478615190193632</v>
+        <v>0.3465671505765005</v>
       </c>
       <c r="X25" t="n">
         <v>0.0002194547689444097</v>
       </c>
       <c r="Y25" t="n">
-        <v>147.1643323996265</v>
+        <v>146.6167441860465</v>
       </c>
       <c r="Z25" t="n">
         <v>2.363762423592839</v>
@@ -2746,7 +2746,7 @@
         <v>33.6962858057476</v>
       </c>
       <c r="K26" t="n">
-        <v>3.47205417885086</v>
+        <v>3.98301250658955</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2762,7 +2762,7 @@
         <v>0.084838</v>
       </c>
       <c r="Q26" t="n">
-        <v>582.3</v>
+        <v>507.6</v>
       </c>
       <c r="R26" t="n">
         <v>29565.5</v>
@@ -2778,13 +2778,13 @@
         <v>372.0058048768779</v>
       </c>
       <c r="W26" t="n">
-        <v>0.05786756964751434</v>
+        <v>0.06638354177649251</v>
       </c>
       <c r="X26" t="n">
         <v>0.002688130096063873</v>
       </c>
       <c r="Y26" t="n">
-        <v>50.77365619096686</v>
+        <v>58.2456658786446</v>
       </c>
       <c r="Z26" t="n">
         <v>1.139716419669804</v>
@@ -2898,7 +2898,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K28" t="n">
-        <v>12.64035755888894</v>
+        <v>14.70820128706288</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2914,7 +2914,7 @@
         <v>0.021244</v>
       </c>
       <c r="Q28" t="n">
-        <v>138.7</v>
+        <v>119.2</v>
       </c>
       <c r="R28" t="n">
         <v>18211.1</v>
@@ -2930,13 +2930,13 @@
         <v>1104.110834068831</v>
       </c>
       <c r="W28" t="n">
-        <v>0.2106726259814823</v>
+        <v>0.2451366881177148</v>
       </c>
       <c r="X28" t="n">
         <v>0.0009057061747277989</v>
       </c>
       <c r="Y28" t="n">
-        <v>131.2984859408796</v>
+        <v>152.7776845637584</v>
       </c>
       <c r="Z28" t="n">
         <v>1.604532028467891</v>
@@ -2988,7 +2988,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K29" t="n">
-        <v>10.25367213403765</v>
+        <v>12.83464782531082</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -3004,7 +3004,7 @@
         <v>0.09042</v>
       </c>
       <c r="Q29" t="n">
-        <v>146.2</v>
+        <v>116.8</v>
       </c>
       <c r="R29" t="n">
         <v>22793.6</v>
@@ -3020,13 +3020,13 @@
         <v>263.8642816401065</v>
       </c>
       <c r="W29" t="n">
-        <v>0.1708945355672941</v>
+        <v>0.2139107970885137</v>
       </c>
       <c r="X29" t="n">
         <v>0.00378982707998324</v>
       </c>
       <c r="Y29" t="n">
-        <v>155.906976744186</v>
+        <v>195.1506849315068</v>
       </c>
       <c r="Z29" t="n">
         <v>1.096131418465639</v>
@@ -3078,7 +3078,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K30" t="n">
-        <v>14.61928523418861</v>
+        <v>15.11730484106756</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3094,7 +3094,7 @@
         <v>0.02862</v>
       </c>
       <c r="Q30" t="n">
-        <v>94.09999999999999</v>
+        <v>91</v>
       </c>
       <c r="R30" t="n">
         <v>12593.6</v>
@@ -3110,13 +3110,13 @@
         <v>694.5957872787968</v>
       </c>
       <c r="W30" t="n">
-        <v>0.2436547539031435</v>
+        <v>0.2519550806844593</v>
       </c>
       <c r="X30" t="n">
         <v>0.001439686243876714</v>
       </c>
       <c r="Y30" t="n">
-        <v>133.8320935175346</v>
+        <v>138.3912087912088</v>
       </c>
       <c r="Z30" t="n">
         <v>1.820600332096128</v>
@@ -3168,7 +3168,7 @@
         <v>22.1685424839812</v>
       </c>
       <c r="K31" t="n">
-        <v>63.03850943312189</v>
+        <v>62.15479201116224</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3184,7 +3184,7 @@
         <v>0.017024</v>
       </c>
       <c r="Q31" t="n">
-        <v>21.1</v>
+        <v>21.4</v>
       </c>
       <c r="R31" t="n">
         <v>7379.9</v>
@@ -3200,13 +3200,13 @@
         <v>1152.690436979056</v>
       </c>
       <c r="W31" t="n">
-        <v>1.050641823885365</v>
+        <v>1.035913200186037</v>
       </c>
       <c r="X31" t="n">
         <v>0.0008675356087977764</v>
       </c>
       <c r="Y31" t="n">
-        <v>349.7582938388625</v>
+        <v>344.8551401869159</v>
       </c>
       <c r="Z31" t="n">
         <v>3.003908248618708</v>
@@ -3258,23 +3258,23 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K32" t="n">
-        <v>12.32109349631951</v>
+        <v>14.22693428136757</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
-        <v>0.012326</v>
+        <v>0.011114</v>
       </c>
       <c r="N32" t="n">
-        <v>0.00072</v>
+        <v>0.000669</v>
       </c>
       <c r="O32" t="n">
-        <v>0.00067</v>
+        <v>0.000603</v>
       </c>
       <c r="P32" t="n">
-        <v>0.010936</v>
+        <v>0.009842</v>
       </c>
       <c r="Q32" t="n">
-        <v>85.09999999999999</v>
+        <v>73.7</v>
       </c>
       <c r="R32" t="n">
         <v>7737.1</v>
@@ -3287,16 +3287,16 @@
       </c>
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="n">
-        <v>1417.768749711707</v>
+        <v>1572.37876632594</v>
       </c>
       <c r="W32" t="n">
-        <v>0.2053515582719918</v>
+        <v>0.2371155713561262</v>
       </c>
       <c r="X32" t="n">
-        <v>0.0007053336449991176</v>
+        <v>0.0006359790792244194</v>
       </c>
       <c r="Y32" t="n">
-        <v>90.91774383078732</v>
+        <v>104.9810040705563</v>
       </c>
       <c r="Z32" t="n">
         <v>2.258652157649054</v>
@@ -3348,7 +3348,7 @@
         <v>14.1889227802691</v>
       </c>
       <c r="K33" t="n">
-        <v>9.144311136585888</v>
+        <v>9.124709183452799</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -3364,7 +3364,7 @@
         <v>0.047676</v>
       </c>
       <c r="Q33" t="n">
-        <v>93.09999999999999</v>
+        <v>93.3</v>
       </c>
       <c r="R33" t="n">
         <v>14142</v>
@@ -3380,13 +3380,13 @@
         <v>131.1287985903656</v>
       </c>
       <c r="W33" t="n">
-        <v>0.1524051856097648</v>
+        <v>0.15207848639088</v>
       </c>
       <c r="X33" t="n">
         <v>0.007626089850208333</v>
       </c>
       <c r="Y33" t="n">
-        <v>151.9011815252417</v>
+        <v>151.5755627009646</v>
       </c>
       <c r="Z33" t="n">
         <v>1.003317973431558</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-09-26)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -676,7 +676,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K3" t="n">
-        <v>75.31930571840435</v>
+        <v>75.48856258518728</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -692,7 +692,7 @@
         <v>0.09657399999999999</v>
       </c>
       <c r="Q3" t="n">
-        <v>44.6</v>
+        <v>44.5</v>
       </c>
       <c r="R3" t="n">
         <v>6353.5</v>
@@ -708,13 +708,13 @@
         <v>383.8588628629582</v>
       </c>
       <c r="W3" t="n">
-        <v>1.255321761973406</v>
+        <v>1.258142709753121</v>
       </c>
       <c r="X3" t="n">
         <v>0.002605124166058427</v>
       </c>
       <c r="Y3" t="n">
-        <v>142.4551569506726</v>
+        <v>142.7752808988764</v>
       </c>
       <c r="Z3" t="n">
         <v>8.81204856913731</v>
@@ -766,7 +766,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K4" t="n">
-        <v>144.8194486005587</v>
+        <v>144.1700340328431</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -782,7 +782,7 @@
         <v>0.03274</v>
       </c>
       <c r="Q4" t="n">
-        <v>22.2</v>
+        <v>22.3</v>
       </c>
       <c r="R4" t="n">
         <v>3004</v>
@@ -798,13 +798,13 @@
         <v>686.2074633379441</v>
       </c>
       <c r="W4" t="n">
-        <v>2.413657476675978</v>
+        <v>2.402833900547386</v>
       </c>
       <c r="X4" t="n">
         <v>0.001457285228487116</v>
       </c>
       <c r="Y4" t="n">
-        <v>135.3153153153153</v>
+        <v>134.7085201793722</v>
       </c>
       <c r="Z4" t="n">
         <v>17.83728228435643</v>
@@ -856,7 +856,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K5" t="n">
-        <v>15.0154575878964</v>
+        <v>15.22251810622687</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -872,7 +872,7 @@
         <v>1.087069</v>
       </c>
       <c r="Q5" t="n">
-        <v>213.2</v>
+        <v>210.3</v>
       </c>
       <c r="R5" t="n">
         <v>23039.4</v>
@@ -888,13 +888,13 @@
         <v>44.3365962628782</v>
       </c>
       <c r="W5" t="n">
-        <v>0.25025762646494</v>
+        <v>0.2537086351037812</v>
       </c>
       <c r="X5" t="n">
         <v>0.022554730951173</v>
       </c>
       <c r="Y5" t="n">
-        <v>108.0647279549719</v>
+        <v>109.5549215406562</v>
       </c>
       <c r="Z5" t="n">
         <v>2.315812302504631</v>
@@ -946,7 +946,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K6" t="n">
-        <v>29.259354035139</v>
+        <v>30.43084390117887</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -962,7 +962,7 @@
         <v>0.452635</v>
       </c>
       <c r="Q6" t="n">
-        <v>109.1</v>
+        <v>104.9</v>
       </c>
       <c r="R6" t="n">
         <v>10176.4</v>
@@ -978,13 +978,13 @@
         <v>95.52129303831462</v>
       </c>
       <c r="W6" t="n">
-        <v>0.4876559005856499</v>
+        <v>0.5071807316863146</v>
       </c>
       <c r="X6" t="n">
         <v>0.01046887000994521</v>
       </c>
       <c r="Y6" t="n">
-        <v>93.27589367552704</v>
+        <v>97.01048617731172</v>
       </c>
       <c r="Z6" t="n">
         <v>5.228102153403404</v>
@@ -1036,7 +1036,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K7" t="n">
-        <v>30.74338680671965</v>
+        <v>34.09298990000841</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1052,7 +1052,7 @@
         <v>0.25811</v>
       </c>
       <c r="Q7" t="n">
-        <v>102.8</v>
+        <v>92.7</v>
       </c>
       <c r="R7" t="n">
         <v>5609.9</v>
@@ -1068,13 +1068,13 @@
         <v>173.6055812119343</v>
       </c>
       <c r="W7" t="n">
-        <v>0.5123897801119942</v>
+        <v>0.5682164983334735</v>
       </c>
       <c r="X7" t="n">
         <v>0.005760183474627001</v>
       </c>
       <c r="Y7" t="n">
-        <v>54.57101167315175</v>
+        <v>60.51672060409924</v>
       </c>
       <c r="Z7" t="n">
         <v>9.389413250773277</v>
@@ -1126,7 +1126,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K8" t="n">
-        <v>55.24041586384344</v>
+        <v>60.91433454753279</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1142,7 +1142,7 @@
         <v>0.126814</v>
       </c>
       <c r="Q8" t="n">
-        <v>56.9</v>
+        <v>51.6</v>
       </c>
       <c r="R8" t="n">
         <v>2987.7</v>
@@ -1158,13 +1158,13 @@
         <v>303.7663387233741</v>
       </c>
       <c r="W8" t="n">
-        <v>0.9206735977307241</v>
+        <v>1.015238909125546</v>
       </c>
       <c r="X8" t="n">
         <v>0.003292003992946215</v>
       </c>
       <c r="Y8" t="n">
-        <v>52.5079086115993</v>
+        <v>57.90116279069767</v>
       </c>
       <c r="Z8" t="n">
         <v>17.53399863134793</v>
@@ -1216,7 +1216,7 @@
         <v>51.2434931792768</v>
       </c>
       <c r="K9" t="n">
-        <v>174.6937267475345</v>
+        <v>183.0124756402743</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1232,7 +1232,7 @@
         <v>0.01898</v>
       </c>
       <c r="Q9" t="n">
-        <v>17.6</v>
+        <v>16.8</v>
       </c>
       <c r="R9" t="n">
         <v>2234.8</v>
@@ -1248,13 +1248,13 @@
         <v>824.4601019930624</v>
       </c>
       <c r="W9" t="n">
-        <v>2.911562112458909</v>
+        <v>3.050207927337905</v>
       </c>
       <c r="X9" t="n">
         <v>0.001212914970151478</v>
       </c>
       <c r="Y9" t="n">
-        <v>126.9772727272727</v>
+        <v>133.0238095238095</v>
       </c>
       <c r="Z9" t="n">
         <v>22.92978932310578</v>
@@ -1306,7 +1306,7 @@
         <v>50.7771115797629</v>
       </c>
       <c r="K10" t="n">
-        <v>28.79609352349503</v>
+        <v>30.9931505064677</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1322,7 @@
         <v>0.20946</v>
       </c>
       <c r="Q10" t="n">
-        <v>105.8</v>
+        <v>98.3</v>
       </c>
       <c r="R10" t="n">
         <v>9435.6</v>
@@ -1338,13 +1338,13 @@
         <v>198.7704793771252</v>
       </c>
       <c r="W10" t="n">
-        <v>0.4799348920582505</v>
+        <v>0.5165525084411282</v>
       </c>
       <c r="X10" t="n">
         <v>0.005030928149560429</v>
       </c>
       <c r="Y10" t="n">
-        <v>89.18336483931948</v>
+        <v>95.98779247202442</v>
       </c>
       <c r="Z10" t="n">
         <v>5.381439609538651</v>
@@ -1486,7 +1486,7 @@
         <v>47.5276426437724</v>
       </c>
       <c r="K12" t="n">
-        <v>32.47902686362578</v>
+        <v>30.20824744307568</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1502,7 +1502,7 @@
         <v>0.076765</v>
       </c>
       <c r="Q12" t="n">
-        <v>87.8</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="R12" t="n">
         <v>8045.8</v>
@@ -1518,13 +1518,13 @@
         <v>554.5362997628245</v>
       </c>
       <c r="W12" t="n">
-        <v>0.5413171143937632</v>
+        <v>0.503470790717928</v>
       </c>
       <c r="X12" t="n">
         <v>0.001803308458666638</v>
       </c>
       <c r="Y12" t="n">
-        <v>91.63781321184511</v>
+        <v>85.23093220338983</v>
       </c>
       <c r="Z12" t="n">
         <v>5.907136971310796</v>
@@ -1576,7 +1576,7 @@
         <v>46.9727068915036</v>
       </c>
       <c r="K13" t="n">
-        <v>35.2295301686277</v>
+        <v>40.20488464322705</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1592,7 +1592,7 @@
         <v>0.111119</v>
       </c>
       <c r="Q13" t="n">
-        <v>80</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="R13" t="n">
         <v>5952.7</v>
@@ -1608,13 +1608,13 @@
         <v>370.7747134022449</v>
       </c>
       <c r="W13" t="n">
-        <v>0.5871588361437949</v>
+        <v>0.6700814107204508</v>
       </c>
       <c r="X13" t="n">
         <v>0.002697055553826625</v>
       </c>
       <c r="Y13" t="n">
-        <v>74.40875</v>
+        <v>84.91726105563481</v>
       </c>
       <c r="Z13" t="n">
         <v>7.890991800612092</v>
@@ -1666,7 +1666,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K14" t="n">
-        <v>4.065343600020008</v>
+        <v>4.137777338995867</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1682,7 @@
         <v>0.337573</v>
       </c>
       <c r="Q14" t="n">
-        <v>685.5</v>
+        <v>673.5</v>
       </c>
       <c r="R14" t="n">
         <v>57055.2</v>
@@ -1698,13 +1698,13 @@
         <v>132.374251168453</v>
       </c>
       <c r="W14" t="n">
-        <v>0.06775572666700015</v>
+        <v>0.0689629556499311</v>
       </c>
       <c r="X14" t="n">
         <v>0.007554339240245816</v>
       </c>
       <c r="Y14" t="n">
-        <v>83.23150984682712</v>
+        <v>84.71447661469932</v>
       </c>
       <c r="Z14" t="n">
         <v>0.814063409298865</v>
@@ -1756,7 +1756,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K15" t="n">
-        <v>5.867537242690095</v>
+        <v>6.487984107988558</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1772,7 +1772,7 @@
         <v>0.0152</v>
       </c>
       <c r="Q15" t="n">
-        <v>473.7</v>
+        <v>428.4</v>
       </c>
       <c r="R15" t="n">
         <v>20796.5</v>
@@ -1788,13 +1788,13 @@
         <v>2193.173304187023</v>
       </c>
       <c r="W15" t="n">
-        <v>0.09779228737816825</v>
+        <v>0.108133068466476</v>
       </c>
       <c r="X15" t="n">
         <v>0.0004559603192738502</v>
       </c>
       <c r="Y15" t="n">
-        <v>43.9022588135951</v>
+        <v>48.54458450046685</v>
       </c>
       <c r="Z15" t="n">
         <v>2.227500133726266</v>
@@ -1846,7 +1846,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K16" t="n">
-        <v>5.590710935336738</v>
+        <v>5.579263943249645</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1862,7 @@
         <v>0.141536</v>
       </c>
       <c r="Q16" t="n">
-        <v>487.4</v>
+        <v>488.4</v>
       </c>
       <c r="R16" t="n">
         <v>24843.6</v>
@@ -1878,13 +1878,13 @@
         <v>290.2523742749451</v>
       </c>
       <c r="W16" t="n">
-        <v>0.09317851558894565</v>
+        <v>0.09298773238749407</v>
       </c>
       <c r="X16" t="n">
         <v>0.003445277588161046</v>
       </c>
       <c r="Y16" t="n">
-        <v>50.97168649979483</v>
+        <v>50.86732186732187</v>
       </c>
       <c r="Z16" t="n">
         <v>1.828044586857464</v>
@@ -1936,7 +1936,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K17" t="n">
-        <v>6.699859209817556</v>
+        <v>7.10000936346945</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1952,7 @@
         <v>0.148652</v>
       </c>
       <c r="Q17" t="n">
-        <v>401</v>
+        <v>378.4</v>
       </c>
       <c r="R17" t="n">
         <v>34728.3</v>
@@ -1968,13 +1968,13 @@
         <v>281.760586368072</v>
       </c>
       <c r="W17" t="n">
-        <v>0.1116643201636259</v>
+        <v>0.1183334893911575</v>
       </c>
       <c r="X17" t="n">
         <v>0.003549112432260739</v>
       </c>
       <c r="Y17" t="n">
-        <v>86.60423940149627</v>
+        <v>91.7766913319239</v>
       </c>
       <c r="Z17" t="n">
         <v>1.289363210569305</v>
@@ -2116,7 +2116,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>14.18409889107937</v>
+        <v>14.00244554348817</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2132,7 @@
         <v>0.039576</v>
       </c>
       <c r="Q19" t="n">
-        <v>185</v>
+        <v>187.4</v>
       </c>
       <c r="R19" t="n">
         <v>15469.6</v>
@@ -2148,13 +2148,13 @@
         <v>972.1110696872879</v>
       </c>
       <c r="W19" t="n">
-        <v>0.2364016481846562</v>
+        <v>0.2333740923914696</v>
       </c>
       <c r="X19" t="n">
         <v>0.001028689036862509</v>
       </c>
       <c r="Y19" t="n">
-        <v>83.61945945945946</v>
+        <v>82.54855923159018</v>
       </c>
       <c r="Z19" t="n">
         <v>2.827112848047875</v>
@@ -2206,7 +2206,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>9.655331772287532</v>
+        <v>9.616284474679015</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2222,7 +2222,7 @@
         <v>0.148276</v>
       </c>
       <c r="Q20" t="n">
-        <v>270.9</v>
+        <v>272</v>
       </c>
       <c r="R20" t="n">
         <v>10391.2</v>
@@ -2238,13 +2238,13 @@
         <v>266.8933313244817</v>
       </c>
       <c r="W20" t="n">
-        <v>0.1609221962047922</v>
+        <v>0.1602714079113169</v>
       </c>
       <c r="X20" t="n">
         <v>0.0037468152352755</v>
       </c>
       <c r="Y20" t="n">
-        <v>38.35806570690292</v>
+        <v>38.20294117647059</v>
       </c>
       <c r="Z20" t="n">
         <v>4.195263583789957</v>
@@ -2296,7 +2296,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K21" t="n">
-        <v>2.923599028912937</v>
+        <v>3.331714659061363</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.021793</v>
       </c>
       <c r="Q21" t="n">
-        <v>858</v>
+        <v>752.9</v>
       </c>
       <c r="R21" t="n">
         <v>44420.3</v>
@@ -2328,13 +2328,13 @@
         <v>1834.787418303125</v>
       </c>
       <c r="W21" t="n">
-        <v>0.04872665048188229</v>
+        <v>0.05552857765102271</v>
       </c>
       <c r="X21" t="n">
         <v>0.0005450222679883181</v>
       </c>
       <c r="Y21" t="n">
-        <v>51.77191142191143</v>
+        <v>58.99893744189136</v>
       </c>
       <c r="Z21" t="n">
         <v>0.9411792831983349</v>
@@ -2386,7 +2386,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K22" t="n">
-        <v>30.39076646776515</v>
+        <v>33.86998524959206</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.088764</v>
       </c>
       <c r="Q22" t="n">
-        <v>80.8</v>
+        <v>72.5</v>
       </c>
       <c r="R22" t="n">
         <v>24301.8</v>
@@ -2418,13 +2418,13 @@
         <v>439.4668804599139</v>
       </c>
       <c r="W22" t="n">
-        <v>0.5065127744627526</v>
+        <v>0.5644997541598676</v>
       </c>
       <c r="X22" t="n">
         <v>0.002275484329907804</v>
       </c>
       <c r="Y22" t="n">
-        <v>300.7648514851485</v>
+        <v>335.1972413793104</v>
       </c>
       <c r="Z22" t="n">
         <v>1.684082338616498</v>
@@ -2566,7 +2566,7 @@
         <v>37.3244239690841</v>
       </c>
       <c r="K24" t="n">
-        <v>21.70024649365355</v>
+        <v>21.57481154282318</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2582,7 +2582,7 @@
         <v>0.015269</v>
       </c>
       <c r="Q24" t="n">
-        <v>103.2</v>
+        <v>103.8</v>
       </c>
       <c r="R24" t="n">
         <v>13175.4</v>
@@ -2598,13 +2598,13 @@
         <v>2269.237838587312</v>
       </c>
       <c r="W24" t="n">
-        <v>0.3616707748942258</v>
+        <v>0.3595801923803864</v>
       </c>
       <c r="X24" t="n">
         <v>0.0004406765932576458</v>
       </c>
       <c r="Y24" t="n">
-        <v>127.6686046511628</v>
+        <v>126.9306358381503</v>
       </c>
       <c r="Z24" t="n">
         <v>2.832887348322184</v>
@@ -2656,7 +2656,7 @@
         <v>37.2559686869738</v>
       </c>
       <c r="K25" t="n">
-        <v>20.79402903459003</v>
+        <v>20.94993553156915</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2672,7 +2672,7 @@
         <v>0.007626</v>
       </c>
       <c r="Q25" t="n">
-        <v>107.5</v>
+        <v>106.7</v>
       </c>
       <c r="R25" t="n">
         <v>15761.3</v>
@@ -2688,13 +2688,13 @@
         <v>4556.747637839262</v>
       </c>
       <c r="W25" t="n">
-        <v>0.3465671505765005</v>
+        <v>0.3491655921928191</v>
       </c>
       <c r="X25" t="n">
         <v>0.0002194547689444097</v>
       </c>
       <c r="Y25" t="n">
-        <v>146.6167441860465</v>
+        <v>147.7160262417994</v>
       </c>
       <c r="Z25" t="n">
         <v>2.363762423592839</v>
@@ -2746,7 +2746,7 @@
         <v>33.6962858057476</v>
       </c>
       <c r="K26" t="n">
-        <v>3.98301250658955</v>
+        <v>4.089355073513058</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2762,7 +2762,7 @@
         <v>0.084838</v>
       </c>
       <c r="Q26" t="n">
-        <v>507.6</v>
+        <v>494.4</v>
       </c>
       <c r="R26" t="n">
         <v>29565.5</v>
@@ -2778,13 +2778,13 @@
         <v>372.0058048768779</v>
       </c>
       <c r="W26" t="n">
-        <v>0.06638354177649251</v>
+        <v>0.06815591789188431</v>
       </c>
       <c r="X26" t="n">
         <v>0.002688130096063873</v>
       </c>
       <c r="Y26" t="n">
-        <v>58.2456658786446</v>
+        <v>59.80076860841424</v>
       </c>
       <c r="Z26" t="n">
         <v>1.139716419669804</v>
@@ -2898,7 +2898,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K28" t="n">
-        <v>14.70820128706288</v>
+        <v>17.67356444977718</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2914,7 +2914,7 @@
         <v>0.021244</v>
       </c>
       <c r="Q28" t="n">
-        <v>119.2</v>
+        <v>99.2</v>
       </c>
       <c r="R28" t="n">
         <v>18211.1</v>
@@ -2930,13 +2930,13 @@
         <v>1104.110834068831</v>
       </c>
       <c r="W28" t="n">
-        <v>0.2451366881177148</v>
+        <v>0.2945594074962863</v>
       </c>
       <c r="X28" t="n">
         <v>0.0009057061747277989</v>
       </c>
       <c r="Y28" t="n">
-        <v>152.7776845637584</v>
+        <v>183.5796370967742</v>
       </c>
       <c r="Z28" t="n">
         <v>1.604532028467891</v>
@@ -2988,7 +2988,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K29" t="n">
-        <v>12.83464782531082</v>
+        <v>13.36084550798845</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -3004,7 +3004,7 @@
         <v>0.09042</v>
       </c>
       <c r="Q29" t="n">
-        <v>116.8</v>
+        <v>112.2</v>
       </c>
       <c r="R29" t="n">
         <v>22793.6</v>
@@ -3020,13 +3020,13 @@
         <v>263.8642816401065</v>
       </c>
       <c r="W29" t="n">
-        <v>0.2139107970885137</v>
+        <v>0.2226807584664741</v>
       </c>
       <c r="X29" t="n">
         <v>0.00378982707998324</v>
       </c>
       <c r="Y29" t="n">
-        <v>195.1506849315068</v>
+        <v>203.1515151515151</v>
       </c>
       <c r="Z29" t="n">
         <v>1.096131418465639</v>
@@ -3078,7 +3078,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K30" t="n">
-        <v>15.11730484106756</v>
+        <v>18.51513782687952</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3094,7 +3094,7 @@
         <v>0.02862</v>
       </c>
       <c r="Q30" t="n">
-        <v>91</v>
+        <v>74.3</v>
       </c>
       <c r="R30" t="n">
         <v>12593.6</v>
@@ -3110,13 +3110,13 @@
         <v>694.5957872787968</v>
       </c>
       <c r="W30" t="n">
-        <v>0.2519550806844593</v>
+        <v>0.3085856304479919</v>
       </c>
       <c r="X30" t="n">
         <v>0.001439686243876714</v>
       </c>
       <c r="Y30" t="n">
-        <v>138.3912087912088</v>
+        <v>169.4966352624495</v>
       </c>
       <c r="Z30" t="n">
         <v>1.820600332096128</v>
@@ -3168,7 +3168,7 @@
         <v>22.1685424839812</v>
       </c>
       <c r="K31" t="n">
-        <v>62.15479201116224</v>
+        <v>59.91497968643567</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3184,7 +3184,7 @@
         <v>0.017024</v>
       </c>
       <c r="Q31" t="n">
-        <v>21.4</v>
+        <v>22.2</v>
       </c>
       <c r="R31" t="n">
         <v>7379.9</v>
@@ -3200,13 +3200,13 @@
         <v>1152.690436979056</v>
       </c>
       <c r="W31" t="n">
-        <v>1.035913200186037</v>
+        <v>0.9985829947739279</v>
       </c>
       <c r="X31" t="n">
         <v>0.0008675356087977764</v>
       </c>
       <c r="Y31" t="n">
-        <v>344.8551401869159</v>
+        <v>332.4279279279279</v>
       </c>
       <c r="Z31" t="n">
         <v>3.003908248618708</v>
@@ -3258,7 +3258,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K32" t="n">
-        <v>14.22693428136757</v>
+        <v>14.09307871689234</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3274,7 +3274,7 @@
         <v>0.009842</v>
       </c>
       <c r="Q32" t="n">
-        <v>73.7</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="R32" t="n">
         <v>7737.1</v>
@@ -3290,13 +3290,13 @@
         <v>1572.37876632594</v>
       </c>
       <c r="W32" t="n">
-        <v>0.2371155713561262</v>
+        <v>0.234884645281539</v>
       </c>
       <c r="X32" t="n">
         <v>0.0006359790792244194</v>
       </c>
       <c r="Y32" t="n">
-        <v>104.9810040705563</v>
+        <v>103.9932795698925</v>
       </c>
       <c r="Z32" t="n">
         <v>2.258652157649054</v>
@@ -3348,7 +3348,7 @@
         <v>14.1889227802691</v>
       </c>
       <c r="K33" t="n">
-        <v>9.124709183452799</v>
+        <v>9.243597902455441</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -3364,7 +3364,7 @@
         <v>0.047676</v>
       </c>
       <c r="Q33" t="n">
-        <v>93.3</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="R33" t="n">
         <v>14142</v>
@@ -3380,13 +3380,13 @@
         <v>131.1287985903656</v>
       </c>
       <c r="W33" t="n">
-        <v>0.15207848639088</v>
+        <v>0.154059965040924</v>
       </c>
       <c r="X33" t="n">
         <v>0.007626089850208333</v>
       </c>
       <c r="Y33" t="n">
-        <v>151.5755627009646</v>
+        <v>153.5504885993485</v>
       </c>
       <c r="Z33" t="n">
         <v>1.003317973431558</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-09-27)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -676,7 +676,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K3" t="n">
-        <v>75.48856258518728</v>
+        <v>74.98305881787577</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -692,7 +692,7 @@
         <v>0.09657399999999999</v>
       </c>
       <c r="Q3" t="n">
-        <v>44.5</v>
+        <v>44.8</v>
       </c>
       <c r="R3" t="n">
         <v>6353.5</v>
@@ -708,13 +708,13 @@
         <v>383.8588628629582</v>
       </c>
       <c r="W3" t="n">
-        <v>1.258142709753121</v>
+        <v>1.249717646964596</v>
       </c>
       <c r="X3" t="n">
         <v>0.002605124166058427</v>
       </c>
       <c r="Y3" t="n">
-        <v>142.7752808988764</v>
+        <v>141.8191964285714</v>
       </c>
       <c r="Z3" t="n">
         <v>8.81204856913731</v>
@@ -766,7 +766,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K4" t="n">
-        <v>144.1700340328431</v>
+        <v>141.0084104794913</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -782,7 +782,7 @@
         <v>0.03274</v>
       </c>
       <c r="Q4" t="n">
-        <v>22.3</v>
+        <v>22.8</v>
       </c>
       <c r="R4" t="n">
         <v>3004</v>
@@ -798,13 +798,13 @@
         <v>686.2074633379441</v>
       </c>
       <c r="W4" t="n">
-        <v>2.402833900547386</v>
+        <v>2.350140174658188</v>
       </c>
       <c r="X4" t="n">
         <v>0.001457285228487116</v>
       </c>
       <c r="Y4" t="n">
-        <v>134.7085201793722</v>
+        <v>131.7543859649123</v>
       </c>
       <c r="Z4" t="n">
         <v>17.83728228435643</v>
@@ -856,7 +856,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K5" t="n">
-        <v>15.22251810622687</v>
+        <v>15.3172036255479</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -872,7 +872,7 @@
         <v>1.087069</v>
       </c>
       <c r="Q5" t="n">
-        <v>210.3</v>
+        <v>209</v>
       </c>
       <c r="R5" t="n">
         <v>23039.4</v>
@@ -888,13 +888,13 @@
         <v>44.3365962628782</v>
       </c>
       <c r="W5" t="n">
-        <v>0.2537086351037812</v>
+        <v>0.2552867270924651</v>
       </c>
       <c r="X5" t="n">
         <v>0.022554730951173</v>
       </c>
       <c r="Y5" t="n">
-        <v>109.5549215406562</v>
+        <v>110.2363636363636</v>
       </c>
       <c r="Z5" t="n">
         <v>2.315812302504631</v>
@@ -946,7 +946,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K6" t="n">
-        <v>30.43084390117887</v>
+        <v>31.05248565402397</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -962,7 +962,7 @@
         <v>0.452635</v>
       </c>
       <c r="Q6" t="n">
-        <v>104.9</v>
+        <v>102.8</v>
       </c>
       <c r="R6" t="n">
         <v>10176.4</v>
@@ -978,13 +978,13 @@
         <v>95.52129303831462</v>
       </c>
       <c r="W6" t="n">
-        <v>0.5071807316863146</v>
+        <v>0.5175414275670662</v>
       </c>
       <c r="X6" t="n">
         <v>0.01046887000994521</v>
       </c>
       <c r="Y6" t="n">
-        <v>97.01048617731172</v>
+        <v>98.99221789883268</v>
       </c>
       <c r="Z6" t="n">
         <v>5.228102153403404</v>
@@ -1036,7 +1036,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K7" t="n">
-        <v>34.09298990000841</v>
+        <v>34.99911587741728</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1052,7 +1052,7 @@
         <v>0.25811</v>
       </c>
       <c r="Q7" t="n">
-        <v>92.7</v>
+        <v>90.3</v>
       </c>
       <c r="R7" t="n">
         <v>5609.9</v>
@@ -1068,13 +1068,13 @@
         <v>173.6055812119343</v>
       </c>
       <c r="W7" t="n">
-        <v>0.5682164983334735</v>
+        <v>0.5833185979569546</v>
       </c>
       <c r="X7" t="n">
         <v>0.005760183474627001</v>
       </c>
       <c r="Y7" t="n">
-        <v>60.51672060409924</v>
+        <v>62.12513842746401</v>
       </c>
       <c r="Z7" t="n">
         <v>9.389413250773277</v>
@@ -1126,7 +1126,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K8" t="n">
-        <v>60.91433454753279</v>
+        <v>58.6414116166547</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1142,7 +1142,7 @@
         <v>0.126814</v>
       </c>
       <c r="Q8" t="n">
-        <v>51.6</v>
+        <v>53.6</v>
       </c>
       <c r="R8" t="n">
         <v>2987.7</v>
@@ -1158,13 +1158,13 @@
         <v>303.7663387233741</v>
       </c>
       <c r="W8" t="n">
-        <v>1.015238909125546</v>
+        <v>0.9773568602775783</v>
       </c>
       <c r="X8" t="n">
         <v>0.003292003992946215</v>
       </c>
       <c r="Y8" t="n">
-        <v>57.90116279069767</v>
+        <v>55.74067164179104</v>
       </c>
       <c r="Z8" t="n">
         <v>17.53399863134793</v>
@@ -1216,7 +1216,7 @@
         <v>51.2434931792768</v>
       </c>
       <c r="K9" t="n">
-        <v>183.0124756402743</v>
+        <v>174.6937267475345</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1232,7 +1232,7 @@
         <v>0.01898</v>
       </c>
       <c r="Q9" t="n">
-        <v>16.8</v>
+        <v>17.6</v>
       </c>
       <c r="R9" t="n">
         <v>2234.8</v>
@@ -1248,13 +1248,13 @@
         <v>824.4601019930624</v>
       </c>
       <c r="W9" t="n">
-        <v>3.050207927337905</v>
+        <v>2.911562112458909</v>
       </c>
       <c r="X9" t="n">
         <v>0.001212914970151478</v>
       </c>
       <c r="Y9" t="n">
-        <v>133.0238095238095</v>
+        <v>126.9772727272727</v>
       </c>
       <c r="Z9" t="n">
         <v>22.92978932310578</v>
@@ -1306,7 +1306,7 @@
         <v>50.7771115797629</v>
       </c>
       <c r="K10" t="n">
-        <v>30.9931505064677</v>
+        <v>31.11978237779136</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1322,7 @@
         <v>0.20946</v>
       </c>
       <c r="Q10" t="n">
-        <v>98.3</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="R10" t="n">
         <v>9435.6</v>
@@ -1338,13 +1338,13 @@
         <v>198.7704793771252</v>
       </c>
       <c r="W10" t="n">
-        <v>0.5165525084411282</v>
+        <v>0.5186630396298559</v>
       </c>
       <c r="X10" t="n">
         <v>0.005030928149560429</v>
       </c>
       <c r="Y10" t="n">
-        <v>95.98779247202442</v>
+        <v>96.3799795709908</v>
       </c>
       <c r="Z10" t="n">
         <v>5.381439609538651</v>
@@ -1396,7 +1396,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K11" t="n">
-        <v>33.16711087721966</v>
+        <v>30.40609743222455</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1412,7 +1412,7 @@
         <v>0.07542500000000001</v>
       </c>
       <c r="Q11" t="n">
-        <v>87</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="R11" t="n">
         <v>18553.6</v>
@@ -1428,13 +1428,13 @@
         <v>578.4775641354948</v>
       </c>
       <c r="W11" t="n">
-        <v>0.5527851812869943</v>
+        <v>0.5067682905370758</v>
       </c>
       <c r="X11" t="n">
         <v>0.001728675513102135</v>
       </c>
       <c r="Y11" t="n">
-        <v>213.2597701149425</v>
+        <v>195.5068493150685</v>
       </c>
       <c r="Z11" t="n">
         <v>2.592074356026243</v>
@@ -1576,7 +1576,7 @@
         <v>46.9727068915036</v>
       </c>
       <c r="K13" t="n">
-        <v>40.20488464322705</v>
+        <v>45.02176379377341</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1592,7 +1592,7 @@
         <v>0.111119</v>
       </c>
       <c r="Q13" t="n">
-        <v>70.09999999999999</v>
+        <v>62.6</v>
       </c>
       <c r="R13" t="n">
         <v>5952.7</v>
@@ -1608,13 +1608,13 @@
         <v>370.7747134022449</v>
       </c>
       <c r="W13" t="n">
-        <v>0.6700814107204508</v>
+        <v>0.7503627298962237</v>
       </c>
       <c r="X13" t="n">
         <v>0.002697055553826625</v>
       </c>
       <c r="Y13" t="n">
-        <v>84.91726105563481</v>
+        <v>95.09105431309904</v>
       </c>
       <c r="Z13" t="n">
         <v>7.890991800612092</v>
@@ -1666,7 +1666,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K14" t="n">
-        <v>4.137777338995867</v>
+        <v>4.126748167945678</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1682,7 @@
         <v>0.337573</v>
       </c>
       <c r="Q14" t="n">
-        <v>673.5</v>
+        <v>675.3</v>
       </c>
       <c r="R14" t="n">
         <v>57055.2</v>
@@ -1698,13 +1698,13 @@
         <v>132.374251168453</v>
       </c>
       <c r="W14" t="n">
-        <v>0.0689629556499311</v>
+        <v>0.06877913613242796</v>
       </c>
       <c r="X14" t="n">
         <v>0.007554339240245816</v>
       </c>
       <c r="Y14" t="n">
-        <v>84.71447661469932</v>
+        <v>84.48867170146602</v>
       </c>
       <c r="Z14" t="n">
         <v>0.814063409298865</v>
@@ -1756,7 +1756,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K15" t="n">
-        <v>6.487984107988558</v>
+        <v>6.147870807038925</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1772,7 +1772,7 @@
         <v>0.0152</v>
       </c>
       <c r="Q15" t="n">
-        <v>428.4</v>
+        <v>452.1</v>
       </c>
       <c r="R15" t="n">
         <v>20796.5</v>
@@ -1788,13 +1788,13 @@
         <v>2193.173304187023</v>
       </c>
       <c r="W15" t="n">
-        <v>0.108133068466476</v>
+        <v>0.1024645134506487</v>
       </c>
       <c r="X15" t="n">
         <v>0.0004559603192738502</v>
       </c>
       <c r="Y15" t="n">
-        <v>48.54458450046685</v>
+        <v>45.99977880999779</v>
       </c>
       <c r="Z15" t="n">
         <v>2.227500133726266</v>
@@ -1846,7 +1846,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K16" t="n">
-        <v>5.579263943249645</v>
+        <v>5.460746512791836</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1862,7 @@
         <v>0.141536</v>
       </c>
       <c r="Q16" t="n">
-        <v>488.4</v>
+        <v>499</v>
       </c>
       <c r="R16" t="n">
         <v>24843.6</v>
@@ -1878,13 +1878,13 @@
         <v>290.2523742749451</v>
       </c>
       <c r="W16" t="n">
-        <v>0.09298773238749407</v>
+        <v>0.09101244187986393</v>
       </c>
       <c r="X16" t="n">
         <v>0.003445277588161046</v>
       </c>
       <c r="Y16" t="n">
-        <v>50.86732186732187</v>
+        <v>49.78677354709419</v>
       </c>
       <c r="Z16" t="n">
         <v>1.828044586857464</v>
@@ -1936,7 +1936,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K17" t="n">
-        <v>7.10000936346945</v>
+        <v>7.306618284299266</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1952,7 @@
         <v>0.148652</v>
       </c>
       <c r="Q17" t="n">
-        <v>378.4</v>
+        <v>367.7</v>
       </c>
       <c r="R17" t="n">
         <v>34728.3</v>
@@ -1968,13 +1968,13 @@
         <v>281.760586368072</v>
       </c>
       <c r="W17" t="n">
-        <v>0.1183334893911575</v>
+        <v>0.1217769714049878</v>
       </c>
       <c r="X17" t="n">
         <v>0.003549112432260739</v>
       </c>
       <c r="Y17" t="n">
-        <v>91.7766913319239</v>
+        <v>94.44737557791679</v>
       </c>
       <c r="Z17" t="n">
         <v>1.289363210569305</v>
@@ -2026,7 +2026,7 @@
         <v>44.3113073012592</v>
       </c>
       <c r="K18" t="n">
-        <v>16.54435866879622</v>
+        <v>16.40147093198983</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2042,7 +2042,7 @@
         <v>0.058096</v>
       </c>
       <c r="Q18" t="n">
-        <v>160.7</v>
+        <v>162.1</v>
       </c>
       <c r="R18" t="n">
         <v>10197.8</v>
@@ -2058,13 +2058,13 @@
         <v>662.6188043195191</v>
       </c>
       <c r="W18" t="n">
-        <v>0.2757393111466036</v>
+        <v>0.2733578488664972</v>
       </c>
       <c r="X18" t="n">
         <v>0.001509163328117374</v>
       </c>
       <c r="Y18" t="n">
-        <v>63.45861854387056</v>
+        <v>62.91054904380012</v>
       </c>
       <c r="Z18" t="n">
         <v>4.345183010184472</v>
@@ -2116,7 +2116,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>14.00244554348817</v>
+        <v>13.69550258272278</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2132,7 @@
         <v>0.039576</v>
       </c>
       <c r="Q19" t="n">
-        <v>187.4</v>
+        <v>191.6</v>
       </c>
       <c r="R19" t="n">
         <v>15469.6</v>
@@ -2148,13 +2148,13 @@
         <v>972.1110696872879</v>
       </c>
       <c r="W19" t="n">
-        <v>0.2333740923914696</v>
+        <v>0.2282583763787129</v>
       </c>
       <c r="X19" t="n">
         <v>0.001028689036862509</v>
       </c>
       <c r="Y19" t="n">
-        <v>82.54855923159018</v>
+        <v>80.73903966597078</v>
       </c>
       <c r="Z19" t="n">
         <v>2.827112848047875</v>
@@ -2206,7 +2206,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>9.616284474679015</v>
+        <v>9.487230239799391</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2222,7 +2222,7 @@
         <v>0.148276</v>
       </c>
       <c r="Q20" t="n">
-        <v>272</v>
+        <v>275.7</v>
       </c>
       <c r="R20" t="n">
         <v>10391.2</v>
@@ -2238,13 +2238,13 @@
         <v>266.8933313244817</v>
       </c>
       <c r="W20" t="n">
-        <v>0.1602714079113169</v>
+        <v>0.1581205039966565</v>
       </c>
       <c r="X20" t="n">
         <v>0.0037468152352755</v>
       </c>
       <c r="Y20" t="n">
-        <v>38.20294117647059</v>
+        <v>37.69024301777294</v>
       </c>
       <c r="Z20" t="n">
         <v>4.195263583789957</v>
@@ -2296,7 +2296,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K21" t="n">
-        <v>3.331714659061363</v>
+        <v>3.635958786501377</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.021793</v>
       </c>
       <c r="Q21" t="n">
-        <v>752.9</v>
+        <v>689.9</v>
       </c>
       <c r="R21" t="n">
         <v>44420.3</v>
@@ -2328,13 +2328,13 @@
         <v>1834.787418303125</v>
       </c>
       <c r="W21" t="n">
-        <v>0.05552857765102271</v>
+        <v>0.06059931310835628</v>
       </c>
       <c r="X21" t="n">
         <v>0.0005450222679883181</v>
       </c>
       <c r="Y21" t="n">
-        <v>58.99893744189136</v>
+        <v>64.38657776489347</v>
       </c>
       <c r="Z21" t="n">
         <v>0.9411792831983349</v>
@@ -2386,7 +2386,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K22" t="n">
-        <v>33.86998524959206</v>
+        <v>30.54196431088836</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.088764</v>
       </c>
       <c r="Q22" t="n">
-        <v>72.5</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="R22" t="n">
         <v>24301.8</v>
@@ -2418,13 +2418,13 @@
         <v>439.4668804599139</v>
       </c>
       <c r="W22" t="n">
-        <v>0.5644997541598676</v>
+        <v>0.509032738514806</v>
       </c>
       <c r="X22" t="n">
         <v>0.002275484329907804</v>
       </c>
       <c r="Y22" t="n">
-        <v>335.1972413793104</v>
+        <v>302.2611940298507</v>
       </c>
       <c r="Z22" t="n">
         <v>1.684082338616498</v>
@@ -2476,7 +2476,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K23" t="n">
-        <v>34.21054983167081</v>
+        <v>31.81948989719919</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2492,7 +2492,7 @@
         <v>0.02621</v>
       </c>
       <c r="Q23" t="n">
-        <v>69.2</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="R23" t="n">
         <v>22336.9</v>
@@ -2508,13 +2508,13 @@
         <v>1426.160900474481</v>
       </c>
       <c r="W23" t="n">
-        <v>0.5701758305278468</v>
+        <v>0.5303248316199866</v>
       </c>
       <c r="X23" t="n">
         <v>0.0007011831551876802</v>
       </c>
       <c r="Y23" t="n">
-        <v>322.7875722543353</v>
+        <v>300.2271505376344</v>
       </c>
       <c r="Z23" t="n">
         <v>1.76641196730643</v>
@@ -2566,7 +2566,7 @@
         <v>37.3244239690841</v>
       </c>
       <c r="K24" t="n">
-        <v>21.57481154282318</v>
+        <v>21.368945020468</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2582,7 +2582,7 @@
         <v>0.015269</v>
       </c>
       <c r="Q24" t="n">
-        <v>103.8</v>
+        <v>104.8</v>
       </c>
       <c r="R24" t="n">
         <v>13175.4</v>
@@ -2598,13 +2598,13 @@
         <v>2269.237838587312</v>
       </c>
       <c r="W24" t="n">
-        <v>0.3595801923803864</v>
+        <v>0.3561490836744666</v>
       </c>
       <c r="X24" t="n">
         <v>0.0004406765932576458</v>
       </c>
       <c r="Y24" t="n">
-        <v>126.9306358381503</v>
+        <v>125.719465648855</v>
       </c>
       <c r="Z24" t="n">
         <v>2.832887348322184</v>
@@ -2656,7 +2656,7 @@
         <v>37.2559686869738</v>
       </c>
       <c r="K25" t="n">
-        <v>20.94993553156915</v>
+        <v>22.04495188578331</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2672,7 +2672,7 @@
         <v>0.007626</v>
       </c>
       <c r="Q25" t="n">
-        <v>106.7</v>
+        <v>101.4</v>
       </c>
       <c r="R25" t="n">
         <v>15761.3</v>
@@ -2688,13 +2688,13 @@
         <v>4556.747637839262</v>
       </c>
       <c r="W25" t="n">
-        <v>0.3491655921928191</v>
+        <v>0.3674158647630552</v>
       </c>
       <c r="X25" t="n">
         <v>0.0002194547689444097</v>
       </c>
       <c r="Y25" t="n">
-        <v>147.7160262417994</v>
+        <v>155.4368836291913</v>
       </c>
       <c r="Z25" t="n">
         <v>2.363762423592839</v>
@@ -2746,7 +2746,7 @@
         <v>33.6962858057476</v>
       </c>
       <c r="K26" t="n">
-        <v>4.089355073513058</v>
+        <v>3.98301250658955</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2762,7 +2762,7 @@
         <v>0.084838</v>
       </c>
       <c r="Q26" t="n">
-        <v>494.4</v>
+        <v>507.6</v>
       </c>
       <c r="R26" t="n">
         <v>29565.5</v>
@@ -2778,13 +2778,13 @@
         <v>372.0058048768779</v>
       </c>
       <c r="W26" t="n">
-        <v>0.06815591789188431</v>
+        <v>0.06638354177649251</v>
       </c>
       <c r="X26" t="n">
         <v>0.002688130096063873</v>
       </c>
       <c r="Y26" t="n">
-        <v>59.80076860841424</v>
+        <v>58.2456658786446</v>
       </c>
       <c r="Z26" t="n">
         <v>1.139716419669804</v>
@@ -2898,7 +2898,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K28" t="n">
-        <v>17.67356444977718</v>
+        <v>17.41030380752628</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2914,7 +2914,7 @@
         <v>0.021244</v>
       </c>
       <c r="Q28" t="n">
-        <v>99.2</v>
+        <v>100.7</v>
       </c>
       <c r="R28" t="n">
         <v>18211.1</v>
@@ -2930,13 +2930,13 @@
         <v>1104.110834068831</v>
       </c>
       <c r="W28" t="n">
-        <v>0.2945594074962863</v>
+        <v>0.290171730125438</v>
       </c>
       <c r="X28" t="n">
         <v>0.0009057061747277989</v>
       </c>
       <c r="Y28" t="n">
-        <v>183.5796370967742</v>
+        <v>180.845084409136</v>
       </c>
       <c r="Z28" t="n">
         <v>1.604532028467891</v>
@@ -2988,7 +2988,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K29" t="n">
-        <v>13.36084550798845</v>
+        <v>13.43267801071957</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -3004,7 +3004,7 @@
         <v>0.09042</v>
       </c>
       <c r="Q29" t="n">
-        <v>112.2</v>
+        <v>111.6</v>
       </c>
       <c r="R29" t="n">
         <v>22793.6</v>
@@ -3020,13 +3020,13 @@
         <v>263.8642816401065</v>
       </c>
       <c r="W29" t="n">
-        <v>0.2226807584664741</v>
+        <v>0.2238779668453262</v>
       </c>
       <c r="X29" t="n">
         <v>0.00378982707998324</v>
       </c>
       <c r="Y29" t="n">
-        <v>203.1515151515151</v>
+        <v>204.2437275985663</v>
       </c>
       <c r="Z29" t="n">
         <v>1.096131418465639</v>
@@ -3078,7 +3078,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K30" t="n">
-        <v>18.51513782687952</v>
+        <v>22.01079584859437</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3094,7 +3094,7 @@
         <v>0.02862</v>
       </c>
       <c r="Q30" t="n">
-        <v>74.3</v>
+        <v>62.5</v>
       </c>
       <c r="R30" t="n">
         <v>12593.6</v>
@@ -3110,13 +3110,13 @@
         <v>694.5957872787968</v>
       </c>
       <c r="W30" t="n">
-        <v>0.3085856304479919</v>
+        <v>0.3668465974765728</v>
       </c>
       <c r="X30" t="n">
         <v>0.001439686243876714</v>
       </c>
       <c r="Y30" t="n">
-        <v>169.4966352624495</v>
+        <v>201.4976</v>
       </c>
       <c r="Z30" t="n">
         <v>1.820600332096128</v>
@@ -3168,7 +3168,7 @@
         <v>22.1685424839812</v>
       </c>
       <c r="K31" t="n">
-        <v>59.91497968643567</v>
+        <v>61.01433711187486</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3184,7 +3184,7 @@
         <v>0.017024</v>
       </c>
       <c r="Q31" t="n">
-        <v>22.2</v>
+        <v>21.8</v>
       </c>
       <c r="R31" t="n">
         <v>7379.9</v>
@@ -3200,13 +3200,13 @@
         <v>1152.690436979056</v>
       </c>
       <c r="W31" t="n">
-        <v>0.9985829947739279</v>
+        <v>1.016905618531248</v>
       </c>
       <c r="X31" t="n">
         <v>0.0008675356087977764</v>
       </c>
       <c r="Y31" t="n">
-        <v>332.4279279279279</v>
+        <v>338.5275229357798</v>
       </c>
       <c r="Z31" t="n">
         <v>3.003908248618708</v>
@@ -3258,7 +3258,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K32" t="n">
-        <v>14.09307871689234</v>
+        <v>14.50242125223776</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3274,7 +3274,7 @@
         <v>0.009842</v>
       </c>
       <c r="Q32" t="n">
-        <v>74.40000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="R32" t="n">
         <v>7737.1</v>
@@ -3290,13 +3290,13 @@
         <v>1572.37876632594</v>
       </c>
       <c r="W32" t="n">
-        <v>0.234884645281539</v>
+        <v>0.2417070208706293</v>
       </c>
       <c r="X32" t="n">
         <v>0.0006359790792244194</v>
       </c>
       <c r="Y32" t="n">
-        <v>103.9932795698925</v>
+        <v>107.0138312586445</v>
       </c>
       <c r="Z32" t="n">
         <v>2.258652157649054</v>
@@ -3348,7 +3348,7 @@
         <v>14.1889227802691</v>
       </c>
       <c r="K33" t="n">
-        <v>9.243597902455441</v>
+        <v>9.448783205506617</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -3364,7 +3364,7 @@
         <v>0.047676</v>
       </c>
       <c r="Q33" t="n">
-        <v>92.09999999999999</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="R33" t="n">
         <v>14142</v>
@@ -3380,13 +3380,13 @@
         <v>131.1287985903656</v>
       </c>
       <c r="W33" t="n">
-        <v>0.154059965040924</v>
+        <v>0.1574797200917769</v>
       </c>
       <c r="X33" t="n">
         <v>0.007626089850208333</v>
       </c>
       <c r="Y33" t="n">
-        <v>153.5504885993485</v>
+        <v>156.9589345172031</v>
       </c>
       <c r="Z33" t="n">
         <v>1.003317973431558</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-09-28)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -593,7 +593,9 @@
       <c r="J2" t="n">
         <v>57.6223698102963</v>
       </c>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="n">
+        <v>13.77976161266552</v>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
         <v>0.770958</v>
@@ -607,7 +609,9 @@
       <c r="P2" t="n">
         <v>0.711927</v>
       </c>
-      <c r="Q2" t="inlineStr"/>
+      <c r="Q2" t="n">
+        <v>250.9</v>
+      </c>
       <c r="R2" t="n">
         <v>37461.4</v>
       </c>
@@ -621,11 +625,15 @@
       <c r="V2" t="n">
         <v>74.74125673551127</v>
       </c>
-      <c r="W2" t="inlineStr"/>
+      <c r="W2" t="n">
+        <v>0.2296626935444253</v>
+      </c>
       <c r="X2" t="n">
         <v>0.0133794913770145</v>
       </c>
-      <c r="Y2" t="inlineStr"/>
+      <c r="Y2" t="n">
+        <v>149.3080908728577</v>
+      </c>
       <c r="Z2" t="n">
         <v>1.538179828044235</v>
       </c>
@@ -676,7 +684,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K3" t="n">
-        <v>74.15543123710451</v>
+        <v>74.48428015611606</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -692,7 +700,7 @@
         <v>0.09657399999999999</v>
       </c>
       <c r="Q3" t="n">
-        <v>45.3</v>
+        <v>45.1</v>
       </c>
       <c r="R3" t="n">
         <v>6353.5</v>
@@ -708,13 +716,13 @@
         <v>383.8588628629582</v>
       </c>
       <c r="W3" t="n">
-        <v>1.235923853951742</v>
+        <v>1.241404669268601</v>
       </c>
       <c r="X3" t="n">
         <v>0.002605124166058427</v>
       </c>
       <c r="Y3" t="n">
-        <v>140.2538631346578</v>
+        <v>140.8758314855876</v>
       </c>
       <c r="Z3" t="n">
         <v>8.81204856913731</v>
@@ -766,7 +774,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K4" t="n">
-        <v>133.9579899555168</v>
+        <v>141.6295929045111</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -782,7 +790,7 @@
         <v>0.03274</v>
       </c>
       <c r="Q4" t="n">
-        <v>24</v>
+        <v>22.7</v>
       </c>
       <c r="R4" t="n">
         <v>3004</v>
@@ -798,13 +806,13 @@
         <v>686.2074633379441</v>
       </c>
       <c r="W4" t="n">
-        <v>2.232633165925279</v>
+        <v>2.360493215075185</v>
       </c>
       <c r="X4" t="n">
         <v>0.001457285228487116</v>
       </c>
       <c r="Y4" t="n">
-        <v>125.1666666666667</v>
+        <v>132.3348017621146</v>
       </c>
       <c r="Z4" t="n">
         <v>17.83728228435643</v>
@@ -856,7 +864,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K5" t="n">
-        <v>15.27335666860454</v>
+        <v>15.02250379042474</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -872,7 +880,7 @@
         <v>1.087069</v>
       </c>
       <c r="Q5" t="n">
-        <v>209.6</v>
+        <v>213.1</v>
       </c>
       <c r="R5" t="n">
         <v>23039.4</v>
@@ -888,13 +896,13 @@
         <v>44.3365962628782</v>
       </c>
       <c r="W5" t="n">
-        <v>0.2545559444767423</v>
+        <v>0.2503750631737456</v>
       </c>
       <c r="X5" t="n">
         <v>0.022554730951173</v>
       </c>
       <c r="Y5" t="n">
-        <v>109.9208015267176</v>
+        <v>108.115438761145</v>
       </c>
       <c r="Z5" t="n">
         <v>2.315812302504631</v>
@@ -946,7 +954,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K6" t="n">
-        <v>29.36702415118366</v>
+        <v>32.08236708777552</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -962,7 +970,7 @@
         <v>0.452635</v>
       </c>
       <c r="Q6" t="n">
-        <v>108.7</v>
+        <v>99.5</v>
       </c>
       <c r="R6" t="n">
         <v>10176.4</v>
@@ -978,13 +986,13 @@
         <v>95.52129303831462</v>
       </c>
       <c r="W6" t="n">
-        <v>0.4894504025197277</v>
+        <v>0.534706118129592</v>
       </c>
       <c r="X6" t="n">
         <v>0.01046887000994521</v>
       </c>
       <c r="Y6" t="n">
-        <v>93.61913523459062</v>
+        <v>102.2753768844221</v>
       </c>
       <c r="Z6" t="n">
         <v>5.228102153403404</v>
@@ -1036,7 +1044,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K7" t="n">
-        <v>34.46477823043381</v>
+        <v>36.20183463609141</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1052,7 +1060,7 @@
         <v>0.25811</v>
       </c>
       <c r="Q7" t="n">
-        <v>91.7</v>
+        <v>87.3</v>
       </c>
       <c r="R7" t="n">
         <v>5609.9</v>
@@ -1068,13 +1076,13 @@
         <v>173.6055812119343</v>
       </c>
       <c r="W7" t="n">
-        <v>0.5744129705072301</v>
+        <v>0.6033639106015235</v>
       </c>
       <c r="X7" t="n">
         <v>0.005760183474627001</v>
       </c>
       <c r="Y7" t="n">
-        <v>61.17666303162486</v>
+        <v>64.26002290950744</v>
       </c>
       <c r="Z7" t="n">
         <v>9.389413250773277</v>
@@ -1126,7 +1134,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K8" t="n">
-        <v>57.14872113913986</v>
+        <v>60.09903752682012</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1142,7 +1150,7 @@
         <v>0.126814</v>
       </c>
       <c r="Q8" t="n">
-        <v>55</v>
+        <v>52.3</v>
       </c>
       <c r="R8" t="n">
         <v>2987.7</v>
@@ -1158,13 +1166,13 @@
         <v>303.7663387233741</v>
       </c>
       <c r="W8" t="n">
-        <v>0.9524786856523308</v>
+        <v>1.001650625447002</v>
       </c>
       <c r="X8" t="n">
         <v>0.003292003992946215</v>
       </c>
       <c r="Y8" t="n">
-        <v>54.32181818181818</v>
+        <v>57.12619502868069</v>
       </c>
       <c r="Z8" t="n">
         <v>17.53399863134793</v>
@@ -1216,7 +1224,7 @@
         <v>51.2434931792768</v>
       </c>
       <c r="K9" t="n">
-        <v>173.7067565399213</v>
+        <v>175.6919766146633</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1232,7 +1240,7 @@
         <v>0.01898</v>
       </c>
       <c r="Q9" t="n">
-        <v>17.7</v>
+        <v>17.5</v>
       </c>
       <c r="R9" t="n">
         <v>2234.8</v>
@@ -1248,13 +1256,13 @@
         <v>824.4601019930624</v>
       </c>
       <c r="W9" t="n">
-        <v>2.895112608998689</v>
+        <v>2.928199610244389</v>
       </c>
       <c r="X9" t="n">
         <v>0.001212914970151478</v>
       </c>
       <c r="Y9" t="n">
-        <v>126.2598870056497</v>
+        <v>127.7028571428572</v>
       </c>
       <c r="Z9" t="n">
         <v>22.92978932310578</v>
@@ -1306,7 +1314,7 @@
         <v>50.7771115797629</v>
       </c>
       <c r="K10" t="n">
-        <v>30.61936376669119</v>
+        <v>31.40852262665747</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1330,7 @@
         <v>0.20946</v>
       </c>
       <c r="Q10" t="n">
-        <v>99.5</v>
+        <v>97</v>
       </c>
       <c r="R10" t="n">
         <v>9435.6</v>
@@ -1338,13 +1346,13 @@
         <v>198.7704793771252</v>
       </c>
       <c r="W10" t="n">
-        <v>0.5103227294448532</v>
+        <v>0.5234753771109577</v>
       </c>
       <c r="X10" t="n">
         <v>0.005030928149560429</v>
       </c>
       <c r="Y10" t="n">
-        <v>94.83015075376885</v>
+        <v>97.27422680412371</v>
       </c>
       <c r="Z10" t="n">
         <v>5.381439609538651</v>
@@ -1396,7 +1404,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K11" t="n">
-        <v>29.93297350952396</v>
+        <v>36.38762479594086</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1412,7 +1420,7 @@
         <v>0.07542500000000001</v>
       </c>
       <c r="Q11" t="n">
-        <v>96.40000000000001</v>
+        <v>79.3</v>
       </c>
       <c r="R11" t="n">
         <v>18553.6</v>
@@ -1428,13 +1436,13 @@
         <v>578.4775641354948</v>
       </c>
       <c r="W11" t="n">
-        <v>0.4988828918253994</v>
+        <v>0.606460413265681</v>
       </c>
       <c r="X11" t="n">
         <v>0.001728675513102135</v>
       </c>
       <c r="Y11" t="n">
-        <v>192.4647302904564</v>
+        <v>233.9672131147541</v>
       </c>
       <c r="Z11" t="n">
         <v>2.592074356026243</v>
@@ -1486,7 +1494,7 @@
         <v>47.5276426437724</v>
       </c>
       <c r="K12" t="n">
-        <v>30.11255077746932</v>
+        <v>31.79106531356013</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1502,7 +1510,7 @@
         <v>0.076765</v>
       </c>
       <c r="Q12" t="n">
-        <v>94.7</v>
+        <v>89.7</v>
       </c>
       <c r="R12" t="n">
         <v>8045.8</v>
@@ -1518,13 +1526,13 @@
         <v>554.5362997628245</v>
       </c>
       <c r="W12" t="n">
-        <v>0.5018758462911552</v>
+        <v>0.5298510885593356</v>
       </c>
       <c r="X12" t="n">
         <v>0.001803308458666638</v>
       </c>
       <c r="Y12" t="n">
-        <v>84.96092925026399</v>
+        <v>89.69676700111482</v>
       </c>
       <c r="Z12" t="n">
         <v>5.907136971310796</v>
@@ -1576,7 +1584,7 @@
         <v>46.9727068915036</v>
       </c>
       <c r="K13" t="n">
-        <v>44.59434198560468</v>
+        <v>44.80703360079835</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1592,7 +1600,7 @@
         <v>0.111119</v>
       </c>
       <c r="Q13" t="n">
-        <v>63.2</v>
+        <v>62.9</v>
       </c>
       <c r="R13" t="n">
         <v>5952.7</v>
@@ -1608,13 +1616,13 @@
         <v>370.7747134022449</v>
       </c>
       <c r="W13" t="n">
-        <v>0.7432390330934113</v>
+        <v>0.7467838933466391</v>
       </c>
       <c r="X13" t="n">
         <v>0.002697055553826625</v>
       </c>
       <c r="Y13" t="n">
-        <v>94.1882911392405</v>
+        <v>94.637519872814</v>
       </c>
       <c r="Z13" t="n">
         <v>7.890991800612092</v>
@@ -1666,7 +1674,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K14" t="n">
-        <v>4.091005633901521</v>
+        <v>3.977723433933365</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1690,7 @@
         <v>0.337573</v>
       </c>
       <c r="Q14" t="n">
-        <v>681.2</v>
+        <v>700.6</v>
       </c>
       <c r="R14" t="n">
         <v>57055.2</v>
@@ -1698,13 +1706,13 @@
         <v>132.374251168453</v>
       </c>
       <c r="W14" t="n">
-        <v>0.068183427231692</v>
+        <v>0.0662953905655561</v>
       </c>
       <c r="X14" t="n">
         <v>0.007554339240245816</v>
       </c>
       <c r="Y14" t="n">
-        <v>83.75689958896065</v>
+        <v>81.43762489294889</v>
       </c>
       <c r="Z14" t="n">
         <v>0.814063409298865</v>
@@ -1756,7 +1764,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K15" t="n">
-        <v>5.947897264845492</v>
+        <v>7.353048655720365</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1772,7 +1780,7 @@
         <v>0.0152</v>
       </c>
       <c r="Q15" t="n">
-        <v>467.3</v>
+        <v>378</v>
       </c>
       <c r="R15" t="n">
         <v>20796.5</v>
@@ -1788,13 +1796,13 @@
         <v>2193.173304187023</v>
       </c>
       <c r="W15" t="n">
-        <v>0.09913162108075818</v>
+        <v>0.1225508109286727</v>
       </c>
       <c r="X15" t="n">
         <v>0.0004559603192738502</v>
       </c>
       <c r="Y15" t="n">
-        <v>44.5035309223197</v>
+        <v>55.01719576719577</v>
       </c>
       <c r="Z15" t="n">
         <v>2.227500133726266</v>
@@ -1846,7 +1854,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K16" t="n">
-        <v>5.460746512791836</v>
+        <v>5.131661977181029</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1870,7 @@
         <v>0.141536</v>
       </c>
       <c r="Q16" t="n">
-        <v>499</v>
+        <v>531</v>
       </c>
       <c r="R16" t="n">
         <v>24843.6</v>
@@ -1878,13 +1886,13 @@
         <v>290.2523742749451</v>
       </c>
       <c r="W16" t="n">
-        <v>0.09101244187986393</v>
+        <v>0.0855276996196838</v>
       </c>
       <c r="X16" t="n">
         <v>0.003445277588161046</v>
       </c>
       <c r="Y16" t="n">
-        <v>49.78677354709419</v>
+        <v>46.7864406779661</v>
       </c>
       <c r="Z16" t="n">
         <v>1.828044586857464</v>
@@ -1936,7 +1944,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K17" t="n">
-        <v>7.306618284299266</v>
+        <v>8.553465594195606</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1960,7 @@
         <v>0.148652</v>
       </c>
       <c r="Q17" t="n">
-        <v>367.7</v>
+        <v>314.1</v>
       </c>
       <c r="R17" t="n">
         <v>34728.3</v>
@@ -1968,13 +1976,13 @@
         <v>281.760586368072</v>
       </c>
       <c r="W17" t="n">
-        <v>0.1217769714049878</v>
+        <v>0.1425577599032601</v>
       </c>
       <c r="X17" t="n">
         <v>0.003549112432260739</v>
       </c>
       <c r="Y17" t="n">
-        <v>94.44737557791679</v>
+        <v>110.5644699140401</v>
       </c>
       <c r="Z17" t="n">
         <v>1.289363210569305</v>
@@ -2026,7 +2034,7 @@
         <v>44.3113073012592</v>
       </c>
       <c r="K18" t="n">
-        <v>16.40147093198983</v>
+        <v>17.09761053424792</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2042,7 +2050,7 @@
         <v>0.058096</v>
       </c>
       <c r="Q18" t="n">
-        <v>162.1</v>
+        <v>155.5</v>
       </c>
       <c r="R18" t="n">
         <v>10197.8</v>
@@ -2058,13 +2066,13 @@
         <v>662.6188043195191</v>
       </c>
       <c r="W18" t="n">
-        <v>0.2733578488664972</v>
+        <v>0.2849601755707987</v>
       </c>
       <c r="X18" t="n">
         <v>0.001509163328117374</v>
       </c>
       <c r="Y18" t="n">
-        <v>62.91054904380012</v>
+        <v>65.58070739549839</v>
       </c>
       <c r="Z18" t="n">
         <v>4.345183010184472</v>
@@ -2116,7 +2124,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>13.69550258272278</v>
+        <v>15.12425530172728</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2140,7 @@
         <v>0.039576</v>
       </c>
       <c r="Q19" t="n">
-        <v>191.6</v>
+        <v>173.5</v>
       </c>
       <c r="R19" t="n">
         <v>15469.6</v>
@@ -2148,13 +2156,13 @@
         <v>972.1110696872879</v>
       </c>
       <c r="W19" t="n">
-        <v>0.2282583763787129</v>
+        <v>0.2520709216954548</v>
       </c>
       <c r="X19" t="n">
         <v>0.001028689036862509</v>
       </c>
       <c r="Y19" t="n">
-        <v>80.73903966597078</v>
+        <v>89.16195965417867</v>
       </c>
       <c r="Z19" t="n">
         <v>2.827112848047875</v>
@@ -2205,9 +2213,7 @@
       <c r="J20" t="n">
         <v>43.5938229518782</v>
       </c>
-      <c r="K20" t="n">
-        <v>9.358244640832531</v>
-      </c>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
         <v>0.163338</v>
@@ -2221,9 +2227,7 @@
       <c r="P20" t="n">
         <v>0.148276</v>
       </c>
-      <c r="Q20" t="n">
-        <v>279.5</v>
-      </c>
+      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="n">
         <v>10391.2</v>
       </c>
@@ -2237,15 +2241,11 @@
       <c r="V20" t="n">
         <v>266.8933313244817</v>
       </c>
-      <c r="W20" t="n">
-        <v>0.1559707440138755</v>
-      </c>
+      <c r="W20" t="inlineStr"/>
       <c r="X20" t="n">
         <v>0.0037468152352755</v>
       </c>
-      <c r="Y20" t="n">
-        <v>37.17781753130591</v>
-      </c>
+      <c r="Y20" t="inlineStr"/>
       <c r="Z20" t="n">
         <v>4.195263583789957</v>
       </c>
@@ -2296,7 +2296,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K21" t="n">
-        <v>3.635958786501377</v>
+        <v>4.503497247409874</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.021793</v>
       </c>
       <c r="Q21" t="n">
-        <v>689.9</v>
+        <v>557</v>
       </c>
       <c r="R21" t="n">
         <v>44420.3</v>
@@ -2328,13 +2328,13 @@
         <v>1834.787418303125</v>
       </c>
       <c r="W21" t="n">
-        <v>0.06059931310835628</v>
+        <v>0.07505828745683124</v>
       </c>
       <c r="X21" t="n">
         <v>0.0005450222679883181</v>
       </c>
       <c r="Y21" t="n">
-        <v>64.38657776489347</v>
+        <v>79.74919210053861</v>
       </c>
       <c r="Z21" t="n">
         <v>0.9411792831983349</v>
@@ -2386,7 +2386,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K22" t="n">
-        <v>29.02569657914213</v>
+        <v>31.00472134590182</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.088764</v>
       </c>
       <c r="Q22" t="n">
-        <v>84.59999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="R22" t="n">
         <v>24301.8</v>
@@ -2418,13 +2418,13 @@
         <v>439.4668804599139</v>
       </c>
       <c r="W22" t="n">
-        <v>0.4837616096523689</v>
+        <v>0.5167453557650303</v>
       </c>
       <c r="X22" t="n">
         <v>0.002275484329907804</v>
       </c>
       <c r="Y22" t="n">
-        <v>287.2553191489362</v>
+        <v>306.8409090909091</v>
       </c>
       <c r="Z22" t="n">
         <v>1.684082338616498</v>
@@ -2476,7 +2476,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K23" t="n">
-        <v>30.234611090059</v>
+        <v>30.54671030131122</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2492,7 +2492,7 @@
         <v>0.02621</v>
       </c>
       <c r="Q23" t="n">
-        <v>78.3</v>
+        <v>77.5</v>
       </c>
       <c r="R23" t="n">
         <v>22336.9</v>
@@ -2508,13 +2508,13 @@
         <v>1426.160900474481</v>
       </c>
       <c r="W23" t="n">
-        <v>0.5039101848343167</v>
+        <v>0.5091118383551871</v>
       </c>
       <c r="X23" t="n">
         <v>0.0007011831551876802</v>
       </c>
       <c r="Y23" t="n">
-        <v>285.2733077905492</v>
+        <v>288.2180645161291</v>
       </c>
       <c r="Z23" t="n">
         <v>1.76641196730643</v>
@@ -2656,7 +2656,7 @@
         <v>37.2559686869738</v>
       </c>
       <c r="K25" t="n">
-        <v>22.04495188578331</v>
+        <v>23.62957844839776</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2672,7 +2672,7 @@
         <v>0.007626</v>
       </c>
       <c r="Q25" t="n">
-        <v>101.4</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="R25" t="n">
         <v>15761.3</v>
@@ -2688,13 +2688,13 @@
         <v>4556.747637839262</v>
       </c>
       <c r="W25" t="n">
-        <v>0.3674158647630552</v>
+        <v>0.393826307473296</v>
       </c>
       <c r="X25" t="n">
         <v>0.0002194547689444097</v>
       </c>
       <c r="Y25" t="n">
-        <v>155.4368836291913</v>
+        <v>166.6099365750529</v>
       </c>
       <c r="Z25" t="n">
         <v>2.363762423592839</v>
@@ -2746,7 +2746,7 @@
         <v>33.6962858057476</v>
       </c>
       <c r="K26" t="n">
-        <v>3.91135064489235</v>
+        <v>3.719236843901501</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2762,7 +2762,7 @@
         <v>0.084838</v>
       </c>
       <c r="Q26" t="n">
-        <v>516.9</v>
+        <v>543.6</v>
       </c>
       <c r="R26" t="n">
         <v>29565.5</v>
@@ -2778,13 +2778,13 @@
         <v>372.0058048768779</v>
       </c>
       <c r="W26" t="n">
-        <v>0.06518917741487251</v>
+        <v>0.06198728073169169</v>
       </c>
       <c r="X26" t="n">
         <v>0.002688130096063873</v>
       </c>
       <c r="Y26" t="n">
-        <v>57.19771715999227</v>
+        <v>54.3883370125092</v>
       </c>
       <c r="Z26" t="n">
         <v>1.139716419669804</v>
@@ -2898,7 +2898,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K28" t="n">
-        <v>17.41030380752628</v>
+        <v>14.04821789597673</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2914,7 +2914,7 @@
         <v>0.021244</v>
       </c>
       <c r="Q28" t="n">
-        <v>100.7</v>
+        <v>124.8</v>
       </c>
       <c r="R28" t="n">
         <v>18211.1</v>
@@ -2930,13 +2930,13 @@
         <v>1104.110834068831</v>
       </c>
       <c r="W28" t="n">
-        <v>0.290171730125438</v>
+        <v>0.2341369649329455</v>
       </c>
       <c r="X28" t="n">
         <v>0.0009057061747277989</v>
       </c>
       <c r="Y28" t="n">
-        <v>180.845084409136</v>
+        <v>145.9222756410256</v>
       </c>
       <c r="Z28" t="n">
         <v>1.604532028467891</v>
@@ -2988,7 +2988,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K29" t="n">
-        <v>13.43267801071957</v>
+        <v>13.36084550798845</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -3004,7 +3004,7 @@
         <v>0.09042</v>
       </c>
       <c r="Q29" t="n">
-        <v>111.6</v>
+        <v>112.2</v>
       </c>
       <c r="R29" t="n">
         <v>22793.6</v>
@@ -3020,13 +3020,13 @@
         <v>263.8642816401065</v>
       </c>
       <c r="W29" t="n">
-        <v>0.2238779668453262</v>
+        <v>0.2226807584664741</v>
       </c>
       <c r="X29" t="n">
         <v>0.00378982707998324</v>
       </c>
       <c r="Y29" t="n">
-        <v>204.2437275985663</v>
+        <v>203.1515151515151</v>
       </c>
       <c r="Z29" t="n">
         <v>1.096131418465639</v>
@@ -3078,7 +3078,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K30" t="n">
-        <v>22.04606955989019</v>
+        <v>24.26234110294794</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3094,7 +3094,7 @@
         <v>0.02862</v>
       </c>
       <c r="Q30" t="n">
-        <v>62.4</v>
+        <v>56.7</v>
       </c>
       <c r="R30" t="n">
         <v>12593.6</v>
@@ -3110,13 +3110,13 @@
         <v>694.5957872787968</v>
       </c>
       <c r="W30" t="n">
-        <v>0.3674344926648366</v>
+        <v>0.4043723517157989</v>
       </c>
       <c r="X30" t="n">
         <v>0.001439686243876714</v>
       </c>
       <c r="Y30" t="n">
-        <v>201.8205128205128</v>
+        <v>222.1093474426808</v>
       </c>
       <c r="Z30" t="n">
         <v>1.820600332096128</v>
@@ -3168,7 +3168,7 @@
         <v>22.1685424839812</v>
       </c>
       <c r="K31" t="n">
-        <v>59.91497968643567</v>
+        <v>58.33826969468736</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3184,7 +3184,7 @@
         <v>0.017024</v>
       </c>
       <c r="Q31" t="n">
-        <v>22.2</v>
+        <v>22.8</v>
       </c>
       <c r="R31" t="n">
         <v>7379.9</v>
@@ -3200,13 +3200,13 @@
         <v>1152.690436979056</v>
       </c>
       <c r="W31" t="n">
-        <v>0.9985829947739279</v>
+        <v>0.9723044949114561</v>
       </c>
       <c r="X31" t="n">
         <v>0.0008675356087977764</v>
       </c>
       <c r="Y31" t="n">
-        <v>332.4279279279279</v>
+        <v>323.6798245614035</v>
       </c>
       <c r="Z31" t="n">
         <v>3.003908248618708</v>
@@ -3258,7 +3258,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K32" t="n">
-        <v>15.02184894751848</v>
+        <v>17.2738889050542</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3274,7 +3274,7 @@
         <v>0.009842</v>
       </c>
       <c r="Q32" t="n">
-        <v>69.8</v>
+        <v>60.7</v>
       </c>
       <c r="R32" t="n">
         <v>7737.1</v>
@@ -3290,13 +3290,13 @@
         <v>1572.37876632594</v>
       </c>
       <c r="W32" t="n">
-        <v>0.250364149125308</v>
+        <v>0.28789814841757</v>
       </c>
       <c r="X32" t="n">
         <v>0.0006359790792244194</v>
       </c>
       <c r="Y32" t="n">
-        <v>110.8467048710602</v>
+        <v>127.4645799011532</v>
       </c>
       <c r="Z32" t="n">
         <v>2.258652157649054</v>
@@ -3348,7 +3348,7 @@
         <v>14.1889227802691</v>
       </c>
       <c r="K33" t="n">
-        <v>9.448783205506617</v>
+        <v>10.05118496831341</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -3364,7 +3364,7 @@
         <v>0.047676</v>
       </c>
       <c r="Q33" t="n">
-        <v>90.09999999999999</v>
+        <v>84.7</v>
       </c>
       <c r="R33" t="n">
         <v>14142</v>
@@ -3380,13 +3380,13 @@
         <v>131.1287985903656</v>
       </c>
       <c r="W33" t="n">
-        <v>0.1574797200917769</v>
+        <v>0.1675197494718902</v>
       </c>
       <c r="X33" t="n">
         <v>0.007626089850208333</v>
       </c>
       <c r="Y33" t="n">
-        <v>156.9589345172031</v>
+        <v>166.965761511216</v>
       </c>
       <c r="Z33" t="n">
         <v>1.003317973431558</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-09-29)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>13.77976161266552</v>
+        <v>13.74142364315492</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>0.711927</v>
       </c>
       <c r="Q2" t="n">
-        <v>250.9</v>
+        <v>251.6</v>
       </c>
       <c r="R2" t="n">
         <v>37461.4</v>
@@ -626,13 +626,13 @@
         <v>74.74125673551127</v>
       </c>
       <c r="W2" t="n">
-        <v>0.2296626935444253</v>
+        <v>0.2290237273859153</v>
       </c>
       <c r="X2" t="n">
         <v>0.0133794913770145</v>
       </c>
       <c r="Y2" t="n">
-        <v>149.3080908728577</v>
+        <v>148.8926868044515</v>
       </c>
       <c r="Z2" t="n">
         <v>1.538179828044235</v>
@@ -684,7 +684,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K3" t="n">
-        <v>74.48428015611606</v>
+        <v>68.55593949062927</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>0.09657399999999999</v>
       </c>
       <c r="Q3" t="n">
-        <v>45.1</v>
+        <v>49</v>
       </c>
       <c r="R3" t="n">
         <v>6353.5</v>
@@ -716,13 +716,13 @@
         <v>383.8588628629582</v>
       </c>
       <c r="W3" t="n">
-        <v>1.241404669268601</v>
+        <v>1.142598991510488</v>
       </c>
       <c r="X3" t="n">
         <v>0.002605124166058427</v>
       </c>
       <c r="Y3" t="n">
-        <v>140.8758314855876</v>
+        <v>129.6632653061224</v>
       </c>
       <c r="Z3" t="n">
         <v>8.81204856913731</v>
@@ -731,17 +731,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>claude-opus-5-5-high</t>
+          <t>claude-sonnet-5-5</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (Adaptive Reasoning, High Effort, Default Fallback)</t>
+          <t>Claude Sonnet 5.5 (Adaptive Reasoning, Max Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (high with fallback)</t>
+          <t>Claude Sonnet 5.5 (max with fallback)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -771,67 +771,67 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>53.5831959822067</v>
+        <v>55.9779549012591</v>
       </c>
       <c r="K4" t="n">
-        <v>141.6295929045111</v>
+        <v>11.07377940677727</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
-        <v>0.078086</v>
+        <v>0.696017</v>
       </c>
       <c r="N4" t="n">
-        <v>0.018005</v>
+        <v>0.014944</v>
       </c>
       <c r="O4" t="n">
-        <v>0.027341</v>
+        <v>0.019359</v>
       </c>
       <c r="P4" t="n">
-        <v>0.03274</v>
+        <v>0.661713</v>
       </c>
       <c r="Q4" t="n">
-        <v>22.7</v>
+        <v>303.3</v>
       </c>
       <c r="R4" t="n">
-        <v>3004</v>
+        <v>68107.2</v>
       </c>
       <c r="S4" t="n">
-        <v>1367.1</v>
+        <v>1935.9</v>
       </c>
       <c r="T4" t="n">
-        <v>1637</v>
+        <v>66171.3</v>
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="n">
-        <v>686.2074633379441</v>
+        <v>80.4261316911212</v>
       </c>
       <c r="W4" t="n">
-        <v>2.360493215075185</v>
+        <v>0.1845629901129545</v>
       </c>
       <c r="X4" t="n">
-        <v>0.001457285228487116</v>
+        <v>0.01243376970858835</v>
       </c>
       <c r="Y4" t="n">
-        <v>132.3348017621146</v>
+        <v>224.5539070227497</v>
       </c>
       <c r="Z4" t="n">
-        <v>17.83728228435643</v>
+        <v>0.8219095029785266</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>claude-fable-5-1</t>
+          <t>claude-opus-5-5-high</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (Adaptive Reasoning, Max Effort, Default Fallback)</t>
+          <t>Claude Opus 5.5 (Adaptive Reasoning, High Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (max with fallback)</t>
+          <t>Claude Opus 5.5 (high with fallback)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -861,67 +861,67 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>53.3549259623252</v>
+        <v>53.5831959822067</v>
       </c>
       <c r="K5" t="n">
-        <v>15.02250379042474</v>
+        <v>131.2241534258123</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
-        <v>1.203406</v>
+        <v>0.078086</v>
       </c>
       <c r="N5" t="n">
-        <v>0.051436</v>
+        <v>0.018005</v>
       </c>
       <c r="O5" t="n">
-        <v>0.064901</v>
+        <v>0.027341</v>
       </c>
       <c r="P5" t="n">
-        <v>1.087069</v>
+        <v>0.03274</v>
       </c>
       <c r="Q5" t="n">
-        <v>213.1</v>
+        <v>24.5</v>
       </c>
       <c r="R5" t="n">
-        <v>23039.4</v>
+        <v>3004</v>
       </c>
       <c r="S5" t="n">
-        <v>1298</v>
+        <v>1367.1</v>
       </c>
       <c r="T5" t="n">
-        <v>21741.4</v>
+        <v>1637</v>
       </c>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="n">
-        <v>44.3365962628782</v>
+        <v>686.2074633379441</v>
       </c>
       <c r="W5" t="n">
-        <v>0.2503750631737456</v>
+        <v>2.187069223763539</v>
       </c>
       <c r="X5" t="n">
-        <v>0.022554730951173</v>
+        <v>0.001457285228487116</v>
       </c>
       <c r="Y5" t="n">
-        <v>108.115438761145</v>
+        <v>122.6122448979592</v>
       </c>
       <c r="Z5" t="n">
-        <v>2.315812302504631</v>
+        <v>17.83728228435643</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>claude-fable-5-1-xhigh</t>
+          <t>claude-fable-5-1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (Adaptive Reasoning, Xhigh Effort, Default Fallback)</t>
+          <t>Claude Fable 5.1 (Adaptive Reasoning, Max Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (xhigh with fallback)</t>
+          <t>Claude Fable 5.1 (max with fallback)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -951,82 +951,82 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>53.2032587538944</v>
+        <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>32.08236708777552</v>
+        <v>14.88282453621344</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
-        <v>0.556978</v>
+        <v>1.203406</v>
       </c>
       <c r="N6" t="n">
-        <v>0.048158</v>
+        <v>0.051436</v>
       </c>
       <c r="O6" t="n">
-        <v>0.056185</v>
+        <v>0.064901</v>
       </c>
       <c r="P6" t="n">
-        <v>0.452635</v>
+        <v>1.087069</v>
       </c>
       <c r="Q6" t="n">
-        <v>99.5</v>
+        <v>215.1</v>
       </c>
       <c r="R6" t="n">
-        <v>10176.4</v>
+        <v>23039.4</v>
       </c>
       <c r="S6" t="n">
-        <v>1123.7</v>
+        <v>1298</v>
       </c>
       <c r="T6" t="n">
-        <v>9052.700000000001</v>
+        <v>21741.4</v>
       </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="n">
-        <v>95.52129303831462</v>
+        <v>44.3365962628782</v>
       </c>
       <c r="W6" t="n">
-        <v>0.534706118129592</v>
+        <v>0.2480470756035574</v>
       </c>
       <c r="X6" t="n">
-        <v>0.01046887000994521</v>
+        <v>0.022554730951173</v>
       </c>
       <c r="Y6" t="n">
-        <v>102.2753768844221</v>
+        <v>107.1101813110181</v>
       </c>
       <c r="Z6" t="n">
-        <v>5.228102153403404</v>
+        <v>2.315812302504631</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>gpt-6-astra</t>
+          <t>claude-fable-5-1-xhigh</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (max)</t>
+          <t>Claude Fable 5.1 (Adaptive Reasoning, Xhigh Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (max)</t>
+          <t>Claude Fable 5.1 (xhigh with fallback)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1041,67 +1041,67 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>52.673669395513</v>
+        <v>53.2032587538944</v>
       </c>
       <c r="K7" t="n">
-        <v>36.20183463609141</v>
+        <v>28.65525606134348</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
-        <v>0.30341</v>
+        <v>0.556978</v>
       </c>
       <c r="N7" t="n">
-        <v>0.022917</v>
+        <v>0.048158</v>
       </c>
       <c r="O7" t="n">
-        <v>0.022384</v>
+        <v>0.056185</v>
       </c>
       <c r="P7" t="n">
-        <v>0.25811</v>
+        <v>0.452635</v>
       </c>
       <c r="Q7" t="n">
-        <v>87.3</v>
+        <v>111.4</v>
       </c>
       <c r="R7" t="n">
-        <v>5609.9</v>
+        <v>10176.4</v>
       </c>
       <c r="S7" t="n">
-        <v>447.7</v>
+        <v>1123.7</v>
       </c>
       <c r="T7" t="n">
-        <v>5162.2</v>
+        <v>9052.700000000001</v>
       </c>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="n">
-        <v>173.6055812119343</v>
+        <v>95.52129303831462</v>
       </c>
       <c r="W7" t="n">
-        <v>0.6033639106015235</v>
+        <v>0.4775876010223914</v>
       </c>
       <c r="X7" t="n">
-        <v>0.005760183474627001</v>
+        <v>0.01046887000994521</v>
       </c>
       <c r="Y7" t="n">
-        <v>64.26002290950744</v>
+        <v>91.35008976660681</v>
       </c>
       <c r="Z7" t="n">
-        <v>9.389413250773277</v>
+        <v>5.228102153403404</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>gpt-6-astra-xhigh</t>
+          <t>gpt-6-astra</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (xhigh)</t>
+          <t>GPT-6 Astra (max)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (xhigh)</t>
+          <t>GPT-6 Astra (max)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1131,82 +1131,82 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>52.3863277108782</v>
+        <v>52.673669395513</v>
       </c>
       <c r="K8" t="n">
-        <v>60.09903752682012</v>
+        <v>33.23259898770537</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
-        <v>0.172456</v>
+        <v>0.30341</v>
       </c>
       <c r="N8" t="n">
-        <v>0.023073</v>
+        <v>0.022917</v>
       </c>
       <c r="O8" t="n">
-        <v>0.02257</v>
+        <v>0.022384</v>
       </c>
       <c r="P8" t="n">
-        <v>0.126814</v>
+        <v>0.25811</v>
       </c>
       <c r="Q8" t="n">
-        <v>52.3</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="R8" t="n">
-        <v>2987.7</v>
+        <v>5609.9</v>
       </c>
       <c r="S8" t="n">
-        <v>451.4</v>
+        <v>447.7</v>
       </c>
       <c r="T8" t="n">
-        <v>2536.3</v>
+        <v>5162.2</v>
       </c>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="n">
-        <v>303.7663387233741</v>
+        <v>173.6055812119343</v>
       </c>
       <c r="W8" t="n">
-        <v>1.001650625447002</v>
+        <v>0.5538766497950894</v>
       </c>
       <c r="X8" t="n">
-        <v>0.003292003992946215</v>
+        <v>0.005760183474627001</v>
       </c>
       <c r="Y8" t="n">
-        <v>57.12619502868069</v>
+        <v>58.98948475289169</v>
       </c>
       <c r="Z8" t="n">
-        <v>17.53399863134793</v>
+        <v>9.389413250773277</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>claude-opus-5-5-medium</t>
+          <t>gpt-6-astra-xhigh</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (Adaptive Reasoning, Medium Effort, Default Fallback)</t>
+          <t>GPT-6 Astra (xhigh)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (medium with fallback)</t>
+          <t>GPT-6 Astra (xhigh)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1221,67 +1221,67 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>51.2434931792768</v>
+        <v>52.3863277108782</v>
       </c>
       <c r="K9" t="n">
-        <v>175.6919766146633</v>
+        <v>53.91388786711308</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
-        <v>0.062154</v>
+        <v>0.172456</v>
       </c>
       <c r="N9" t="n">
-        <v>0.017457</v>
+        <v>0.023073</v>
       </c>
       <c r="O9" t="n">
-        <v>0.025716</v>
+        <v>0.02257</v>
       </c>
       <c r="P9" t="n">
-        <v>0.01898</v>
+        <v>0.126814</v>
       </c>
       <c r="Q9" t="n">
-        <v>17.5</v>
+        <v>58.3</v>
       </c>
       <c r="R9" t="n">
-        <v>2234.8</v>
+        <v>2987.7</v>
       </c>
       <c r="S9" t="n">
-        <v>1285.8</v>
+        <v>451.4</v>
       </c>
       <c r="T9" t="n">
-        <v>949</v>
+        <v>2536.3</v>
       </c>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="n">
-        <v>824.4601019930624</v>
+        <v>303.7663387233741</v>
       </c>
       <c r="W9" t="n">
-        <v>2.928199610244389</v>
+        <v>0.8985647977852178</v>
       </c>
       <c r="X9" t="n">
-        <v>0.001212914970151478</v>
+        <v>0.003292003992946215</v>
       </c>
       <c r="Y9" t="n">
-        <v>127.7028571428572</v>
+        <v>51.24699828473413</v>
       </c>
       <c r="Z9" t="n">
-        <v>22.92978932310578</v>
+        <v>17.53399863134793</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>claude-opus-5</t>
+          <t>claude-sonnet-5-5-xhigh</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Claude Opus 5 (Adaptive Reasoning, Max Effort)</t>
+          <t>Claude Sonnet 5.5 (Adaptive Reasoning, Xhigh Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Claude Opus 5 (max)</t>
+          <t>Claude Sonnet 5.5 (xhigh with fallback)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1311,82 +1311,82 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>50.7771115797629</v>
+        <v>51.8522867021152</v>
       </c>
       <c r="K10" t="n">
-        <v>31.40852262665747</v>
+        <v>75.69676890819737</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
-        <v>0.255456</v>
+        <v>0.08497200000000001</v>
       </c>
       <c r="N10" t="n">
-        <v>0.019565</v>
+        <v>0.013004</v>
       </c>
       <c r="O10" t="n">
-        <v>0.02643</v>
+        <v>0.013776</v>
       </c>
       <c r="P10" t="n">
-        <v>0.20946</v>
+        <v>0.058192</v>
       </c>
       <c r="Q10" t="n">
-        <v>97</v>
+        <v>41.1</v>
       </c>
       <c r="R10" t="n">
-        <v>9435.6</v>
+        <v>7196.8</v>
       </c>
       <c r="S10" t="n">
-        <v>1057.2</v>
+        <v>1377.6</v>
       </c>
       <c r="T10" t="n">
-        <v>8378.4</v>
+        <v>5819.2</v>
       </c>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="n">
-        <v>198.7704793771252</v>
+        <v>610.2279186333757</v>
       </c>
       <c r="W10" t="n">
-        <v>0.5234753771109577</v>
+        <v>1.261612815136623</v>
       </c>
       <c r="X10" t="n">
-        <v>0.005030928149560429</v>
+        <v>0.001638731971227293</v>
       </c>
       <c r="Y10" t="n">
-        <v>97.27422680412371</v>
+        <v>175.1046228710462</v>
       </c>
       <c r="Z10" t="n">
-        <v>5.381439609538651</v>
+        <v>7.204908668035126</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>muse-spark-1-3</t>
+          <t>claude-opus-5</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Muse Spark 1.3 (max)</t>
+          <t>Claude Opus 5 (Adaptive Reasoning, Max Effort)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Muse Spark 1.3 (max)</t>
+          <t>Claude Opus 5 (max)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1401,82 +1401,82 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>48.0923107719685</v>
+        <v>50.7771115797629</v>
       </c>
       <c r="K11" t="n">
-        <v>36.38762479594086</v>
+        <v>29.3509315489959</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
-        <v>0.083136</v>
+        <v>0.255456</v>
       </c>
       <c r="N11" t="n">
-        <v>0.004284</v>
+        <v>0.019565</v>
       </c>
       <c r="O11" t="n">
-        <v>0.003428</v>
+        <v>0.02643</v>
       </c>
       <c r="P11" t="n">
-        <v>0.07542500000000001</v>
+        <v>0.20946</v>
       </c>
       <c r="Q11" t="n">
-        <v>79.3</v>
+        <v>103.8</v>
       </c>
       <c r="R11" t="n">
-        <v>18553.6</v>
+        <v>9435.6</v>
       </c>
       <c r="S11" t="n">
-        <v>806.5</v>
+        <v>1057.2</v>
       </c>
       <c r="T11" t="n">
-        <v>17747</v>
+        <v>8378.4</v>
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>578.4775641354948</v>
+        <v>198.7704793771252</v>
       </c>
       <c r="W11" t="n">
-        <v>0.606460413265681</v>
+        <v>0.4891821924832649</v>
       </c>
       <c r="X11" t="n">
-        <v>0.001728675513102135</v>
+        <v>0.005030928149560429</v>
       </c>
       <c r="Y11" t="n">
-        <v>233.9672131147541</v>
+        <v>90.90173410404626</v>
       </c>
       <c r="Z11" t="n">
-        <v>2.592074356026243</v>
+        <v>5.381439609538651</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>gpt-6-sol</t>
+          <t>muse-spark-1-3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>GPT-6 Sol (max)</t>
+          <t>Muse Spark 1.3 (max)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GPT-6 Sol (max)</t>
+          <t>Muse Spark 1.3 (max)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1491,67 +1491,67 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>47.5276426437724</v>
+        <v>48.0923107719685</v>
       </c>
       <c r="K12" t="n">
-        <v>31.79106531356013</v>
+        <v>29.38430393399297</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
-        <v>0.08570700000000001</v>
+        <v>0.083136</v>
       </c>
       <c r="N12" t="n">
-        <v>0.00525</v>
+        <v>0.004284</v>
       </c>
       <c r="O12" t="n">
-        <v>0.003693</v>
+        <v>0.003428</v>
       </c>
       <c r="P12" t="n">
-        <v>0.076765</v>
+        <v>0.07542500000000001</v>
       </c>
       <c r="Q12" t="n">
-        <v>89.7</v>
+        <v>98.2</v>
       </c>
       <c r="R12" t="n">
-        <v>8045.8</v>
+        <v>18553.6</v>
       </c>
       <c r="S12" t="n">
-        <v>369.3</v>
+        <v>806.5</v>
       </c>
       <c r="T12" t="n">
-        <v>7676.5</v>
+        <v>17747</v>
       </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="n">
-        <v>554.5362997628245</v>
+        <v>578.4775641354948</v>
       </c>
       <c r="W12" t="n">
-        <v>0.5298510885593356</v>
+        <v>0.4897383988998829</v>
       </c>
       <c r="X12" t="n">
-        <v>0.001803308458666638</v>
+        <v>0.001728675513102135</v>
       </c>
       <c r="Y12" t="n">
-        <v>89.69676700111482</v>
+        <v>188.9368635437882</v>
       </c>
       <c r="Z12" t="n">
-        <v>5.907136971310796</v>
+        <v>2.592074356026243</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>gpt-5-6-sol</t>
+          <t>gpt-6-sol</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GPT-5.6 Sol (max)</t>
+          <t>GPT-6 Sol (max)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GPT-5.6 Sol (max)</t>
+          <t>GPT-6 Sol (max)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1581,82 +1581,82 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>46.9727068915036</v>
+        <v>47.5276426437724</v>
       </c>
       <c r="K13" t="n">
-        <v>44.80703360079835</v>
+        <v>28.06750549829079</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
-        <v>0.126688</v>
+        <v>0.08570700000000001</v>
       </c>
       <c r="N13" t="n">
-        <v>0.007634</v>
+        <v>0.00525</v>
       </c>
       <c r="O13" t="n">
-        <v>0.007934999999999999</v>
+        <v>0.003693</v>
       </c>
       <c r="P13" t="n">
-        <v>0.111119</v>
+        <v>0.076765</v>
       </c>
       <c r="Q13" t="n">
-        <v>62.9</v>
+        <v>101.6</v>
       </c>
       <c r="R13" t="n">
-        <v>5952.7</v>
+        <v>8045.8</v>
       </c>
       <c r="S13" t="n">
-        <v>396.7</v>
+        <v>369.3</v>
       </c>
       <c r="T13" t="n">
-        <v>5555.9</v>
+        <v>7676.5</v>
       </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="n">
-        <v>370.7747134022449</v>
+        <v>554.5362997628245</v>
       </c>
       <c r="W13" t="n">
-        <v>0.7467838933466391</v>
+        <v>0.4677917583048465</v>
       </c>
       <c r="X13" t="n">
-        <v>0.002697055553826625</v>
+        <v>0.001803308458666638</v>
       </c>
       <c r="Y13" t="n">
-        <v>94.637519872814</v>
+        <v>79.19094488188976</v>
       </c>
       <c r="Z13" t="n">
-        <v>7.890991800612092</v>
+        <v>5.907136971310796</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>grok-4-7</t>
+          <t>gpt-5-6-sol</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Grok 4.7 (xhigh)</t>
+          <t>GPT-5.6 Sol (max)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Grok 4.7 (xhigh)</t>
+          <t>GPT-5.6 Sol (max)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>SpaceXAI</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>xai</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1671,77 +1671,77 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>46.4465506302286</v>
+        <v>46.9727068915036</v>
       </c>
       <c r="K14" t="n">
-        <v>3.977723433933365</v>
+        <v>41.26445700571327</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>0.350873</v>
+        <v>0.126688</v>
       </c>
       <c r="N14" t="n">
-        <v>0.008541999999999999</v>
+        <v>0.007634</v>
       </c>
       <c r="O14" t="n">
-        <v>0.004758</v>
+        <v>0.007934999999999999</v>
       </c>
       <c r="P14" t="n">
-        <v>0.337573</v>
+        <v>0.111119</v>
       </c>
       <c r="Q14" t="n">
-        <v>700.6</v>
+        <v>68.3</v>
       </c>
       <c r="R14" t="n">
-        <v>57055.2</v>
+        <v>5952.7</v>
       </c>
       <c r="S14" t="n">
-        <v>793</v>
+        <v>396.7</v>
       </c>
       <c r="T14" t="n">
-        <v>56262.1</v>
+        <v>5555.9</v>
       </c>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="n">
-        <v>132.374251168453</v>
+        <v>370.7747134022449</v>
       </c>
       <c r="W14" t="n">
-        <v>0.0662953905655561</v>
+        <v>0.6877409500952211</v>
       </c>
       <c r="X14" t="n">
-        <v>0.007554339240245816</v>
+        <v>0.002697055553826625</v>
       </c>
       <c r="Y14" t="n">
-        <v>81.43762489294889</v>
+        <v>87.15519765739386</v>
       </c>
       <c r="Z14" t="n">
-        <v>0.814063409298865</v>
+        <v>7.890991800612092</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>mimo-v2-6-pro</t>
+          <t>grok-4-7</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Grok 4.7 (xhigh)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Grok 4.7 (xhigh)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Xiaomi</t>
+          <t>SpaceXAI</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>xiaomi</t>
+          <t>xai</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1758,85 +1758,85 @@
         <v>1</v>
       </c>
       <c r="I15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>46.3242065310383</v>
+        <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>7.353048655720365</v>
+        <v>3.536988244464673</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>0.021122</v>
+        <v>0.350873</v>
       </c>
       <c r="N15" t="n">
-        <v>0.003029</v>
+        <v>0.008541999999999999</v>
       </c>
       <c r="O15" t="n">
-        <v>0.002893</v>
+        <v>0.004758</v>
       </c>
       <c r="P15" t="n">
-        <v>0.0152</v>
+        <v>0.337573</v>
       </c>
       <c r="Q15" t="n">
-        <v>378</v>
+        <v>787.9</v>
       </c>
       <c r="R15" t="n">
-        <v>20796.5</v>
+        <v>57055.2</v>
       </c>
       <c r="S15" t="n">
-        <v>3325.3</v>
+        <v>793</v>
       </c>
       <c r="T15" t="n">
-        <v>17471.2</v>
+        <v>56262.1</v>
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="n">
-        <v>2193.173304187023</v>
+        <v>132.374251168453</v>
       </c>
       <c r="W15" t="n">
-        <v>0.1225508109286727</v>
+        <v>0.05894980407441122</v>
       </c>
       <c r="X15" t="n">
-        <v>0.0004559603192738502</v>
+        <v>0.007554339240245816</v>
       </c>
       <c r="Y15" t="n">
-        <v>55.01719576719577</v>
+        <v>72.41426576976774</v>
       </c>
       <c r="Z15" t="n">
-        <v>2.227500133726266</v>
+        <v>0.814063409298865</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>qwen3-8-max</t>
+          <t>mimo-v2-6-pro</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>Xiaomi</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>xiaomi</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1848,85 +1848,85 @@
         <v>1</v>
       </c>
       <c r="I16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" t="n">
-        <v>45.4152084980521</v>
+        <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>5.131661977181029</v>
+        <v>5.645850887390409</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
-        <v>0.156468</v>
+        <v>0.021122</v>
       </c>
       <c r="N16" t="n">
-        <v>0.007406</v>
+        <v>0.003029</v>
       </c>
       <c r="O16" t="n">
-        <v>0.007526</v>
+        <v>0.002893</v>
       </c>
       <c r="P16" t="n">
-        <v>0.141536</v>
+        <v>0.0152</v>
       </c>
       <c r="Q16" t="n">
-        <v>531</v>
+        <v>492.3</v>
       </c>
       <c r="R16" t="n">
-        <v>24843.6</v>
+        <v>20796.5</v>
       </c>
       <c r="S16" t="n">
-        <v>1254.3</v>
+        <v>3325.3</v>
       </c>
       <c r="T16" t="n">
-        <v>23589.3</v>
+        <v>17471.2</v>
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="n">
-        <v>290.2523742749451</v>
+        <v>2193.173304187023</v>
       </c>
       <c r="W16" t="n">
-        <v>0.0855276996196838</v>
+        <v>0.09409751478984013</v>
       </c>
       <c r="X16" t="n">
-        <v>0.003445277588161046</v>
+        <v>0.0004559603192738502</v>
       </c>
       <c r="Y16" t="n">
-        <v>46.7864406779661</v>
+        <v>42.24355068047938</v>
       </c>
       <c r="Z16" t="n">
-        <v>1.828044586857464</v>
+        <v>2.227500133726266</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>glm-5-3</t>
+          <t>qwen3-8-max</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1938,85 +1938,85 @@
         <v>1</v>
       </c>
       <c r="I17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>44.777392385614</v>
+        <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>8.553465594195606</v>
+        <v>4.982469390899847</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
-        <v>0.15892</v>
+        <v>0.156468</v>
       </c>
       <c r="N17" t="n">
-        <v>0.006115</v>
+        <v>0.007406</v>
       </c>
       <c r="O17" t="n">
-        <v>0.004153</v>
+        <v>0.007526</v>
       </c>
       <c r="P17" t="n">
-        <v>0.148652</v>
+        <v>0.141536</v>
       </c>
       <c r="Q17" t="n">
-        <v>314.1</v>
+        <v>546.9</v>
       </c>
       <c r="R17" t="n">
-        <v>34728.3</v>
+        <v>24843.6</v>
       </c>
       <c r="S17" t="n">
-        <v>943.8</v>
+        <v>1254.3</v>
       </c>
       <c r="T17" t="n">
-        <v>33784.5</v>
+        <v>23589.3</v>
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="n">
-        <v>281.760586368072</v>
+        <v>290.2523742749451</v>
       </c>
       <c r="W17" t="n">
-        <v>0.1425577599032601</v>
+        <v>0.08304115651499745</v>
       </c>
       <c r="X17" t="n">
-        <v>0.003549112432260739</v>
+        <v>0.003445277588161046</v>
       </c>
       <c r="Y17" t="n">
-        <v>110.5644699140401</v>
+        <v>45.42622051563357</v>
       </c>
       <c r="Z17" t="n">
-        <v>1.289363210569305</v>
+        <v>1.828044586857464</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>grok-4-6</t>
+          <t>glm-5-3</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Grok 4.6 (high)</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Grok 4.6 (high)</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>SpaceXAI</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>xai</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2028,54 +2028,54 @@
         <v>1</v>
       </c>
       <c r="I18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" t="n">
-        <v>44.3113073012592</v>
+        <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>17.09761053424792</v>
+        <v>8.567103135002677</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
-        <v>0.066873</v>
+        <v>0.15892</v>
       </c>
       <c r="N18" t="n">
-        <v>0.005686</v>
+        <v>0.006115</v>
       </c>
       <c r="O18" t="n">
-        <v>0.003091</v>
+        <v>0.004153</v>
       </c>
       <c r="P18" t="n">
-        <v>0.058096</v>
+        <v>0.148652</v>
       </c>
       <c r="Q18" t="n">
-        <v>155.5</v>
+        <v>313.6</v>
       </c>
       <c r="R18" t="n">
-        <v>10197.8</v>
+        <v>34728.3</v>
       </c>
       <c r="S18" t="n">
-        <v>515.2</v>
+        <v>943.8</v>
       </c>
       <c r="T18" t="n">
-        <v>9682.6</v>
+        <v>33784.5</v>
       </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="n">
-        <v>662.6188043195191</v>
+        <v>281.760586368072</v>
       </c>
       <c r="W18" t="n">
-        <v>0.2849601755707987</v>
+        <v>0.1427850522500446</v>
       </c>
       <c r="X18" t="n">
-        <v>0.001509163328117374</v>
+        <v>0.003549112432260739</v>
       </c>
       <c r="Y18" t="n">
-        <v>65.58070739549839</v>
+        <v>110.7407525510204</v>
       </c>
       <c r="Z18" t="n">
-        <v>4.345183010184472</v>
+        <v>1.289363210569305</v>
       </c>
     </row>
     <row r="19">
@@ -2124,7 +2124,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>15.12425530172728</v>
+        <v>16.4106209809236</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2140,7 +2140,7 @@
         <v>0.039576</v>
       </c>
       <c r="Q19" t="n">
-        <v>173.5</v>
+        <v>159.9</v>
       </c>
       <c r="R19" t="n">
         <v>15469.6</v>
@@ -2156,13 +2156,13 @@
         <v>972.1110696872879</v>
       </c>
       <c r="W19" t="n">
-        <v>0.2520709216954548</v>
+        <v>0.27351034968206</v>
       </c>
       <c r="X19" t="n">
         <v>0.001028689036862509</v>
       </c>
       <c r="Y19" t="n">
-        <v>89.16195965417867</v>
+        <v>96.74546591619762</v>
       </c>
       <c r="Z19" t="n">
         <v>2.827112848047875</v>
@@ -2296,7 +2296,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K21" t="n">
-        <v>4.503497247409874</v>
+        <v>3.613957595169716</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.021793</v>
       </c>
       <c r="Q21" t="n">
-        <v>557</v>
+        <v>694.1</v>
       </c>
       <c r="R21" t="n">
         <v>44420.3</v>
@@ -2328,13 +2328,13 @@
         <v>1834.787418303125</v>
       </c>
       <c r="W21" t="n">
-        <v>0.07505828745683124</v>
+        <v>0.06023262658616194</v>
       </c>
       <c r="X21" t="n">
         <v>0.0005450222679883181</v>
       </c>
       <c r="Y21" t="n">
-        <v>79.74919210053861</v>
+        <v>63.99697449935168</v>
       </c>
       <c r="Z21" t="n">
         <v>0.9411792831983349</v>
@@ -2386,7 +2386,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K22" t="n">
-        <v>31.00472134590182</v>
+        <v>24.45790767525323</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.088764</v>
       </c>
       <c r="Q22" t="n">
-        <v>79.2</v>
+        <v>100.4</v>
       </c>
       <c r="R22" t="n">
         <v>24301.8</v>
@@ -2418,13 +2418,13 @@
         <v>439.4668804599139</v>
       </c>
       <c r="W22" t="n">
-        <v>0.5167453557650303</v>
+        <v>0.4076317945875538</v>
       </c>
       <c r="X22" t="n">
         <v>0.002275484329907804</v>
       </c>
       <c r="Y22" t="n">
-        <v>306.8409090909091</v>
+        <v>242.0498007968127</v>
       </c>
       <c r="Z22" t="n">
         <v>1.684082338616498</v>
@@ -2476,7 +2476,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K23" t="n">
-        <v>30.54671030131122</v>
+        <v>29.66629133272707</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2492,7 +2492,7 @@
         <v>0.02621</v>
       </c>
       <c r="Q23" t="n">
-        <v>77.5</v>
+        <v>79.8</v>
       </c>
       <c r="R23" t="n">
         <v>22336.9</v>
@@ -2508,13 +2508,13 @@
         <v>1426.160900474481</v>
       </c>
       <c r="W23" t="n">
-        <v>0.5091118383551871</v>
+        <v>0.4944381888787845</v>
       </c>
       <c r="X23" t="n">
         <v>0.0007011831551876802</v>
       </c>
       <c r="Y23" t="n">
-        <v>288.2180645161291</v>
+        <v>279.9110275689223</v>
       </c>
       <c r="Z23" t="n">
         <v>1.76641196730643</v>
@@ -2656,7 +2656,7 @@
         <v>37.2559686869738</v>
       </c>
       <c r="K25" t="n">
-        <v>23.62957844839776</v>
+        <v>20.43288959066205</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2672,7 +2672,7 @@
         <v>0.007626</v>
       </c>
       <c r="Q25" t="n">
-        <v>94.59999999999999</v>
+        <v>109.4</v>
       </c>
       <c r="R25" t="n">
         <v>15761.3</v>
@@ -2688,13 +2688,13 @@
         <v>4556.747637839262</v>
       </c>
       <c r="W25" t="n">
-        <v>0.393826307473296</v>
+        <v>0.3405481598443675</v>
       </c>
       <c r="X25" t="n">
         <v>0.0002194547689444097</v>
       </c>
       <c r="Y25" t="n">
-        <v>166.6099365750529</v>
+        <v>144.0703839122486</v>
       </c>
       <c r="Z25" t="n">
         <v>2.363762423592839</v>
@@ -2746,7 +2746,7 @@
         <v>33.6962858057476</v>
       </c>
       <c r="K26" t="n">
-        <v>3.719236843901501</v>
+        <v>3.618069342063093</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2762,7 +2762,7 @@
         <v>0.084838</v>
       </c>
       <c r="Q26" t="n">
-        <v>543.6</v>
+        <v>558.8</v>
       </c>
       <c r="R26" t="n">
         <v>29565.5</v>
@@ -2778,13 +2778,13 @@
         <v>372.0058048768779</v>
       </c>
       <c r="W26" t="n">
-        <v>0.06198728073169169</v>
+        <v>0.06030115570105155</v>
       </c>
       <c r="X26" t="n">
         <v>0.002688130096063873</v>
       </c>
       <c r="Y26" t="n">
-        <v>54.3883370125092</v>
+        <v>52.90891195418755</v>
       </c>
       <c r="Z26" t="n">
         <v>1.139716419669804</v>
@@ -2898,7 +2898,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K28" t="n">
-        <v>14.04821789597673</v>
+        <v>10.30092593077495</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2914,7 +2914,7 @@
         <v>0.021244</v>
       </c>
       <c r="Q28" t="n">
-        <v>124.8</v>
+        <v>170.2</v>
       </c>
       <c r="R28" t="n">
         <v>18211.1</v>
@@ -2930,13 +2930,13 @@
         <v>1104.110834068831</v>
       </c>
       <c r="W28" t="n">
-        <v>0.2341369649329455</v>
+        <v>0.1716820988462491</v>
       </c>
       <c r="X28" t="n">
         <v>0.0009057061747277989</v>
       </c>
       <c r="Y28" t="n">
-        <v>145.9222756410256</v>
+        <v>106.9982373678026</v>
       </c>
       <c r="Z28" t="n">
         <v>1.604532028467891</v>
@@ -2988,7 +2988,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K29" t="n">
-        <v>13.36084550798845</v>
+        <v>13.40864817528</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -3004,7 +3004,7 @@
         <v>0.09042</v>
       </c>
       <c r="Q29" t="n">
-        <v>112.2</v>
+        <v>111.8</v>
       </c>
       <c r="R29" t="n">
         <v>22793.6</v>
@@ -3020,13 +3020,13 @@
         <v>263.8642816401065</v>
       </c>
       <c r="W29" t="n">
-        <v>0.2226807584664741</v>
+        <v>0.223477469588</v>
       </c>
       <c r="X29" t="n">
         <v>0.00378982707998324</v>
       </c>
       <c r="Y29" t="n">
-        <v>203.1515151515151</v>
+        <v>203.8783542039356</v>
       </c>
       <c r="Z29" t="n">
         <v>1.096131418465639</v>
@@ -3078,7 +3078,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K30" t="n">
-        <v>24.26234110294794</v>
+        <v>24.13464457082716</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3094,7 +3094,7 @@
         <v>0.02862</v>
       </c>
       <c r="Q30" t="n">
-        <v>56.7</v>
+        <v>57</v>
       </c>
       <c r="R30" t="n">
         <v>12593.6</v>
@@ -3110,13 +3110,13 @@
         <v>694.5957872787968</v>
       </c>
       <c r="W30" t="n">
-        <v>0.4043723517157989</v>
+        <v>0.4022440761804527</v>
       </c>
       <c r="X30" t="n">
         <v>0.001439686243876714</v>
       </c>
       <c r="Y30" t="n">
-        <v>222.1093474426808</v>
+        <v>220.940350877193</v>
       </c>
       <c r="Z30" t="n">
         <v>1.820600332096128</v>
@@ -3168,7 +3168,7 @@
         <v>22.1685424839812</v>
       </c>
       <c r="K31" t="n">
-        <v>58.33826969468736</v>
+        <v>56.36070123046067</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3184,7 +3184,7 @@
         <v>0.017024</v>
       </c>
       <c r="Q31" t="n">
-        <v>22.8</v>
+        <v>23.6</v>
       </c>
       <c r="R31" t="n">
         <v>7379.9</v>
@@ -3200,13 +3200,13 @@
         <v>1152.690436979056</v>
       </c>
       <c r="W31" t="n">
-        <v>0.9723044949114561</v>
+        <v>0.9393450205076779</v>
       </c>
       <c r="X31" t="n">
         <v>0.0008675356087977764</v>
       </c>
       <c r="Y31" t="n">
-        <v>323.6798245614035</v>
+        <v>312.707627118644</v>
       </c>
       <c r="Z31" t="n">
         <v>3.003908248618708</v>
@@ -3258,7 +3258,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K32" t="n">
-        <v>17.2738889050542</v>
+        <v>19.09881705895793</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3274,7 +3274,7 @@
         <v>0.009842</v>
       </c>
       <c r="Q32" t="n">
-        <v>60.7</v>
+        <v>54.9</v>
       </c>
       <c r="R32" t="n">
         <v>7737.1</v>
@@ -3290,13 +3290,13 @@
         <v>1572.37876632594</v>
       </c>
       <c r="W32" t="n">
-        <v>0.28789814841757</v>
+        <v>0.3183136176492987</v>
       </c>
       <c r="X32" t="n">
         <v>0.0006359790792244194</v>
       </c>
       <c r="Y32" t="n">
-        <v>127.4645799011532</v>
+        <v>140.9307832422587</v>
       </c>
       <c r="Z32" t="n">
         <v>2.258652157649054</v>
@@ -3348,7 +3348,7 @@
         <v>14.1889227802691</v>
       </c>
       <c r="K33" t="n">
-        <v>10.05118496831341</v>
+        <v>10.08691192910126</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -3364,7 +3364,7 @@
         <v>0.047676</v>
       </c>
       <c r="Q33" t="n">
-        <v>84.7</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="R33" t="n">
         <v>14142</v>
@@ -3380,13 +3380,13 @@
         <v>131.1287985903656</v>
       </c>
       <c r="W33" t="n">
-        <v>0.1675197494718902</v>
+        <v>0.1681151988183543</v>
       </c>
       <c r="X33" t="n">
         <v>0.007626089850208333</v>
       </c>
       <c r="Y33" t="n">
-        <v>166.965761511216</v>
+        <v>167.5592417061611</v>
       </c>
       <c r="Z33" t="n">
         <v>1.003317973431558</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-09-30)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z33"/>
+  <dimension ref="A1:Z31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>13.74142364315492</v>
+        <v>13.5210879492287</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>0.711927</v>
       </c>
       <c r="Q2" t="n">
-        <v>251.6</v>
+        <v>255.7</v>
       </c>
       <c r="R2" t="n">
         <v>37461.4</v>
@@ -626,13 +626,13 @@
         <v>74.74125673551127</v>
       </c>
       <c r="W2" t="n">
-        <v>0.2290237273859153</v>
+        <v>0.2253514658204783</v>
       </c>
       <c r="X2" t="n">
         <v>0.0133794913770145</v>
       </c>
       <c r="Y2" t="n">
-        <v>148.8926868044515</v>
+        <v>146.50527962456</v>
       </c>
       <c r="Z2" t="n">
         <v>1.538179828044235</v>
@@ -684,7 +684,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K3" t="n">
-        <v>68.55593949062927</v>
+        <v>67.45463925784809</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>0.09657399999999999</v>
       </c>
       <c r="Q3" t="n">
-        <v>49</v>
+        <v>49.8</v>
       </c>
       <c r="R3" t="n">
         <v>6353.5</v>
@@ -716,13 +716,13 @@
         <v>383.8588628629582</v>
       </c>
       <c r="W3" t="n">
-        <v>1.142598991510488</v>
+        <v>1.124243987630801</v>
       </c>
       <c r="X3" t="n">
         <v>0.002605124166058427</v>
       </c>
       <c r="Y3" t="n">
-        <v>129.6632653061224</v>
+        <v>127.5803212851406</v>
       </c>
       <c r="Z3" t="n">
         <v>8.81204856913731</v>
@@ -774,7 +774,7 @@
         <v>55.9779549012591</v>
       </c>
       <c r="K4" t="n">
-        <v>11.07377940677727</v>
+        <v>11.10306543496048</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.661713</v>
       </c>
       <c r="Q4" t="n">
-        <v>303.3</v>
+        <v>302.5</v>
       </c>
       <c r="R4" t="n">
         <v>68107.2</v>
@@ -806,13 +806,13 @@
         <v>80.4261316911212</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1845629901129545</v>
+        <v>0.1850510905826747</v>
       </c>
       <c r="X4" t="n">
         <v>0.01243376970858835</v>
       </c>
       <c r="Y4" t="n">
-        <v>224.5539070227497</v>
+        <v>225.1477685950413</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8219095029785266</v>
@@ -864,7 +864,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K5" t="n">
-        <v>131.2241534258123</v>
+        <v>128.5996703572961</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -880,7 +880,7 @@
         <v>0.03274</v>
       </c>
       <c r="Q5" t="n">
-        <v>24.5</v>
+        <v>25</v>
       </c>
       <c r="R5" t="n">
         <v>3004</v>
@@ -896,13 +896,13 @@
         <v>686.2074633379441</v>
       </c>
       <c r="W5" t="n">
-        <v>2.187069223763539</v>
+        <v>2.143327839288268</v>
       </c>
       <c r="X5" t="n">
         <v>0.001457285228487116</v>
       </c>
       <c r="Y5" t="n">
-        <v>122.6122448979592</v>
+        <v>120.16</v>
       </c>
       <c r="Z5" t="n">
         <v>17.83728228435643</v>
@@ -954,7 +954,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>14.88282453621344</v>
+        <v>15.25879674804343</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -970,7 +970,7 @@
         <v>1.087069</v>
       </c>
       <c r="Q6" t="n">
-        <v>215.1</v>
+        <v>209.8</v>
       </c>
       <c r="R6" t="n">
         <v>23039.4</v>
@@ -986,13 +986,13 @@
         <v>44.3365962628782</v>
       </c>
       <c r="W6" t="n">
-        <v>0.2480470756035574</v>
+        <v>0.2543132791340572</v>
       </c>
       <c r="X6" t="n">
         <v>0.022554730951173</v>
       </c>
       <c r="Y6" t="n">
-        <v>107.1101813110181</v>
+        <v>109.8160152526215</v>
       </c>
       <c r="Z6" t="n">
         <v>2.315812302504631</v>
@@ -1044,7 +1044,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K7" t="n">
-        <v>28.65525606134348</v>
+        <v>30.93212718249675</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1060,7 +1060,7 @@
         <v>0.452635</v>
       </c>
       <c r="Q7" t="n">
-        <v>111.4</v>
+        <v>103.2</v>
       </c>
       <c r="R7" t="n">
         <v>10176.4</v>
@@ -1076,13 +1076,13 @@
         <v>95.52129303831462</v>
       </c>
       <c r="W7" t="n">
-        <v>0.4775876010223914</v>
+        <v>0.5155354530416124</v>
       </c>
       <c r="X7" t="n">
         <v>0.01046887000994521</v>
       </c>
       <c r="Y7" t="n">
-        <v>91.35008976660681</v>
+        <v>98.60852713178294</v>
       </c>
       <c r="Z7" t="n">
         <v>5.228102153403404</v>
@@ -1134,7 +1134,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K8" t="n">
-        <v>33.23259898770537</v>
+        <v>29.10147480415083</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1150,7 +1150,7 @@
         <v>0.25811</v>
       </c>
       <c r="Q8" t="n">
-        <v>95.09999999999999</v>
+        <v>108.6</v>
       </c>
       <c r="R8" t="n">
         <v>5609.9</v>
@@ -1166,13 +1166,13 @@
         <v>173.6055812119343</v>
       </c>
       <c r="W8" t="n">
-        <v>0.5538766497950894</v>
+        <v>0.4850245800691805</v>
       </c>
       <c r="X8" t="n">
         <v>0.005760183474627001</v>
       </c>
       <c r="Y8" t="n">
-        <v>58.98948475289169</v>
+        <v>51.65653775322284</v>
       </c>
       <c r="Z8" t="n">
         <v>9.389413250773277</v>
@@ -1224,7 +1224,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K9" t="n">
-        <v>53.91388786711308</v>
+        <v>51.1918511832686</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1240,7 +1240,7 @@
         <v>0.126814</v>
       </c>
       <c r="Q9" t="n">
-        <v>58.3</v>
+        <v>61.4</v>
       </c>
       <c r="R9" t="n">
         <v>2987.7</v>
@@ -1256,13 +1256,13 @@
         <v>303.7663387233741</v>
       </c>
       <c r="W9" t="n">
-        <v>0.8985647977852178</v>
+        <v>0.8531975197211433</v>
       </c>
       <c r="X9" t="n">
         <v>0.003292003992946215</v>
       </c>
       <c r="Y9" t="n">
-        <v>51.24699828473413</v>
+        <v>48.65960912052117</v>
       </c>
       <c r="Z9" t="n">
         <v>17.53399863134793</v>
@@ -1314,7 +1314,7 @@
         <v>51.8522867021152</v>
       </c>
       <c r="K10" t="n">
-        <v>75.69676890819737</v>
+        <v>73.54934283987973</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1330,7 +1330,7 @@
         <v>0.058192</v>
       </c>
       <c r="Q10" t="n">
-        <v>41.1</v>
+        <v>42.3</v>
       </c>
       <c r="R10" t="n">
         <v>7196.8</v>
@@ -1346,13 +1346,13 @@
         <v>610.2279186333757</v>
       </c>
       <c r="W10" t="n">
-        <v>1.261612815136623</v>
+        <v>1.225822380664662</v>
       </c>
       <c r="X10" t="n">
         <v>0.001638731971227293</v>
       </c>
       <c r="Y10" t="n">
-        <v>175.1046228710462</v>
+        <v>170.1371158392435</v>
       </c>
       <c r="Z10" t="n">
         <v>7.204908668035126</v>
@@ -1361,32 +1361,32 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>claude-opus-5</t>
+          <t>gpt-6-1-sol</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Claude Opus 5 (Adaptive Reasoning, Max Effort)</t>
+          <t>GPT-6.1 Sol (max)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Claude Opus 5 (max)</t>
+          <t>GPT-6.1 Sol (max)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1401,51 +1401,51 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>50.7771115797629</v>
+        <v>51.8332597011541</v>
       </c>
       <c r="K11" t="n">
-        <v>29.3509315489959</v>
+        <v>30.22347504440472</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
-        <v>0.255456</v>
+        <v>0.074921</v>
       </c>
       <c r="N11" t="n">
-        <v>0.019565</v>
+        <v>0.006023</v>
       </c>
       <c r="O11" t="n">
-        <v>0.02643</v>
+        <v>0.005667</v>
       </c>
       <c r="P11" t="n">
-        <v>0.20946</v>
+        <v>0.06322999999999999</v>
       </c>
       <c r="Q11" t="n">
-        <v>103.8</v>
+        <v>102.9</v>
       </c>
       <c r="R11" t="n">
-        <v>9435.6</v>
+        <v>6889.8</v>
       </c>
       <c r="S11" t="n">
-        <v>1057.2</v>
+        <v>566.7</v>
       </c>
       <c r="T11" t="n">
-        <v>8378.4</v>
+        <v>6323</v>
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>198.7704793771252</v>
+        <v>691.8388662878779</v>
       </c>
       <c r="W11" t="n">
-        <v>0.4891821924832649</v>
+        <v>0.503724584073412</v>
       </c>
       <c r="X11" t="n">
-        <v>0.005030928149560429</v>
+        <v>0.001445423275170399</v>
       </c>
       <c r="Y11" t="n">
-        <v>90.90173410404626</v>
+        <v>66.95626822157435</v>
       </c>
       <c r="Z11" t="n">
-        <v>5.381439609538651</v>
+        <v>7.523187857579915</v>
       </c>
     </row>
     <row r="12">
@@ -1494,7 +1494,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K12" t="n">
-        <v>29.38430393399297</v>
+        <v>27.3251765749821</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1510,7 +1510,7 @@
         <v>0.07542500000000001</v>
       </c>
       <c r="Q12" t="n">
-        <v>98.2</v>
+        <v>105.6</v>
       </c>
       <c r="R12" t="n">
         <v>18553.6</v>
@@ -1526,13 +1526,13 @@
         <v>578.4775641354948</v>
       </c>
       <c r="W12" t="n">
-        <v>0.4897383988998829</v>
+        <v>0.4554196095830351</v>
       </c>
       <c r="X12" t="n">
         <v>0.001728675513102135</v>
       </c>
       <c r="Y12" t="n">
-        <v>188.9368635437882</v>
+        <v>175.6969696969697</v>
       </c>
       <c r="Z12" t="n">
         <v>2.592074356026243</v>
@@ -1584,7 +1584,7 @@
         <v>47.5276426437724</v>
       </c>
       <c r="K13" t="n">
-        <v>28.06750549829079</v>
+        <v>26.97879431056144</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1600,7 +1600,7 @@
         <v>0.076765</v>
       </c>
       <c r="Q13" t="n">
-        <v>101.6</v>
+        <v>105.7</v>
       </c>
       <c r="R13" t="n">
         <v>8045.8</v>
@@ -1616,13 +1616,13 @@
         <v>554.5362997628245</v>
       </c>
       <c r="W13" t="n">
-        <v>0.4677917583048465</v>
+        <v>0.4496465718426906</v>
       </c>
       <c r="X13" t="n">
         <v>0.001803308458666638</v>
       </c>
       <c r="Y13" t="n">
-        <v>79.19094488188976</v>
+        <v>76.11920529801324</v>
       </c>
       <c r="Z13" t="n">
         <v>5.907136971310796</v>
@@ -1631,32 +1631,32 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>gpt-5-6-sol</t>
+          <t>grok-4-7</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>GPT-5.6 Sol (max)</t>
+          <t>Grok 4.7 (xhigh)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GPT-5.6 Sol (max)</t>
+          <t>Grok 4.7 (xhigh)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>SpaceXAI</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>xai</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1671,77 +1671,77 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>46.9727068915036</v>
+        <v>46.4465506302286</v>
       </c>
       <c r="K14" t="n">
-        <v>41.26445700571327</v>
+        <v>3.467885811117118</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>0.126688</v>
+        <v>0.350873</v>
       </c>
       <c r="N14" t="n">
-        <v>0.007634</v>
+        <v>0.008541999999999999</v>
       </c>
       <c r="O14" t="n">
-        <v>0.007934999999999999</v>
+        <v>0.004758</v>
       </c>
       <c r="P14" t="n">
-        <v>0.111119</v>
+        <v>0.337573</v>
       </c>
       <c r="Q14" t="n">
-        <v>68.3</v>
+        <v>803.6</v>
       </c>
       <c r="R14" t="n">
-        <v>5952.7</v>
+        <v>57055.2</v>
       </c>
       <c r="S14" t="n">
-        <v>396.7</v>
+        <v>793</v>
       </c>
       <c r="T14" t="n">
-        <v>5555.9</v>
+        <v>56262.1</v>
       </c>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="n">
-        <v>370.7747134022449</v>
+        <v>132.374251168453</v>
       </c>
       <c r="W14" t="n">
-        <v>0.6877409500952211</v>
+        <v>0.05779809685195197</v>
       </c>
       <c r="X14" t="n">
-        <v>0.002697055553826625</v>
+        <v>0.007554339240245816</v>
       </c>
       <c r="Y14" t="n">
-        <v>87.15519765739386</v>
+        <v>70.99950223992035</v>
       </c>
       <c r="Z14" t="n">
-        <v>7.890991800612092</v>
+        <v>0.814063409298865</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>grok-4-7</t>
+          <t>mimo-v2-6-pro</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Grok 4.7 (xhigh)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Grok 4.7 (xhigh)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>SpaceXAI</t>
+          <t>Xiaomi</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>xai</t>
+          <t>xiaomi</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1758,85 +1758,85 @@
         <v>1</v>
       </c>
       <c r="I15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" t="n">
-        <v>46.4465506302286</v>
+        <v>46.3242065310383</v>
       </c>
       <c r="K15" t="n">
-        <v>3.536988244464673</v>
+        <v>5.645850887390409</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>0.350873</v>
+        <v>0.021122</v>
       </c>
       <c r="N15" t="n">
-        <v>0.008541999999999999</v>
+        <v>0.003029</v>
       </c>
       <c r="O15" t="n">
-        <v>0.004758</v>
+        <v>0.002893</v>
       </c>
       <c r="P15" t="n">
-        <v>0.337573</v>
+        <v>0.0152</v>
       </c>
       <c r="Q15" t="n">
-        <v>787.9</v>
+        <v>492.3</v>
       </c>
       <c r="R15" t="n">
-        <v>57055.2</v>
+        <v>20796.5</v>
       </c>
       <c r="S15" t="n">
-        <v>793</v>
+        <v>3325.3</v>
       </c>
       <c r="T15" t="n">
-        <v>56262.1</v>
+        <v>17471.2</v>
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="n">
-        <v>132.374251168453</v>
+        <v>2193.173304187023</v>
       </c>
       <c r="W15" t="n">
-        <v>0.05894980407441122</v>
+        <v>0.09409751478984013</v>
       </c>
       <c r="X15" t="n">
-        <v>0.007554339240245816</v>
+        <v>0.0004559603192738502</v>
       </c>
       <c r="Y15" t="n">
-        <v>72.41426576976774</v>
+        <v>42.24355068047938</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.814063409298865</v>
+        <v>2.227500133726266</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>mimo-v2-6-pro</t>
+          <t>qwen3-8-max</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Xiaomi</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>xiaomi</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1848,85 +1848,85 @@
         <v>1</v>
       </c>
       <c r="I16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>46.3242065310383</v>
+        <v>45.4152084980521</v>
       </c>
       <c r="K16" t="n">
-        <v>5.645850887390409</v>
+        <v>5.31068507090845</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
-        <v>0.021122</v>
+        <v>0.156468</v>
       </c>
       <c r="N16" t="n">
-        <v>0.003029</v>
+        <v>0.007406</v>
       </c>
       <c r="O16" t="n">
-        <v>0.002893</v>
+        <v>0.007526</v>
       </c>
       <c r="P16" t="n">
-        <v>0.0152</v>
+        <v>0.141536</v>
       </c>
       <c r="Q16" t="n">
-        <v>492.3</v>
+        <v>513.1</v>
       </c>
       <c r="R16" t="n">
-        <v>20796.5</v>
+        <v>24843.6</v>
       </c>
       <c r="S16" t="n">
-        <v>3325.3</v>
+        <v>1254.3</v>
       </c>
       <c r="T16" t="n">
-        <v>17471.2</v>
+        <v>23589.3</v>
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="n">
-        <v>2193.173304187023</v>
+        <v>290.2523742749451</v>
       </c>
       <c r="W16" t="n">
-        <v>0.09409751478984013</v>
+        <v>0.08851141784847417</v>
       </c>
       <c r="X16" t="n">
-        <v>0.0004559603192738502</v>
+        <v>0.003445277588161046</v>
       </c>
       <c r="Y16" t="n">
-        <v>42.24355068047938</v>
+        <v>48.41863184564412</v>
       </c>
       <c r="Z16" t="n">
-        <v>2.227500133726266</v>
+        <v>1.828044586857464</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>qwen3-8-max</t>
+          <t>glm-5-3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1938,85 +1938,85 @@
         <v>1</v>
       </c>
       <c r="I17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17" t="n">
-        <v>45.4152084980521</v>
+        <v>44.777392385614</v>
       </c>
       <c r="K17" t="n">
-        <v>4.982469390899847</v>
+        <v>7.47327828410804</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
-        <v>0.156468</v>
+        <v>0.15892</v>
       </c>
       <c r="N17" t="n">
-        <v>0.007406</v>
+        <v>0.006115</v>
       </c>
       <c r="O17" t="n">
-        <v>0.007526</v>
+        <v>0.004153</v>
       </c>
       <c r="P17" t="n">
-        <v>0.141536</v>
+        <v>0.148652</v>
       </c>
       <c r="Q17" t="n">
-        <v>546.9</v>
+        <v>359.5</v>
       </c>
       <c r="R17" t="n">
-        <v>24843.6</v>
+        <v>34728.3</v>
       </c>
       <c r="S17" t="n">
-        <v>1254.3</v>
+        <v>943.8</v>
       </c>
       <c r="T17" t="n">
-        <v>23589.3</v>
+        <v>33784.5</v>
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="n">
-        <v>290.2523742749451</v>
+        <v>281.760586368072</v>
       </c>
       <c r="W17" t="n">
-        <v>0.08304115651499745</v>
+        <v>0.1245546380684673</v>
       </c>
       <c r="X17" t="n">
-        <v>0.003445277588161046</v>
+        <v>0.003549112432260739</v>
       </c>
       <c r="Y17" t="n">
-        <v>45.42622051563357</v>
+        <v>96.60166898470098</v>
       </c>
       <c r="Z17" t="n">
-        <v>1.828044586857464</v>
+        <v>1.289363210569305</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>glm-5-3</t>
+          <t>step-5</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>StepFun</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>stepfun</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2028,85 +2028,85 @@
         <v>1</v>
       </c>
       <c r="I18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>44.777392385614</v>
+        <v>43.7343049141614</v>
       </c>
       <c r="K18" t="n">
-        <v>8.567103135002677</v>
+        <v>16.4106209809236</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
-        <v>0.15892</v>
+        <v>0.044989</v>
       </c>
       <c r="N18" t="n">
-        <v>0.006115</v>
+        <v>0.003221</v>
       </c>
       <c r="O18" t="n">
-        <v>0.004153</v>
+        <v>0.002192</v>
       </c>
       <c r="P18" t="n">
-        <v>0.148652</v>
+        <v>0.039576</v>
       </c>
       <c r="Q18" t="n">
-        <v>313.6</v>
+        <v>159.9</v>
       </c>
       <c r="R18" t="n">
-        <v>34728.3</v>
+        <v>15469.6</v>
       </c>
       <c r="S18" t="n">
-        <v>943.8</v>
+        <v>811.7</v>
       </c>
       <c r="T18" t="n">
-        <v>33784.5</v>
+        <v>14657.8</v>
       </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="n">
-        <v>281.760586368072</v>
+        <v>972.1110696872879</v>
       </c>
       <c r="W18" t="n">
-        <v>0.1427850522500446</v>
+        <v>0.27351034968206</v>
       </c>
       <c r="X18" t="n">
-        <v>0.003549112432260739</v>
+        <v>0.001028689036862509</v>
       </c>
       <c r="Y18" t="n">
-        <v>110.7407525510204</v>
+        <v>96.74546591619762</v>
       </c>
       <c r="Z18" t="n">
-        <v>1.289363210569305</v>
+        <v>2.827112848047875</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>step-5</t>
+          <t>kimi-k3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>Kimi K3 (max)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>Kimi K3 (max)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>StepFun</t>
+          <t>Kimi</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>stepfun</t>
+          <t>kimi</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2118,85 +2118,85 @@
         <v>1</v>
       </c>
       <c r="I19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>43.7343049141614</v>
+        <v>43.5938229518782</v>
       </c>
       <c r="K19" t="n">
-        <v>16.4106209809236</v>
+        <v>10.64995674720152</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
-        <v>0.044989</v>
+        <v>0.163338</v>
       </c>
       <c r="N19" t="n">
-        <v>0.003221</v>
+        <v>0.007471</v>
       </c>
       <c r="O19" t="n">
-        <v>0.002192</v>
+        <v>0.007591</v>
       </c>
       <c r="P19" t="n">
-        <v>0.039576</v>
+        <v>0.148276</v>
       </c>
       <c r="Q19" t="n">
-        <v>159.9</v>
+        <v>245.6</v>
       </c>
       <c r="R19" t="n">
-        <v>15469.6</v>
+        <v>10391.2</v>
       </c>
       <c r="S19" t="n">
-        <v>811.7</v>
+        <v>506.1</v>
       </c>
       <c r="T19" t="n">
-        <v>14657.8</v>
+        <v>9885.1</v>
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="n">
-        <v>972.1110696872879</v>
+        <v>266.8933313244817</v>
       </c>
       <c r="W19" t="n">
-        <v>0.27351034968206</v>
+        <v>0.1774992791200252</v>
       </c>
       <c r="X19" t="n">
-        <v>0.001028689036862509</v>
+        <v>0.0037468152352755</v>
       </c>
       <c r="Y19" t="n">
-        <v>96.74546591619762</v>
+        <v>42.30944625407167</v>
       </c>
       <c r="Z19" t="n">
-        <v>2.827112848047875</v>
+        <v>4.195263583789957</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>kimi-k3</t>
+          <t>glm-5-3-flash</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Kimi K3 (max)</t>
+          <t>GLM 5.3 Flash</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Kimi K3 (max)</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Kimi</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>kimi</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2211,74 +2211,82 @@
         <v>1</v>
       </c>
       <c r="J20" t="n">
-        <v>43.5938229518782</v>
-      </c>
-      <c r="K20" t="inlineStr"/>
+        <v>41.807466113455</v>
+      </c>
+      <c r="K20" t="n">
+        <v>3.483955509454583</v>
+      </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
-        <v>0.163338</v>
+        <v>0.022786</v>
       </c>
       <c r="N20" t="n">
-        <v>0.007471</v>
+        <v>0.000576</v>
       </c>
       <c r="O20" t="n">
-        <v>0.007591</v>
+        <v>0.000417</v>
       </c>
       <c r="P20" t="n">
-        <v>0.148276</v>
-      </c>
-      <c r="Q20" t="inlineStr"/>
+        <v>0.021793</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>720</v>
+      </c>
       <c r="R20" t="n">
-        <v>10391.2</v>
+        <v>44420.3</v>
       </c>
       <c r="S20" t="n">
-        <v>506.1</v>
+        <v>834.1</v>
       </c>
       <c r="T20" t="n">
-        <v>9885.1</v>
+        <v>43586.3</v>
       </c>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="n">
-        <v>266.8933313244817</v>
-      </c>
-      <c r="W20" t="inlineStr"/>
+        <v>1834.787418303125</v>
+      </c>
+      <c r="W20" t="n">
+        <v>0.05806592515757639</v>
+      </c>
       <c r="X20" t="n">
-        <v>0.0037468152352755</v>
-      </c>
-      <c r="Y20" t="inlineStr"/>
+        <v>0.0005450222679883181</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>61.69486111111112</v>
+      </c>
       <c r="Z20" t="n">
-        <v>4.195263583789957</v>
+        <v>0.9411792831983349</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>glm-5-3-flash</t>
+          <t>gemini-3-8-flash</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>GLM 5.3 Flash</t>
+          <t>Gemini 3.8 Flash (high)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Gemini 3.8 Flash (high)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2290,85 +2298,85 @@
         <v>1</v>
       </c>
       <c r="I21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>41.807466113455</v>
+        <v>40.9262321765904</v>
       </c>
       <c r="K21" t="n">
-        <v>3.613957595169716</v>
+        <v>24.45790767525323</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
-        <v>0.022786</v>
+        <v>0.093127</v>
       </c>
       <c r="N21" t="n">
-        <v>0.000576</v>
+        <v>0.001995</v>
       </c>
       <c r="O21" t="n">
-        <v>0.000417</v>
+        <v>0.002368</v>
       </c>
       <c r="P21" t="n">
-        <v>0.021793</v>
+        <v>0.088764</v>
       </c>
       <c r="Q21" t="n">
-        <v>694.1</v>
+        <v>100.4</v>
       </c>
       <c r="R21" t="n">
-        <v>44420.3</v>
+        <v>24301.8</v>
       </c>
       <c r="S21" t="n">
-        <v>834.1</v>
+        <v>631.5</v>
       </c>
       <c r="T21" t="n">
-        <v>43586.3</v>
+        <v>23670.3</v>
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="n">
-        <v>1834.787418303125</v>
+        <v>439.4668804599139</v>
       </c>
       <c r="W21" t="n">
-        <v>0.06023262658616194</v>
+        <v>0.4076317945875538</v>
       </c>
       <c r="X21" t="n">
-        <v>0.0005450222679883181</v>
+        <v>0.002275484329907804</v>
       </c>
       <c r="Y21" t="n">
-        <v>63.99697449935168</v>
+        <v>242.0498007968127</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.9411792831983349</v>
+        <v>1.684082338616498</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>gemini-3-8-flash</t>
+          <t>deepseek-v4-1-flash</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>DeepSeek V4.1 Flash (Reasoning, Max Effort)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>DeepSeek V4.1 Flash (max)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>DeepSeek</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>deepseek</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2380,360 +2388,332 @@
         <v>1</v>
       </c>
       <c r="I22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>40.9262321765904</v>
+        <v>39.456167472527</v>
       </c>
       <c r="K22" t="n">
-        <v>24.45790767525323</v>
+        <v>29.44490109890074</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
-        <v>0.093127</v>
+        <v>0.027666</v>
       </c>
       <c r="N22" t="n">
-        <v>0.001995</v>
+        <v>0.000862</v>
       </c>
       <c r="O22" t="n">
-        <v>0.002368</v>
+        <v>0.000595</v>
       </c>
       <c r="P22" t="n">
-        <v>0.088764</v>
+        <v>0.02621</v>
       </c>
       <c r="Q22" t="n">
-        <v>100.4</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="R22" t="n">
-        <v>24301.8</v>
+        <v>22336.9</v>
       </c>
       <c r="S22" t="n">
-        <v>631.5</v>
+        <v>495.4</v>
       </c>
       <c r="T22" t="n">
-        <v>23670.3</v>
+        <v>21841.5</v>
       </c>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="n">
-        <v>439.4668804599139</v>
+        <v>1426.160900474481</v>
       </c>
       <c r="W22" t="n">
-        <v>0.4076317945875538</v>
+        <v>0.4907483516483457</v>
       </c>
       <c r="X22" t="n">
-        <v>0.002275484329907804</v>
+        <v>0.0007011831551876802</v>
       </c>
       <c r="Y22" t="n">
-        <v>242.0498007968127</v>
+        <v>277.8221393034826</v>
       </c>
       <c r="Z22" t="n">
-        <v>1.684082338616498</v>
+        <v>1.76641196730643</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>deepseek-v4-1-flash</t>
+          <t>gpt-6-luna</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (Reasoning, Max Effort)</t>
+          <t>GPT-6 Luna (max)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (max)</t>
+          <t>GPT-6 Luna (max)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>DeepSeek</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>deepseek</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H23" t="b">
         <v>1</v>
       </c>
       <c r="I23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>39.456167472527</v>
+        <v>37.2559686869738</v>
       </c>
       <c r="K23" t="n">
-        <v>29.66629133272707</v>
+        <v>19.17116742039818</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
-        <v>0.027666</v>
+        <v>0.008175999999999999</v>
       </c>
       <c r="N23" t="n">
-        <v>0.000862</v>
+        <v>0.000295</v>
       </c>
       <c r="O23" t="n">
-        <v>0.000595</v>
+        <v>0.000254</v>
       </c>
       <c r="P23" t="n">
-        <v>0.02621</v>
+        <v>0.007626</v>
       </c>
       <c r="Q23" t="n">
-        <v>79.8</v>
+        <v>116.6</v>
       </c>
       <c r="R23" t="n">
-        <v>22336.9</v>
+        <v>15761.3</v>
       </c>
       <c r="S23" t="n">
-        <v>495.4</v>
+        <v>508.9</v>
       </c>
       <c r="T23" t="n">
-        <v>21841.5</v>
+        <v>15252.5</v>
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="n">
-        <v>1426.160900474481</v>
+        <v>4556.747637839262</v>
       </c>
       <c r="W23" t="n">
-        <v>0.4944381888787845</v>
+        <v>0.3195194570066364</v>
       </c>
       <c r="X23" t="n">
-        <v>0.0007011831551876802</v>
+        <v>0.0002194547689444097</v>
       </c>
       <c r="Y23" t="n">
-        <v>279.9110275689223</v>
+        <v>135.1740994854202</v>
       </c>
       <c r="Z23" t="n">
-        <v>1.76641196730643</v>
+        <v>2.363762423592839</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>gpt-5-6-luna</t>
+          <t>qwen3-8-27b</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GPT-5.6 Luna (max)</t>
+          <t>Qwen3.8 27B (xhigh)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GPT-5.6 Luna (max)</t>
+          <t>Qwen3.8 27B (xhigh)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H24" t="b">
         <v>1</v>
       </c>
       <c r="I24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>37.3244239690841</v>
+        <v>33.6962858057476</v>
       </c>
       <c r="K24" t="n">
-        <v>21.368945020468</v>
+        <v>3.68131308875611</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>0.016448</v>
+        <v>0.09057999999999999</v>
       </c>
       <c r="N24" t="n">
-        <v>0.000637</v>
+        <v>0.001883</v>
       </c>
       <c r="O24" t="n">
-        <v>0.000541</v>
+        <v>0.003858</v>
       </c>
       <c r="P24" t="n">
-        <v>0.015269</v>
+        <v>0.084838</v>
       </c>
       <c r="Q24" t="n">
-        <v>104.8</v>
+        <v>549.2</v>
       </c>
       <c r="R24" t="n">
-        <v>13175.4</v>
+        <v>29565.5</v>
       </c>
       <c r="S24" t="n">
-        <v>451.2</v>
+        <v>1286.1</v>
       </c>
       <c r="T24" t="n">
-        <v>12724.3</v>
+        <v>28279.4</v>
       </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="n">
-        <v>2269.237838587312</v>
+        <v>372.0058048768779</v>
       </c>
       <c r="W24" t="n">
-        <v>0.3561490836744666</v>
+        <v>0.06135521814593517</v>
       </c>
       <c r="X24" t="n">
-        <v>0.0004406765932576458</v>
+        <v>0.002688130096063873</v>
       </c>
       <c r="Y24" t="n">
-        <v>125.719465648855</v>
+        <v>53.83375819373634</v>
       </c>
       <c r="Z24" t="n">
-        <v>2.832887348322184</v>
+        <v>1.139716419669804</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>gpt-6-luna</t>
+          <t>k2-horizon-375b-a23b</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (max)</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (max)</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Institute of Foundation Models</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>ifm</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H25" t="b">
         <v>1</v>
       </c>
       <c r="I25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>37.2559686869738</v>
-      </c>
-      <c r="K25" t="n">
-        <v>20.43288959066205</v>
-      </c>
+        <v>30.5015302696723</v>
+      </c>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
-      <c r="M25" t="n">
-        <v>0.008175999999999999</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0.000295</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0.000254</v>
-      </c>
-      <c r="P25" t="n">
-        <v>0.007626</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>109.4</v>
-      </c>
-      <c r="R25" t="n">
-        <v>15761.3</v>
-      </c>
-      <c r="S25" t="n">
-        <v>508.9</v>
-      </c>
-      <c r="T25" t="n">
-        <v>15252.5</v>
-      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
-      <c r="V25" t="n">
-        <v>4556.747637839262</v>
-      </c>
-      <c r="W25" t="n">
-        <v>0.3405481598443675</v>
-      </c>
-      <c r="X25" t="n">
-        <v>0.0002194547689444097</v>
-      </c>
-      <c r="Y25" t="n">
-        <v>144.0703839122486</v>
-      </c>
-      <c r="Z25" t="n">
-        <v>2.363762423592839</v>
-      </c>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>qwen3-8-27b</t>
+          <t>minimax-m3</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (xhigh)</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (xhigh)</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>minimax</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H26" t="b">
@@ -2743,82 +2723,82 @@
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>33.6962858057476</v>
+        <v>29.2202932236316</v>
       </c>
       <c r="K26" t="n">
-        <v>3.618069342063093</v>
+        <v>10.02411431342422</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
-        <v>0.09057999999999999</v>
+        <v>0.026465</v>
       </c>
       <c r="N26" t="n">
-        <v>0.001883</v>
+        <v>0.004611</v>
       </c>
       <c r="O26" t="n">
-        <v>0.003858</v>
+        <v>0.00061</v>
       </c>
       <c r="P26" t="n">
-        <v>0.084838</v>
+        <v>0.021244</v>
       </c>
       <c r="Q26" t="n">
-        <v>558.8</v>
+        <v>174.9</v>
       </c>
       <c r="R26" t="n">
-        <v>29565.5</v>
+        <v>18211.1</v>
       </c>
       <c r="S26" t="n">
-        <v>1286.1</v>
+        <v>508</v>
       </c>
       <c r="T26" t="n">
-        <v>28279.4</v>
+        <v>17703.1</v>
       </c>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="n">
-        <v>372.0058048768779</v>
+        <v>1104.110834068831</v>
       </c>
       <c r="W26" t="n">
-        <v>0.06030115570105155</v>
+        <v>0.1670685718904037</v>
       </c>
       <c r="X26" t="n">
-        <v>0.002688130096063873</v>
+        <v>0.0009057061747277989</v>
       </c>
       <c r="Y26" t="n">
-        <v>52.90891195418755</v>
+        <v>104.1229273870783</v>
       </c>
       <c r="Z26" t="n">
-        <v>1.139716419669804</v>
+        <v>1.604532028467891</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>k2-horizon-375b-a23b</t>
+          <t>inkling</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Inkling (xhigh)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Inkling</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Institute of Foundation Models</t>
+          <t>Thinking Machines</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ifm</t>
+          <t>thinking-machines</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2833,54 +2813,82 @@
         <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>30.5015302696723</v>
-      </c>
-      <c r="K27" t="inlineStr"/>
+        <v>24.9847810999384</v>
+      </c>
+      <c r="K27" t="n">
+        <v>13.36084550798845</v>
+      </c>
       <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
-      <c r="T27" t="inlineStr"/>
+      <c r="M27" t="n">
+        <v>0.09468799999999999</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0.002374</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0.001895</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0.09042</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>112.2</v>
+      </c>
+      <c r="R27" t="n">
+        <v>22793.6</v>
+      </c>
+      <c r="S27" t="n">
+        <v>467.8</v>
+      </c>
+      <c r="T27" t="n">
+        <v>22325.9</v>
+      </c>
       <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="inlineStr"/>
+      <c r="V27" t="n">
+        <v>263.8642816401065</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0.2226807584664741</v>
+      </c>
+      <c r="X27" t="n">
+        <v>0.00378982707998324</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>203.1515151515151</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>1.096131418465639</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>minimax-m3</t>
+          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>Nemotron 3 Ultra</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>minimax</t>
+          <t>nvidia</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2895,177 +2903,177 @@
         <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>29.2202932236316</v>
+        <v>22.9279123422858</v>
       </c>
       <c r="K28" t="n">
-        <v>10.30092593077495</v>
+        <v>22.44167602833847</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
-        <v>0.026465</v>
+        <v>0.033009</v>
       </c>
       <c r="N28" t="n">
-        <v>0.004611</v>
+        <v>0.001525</v>
       </c>
       <c r="O28" t="n">
-        <v>0.00061</v>
+        <v>0.002864</v>
       </c>
       <c r="P28" t="n">
-        <v>0.021244</v>
+        <v>0.02862</v>
       </c>
       <c r="Q28" t="n">
-        <v>170.2</v>
+        <v>61.3</v>
       </c>
       <c r="R28" t="n">
-        <v>18211.1</v>
+        <v>12593.6</v>
       </c>
       <c r="S28" t="n">
-        <v>508</v>
+        <v>1145.5</v>
       </c>
       <c r="T28" t="n">
-        <v>17703.1</v>
+        <v>11448.1</v>
       </c>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="n">
-        <v>1104.110834068831</v>
+        <v>694.5957872787968</v>
       </c>
       <c r="W28" t="n">
-        <v>0.1716820988462491</v>
+        <v>0.3740279338056411</v>
       </c>
       <c r="X28" t="n">
-        <v>0.0009057061747277989</v>
+        <v>0.001439686243876714</v>
       </c>
       <c r="Y28" t="n">
-        <v>106.9982373678026</v>
+        <v>205.442088091354</v>
       </c>
       <c r="Z28" t="n">
-        <v>1.604532028467891</v>
+        <v>1.820600332096128</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>inkling</t>
+          <t>gemini-3-5-flash-lite</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Inkling (xhigh)</t>
+          <t>Gemini 3.5 Flash-Lite</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Inkling</t>
+          <t>Gemini 3.5 Flash-Lite</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Thinking Machines</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>thinking-machines</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H29" t="b">
         <v>1</v>
       </c>
       <c r="I29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>24.9847810999384</v>
+        <v>22.1685424839812</v>
       </c>
       <c r="K29" t="n">
-        <v>13.40864817528</v>
+        <v>56.36070123046067</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
-        <v>0.09468799999999999</v>
+        <v>0.019232</v>
       </c>
       <c r="N29" t="n">
-        <v>0.002374</v>
+        <v>0.000782</v>
       </c>
       <c r="O29" t="n">
-        <v>0.001895</v>
+        <v>0.001426</v>
       </c>
       <c r="P29" t="n">
-        <v>0.09042</v>
+        <v>0.017024</v>
       </c>
       <c r="Q29" t="n">
-        <v>111.8</v>
+        <v>23.6</v>
       </c>
       <c r="R29" t="n">
-        <v>22793.6</v>
+        <v>7379.9</v>
       </c>
       <c r="S29" t="n">
-        <v>467.8</v>
+        <v>570.5</v>
       </c>
       <c r="T29" t="n">
-        <v>22325.9</v>
+        <v>6809.5</v>
       </c>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="n">
-        <v>263.8642816401065</v>
+        <v>1152.690436979056</v>
       </c>
       <c r="W29" t="n">
-        <v>0.223477469588</v>
+        <v>0.9393450205076779</v>
       </c>
       <c r="X29" t="n">
-        <v>0.00378982707998324</v>
+        <v>0.0008675356087977764</v>
       </c>
       <c r="Y29" t="n">
-        <v>203.8783542039356</v>
+        <v>312.707627118644</v>
       </c>
       <c r="Z29" t="n">
-        <v>1.096131418465639</v>
+        <v>3.003908248618708</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
+          <t>muse-glimmer</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
+          <t>Muse Glimmer (high)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra</t>
+          <t>Muse Glimmer (high)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H30" t="b">
@@ -3075,82 +3083,82 @@
         <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>22.9279123422858</v>
+        <v>17.4754176089465</v>
       </c>
       <c r="K30" t="n">
-        <v>24.13464457082716</v>
+        <v>19.27435765692629</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
-        <v>0.033009</v>
+        <v>0.011114</v>
       </c>
       <c r="N30" t="n">
-        <v>0.001525</v>
+        <v>0.000669</v>
       </c>
       <c r="O30" t="n">
-        <v>0.002864</v>
+        <v>0.000603</v>
       </c>
       <c r="P30" t="n">
-        <v>0.02862</v>
+        <v>0.009842</v>
       </c>
       <c r="Q30" t="n">
-        <v>57</v>
+        <v>54.4</v>
       </c>
       <c r="R30" t="n">
-        <v>12593.6</v>
+        <v>7737.1</v>
       </c>
       <c r="S30" t="n">
-        <v>1145.5</v>
+        <v>446.4</v>
       </c>
       <c r="T30" t="n">
-        <v>11448.1</v>
+        <v>7290.7</v>
       </c>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="n">
-        <v>694.5957872787968</v>
+        <v>1572.37876632594</v>
       </c>
       <c r="W30" t="n">
-        <v>0.4022440761804527</v>
+        <v>0.3212392942821048</v>
       </c>
       <c r="X30" t="n">
-        <v>0.001439686243876714</v>
+        <v>0.0006359790792244194</v>
       </c>
       <c r="Y30" t="n">
-        <v>220.940350877193</v>
+        <v>142.2261029411765</v>
       </c>
       <c r="Z30" t="n">
-        <v>1.820600332096128</v>
+        <v>2.258652157649054</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>gemini-3-5-flash-lite</t>
+          <t>mistral-medium-3-5</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash-Lite</t>
+          <t>Mistral Medium 3.5</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash-Lite</t>
+          <t>Mistral Medium 3.5</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Mistral</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>mistral</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3162,233 +3170,53 @@
         <v>1</v>
       </c>
       <c r="I31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>22.1685424839812</v>
+        <v>14.1889227802691</v>
       </c>
       <c r="K31" t="n">
-        <v>56.36070123046067</v>
+        <v>10.45866544000179</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
-        <v>0.019232</v>
+        <v>0.108206</v>
       </c>
       <c r="N31" t="n">
-        <v>0.000782</v>
+        <v>0.002141</v>
       </c>
       <c r="O31" t="n">
-        <v>0.001426</v>
+        <v>0.058389</v>
       </c>
       <c r="P31" t="n">
-        <v>0.017024</v>
+        <v>0.047676</v>
       </c>
       <c r="Q31" t="n">
-        <v>23.6</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="R31" t="n">
-        <v>7379.9</v>
+        <v>14142</v>
       </c>
       <c r="S31" t="n">
-        <v>570.5</v>
+        <v>7785.3</v>
       </c>
       <c r="T31" t="n">
-        <v>6809.5</v>
+        <v>6356.8</v>
       </c>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="n">
-        <v>1152.690436979056</v>
+        <v>131.1287985903656</v>
       </c>
       <c r="W31" t="n">
-        <v>0.9393450205076779</v>
+        <v>0.1743110906666966</v>
       </c>
       <c r="X31" t="n">
-        <v>0.0008675356087977764</v>
+        <v>0.007626089850208333</v>
       </c>
       <c r="Y31" t="n">
-        <v>312.707627118644</v>
+        <v>173.7346437346437</v>
       </c>
       <c r="Z31" t="n">
-        <v>3.003908248618708</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>muse-glimmer</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Muse Glimmer (high)</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Muse Glimmer (high)</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>meta</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>small</t>
-        </is>
-      </c>
-      <c r="H32" t="b">
-        <v>1</v>
-      </c>
-      <c r="I32" t="b">
-        <v>1</v>
-      </c>
-      <c r="J32" t="n">
-        <v>17.4754176089465</v>
-      </c>
-      <c r="K32" t="n">
-        <v>19.09881705895793</v>
-      </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="n">
-        <v>0.011114</v>
-      </c>
-      <c r="N32" t="n">
-        <v>0.000669</v>
-      </c>
-      <c r="O32" t="n">
-        <v>0.000603</v>
-      </c>
-      <c r="P32" t="n">
-        <v>0.009842</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>54.9</v>
-      </c>
-      <c r="R32" t="n">
-        <v>7737.1</v>
-      </c>
-      <c r="S32" t="n">
-        <v>446.4</v>
-      </c>
-      <c r="T32" t="n">
-        <v>7290.7</v>
-      </c>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="n">
-        <v>1572.37876632594</v>
-      </c>
-      <c r="W32" t="n">
-        <v>0.3183136176492987</v>
-      </c>
-      <c r="X32" t="n">
-        <v>0.0006359790792244194</v>
-      </c>
-      <c r="Y32" t="n">
-        <v>140.9307832422587</v>
-      </c>
-      <c r="Z32" t="n">
-        <v>2.258652157649054</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>mistral-medium-3-5</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Mistral Medium 3.5</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Mistral Medium 3.5</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Mistral</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>mistral</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>2026-04-29</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H33" t="b">
-        <v>1</v>
-      </c>
-      <c r="I33" t="b">
-        <v>1</v>
-      </c>
-      <c r="J33" t="n">
-        <v>14.1889227802691</v>
-      </c>
-      <c r="K33" t="n">
-        <v>10.08691192910126</v>
-      </c>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="n">
-        <v>0.108206</v>
-      </c>
-      <c r="N33" t="n">
-        <v>0.002141</v>
-      </c>
-      <c r="O33" t="n">
-        <v>0.058389</v>
-      </c>
-      <c r="P33" t="n">
-        <v>0.047676</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>84.40000000000001</v>
-      </c>
-      <c r="R33" t="n">
-        <v>14142</v>
-      </c>
-      <c r="S33" t="n">
-        <v>7785.3</v>
-      </c>
-      <c r="T33" t="n">
-        <v>6356.8</v>
-      </c>
-      <c r="U33" t="inlineStr"/>
-      <c r="V33" t="n">
-        <v>131.1287985903656</v>
-      </c>
-      <c r="W33" t="n">
-        <v>0.1681151988183543</v>
-      </c>
-      <c r="X33" t="n">
-        <v>0.007626089850208333</v>
-      </c>
-      <c r="Y33" t="n">
-        <v>167.5592417061611</v>
-      </c>
-      <c r="Z33" t="n">
         <v>1.003317973431558</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-01)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>13.5210879492287</v>
+        <v>13.27704373509131</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>0.711927</v>
       </c>
       <c r="Q2" t="n">
-        <v>255.7</v>
+        <v>260.4</v>
       </c>
       <c r="R2" t="n">
         <v>37461.4</v>
@@ -626,13 +626,13 @@
         <v>74.74125673551127</v>
       </c>
       <c r="W2" t="n">
-        <v>0.2253514658204783</v>
+        <v>0.2212840622515219</v>
       </c>
       <c r="X2" t="n">
         <v>0.0133794913770145</v>
       </c>
       <c r="Y2" t="n">
-        <v>146.50527962456</v>
+        <v>143.8609831029186</v>
       </c>
       <c r="Z2" t="n">
         <v>1.538179828044235</v>
@@ -774,7 +774,7 @@
         <v>55.9779549012591</v>
       </c>
       <c r="K4" t="n">
-        <v>11.10306543496048</v>
+        <v>10.97606958848218</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.661713</v>
       </c>
       <c r="Q4" t="n">
-        <v>302.5</v>
+        <v>306</v>
       </c>
       <c r="R4" t="n">
         <v>68107.2</v>
@@ -806,13 +806,13 @@
         <v>80.4261316911212</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1850510905826747</v>
+        <v>0.1829344931413696</v>
       </c>
       <c r="X4" t="n">
         <v>0.01243376970858835</v>
       </c>
       <c r="Y4" t="n">
-        <v>225.1477685950413</v>
+        <v>222.5725490196078</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8219095029785266</v>
@@ -864,7 +864,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K5" t="n">
-        <v>128.5996703572961</v>
+        <v>126.5744786981261</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -880,7 +880,7 @@
         <v>0.03274</v>
       </c>
       <c r="Q5" t="n">
-        <v>25</v>
+        <v>25.4</v>
       </c>
       <c r="R5" t="n">
         <v>3004</v>
@@ -896,13 +896,13 @@
         <v>686.2074633379441</v>
       </c>
       <c r="W5" t="n">
-        <v>2.143327839288268</v>
+        <v>2.109574644968768</v>
       </c>
       <c r="X5" t="n">
         <v>0.001457285228487116</v>
       </c>
       <c r="Y5" t="n">
-        <v>120.16</v>
+        <v>118.2677165354331</v>
       </c>
       <c r="Z5" t="n">
         <v>17.83728228435643</v>
@@ -954,7 +954,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>15.25879674804343</v>
+        <v>15.09333124818252</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -970,7 +970,7 @@
         <v>1.087069</v>
       </c>
       <c r="Q6" t="n">
-        <v>209.8</v>
+        <v>212.1</v>
       </c>
       <c r="R6" t="n">
         <v>23039.4</v>
@@ -986,13 +986,13 @@
         <v>44.3365962628782</v>
       </c>
       <c r="W6" t="n">
-        <v>0.2543132791340572</v>
+        <v>0.2515555208030419</v>
       </c>
       <c r="X6" t="n">
         <v>0.022554730951173</v>
       </c>
       <c r="Y6" t="n">
-        <v>109.8160152526215</v>
+        <v>108.6251768033946</v>
       </c>
       <c r="Z6" t="n">
         <v>2.315812302504631</v>
@@ -1044,7 +1044,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K7" t="n">
-        <v>30.93212718249675</v>
+        <v>30.11505212484589</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1060,7 +1060,7 @@
         <v>0.452635</v>
       </c>
       <c r="Q7" t="n">
-        <v>103.2</v>
+        <v>106</v>
       </c>
       <c r="R7" t="n">
         <v>10176.4</v>
@@ -1076,13 +1076,13 @@
         <v>95.52129303831462</v>
       </c>
       <c r="W7" t="n">
-        <v>0.5155354530416124</v>
+        <v>0.5019175354140981</v>
       </c>
       <c r="X7" t="n">
         <v>0.01046887000994521</v>
       </c>
       <c r="Y7" t="n">
-        <v>98.60852713178294</v>
+        <v>96.00377358490566</v>
       </c>
       <c r="Z7" t="n">
         <v>5.228102153403404</v>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (max)</t>
+          <t>GPT-6 Astra (Max)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1134,7 +1134,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K8" t="n">
-        <v>29.10147480415083</v>
+        <v>29.04797944605497</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1150,7 +1150,7 @@
         <v>0.25811</v>
       </c>
       <c r="Q8" t="n">
-        <v>108.6</v>
+        <v>108.8</v>
       </c>
       <c r="R8" t="n">
         <v>5609.9</v>
@@ -1166,13 +1166,13 @@
         <v>173.6055812119343</v>
       </c>
       <c r="W8" t="n">
-        <v>0.4850245800691805</v>
+        <v>0.4841329907675828</v>
       </c>
       <c r="X8" t="n">
         <v>0.005760183474627001</v>
       </c>
       <c r="Y8" t="n">
-        <v>51.65653775322284</v>
+        <v>51.56158088235294</v>
       </c>
       <c r="Z8" t="n">
         <v>9.389413250773277</v>
@@ -1181,32 +1181,32 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>gpt-6-astra-xhigh</t>
+          <t>gemini-4-argon</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (xhigh)</t>
+          <t>Gemini 4 Argon (High)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (xhigh)</t>
+          <t>Gemini 4 Argon (high)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1221,82 +1221,74 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>52.3863277108782</v>
-      </c>
-      <c r="K9" t="n">
-        <v>51.1918511832686</v>
-      </c>
+        <v>52.5605655745982</v>
+      </c>
+      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
-        <v>0.172456</v>
+        <v>0.253676</v>
       </c>
       <c r="N9" t="n">
-        <v>0.023073</v>
+        <v>0.024676</v>
       </c>
       <c r="O9" t="n">
-        <v>0.02257</v>
+        <v>0.009820000000000001</v>
       </c>
       <c r="P9" t="n">
-        <v>0.126814</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>61.4</v>
-      </c>
+        <v>0.21918</v>
+      </c>
+      <c r="Q9" t="inlineStr"/>
       <c r="R9" t="n">
-        <v>2987.7</v>
+        <v>22900</v>
       </c>
       <c r="S9" t="n">
-        <v>451.4</v>
+        <v>982</v>
       </c>
       <c r="T9" t="n">
-        <v>2536.3</v>
+        <v>21918</v>
       </c>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="n">
-        <v>303.7663387233741</v>
-      </c>
-      <c r="W9" t="n">
-        <v>0.8531975197211433</v>
-      </c>
+        <v>207.195657352679</v>
+      </c>
+      <c r="W9" t="inlineStr"/>
       <c r="X9" t="n">
-        <v>0.003292003992946215</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>48.65960912052117</v>
-      </c>
+        <v>0.00482635598051095</v>
+      </c>
+      <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="n">
-        <v>17.53399863134793</v>
+        <v>2.295221204130926</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>claude-sonnet-5-5-xhigh</t>
+          <t>gpt-6-astra-xhigh</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5.5 (Adaptive Reasoning, Xhigh Effort, Default Fallback)</t>
+          <t>GPT-6 Astra (Xhigh)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5.5 (xhigh with fallback)</t>
+          <t>GPT-6 Astra (xhigh)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1311,82 +1303,82 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>51.8522867021152</v>
+        <v>52.3863277108782</v>
       </c>
       <c r="K10" t="n">
-        <v>73.54934283987973</v>
+        <v>49.42106387818698</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
-        <v>0.08497200000000001</v>
+        <v>0.172456</v>
       </c>
       <c r="N10" t="n">
-        <v>0.013004</v>
+        <v>0.023073</v>
       </c>
       <c r="O10" t="n">
-        <v>0.013776</v>
+        <v>0.02257</v>
       </c>
       <c r="P10" t="n">
-        <v>0.058192</v>
+        <v>0.126814</v>
       </c>
       <c r="Q10" t="n">
-        <v>42.3</v>
+        <v>63.6</v>
       </c>
       <c r="R10" t="n">
-        <v>7196.8</v>
+        <v>2987.7</v>
       </c>
       <c r="S10" t="n">
-        <v>1377.6</v>
+        <v>451.4</v>
       </c>
       <c r="T10" t="n">
-        <v>5819.2</v>
+        <v>2536.3</v>
       </c>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="n">
-        <v>610.2279186333757</v>
+        <v>303.7663387233741</v>
       </c>
       <c r="W10" t="n">
-        <v>1.225822380664662</v>
+        <v>0.823684397969783</v>
       </c>
       <c r="X10" t="n">
-        <v>0.001638731971227293</v>
+        <v>0.003292003992946215</v>
       </c>
       <c r="Y10" t="n">
-        <v>170.1371158392435</v>
+        <v>46.97641509433962</v>
       </c>
       <c r="Z10" t="n">
-        <v>7.204908668035126</v>
+        <v>17.53399863134793</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>gpt-6-1-sol</t>
+          <t>claude-sonnet-5-5-xhigh</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>GPT-6.1 Sol (max)</t>
+          <t>Claude Sonnet 5.5 (Adaptive Reasoning, Xhigh Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GPT-6.1 Sol (max)</t>
+          <t>Claude Sonnet 5.5 (xhigh with fallback)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1401,82 +1393,82 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>51.8332597011541</v>
+        <v>51.8522867021152</v>
       </c>
       <c r="K11" t="n">
-        <v>30.22347504440472</v>
+        <v>73.54934283987973</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
-        <v>0.074921</v>
+        <v>0.08497200000000001</v>
       </c>
       <c r="N11" t="n">
-        <v>0.006023</v>
+        <v>0.013004</v>
       </c>
       <c r="O11" t="n">
-        <v>0.005667</v>
+        <v>0.013776</v>
       </c>
       <c r="P11" t="n">
-        <v>0.06322999999999999</v>
+        <v>0.058192</v>
       </c>
       <c r="Q11" t="n">
-        <v>102.9</v>
+        <v>42.3</v>
       </c>
       <c r="R11" t="n">
-        <v>6889.8</v>
+        <v>7196.8</v>
       </c>
       <c r="S11" t="n">
-        <v>566.7</v>
+        <v>1377.6</v>
       </c>
       <c r="T11" t="n">
-        <v>6323</v>
+        <v>5819.2</v>
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>691.8388662878779</v>
+        <v>610.2279186333757</v>
       </c>
       <c r="W11" t="n">
-        <v>0.503724584073412</v>
+        <v>1.225822380664662</v>
       </c>
       <c r="X11" t="n">
-        <v>0.001445423275170399</v>
+        <v>0.001638731971227293</v>
       </c>
       <c r="Y11" t="n">
-        <v>66.95626822157435</v>
+        <v>170.1371158392435</v>
       </c>
       <c r="Z11" t="n">
-        <v>7.523187857579915</v>
+        <v>7.204908668035126</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>muse-spark-1-3</t>
+          <t>gpt-6-1-sol</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Muse Spark 1.3 (max)</t>
+          <t>GPT-6.1 Sol (Max)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Muse Spark 1.3 (max)</t>
+          <t>GPT-6.1 Sol (max)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1491,82 +1483,82 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>48.0923107719685</v>
+        <v>51.8332597011541</v>
       </c>
       <c r="K12" t="n">
-        <v>27.3251765749821</v>
+        <v>29.01115281781013</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
-        <v>0.083136</v>
+        <v>0.074921</v>
       </c>
       <c r="N12" t="n">
-        <v>0.004284</v>
+        <v>0.006023</v>
       </c>
       <c r="O12" t="n">
-        <v>0.003428</v>
+        <v>0.005667</v>
       </c>
       <c r="P12" t="n">
-        <v>0.07542500000000001</v>
+        <v>0.06322999999999999</v>
       </c>
       <c r="Q12" t="n">
-        <v>105.6</v>
+        <v>107.2</v>
       </c>
       <c r="R12" t="n">
-        <v>18553.6</v>
+        <v>6889.8</v>
       </c>
       <c r="S12" t="n">
-        <v>806.5</v>
+        <v>566.7</v>
       </c>
       <c r="T12" t="n">
-        <v>17747</v>
+        <v>6323</v>
       </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="n">
-        <v>578.4775641354948</v>
+        <v>691.8388662878779</v>
       </c>
       <c r="W12" t="n">
-        <v>0.4554196095830351</v>
+        <v>0.4835192136301688</v>
       </c>
       <c r="X12" t="n">
-        <v>0.001728675513102135</v>
+        <v>0.001445423275170399</v>
       </c>
       <c r="Y12" t="n">
-        <v>175.6969696969697</v>
+        <v>64.2705223880597</v>
       </c>
       <c r="Z12" t="n">
-        <v>2.592074356026243</v>
+        <v>7.523187857579915</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>gpt-6-sol</t>
+          <t>muse-spark-1-3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GPT-6 Sol (max)</t>
+          <t>Muse Spark 1.3 (Max)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GPT-6 Sol (max)</t>
+          <t>Muse Spark 1.3 (max)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1581,82 +1573,82 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>47.5276426437724</v>
+        <v>48.0923107719685</v>
       </c>
       <c r="K13" t="n">
-        <v>26.97879431056144</v>
+        <v>25.67205201350631</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
-        <v>0.08570700000000001</v>
+        <v>0.083136</v>
       </c>
       <c r="N13" t="n">
-        <v>0.00525</v>
+        <v>0.004284</v>
       </c>
       <c r="O13" t="n">
-        <v>0.003693</v>
+        <v>0.003428</v>
       </c>
       <c r="P13" t="n">
-        <v>0.076765</v>
+        <v>0.07542500000000001</v>
       </c>
       <c r="Q13" t="n">
-        <v>105.7</v>
+        <v>112.4</v>
       </c>
       <c r="R13" t="n">
-        <v>8045.8</v>
+        <v>18553.6</v>
       </c>
       <c r="S13" t="n">
-        <v>369.3</v>
+        <v>806.5</v>
       </c>
       <c r="T13" t="n">
-        <v>7676.5</v>
+        <v>17747</v>
       </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="n">
-        <v>554.5362997628245</v>
+        <v>578.4775641354948</v>
       </c>
       <c r="W13" t="n">
-        <v>0.4496465718426906</v>
+        <v>0.4278675335584386</v>
       </c>
       <c r="X13" t="n">
-        <v>0.001803308458666638</v>
+        <v>0.001728675513102135</v>
       </c>
       <c r="Y13" t="n">
-        <v>76.11920529801324</v>
+        <v>165.067615658363</v>
       </c>
       <c r="Z13" t="n">
-        <v>5.907136971310796</v>
+        <v>2.592074356026243</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>grok-4-7</t>
+          <t>gpt-6-sol</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Grok 4.7 (xhigh)</t>
+          <t>GPT-6 Sol (Max)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Grok 4.7 (xhigh)</t>
+          <t>GPT-6 Sol (max)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>SpaceXAI</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>xai</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1671,77 +1663,77 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>46.4465506302286</v>
+        <v>47.6305176437724</v>
       </c>
       <c r="K14" t="n">
-        <v>3.467885811117118</v>
+        <v>26.73368623598077</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>0.350873</v>
+        <v>0.085367</v>
       </c>
       <c r="N14" t="n">
-        <v>0.008541999999999999</v>
+        <v>0.00525</v>
       </c>
       <c r="O14" t="n">
-        <v>0.004758</v>
+        <v>0.003689</v>
       </c>
       <c r="P14" t="n">
-        <v>0.337573</v>
+        <v>0.076429</v>
       </c>
       <c r="Q14" t="n">
-        <v>803.6</v>
+        <v>106.9</v>
       </c>
       <c r="R14" t="n">
-        <v>57055.2</v>
+        <v>8011.8</v>
       </c>
       <c r="S14" t="n">
-        <v>793</v>
+        <v>368.9</v>
       </c>
       <c r="T14" t="n">
-        <v>56262.1</v>
+        <v>7642.9</v>
       </c>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="n">
-        <v>132.374251168453</v>
+        <v>557.9499999270491</v>
       </c>
       <c r="W14" t="n">
-        <v>0.05779809685195197</v>
+        <v>0.4455614372663461</v>
       </c>
       <c r="X14" t="n">
-        <v>0.007554339240245816</v>
+        <v>0.001792275293719416</v>
       </c>
       <c r="Y14" t="n">
-        <v>70.99950223992035</v>
+        <v>74.9466791393826</v>
       </c>
       <c r="Z14" t="n">
-        <v>0.814063409298865</v>
+        <v>5.945045762971167</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>mimo-v2-6-pro</t>
+          <t>grok-4-7</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Grok 4.7 (Xhigh)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Grok 4.7 (xhigh)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Xiaomi</t>
+          <t>SpaceXAI</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>xiaomi</t>
+          <t>xai</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1758,85 +1750,85 @@
         <v>1</v>
       </c>
       <c r="I15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>46.3242065310383</v>
+        <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>5.645850887390409</v>
+        <v>3.398942600089909</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>0.021122</v>
+        <v>0.350873</v>
       </c>
       <c r="N15" t="n">
-        <v>0.003029</v>
+        <v>0.008541999999999999</v>
       </c>
       <c r="O15" t="n">
-        <v>0.002893</v>
+        <v>0.004758</v>
       </c>
       <c r="P15" t="n">
-        <v>0.0152</v>
+        <v>0.337573</v>
       </c>
       <c r="Q15" t="n">
-        <v>492.3</v>
+        <v>819.9</v>
       </c>
       <c r="R15" t="n">
-        <v>20796.5</v>
+        <v>57055.2</v>
       </c>
       <c r="S15" t="n">
-        <v>3325.3</v>
+        <v>793</v>
       </c>
       <c r="T15" t="n">
-        <v>17471.2</v>
+        <v>56262.1</v>
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="n">
-        <v>2193.173304187023</v>
+        <v>132.374251168453</v>
       </c>
       <c r="W15" t="n">
-        <v>0.09409751478984013</v>
+        <v>0.05664904333483181</v>
       </c>
       <c r="X15" t="n">
-        <v>0.0004559603192738502</v>
+        <v>0.007554339240245816</v>
       </c>
       <c r="Y15" t="n">
-        <v>42.24355068047938</v>
+        <v>69.58799853640687</v>
       </c>
       <c r="Z15" t="n">
-        <v>2.227500133726266</v>
+        <v>0.814063409298865</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>qwen3-8-max</t>
+          <t>mimo-v2-6-pro</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>Xiaomi</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>xiaomi</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1848,85 +1840,85 @@
         <v>1</v>
       </c>
       <c r="I16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" t="n">
-        <v>45.4152084980521</v>
+        <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>5.31068507090845</v>
+        <v>5.841640167848461</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
-        <v>0.156468</v>
+        <v>0.021122</v>
       </c>
       <c r="N16" t="n">
-        <v>0.007406</v>
+        <v>0.003029</v>
       </c>
       <c r="O16" t="n">
-        <v>0.007526</v>
+        <v>0.002893</v>
       </c>
       <c r="P16" t="n">
-        <v>0.141536</v>
+        <v>0.0152</v>
       </c>
       <c r="Q16" t="n">
-        <v>513.1</v>
+        <v>475.8</v>
       </c>
       <c r="R16" t="n">
-        <v>24843.6</v>
+        <v>20796.5</v>
       </c>
       <c r="S16" t="n">
-        <v>1254.3</v>
+        <v>3325.3</v>
       </c>
       <c r="T16" t="n">
-        <v>23589.3</v>
+        <v>17471.2</v>
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="n">
-        <v>290.2523742749451</v>
+        <v>2193.173304187023</v>
       </c>
       <c r="W16" t="n">
-        <v>0.08851141784847417</v>
+        <v>0.09736066946414103</v>
       </c>
       <c r="X16" t="n">
-        <v>0.003445277588161046</v>
+        <v>0.0004559603192738502</v>
       </c>
       <c r="Y16" t="n">
-        <v>48.41863184564412</v>
+        <v>43.70849096258932</v>
       </c>
       <c r="Z16" t="n">
-        <v>1.828044586857464</v>
+        <v>2.227500133726266</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>glm-5-3</t>
+          <t>qwen3-8-max</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1938,85 +1930,85 @@
         <v>1</v>
       </c>
       <c r="I17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>44.777392385614</v>
+        <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>7.47327828410804</v>
+        <v>5.370343929608053</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
-        <v>0.15892</v>
+        <v>0.156468</v>
       </c>
       <c r="N17" t="n">
-        <v>0.006115</v>
+        <v>0.007406</v>
       </c>
       <c r="O17" t="n">
-        <v>0.004153</v>
+        <v>0.007526</v>
       </c>
       <c r="P17" t="n">
-        <v>0.148652</v>
+        <v>0.141536</v>
       </c>
       <c r="Q17" t="n">
-        <v>359.5</v>
+        <v>507.4</v>
       </c>
       <c r="R17" t="n">
-        <v>34728.3</v>
+        <v>24843.6</v>
       </c>
       <c r="S17" t="n">
-        <v>943.8</v>
+        <v>1254.3</v>
       </c>
       <c r="T17" t="n">
-        <v>33784.5</v>
+        <v>23589.3</v>
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="n">
-        <v>281.760586368072</v>
+        <v>290.2523742749451</v>
       </c>
       <c r="W17" t="n">
-        <v>0.1245546380684673</v>
+        <v>0.08950573216013422</v>
       </c>
       <c r="X17" t="n">
-        <v>0.003549112432260739</v>
+        <v>0.003445277588161046</v>
       </c>
       <c r="Y17" t="n">
-        <v>96.60166898470098</v>
+        <v>48.9625541978715</v>
       </c>
       <c r="Z17" t="n">
-        <v>1.289363210569305</v>
+        <v>1.828044586857464</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>step-5</t>
+          <t>glm-5-3</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>GLM-5.3 (Max)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>StepFun</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>stepfun</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2028,85 +2020,85 @@
         <v>1</v>
       </c>
       <c r="I18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" t="n">
-        <v>43.7343049141614</v>
+        <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>16.4106209809236</v>
+        <v>6.498895846968651</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
-        <v>0.044989</v>
+        <v>0.15892</v>
       </c>
       <c r="N18" t="n">
-        <v>0.003221</v>
+        <v>0.006115</v>
       </c>
       <c r="O18" t="n">
-        <v>0.002192</v>
+        <v>0.004153</v>
       </c>
       <c r="P18" t="n">
-        <v>0.039576</v>
+        <v>0.148652</v>
       </c>
       <c r="Q18" t="n">
-        <v>159.9</v>
+        <v>413.4</v>
       </c>
       <c r="R18" t="n">
-        <v>15469.6</v>
+        <v>34728.3</v>
       </c>
       <c r="S18" t="n">
-        <v>811.7</v>
+        <v>943.8</v>
       </c>
       <c r="T18" t="n">
-        <v>14657.8</v>
+        <v>33784.5</v>
       </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="n">
-        <v>972.1110696872879</v>
+        <v>281.760586368072</v>
       </c>
       <c r="W18" t="n">
-        <v>0.27351034968206</v>
+        <v>0.1083149307828108</v>
       </c>
       <c r="X18" t="n">
-        <v>0.001028689036862509</v>
+        <v>0.003549112432260739</v>
       </c>
       <c r="Y18" t="n">
-        <v>96.74546591619762</v>
+        <v>84.00653120464442</v>
       </c>
       <c r="Z18" t="n">
-        <v>2.827112848047875</v>
+        <v>1.289363210569305</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>kimi-k3</t>
+          <t>step-5</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Kimi K3 (max)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Kimi K3 (max)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Kimi</t>
+          <t>StepFun</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>kimi</t>
+          <t>stepfun</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2118,85 +2110,85 @@
         <v>1</v>
       </c>
       <c r="I19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>43.5938229518782</v>
+        <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>10.64995674720152</v>
+        <v>15.4084456538443</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
-        <v>0.163338</v>
+        <v>0.044989</v>
       </c>
       <c r="N19" t="n">
-        <v>0.007471</v>
+        <v>0.003221</v>
       </c>
       <c r="O19" t="n">
-        <v>0.007591</v>
+        <v>0.002192</v>
       </c>
       <c r="P19" t="n">
-        <v>0.148276</v>
+        <v>0.039576</v>
       </c>
       <c r="Q19" t="n">
-        <v>245.6</v>
+        <v>170.3</v>
       </c>
       <c r="R19" t="n">
-        <v>10391.2</v>
+        <v>15469.6</v>
       </c>
       <c r="S19" t="n">
-        <v>506.1</v>
+        <v>811.7</v>
       </c>
       <c r="T19" t="n">
-        <v>9885.1</v>
+        <v>14657.8</v>
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="n">
-        <v>266.8933313244817</v>
+        <v>972.1110696872879</v>
       </c>
       <c r="W19" t="n">
-        <v>0.1774992791200252</v>
+        <v>0.2568074275640716</v>
       </c>
       <c r="X19" t="n">
-        <v>0.0037468152352755</v>
+        <v>0.001028689036862509</v>
       </c>
       <c r="Y19" t="n">
-        <v>42.30944625407167</v>
+        <v>90.83734586024661</v>
       </c>
       <c r="Z19" t="n">
-        <v>4.195263583789957</v>
+        <v>2.827112848047875</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>glm-5-3-flash</t>
+          <t>kimi-k3</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>GLM 5.3 Flash</t>
+          <t>Kimi K3 (Max)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Kimi K3 (max)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>Kimi</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>kimi</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2211,82 +2203,82 @@
         <v>1</v>
       </c>
       <c r="J20" t="n">
-        <v>41.807466113455</v>
+        <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>3.483955509454583</v>
+        <v>9.745265935591254</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
-        <v>0.022786</v>
+        <v>0.163338</v>
       </c>
       <c r="N20" t="n">
-        <v>0.000576</v>
+        <v>0.007471</v>
       </c>
       <c r="O20" t="n">
-        <v>0.000417</v>
+        <v>0.007591</v>
       </c>
       <c r="P20" t="n">
-        <v>0.021793</v>
+        <v>0.148276</v>
       </c>
       <c r="Q20" t="n">
-        <v>720</v>
+        <v>268.4</v>
       </c>
       <c r="R20" t="n">
-        <v>44420.3</v>
+        <v>10391.2</v>
       </c>
       <c r="S20" t="n">
-        <v>834.1</v>
+        <v>506.1</v>
       </c>
       <c r="T20" t="n">
-        <v>43586.3</v>
+        <v>9885.1</v>
       </c>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="n">
-        <v>1834.787418303125</v>
+        <v>266.8933313244817</v>
       </c>
       <c r="W20" t="n">
-        <v>0.05806592515757639</v>
+        <v>0.1624210989265209</v>
       </c>
       <c r="X20" t="n">
-        <v>0.0005450222679883181</v>
+        <v>0.0037468152352755</v>
       </c>
       <c r="Y20" t="n">
-        <v>61.69486111111112</v>
+        <v>38.71535022354695</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.9411792831983349</v>
+        <v>4.195263583789957</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>gemini-3-8-flash</t>
+          <t>glm-5-3-flash</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>GLM 5.3 Flash</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2298,85 +2290,85 @@
         <v>1</v>
       </c>
       <c r="I21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" t="n">
-        <v>40.9262321765904</v>
+        <v>41.807466113455</v>
       </c>
       <c r="K21" t="n">
-        <v>24.45790767525323</v>
+        <v>3.492687227523392</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
-        <v>0.093127</v>
+        <v>0.022786</v>
       </c>
       <c r="N21" t="n">
-        <v>0.001995</v>
+        <v>0.000576</v>
       </c>
       <c r="O21" t="n">
-        <v>0.002368</v>
+        <v>0.000417</v>
       </c>
       <c r="P21" t="n">
-        <v>0.088764</v>
+        <v>0.021793</v>
       </c>
       <c r="Q21" t="n">
-        <v>100.4</v>
+        <v>718.2</v>
       </c>
       <c r="R21" t="n">
-        <v>24301.8</v>
+        <v>44420.3</v>
       </c>
       <c r="S21" t="n">
-        <v>631.5</v>
+        <v>834.1</v>
       </c>
       <c r="T21" t="n">
-        <v>23670.3</v>
+        <v>43586.3</v>
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="n">
-        <v>439.4668804599139</v>
+        <v>1834.787418303125</v>
       </c>
       <c r="W21" t="n">
-        <v>0.4076317945875538</v>
+        <v>0.05821145379205653</v>
       </c>
       <c r="X21" t="n">
-        <v>0.002275484329907804</v>
+        <v>0.0005450222679883181</v>
       </c>
       <c r="Y21" t="n">
-        <v>242.0498007968127</v>
+        <v>61.84948482316904</v>
       </c>
       <c r="Z21" t="n">
-        <v>1.684082338616498</v>
+        <v>0.9411792831983349</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>deepseek-v4-1-flash</t>
+          <t>gemini-3-8-flash</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (Reasoning, Max Effort)</t>
+          <t>Gemini 3.8 Flash (High)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (max)</t>
+          <t>Gemini 3.8 Flash (high)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>DeepSeek</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>deepseek</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2388,270 +2380,270 @@
         <v>1</v>
       </c>
       <c r="I22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>39.456167472527</v>
+        <v>40.9262321765904</v>
       </c>
       <c r="K22" t="n">
-        <v>29.44490109890074</v>
+        <v>23.07870235522015</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
-        <v>0.027666</v>
+        <v>0.093127</v>
       </c>
       <c r="N22" t="n">
-        <v>0.000862</v>
+        <v>0.001995</v>
       </c>
       <c r="O22" t="n">
-        <v>0.000595</v>
+        <v>0.002368</v>
       </c>
       <c r="P22" t="n">
-        <v>0.02621</v>
+        <v>0.088764</v>
       </c>
       <c r="Q22" t="n">
-        <v>80.40000000000001</v>
+        <v>106.4</v>
       </c>
       <c r="R22" t="n">
-        <v>22336.9</v>
+        <v>24301.8</v>
       </c>
       <c r="S22" t="n">
-        <v>495.4</v>
+        <v>631.5</v>
       </c>
       <c r="T22" t="n">
-        <v>21841.5</v>
+        <v>23670.3</v>
       </c>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="n">
-        <v>1426.160900474481</v>
+        <v>439.4668804599139</v>
       </c>
       <c r="W22" t="n">
-        <v>0.4907483516483457</v>
+        <v>0.3846450392536692</v>
       </c>
       <c r="X22" t="n">
-        <v>0.0007011831551876802</v>
+        <v>0.002275484329907804</v>
       </c>
       <c r="Y22" t="n">
-        <v>277.8221393034826</v>
+        <v>228.4003759398496</v>
       </c>
       <c r="Z22" t="n">
-        <v>1.76641196730643</v>
+        <v>1.684082338616498</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>gpt-6-luna</t>
+          <t>deepseek-v4-1-flash</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (max)</t>
+          <t>DeepSeek V4.1 Flash (Max)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (max)</t>
+          <t>DeepSeek V4.1 Flash (max)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>DeepSeek</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>deepseek</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H23" t="b">
         <v>1</v>
       </c>
       <c r="I23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J23" t="n">
-        <v>37.2559686869738</v>
+        <v>39.456167472527</v>
       </c>
       <c r="K23" t="n">
-        <v>19.17116742039818</v>
+        <v>30.11921181108931</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
-        <v>0.008175999999999999</v>
+        <v>0.027666</v>
       </c>
       <c r="N23" t="n">
-        <v>0.000295</v>
+        <v>0.000862</v>
       </c>
       <c r="O23" t="n">
-        <v>0.000254</v>
+        <v>0.000595</v>
       </c>
       <c r="P23" t="n">
-        <v>0.007626</v>
+        <v>0.02621</v>
       </c>
       <c r="Q23" t="n">
-        <v>116.6</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="R23" t="n">
-        <v>15761.3</v>
+        <v>22336.9</v>
       </c>
       <c r="S23" t="n">
-        <v>508.9</v>
+        <v>495.4</v>
       </c>
       <c r="T23" t="n">
-        <v>15252.5</v>
+        <v>21841.5</v>
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="n">
-        <v>4556.747637839262</v>
+        <v>1426.160900474481</v>
       </c>
       <c r="W23" t="n">
-        <v>0.3195194570066364</v>
+        <v>0.5019868635181552</v>
       </c>
       <c r="X23" t="n">
-        <v>0.0002194547689444097</v>
+        <v>0.0007011831551876802</v>
       </c>
       <c r="Y23" t="n">
-        <v>135.1740994854202</v>
+        <v>284.1844783715013</v>
       </c>
       <c r="Z23" t="n">
-        <v>2.363762423592839</v>
+        <v>1.76641196730643</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>qwen3-8-27b</t>
+          <t>gpt-6-luna</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (xhigh)</t>
+          <t>GPT-6 Luna (Max)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (xhigh)</t>
+          <t>GPT-6 Luna (max)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H24" t="b">
         <v>1</v>
       </c>
       <c r="I24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>33.6962858057476</v>
+        <v>38.1245186869738</v>
       </c>
       <c r="K24" t="n">
-        <v>3.68131308875611</v>
+        <v>18.82692280838213</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>0.09057999999999999</v>
+        <v>0.007925</v>
       </c>
       <c r="N24" t="n">
-        <v>0.001883</v>
+        <v>0.000295</v>
       </c>
       <c r="O24" t="n">
-        <v>0.003858</v>
+        <v>0.000255</v>
       </c>
       <c r="P24" t="n">
-        <v>0.084838</v>
+        <v>0.007375</v>
       </c>
       <c r="Q24" t="n">
-        <v>549.2</v>
+        <v>121.5</v>
       </c>
       <c r="R24" t="n">
-        <v>29565.5</v>
+        <v>15260.2</v>
       </c>
       <c r="S24" t="n">
-        <v>1286.1</v>
+        <v>509.3</v>
       </c>
       <c r="T24" t="n">
-        <v>28279.4</v>
+        <v>14750.9</v>
       </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="n">
-        <v>372.0058048768779</v>
+        <v>4810.66481854559</v>
       </c>
       <c r="W24" t="n">
-        <v>0.06135521814593517</v>
+        <v>0.3137820468063687</v>
       </c>
       <c r="X24" t="n">
-        <v>0.002688130096063873</v>
+        <v>0.0002078714767540862</v>
       </c>
       <c r="Y24" t="n">
-        <v>53.83375819373634</v>
+        <v>125.598353909465</v>
       </c>
       <c r="Z24" t="n">
-        <v>1.139716419669804</v>
+        <v>2.498297446099907</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>k2-horizon-375b-a23b</t>
+          <t>qwen3-8-27b</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Qwen3.8 27B (Xhigh)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Qwen3.8 27B (xhigh)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Institute of Foundation Models</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ifm</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H25" t="b">
@@ -2661,54 +2653,82 @@
         <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>30.5015302696723</v>
-      </c>
-      <c r="K25" t="inlineStr"/>
+        <v>33.6962858057476</v>
+      </c>
+      <c r="K25" t="n">
+        <v>3.723346497872662</v>
+      </c>
       <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
+      <c r="M25" t="n">
+        <v>0.09057999999999999</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0.001883</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0.003858</v>
+      </c>
+      <c r="P25" t="n">
+        <v>0.084838</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>543</v>
+      </c>
+      <c r="R25" t="n">
+        <v>29565.5</v>
+      </c>
+      <c r="S25" t="n">
+        <v>1286.1</v>
+      </c>
+      <c r="T25" t="n">
+        <v>28279.4</v>
+      </c>
       <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
-      <c r="Z25" t="inlineStr"/>
+      <c r="V25" t="n">
+        <v>372.0058048768779</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0.06205577496454438</v>
+      </c>
+      <c r="X25" t="n">
+        <v>0.002688130096063873</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>54.44843462246777</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>1.139716419669804</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>minimax-m3</t>
+          <t>k2-horizon-375b-a23b</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>Institute of Foundation Models</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>minimax</t>
+          <t>ifm</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2723,82 +2743,54 @@
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>29.2202932236316</v>
-      </c>
-      <c r="K26" t="n">
-        <v>10.02411431342422</v>
-      </c>
+        <v>30.5015302696723</v>
+      </c>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
-      <c r="M26" t="n">
-        <v>0.026465</v>
-      </c>
-      <c r="N26" t="n">
-        <v>0.004611</v>
-      </c>
-      <c r="O26" t="n">
-        <v>0.00061</v>
-      </c>
-      <c r="P26" t="n">
-        <v>0.021244</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>174.9</v>
-      </c>
-      <c r="R26" t="n">
-        <v>18211.1</v>
-      </c>
-      <c r="S26" t="n">
-        <v>508</v>
-      </c>
-      <c r="T26" t="n">
-        <v>17703.1</v>
-      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
-      <c r="V26" t="n">
-        <v>1104.110834068831</v>
-      </c>
-      <c r="W26" t="n">
-        <v>0.1670685718904037</v>
-      </c>
-      <c r="X26" t="n">
-        <v>0.0009057061747277989</v>
-      </c>
-      <c r="Y26" t="n">
-        <v>104.1229273870783</v>
-      </c>
-      <c r="Z26" t="n">
-        <v>1.604532028467891</v>
-      </c>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>inkling</t>
+          <t>minimax-m3</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Inkling (xhigh)</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Inkling</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Thinking Machines</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>thinking-machines</t>
+          <t>minimax</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2813,82 +2805,82 @@
         <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>24.9847810999384</v>
+        <v>29.2202932236316</v>
       </c>
       <c r="K27" t="n">
-        <v>13.36084550798845</v>
+        <v>8.836782224888589</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
-        <v>0.09468799999999999</v>
+        <v>0.026465</v>
       </c>
       <c r="N27" t="n">
-        <v>0.002374</v>
+        <v>0.004611</v>
       </c>
       <c r="O27" t="n">
-        <v>0.001895</v>
+        <v>0.00061</v>
       </c>
       <c r="P27" t="n">
-        <v>0.09042</v>
+        <v>0.021244</v>
       </c>
       <c r="Q27" t="n">
-        <v>112.2</v>
+        <v>198.4</v>
       </c>
       <c r="R27" t="n">
-        <v>22793.6</v>
+        <v>18211.1</v>
       </c>
       <c r="S27" t="n">
-        <v>467.8</v>
+        <v>508</v>
       </c>
       <c r="T27" t="n">
-        <v>22325.9</v>
+        <v>17703.1</v>
       </c>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="n">
-        <v>263.8642816401065</v>
+        <v>1104.110834068831</v>
       </c>
       <c r="W27" t="n">
-        <v>0.2226807584664741</v>
+        <v>0.1472797037481431</v>
       </c>
       <c r="X27" t="n">
-        <v>0.00378982707998324</v>
+        <v>0.0009057061747277989</v>
       </c>
       <c r="Y27" t="n">
-        <v>203.1515151515151</v>
+        <v>91.78981854838709</v>
       </c>
       <c r="Z27" t="n">
-        <v>1.096131418465639</v>
+        <v>1.604532028467891</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
+          <t>inkling</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
+          <t>Inkling (Xhigh)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra</t>
+          <t>Inkling (xhigh)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Thinking Machines</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>thinking-machines</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2903,141 +2895,141 @@
         <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>22.9279123422858</v>
+        <v>24.9847810999384</v>
       </c>
       <c r="K28" t="n">
-        <v>22.44167602833847</v>
+        <v>13.5786853804013</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
-        <v>0.033009</v>
+        <v>0.09468799999999999</v>
       </c>
       <c r="N28" t="n">
-        <v>0.001525</v>
+        <v>0.002374</v>
       </c>
       <c r="O28" t="n">
-        <v>0.002864</v>
+        <v>0.001895</v>
       </c>
       <c r="P28" t="n">
-        <v>0.02862</v>
+        <v>0.09042</v>
       </c>
       <c r="Q28" t="n">
-        <v>61.3</v>
+        <v>110.4</v>
       </c>
       <c r="R28" t="n">
-        <v>12593.6</v>
+        <v>22793.6</v>
       </c>
       <c r="S28" t="n">
-        <v>1145.5</v>
+        <v>467.8</v>
       </c>
       <c r="T28" t="n">
-        <v>11448.1</v>
+        <v>22325.9</v>
       </c>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="n">
-        <v>694.5957872787968</v>
+        <v>263.8642816401065</v>
       </c>
       <c r="W28" t="n">
-        <v>0.3740279338056411</v>
+        <v>0.2263114230066884</v>
       </c>
       <c r="X28" t="n">
-        <v>0.001439686243876714</v>
+        <v>0.00378982707998324</v>
       </c>
       <c r="Y28" t="n">
-        <v>205.442088091354</v>
+        <v>206.463768115942</v>
       </c>
       <c r="Z28" t="n">
-        <v>1.820600332096128</v>
+        <v>1.096131418465639</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>gemini-3-5-flash-lite</t>
+          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash-Lite</t>
+          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash-Lite</t>
+          <t>Nemotron 3 Ultra</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>nvidia</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H29" t="b">
         <v>1</v>
       </c>
       <c r="I29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J29" t="n">
-        <v>22.1685424839812</v>
+        <v>22.9279123422858</v>
       </c>
       <c r="K29" t="n">
-        <v>56.36070123046067</v>
+        <v>17.26066173823272</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
-        <v>0.019232</v>
+        <v>0.033009</v>
       </c>
       <c r="N29" t="n">
-        <v>0.000782</v>
+        <v>0.001525</v>
       </c>
       <c r="O29" t="n">
-        <v>0.001426</v>
+        <v>0.002864</v>
       </c>
       <c r="P29" t="n">
-        <v>0.017024</v>
+        <v>0.02862</v>
       </c>
       <c r="Q29" t="n">
-        <v>23.6</v>
+        <v>79.7</v>
       </c>
       <c r="R29" t="n">
-        <v>7379.9</v>
+        <v>12593.6</v>
       </c>
       <c r="S29" t="n">
-        <v>570.5</v>
+        <v>1145.5</v>
       </c>
       <c r="T29" t="n">
-        <v>6809.5</v>
+        <v>11448.1</v>
       </c>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="n">
-        <v>1152.690436979056</v>
+        <v>694.5957872787968</v>
       </c>
       <c r="W29" t="n">
-        <v>0.9393450205076779</v>
+        <v>0.287677695637212</v>
       </c>
       <c r="X29" t="n">
-        <v>0.0008675356087977764</v>
+        <v>0.001439686243876714</v>
       </c>
       <c r="Y29" t="n">
-        <v>312.707627118644</v>
+        <v>158.0125470514429</v>
       </c>
       <c r="Z29" t="n">
-        <v>3.003908248618708</v>
+        <v>1.820600332096128</v>
       </c>
     </row>
     <row r="30">
@@ -3048,7 +3040,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Muse Glimmer (high)</t>
+          <t>Muse Glimmer (High)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3086,7 +3078,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K30" t="n">
-        <v>19.27435765692629</v>
+        <v>18.92644506384098</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3102,7 +3094,7 @@
         <v>0.009842</v>
       </c>
       <c r="Q30" t="n">
-        <v>54.4</v>
+        <v>55.4</v>
       </c>
       <c r="R30" t="n">
         <v>7737.1</v>
@@ -3118,13 +3110,13 @@
         <v>1572.37876632594</v>
       </c>
       <c r="W30" t="n">
-        <v>0.3212392942821048</v>
+        <v>0.3154407510640163</v>
       </c>
       <c r="X30" t="n">
         <v>0.0006359790792244194</v>
       </c>
       <c r="Y30" t="n">
-        <v>142.2261029411765</v>
+        <v>139.658844765343</v>
       </c>
       <c r="Z30" t="n">
         <v>2.258652157649054</v>
@@ -3176,7 +3168,7 @@
         <v>14.1889227802691</v>
       </c>
       <c r="K31" t="n">
-        <v>10.45866544000179</v>
+        <v>10.57559461883411</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3192,7 +3184,7 @@
         <v>0.047676</v>
       </c>
       <c r="Q31" t="n">
-        <v>81.40000000000001</v>
+        <v>80.5</v>
       </c>
       <c r="R31" t="n">
         <v>14142</v>
@@ -3208,13 +3200,13 @@
         <v>131.1287985903656</v>
       </c>
       <c r="W31" t="n">
-        <v>0.1743110906666966</v>
+        <v>0.1762599103139019</v>
       </c>
       <c r="X31" t="n">
         <v>0.007626089850208333</v>
       </c>
       <c r="Y31" t="n">
-        <v>173.7346437346437</v>
+        <v>175.6770186335404</v>
       </c>
       <c r="Z31" t="n">
         <v>1.003317973431558</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-02)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.196822273146125</v>
+        <v>4.287378706123237</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>823.8000000000001</v>
+        <v>806.4</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.06994703788576875</v>
+        <v>0.07145631176872061</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>144.6540422432629</v>
+        <v>147.7752976190476</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -641,17 +641,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>claude-opus-5-5-xhigh</t>
+          <t>claude-sonnet-5-5</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (Adaptive Reasoning, Xhigh Effort, Default Fallback)</t>
+          <t>Claude Sonnet 5.5 (Adaptive Reasoning, Max Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (xhigh with fallback)</t>
+          <t>Claude Sonnet 5.5 (max with fallback)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -681,67 +681,67 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>55.9873505840139</v>
+        <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>6.641441350416834</v>
+        <v>3.753359829629987</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
-        <v>29.342164</v>
+        <v>47.127587</v>
       </c>
       <c r="N3" t="n">
-        <v>28.028816</v>
+        <v>45.153283</v>
       </c>
       <c r="O3" t="n">
-        <v>0.507053</v>
+        <v>0.507969</v>
       </c>
       <c r="P3" t="n">
-        <v>0.806295</v>
+        <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>505.8</v>
+        <v>895.2</v>
       </c>
       <c r="R3" t="n">
-        <v>65667.39999999999</v>
+        <v>197430.4</v>
       </c>
       <c r="S3" t="n">
-        <v>25352.7</v>
+        <v>50796.9</v>
       </c>
       <c r="T3" t="n">
-        <v>40314.7</v>
+        <v>146633.5</v>
       </c>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="n">
-        <v>1.908085258606485</v>
+        <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.1106906891736139</v>
+        <v>0.06255599716049977</v>
       </c>
       <c r="X3" t="n">
-        <v>0.5240855960127908</v>
+        <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>129.8287860814551</v>
+        <v>220.5433422698838</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.8525897261657063</v>
+        <v>0.2836449131343471</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>claude-sonnet-5-5</t>
+          <t>claude-opus-5-5-xhigh</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5.5 (Adaptive Reasoning, Max Effort, Default Fallback)</t>
+          <t>Claude Opus 5.5 (Adaptive Reasoning, Xhigh Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5.5 (max with fallback)</t>
+          <t>Claude Opus 5.5 (xhigh with fallback)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -771,51 +771,51 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>55.9779549012591</v>
+        <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>3.860548613879938</v>
+        <v>6.721170538296987</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
-        <v>47.153136</v>
+        <v>29.342164</v>
       </c>
       <c r="N4" t="n">
-        <v>45.217867</v>
+        <v>28.028816</v>
       </c>
       <c r="O4" t="n">
-        <v>0.503104</v>
+        <v>0.507053</v>
       </c>
       <c r="P4" t="n">
-        <v>1.432164</v>
+        <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>870</v>
+        <v>499.8</v>
       </c>
       <c r="R4" t="n">
-        <v>193526.9</v>
+        <v>65667.39999999999</v>
       </c>
       <c r="S4" t="n">
-        <v>50310.4</v>
+        <v>25352.7</v>
       </c>
       <c r="T4" t="n">
-        <v>143216.4</v>
+        <v>40314.7</v>
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="n">
-        <v>1.187152322196748</v>
+        <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.06434247689799896</v>
+        <v>0.1120195089716164</v>
       </c>
       <c r="X4" t="n">
-        <v>0.842351888045474</v>
+        <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>222.4447126436781</v>
+        <v>131.3873549419768</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.2892515453989037</v>
+        <v>0.8525897261657063</v>
       </c>
     </row>
     <row r="5">
@@ -864,7 +864,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K5" t="n">
-        <v>10.73811542729593</v>
+        <v>10.91307453812764</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -880,7 +880,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q5" t="n">
-        <v>299.4</v>
+        <v>294.6</v>
       </c>
       <c r="R5" t="n">
         <v>35584.1</v>
@@ -896,13 +896,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1789685904549322</v>
+        <v>0.1818845756354606</v>
       </c>
       <c r="X5" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y5" t="n">
-        <v>118.8513694054776</v>
+        <v>120.7878479293958</v>
       </c>
       <c r="Z5" t="n">
         <v>1.505818497087371</v>
@@ -954,7 +954,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>4.476084392812517</v>
+        <v>4.391351931055572</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -970,7 +970,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q6" t="n">
-        <v>715.2</v>
+        <v>729</v>
       </c>
       <c r="R6" t="n">
         <v>78110.8</v>
@@ -986,13 +986,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07460140654687528</v>
+        <v>0.0731891988509262</v>
       </c>
       <c r="X6" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y6" t="n">
-        <v>109.2153243847875</v>
+        <v>107.1478737997257</v>
       </c>
       <c r="Z6" t="n">
         <v>0.6830672066132366</v>
@@ -1044,7 +1044,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K7" t="n">
-        <v>5.32032587538944</v>
+        <v>5.347061181295921</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1060,7 +1060,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q7" t="n">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="R7" t="n">
         <v>60537.6</v>
@@ -1076,13 +1076,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W7" t="n">
-        <v>0.08867209792315733</v>
+        <v>0.089117686354932</v>
       </c>
       <c r="X7" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y7" t="n">
-        <v>100.896</v>
+        <v>101.4030150753769</v>
       </c>
       <c r="Z7" t="n">
         <v>0.8788465144619939</v>
@@ -1306,7 +1306,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K10" t="n">
-        <v>9.158448900503181</v>
+        <v>9.222945019520811</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1322,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q10" t="n">
-        <v>343.2</v>
+        <v>340.8</v>
       </c>
       <c r="R10" t="n">
         <v>16901.2</v>
@@ -1338,13 +1338,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W10" t="n">
-        <v>0.1526408150083864</v>
+        <v>0.1537157503253468</v>
       </c>
       <c r="X10" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y10" t="n">
-        <v>49.24592074592075</v>
+        <v>49.59272300469485</v>
       </c>
       <c r="Z10" t="n">
         <v>3.099562617499243</v>
@@ -1393,51 +1393,51 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>51.8522867021152</v>
+        <v>51.8955544183089</v>
       </c>
       <c r="K11" t="n">
-        <v>7.035588426338562</v>
+        <v>6.937908344693702</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
-        <v>15.934687</v>
+        <v>15.865464</v>
       </c>
       <c r="N11" t="n">
-        <v>15.197443</v>
+        <v>15.117367</v>
       </c>
       <c r="O11" t="n">
-        <v>0.260605</v>
+        <v>0.268563</v>
       </c>
       <c r="P11" t="n">
-        <v>0.476639</v>
+        <v>0.479533</v>
       </c>
       <c r="Q11" t="n">
-        <v>442.2</v>
+        <v>448.8</v>
       </c>
       <c r="R11" t="n">
-        <v>73724.39999999999</v>
+        <v>74809.60000000001</v>
       </c>
       <c r="S11" t="n">
-        <v>26060.5</v>
+        <v>26856.3</v>
       </c>
       <c r="T11" t="n">
-        <v>47663.9</v>
+        <v>47953.3</v>
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>3.25405115909181</v>
+        <v>3.270976154136362</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1172598071056427</v>
+        <v>0.115631805744895</v>
       </c>
       <c r="X11" t="n">
-        <v>0.3073092434966803</v>
+        <v>0.3057191348629781</v>
       </c>
       <c r="Y11" t="n">
-        <v>166.7218453188602</v>
+        <v>166.6880570409982</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.7033259911523893</v>
+        <v>0.6937018032218979</v>
       </c>
     </row>
     <row r="12">
@@ -1486,7 +1486,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K12" t="n">
-        <v>5.246281346270657</v>
+        <v>5.18851448460001</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1502,7 +1502,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q12" t="n">
-        <v>592.8000000000001</v>
+        <v>599.4</v>
       </c>
       <c r="R12" t="n">
         <v>38128.4</v>
@@ -1518,13 +1518,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W12" t="n">
-        <v>0.08743802243784428</v>
+        <v>0.08647524141000017</v>
       </c>
       <c r="X12" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y12" t="n">
-        <v>64.31916329284749</v>
+        <v>63.61094427761095</v>
       </c>
       <c r="Z12" t="n">
         <v>1.359439674918279</v>
@@ -1576,7 +1576,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K13" t="n">
-        <v>7.658011269421735</v>
+        <v>7.221067683478753</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1592,7 +1592,7 @@
         <v>0.145035</v>
       </c>
       <c r="Q13" t="n">
-        <v>376.8</v>
+        <v>399.6</v>
       </c>
       <c r="R13" t="n">
         <v>60200.2</v>
@@ -1608,13 +1608,13 @@
         <v>6.17518114688861</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1276335211570289</v>
+        <v>0.1203511280579792</v>
       </c>
       <c r="X13" t="n">
         <v>0.161938569284539</v>
       </c>
       <c r="Y13" t="n">
-        <v>159.7669851380042</v>
+        <v>150.6511511511511</v>
       </c>
       <c r="Z13" t="n">
         <v>0.7988729401558218</v>
@@ -1666,7 +1666,7 @@
         <v>47.6305176437724</v>
       </c>
       <c r="K14" t="n">
-        <v>7.572419339232496</v>
+        <v>8.460127467810374</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1682,7 @@
         <v>0.208445</v>
       </c>
       <c r="Q14" t="n">
-        <v>377.4</v>
+        <v>337.8</v>
       </c>
       <c r="R14" t="n">
         <v>30999.6</v>
@@ -1698,13 +1698,13 @@
         <v>8.555202665891516</v>
       </c>
       <c r="W14" t="n">
-        <v>0.1262069889872083</v>
+        <v>0.1410021244635062</v>
       </c>
       <c r="X14" t="n">
         <v>0.1168879381416492</v>
       </c>
       <c r="Y14" t="n">
-        <v>82.13990461049285</v>
+        <v>91.76909413854351</v>
       </c>
       <c r="Z14" t="n">
         <v>1.53648813674281</v>
@@ -1846,7 +1846,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>1.858171140434749</v>
+        <v>1.996733040130961</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1862,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1495.8</v>
+        <v>1392</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1878,13 +1878,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.03096951900724582</v>
+        <v>0.03327888400218269</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>42.97078486428667</v>
+        <v>46.17507183908046</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1936,7 +1936,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.236797617049349</v>
+        <v>1.251797367642009</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1952,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2203.2</v>
+        <v>2176.8</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1968,13 +1968,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.02061329361748915</v>
+        <v>0.02086328946070016</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>48.89714960058097</v>
+        <v>49.4901690554943</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -2026,7 +2026,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>3.500968912088663</v>
+        <v>3.200671364232595</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2042,7 +2042,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q18" t="n">
-        <v>767.4</v>
+        <v>839.4</v>
       </c>
       <c r="R18" t="n">
         <v>71127.60000000001</v>
@@ -2058,13 +2058,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W18" t="n">
-        <v>0.05834948186814438</v>
+        <v>0.05334452273720992</v>
       </c>
       <c r="X18" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y18" t="n">
-        <v>92.68647380766225</v>
+        <v>84.73624017155112</v>
       </c>
       <c r="Z18" t="n">
         <v>0.629536106737947</v>
@@ -2116,7 +2116,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>3.706297026623847</v>
+        <v>3.715743832978879</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2132,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q19" t="n">
-        <v>708</v>
+        <v>706.1999999999999</v>
       </c>
       <c r="R19" t="n">
         <v>64144.3</v>
@@ -2148,13 +2148,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W19" t="n">
-        <v>0.06177161711039746</v>
+        <v>0.06192906388298131</v>
       </c>
       <c r="X19" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y19" t="n">
-        <v>90.59929378531073</v>
+        <v>90.83021806853584</v>
       </c>
       <c r="Z19" t="n">
         <v>0.6818112429968274</v>
@@ -2296,7 +2296,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K21" t="n">
-        <v>2.346097986164703</v>
+        <v>2.555468588841993</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q21" t="n">
-        <v>1069.2</v>
+        <v>981.5999999999999</v>
       </c>
       <c r="R21" t="n">
         <v>68673.2</v>
@@ -2328,13 +2328,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W21" t="n">
-        <v>0.03910163310274504</v>
+        <v>0.04259114314736655</v>
       </c>
       <c r="X21" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y21" t="n">
-        <v>64.22858211747101</v>
+        <v>69.96047269763652</v>
       </c>
       <c r="Z21" t="n">
         <v>0.6087886703030441</v>
@@ -2386,7 +2386,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K22" t="n">
-        <v>8.218118910961927</v>
+        <v>8.994776302547342</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q22" t="n">
-        <v>298.8</v>
+        <v>273</v>
       </c>
       <c r="R22" t="n">
         <v>71002.60000000001</v>
@@ -2418,13 +2418,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W22" t="n">
-        <v>0.1369686485160321</v>
+        <v>0.149912938375789</v>
       </c>
       <c r="X22" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y22" t="n">
-        <v>237.6258366800536</v>
+        <v>260.0827838827839</v>
       </c>
       <c r="Z22" t="n">
         <v>0.5764046975264343</v>
@@ -2476,7 +2476,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K23" t="n">
-        <v>7.587724513947499</v>
+        <v>7.782281552766665</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2492,7 +2492,7 @@
         <v>0.07520300000000001</v>
       </c>
       <c r="Q23" t="n">
-        <v>312</v>
+        <v>304.2</v>
       </c>
       <c r="R23" t="n">
         <v>88574</v>
@@ -2508,13 +2508,13 @@
         <v>12.61396912906789</v>
       </c>
       <c r="W23" t="n">
-        <v>0.1264620752324583</v>
+        <v>0.1297046925461111</v>
       </c>
       <c r="X23" t="n">
         <v>0.07927718783579227</v>
       </c>
       <c r="Y23" t="n">
-        <v>283.8910256410256</v>
+        <v>291.1702827087442</v>
       </c>
       <c r="Z23" t="n">
         <v>0.4454599258532639</v>
@@ -2566,7 +2566,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K24" t="n">
-        <v>5.758990738213565</v>
+        <v>6.099922989915808</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2582,7 +2582,7 @@
         <v>0.019426</v>
       </c>
       <c r="Q24" t="n">
-        <v>397.2</v>
+        <v>375</v>
       </c>
       <c r="R24" t="n">
         <v>49956</v>
@@ -2598,13 +2598,13 @@
         <v>117.2034329494868</v>
       </c>
       <c r="W24" t="n">
-        <v>0.09598317897022608</v>
+        <v>0.1016653831652635</v>
       </c>
       <c r="X24" t="n">
         <v>0.008532173289079235</v>
       </c>
       <c r="Y24" t="n">
-        <v>125.7703927492447</v>
+        <v>133.216</v>
       </c>
       <c r="Z24" t="n">
         <v>0.7631619562609856</v>
@@ -2656,7 +2656,7 @@
         <v>33.6962858057476</v>
       </c>
       <c r="K25" t="n">
-        <v>1.697545884420534</v>
+        <v>1.830325138823878</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2672,7 +2672,7 @@
         <v>0.143133</v>
       </c>
       <c r="Q25" t="n">
-        <v>1191</v>
+        <v>1104.6</v>
       </c>
       <c r="R25" t="n">
         <v>66797.5</v>
@@ -2688,13 +2688,13 @@
         <v>13.44796592290856</v>
       </c>
       <c r="W25" t="n">
-        <v>0.0282924314070089</v>
+        <v>0.03050541898039797</v>
       </c>
       <c r="X25" t="n">
         <v>0.0743606881317645</v>
       </c>
       <c r="Y25" t="n">
-        <v>56.08522250209908</v>
+        <v>60.47211660329531</v>
       </c>
       <c r="Z25" t="n">
         <v>0.504454295531234</v>
@@ -2808,7 +2808,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K27" t="n">
-        <v>3.196968624029715</v>
+        <v>3.172670274009946</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2824,7 +2824,7 @@
         <v>0.026182</v>
       </c>
       <c r="Q27" t="n">
-        <v>548.4000000000001</v>
+        <v>552.6</v>
       </c>
       <c r="R27" t="n">
         <v>48192</v>
@@ -2840,13 +2840,13 @@
         <v>15.27539782478406</v>
       </c>
       <c r="W27" t="n">
-        <v>0.05328281040049525</v>
+        <v>0.05287783790016576</v>
       </c>
       <c r="X27" t="n">
         <v>0.06546474346988973</v>
       </c>
       <c r="Y27" t="n">
-        <v>87.87746170678335</v>
+        <v>87.20955483170466</v>
       </c>
       <c r="Z27" t="n">
         <v>0.6063307856829266</v>
@@ -2898,7 +2898,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K28" t="n">
-        <v>8.82854455828212</v>
+        <v>8.923136107120857</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2914,7 +2914,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q28" t="n">
-        <v>169.8</v>
+        <v>168</v>
       </c>
       <c r="R28" t="n">
         <v>34656</v>
@@ -2930,13 +2930,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W28" t="n">
-        <v>0.147142409304702</v>
+        <v>0.148718935118681</v>
       </c>
       <c r="X28" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y28" t="n">
-        <v>204.0989399293286</v>
+        <v>206.2857142857143</v>
       </c>
       <c r="Z28" t="n">
         <v>0.7209366660877885</v>
@@ -2988,7 +2988,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K29" t="n">
-        <v>8.130465369604895</v>
+        <v>8.367851219812335</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -3004,7 +3004,7 @@
         <v>0.037626</v>
       </c>
       <c r="Q29" t="n">
-        <v>169.2</v>
+        <v>164.4</v>
       </c>
       <c r="R29" t="n">
         <v>28366.1</v>
@@ -3020,13 +3020,13 @@
         <v>31.96610467696488</v>
       </c>
       <c r="W29" t="n">
-        <v>0.1355077561600816</v>
+        <v>0.1394641869968723</v>
       </c>
       <c r="X29" t="n">
         <v>0.0312831360000085</v>
       </c>
       <c r="Y29" t="n">
-        <v>167.6483451536643</v>
+        <v>172.5431873479318</v>
       </c>
       <c r="Z29" t="n">
         <v>0.8082856769977473</v>
@@ -3078,7 +3078,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K30" t="n">
-        <v>10.46432192152485</v>
+        <v>9.985952919398001</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3094,7 +3094,7 @@
         <v>0.01289</v>
       </c>
       <c r="Q30" t="n">
-        <v>100.2</v>
+        <v>105</v>
       </c>
       <c r="R30" t="n">
         <v>13925.2</v>
@@ -3110,13 +3110,13 @@
         <v>76.71116733805002</v>
       </c>
       <c r="W30" t="n">
-        <v>0.1744053653587475</v>
+        <v>0.1664325486566333</v>
       </c>
       <c r="X30" t="n">
         <v>0.01303591165016704</v>
       </c>
       <c r="Y30" t="n">
-        <v>138.9740518962076</v>
+        <v>132.6209523809524</v>
       </c>
       <c r="Z30" t="n">
         <v>1.254949128841704</v>
@@ -3168,7 +3168,7 @@
         <v>14.1889227802691</v>
       </c>
       <c r="K31" t="n">
-        <v>5.791397053171061</v>
+        <v>5.744503149906518</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3184,7 +3184,7 @@
         <v>0.105148</v>
       </c>
       <c r="Q31" t="n">
-        <v>147</v>
+        <v>148.2</v>
       </c>
       <c r="R31" t="n">
         <v>26085.5</v>
@@ -3200,13 +3200,13 @@
         <v>9.066560752338283</v>
       </c>
       <c r="W31" t="n">
-        <v>0.0965232842195177</v>
+        <v>0.09574171916510862</v>
       </c>
       <c r="X31" t="n">
         <v>0.1102954060879257</v>
       </c>
       <c r="Y31" t="n">
-        <v>177.452380952381</v>
+        <v>176.0155195681511</v>
       </c>
       <c r="Z31" t="n">
         <v>0.5439390765087539</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-03)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -556,7 +556,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (Adaptive Reasoning, Max Effort, Default Fallback)</t>
+          <t>Claude Opus 5.5 (Max, Default Fallback)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.287378706123237</v>
+        <v>4.303388335346997</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>806.4</v>
+        <v>803.4000000000001</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07145631176872061</v>
+        <v>0.07172313892244996</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>147.7752976190476</v>
+        <v>148.3271097834204</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -646,7 +646,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5.5 (Adaptive Reasoning, Max Effort, Default Fallback)</t>
+          <t>Claude Sonnet 5.5 (Max, Default Fallback)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.753359829629987</v>
+        <v>3.686644414620105</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>895.2</v>
+        <v>911.4</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.06255599716049977</v>
+        <v>0.06144407357700175</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>220.5433422698838</v>
+        <v>216.623217028747</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -736,7 +736,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (Adaptive Reasoning, Xhigh Effort, Default Fallback)</t>
+          <t>Claude Opus 5.5 (Xhigh, Default Fallback)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.721170538296987</v>
+        <v>6.617890139954361</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>499.8</v>
+        <v>507.6</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1120195089716164</v>
+        <v>0.1102981689992394</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>131.3873549419768</v>
+        <v>129.3684003152088</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -826,7 +826,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (Adaptive Reasoning, High Effort, Default Fallback)</t>
+          <t>Claude Opus 5.5 (High, Default Fallback)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (Adaptive Reasoning, Max Effort, Default Fallback)</t>
+          <t>Claude Fable 5.1 (Max, Default Fallback)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -954,7 +954,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>4.391351931055572</v>
+        <v>4.227807128551918</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -970,7 +970,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q6" t="n">
-        <v>729</v>
+        <v>757.1999999999999</v>
       </c>
       <c r="R6" t="n">
         <v>78110.8</v>
@@ -986,13 +986,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W6" t="n">
-        <v>0.0731891988509262</v>
+        <v>0.07046345214253197</v>
       </c>
       <c r="X6" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y6" t="n">
-        <v>107.1478737997257</v>
+        <v>103.1574220813524</v>
       </c>
       <c r="Z6" t="n">
         <v>0.6830672066132366</v>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (Adaptive Reasoning, Xhigh Effort, Default Fallback)</t>
+          <t>Claude Fable 5.1 (Xhigh, Default Fallback)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1044,7 +1044,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K7" t="n">
-        <v>5.347061181295921</v>
+        <v>5.170384718551449</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1060,7 +1060,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q7" t="n">
-        <v>597</v>
+        <v>617.4</v>
       </c>
       <c r="R7" t="n">
         <v>60537.6</v>
@@ -1076,13 +1076,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W7" t="n">
-        <v>0.089117686354932</v>
+        <v>0.08617307864252415</v>
       </c>
       <c r="X7" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y7" t="n">
-        <v>101.4030150753769</v>
+        <v>98.05247813411079</v>
       </c>
       <c r="Z7" t="n">
         <v>0.8788465144619939</v>
@@ -1134,7 +1134,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K8" t="n">
-        <v>6.026735628777232</v>
+        <v>6.535194714083499</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1150,7 +1150,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q8" t="n">
-        <v>524.4</v>
+        <v>483.6</v>
       </c>
       <c r="R8" t="n">
         <v>27205.5</v>
@@ -1166,13 +1166,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W8" t="n">
-        <v>0.1004455938129539</v>
+        <v>0.1089199119013917</v>
       </c>
       <c r="X8" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y8" t="n">
-        <v>51.87929061784897</v>
+        <v>56.2562034739454</v>
       </c>
       <c r="Z8" t="n">
         <v>1.936140464079432</v>
@@ -1306,7 +1306,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K10" t="n">
-        <v>9.222945019520811</v>
+        <v>9.271916409004991</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1322,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q10" t="n">
-        <v>340.8</v>
+        <v>339</v>
       </c>
       <c r="R10" t="n">
         <v>16901.2</v>
@@ -1338,13 +1338,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W10" t="n">
-        <v>0.1537157503253468</v>
+        <v>0.1545319401500832</v>
       </c>
       <c r="X10" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y10" t="n">
-        <v>49.59272300469485</v>
+        <v>49.85604719764012</v>
       </c>
       <c r="Z10" t="n">
         <v>3.099562617499243</v>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5.5 (Adaptive Reasoning, Xhigh Effort, Default Fallback)</t>
+          <t>Claude Sonnet 5.5 (Xhigh, Default Fallback)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1396,7 +1396,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K11" t="n">
-        <v>6.937908344693702</v>
+        <v>6.837358948393795</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1412,7 +1412,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q11" t="n">
-        <v>448.8</v>
+        <v>455.4</v>
       </c>
       <c r="R11" t="n">
         <v>74809.60000000001</v>
@@ -1428,13 +1428,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W11" t="n">
-        <v>0.115631805744895</v>
+        <v>0.1139559824732299</v>
       </c>
       <c r="X11" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y11" t="n">
-        <v>166.6880570409982</v>
+        <v>164.2722880983751</v>
       </c>
       <c r="Z11" t="n">
         <v>0.6937018032218979</v>
@@ -1486,7 +1486,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K12" t="n">
-        <v>5.18851448460001</v>
+        <v>4.25211318303151</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1502,7 +1502,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q12" t="n">
-        <v>599.4</v>
+        <v>731.4</v>
       </c>
       <c r="R12" t="n">
         <v>38128.4</v>
@@ -1518,13 +1518,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W12" t="n">
-        <v>0.08647524141000017</v>
+        <v>0.07086855305052515</v>
       </c>
       <c r="X12" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y12" t="n">
-        <v>63.61094427761095</v>
+        <v>52.13070823079027</v>
       </c>
       <c r="Z12" t="n">
         <v>1.359439674918279</v>
@@ -1576,7 +1576,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K13" t="n">
-        <v>7.221067683478753</v>
+        <v>5.711675863654216</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1592,7 +1592,7 @@
         <v>0.145035</v>
       </c>
       <c r="Q13" t="n">
-        <v>399.6</v>
+        <v>505.2</v>
       </c>
       <c r="R13" t="n">
         <v>60200.2</v>
@@ -1608,13 +1608,13 @@
         <v>6.17518114688861</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1203511280579792</v>
+        <v>0.09519459772757027</v>
       </c>
       <c r="X13" t="n">
         <v>0.161938569284539</v>
       </c>
       <c r="Y13" t="n">
-        <v>150.6511511511511</v>
+        <v>119.1611243072051</v>
       </c>
       <c r="Z13" t="n">
         <v>0.7988729401558218</v>
@@ -1666,7 +1666,7 @@
         <v>47.6305176437724</v>
       </c>
       <c r="K14" t="n">
-        <v>8.460127467810374</v>
+        <v>8.707590062846874</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1682,7 @@
         <v>0.208445</v>
       </c>
       <c r="Q14" t="n">
-        <v>337.8</v>
+        <v>328.2</v>
       </c>
       <c r="R14" t="n">
         <v>30999.6</v>
@@ -1698,13 +1698,13 @@
         <v>8.555202665891516</v>
       </c>
       <c r="W14" t="n">
-        <v>0.1410021244635062</v>
+        <v>0.1451265010474479</v>
       </c>
       <c r="X14" t="n">
         <v>0.1168879381416492</v>
       </c>
       <c r="Y14" t="n">
-        <v>91.76909413854351</v>
+        <v>94.45338208409507</v>
       </c>
       <c r="Z14" t="n">
         <v>1.53648813674281</v>
@@ -1756,7 +1756,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>2.634517903019206</v>
+        <v>2.521528264398947</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1772,7 +1772,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>1057.8</v>
+        <v>1105.2</v>
       </c>
       <c r="R15" t="n">
         <v>80561.39999999999</v>
@@ -1788,13 +1788,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.04390863171698677</v>
+        <v>0.04202547107331578</v>
       </c>
       <c r="X15" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>76.15938740782757</v>
+        <v>72.8930510314875</v>
       </c>
       <c r="Z15" t="n">
         <v>0.5765360412086756</v>
@@ -1846,7 +1846,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>1.996733040130961</v>
+        <v>1.830272877559791</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1862,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1392</v>
+        <v>1518.6</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1878,13 +1878,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.03327888400218269</v>
+        <v>0.03050454795932984</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>46.17507183908046</v>
+        <v>42.32562886869485</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1936,7 +1936,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.251797367642009</v>
+        <v>1.200190499419981</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1952,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2176.8</v>
+        <v>2270.4</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1968,13 +1968,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.02086328946070016</v>
+        <v>0.02000317499033303</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>49.4901690554943</v>
+        <v>47.44987667371388</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -2026,7 +2026,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>3.200671364232595</v>
+        <v>3.287620586315272</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2042,7 +2042,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q18" t="n">
-        <v>839.4</v>
+        <v>817.1999999999999</v>
       </c>
       <c r="R18" t="n">
         <v>71127.60000000001</v>
@@ -2058,13 +2058,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W18" t="n">
-        <v>0.05334452273720992</v>
+        <v>0.05479367643858787</v>
       </c>
       <c r="X18" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y18" t="n">
-        <v>84.73624017155112</v>
+        <v>87.03817914831131</v>
       </c>
       <c r="Z18" t="n">
         <v>0.629536106737947</v>
@@ -2116,7 +2116,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>3.715743832978879</v>
+        <v>3.799678967346777</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2132,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q19" t="n">
-        <v>706.1999999999999</v>
+        <v>690.6</v>
       </c>
       <c r="R19" t="n">
         <v>64144.3</v>
@@ -2148,13 +2148,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W19" t="n">
-        <v>0.06192906388298131</v>
+        <v>0.06332798278911295</v>
       </c>
       <c r="X19" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y19" t="n">
-        <v>90.83021806853584</v>
+        <v>92.8819866782508</v>
       </c>
       <c r="Z19" t="n">
         <v>0.6818112429968274</v>
@@ -2206,7 +2206,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>2.054374314414619</v>
+        <v>2.125491123933603</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2222,7 +2222,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q20" t="n">
-        <v>1273.2</v>
+        <v>1230.6</v>
       </c>
       <c r="R20" t="n">
         <v>48455.2</v>
@@ -2238,13 +2238,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W20" t="n">
-        <v>0.03423957190691031</v>
+        <v>0.03542485206556005</v>
       </c>
       <c r="X20" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y20" t="n">
-        <v>38.05780710021992</v>
+        <v>39.37526409881358</v>
       </c>
       <c r="Z20" t="n">
         <v>0.8996727482680539</v>
@@ -2296,7 +2296,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K21" t="n">
-        <v>2.555468588841993</v>
+        <v>2.473814562926332</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q21" t="n">
-        <v>981.5999999999999</v>
+        <v>1014</v>
       </c>
       <c r="R21" t="n">
         <v>68673.2</v>
@@ -2328,13 +2328,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W21" t="n">
-        <v>0.04259114314736655</v>
+        <v>0.04123024271543886</v>
       </c>
       <c r="X21" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y21" t="n">
-        <v>69.96047269763652</v>
+        <v>67.7250493096647</v>
       </c>
       <c r="Z21" t="n">
         <v>0.6087886703030441</v>
@@ -2386,7 +2386,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K22" t="n">
-        <v>8.994776302547342</v>
+        <v>8.185246435318081</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q22" t="n">
-        <v>273</v>
+        <v>300</v>
       </c>
       <c r="R22" t="n">
         <v>71002.60000000001</v>
@@ -2418,13 +2418,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W22" t="n">
-        <v>0.149912938375789</v>
+        <v>0.136420773921968</v>
       </c>
       <c r="X22" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y22" t="n">
-        <v>260.0827838827839</v>
+        <v>236.6753333333334</v>
       </c>
       <c r="Z22" t="n">
         <v>0.5764046975264343</v>
@@ -2476,7 +2476,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K23" t="n">
-        <v>7.782281552766665</v>
+        <v>7.721363497559099</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2492,7 +2492,7 @@
         <v>0.07520300000000001</v>
       </c>
       <c r="Q23" t="n">
-        <v>304.2</v>
+        <v>306.6</v>
       </c>
       <c r="R23" t="n">
         <v>88574</v>
@@ -2508,13 +2508,13 @@
         <v>12.61396912906789</v>
       </c>
       <c r="W23" t="n">
-        <v>0.1297046925461111</v>
+        <v>0.128689391625985</v>
       </c>
       <c r="X23" t="n">
         <v>0.07927718783579227</v>
       </c>
       <c r="Y23" t="n">
-        <v>291.1702827087442</v>
+        <v>288.8910632746249</v>
       </c>
       <c r="Z23" t="n">
         <v>0.4454599258532639</v>
@@ -2566,48 +2566,48 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K24" t="n">
-        <v>6.099922989915808</v>
+        <v>5.829437108099969</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>0.325285</v>
+        <v>0.326276</v>
       </c>
       <c r="N24" t="n">
-        <v>0.300307</v>
+        <v>0.30127</v>
       </c>
       <c r="O24" t="n">
-        <v>0.005552</v>
+        <v>0.005561</v>
       </c>
       <c r="P24" t="n">
-        <v>0.019426</v>
+        <v>0.019445</v>
       </c>
       <c r="Q24" t="n">
-        <v>375</v>
+        <v>392.4</v>
       </c>
       <c r="R24" t="n">
-        <v>49956</v>
+        <v>50011.7</v>
       </c>
       <c r="S24" t="n">
-        <v>11104.7</v>
+        <v>11122</v>
       </c>
       <c r="T24" t="n">
-        <v>38851.3</v>
+        <v>38889.7</v>
       </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="n">
-        <v>117.2034329494868</v>
+        <v>116.8474502782117</v>
       </c>
       <c r="W24" t="n">
-        <v>0.1016653831652635</v>
+        <v>0.09715728513499949</v>
       </c>
       <c r="X24" t="n">
-        <v>0.008532173289079235</v>
+        <v>0.008558167059863248</v>
       </c>
       <c r="Y24" t="n">
-        <v>133.216</v>
+        <v>127.4508154943935</v>
       </c>
       <c r="Z24" t="n">
-        <v>0.7631619562609856</v>
+        <v>0.7623119927331765</v>
       </c>
     </row>
     <row r="25">
@@ -2656,7 +2656,7 @@
         <v>33.6962858057476</v>
       </c>
       <c r="K25" t="n">
-        <v>1.830325138823878</v>
+        <v>1.751366206119938</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2672,7 +2672,7 @@
         <v>0.143133</v>
       </c>
       <c r="Q25" t="n">
-        <v>1104.6</v>
+        <v>1154.4</v>
       </c>
       <c r="R25" t="n">
         <v>66797.5</v>
@@ -2688,13 +2688,13 @@
         <v>13.44796592290856</v>
       </c>
       <c r="W25" t="n">
-        <v>0.03050541898039797</v>
+        <v>0.02918943676866563</v>
       </c>
       <c r="X25" t="n">
         <v>0.0743606881317645</v>
       </c>
       <c r="Y25" t="n">
-        <v>60.47211660329531</v>
+        <v>57.86339223839224</v>
       </c>
       <c r="Z25" t="n">
         <v>0.504454295531234</v>
@@ -2808,7 +2808,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K27" t="n">
-        <v>3.172670274009946</v>
+        <v>2.88453042681457</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2824,7 +2824,7 @@
         <v>0.026182</v>
       </c>
       <c r="Q27" t="n">
-        <v>552.6</v>
+        <v>607.8000000000001</v>
       </c>
       <c r="R27" t="n">
         <v>48192</v>
@@ -2840,13 +2840,13 @@
         <v>15.27539782478406</v>
       </c>
       <c r="W27" t="n">
-        <v>0.05287783790016576</v>
+        <v>0.04807550711357617</v>
       </c>
       <c r="X27" t="n">
         <v>0.06546474346988973</v>
       </c>
       <c r="Y27" t="n">
-        <v>87.20955483170466</v>
+        <v>79.28923988153997</v>
       </c>
       <c r="Z27" t="n">
         <v>0.6063307856829266</v>
@@ -2898,7 +2898,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K28" t="n">
-        <v>8.923136107120857</v>
+        <v>8.766589859627508</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2914,7 +2914,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q28" t="n">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="R28" t="n">
         <v>34656</v>
@@ -2930,13 +2930,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W28" t="n">
-        <v>0.148718935118681</v>
+        <v>0.1461098309937918</v>
       </c>
       <c r="X28" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y28" t="n">
-        <v>206.2857142857143</v>
+        <v>202.6666666666667</v>
       </c>
       <c r="Z28" t="n">
         <v>0.7209366660877885</v>
@@ -2988,7 +2988,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K29" t="n">
-        <v>8.367851219812335</v>
+        <v>8.818427823956076</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -3004,7 +3004,7 @@
         <v>0.037626</v>
       </c>
       <c r="Q29" t="n">
-        <v>164.4</v>
+        <v>156</v>
       </c>
       <c r="R29" t="n">
         <v>28366.1</v>
@@ -3020,13 +3020,13 @@
         <v>31.96610467696488</v>
       </c>
       <c r="W29" t="n">
-        <v>0.1394641869968723</v>
+        <v>0.1469737970659346</v>
       </c>
       <c r="X29" t="n">
         <v>0.0312831360000085</v>
       </c>
       <c r="Y29" t="n">
-        <v>172.5431873479318</v>
+        <v>181.8339743589744</v>
       </c>
       <c r="Z29" t="n">
         <v>0.8082856769977473</v>
@@ -3078,7 +3078,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K30" t="n">
-        <v>9.985952919398001</v>
+        <v>9.654926855771548</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3094,7 +3094,7 @@
         <v>0.01289</v>
       </c>
       <c r="Q30" t="n">
-        <v>105</v>
+        <v>108.6</v>
       </c>
       <c r="R30" t="n">
         <v>13925.2</v>
@@ -3110,13 +3110,13 @@
         <v>76.71116733805002</v>
       </c>
       <c r="W30" t="n">
-        <v>0.1664325486566333</v>
+        <v>0.1609154475961924</v>
       </c>
       <c r="X30" t="n">
         <v>0.01303591165016704</v>
       </c>
       <c r="Y30" t="n">
-        <v>132.6209523809524</v>
+        <v>128.2246777163904</v>
       </c>
       <c r="Z30" t="n">
         <v>1.254949128841704</v>
@@ -3168,7 +3168,7 @@
         <v>14.1889227802691</v>
       </c>
       <c r="K31" t="n">
-        <v>5.744503149906518</v>
+        <v>5.542547961042617</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3184,7 +3184,7 @@
         <v>0.105148</v>
       </c>
       <c r="Q31" t="n">
-        <v>148.2</v>
+        <v>153.6</v>
       </c>
       <c r="R31" t="n">
         <v>26085.5</v>
@@ -3200,13 +3200,13 @@
         <v>9.066560752338283</v>
       </c>
       <c r="W31" t="n">
-        <v>0.09574171916510862</v>
+        <v>0.09237579935071029</v>
       </c>
       <c r="X31" t="n">
         <v>0.1102954060879257</v>
       </c>
       <c r="Y31" t="n">
-        <v>176.0155195681511</v>
+        <v>169.8274739583333</v>
       </c>
       <c r="Z31" t="n">
         <v>0.5439390765087539</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-04)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.686644414620105</v>
+        <v>3.605932302516381</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>911.4</v>
+        <v>931.8</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.06144407357700175</v>
+        <v>0.06009887170860635</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>216.623217028747</v>
+        <v>211.88066108607</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.617890139954361</v>
+        <v>6.571285279813838</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>507.6</v>
+        <v>511.2</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1102981689992394</v>
+        <v>0.1095214213302306</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>129.3684003152088</v>
+        <v>128.4573552425665</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -864,7 +864,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K5" t="n">
-        <v>10.91307453812764</v>
+        <v>10.73811542729593</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -880,7 +880,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q5" t="n">
-        <v>294.6</v>
+        <v>299.4</v>
       </c>
       <c r="R5" t="n">
         <v>35584.1</v>
@@ -896,13 +896,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1818845756354606</v>
+        <v>0.1789685904549322</v>
       </c>
       <c r="X5" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y5" t="n">
-        <v>120.7878479293958</v>
+        <v>118.8513694054776</v>
       </c>
       <c r="Z5" t="n">
         <v>1.505818497087371</v>
@@ -954,7 +954,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>4.227807128551918</v>
+        <v>4.231159870128883</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -970,7 +970,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q6" t="n">
-        <v>757.1999999999999</v>
+        <v>756.5999999999999</v>
       </c>
       <c r="R6" t="n">
         <v>78110.8</v>
@@ -986,13 +986,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07046345214253197</v>
+        <v>0.0705193311688147</v>
       </c>
       <c r="X6" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y6" t="n">
-        <v>103.1574220813524</v>
+        <v>103.2392281258261</v>
       </c>
       <c r="Z6" t="n">
         <v>0.6830672066132366</v>
@@ -1044,7 +1044,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K7" t="n">
-        <v>5.170384718551449</v>
+        <v>4.995611150600413</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1060,7 +1060,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q7" t="n">
-        <v>617.4</v>
+        <v>639</v>
       </c>
       <c r="R7" t="n">
         <v>60537.6</v>
@@ -1076,13 +1076,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W7" t="n">
-        <v>0.08617307864252415</v>
+        <v>0.08326018584334022</v>
       </c>
       <c r="X7" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y7" t="n">
-        <v>98.05247813411079</v>
+        <v>94.73802816901409</v>
       </c>
       <c r="Z7" t="n">
         <v>0.8788465144619939</v>
@@ -1134,7 +1134,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K8" t="n">
-        <v>6.535194714083499</v>
+        <v>6.995175218527623</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1150,7 +1150,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q8" t="n">
-        <v>483.6</v>
+        <v>451.8</v>
       </c>
       <c r="R8" t="n">
         <v>27205.5</v>
@@ -1166,13 +1166,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W8" t="n">
-        <v>0.1089199119013917</v>
+        <v>0.116586253642127</v>
       </c>
       <c r="X8" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y8" t="n">
-        <v>56.2562034739454</v>
+        <v>60.21580345285525</v>
       </c>
       <c r="Z8" t="n">
         <v>1.936140464079432</v>
@@ -1306,7 +1306,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K10" t="n">
-        <v>9.271916409004991</v>
+        <v>10.19189255075451</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1322,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q10" t="n">
-        <v>339</v>
+        <v>308.4</v>
       </c>
       <c r="R10" t="n">
         <v>16901.2</v>
@@ -1338,13 +1338,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W10" t="n">
-        <v>0.1545319401500832</v>
+        <v>0.1698648758459086</v>
       </c>
       <c r="X10" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y10" t="n">
-        <v>49.85604719764012</v>
+        <v>54.80285343709469</v>
       </c>
       <c r="Z10" t="n">
         <v>3.099562617499243</v>
@@ -1396,7 +1396,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K11" t="n">
-        <v>6.837358948393795</v>
+        <v>6.748446608362666</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1412,7 +1412,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q11" t="n">
-        <v>455.4</v>
+        <v>461.4</v>
       </c>
       <c r="R11" t="n">
         <v>74809.60000000001</v>
@@ -1428,13 +1428,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1139559824732299</v>
+        <v>0.1124741101393777</v>
       </c>
       <c r="X11" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y11" t="n">
-        <v>164.2722880983751</v>
+        <v>162.1361074989163</v>
       </c>
       <c r="Z11" t="n">
         <v>0.6937018032218979</v>
@@ -1486,7 +1486,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K12" t="n">
-        <v>4.25211318303151</v>
+        <v>4.200426231860138</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1502,7 +1502,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q12" t="n">
-        <v>731.4</v>
+        <v>740.4</v>
       </c>
       <c r="R12" t="n">
         <v>38128.4</v>
@@ -1518,13 +1518,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W12" t="n">
-        <v>0.07086855305052515</v>
+        <v>0.07000710386433563</v>
       </c>
       <c r="X12" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y12" t="n">
-        <v>52.13070823079027</v>
+        <v>51.49702863317126</v>
       </c>
       <c r="Z12" t="n">
         <v>1.359439674918279</v>
@@ -1576,7 +1576,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K13" t="n">
-        <v>5.711675863654216</v>
+        <v>6.004033804240762</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1592,7 +1592,7 @@
         <v>0.145035</v>
       </c>
       <c r="Q13" t="n">
-        <v>505.2</v>
+        <v>480.6</v>
       </c>
       <c r="R13" t="n">
         <v>60200.2</v>
@@ -1608,13 +1608,13 @@
         <v>6.17518114688861</v>
       </c>
       <c r="W13" t="n">
-        <v>0.09519459772757027</v>
+        <v>0.1000672300706794</v>
       </c>
       <c r="X13" t="n">
         <v>0.161938569284539</v>
       </c>
       <c r="Y13" t="n">
-        <v>119.1611243072051</v>
+        <v>125.2605076987099</v>
       </c>
       <c r="Z13" t="n">
         <v>0.7988729401558218</v>
@@ -1666,7 +1666,7 @@
         <v>47.6305176437724</v>
       </c>
       <c r="K14" t="n">
-        <v>8.707590062846874</v>
+        <v>9.394579416917631</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1682,7 @@
         <v>0.208445</v>
       </c>
       <c r="Q14" t="n">
-        <v>328.2</v>
+        <v>304.2</v>
       </c>
       <c r="R14" t="n">
         <v>30999.6</v>
@@ -1698,13 +1698,13 @@
         <v>8.555202665891516</v>
       </c>
       <c r="W14" t="n">
-        <v>0.1451265010474479</v>
+        <v>0.1565763236152939</v>
       </c>
       <c r="X14" t="n">
         <v>0.1168879381416492</v>
       </c>
       <c r="Y14" t="n">
-        <v>94.45338208409507</v>
+        <v>101.905325443787</v>
       </c>
       <c r="Z14" t="n">
         <v>1.53648813674281</v>
@@ -1756,7 +1756,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>2.521528264398947</v>
+        <v>2.539450553867064</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1772,7 +1772,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>1105.2</v>
+        <v>1097.4</v>
       </c>
       <c r="R15" t="n">
         <v>80561.39999999999</v>
@@ -1788,13 +1788,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.04202547107331578</v>
+        <v>0.04232417589778441</v>
       </c>
       <c r="X15" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>72.8930510314875</v>
+        <v>73.4111536358666</v>
       </c>
       <c r="Z15" t="n">
         <v>0.5765360412086756</v>
@@ -1846,7 +1846,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>1.830272877559791</v>
+        <v>1.817348235819471</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1862,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1518.6</v>
+        <v>1529.4</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1878,13 +1878,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.03050454795932984</v>
+        <v>0.03028913726365784</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>42.32562886869485</v>
+        <v>42.02674251340395</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1936,7 +1936,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.200190499419981</v>
+        <v>1.16151428383765</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1952,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2270.4</v>
+        <v>2346</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1968,13 +1968,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.02000317499033303</v>
+        <v>0.01935857139729416</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>47.44987667371388</v>
+        <v>45.92080136402387</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -2026,7 +2026,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>3.287620586315272</v>
+        <v>3.72834241345662</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2042,7 +2042,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q18" t="n">
-        <v>817.1999999999999</v>
+        <v>720.6</v>
       </c>
       <c r="R18" t="n">
         <v>71127.60000000001</v>
@@ -2058,13 +2058,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W18" t="n">
-        <v>0.05479367643858787</v>
+        <v>0.06213904022427699</v>
       </c>
       <c r="X18" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y18" t="n">
-        <v>87.03817914831131</v>
+        <v>98.70607826810992</v>
       </c>
       <c r="Z18" t="n">
         <v>0.629536106737947</v>
@@ -2116,7 +2116,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>3.799678967346777</v>
+        <v>3.839710703613818</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2132,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q19" t="n">
-        <v>690.6</v>
+        <v>683.4000000000001</v>
       </c>
       <c r="R19" t="n">
         <v>64144.3</v>
@@ -2148,13 +2148,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W19" t="n">
-        <v>0.06332798278911295</v>
+        <v>0.06399517839356364</v>
       </c>
       <c r="X19" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y19" t="n">
-        <v>92.8819866782508</v>
+        <v>93.86055019022534</v>
       </c>
       <c r="Z19" t="n">
         <v>0.6818112429968274</v>
@@ -2206,7 +2206,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>2.125491123933603</v>
+        <v>2.284791559322757</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2222,7 +2222,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q20" t="n">
-        <v>1230.6</v>
+        <v>1144.8</v>
       </c>
       <c r="R20" t="n">
         <v>48455.2</v>
@@ -2238,13 +2238,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W20" t="n">
-        <v>0.03542485206556005</v>
+        <v>0.03807985932204595</v>
       </c>
       <c r="X20" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y20" t="n">
-        <v>39.37526409881358</v>
+        <v>42.32634521313766</v>
       </c>
       <c r="Z20" t="n">
         <v>0.8996727482680539</v>
@@ -2296,7 +2296,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K21" t="n">
-        <v>2.473814562926332</v>
+        <v>2.539943263271871</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q21" t="n">
-        <v>1014</v>
+        <v>987.6</v>
       </c>
       <c r="R21" t="n">
         <v>68673.2</v>
@@ -2328,13 +2328,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W21" t="n">
-        <v>0.04123024271543886</v>
+        <v>0.04233238772119785</v>
       </c>
       <c r="X21" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y21" t="n">
-        <v>67.7250493096647</v>
+        <v>69.5354394491697</v>
       </c>
       <c r="Z21" t="n">
         <v>0.6087886703030441</v>
@@ -2386,7 +2386,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K22" t="n">
-        <v>8.185246435318081</v>
+        <v>8.301466972939233</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q22" t="n">
-        <v>300</v>
+        <v>295.8</v>
       </c>
       <c r="R22" t="n">
         <v>71002.60000000001</v>
@@ -2418,13 +2418,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W22" t="n">
-        <v>0.136420773921968</v>
+        <v>0.1383577828823205</v>
       </c>
       <c r="X22" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y22" t="n">
-        <v>236.6753333333334</v>
+        <v>240.0358350236647</v>
       </c>
       <c r="Z22" t="n">
         <v>0.5764046975264343</v>
@@ -2476,7 +2476,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K23" t="n">
-        <v>7.721363497559099</v>
+        <v>7.134930826858408</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2492,7 +2492,7 @@
         <v>0.07520300000000001</v>
       </c>
       <c r="Q23" t="n">
-        <v>306.6</v>
+        <v>331.8</v>
       </c>
       <c r="R23" t="n">
         <v>88574</v>
@@ -2508,13 +2508,13 @@
         <v>12.61396912906789</v>
       </c>
       <c r="W23" t="n">
-        <v>0.128689391625985</v>
+        <v>0.1189155137809735</v>
       </c>
       <c r="X23" t="n">
         <v>0.07927718783579227</v>
       </c>
       <c r="Y23" t="n">
-        <v>288.8910632746249</v>
+        <v>266.9499698613623</v>
       </c>
       <c r="Z23" t="n">
         <v>0.4454599258532639</v>
@@ -2566,7 +2566,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K24" t="n">
-        <v>5.829437108099969</v>
+        <v>6.061131746736693</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2582,7 +2582,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q24" t="n">
-        <v>392.4</v>
+        <v>377.4</v>
       </c>
       <c r="R24" t="n">
         <v>50011.7</v>
@@ -2598,13 +2598,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W24" t="n">
-        <v>0.09715728513499949</v>
+        <v>0.1010188624456116</v>
       </c>
       <c r="X24" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y24" t="n">
-        <v>127.4508154943935</v>
+        <v>132.5164281928988</v>
       </c>
       <c r="Z24" t="n">
         <v>0.7623119927331765</v>
@@ -2656,7 +2656,7 @@
         <v>33.6962858057476</v>
       </c>
       <c r="K25" t="n">
-        <v>1.751366206119938</v>
+        <v>1.777230264016224</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2672,7 +2672,7 @@
         <v>0.143133</v>
       </c>
       <c r="Q25" t="n">
-        <v>1154.4</v>
+        <v>1137.6</v>
       </c>
       <c r="R25" t="n">
         <v>66797.5</v>
@@ -2688,13 +2688,13 @@
         <v>13.44796592290856</v>
       </c>
       <c r="W25" t="n">
-        <v>0.02918943676866563</v>
+        <v>0.02962050440027039</v>
       </c>
       <c r="X25" t="n">
         <v>0.0743606881317645</v>
       </c>
       <c r="Y25" t="n">
-        <v>57.86339223839224</v>
+        <v>58.71791490857946</v>
       </c>
       <c r="Z25" t="n">
         <v>0.504454295531234</v>
@@ -2808,7 +2808,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K27" t="n">
-        <v>2.88453042681457</v>
+        <v>2.743689504566347</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2824,7 +2824,7 @@
         <v>0.026182</v>
       </c>
       <c r="Q27" t="n">
-        <v>607.8000000000001</v>
+        <v>639</v>
       </c>
       <c r="R27" t="n">
         <v>48192</v>
@@ -2840,13 +2840,13 @@
         <v>15.27539782478406</v>
       </c>
       <c r="W27" t="n">
-        <v>0.04807550711357617</v>
+        <v>0.04572815840943913</v>
       </c>
       <c r="X27" t="n">
         <v>0.06546474346988973</v>
       </c>
       <c r="Y27" t="n">
-        <v>79.28923988153997</v>
+        <v>75.41784037558685</v>
       </c>
       <c r="Z27" t="n">
         <v>0.6063307856829266</v>
@@ -2988,7 +2988,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K29" t="n">
-        <v>8.818427823956076</v>
+        <v>9.593268762462678</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -3004,7 +3004,7 @@
         <v>0.037626</v>
       </c>
       <c r="Q29" t="n">
-        <v>156</v>
+        <v>143.4</v>
       </c>
       <c r="R29" t="n">
         <v>28366.1</v>
@@ -3020,13 +3020,13 @@
         <v>31.96610467696488</v>
       </c>
       <c r="W29" t="n">
-        <v>0.1469737970659346</v>
+        <v>0.1598878127077113</v>
       </c>
       <c r="X29" t="n">
         <v>0.0312831360000085</v>
       </c>
       <c r="Y29" t="n">
-        <v>181.8339743589744</v>
+        <v>197.8110181311018</v>
       </c>
       <c r="Z29" t="n">
         <v>0.8082856769977473</v>
@@ -3078,7 +3078,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K30" t="n">
-        <v>9.654926855771548</v>
+        <v>8.916029392319643</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3094,7 +3094,7 @@
         <v>0.01289</v>
       </c>
       <c r="Q30" t="n">
-        <v>108.6</v>
+        <v>117.6</v>
       </c>
       <c r="R30" t="n">
         <v>13925.2</v>
@@ -3110,13 +3110,13 @@
         <v>76.71116733805002</v>
       </c>
       <c r="W30" t="n">
-        <v>0.1609154475961924</v>
+        <v>0.1486004898719941</v>
       </c>
       <c r="X30" t="n">
         <v>0.01303591165016704</v>
       </c>
       <c r="Y30" t="n">
-        <v>128.2246777163904</v>
+        <v>118.4115646258503</v>
       </c>
       <c r="Z30" t="n">
         <v>1.254949128841704</v>
@@ -3168,7 +3168,7 @@
         <v>14.1889227802691</v>
       </c>
       <c r="K31" t="n">
-        <v>5.542547961042617</v>
+        <v>5.586190070972087</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3184,7 +3184,7 @@
         <v>0.105148</v>
       </c>
       <c r="Q31" t="n">
-        <v>153.6</v>
+        <v>152.4</v>
       </c>
       <c r="R31" t="n">
         <v>26085.5</v>
@@ -3200,13 +3200,13 @@
         <v>9.066560752338283</v>
       </c>
       <c r="W31" t="n">
-        <v>0.09237579935071029</v>
+        <v>0.09310316784953478</v>
       </c>
       <c r="X31" t="n">
         <v>0.1102954060879257</v>
       </c>
       <c r="Y31" t="n">
-        <v>169.8274739583333</v>
+        <v>171.1646981627296</v>
       </c>
       <c r="Z31" t="n">
         <v>0.5439390765087539</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-05)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.35543233637916</v>
+        <v>4.227613338979919</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>793.8000000000001</v>
+        <v>817.8000000000001</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07259053893965267</v>
+        <v>0.07046022231633198</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>150.1209372637944</v>
+        <v>145.7153338224505</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.645841709510378</v>
+        <v>3.471799668820794</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>921.5999999999999</v>
+        <v>967.8</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.06076402849183963</v>
+        <v>0.05786332781367989</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>214.2256944444445</v>
+        <v>203.9991733829304</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.427939217452801</v>
+        <v>6.383962438314015</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>522.6</v>
+        <v>526.1999999999999</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.10713232029088</v>
+        <v>0.1063993739719002</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>125.6551856104095</v>
+        <v>124.7955150133029</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -864,7 +864,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K5" t="n">
-        <v>10.89089349231844</v>
+        <v>10.54787322484384</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -880,7 +880,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q5" t="n">
-        <v>295.2</v>
+        <v>304.8</v>
       </c>
       <c r="R5" t="n">
         <v>35584.1</v>
@@ -896,13 +896,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1815148915386406</v>
+        <v>0.1757978870807307</v>
       </c>
       <c r="X5" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y5" t="n">
-        <v>120.5423441734417</v>
+        <v>116.7457349081365</v>
       </c>
       <c r="Z5" t="n">
         <v>1.505818497087371</v>
@@ -954,7 +954,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>4.227807128551918</v>
+        <v>4.126444389971013</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -970,7 +970,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q6" t="n">
-        <v>757.1999999999999</v>
+        <v>775.8</v>
       </c>
       <c r="R6" t="n">
         <v>78110.8</v>
@@ -986,13 +986,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07046345214253197</v>
+        <v>0.06877407316618356</v>
       </c>
       <c r="X6" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y6" t="n">
-        <v>103.1574220813524</v>
+        <v>100.6841969579789</v>
       </c>
       <c r="Z6" t="n">
         <v>0.6830672066132366</v>
@@ -1044,7 +1044,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K7" t="n">
-        <v>5.315010864524916</v>
+        <v>5.019175354140981</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1060,7 +1060,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q7" t="n">
-        <v>600.6</v>
+        <v>636</v>
       </c>
       <c r="R7" t="n">
         <v>60537.6</v>
@@ -1076,13 +1076,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W7" t="n">
-        <v>0.08858351440874859</v>
+        <v>0.08365292256901635</v>
       </c>
       <c r="X7" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y7" t="n">
-        <v>100.7952047952048</v>
+        <v>95.18490566037735</v>
       </c>
       <c r="Z7" t="n">
         <v>0.8788465144619939</v>
@@ -1134,7 +1134,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K8" t="n">
-        <v>7.12769545270812</v>
+        <v>7.118063431826081</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1150,7 +1150,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q8" t="n">
-        <v>443.4</v>
+        <v>444</v>
       </c>
       <c r="R8" t="n">
         <v>27205.5</v>
@@ -1166,13 +1166,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W8" t="n">
-        <v>0.118794924211802</v>
+        <v>0.1186343905304347</v>
       </c>
       <c r="X8" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y8" t="n">
-        <v>61.35656292286875</v>
+        <v>61.27364864864865</v>
       </c>
       <c r="Z8" t="n">
         <v>1.936140464079432</v>
@@ -1306,7 +1306,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K10" t="n">
-        <v>10.35302919187316</v>
+        <v>11.12236257131172</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1322,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q10" t="n">
-        <v>303.6</v>
+        <v>282.6</v>
       </c>
       <c r="R10" t="n">
         <v>16901.2</v>
@@ -1338,13 +1338,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W10" t="n">
-        <v>0.1725504865312194</v>
+        <v>0.185372709521862</v>
       </c>
       <c r="X10" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y10" t="n">
-        <v>55.66930171277998</v>
+        <v>59.80608634111819</v>
       </c>
       <c r="Z10" t="n">
         <v>3.099562617499243</v>
@@ -1396,7 +1396,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K11" t="n">
-        <v>6.837358948393795</v>
+        <v>6.748446608362666</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1412,7 +1412,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q11" t="n">
-        <v>455.4</v>
+        <v>461.4</v>
       </c>
       <c r="R11" t="n">
         <v>74809.60000000001</v>
@@ -1428,13 +1428,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1139559824732299</v>
+        <v>0.1124741101393777</v>
       </c>
       <c r="X11" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y11" t="n">
-        <v>164.2722880983751</v>
+        <v>162.1361074989163</v>
       </c>
       <c r="Z11" t="n">
         <v>0.6937018032218979</v>
@@ -1486,7 +1486,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K12" t="n">
-        <v>4.231286506216661</v>
+        <v>4.483845994909524</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1502,7 +1502,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q12" t="n">
-        <v>735</v>
+        <v>693.6</v>
       </c>
       <c r="R12" t="n">
         <v>38128.4</v>
@@ -1518,13 +1518,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W12" t="n">
-        <v>0.07052144177027768</v>
+        <v>0.0747307665818254</v>
       </c>
       <c r="X12" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y12" t="n">
-        <v>51.87537414965987</v>
+        <v>54.97174163783161</v>
       </c>
       <c r="Z12" t="n">
         <v>1.359439674918279</v>
@@ -1576,7 +1576,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K13" t="n">
-        <v>6.294805074864987</v>
+        <v>7.114247155616642</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1592,7 +1592,7 @@
         <v>0.145035</v>
       </c>
       <c r="Q13" t="n">
-        <v>458.4</v>
+        <v>405.6</v>
       </c>
       <c r="R13" t="n">
         <v>60200.2</v>
@@ -1608,13 +1608,13 @@
         <v>6.17518114688861</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1049134179144165</v>
+        <v>0.118570785926944</v>
       </c>
       <c r="X13" t="n">
         <v>0.161938569284539</v>
       </c>
       <c r="Y13" t="n">
-        <v>131.3267888307155</v>
+        <v>148.42258382643</v>
       </c>
       <c r="Z13" t="n">
         <v>0.7988729401558218</v>
@@ -1666,7 +1666,7 @@
         <v>47.6305176437724</v>
       </c>
       <c r="K14" t="n">
-        <v>9.700716424393564</v>
+        <v>9.820725287375753</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1682,7 @@
         <v>0.208445</v>
       </c>
       <c r="Q14" t="n">
-        <v>294.6</v>
+        <v>291</v>
       </c>
       <c r="R14" t="n">
         <v>30999.6</v>
@@ -1698,13 +1698,13 @@
         <v>8.555202665891516</v>
       </c>
       <c r="W14" t="n">
-        <v>0.1616786070732261</v>
+        <v>0.1636787547895959</v>
       </c>
       <c r="X14" t="n">
         <v>0.1168879381416492</v>
       </c>
       <c r="Y14" t="n">
-        <v>105.2260692464358</v>
+        <v>106.5278350515464</v>
       </c>
       <c r="Z14" t="n">
         <v>1.53648813674281</v>
@@ -1756,7 +1756,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>2.593330576785517</v>
+        <v>2.849481633756356</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1772,7 +1772,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>1074.6</v>
+        <v>978</v>
       </c>
       <c r="R15" t="n">
         <v>80561.39999999999</v>
@@ -1788,13 +1788,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.04322217627975861</v>
+        <v>0.04749136056260593</v>
       </c>
       <c r="X15" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>74.96873255164712</v>
+        <v>82.37361963190183</v>
       </c>
       <c r="Z15" t="n">
         <v>0.5765360412086756</v>
@@ -1846,7 +1846,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>1.795511881047996</v>
+        <v>1.852968261241532</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1862,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1548</v>
+        <v>1500</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1878,13 +1878,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.0299251980174666</v>
+        <v>0.03088280435402553</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>41.52177002583979</v>
+        <v>42.85046666666666</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1936,7 +1936,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.124974201091209</v>
+        <v>1.16151428383765</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1952,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2422.2</v>
+        <v>2346</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1968,13 +1968,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.01874957001818682</v>
+        <v>0.01935857139729416</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>44.47617868053835</v>
+        <v>45.92080136402387</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -2026,7 +2026,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>3.495502918471038</v>
+        <v>3.567919712001115</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2042,7 +2042,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q18" t="n">
-        <v>768.6</v>
+        <v>753</v>
       </c>
       <c r="R18" t="n">
         <v>71127.60000000001</v>
@@ -2058,13 +2058,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W18" t="n">
-        <v>0.05825838197451731</v>
+        <v>0.05946532853335192</v>
       </c>
       <c r="X18" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y18" t="n">
-        <v>92.54176424668229</v>
+        <v>94.4589641434263</v>
       </c>
       <c r="Z18" t="n">
         <v>0.629536106737947</v>
@@ -2116,7 +2116,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>3.819589948835057</v>
+        <v>3.968630209996497</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2132,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q19" t="n">
-        <v>687</v>
+        <v>661.1999999999999</v>
       </c>
       <c r="R19" t="n">
         <v>64144.3</v>
@@ -2148,13 +2148,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W19" t="n">
-        <v>0.06365983248058428</v>
+        <v>0.06614383683327496</v>
       </c>
       <c r="X19" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y19" t="n">
-        <v>93.36870451237264</v>
+        <v>97.01194797338175</v>
       </c>
       <c r="Z19" t="n">
         <v>0.6818112429968274</v>
@@ -2206,7 +2206,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>2.353878129151091</v>
+        <v>2.640449603384506</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2222,7 +2222,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q20" t="n">
-        <v>1111.2</v>
+        <v>990.6000000000001</v>
       </c>
       <c r="R20" t="n">
         <v>48455.2</v>
@@ -2238,13 +2238,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W20" t="n">
-        <v>0.03923130215251818</v>
+        <v>0.04400749338974177</v>
       </c>
       <c r="X20" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y20" t="n">
-        <v>43.60619150467962</v>
+        <v>48.91500100948919</v>
       </c>
       <c r="Z20" t="n">
         <v>0.8996727482680539</v>
@@ -2296,7 +2296,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K21" t="n">
-        <v>2.612966632090937</v>
+        <v>2.572767145443385</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q21" t="n">
-        <v>960</v>
+        <v>975</v>
       </c>
       <c r="R21" t="n">
         <v>68673.2</v>
@@ -2328,13 +2328,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W21" t="n">
-        <v>0.04354944386818229</v>
+        <v>0.04287945242405641</v>
       </c>
       <c r="X21" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y21" t="n">
-        <v>71.53458333333333</v>
+        <v>70.43405128205129</v>
       </c>
       <c r="Z21" t="n">
         <v>0.6087886703030441</v>
@@ -2386,7 +2386,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K22" t="n">
-        <v>8.421035427281975</v>
+        <v>8.335281502360571</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q22" t="n">
-        <v>291.6</v>
+        <v>294.6</v>
       </c>
       <c r="R22" t="n">
         <v>71002.60000000001</v>
@@ -2418,13 +2418,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W22" t="n">
-        <v>0.1403505904546996</v>
+        <v>0.1389213583726762</v>
       </c>
       <c r="X22" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y22" t="n">
-        <v>243.4931412894376</v>
+        <v>241.0135777325187</v>
       </c>
       <c r="Z22" t="n">
         <v>0.5764046975264343</v>
@@ -2476,7 +2476,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K23" t="n">
-        <v>7.721363497559099</v>
+        <v>7.602344407037957</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2492,7 +2492,7 @@
         <v>0.07520300000000001</v>
       </c>
       <c r="Q23" t="n">
-        <v>306.6</v>
+        <v>311.4</v>
       </c>
       <c r="R23" t="n">
         <v>88574</v>
@@ -2508,13 +2508,13 @@
         <v>12.61396912906789</v>
       </c>
       <c r="W23" t="n">
-        <v>0.128689391625985</v>
+        <v>0.1267057401172993</v>
       </c>
       <c r="X23" t="n">
         <v>0.07927718783579227</v>
       </c>
       <c r="Y23" t="n">
-        <v>288.8910632746249</v>
+        <v>284.4380218368657</v>
       </c>
       <c r="Z23" t="n">
         <v>0.4454599258532639</v>
@@ -2656,7 +2656,7 @@
         <v>33.6962858057476</v>
       </c>
       <c r="K25" t="n">
-        <v>1.777230264016224</v>
+        <v>1.736921948749876</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2672,7 +2672,7 @@
         <v>0.143133</v>
       </c>
       <c r="Q25" t="n">
-        <v>1137.6</v>
+        <v>1164</v>
       </c>
       <c r="R25" t="n">
         <v>66797.5</v>
@@ -2688,13 +2688,13 @@
         <v>13.44796592290856</v>
       </c>
       <c r="W25" t="n">
-        <v>0.02962050440027039</v>
+        <v>0.02894869914583127</v>
       </c>
       <c r="X25" t="n">
         <v>0.0743606881317645</v>
       </c>
       <c r="Y25" t="n">
-        <v>58.71791490857946</v>
+        <v>57.38616838487972</v>
       </c>
       <c r="Z25" t="n">
         <v>0.504454295531234</v>
@@ -2808,7 +2808,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K27" t="n">
-        <v>3.009298993164943</v>
+        <v>3.312958415377732</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2824,7 +2824,7 @@
         <v>0.026182</v>
       </c>
       <c r="Q27" t="n">
-        <v>582.6</v>
+        <v>529.2</v>
       </c>
       <c r="R27" t="n">
         <v>48192</v>
@@ -2840,13 +2840,13 @@
         <v>15.27539782478406</v>
       </c>
       <c r="W27" t="n">
-        <v>0.05015498321941572</v>
+        <v>0.05521597358962887</v>
       </c>
       <c r="X27" t="n">
         <v>0.06546474346988973</v>
       </c>
       <c r="Y27" t="n">
-        <v>82.71884654994851</v>
+        <v>91.06575963718821</v>
       </c>
       <c r="Z27" t="n">
         <v>0.6063307856829266</v>
@@ -2898,7 +2898,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K28" t="n">
-        <v>8.766589859627508</v>
+        <v>8.735937447530908</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2914,7 +2914,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q28" t="n">
-        <v>171</v>
+        <v>171.6</v>
       </c>
       <c r="R28" t="n">
         <v>34656</v>
@@ -2930,13 +2930,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W28" t="n">
-        <v>0.1461098309937918</v>
+        <v>0.1455989574588485</v>
       </c>
       <c r="X28" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y28" t="n">
-        <v>202.6666666666667</v>
+        <v>201.958041958042</v>
       </c>
       <c r="Z28" t="n">
         <v>0.7209366660877885</v>
@@ -2988,7 +2988,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K29" t="n">
-        <v>9.593268762462678</v>
+        <v>10.23567515280616</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -3004,7 +3004,7 @@
         <v>0.037626</v>
       </c>
       <c r="Q29" t="n">
-        <v>143.4</v>
+        <v>134.4</v>
       </c>
       <c r="R29" t="n">
         <v>28366.1</v>
@@ -3020,13 +3020,13 @@
         <v>31.96610467696488</v>
       </c>
       <c r="W29" t="n">
-        <v>0.1598878127077113</v>
+        <v>0.1705945858801027</v>
       </c>
       <c r="X29" t="n">
         <v>0.0312831360000085</v>
       </c>
       <c r="Y29" t="n">
-        <v>197.8110181311018</v>
+        <v>211.0572916666667</v>
       </c>
       <c r="Z29" t="n">
         <v>0.8082856769977473</v>
@@ -3078,7 +3078,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K30" t="n">
-        <v>8.916029392319643</v>
+        <v>9.49750957007962</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3094,7 +3094,7 @@
         <v>0.01289</v>
       </c>
       <c r="Q30" t="n">
-        <v>117.6</v>
+        <v>110.4</v>
       </c>
       <c r="R30" t="n">
         <v>13925.2</v>
@@ -3110,13 +3110,13 @@
         <v>76.71116733805002</v>
       </c>
       <c r="W30" t="n">
-        <v>0.1486004898719941</v>
+        <v>0.1582918261679936</v>
       </c>
       <c r="X30" t="n">
         <v>0.01303591165016704</v>
       </c>
       <c r="Y30" t="n">
-        <v>118.4115646258503</v>
+        <v>126.1340579710145</v>
       </c>
       <c r="Z30" t="n">
         <v>1.254949128841704</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-06)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.227613338979919</v>
+        <v>4.358726914545862</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>817.8000000000001</v>
+        <v>793.2</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07046022231633198</v>
+        <v>0.07264544857576437</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>145.7153338224505</v>
+        <v>150.2344931921331</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.471799668820794</v>
+        <v>3.431380432480355</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>967.8</v>
+        <v>979.2</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.05786332781367989</v>
+        <v>0.05718967387467259</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>203.9991733829304</v>
+        <v>201.6241830065359</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.383962438314015</v>
+        <v>6.586747127531048</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>526.1999999999999</v>
+        <v>510</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1063993739719002</v>
+        <v>0.1097791187921841</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>124.7955150133029</v>
+        <v>128.7596078431372</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -864,7 +864,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K5" t="n">
-        <v>10.54787322484384</v>
+        <v>11.18647097749618</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -880,7 +880,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q5" t="n">
-        <v>304.8</v>
+        <v>287.4</v>
       </c>
       <c r="R5" t="n">
         <v>35584.1</v>
@@ -896,13 +896,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1757978870807307</v>
+        <v>0.1864411829582697</v>
       </c>
       <c r="X5" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y5" t="n">
-        <v>116.7457349081365</v>
+        <v>123.8138482950592</v>
       </c>
       <c r="Z5" t="n">
         <v>1.505818497087371</v>
@@ -1044,7 +1044,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K7" t="n">
-        <v>5.019175354140981</v>
+        <v>5.417847123614501</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1060,7 +1060,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q7" t="n">
-        <v>636</v>
+        <v>589.2</v>
       </c>
       <c r="R7" t="n">
         <v>60537.6</v>
@@ -1076,13 +1076,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W7" t="n">
-        <v>0.08365292256901635</v>
+        <v>0.09029745206024169</v>
       </c>
       <c r="X7" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y7" t="n">
-        <v>95.18490566037735</v>
+        <v>102.7454175152749</v>
       </c>
       <c r="Z7" t="n">
         <v>0.8788465144619939</v>
@@ -1134,7 +1134,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K8" t="n">
-        <v>7.118063431826081</v>
+        <v>7.439783812925565</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1150,7 +1150,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q8" t="n">
-        <v>444</v>
+        <v>424.8</v>
       </c>
       <c r="R8" t="n">
         <v>27205.5</v>
@@ -1166,13 +1166,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W8" t="n">
-        <v>0.1186343905304347</v>
+        <v>0.1239963968820928</v>
       </c>
       <c r="X8" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y8" t="n">
-        <v>61.27364864864865</v>
+        <v>64.04307909604519</v>
       </c>
       <c r="Z8" t="n">
         <v>1.936140464079432</v>
@@ -1306,7 +1306,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K10" t="n">
-        <v>11.12236257131172</v>
+        <v>11.71953640064389</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1322,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q10" t="n">
-        <v>282.6</v>
+        <v>268.2</v>
       </c>
       <c r="R10" t="n">
         <v>16901.2</v>
@@ -1338,13 +1338,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W10" t="n">
-        <v>0.185372709521862</v>
+        <v>0.1953256066773982</v>
       </c>
       <c r="X10" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y10" t="n">
-        <v>59.80608634111819</v>
+        <v>63.01715137956749</v>
       </c>
       <c r="Z10" t="n">
         <v>3.099562617499243</v>
@@ -1396,7 +1396,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K11" t="n">
-        <v>6.748446608362666</v>
+        <v>7.148147991502603</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1412,7 +1412,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q11" t="n">
-        <v>461.4</v>
+        <v>435.6</v>
       </c>
       <c r="R11" t="n">
         <v>74809.60000000001</v>
@@ -1428,13 +1428,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1124741101393777</v>
+        <v>0.1191357998583767</v>
       </c>
       <c r="X11" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y11" t="n">
-        <v>162.1361074989163</v>
+        <v>171.7392102846649</v>
       </c>
       <c r="Z11" t="n">
         <v>0.6937018032218979</v>
@@ -1486,7 +1486,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K12" t="n">
-        <v>4.483845994909524</v>
+        <v>4.772860009314375</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1502,7 +1502,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q12" t="n">
-        <v>693.6</v>
+        <v>651.5999999999999</v>
       </c>
       <c r="R12" t="n">
         <v>38128.4</v>
@@ -1518,13 +1518,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W12" t="n">
-        <v>0.0747307665818254</v>
+        <v>0.07954766682190624</v>
       </c>
       <c r="X12" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y12" t="n">
-        <v>54.97174163783161</v>
+        <v>58.51503990178024</v>
       </c>
       <c r="Z12" t="n">
         <v>1.359439674918279</v>
@@ -1576,7 +1576,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K13" t="n">
-        <v>7.114247155616642</v>
+        <v>9.195470510892637</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1592,7 +1592,7 @@
         <v>0.145035</v>
       </c>
       <c r="Q13" t="n">
-        <v>405.6</v>
+        <v>313.8</v>
       </c>
       <c r="R13" t="n">
         <v>60200.2</v>
@@ -1608,13 +1608,13 @@
         <v>6.17518114688861</v>
       </c>
       <c r="W13" t="n">
-        <v>0.118570785926944</v>
+        <v>0.1532578418482106</v>
       </c>
       <c r="X13" t="n">
         <v>0.161938569284539</v>
       </c>
       <c r="Y13" t="n">
-        <v>148.42258382643</v>
+        <v>191.842574888464</v>
       </c>
       <c r="Z13" t="n">
         <v>0.7988729401558218</v>
@@ -1666,7 +1666,7 @@
         <v>47.6305176437724</v>
       </c>
       <c r="K14" t="n">
-        <v>9.820725287375753</v>
+        <v>10.00641126970008</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1682,7 @@
         <v>0.208445</v>
       </c>
       <c r="Q14" t="n">
-        <v>291</v>
+        <v>285.6</v>
       </c>
       <c r="R14" t="n">
         <v>30999.6</v>
@@ -1698,13 +1698,13 @@
         <v>8.555202665891516</v>
       </c>
       <c r="W14" t="n">
-        <v>0.1636787547895959</v>
+        <v>0.1667735211616681</v>
       </c>
       <c r="X14" t="n">
         <v>0.1168879381416492</v>
       </c>
       <c r="Y14" t="n">
-        <v>106.5278350515464</v>
+        <v>108.5420168067227</v>
       </c>
       <c r="Z14" t="n">
         <v>1.53648813674281</v>
@@ -1756,7 +1756,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>2.849481633756356</v>
+        <v>3.176918647758455</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1772,7 +1772,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>978</v>
+        <v>877.1999999999999</v>
       </c>
       <c r="R15" t="n">
         <v>80561.39999999999</v>
@@ -1788,13 +1788,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.04749136056260593</v>
+        <v>0.05294864412930757</v>
       </c>
       <c r="X15" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>82.37361963190183</v>
+        <v>91.83926128590971</v>
       </c>
       <c r="Z15" t="n">
         <v>0.5765360412086756</v>
@@ -1846,7 +1846,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>1.852968261241532</v>
+        <v>2.187167447168947</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1862,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1500</v>
+        <v>1270.8</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1878,13 +1878,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.03088280435402553</v>
+        <v>0.03645279078614912</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>42.85046666666666</v>
+        <v>50.57892666037142</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1936,7 +1936,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.16151428383765</v>
+        <v>1.177474941614003</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1952,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2346</v>
+        <v>2314.2</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1968,13 +1968,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.01935857139729416</v>
+        <v>0.01962458236023339</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>45.92080136402387</v>
+        <v>46.55181056088497</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -2026,7 +2026,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>3.567919712001115</v>
+        <v>3.124730801508304</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2042,7 +2042,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q18" t="n">
-        <v>753</v>
+        <v>859.8</v>
       </c>
       <c r="R18" t="n">
         <v>71127.60000000001</v>
@@ -2058,13 +2058,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W18" t="n">
-        <v>0.05946532853335192</v>
+        <v>0.05207884669180508</v>
       </c>
       <c r="X18" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y18" t="n">
-        <v>94.4589641434263</v>
+        <v>82.72575017445919</v>
       </c>
       <c r="Z18" t="n">
         <v>0.629536106737947</v>
@@ -2116,7 +2116,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>3.968630209996497</v>
+        <v>4.064526479011283</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2132,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q19" t="n">
-        <v>661.1999999999999</v>
+        <v>645.6</v>
       </c>
       <c r="R19" t="n">
         <v>64144.3</v>
@@ -2148,13 +2148,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W19" t="n">
-        <v>0.06614383683327496</v>
+        <v>0.06774210798352137</v>
       </c>
       <c r="X19" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y19" t="n">
-        <v>97.01194797338175</v>
+        <v>99.35610285006196</v>
       </c>
       <c r="Z19" t="n">
         <v>0.6818112429968274</v>
@@ -2206,7 +2206,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>2.640449603384506</v>
+        <v>2.959526337534162</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2222,7 +2222,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q20" t="n">
-        <v>990.6000000000001</v>
+        <v>883.8000000000001</v>
       </c>
       <c r="R20" t="n">
         <v>48455.2</v>
@@ -2238,13 +2238,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W20" t="n">
-        <v>0.04400749338974177</v>
+        <v>0.04932543895890269</v>
       </c>
       <c r="X20" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y20" t="n">
-        <v>48.91500100948919</v>
+        <v>54.82597872821905</v>
       </c>
       <c r="Z20" t="n">
         <v>0.8996727482680539</v>
@@ -2296,7 +2296,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K21" t="n">
-        <v>2.572767145443385</v>
+        <v>2.577525654343712</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q21" t="n">
-        <v>975</v>
+        <v>973.1999999999999</v>
       </c>
       <c r="R21" t="n">
         <v>68673.2</v>
@@ -2328,13 +2328,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W21" t="n">
-        <v>0.04287945242405641</v>
+        <v>0.04295876090572853</v>
       </c>
       <c r="X21" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y21" t="n">
-        <v>70.43405128205129</v>
+        <v>70.56432387998356</v>
       </c>
       <c r="Z21" t="n">
         <v>0.6087886703030441</v>
@@ -2386,7 +2386,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K22" t="n">
-        <v>8.335281502360571</v>
+        <v>8.403743773427188</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q22" t="n">
-        <v>294.6</v>
+        <v>292.2</v>
       </c>
       <c r="R22" t="n">
         <v>71002.60000000001</v>
@@ -2418,13 +2418,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W22" t="n">
-        <v>0.1389213583726762</v>
+        <v>0.1400623962237865</v>
       </c>
       <c r="X22" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y22" t="n">
-        <v>241.0135777325187</v>
+        <v>242.9931553730322</v>
       </c>
       <c r="Z22" t="n">
         <v>0.5764046975264343</v>
@@ -2476,7 +2476,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K23" t="n">
-        <v>7.602344407037957</v>
+        <v>8.306561573163579</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2492,7 +2492,7 @@
         <v>0.07520300000000001</v>
       </c>
       <c r="Q23" t="n">
-        <v>311.4</v>
+        <v>285</v>
       </c>
       <c r="R23" t="n">
         <v>88574</v>
@@ -2508,13 +2508,13 @@
         <v>12.61396912906789</v>
       </c>
       <c r="W23" t="n">
-        <v>0.1267057401172993</v>
+        <v>0.1384426928860596</v>
       </c>
       <c r="X23" t="n">
         <v>0.07927718783579227</v>
       </c>
       <c r="Y23" t="n">
-        <v>284.4380218368657</v>
+        <v>310.7859649122807</v>
       </c>
       <c r="Z23" t="n">
         <v>0.4454599258532639</v>
@@ -2566,7 +2566,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K24" t="n">
-        <v>6.429092527314301</v>
+        <v>6.759666433860604</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2582,7 +2582,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q24" t="n">
-        <v>355.8</v>
+        <v>338.4</v>
       </c>
       <c r="R24" t="n">
         <v>50011.7</v>
@@ -2598,13 +2598,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W24" t="n">
-        <v>0.107151542121905</v>
+        <v>0.1126611072310101</v>
       </c>
       <c r="X24" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y24" t="n">
-        <v>140.5612703766161</v>
+        <v>147.7887115839243</v>
       </c>
       <c r="Z24" t="n">
         <v>0.7623119927331765</v>
@@ -2656,7 +2656,7 @@
         <v>33.6962858057476</v>
       </c>
       <c r="K25" t="n">
-        <v>1.736921948749876</v>
+        <v>1.767905865988856</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2672,7 +2672,7 @@
         <v>0.143133</v>
       </c>
       <c r="Q25" t="n">
-        <v>1164</v>
+        <v>1143.6</v>
       </c>
       <c r="R25" t="n">
         <v>66797.5</v>
@@ -2688,13 +2688,13 @@
         <v>13.44796592290856</v>
       </c>
       <c r="W25" t="n">
-        <v>0.02894869914583127</v>
+        <v>0.02946509776648094</v>
       </c>
       <c r="X25" t="n">
         <v>0.0743606881317645</v>
       </c>
       <c r="Y25" t="n">
-        <v>57.38616838487972</v>
+        <v>58.40984610003498</v>
       </c>
       <c r="Z25" t="n">
         <v>0.504454295531234</v>
@@ -2808,7 +2808,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K27" t="n">
-        <v>3.312958415377732</v>
+        <v>3.834684150082887</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2824,7 +2824,7 @@
         <v>0.026182</v>
       </c>
       <c r="Q27" t="n">
-        <v>529.2</v>
+        <v>457.2</v>
       </c>
       <c r="R27" t="n">
         <v>48192</v>
@@ -2840,13 +2840,13 @@
         <v>15.27539782478406</v>
       </c>
       <c r="W27" t="n">
-        <v>0.05521597358962887</v>
+        <v>0.06391140250138146</v>
       </c>
       <c r="X27" t="n">
         <v>0.06546474346988973</v>
       </c>
       <c r="Y27" t="n">
-        <v>91.06575963718821</v>
+        <v>105.4068241469816</v>
       </c>
       <c r="Z27" t="n">
         <v>0.6063307856829266</v>
@@ -2898,7 +2898,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K28" t="n">
-        <v>8.735937447530908</v>
+        <v>10.91038475979843</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2914,7 +2914,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q28" t="n">
-        <v>171.6</v>
+        <v>137.4</v>
       </c>
       <c r="R28" t="n">
         <v>34656</v>
@@ -2930,13 +2930,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W28" t="n">
-        <v>0.1455989574588485</v>
+        <v>0.1818397459966405</v>
       </c>
       <c r="X28" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y28" t="n">
-        <v>201.958041958042</v>
+        <v>252.2270742358079</v>
       </c>
       <c r="Z28" t="n">
         <v>0.7209366660877885</v>
@@ -2988,7 +2988,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K29" t="n">
-        <v>10.23567515280616</v>
+        <v>9.396685386182705</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -3004,7 +3004,7 @@
         <v>0.037626</v>
       </c>
       <c r="Q29" t="n">
-        <v>134.4</v>
+        <v>146.4</v>
       </c>
       <c r="R29" t="n">
         <v>28366.1</v>
@@ -3020,13 +3020,13 @@
         <v>31.96610467696488</v>
       </c>
       <c r="W29" t="n">
-        <v>0.1705945858801027</v>
+        <v>0.1566114231030451</v>
       </c>
       <c r="X29" t="n">
         <v>0.0312831360000085</v>
       </c>
       <c r="Y29" t="n">
-        <v>211.0572916666667</v>
+        <v>193.7575136612022</v>
       </c>
       <c r="Z29" t="n">
         <v>0.8082856769977473</v>
@@ -3078,7 +3078,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K30" t="n">
-        <v>9.49750957007962</v>
+        <v>8.916029392319643</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3094,7 +3094,7 @@
         <v>0.01289</v>
       </c>
       <c r="Q30" t="n">
-        <v>110.4</v>
+        <v>117.6</v>
       </c>
       <c r="R30" t="n">
         <v>13925.2</v>
@@ -3110,13 +3110,13 @@
         <v>76.71116733805002</v>
       </c>
       <c r="W30" t="n">
-        <v>0.1582918261679936</v>
+        <v>0.1486004898719941</v>
       </c>
       <c r="X30" t="n">
         <v>0.01303591165016704</v>
       </c>
       <c r="Y30" t="n">
-        <v>126.1340579710145</v>
+        <v>118.4115646258503</v>
       </c>
       <c r="Z30" t="n">
         <v>1.254949128841704</v>
@@ -3168,7 +3168,7 @@
         <v>14.1889227802691</v>
       </c>
       <c r="K31" t="n">
-        <v>5.586190070972087</v>
+        <v>6.063642213790216</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3184,7 +3184,7 @@
         <v>0.105148</v>
       </c>
       <c r="Q31" t="n">
-        <v>152.4</v>
+        <v>140.4</v>
       </c>
       <c r="R31" t="n">
         <v>26085.5</v>
@@ -3200,13 +3200,13 @@
         <v>9.066560752338283</v>
       </c>
       <c r="W31" t="n">
-        <v>0.09310316784953478</v>
+        <v>0.1010607035631702</v>
       </c>
       <c r="X31" t="n">
         <v>0.1102954060879257</v>
       </c>
       <c r="Y31" t="n">
-        <v>171.1646981627296</v>
+        <v>185.7941595441596</v>
       </c>
       <c r="Z31" t="n">
         <v>0.5439390765087539</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-07)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.358726914545862</v>
+        <v>4.408750559318768</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>793.2</v>
+        <v>784.2</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07264544857576437</v>
+        <v>0.07347917598864613</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>150.2344931921331</v>
+        <v>151.9586840091813</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.431380432480355</v>
+        <v>3.420899734763555</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>979.2</v>
+        <v>982.2</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.05718967387467259</v>
+        <v>0.05701499557939258</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>201.6241830065359</v>
+        <v>201.008348605172</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.586747127531048</v>
+        <v>6.54057833925396</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>510</v>
+        <v>513.6</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1097791187921841</v>
+        <v>0.109009638987566</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>128.7596078431372</v>
+        <v>127.8570872274143</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -954,7 +954,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>4.126444389971013</v>
+        <v>4.278662867868901</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -970,7 +970,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q6" t="n">
-        <v>775.8</v>
+        <v>748.2</v>
       </c>
       <c r="R6" t="n">
         <v>78110.8</v>
@@ -986,13 +986,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W6" t="n">
-        <v>0.06877407316618356</v>
+        <v>0.07131104779781501</v>
       </c>
       <c r="X6" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y6" t="n">
-        <v>100.6841969579789</v>
+        <v>104.3982892274793</v>
       </c>
       <c r="Z6" t="n">
         <v>0.6830672066132366</v>
@@ -1044,7 +1044,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K7" t="n">
-        <v>5.417847123614501</v>
+        <v>5.028663398288696</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1060,7 +1060,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q7" t="n">
-        <v>589.2</v>
+        <v>634.8</v>
       </c>
       <c r="R7" t="n">
         <v>60537.6</v>
@@ -1076,13 +1076,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W7" t="n">
-        <v>0.09029745206024169</v>
+        <v>0.08381105663814493</v>
       </c>
       <c r="X7" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y7" t="n">
-        <v>102.7454175152749</v>
+        <v>95.3648393194707</v>
       </c>
       <c r="Z7" t="n">
         <v>0.8788465144619939</v>
@@ -1134,7 +1134,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K8" t="n">
-        <v>7.439783812925565</v>
+        <v>6.146285810444924</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1150,7 +1150,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q8" t="n">
-        <v>424.8</v>
+        <v>514.2</v>
       </c>
       <c r="R8" t="n">
         <v>27205.5</v>
@@ -1166,13 +1166,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W8" t="n">
-        <v>0.1239963968820928</v>
+        <v>0.1024380968407487</v>
       </c>
       <c r="X8" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y8" t="n">
-        <v>64.04307909604519</v>
+        <v>52.90840140023337</v>
       </c>
       <c r="Z8" t="n">
         <v>1.936140464079432</v>
@@ -1306,7 +1306,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K10" t="n">
-        <v>11.71953640064389</v>
+        <v>9.791836955304337</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1322,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q10" t="n">
-        <v>268.2</v>
+        <v>321</v>
       </c>
       <c r="R10" t="n">
         <v>16901.2</v>
@@ -1338,13 +1338,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W10" t="n">
-        <v>0.1953256066773982</v>
+        <v>0.1631972825884056</v>
       </c>
       <c r="X10" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y10" t="n">
-        <v>63.01715137956749</v>
+        <v>52.65171339563863</v>
       </c>
       <c r="Z10" t="n">
         <v>3.099562617499243</v>
@@ -1396,7 +1396,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K11" t="n">
-        <v>7.148147991502603</v>
+        <v>6.828362423461697</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1412,7 +1412,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q11" t="n">
-        <v>435.6</v>
+        <v>456</v>
       </c>
       <c r="R11" t="n">
         <v>74809.60000000001</v>
@@ -1428,13 +1428,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1191357998583767</v>
+        <v>0.1138060403910283</v>
       </c>
       <c r="X11" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y11" t="n">
-        <v>171.7392102846649</v>
+        <v>164.0561403508772</v>
       </c>
       <c r="Z11" t="n">
         <v>0.6937018032218979</v>
@@ -1486,7 +1486,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K12" t="n">
-        <v>4.772860009314375</v>
+        <v>4.803823883332169</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1502,7 +1502,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q12" t="n">
-        <v>651.5999999999999</v>
+        <v>647.4</v>
       </c>
       <c r="R12" t="n">
         <v>38128.4</v>
@@ -1518,13 +1518,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W12" t="n">
-        <v>0.07954766682190624</v>
+        <v>0.08006373138886948</v>
       </c>
       <c r="X12" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y12" t="n">
-        <v>58.51503990178024</v>
+        <v>58.89465554525796</v>
       </c>
       <c r="Z12" t="n">
         <v>1.359439674918279</v>
@@ -1576,7 +1576,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K13" t="n">
-        <v>9.195470510892637</v>
+        <v>9.374719448726804</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1592,7 +1592,7 @@
         <v>0.145035</v>
       </c>
       <c r="Q13" t="n">
-        <v>313.8</v>
+        <v>307.8</v>
       </c>
       <c r="R13" t="n">
         <v>60200.2</v>
@@ -1608,13 +1608,13 @@
         <v>6.17518114688861</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1532578418482106</v>
+        <v>0.1562453241454467</v>
       </c>
       <c r="X13" t="n">
         <v>0.161938569284539</v>
       </c>
       <c r="Y13" t="n">
-        <v>191.842574888464</v>
+        <v>195.582196231319</v>
       </c>
       <c r="Z13" t="n">
         <v>0.7988729401558218</v>
@@ -1666,7 +1666,7 @@
         <v>47.6305176437724</v>
       </c>
       <c r="K14" t="n">
-        <v>10.00641126970008</v>
+        <v>8.490288350048555</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1682,7 @@
         <v>0.208445</v>
       </c>
       <c r="Q14" t="n">
-        <v>285.6</v>
+        <v>336.6</v>
       </c>
       <c r="R14" t="n">
         <v>30999.6</v>
@@ -1698,13 +1698,13 @@
         <v>8.555202665891516</v>
       </c>
       <c r="W14" t="n">
-        <v>0.1667735211616681</v>
+        <v>0.1415048058341426</v>
       </c>
       <c r="X14" t="n">
         <v>0.1168879381416492</v>
       </c>
       <c r="Y14" t="n">
-        <v>108.5420168067227</v>
+        <v>92.09625668449196</v>
       </c>
       <c r="Z14" t="n">
         <v>1.53648813674281</v>
@@ -1756,7 +1756,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>3.176918647758455</v>
+        <v>2.481119157597682</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1772,7 +1772,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>877.1999999999999</v>
+        <v>1123.2</v>
       </c>
       <c r="R15" t="n">
         <v>80561.39999999999</v>
@@ -1788,13 +1788,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.05294864412930757</v>
+        <v>0.04135198595996137</v>
       </c>
       <c r="X15" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>91.83926128590971</v>
+        <v>71.72489316239317</v>
       </c>
       <c r="Z15" t="n">
         <v>0.5765360412086756</v>
@@ -1846,7 +1846,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>2.187167447168947</v>
+        <v>1.764059654647308</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1862,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1270.8</v>
+        <v>1575.6</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1878,13 +1878,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.03645279078614912</v>
+        <v>0.02940099424412179</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>50.57892666037142</v>
+        <v>40.79442751967504</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1936,7 +1936,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.177474941614003</v>
+        <v>1.264695307659485</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1952,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2314.2</v>
+        <v>2154.6</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1968,13 +1968,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.01962458236023339</v>
+        <v>0.02107825512765808</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>46.55181056088497</v>
+        <v>50.00009282465423</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -2026,7 +2026,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>3.124730801508304</v>
+        <v>3.460385810325657</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2042,7 +2042,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q18" t="n">
-        <v>859.8</v>
+        <v>776.4</v>
       </c>
       <c r="R18" t="n">
         <v>71127.60000000001</v>
@@ -2058,13 +2058,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W18" t="n">
-        <v>0.05207884669180508</v>
+        <v>0.05767309683876095</v>
       </c>
       <c r="X18" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y18" t="n">
-        <v>82.72575017445919</v>
+        <v>91.61205564142196</v>
       </c>
       <c r="Z18" t="n">
         <v>0.629536106737947</v>
@@ -2116,7 +2116,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>4.064526479011283</v>
+        <v>4.494789816460576</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2132,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q19" t="n">
-        <v>645.6</v>
+        <v>583.8000000000001</v>
       </c>
       <c r="R19" t="n">
         <v>64144.3</v>
@@ -2148,13 +2148,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W19" t="n">
-        <v>0.06774210798352137</v>
+        <v>0.07491316360767625</v>
       </c>
       <c r="X19" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y19" t="n">
-        <v>99.35610285006196</v>
+        <v>109.8737581363481</v>
       </c>
       <c r="Z19" t="n">
         <v>0.6818112429968274</v>
@@ -2206,7 +2206,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>2.959526337534162</v>
+        <v>2.491075597250183</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2222,7 +2222,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q20" t="n">
-        <v>883.8000000000001</v>
+        <v>1050</v>
       </c>
       <c r="R20" t="n">
         <v>48455.2</v>
@@ -2238,13 +2238,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W20" t="n">
-        <v>0.04932543895890269</v>
+        <v>0.04151792662083639</v>
       </c>
       <c r="X20" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y20" t="n">
-        <v>54.82597872821905</v>
+        <v>46.14780952380952</v>
       </c>
       <c r="Z20" t="n">
         <v>0.8996727482680539</v>
@@ -2296,7 +2296,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K21" t="n">
-        <v>2.577525654343712</v>
+        <v>2.475279225189757</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q21" t="n">
-        <v>973.1999999999999</v>
+        <v>1013.4</v>
       </c>
       <c r="R21" t="n">
         <v>68673.2</v>
@@ -2328,13 +2328,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W21" t="n">
-        <v>0.04295876090572853</v>
+        <v>0.04125465375316262</v>
       </c>
       <c r="X21" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y21" t="n">
-        <v>70.56432387998356</v>
+        <v>67.76514702980066</v>
       </c>
       <c r="Z21" t="n">
         <v>0.6087886703030441</v>
@@ -2386,7 +2386,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K22" t="n">
-        <v>8.403743773427188</v>
+        <v>6.200944269180365</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q22" t="n">
-        <v>292.2</v>
+        <v>396</v>
       </c>
       <c r="R22" t="n">
         <v>71002.60000000001</v>
@@ -2418,13 +2418,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W22" t="n">
-        <v>0.1400623962237865</v>
+        <v>0.1033490711530061</v>
       </c>
       <c r="X22" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y22" t="n">
-        <v>242.9931553730322</v>
+        <v>179.299494949495</v>
       </c>
       <c r="Z22" t="n">
         <v>0.5764046975264343</v>
@@ -2476,7 +2476,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K23" t="n">
-        <v>8.306561573163579</v>
+        <v>8.596114917761874</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2492,7 +2492,7 @@
         <v>0.07520300000000001</v>
       </c>
       <c r="Q23" t="n">
-        <v>285</v>
+        <v>275.4</v>
       </c>
       <c r="R23" t="n">
         <v>88574</v>
@@ -2508,13 +2508,13 @@
         <v>12.61396912906789</v>
       </c>
       <c r="W23" t="n">
-        <v>0.1384426928860596</v>
+        <v>0.1432685819626979</v>
       </c>
       <c r="X23" t="n">
         <v>0.07927718783579227</v>
       </c>
       <c r="Y23" t="n">
-        <v>310.7859649122807</v>
+        <v>321.6194625998548</v>
       </c>
       <c r="Z23" t="n">
         <v>0.4454599258532639</v>
@@ -2523,37 +2523,37 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>gpt-6-luna</t>
+          <t>mistral-large-4</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (Max)</t>
+          <t>Mistral Large 4 Preview</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (max)</t>
+          <t>Mistral Large 4 Preview</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Mistral</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>mistral</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H24" t="b">
@@ -2563,177 +2563,177 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>38.1245186869738</v>
+        <v>38.3770408917494</v>
       </c>
       <c r="K24" t="n">
-        <v>6.759666433860604</v>
+        <v>4.541661643994012</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>0.326276</v>
+        <v>6.131298</v>
       </c>
       <c r="N24" t="n">
-        <v>0.30127</v>
+        <v>5.841498</v>
       </c>
       <c r="O24" t="n">
-        <v>0.005561</v>
+        <v>0.072395</v>
       </c>
       <c r="P24" t="n">
-        <v>0.019445</v>
+        <v>0.217404</v>
       </c>
       <c r="Q24" t="n">
-        <v>338.4</v>
+        <v>506.9999999999999</v>
       </c>
       <c r="R24" t="n">
-        <v>50011.7</v>
+        <v>69330</v>
       </c>
       <c r="S24" t="n">
-        <v>11122</v>
+        <v>17319.4</v>
       </c>
       <c r="T24" t="n">
-        <v>38889.7</v>
+        <v>52010.6</v>
       </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="n">
-        <v>116.8474502782117</v>
+        <v>6.259203335370325</v>
       </c>
       <c r="W24" t="n">
-        <v>0.1126611072310101</v>
+        <v>0.07569436073323355</v>
       </c>
       <c r="X24" t="n">
-        <v>0.008558167059863248</v>
+        <v>0.1597647410412551</v>
       </c>
       <c r="Y24" t="n">
-        <v>147.7887115839243</v>
+        <v>136.7455621301775</v>
       </c>
       <c r="Z24" t="n">
-        <v>0.7623119927331765</v>
+        <v>0.5535416254399164</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>qwen3-8-27b</t>
+          <t>gpt-6-luna</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (Xhigh)</t>
+          <t>GPT-6 Luna (Max)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (xhigh)</t>
+          <t>GPT-6 Luna (max)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H25" t="b">
         <v>1</v>
       </c>
       <c r="I25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>33.6962858057476</v>
+        <v>38.1245186869738</v>
       </c>
       <c r="K25" t="n">
-        <v>1.767905865988856</v>
+        <v>5.883413377619413</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
-        <v>2.505679</v>
+        <v>0.326276</v>
       </c>
       <c r="N25" t="n">
-        <v>2.305287</v>
+        <v>0.30127</v>
       </c>
       <c r="O25" t="n">
-        <v>0.05726</v>
+        <v>0.005561</v>
       </c>
       <c r="P25" t="n">
-        <v>0.143133</v>
+        <v>0.019445</v>
       </c>
       <c r="Q25" t="n">
-        <v>1143.6</v>
+        <v>388.8</v>
       </c>
       <c r="R25" t="n">
-        <v>66797.5</v>
+        <v>50011.7</v>
       </c>
       <c r="S25" t="n">
-        <v>19086.6</v>
+        <v>11122</v>
       </c>
       <c r="T25" t="n">
-        <v>47710.9</v>
+        <v>38889.7</v>
       </c>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="n">
-        <v>13.44796592290856</v>
+        <v>116.8474502782117</v>
       </c>
       <c r="W25" t="n">
-        <v>0.02946509776648094</v>
+        <v>0.09805688962699023</v>
       </c>
       <c r="X25" t="n">
-        <v>0.0743606881317645</v>
+        <v>0.008558167059863248</v>
       </c>
       <c r="Y25" t="n">
-        <v>58.40984610003498</v>
+        <v>128.6309156378601</v>
       </c>
       <c r="Z25" t="n">
-        <v>0.504454295531234</v>
+        <v>0.7623119927331765</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>k2-horizon-375b-a23b</t>
+          <t>qwen3-8-27b</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Qwen3.8 27B (Xhigh)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Qwen3.8 27B (xhigh)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Institute of Foundation Models</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ifm</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H26" t="b">
@@ -2743,54 +2743,82 @@
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>30.5015302696723</v>
-      </c>
-      <c r="K26" t="inlineStr"/>
+        <v>33.6962858057476</v>
+      </c>
+      <c r="K26" t="n">
+        <v>1.78287226485437</v>
+      </c>
       <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
-      <c r="T26" t="inlineStr"/>
+      <c r="M26" t="n">
+        <v>2.505679</v>
+      </c>
+      <c r="N26" t="n">
+        <v>2.305287</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0.05726</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0.143133</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>1134</v>
+      </c>
+      <c r="R26" t="n">
+        <v>66797.5</v>
+      </c>
+      <c r="S26" t="n">
+        <v>19086.6</v>
+      </c>
+      <c r="T26" t="n">
+        <v>47710.9</v>
+      </c>
       <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
-      <c r="X26" t="inlineStr"/>
-      <c r="Y26" t="inlineStr"/>
-      <c r="Z26" t="inlineStr"/>
+      <c r="V26" t="n">
+        <v>13.44796592290856</v>
+      </c>
+      <c r="W26" t="n">
+        <v>0.02971453774757284</v>
+      </c>
+      <c r="X26" t="n">
+        <v>0.0743606881317645</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>58.90432098765432</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>0.504454295531234</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>minimax-m3</t>
+          <t>k2-horizon-375b-a23b</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>Institute of Foundation Models</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>minimax</t>
+          <t>ifm</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2805,82 +2833,54 @@
         <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>29.2202932236316</v>
-      </c>
-      <c r="K27" t="n">
-        <v>3.834684150082887</v>
-      </c>
+        <v>30.5015302696723</v>
+      </c>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
-      <c r="M27" t="n">
-        <v>1.912899</v>
-      </c>
-      <c r="N27" t="n">
-        <v>1.855069</v>
-      </c>
-      <c r="O27" t="n">
-        <v>0.031649</v>
-      </c>
-      <c r="P27" t="n">
-        <v>0.026182</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>457.2</v>
-      </c>
-      <c r="R27" t="n">
-        <v>48192</v>
-      </c>
-      <c r="S27" t="n">
-        <v>26373.8</v>
-      </c>
-      <c r="T27" t="n">
-        <v>21818.2</v>
-      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
-      <c r="V27" t="n">
-        <v>15.27539782478406</v>
-      </c>
-      <c r="W27" t="n">
-        <v>0.06391140250138146</v>
-      </c>
-      <c r="X27" t="n">
-        <v>0.06546474346988973</v>
-      </c>
-      <c r="Y27" t="n">
-        <v>105.4068241469816</v>
-      </c>
-      <c r="Z27" t="n">
-        <v>0.6063307856829266</v>
-      </c>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>inkling</t>
+          <t>minimax-m3</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Inkling (Xhigh)</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Inkling (xhigh)</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Thinking Machines</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>thinking-machines</t>
+          <t>minimax</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2895,82 +2895,82 @@
         <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>24.9847810999384</v>
+        <v>29.2202932236316</v>
       </c>
       <c r="K28" t="n">
-        <v>10.91038475979843</v>
+        <v>3.449857523451192</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
-        <v>2.418996</v>
+        <v>1.912899</v>
       </c>
       <c r="N28" t="n">
-        <v>2.278639</v>
+        <v>1.855069</v>
       </c>
       <c r="O28" t="n">
-        <v>0.04559</v>
+        <v>0.031649</v>
       </c>
       <c r="P28" t="n">
-        <v>0.094767</v>
+        <v>0.026182</v>
       </c>
       <c r="Q28" t="n">
-        <v>137.4</v>
+        <v>508.2</v>
       </c>
       <c r="R28" t="n">
-        <v>34656</v>
+        <v>48192</v>
       </c>
       <c r="S28" t="n">
-        <v>11256.8</v>
+        <v>26373.8</v>
       </c>
       <c r="T28" t="n">
-        <v>23399.2</v>
+        <v>21818.2</v>
       </c>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="n">
-        <v>10.32857478885389</v>
+        <v>15.27539782478406</v>
       </c>
       <c r="W28" t="n">
-        <v>0.1818397459966405</v>
+        <v>0.0574976253908532</v>
       </c>
       <c r="X28" t="n">
-        <v>0.09681877901287532</v>
+        <v>0.06546474346988973</v>
       </c>
       <c r="Y28" t="n">
-        <v>252.2270742358079</v>
+        <v>94.82880755608028</v>
       </c>
       <c r="Z28" t="n">
-        <v>0.7209366660877885</v>
+        <v>0.6063307856829266</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
+          <t>inkling</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
+          <t>Inkling (Xhigh)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra</t>
+          <t>Inkling (xhigh)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Thinking Machines</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>thinking-machines</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2985,87 +2985,87 @@
         <v>1</v>
       </c>
       <c r="J29" t="n">
-        <v>22.9279123422858</v>
+        <v>24.9847810999384</v>
       </c>
       <c r="K29" t="n">
-        <v>9.396685386182705</v>
+        <v>7.037966507024901</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
-        <v>0.717257</v>
+        <v>2.418996</v>
       </c>
       <c r="N29" t="n">
-        <v>0.646342</v>
+        <v>2.278639</v>
       </c>
       <c r="O29" t="n">
-        <v>0.03329</v>
+        <v>0.04559</v>
       </c>
       <c r="P29" t="n">
-        <v>0.037626</v>
+        <v>0.094767</v>
       </c>
       <c r="Q29" t="n">
-        <v>146.4</v>
+        <v>213</v>
       </c>
       <c r="R29" t="n">
-        <v>28366.1</v>
+        <v>34656</v>
       </c>
       <c r="S29" t="n">
-        <v>13315.8</v>
+        <v>11256.8</v>
       </c>
       <c r="T29" t="n">
-        <v>15050.3</v>
+        <v>23399.2</v>
       </c>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="n">
-        <v>31.96610467696488</v>
+        <v>10.32857478885389</v>
       </c>
       <c r="W29" t="n">
-        <v>0.1566114231030451</v>
+        <v>0.1172994417837483</v>
       </c>
       <c r="X29" t="n">
-        <v>0.0312831360000085</v>
+        <v>0.09681877901287532</v>
       </c>
       <c r="Y29" t="n">
-        <v>193.7575136612022</v>
+        <v>162.7042253521127</v>
       </c>
       <c r="Z29" t="n">
-        <v>0.8082856769977473</v>
+        <v>0.7209366660877885</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>muse-glimmer</t>
+          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Muse Glimmer (High)</t>
+          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Muse Glimmer (high)</t>
+          <t>Nemotron 3 Ultra</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>nvidia</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H30" t="b">
@@ -3075,87 +3075,87 @@
         <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>17.4754176089465</v>
+        <v>22.9279123422858</v>
       </c>
       <c r="K30" t="n">
-        <v>8.916029392319643</v>
+        <v>8.491819386031777</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
-        <v>0.227808</v>
+        <v>0.717257</v>
       </c>
       <c r="N30" t="n">
-        <v>0.209009</v>
+        <v>0.646342</v>
       </c>
       <c r="O30" t="n">
-        <v>0.005909</v>
+        <v>0.03329</v>
       </c>
       <c r="P30" t="n">
-        <v>0.01289</v>
+        <v>0.037626</v>
       </c>
       <c r="Q30" t="n">
-        <v>117.6</v>
+        <v>162</v>
       </c>
       <c r="R30" t="n">
-        <v>13925.2</v>
+        <v>28366.1</v>
       </c>
       <c r="S30" t="n">
-        <v>4377.3</v>
+        <v>13315.8</v>
       </c>
       <c r="T30" t="n">
-        <v>9547.9</v>
+        <v>15050.3</v>
       </c>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="n">
-        <v>76.71116733805002</v>
+        <v>31.96610467696488</v>
       </c>
       <c r="W30" t="n">
-        <v>0.1486004898719941</v>
+        <v>0.1415303231005296</v>
       </c>
       <c r="X30" t="n">
-        <v>0.01303591165016704</v>
+        <v>0.0312831360000085</v>
       </c>
       <c r="Y30" t="n">
-        <v>118.4115646258503</v>
+        <v>175.0993827160494</v>
       </c>
       <c r="Z30" t="n">
-        <v>1.254949128841704</v>
+        <v>0.8082856769977473</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>mistral-medium-3-5</t>
+          <t>muse-glimmer</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mistral Medium 3.5</t>
+          <t>Muse Glimmer (High)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Mistral Medium 3.5</t>
+          <t>Muse Glimmer (high)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Mistral</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>mistral</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H31" t="b">
@@ -3165,51 +3165,51 @@
         <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>14.1889227802691</v>
+        <v>17.4754176089465</v>
       </c>
       <c r="K31" t="n">
-        <v>6.063642213790216</v>
+        <v>7.836510138541032</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
-        <v>1.564973</v>
+        <v>0.227808</v>
       </c>
       <c r="N31" t="n">
-        <v>1.369332</v>
+        <v>0.209009</v>
       </c>
       <c r="O31" t="n">
-        <v>0.090493</v>
+        <v>0.005909</v>
       </c>
       <c r="P31" t="n">
-        <v>0.105148</v>
+        <v>0.01289</v>
       </c>
       <c r="Q31" t="n">
-        <v>140.4</v>
+        <v>133.8</v>
       </c>
       <c r="R31" t="n">
-        <v>26085.5</v>
+        <v>13925.2</v>
       </c>
       <c r="S31" t="n">
-        <v>12065.8</v>
+        <v>4377.3</v>
       </c>
       <c r="T31" t="n">
-        <v>14019.8</v>
+        <v>9547.9</v>
       </c>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="n">
-        <v>9.066560752338283</v>
+        <v>76.71116733805002</v>
       </c>
       <c r="W31" t="n">
-        <v>0.1010607035631702</v>
+        <v>0.1306085023090172</v>
       </c>
       <c r="X31" t="n">
-        <v>0.1102954060879257</v>
+        <v>0.01303591165016704</v>
       </c>
       <c r="Y31" t="n">
-        <v>185.7941595441596</v>
+        <v>104.0747384155456</v>
       </c>
       <c r="Z31" t="n">
-        <v>0.5439390765087539</v>
+        <v>1.254949128841704</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-08)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z31"/>
+  <dimension ref="A1:Z32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.408750559318768</v>
+        <v>4.418893390360146</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>784.2</v>
+        <v>782.4</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07347917598864613</v>
+        <v>0.0736482231726691</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>151.9586840091813</v>
+        <v>152.308282208589</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.420899734763555</v>
+        <v>3.575997998600217</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>982.2</v>
+        <v>939.6</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.05701499557939258</v>
+        <v>0.05959996664333695</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>201.008348605172</v>
+        <v>210.1217539378459</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.54057833925396</v>
+        <v>6.548228138481158</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>513.6</v>
+        <v>513</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.109009638987566</v>
+        <v>0.1091371356413526</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>127.8570872274143</v>
+        <v>128.0066276803119</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -864,7 +864,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K5" t="n">
-        <v>11.18647097749618</v>
+        <v>11.23337441974983</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -880,7 +880,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q5" t="n">
-        <v>287.4</v>
+        <v>286.2</v>
       </c>
       <c r="R5" t="n">
         <v>35584.1</v>
@@ -896,13 +896,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1864411829582697</v>
+        <v>0.1872229069958306</v>
       </c>
       <c r="X5" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y5" t="n">
-        <v>123.8138482950592</v>
+        <v>124.3329839273236</v>
       </c>
       <c r="Z5" t="n">
         <v>1.505818497087371</v>
@@ -954,7 +954,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>4.278662867868901</v>
+        <v>4.494939002723269</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -970,7 +970,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q6" t="n">
-        <v>748.2</v>
+        <v>712.1999999999999</v>
       </c>
       <c r="R6" t="n">
         <v>78110.8</v>
@@ -986,13 +986,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07131104779781501</v>
+        <v>0.07491565004538782</v>
       </c>
       <c r="X6" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y6" t="n">
-        <v>104.3982892274793</v>
+        <v>109.6753720864926</v>
       </c>
       <c r="Z6" t="n">
         <v>0.6830672066132366</v>
@@ -1044,7 +1044,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K7" t="n">
-        <v>5.028663398288696</v>
+        <v>5.257239007301819</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1060,7 +1060,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q7" t="n">
-        <v>634.8</v>
+        <v>607.1999999999999</v>
       </c>
       <c r="R7" t="n">
         <v>60537.6</v>
@@ -1076,13 +1076,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W7" t="n">
-        <v>0.08381105663814493</v>
+        <v>0.08762065012169698</v>
       </c>
       <c r="X7" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y7" t="n">
-        <v>95.3648393194707</v>
+        <v>99.69960474308301</v>
       </c>
       <c r="Z7" t="n">
         <v>0.8788465144619939</v>
@@ -1134,7 +1134,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K8" t="n">
-        <v>6.146285810444924</v>
+        <v>5.396892356097644</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1150,7 +1150,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q8" t="n">
-        <v>514.2</v>
+        <v>585.6</v>
       </c>
       <c r="R8" t="n">
         <v>27205.5</v>
@@ -1166,13 +1166,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W8" t="n">
-        <v>0.1024380968407487</v>
+        <v>0.08994820593496072</v>
       </c>
       <c r="X8" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y8" t="n">
-        <v>52.90840140023337</v>
+        <v>46.45747950819672</v>
       </c>
       <c r="Z8" t="n">
         <v>1.936140464079432</v>
@@ -1306,7 +1306,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K10" t="n">
-        <v>9.791836955304337</v>
+        <v>8.211023152175267</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1322,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q10" t="n">
-        <v>321</v>
+        <v>382.8</v>
       </c>
       <c r="R10" t="n">
         <v>16901.2</v>
@@ -1338,13 +1338,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W10" t="n">
-        <v>0.1631972825884056</v>
+        <v>0.1368503858695878</v>
       </c>
       <c r="X10" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y10" t="n">
-        <v>52.65171339563863</v>
+        <v>44.15151515151515</v>
       </c>
       <c r="Z10" t="n">
         <v>3.099562617499243</v>
@@ -1396,7 +1396,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K11" t="n">
-        <v>6.828362423461697</v>
+        <v>7.227793094471992</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1412,7 +1412,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q11" t="n">
-        <v>456</v>
+        <v>430.8</v>
       </c>
       <c r="R11" t="n">
         <v>74809.60000000001</v>
@@ -1428,13 +1428,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1138060403910283</v>
+        <v>0.1204632182411999</v>
       </c>
       <c r="X11" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y11" t="n">
-        <v>164.0561403508772</v>
+        <v>173.652739090065</v>
       </c>
       <c r="Z11" t="n">
         <v>0.6937018032218979</v>
@@ -1486,7 +1486,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K12" t="n">
-        <v>4.803823883332169</v>
+        <v>4.52692224464228</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1502,7 +1502,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q12" t="n">
-        <v>647.4</v>
+        <v>687</v>
       </c>
       <c r="R12" t="n">
         <v>38128.4</v>
@@ -1518,13 +1518,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W12" t="n">
-        <v>0.08006373138886948</v>
+        <v>0.07544870407737132</v>
       </c>
       <c r="X12" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y12" t="n">
-        <v>58.89465554525796</v>
+        <v>55.49985443959243</v>
       </c>
       <c r="Z12" t="n">
         <v>1.359439674918279</v>
@@ -1576,7 +1576,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K13" t="n">
-        <v>9.374719448726804</v>
+        <v>8.680922522015974</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1592,7 +1592,7 @@
         <v>0.145035</v>
       </c>
       <c r="Q13" t="n">
-        <v>307.8</v>
+        <v>332.4</v>
       </c>
       <c r="R13" t="n">
         <v>60200.2</v>
@@ -1608,13 +1608,13 @@
         <v>6.17518114688861</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1562453241454467</v>
+        <v>0.1446820420335996</v>
       </c>
       <c r="X13" t="n">
         <v>0.161938569284539</v>
       </c>
       <c r="Y13" t="n">
-        <v>195.582196231319</v>
+        <v>181.1077015643803</v>
       </c>
       <c r="Z13" t="n">
         <v>0.7988729401558218</v>
@@ -1666,7 +1666,7 @@
         <v>47.6305176437724</v>
       </c>
       <c r="K14" t="n">
-        <v>8.490288350048555</v>
+        <v>8.114227877985076</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1682,7 @@
         <v>0.208445</v>
       </c>
       <c r="Q14" t="n">
-        <v>336.6</v>
+        <v>352.2</v>
       </c>
       <c r="R14" t="n">
         <v>30999.6</v>
@@ -1698,13 +1698,13 @@
         <v>8.555202665891516</v>
       </c>
       <c r="W14" t="n">
-        <v>0.1415048058341426</v>
+        <v>0.1352371312997513</v>
       </c>
       <c r="X14" t="n">
         <v>0.1168879381416492</v>
       </c>
       <c r="Y14" t="n">
-        <v>92.09625668449196</v>
+        <v>88.01703577512777</v>
       </c>
       <c r="Z14" t="n">
         <v>1.53648813674281</v>
@@ -1756,7 +1756,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>2.481119157597682</v>
+        <v>2.400338533861943</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1772,7 +1772,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>1123.2</v>
+        <v>1161</v>
       </c>
       <c r="R15" t="n">
         <v>80561.39999999999</v>
@@ -1788,13 +1788,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.04135198595996137</v>
+        <v>0.04000564223103239</v>
       </c>
       <c r="X15" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>71.72489316239317</v>
+        <v>69.38966408268733</v>
       </c>
       <c r="Z15" t="n">
         <v>0.5765360412086756</v>
@@ -1846,7 +1846,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>1.764059654647308</v>
+        <v>1.761376674183966</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1862,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1575.6</v>
+        <v>1578</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1878,13 +1878,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.02940099424412179</v>
+        <v>0.0293562779030661</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>40.79442751967504</v>
+        <v>40.73238276299113</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1936,7 +1936,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.264695307659485</v>
+        <v>1.208815770509771</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1952,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2154.6</v>
+        <v>2254.2</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1968,13 +1968,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.02107825512765808</v>
+        <v>0.02014692950849619</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>50.00009282465423</v>
+        <v>47.79087924762666</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -2026,7 +2026,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>3.460385810325657</v>
+        <v>3.688417824185667</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2042,7 +2042,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q18" t="n">
-        <v>776.4</v>
+        <v>728.4000000000001</v>
       </c>
       <c r="R18" t="n">
         <v>71127.60000000001</v>
@@ -2058,13 +2058,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W18" t="n">
-        <v>0.05767309683876095</v>
+        <v>0.06147363040309445</v>
       </c>
       <c r="X18" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y18" t="n">
-        <v>91.61205564142196</v>
+        <v>97.64909390444811</v>
       </c>
       <c r="Z18" t="n">
         <v>0.629536106737947</v>
@@ -2116,7 +2116,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>4.494789816460576</v>
+        <v>4.317305519660552</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2132,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q19" t="n">
-        <v>583.8000000000001</v>
+        <v>607.8000000000001</v>
       </c>
       <c r="R19" t="n">
         <v>64144.3</v>
@@ -2148,13 +2148,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W19" t="n">
-        <v>0.07491316360767625</v>
+        <v>0.07195509199434254</v>
       </c>
       <c r="X19" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y19" t="n">
-        <v>109.8737581363481</v>
+        <v>105.5352089503126</v>
       </c>
       <c r="Z19" t="n">
         <v>0.6818112429968274</v>
@@ -2206,7 +2206,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>2.491075597250183</v>
+        <v>2.364090181772136</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2222,7 +2222,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q20" t="n">
-        <v>1050</v>
+        <v>1106.4</v>
       </c>
       <c r="R20" t="n">
         <v>48455.2</v>
@@ -2238,13 +2238,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W20" t="n">
-        <v>0.04151792662083639</v>
+        <v>0.03940150302953561</v>
       </c>
       <c r="X20" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y20" t="n">
-        <v>46.14780952380952</v>
+        <v>43.79537237888647</v>
       </c>
       <c r="Z20" t="n">
         <v>0.8996727482680539</v>
@@ -2253,122 +2253,122 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>glm-5-3-flash</t>
+          <t>claude-haiku-5-5</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>GLM 5.3 Flash</t>
+          <t>Claude Haiku 5.5 (Max)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Claude Haiku 5.5 (max)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H21" t="b">
         <v>1</v>
       </c>
       <c r="I21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>41.807466113455</v>
+        <v>43.3950199670746</v>
       </c>
       <c r="K21" t="n">
-        <v>2.475279225189757</v>
+        <v>6.146603394769774</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
-        <v>1.193653</v>
+        <v>1.064978</v>
       </c>
       <c r="N21" t="n">
-        <v>1.159316</v>
+        <v>0.983896</v>
       </c>
       <c r="O21" t="n">
-        <v>0.011012</v>
+        <v>0.016559</v>
       </c>
       <c r="P21" t="n">
-        <v>0.023325</v>
+        <v>0.064523</v>
       </c>
       <c r="Q21" t="n">
-        <v>1013.4</v>
+        <v>423.6</v>
       </c>
       <c r="R21" t="n">
-        <v>68673.2</v>
+        <v>162164.2</v>
       </c>
       <c r="S21" t="n">
-        <v>22023.7</v>
+        <v>33117.6</v>
       </c>
       <c r="T21" t="n">
-        <v>46649.5</v>
+        <v>129046.6</v>
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="n">
-        <v>35.02480713696107</v>
+        <v>40.74733935074209</v>
       </c>
       <c r="W21" t="n">
-        <v>0.04125465375316262</v>
+        <v>0.1024433899128296</v>
       </c>
       <c r="X21" t="n">
-        <v>0.02855119219042658</v>
+        <v>0.02454147966305898</v>
       </c>
       <c r="Y21" t="n">
-        <v>67.76514702980066</v>
+        <v>382.8238904627007</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.6087886703030441</v>
+        <v>0.2675992602995889</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>gemini-3-8-flash</t>
+          <t>glm-5-3-flash</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (High)</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2380,85 +2380,85 @@
         <v>1</v>
       </c>
       <c r="I22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>40.9262321765904</v>
+        <v>41.807466113455</v>
       </c>
       <c r="K22" t="n">
-        <v>6.200944269180365</v>
+        <v>2.422217040176998</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
-        <v>4.90102</v>
+        <v>1.193653</v>
       </c>
       <c r="N22" t="n">
-        <v>4.63476</v>
+        <v>1.159316</v>
       </c>
       <c r="O22" t="n">
-        <v>0.106033</v>
+        <v>0.011012</v>
       </c>
       <c r="P22" t="n">
-        <v>0.160227</v>
+        <v>0.023325</v>
       </c>
       <c r="Q22" t="n">
-        <v>396</v>
+        <v>1035.6</v>
       </c>
       <c r="R22" t="n">
-        <v>71002.60000000001</v>
+        <v>68673.2</v>
       </c>
       <c r="S22" t="n">
-        <v>28275.4</v>
+        <v>22023.7</v>
       </c>
       <c r="T22" t="n">
-        <v>42727.1</v>
+        <v>46649.5</v>
       </c>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="n">
-        <v>8.350554002348574</v>
+        <v>35.02480713696107</v>
       </c>
       <c r="W22" t="n">
-        <v>0.1033490711530061</v>
+        <v>0.04037028400294997</v>
       </c>
       <c r="X22" t="n">
-        <v>0.119752533750306</v>
+        <v>0.02855119219042658</v>
       </c>
       <c r="Y22" t="n">
-        <v>179.299494949495</v>
+        <v>66.31247585940517</v>
       </c>
       <c r="Z22" t="n">
-        <v>0.5764046975264343</v>
+        <v>0.6087886703030441</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>deepseek-v4-1-flash</t>
+          <t>gemini-3-8-flash</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (Max)</t>
+          <t>Gemini 3.8 Flash (High)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (max)</t>
+          <t>Gemini 3.8 Flash (high)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>DeepSeek</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>deepseek</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2470,85 +2470,85 @@
         <v>1</v>
       </c>
       <c r="I23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>39.456167472527</v>
+        <v>40.9262321765904</v>
       </c>
       <c r="K23" t="n">
-        <v>8.596114917761874</v>
+        <v>4.372460702627181</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
-        <v>3.127974</v>
+        <v>4.90102</v>
       </c>
       <c r="N23" t="n">
-        <v>3.021685</v>
+        <v>4.63476</v>
       </c>
       <c r="O23" t="n">
-        <v>0.031085</v>
+        <v>0.106033</v>
       </c>
       <c r="P23" t="n">
-        <v>0.07520300000000001</v>
+        <v>0.160227</v>
       </c>
       <c r="Q23" t="n">
-        <v>275.4</v>
+        <v>561.5999999999999</v>
       </c>
       <c r="R23" t="n">
-        <v>88574</v>
+        <v>71002.60000000001</v>
       </c>
       <c r="S23" t="n">
-        <v>25904.4</v>
+        <v>28275.4</v>
       </c>
       <c r="T23" t="n">
-        <v>62669.6</v>
+        <v>42727.1</v>
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="n">
-        <v>12.61396912906789</v>
+        <v>8.350554002348574</v>
       </c>
       <c r="W23" t="n">
-        <v>0.1432685819626979</v>
+        <v>0.07287434504378634</v>
       </c>
       <c r="X23" t="n">
-        <v>0.07927718783579227</v>
+        <v>0.119752533750306</v>
       </c>
       <c r="Y23" t="n">
-        <v>321.6194625998548</v>
+        <v>126.4291310541311</v>
       </c>
       <c r="Z23" t="n">
-        <v>0.4454599258532639</v>
+        <v>0.5764046975264343</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>mistral-large-4</t>
+          <t>deepseek-v4-1-flash</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Mistral Large 4 Preview</t>
+          <t>DeepSeek V4.1 Flash (Max)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mistral Large 4 Preview</t>
+          <t>DeepSeek V4.1 Flash (max)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Mistral</t>
+          <t>DeepSeek</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>mistral</t>
+          <t>deepseek</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2560,90 +2560,90 @@
         <v>1</v>
       </c>
       <c r="I24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>38.3770408917494</v>
+        <v>39.456167472527</v>
       </c>
       <c r="K24" t="n">
-        <v>4.541661643994012</v>
+        <v>8.558821577554664</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>6.131298</v>
+        <v>3.127974</v>
       </c>
       <c r="N24" t="n">
-        <v>5.841498</v>
+        <v>3.021685</v>
       </c>
       <c r="O24" t="n">
-        <v>0.072395</v>
+        <v>0.031085</v>
       </c>
       <c r="P24" t="n">
-        <v>0.217404</v>
+        <v>0.07520300000000001</v>
       </c>
       <c r="Q24" t="n">
-        <v>506.9999999999999</v>
+        <v>276.6</v>
       </c>
       <c r="R24" t="n">
-        <v>69330</v>
+        <v>88574</v>
       </c>
       <c r="S24" t="n">
-        <v>17319.4</v>
+        <v>25904.4</v>
       </c>
       <c r="T24" t="n">
-        <v>52010.6</v>
+        <v>62669.6</v>
       </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="n">
-        <v>6.259203335370325</v>
+        <v>12.61396912906789</v>
       </c>
       <c r="W24" t="n">
-        <v>0.07569436073323355</v>
+        <v>0.1426470262925777</v>
       </c>
       <c r="X24" t="n">
-        <v>0.1597647410412551</v>
+        <v>0.07927718783579227</v>
       </c>
       <c r="Y24" t="n">
-        <v>136.7455621301775</v>
+        <v>320.2241503976862</v>
       </c>
       <c r="Z24" t="n">
-        <v>0.5535416254399164</v>
+        <v>0.4454599258532639</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>gpt-6-luna</t>
+          <t>mistral-large-4</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (Max)</t>
+          <t>Mistral Large 4 Preview</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (max)</t>
+          <t>Mistral Large 4 Preview</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Mistral</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>mistral</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H25" t="b">
@@ -2653,177 +2653,177 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>38.1245186869738</v>
+        <v>38.3770408917494</v>
       </c>
       <c r="K25" t="n">
-        <v>5.883413377619413</v>
+        <v>4.541661643994012</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
-        <v>0.326276</v>
+        <v>6.131298</v>
       </c>
       <c r="N25" t="n">
-        <v>0.30127</v>
+        <v>5.841498</v>
       </c>
       <c r="O25" t="n">
-        <v>0.005561</v>
+        <v>0.072395</v>
       </c>
       <c r="P25" t="n">
-        <v>0.019445</v>
+        <v>0.217404</v>
       </c>
       <c r="Q25" t="n">
-        <v>388.8</v>
+        <v>506.9999999999999</v>
       </c>
       <c r="R25" t="n">
-        <v>50011.7</v>
+        <v>69330</v>
       </c>
       <c r="S25" t="n">
-        <v>11122</v>
+        <v>17319.4</v>
       </c>
       <c r="T25" t="n">
-        <v>38889.7</v>
+        <v>52010.6</v>
       </c>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="n">
-        <v>116.8474502782117</v>
+        <v>6.259203335370325</v>
       </c>
       <c r="W25" t="n">
-        <v>0.09805688962699023</v>
+        <v>0.07569436073323355</v>
       </c>
       <c r="X25" t="n">
-        <v>0.008558167059863248</v>
+        <v>0.1597647410412551</v>
       </c>
       <c r="Y25" t="n">
-        <v>128.6309156378601</v>
+        <v>136.7455621301775</v>
       </c>
       <c r="Z25" t="n">
-        <v>0.7623119927331765</v>
+        <v>0.5535416254399164</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>qwen3-8-27b</t>
+          <t>gpt-6-luna</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (Xhigh)</t>
+          <t>GPT-6 Luna (Max)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (xhigh)</t>
+          <t>GPT-6 Luna (max)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H26" t="b">
         <v>1</v>
       </c>
       <c r="I26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>33.6962858057476</v>
+        <v>38.1245186869738</v>
       </c>
       <c r="K26" t="n">
-        <v>1.78287226485437</v>
+        <v>5.811664433989909</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
-        <v>2.505679</v>
+        <v>0.326276</v>
       </c>
       <c r="N26" t="n">
-        <v>2.305287</v>
+        <v>0.30127</v>
       </c>
       <c r="O26" t="n">
-        <v>0.05726</v>
+        <v>0.005561</v>
       </c>
       <c r="P26" t="n">
-        <v>0.143133</v>
+        <v>0.019445</v>
       </c>
       <c r="Q26" t="n">
-        <v>1134</v>
+        <v>393.6</v>
       </c>
       <c r="R26" t="n">
-        <v>66797.5</v>
+        <v>50011.7</v>
       </c>
       <c r="S26" t="n">
-        <v>19086.6</v>
+        <v>11122</v>
       </c>
       <c r="T26" t="n">
-        <v>47710.9</v>
+        <v>38889.7</v>
       </c>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="n">
-        <v>13.44796592290856</v>
+        <v>116.8474502782117</v>
       </c>
       <c r="W26" t="n">
-        <v>0.02971453774757284</v>
+        <v>0.09686107389983181</v>
       </c>
       <c r="X26" t="n">
-        <v>0.0743606881317645</v>
+        <v>0.008558167059863248</v>
       </c>
       <c r="Y26" t="n">
-        <v>58.90432098765432</v>
+        <v>127.0622459349593</v>
       </c>
       <c r="Z26" t="n">
-        <v>0.504454295531234</v>
+        <v>0.7623119927331765</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>k2-horizon-375b-a23b</t>
+          <t>qwen3-8-27b</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Qwen3.8 27B (Xhigh)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Qwen3.8 27B (xhigh)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Institute of Foundation Models</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ifm</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H27" t="b">
@@ -2833,54 +2833,82 @@
         <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>30.5015302696723</v>
-      </c>
-      <c r="K27" t="inlineStr"/>
+        <v>33.6962858057476</v>
+      </c>
+      <c r="K27" t="n">
+        <v>1.78287226485437</v>
+      </c>
       <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
-      <c r="T27" t="inlineStr"/>
+      <c r="M27" t="n">
+        <v>2.505679</v>
+      </c>
+      <c r="N27" t="n">
+        <v>2.305287</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0.05726</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0.143133</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>1134</v>
+      </c>
+      <c r="R27" t="n">
+        <v>66797.5</v>
+      </c>
+      <c r="S27" t="n">
+        <v>19086.6</v>
+      </c>
+      <c r="T27" t="n">
+        <v>47710.9</v>
+      </c>
       <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="inlineStr"/>
+      <c r="V27" t="n">
+        <v>13.44796592290856</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0.02971453774757284</v>
+      </c>
+      <c r="X27" t="n">
+        <v>0.0743606881317645</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>58.90432098765432</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>0.504454295531234</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>minimax-m3</t>
+          <t>k2-horizon-375b-a23b</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>Institute of Foundation Models</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>minimax</t>
+          <t>ifm</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2895,82 +2923,54 @@
         <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>29.2202932236316</v>
-      </c>
-      <c r="K28" t="n">
-        <v>3.449857523451192</v>
-      </c>
+        <v>30.5015302696723</v>
+      </c>
+      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
-      <c r="M28" t="n">
-        <v>1.912899</v>
-      </c>
-      <c r="N28" t="n">
-        <v>1.855069</v>
-      </c>
-      <c r="O28" t="n">
-        <v>0.031649</v>
-      </c>
-      <c r="P28" t="n">
-        <v>0.026182</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>508.2</v>
-      </c>
-      <c r="R28" t="n">
-        <v>48192</v>
-      </c>
-      <c r="S28" t="n">
-        <v>26373.8</v>
-      </c>
-      <c r="T28" t="n">
-        <v>21818.2</v>
-      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
-      <c r="V28" t="n">
-        <v>15.27539782478406</v>
-      </c>
-      <c r="W28" t="n">
-        <v>0.0574976253908532</v>
-      </c>
-      <c r="X28" t="n">
-        <v>0.06546474346988973</v>
-      </c>
-      <c r="Y28" t="n">
-        <v>94.82880755608028</v>
-      </c>
-      <c r="Z28" t="n">
-        <v>0.6063307856829266</v>
-      </c>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>inkling</t>
+          <t>minimax-m3</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Inkling (Xhigh)</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Inkling (xhigh)</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Thinking Machines</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>thinking-machines</t>
+          <t>minimax</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2985,82 +2985,82 @@
         <v>1</v>
       </c>
       <c r="J29" t="n">
-        <v>24.9847810999384</v>
+        <v>29.2202932236316</v>
       </c>
       <c r="K29" t="n">
-        <v>7.037966507024901</v>
+        <v>3.169229199960043</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
-        <v>2.418996</v>
+        <v>1.912899</v>
       </c>
       <c r="N29" t="n">
-        <v>2.278639</v>
+        <v>1.855069</v>
       </c>
       <c r="O29" t="n">
-        <v>0.04559</v>
+        <v>0.031649</v>
       </c>
       <c r="P29" t="n">
-        <v>0.094767</v>
+        <v>0.026182</v>
       </c>
       <c r="Q29" t="n">
-        <v>213</v>
+        <v>553.2</v>
       </c>
       <c r="R29" t="n">
-        <v>34656</v>
+        <v>48192</v>
       </c>
       <c r="S29" t="n">
-        <v>11256.8</v>
+        <v>26373.8</v>
       </c>
       <c r="T29" t="n">
-        <v>23399.2</v>
+        <v>21818.2</v>
       </c>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="n">
-        <v>10.32857478885389</v>
+        <v>15.27539782478406</v>
       </c>
       <c r="W29" t="n">
-        <v>0.1172994417837483</v>
+        <v>0.05282048666600072</v>
       </c>
       <c r="X29" t="n">
-        <v>0.09681877901287532</v>
+        <v>0.06546474346988973</v>
       </c>
       <c r="Y29" t="n">
-        <v>162.7042253521127</v>
+        <v>87.11496746203903</v>
       </c>
       <c r="Z29" t="n">
-        <v>0.7209366660877885</v>
+        <v>0.6063307856829266</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
+          <t>inkling</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
+          <t>Inkling (Xhigh)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra</t>
+          <t>Inkling (xhigh)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Thinking Machines</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>thinking-machines</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3075,87 +3075,87 @@
         <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>22.9279123422858</v>
+        <v>24.9847810999384</v>
       </c>
       <c r="K30" t="n">
-        <v>8.491819386031777</v>
+        <v>7.037966507024901</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
-        <v>0.717257</v>
+        <v>2.418996</v>
       </c>
       <c r="N30" t="n">
-        <v>0.646342</v>
+        <v>2.278639</v>
       </c>
       <c r="O30" t="n">
-        <v>0.03329</v>
+        <v>0.04559</v>
       </c>
       <c r="P30" t="n">
-        <v>0.037626</v>
+        <v>0.094767</v>
       </c>
       <c r="Q30" t="n">
-        <v>162</v>
+        <v>213</v>
       </c>
       <c r="R30" t="n">
-        <v>28366.1</v>
+        <v>34656</v>
       </c>
       <c r="S30" t="n">
-        <v>13315.8</v>
+        <v>11256.8</v>
       </c>
       <c r="T30" t="n">
-        <v>15050.3</v>
+        <v>23399.2</v>
       </c>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="n">
-        <v>31.96610467696488</v>
+        <v>10.32857478885389</v>
       </c>
       <c r="W30" t="n">
-        <v>0.1415303231005296</v>
+        <v>0.1172994417837483</v>
       </c>
       <c r="X30" t="n">
-        <v>0.0312831360000085</v>
+        <v>0.09681877901287532</v>
       </c>
       <c r="Y30" t="n">
-        <v>175.0993827160494</v>
+        <v>162.7042253521127</v>
       </c>
       <c r="Z30" t="n">
-        <v>0.8082856769977473</v>
+        <v>0.7209366660877885</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>muse-glimmer</t>
+          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Muse Glimmer (High)</t>
+          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Muse Glimmer (high)</t>
+          <t>Nemotron 3 Ultra</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>nvidia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H31" t="b">
@@ -3165,50 +3165,140 @@
         <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>17.4754176089465</v>
+        <v>22.9279123422858</v>
       </c>
       <c r="K31" t="n">
-        <v>7.836510138541032</v>
+        <v>7.49278181120451</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
-        <v>0.227808</v>
+        <v>0.717257</v>
       </c>
       <c r="N31" t="n">
-        <v>0.209009</v>
+        <v>0.646342</v>
       </c>
       <c r="O31" t="n">
-        <v>0.005909</v>
+        <v>0.03329</v>
       </c>
       <c r="P31" t="n">
-        <v>0.01289</v>
+        <v>0.037626</v>
       </c>
       <c r="Q31" t="n">
-        <v>133.8</v>
+        <v>183.6</v>
       </c>
       <c r="R31" t="n">
-        <v>13925.2</v>
+        <v>28366.1</v>
       </c>
       <c r="S31" t="n">
-        <v>4377.3</v>
+        <v>13315.8</v>
       </c>
       <c r="T31" t="n">
-        <v>9547.9</v>
+        <v>15050.3</v>
       </c>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="n">
+        <v>31.96610467696488</v>
+      </c>
+      <c r="W31" t="n">
+        <v>0.1248796968534085</v>
+      </c>
+      <c r="X31" t="n">
+        <v>0.0312831360000085</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>154.4994553376906</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>0.8082856769977473</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>muse-glimmer</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Muse Glimmer (High)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Muse Glimmer (high)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>small</t>
+        </is>
+      </c>
+      <c r="H32" t="b">
+        <v>1</v>
+      </c>
+      <c r="I32" t="b">
+        <v>1</v>
+      </c>
+      <c r="J32" t="n">
+        <v>17.4754176089465</v>
+      </c>
+      <c r="K32" t="n">
+        <v>7.162056397109222</v>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="n">
+        <v>0.227808</v>
+      </c>
+      <c r="N32" t="n">
+        <v>0.209009</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0.005909</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0.01289</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>146.4</v>
+      </c>
+      <c r="R32" t="n">
+        <v>13925.2</v>
+      </c>
+      <c r="S32" t="n">
+        <v>4377.3</v>
+      </c>
+      <c r="T32" t="n">
+        <v>9547.9</v>
+      </c>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="n">
         <v>76.71116733805002</v>
       </c>
-      <c r="W31" t="n">
-        <v>0.1306085023090172</v>
-      </c>
-      <c r="X31" t="n">
+      <c r="W32" t="n">
+        <v>0.119367606618487</v>
+      </c>
+      <c r="X32" t="n">
         <v>0.01303591165016704</v>
       </c>
-      <c r="Y31" t="n">
-        <v>104.0747384155456</v>
-      </c>
-      <c r="Z31" t="n">
+      <c r="Y32" t="n">
+        <v>95.11748633879782</v>
+      </c>
+      <c r="Z32" t="n">
         <v>1.254949128841704</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-09)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.575997998600217</v>
+        <v>3.730854674089234</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>939.6</v>
+        <v>900.6</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.05959996664333695</v>
+        <v>0.06218091123482056</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>210.1217539378459</v>
+        <v>219.2209638019098</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.548228138481158</v>
+        <v>6.617890139954361</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>513</v>
+        <v>507.6</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1091371356413526</v>
+        <v>0.1102981689992394</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>128.0066276803119</v>
+        <v>129.3684003152088</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -864,7 +864,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K5" t="n">
-        <v>11.23337441974983</v>
+        <v>11.30447172620395</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -880,7 +880,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q5" t="n">
-        <v>286.2</v>
+        <v>284.4</v>
       </c>
       <c r="R5" t="n">
         <v>35584.1</v>
@@ -896,13 +896,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1872229069958306</v>
+        <v>0.1884078621033991</v>
       </c>
       <c r="X5" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y5" t="n">
-        <v>124.3329839273236</v>
+        <v>125.1199015471167</v>
       </c>
       <c r="Z5" t="n">
         <v>1.505818497087371</v>
@@ -954,7 +954,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>4.494939002723269</v>
+        <v>4.536983500197721</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -970,7 +970,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q6" t="n">
-        <v>712.1999999999999</v>
+        <v>705.6</v>
       </c>
       <c r="R6" t="n">
         <v>78110.8</v>
@@ -986,13 +986,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07491565004538782</v>
+        <v>0.07561639166996201</v>
       </c>
       <c r="X6" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y6" t="n">
-        <v>109.6753720864926</v>
+        <v>110.7012471655329</v>
       </c>
       <c r="Z6" t="n">
         <v>0.6830672066132366</v>
@@ -1044,7 +1044,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K7" t="n">
-        <v>5.257239007301819</v>
+        <v>5.205798312514129</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1060,7 +1060,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q7" t="n">
-        <v>607.1999999999999</v>
+        <v>613.2</v>
       </c>
       <c r="R7" t="n">
         <v>60537.6</v>
@@ -1076,13 +1076,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W7" t="n">
-        <v>0.08762065012169698</v>
+        <v>0.08676330520856881</v>
       </c>
       <c r="X7" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y7" t="n">
-        <v>99.69960474308301</v>
+        <v>98.72407045009784</v>
       </c>
       <c r="Z7" t="n">
         <v>0.8788465144619939</v>
@@ -1134,7 +1134,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K8" t="n">
-        <v>5.396892356097644</v>
+        <v>5.504040689186311</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1150,7 +1150,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q8" t="n">
-        <v>585.6</v>
+        <v>574.2</v>
       </c>
       <c r="R8" t="n">
         <v>27205.5</v>
@@ -1166,13 +1166,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W8" t="n">
-        <v>0.08994820593496072</v>
+        <v>0.09173401148643852</v>
       </c>
       <c r="X8" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y8" t="n">
-        <v>46.45747950819672</v>
+        <v>47.37983281086729</v>
       </c>
       <c r="Z8" t="n">
         <v>1.936140464079432</v>
@@ -1306,7 +1306,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K10" t="n">
-        <v>8.211023152175267</v>
+        <v>8.034712839091748</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1322,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q10" t="n">
-        <v>382.8</v>
+        <v>391.2</v>
       </c>
       <c r="R10" t="n">
         <v>16901.2</v>
@@ -1338,13 +1338,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W10" t="n">
-        <v>0.1368503858695878</v>
+        <v>0.1339118806515291</v>
       </c>
       <c r="X10" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y10" t="n">
-        <v>44.15151515151515</v>
+        <v>43.20347648261759</v>
       </c>
       <c r="Z10" t="n">
         <v>3.099562617499243</v>
@@ -1396,7 +1396,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K11" t="n">
-        <v>7.227793094471992</v>
+        <v>7.031917942860284</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1412,7 +1412,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q11" t="n">
-        <v>430.8</v>
+        <v>442.8</v>
       </c>
       <c r="R11" t="n">
         <v>74809.60000000001</v>
@@ -1428,13 +1428,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1204632182411999</v>
+        <v>0.1171986323810047</v>
       </c>
       <c r="X11" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y11" t="n">
-        <v>173.652739090065</v>
+        <v>168.9467028003614</v>
       </c>
       <c r="Z11" t="n">
         <v>0.6937018032218979</v>
@@ -1486,7 +1486,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K12" t="n">
-        <v>4.52692224464228</v>
+        <v>4.546777166767903</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1502,7 +1502,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q12" t="n">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="R12" t="n">
         <v>38128.4</v>
@@ -1518,13 +1518,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W12" t="n">
-        <v>0.07544870407737132</v>
+        <v>0.07577961944613172</v>
       </c>
       <c r="X12" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y12" t="n">
-        <v>55.49985443959243</v>
+        <v>55.74327485380118</v>
       </c>
       <c r="Z12" t="n">
         <v>1.359439674918279</v>
@@ -1576,7 +1576,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K13" t="n">
-        <v>8.680922522015974</v>
+        <v>8.334889215245841</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1592,7 +1592,7 @@
         <v>0.145035</v>
       </c>
       <c r="Q13" t="n">
-        <v>332.4</v>
+        <v>346.2</v>
       </c>
       <c r="R13" t="n">
         <v>60200.2</v>
@@ -1608,13 +1608,13 @@
         <v>6.17518114688861</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1446820420335996</v>
+        <v>0.1389148202540973</v>
       </c>
       <c r="X13" t="n">
         <v>0.161938569284539</v>
       </c>
       <c r="Y13" t="n">
-        <v>181.1077015643803</v>
+        <v>173.8885037550549</v>
       </c>
       <c r="Z13" t="n">
         <v>0.7988729401558218</v>
@@ -1666,7 +1666,7 @@
         <v>47.6305176437724</v>
       </c>
       <c r="K14" t="n">
-        <v>8.114227877985076</v>
+        <v>8.15591055544048</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1682,7 @@
         <v>0.208445</v>
       </c>
       <c r="Q14" t="n">
-        <v>352.2</v>
+        <v>350.4</v>
       </c>
       <c r="R14" t="n">
         <v>30999.6</v>
@@ -1698,13 +1698,13 @@
         <v>8.555202665891516</v>
       </c>
       <c r="W14" t="n">
-        <v>0.1352371312997513</v>
+        <v>0.1359318425906747</v>
       </c>
       <c r="X14" t="n">
         <v>0.1168879381416492</v>
       </c>
       <c r="Y14" t="n">
-        <v>88.01703577512777</v>
+        <v>88.46917808219179</v>
       </c>
       <c r="Z14" t="n">
         <v>1.53648813674281</v>
@@ -1846,7 +1846,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>1.761376674183966</v>
+        <v>1.921368997554471</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1862,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1578</v>
+        <v>1446.6</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1878,13 +1878,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.0293562779030661</v>
+        <v>0.03202281662590786</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>40.73238276299113</v>
+        <v>44.43225494262408</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1936,7 +1936,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.208815770509771</v>
+        <v>1.236797617049349</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1952,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2254.2</v>
+        <v>2203.2</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1968,13 +1968,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.02014692950849619</v>
+        <v>0.02061329361748915</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>47.79087924762666</v>
+        <v>48.89714960058097</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -2026,7 +2026,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>3.688417824185667</v>
+        <v>3.9837537709621</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2042,7 +2042,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q18" t="n">
-        <v>728.4000000000001</v>
+        <v>674.4</v>
       </c>
       <c r="R18" t="n">
         <v>71127.60000000001</v>
@@ -2058,13 +2058,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W18" t="n">
-        <v>0.06147363040309445</v>
+        <v>0.06639589618270167</v>
       </c>
       <c r="X18" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y18" t="n">
-        <v>97.64909390444811</v>
+        <v>105.4679715302491</v>
       </c>
       <c r="Z18" t="n">
         <v>0.629536106737947</v>
@@ -2116,7 +2116,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>4.317305519660552</v>
+        <v>4.118107807359831</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2132,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q19" t="n">
-        <v>607.8000000000001</v>
+        <v>637.1999999999999</v>
       </c>
       <c r="R19" t="n">
         <v>64144.3</v>
@@ -2148,13 +2148,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W19" t="n">
-        <v>0.07195509199434254</v>
+        <v>0.06863513012266385</v>
       </c>
       <c r="X19" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y19" t="n">
-        <v>105.5352089503126</v>
+        <v>100.6658819836786</v>
       </c>
       <c r="Z19" t="n">
         <v>0.6818112429968274</v>
@@ -2206,7 +2206,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>2.364090181772136</v>
+        <v>2.284791559322757</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2222,7 +2222,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q20" t="n">
-        <v>1106.4</v>
+        <v>1144.8</v>
       </c>
       <c r="R20" t="n">
         <v>48455.2</v>
@@ -2238,13 +2238,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W20" t="n">
-        <v>0.03940150302953561</v>
+        <v>0.03807985932204595</v>
       </c>
       <c r="X20" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y20" t="n">
-        <v>43.79537237888647</v>
+        <v>42.32634521313766</v>
       </c>
       <c r="Z20" t="n">
         <v>0.8996727482680539</v>
@@ -2296,7 +2296,7 @@
         <v>43.3950199670746</v>
       </c>
       <c r="K21" t="n">
-        <v>6.146603394769774</v>
+        <v>6.120595199869479</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.064523</v>
       </c>
       <c r="Q21" t="n">
-        <v>423.6</v>
+        <v>425.4</v>
       </c>
       <c r="R21" t="n">
         <v>162164.2</v>
@@ -2328,13 +2328,13 @@
         <v>40.74733935074209</v>
       </c>
       <c r="W21" t="n">
-        <v>0.1024433899128296</v>
+        <v>0.1020099199978246</v>
       </c>
       <c r="X21" t="n">
         <v>0.02454147966305898</v>
       </c>
       <c r="Y21" t="n">
-        <v>382.8238904627007</v>
+        <v>381.2040432534086</v>
       </c>
       <c r="Z21" t="n">
         <v>0.2675992602995889</v>
@@ -2386,7 +2386,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K22" t="n">
-        <v>2.422217040176998</v>
+        <v>2.561731992246017</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q22" t="n">
-        <v>1035.6</v>
+        <v>979.2</v>
       </c>
       <c r="R22" t="n">
         <v>68673.2</v>
@@ -2418,13 +2418,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W22" t="n">
-        <v>0.04037028400294997</v>
+        <v>0.04269553320410029</v>
       </c>
       <c r="X22" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y22" t="n">
-        <v>66.31247585940517</v>
+        <v>70.13194444444444</v>
       </c>
       <c r="Z22" t="n">
         <v>0.6087886703030441</v>
@@ -2476,7 +2476,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K23" t="n">
-        <v>4.372460702627181</v>
+        <v>4.308024439641095</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2492,7 +2492,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q23" t="n">
-        <v>561.5999999999999</v>
+        <v>570</v>
       </c>
       <c r="R23" t="n">
         <v>71002.60000000001</v>
@@ -2508,13 +2508,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W23" t="n">
-        <v>0.07287434504378634</v>
+        <v>0.07180040732735159</v>
       </c>
       <c r="X23" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y23" t="n">
-        <v>126.4291310541311</v>
+        <v>124.5659649122807</v>
       </c>
       <c r="Z23" t="n">
         <v>0.5764046975264343</v>
@@ -2566,7 +2566,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K24" t="n">
-        <v>8.558821577554664</v>
+        <v>8.254428341532845</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2582,7 +2582,7 @@
         <v>0.07520300000000001</v>
       </c>
       <c r="Q24" t="n">
-        <v>276.6</v>
+        <v>286.8</v>
       </c>
       <c r="R24" t="n">
         <v>88574</v>
@@ -2598,13 +2598,13 @@
         <v>12.61396912906789</v>
       </c>
       <c r="W24" t="n">
-        <v>0.1426470262925777</v>
+        <v>0.1375738056922141</v>
       </c>
       <c r="X24" t="n">
         <v>0.07927718783579227</v>
       </c>
       <c r="Y24" t="n">
-        <v>320.2241503976862</v>
+        <v>308.8354253835425</v>
       </c>
       <c r="Z24" t="n">
         <v>0.4454599258532639</v>
@@ -2655,9 +2655,7 @@
       <c r="J25" t="n">
         <v>38.3770408917494</v>
       </c>
-      <c r="K25" t="n">
-        <v>4.541661643994012</v>
-      </c>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
         <v>6.131298</v>
@@ -2671,9 +2669,7 @@
       <c r="P25" t="n">
         <v>0.217404</v>
       </c>
-      <c r="Q25" t="n">
-        <v>506.9999999999999</v>
-      </c>
+      <c r="Q25" t="inlineStr"/>
       <c r="R25" t="n">
         <v>69330</v>
       </c>
@@ -2687,15 +2683,11 @@
       <c r="V25" t="n">
         <v>6.259203335370325</v>
       </c>
-      <c r="W25" t="n">
-        <v>0.07569436073323355</v>
-      </c>
+      <c r="W25" t="inlineStr"/>
       <c r="X25" t="n">
         <v>0.1597647410412551</v>
       </c>
-      <c r="Y25" t="n">
-        <v>136.7455621301775</v>
-      </c>
+      <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="n">
         <v>0.5535416254399164</v>
       </c>
@@ -2746,7 +2738,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K26" t="n">
-        <v>5.811664433989909</v>
+        <v>5.68174645111383</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2762,7 +2754,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q26" t="n">
-        <v>393.6</v>
+        <v>402.6</v>
       </c>
       <c r="R26" t="n">
         <v>50011.7</v>
@@ -2778,13 +2770,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W26" t="n">
-        <v>0.09686107389983181</v>
+        <v>0.09469577418523049</v>
       </c>
       <c r="X26" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y26" t="n">
-        <v>127.0622459349593</v>
+        <v>124.2218082463984</v>
       </c>
       <c r="Z26" t="n">
         <v>0.7623119927331765</v>
@@ -2836,7 +2828,7 @@
         <v>33.6962858057476</v>
       </c>
       <c r="K27" t="n">
-        <v>1.78287226485437</v>
+        <v>1.840321453071961</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2852,7 +2844,7 @@
         <v>0.143133</v>
       </c>
       <c r="Q27" t="n">
-        <v>1134</v>
+        <v>1098.6</v>
       </c>
       <c r="R27" t="n">
         <v>66797.5</v>
@@ -2868,13 +2860,13 @@
         <v>13.44796592290856</v>
       </c>
       <c r="W27" t="n">
-        <v>0.02971453774757284</v>
+        <v>0.03067202421786601</v>
       </c>
       <c r="X27" t="n">
         <v>0.0743606881317645</v>
       </c>
       <c r="Y27" t="n">
-        <v>58.90432098765432</v>
+        <v>60.80238485344985</v>
       </c>
       <c r="Z27" t="n">
         <v>0.504454295531234</v>
@@ -2988,7 +2980,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K29" t="n">
-        <v>3.169229199960043</v>
+        <v>3.239500357387096</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -3004,7 +2996,7 @@
         <v>0.026182</v>
       </c>
       <c r="Q29" t="n">
-        <v>553.2</v>
+        <v>541.1999999999999</v>
       </c>
       <c r="R29" t="n">
         <v>48192</v>
@@ -3020,13 +3012,13 @@
         <v>15.27539782478406</v>
       </c>
       <c r="W29" t="n">
-        <v>0.05282048666600072</v>
+        <v>0.05399167262311826</v>
       </c>
       <c r="X29" t="n">
         <v>0.06546474346988973</v>
       </c>
       <c r="Y29" t="n">
-        <v>87.11496746203903</v>
+        <v>89.04656319290467</v>
       </c>
       <c r="Z29" t="n">
         <v>0.6063307856829266</v>
@@ -3078,7 +3070,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K30" t="n">
-        <v>7.037966507024901</v>
+        <v>7.348465029393647</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3094,7 +3086,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q30" t="n">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="R30" t="n">
         <v>34656</v>
@@ -3110,13 +3102,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W30" t="n">
-        <v>0.1172994417837483</v>
+        <v>0.1224744171565608</v>
       </c>
       <c r="X30" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y30" t="n">
-        <v>162.7042253521127</v>
+        <v>169.8823529411765</v>
       </c>
       <c r="Z30" t="n">
         <v>0.7209366660877885</v>
@@ -3168,7 +3160,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K31" t="n">
-        <v>7.49278181120451</v>
+        <v>7.21003532776283</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3184,7 +3176,7 @@
         <v>0.037626</v>
       </c>
       <c r="Q31" t="n">
-        <v>183.6</v>
+        <v>190.8</v>
       </c>
       <c r="R31" t="n">
         <v>28366.1</v>
@@ -3200,13 +3192,13 @@
         <v>31.96610467696488</v>
       </c>
       <c r="W31" t="n">
-        <v>0.1248796968534085</v>
+        <v>0.1201672554627138</v>
       </c>
       <c r="X31" t="n">
         <v>0.0312831360000085</v>
       </c>
       <c r="Y31" t="n">
-        <v>154.4994553376906</v>
+        <v>148.66928721174</v>
       </c>
       <c r="Z31" t="n">
         <v>0.8082856769977473</v>
@@ -3258,7 +3250,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K32" t="n">
-        <v>7.162056397109222</v>
+        <v>8.282188440259006</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3274,7 +3266,7 @@
         <v>0.01289</v>
       </c>
       <c r="Q32" t="n">
-        <v>146.4</v>
+        <v>126.6</v>
       </c>
       <c r="R32" t="n">
         <v>13925.2</v>
@@ -3290,13 +3282,13 @@
         <v>76.71116733805002</v>
       </c>
       <c r="W32" t="n">
-        <v>0.119367606618487</v>
+        <v>0.1380364740043168</v>
       </c>
       <c r="X32" t="n">
         <v>0.01303591165016704</v>
       </c>
       <c r="Y32" t="n">
-        <v>95.11748633879782</v>
+        <v>109.9936808846762</v>
       </c>
       <c r="Z32" t="n">
         <v>1.254949128841704</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-10)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.418893390360146</v>
+        <v>4.505267381571251</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>782.4</v>
+        <v>767.4</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.0736482231726691</v>
+        <v>0.07508778969285418</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>152.308282208589</v>
+        <v>155.285379202502</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.730854674089234</v>
+        <v>3.886199074120708</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>900.6</v>
+        <v>864.6</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.06218091123482056</v>
+        <v>0.06476998456867845</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>219.2209638019098</v>
+        <v>228.3488318297478</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.617890139954361</v>
+        <v>6.70507192622921</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>507.6</v>
+        <v>501</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1102981689992394</v>
+        <v>0.1117511987704868</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>129.3684003152088</v>
+        <v>131.0726546906187</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -864,7 +864,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K5" t="n">
-        <v>11.30447172620395</v>
+        <v>11.35237203012854</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -880,7 +880,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q5" t="n">
-        <v>284.4</v>
+        <v>283.2</v>
       </c>
       <c r="R5" t="n">
         <v>35584.1</v>
@@ -896,13 +896,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1884078621033991</v>
+        <v>0.1892062005021423</v>
       </c>
       <c r="X5" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y5" t="n">
-        <v>125.1199015471167</v>
+        <v>125.6500706214689</v>
       </c>
       <c r="Z5" t="n">
         <v>1.505818497087371</v>
@@ -954,7 +954,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>4.536983500197721</v>
+        <v>4.544712603264497</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -970,7 +970,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q6" t="n">
-        <v>705.6</v>
+        <v>704.4</v>
       </c>
       <c r="R6" t="n">
         <v>78110.8</v>
@@ -986,13 +986,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07561639166996201</v>
+        <v>0.07574521005440829</v>
       </c>
       <c r="X6" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y6" t="n">
-        <v>110.7012471655329</v>
+        <v>110.8898353208404</v>
       </c>
       <c r="Z6" t="n">
         <v>0.6830672066132366</v>
@@ -1044,7 +1044,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K7" t="n">
-        <v>5.205798312514129</v>
+        <v>5.374066540797414</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1060,7 +1060,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q7" t="n">
-        <v>613.2</v>
+        <v>594</v>
       </c>
       <c r="R7" t="n">
         <v>60537.6</v>
@@ -1076,13 +1076,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W7" t="n">
-        <v>0.08676330520856881</v>
+        <v>0.08956777567995691</v>
       </c>
       <c r="X7" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y7" t="n">
-        <v>98.72407045009784</v>
+        <v>101.9151515151515</v>
       </c>
       <c r="Z7" t="n">
         <v>0.8788465144619939</v>
@@ -1134,7 +1134,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K8" t="n">
-        <v>5.504040689186311</v>
+        <v>5.515567475969948</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1150,7 +1150,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q8" t="n">
-        <v>574.2</v>
+        <v>573</v>
       </c>
       <c r="R8" t="n">
         <v>27205.5</v>
@@ -1166,13 +1166,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W8" t="n">
-        <v>0.09173401148643852</v>
+        <v>0.09192612459949913</v>
       </c>
       <c r="X8" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y8" t="n">
-        <v>47.37983281086729</v>
+        <v>47.47905759162304</v>
       </c>
       <c r="Z8" t="n">
         <v>1.936140464079432</v>
@@ -1306,7 +1306,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K10" t="n">
-        <v>8.034712839091748</v>
+        <v>8.644608533148219</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1322,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q10" t="n">
-        <v>391.2</v>
+        <v>363.6</v>
       </c>
       <c r="R10" t="n">
         <v>16901.2</v>
@@ -1338,13 +1338,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W10" t="n">
-        <v>0.1339118806515291</v>
+        <v>0.1440768088858037</v>
       </c>
       <c r="X10" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y10" t="n">
-        <v>43.20347648261759</v>
+        <v>46.48294829482949</v>
       </c>
       <c r="Z10" t="n">
         <v>3.099562617499243</v>
@@ -1396,7 +1396,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K11" t="n">
-        <v>7.031917942860284</v>
+        <v>7.247982460657667</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1412,7 +1412,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q11" t="n">
-        <v>442.8</v>
+        <v>429.6</v>
       </c>
       <c r="R11" t="n">
         <v>74809.60000000001</v>
@@ -1428,13 +1428,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1171986323810047</v>
+        <v>0.1207997076776278</v>
       </c>
       <c r="X11" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y11" t="n">
-        <v>168.9467028003614</v>
+        <v>174.1378026070764</v>
       </c>
       <c r="Z11" t="n">
         <v>0.6937018032218979</v>
@@ -1486,7 +1486,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K12" t="n">
-        <v>4.546777166767903</v>
+        <v>4.835192136301688</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1502,7 +1502,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q12" t="n">
-        <v>684</v>
+        <v>643.2</v>
       </c>
       <c r="R12" t="n">
         <v>38128.4</v>
@@ -1518,13 +1518,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W12" t="n">
-        <v>0.07577961944613172</v>
+        <v>0.08058653560502813</v>
       </c>
       <c r="X12" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y12" t="n">
-        <v>55.74327485380118</v>
+        <v>59.27922885572139</v>
       </c>
       <c r="Z12" t="n">
         <v>1.359439674918279</v>
@@ -1576,7 +1576,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K13" t="n">
-        <v>8.334889215245841</v>
+        <v>6.072261461107134</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1592,7 +1592,7 @@
         <v>0.145035</v>
       </c>
       <c r="Q13" t="n">
-        <v>346.2</v>
+        <v>475.2</v>
       </c>
       <c r="R13" t="n">
         <v>60200.2</v>
@@ -1608,13 +1608,13 @@
         <v>6.17518114688861</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1389148202540973</v>
+        <v>0.1012043576851189</v>
       </c>
       <c r="X13" t="n">
         <v>0.161938569284539</v>
       </c>
       <c r="Y13" t="n">
-        <v>173.8885037550549</v>
+        <v>126.6839225589226</v>
       </c>
       <c r="Z13" t="n">
         <v>0.7988729401558218</v>
@@ -1666,7 +1666,7 @@
         <v>47.6305176437724</v>
       </c>
       <c r="K14" t="n">
-        <v>8.15591055544048</v>
+        <v>9.248644202674251</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1682,7 @@
         <v>0.208445</v>
       </c>
       <c r="Q14" t="n">
-        <v>350.4</v>
+        <v>309</v>
       </c>
       <c r="R14" t="n">
         <v>30999.6</v>
@@ -1698,13 +1698,13 @@
         <v>8.555202665891516</v>
       </c>
       <c r="W14" t="n">
-        <v>0.1359318425906747</v>
+        <v>0.1541440700445709</v>
       </c>
       <c r="X14" t="n">
         <v>0.1168879381416492</v>
       </c>
       <c r="Y14" t="n">
-        <v>88.46917808219179</v>
+        <v>100.3223300970874</v>
       </c>
       <c r="Z14" t="n">
         <v>1.53648813674281</v>
@@ -1756,7 +1756,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>2.400338533861943</v>
+        <v>2.564690813375406</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1772,7 +1772,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>1161</v>
+        <v>1086.6</v>
       </c>
       <c r="R15" t="n">
         <v>80561.39999999999</v>
@@ -1788,13 +1788,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.04000564223103239</v>
+        <v>0.0427448468895901</v>
       </c>
       <c r="X15" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>69.38966408268733</v>
+        <v>74.1408061844285</v>
       </c>
       <c r="Z15" t="n">
         <v>0.5765360412086756</v>
@@ -1846,7 +1846,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>1.921368997554471</v>
+        <v>2.04521883139242</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1862,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1446.6</v>
+        <v>1359</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1878,13 +1878,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.03202281662590786</v>
+        <v>0.03408698052320699</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>44.43225494262408</v>
+        <v>47.29632082413539</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1936,7 +1936,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.236797617049349</v>
+        <v>1.237134527323675</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1952,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2203.2</v>
+        <v>2202.6</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1968,13 +1968,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.02061329361748915</v>
+        <v>0.02061890878872791</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>48.89714960058097</v>
+        <v>48.91046944520113</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -2026,7 +2026,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>3.9837537709621</v>
+        <v>3.924398982087117</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2042,7 +2042,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q18" t="n">
-        <v>674.4</v>
+        <v>684.6</v>
       </c>
       <c r="R18" t="n">
         <v>71127.60000000001</v>
@@ -2058,13 +2058,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W18" t="n">
-        <v>0.06639589618270167</v>
+        <v>0.06540664970145194</v>
       </c>
       <c r="X18" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y18" t="n">
-        <v>105.4679715302491</v>
+        <v>103.8965819456617</v>
       </c>
       <c r="Z18" t="n">
         <v>0.629536106737947</v>
@@ -2116,7 +2116,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>4.118107807359831</v>
+        <v>4.283477464658315</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2132,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q19" t="n">
-        <v>637.1999999999999</v>
+        <v>612.6</v>
       </c>
       <c r="R19" t="n">
         <v>64144.3</v>
@@ -2148,13 +2148,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W19" t="n">
-        <v>0.06863513012266385</v>
+        <v>0.07139129107763859</v>
       </c>
       <c r="X19" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y19" t="n">
-        <v>100.6658819836786</v>
+        <v>104.7082925236696</v>
       </c>
       <c r="Z19" t="n">
         <v>0.6818112429968274</v>
@@ -2206,7 +2206,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>2.284791559322757</v>
+        <v>2.320054441292081</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2222,7 +2222,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q20" t="n">
-        <v>1144.8</v>
+        <v>1127.4</v>
       </c>
       <c r="R20" t="n">
         <v>48455.2</v>
@@ -2238,13 +2238,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W20" t="n">
-        <v>0.03807985932204595</v>
+        <v>0.03866757402153469</v>
       </c>
       <c r="X20" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y20" t="n">
-        <v>42.32634521313766</v>
+        <v>42.97959907752351</v>
       </c>
       <c r="Z20" t="n">
         <v>0.8996727482680539</v>
@@ -2296,7 +2296,7 @@
         <v>43.3950199670746</v>
       </c>
       <c r="K21" t="n">
-        <v>6.120595199869479</v>
+        <v>6.137909472004893</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.064523</v>
       </c>
       <c r="Q21" t="n">
-        <v>425.4</v>
+        <v>424.2</v>
       </c>
       <c r="R21" t="n">
         <v>162164.2</v>
@@ -2328,13 +2328,13 @@
         <v>40.74733935074209</v>
       </c>
       <c r="W21" t="n">
-        <v>0.1020099199978246</v>
+        <v>0.1022984912000816</v>
       </c>
       <c r="X21" t="n">
         <v>0.02454147966305898</v>
       </c>
       <c r="Y21" t="n">
-        <v>381.2040432534086</v>
+        <v>382.2824139556812</v>
       </c>
       <c r="Z21" t="n">
         <v>0.2675992602995889</v>
@@ -2386,7 +2386,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K22" t="n">
-        <v>2.561731992246017</v>
+        <v>2.929745347824457</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q22" t="n">
-        <v>979.2</v>
+        <v>856.1999999999999</v>
       </c>
       <c r="R22" t="n">
         <v>68673.2</v>
@@ -2418,13 +2418,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W22" t="n">
-        <v>0.04269553320410029</v>
+        <v>0.04882908913040762</v>
       </c>
       <c r="X22" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y22" t="n">
-        <v>70.13194444444444</v>
+        <v>80.2069609904228</v>
       </c>
       <c r="Z22" t="n">
         <v>0.6087886703030441</v>
@@ -2476,7 +2476,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K23" t="n">
-        <v>4.308024439641095</v>
+        <v>4.562567689697927</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2492,7 +2492,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q23" t="n">
-        <v>570</v>
+        <v>538.2</v>
       </c>
       <c r="R23" t="n">
         <v>71002.60000000001</v>
@@ -2508,13 +2508,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W23" t="n">
-        <v>0.07180040732735159</v>
+        <v>0.07604279482829877</v>
       </c>
       <c r="X23" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y23" t="n">
-        <v>124.5659649122807</v>
+        <v>131.926049795615</v>
       </c>
       <c r="Z23" t="n">
         <v>0.5764046975264343</v>
@@ -2566,7 +2566,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K24" t="n">
-        <v>8.254428341532845</v>
+        <v>8.202945420483784</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2582,7 +2582,7 @@
         <v>0.07520300000000001</v>
       </c>
       <c r="Q24" t="n">
-        <v>286.8</v>
+        <v>288.6</v>
       </c>
       <c r="R24" t="n">
         <v>88574</v>
@@ -2598,13 +2598,13 @@
         <v>12.61396912906789</v>
       </c>
       <c r="W24" t="n">
-        <v>0.1375738056922141</v>
+        <v>0.1367157570080631</v>
       </c>
       <c r="X24" t="n">
         <v>0.07927718783579227</v>
       </c>
       <c r="Y24" t="n">
-        <v>308.8354253835425</v>
+        <v>306.9092169092169</v>
       </c>
       <c r="Z24" t="n">
         <v>0.4454599258532639</v>
@@ -2738,7 +2738,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K26" t="n">
-        <v>5.68174645111383</v>
+        <v>6.219334206684143</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2754,7 +2754,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q26" t="n">
-        <v>402.6</v>
+        <v>367.8</v>
       </c>
       <c r="R26" t="n">
         <v>50011.7</v>
@@ -2770,13 +2770,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W26" t="n">
-        <v>0.09469577418523049</v>
+        <v>0.1036555701114024</v>
       </c>
       <c r="X26" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y26" t="n">
-        <v>124.2218082463984</v>
+        <v>135.9752582925503</v>
       </c>
       <c r="Z26" t="n">
         <v>0.7623119927331765</v>
@@ -2980,7 +2980,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K29" t="n">
-        <v>3.239500357387096</v>
+        <v>3.541853724076558</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -2996,7 +2996,7 @@
         <v>0.026182</v>
       </c>
       <c r="Q29" t="n">
-        <v>541.1999999999999</v>
+        <v>495</v>
       </c>
       <c r="R29" t="n">
         <v>48192</v>
@@ -3012,13 +3012,13 @@
         <v>15.27539782478406</v>
       </c>
       <c r="W29" t="n">
-        <v>0.05399167262311826</v>
+        <v>0.05903089540127596</v>
       </c>
       <c r="X29" t="n">
         <v>0.06546474346988973</v>
       </c>
       <c r="Y29" t="n">
-        <v>89.04656319290467</v>
+        <v>97.35757575757576</v>
       </c>
       <c r="Z29" t="n">
         <v>0.6063307856829266</v>
@@ -3070,7 +3070,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K30" t="n">
-        <v>7.348465029393647</v>
+        <v>8.527229044347576</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3086,7 +3086,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q30" t="n">
-        <v>204</v>
+        <v>175.8</v>
       </c>
       <c r="R30" t="n">
         <v>34656</v>
@@ -3102,13 +3102,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W30" t="n">
-        <v>0.1224744171565608</v>
+        <v>0.1421204840724596</v>
       </c>
       <c r="X30" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y30" t="n">
-        <v>169.8823529411765</v>
+        <v>197.1331058020478</v>
       </c>
       <c r="Z30" t="n">
         <v>0.7209366660877885</v>
@@ -3160,7 +3160,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K31" t="n">
-        <v>7.21003532776283</v>
+        <v>6.885258961647388</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3176,7 +3176,7 @@
         <v>0.037626</v>
       </c>
       <c r="Q31" t="n">
-        <v>190.8</v>
+        <v>199.8</v>
       </c>
       <c r="R31" t="n">
         <v>28366.1</v>
@@ -3192,13 +3192,13 @@
         <v>31.96610467696488</v>
       </c>
       <c r="W31" t="n">
-        <v>0.1201672554627138</v>
+        <v>0.1147543160274564</v>
       </c>
       <c r="X31" t="n">
         <v>0.0312831360000085</v>
       </c>
       <c r="Y31" t="n">
-        <v>148.66928721174</v>
+        <v>141.9724724724724</v>
       </c>
       <c r="Z31" t="n">
         <v>0.8082856769977473</v>
@@ -3250,7 +3250,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K32" t="n">
-        <v>8.282188440259006</v>
+        <v>8.82596848936692</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3266,7 +3266,7 @@
         <v>0.01289</v>
       </c>
       <c r="Q32" t="n">
-        <v>126.6</v>
+        <v>118.8</v>
       </c>
       <c r="R32" t="n">
         <v>13925.2</v>
@@ -3282,13 +3282,13 @@
         <v>76.71116733805002</v>
       </c>
       <c r="W32" t="n">
-        <v>0.1380364740043168</v>
+        <v>0.147099474822782</v>
       </c>
       <c r="X32" t="n">
         <v>0.01303591165016704</v>
       </c>
       <c r="Y32" t="n">
-        <v>109.9936808846762</v>
+        <v>117.2154882154882</v>
       </c>
       <c r="Z32" t="n">
         <v>1.254949128841704</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-11)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.505267381571251</v>
+        <v>4.522948964701436</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>767.4</v>
+        <v>764.4</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07508778969285418</v>
+        <v>0.07538248274502395</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>155.285379202502</v>
+        <v>155.894819466248</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.886199074120708</v>
+        <v>3.788912629098741</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>864.6</v>
+        <v>886.8</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.06476998456867845</v>
+        <v>0.06314854381831236</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>228.3488318297478</v>
+        <v>222.6323861073523</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.70507192622921</v>
+        <v>6.802837252006549</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>501</v>
+        <v>493.8</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1117511987704868</v>
+        <v>0.1133806208667758</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>131.0726546906187</v>
+        <v>132.983799108951</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -864,7 +864,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K5" t="n">
-        <v>11.35237203012854</v>
+        <v>11.42498848234684</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -880,7 +880,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q5" t="n">
-        <v>283.2</v>
+        <v>281.4</v>
       </c>
       <c r="R5" t="n">
         <v>35584.1</v>
@@ -896,13 +896,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1892062005021423</v>
+        <v>0.1904164747057807</v>
       </c>
       <c r="X5" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y5" t="n">
-        <v>125.6500706214689</v>
+        <v>126.453802416489</v>
       </c>
       <c r="Z5" t="n">
         <v>1.505818497087371</v>
@@ -954,7 +954,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>4.544712603264497</v>
+        <v>4.468586764013835</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -970,7 +970,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q6" t="n">
-        <v>704.4</v>
+        <v>716.4</v>
       </c>
       <c r="R6" t="n">
         <v>78110.8</v>
@@ -986,13 +986,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07574521005440829</v>
+        <v>0.07447644606689727</v>
       </c>
       <c r="X6" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y6" t="n">
-        <v>110.8898353208404</v>
+        <v>109.0323841429369</v>
       </c>
       <c r="Z6" t="n">
         <v>0.6830672066132366</v>
@@ -1044,7 +1044,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K7" t="n">
-        <v>5.374066540797414</v>
+        <v>5.46234689465035</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1060,7 +1060,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q7" t="n">
-        <v>594</v>
+        <v>584.4</v>
       </c>
       <c r="R7" t="n">
         <v>60537.6</v>
@@ -1076,13 +1076,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W7" t="n">
-        <v>0.08956777567995691</v>
+        <v>0.09103911491083916</v>
       </c>
       <c r="X7" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y7" t="n">
-        <v>101.9151515151515</v>
+        <v>103.5893223819302</v>
       </c>
       <c r="Z7" t="n">
         <v>0.8788465144619939</v>
@@ -1134,7 +1134,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K8" t="n">
-        <v>5.515567475969948</v>
+        <v>6.718580280039924</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1150,7 +1150,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q8" t="n">
-        <v>573</v>
+        <v>470.4</v>
       </c>
       <c r="R8" t="n">
         <v>27205.5</v>
@@ -1166,13 +1166,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W8" t="n">
-        <v>0.09192612459949913</v>
+        <v>0.1119763380006654</v>
       </c>
       <c r="X8" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y8" t="n">
-        <v>47.47905759162304</v>
+        <v>57.83482142857143</v>
       </c>
       <c r="Z8" t="n">
         <v>1.936140464079432</v>
@@ -1306,7 +1306,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K10" t="n">
-        <v>8.644608533148219</v>
+        <v>9.865598438960113</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1322,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q10" t="n">
-        <v>363.6</v>
+        <v>318.6</v>
       </c>
       <c r="R10" t="n">
         <v>16901.2</v>
@@ -1338,13 +1338,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W10" t="n">
-        <v>0.1440768088858037</v>
+        <v>0.1644266406493352</v>
       </c>
       <c r="X10" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y10" t="n">
-        <v>46.48294829482949</v>
+        <v>53.04833647206529</v>
       </c>
       <c r="Z10" t="n">
         <v>3.099562617499243</v>
@@ -1396,7 +1396,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K11" t="n">
-        <v>7.247982460657667</v>
+        <v>7.217740531058261</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1412,7 +1412,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q11" t="n">
-        <v>429.6</v>
+        <v>431.4</v>
       </c>
       <c r="R11" t="n">
         <v>74809.60000000001</v>
@@ -1428,13 +1428,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1207997076776278</v>
+        <v>0.1202956755176377</v>
       </c>
       <c r="X11" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y11" t="n">
-        <v>174.1378026070764</v>
+        <v>173.4112192860454</v>
       </c>
       <c r="Z11" t="n">
         <v>0.6937018032218979</v>
@@ -1486,7 +1486,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K12" t="n">
-        <v>4.835192136301688</v>
+        <v>5.061841767690829</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1502,7 +1502,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q12" t="n">
-        <v>643.2</v>
+        <v>614.4</v>
       </c>
       <c r="R12" t="n">
         <v>38128.4</v>
@@ -1518,13 +1518,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W12" t="n">
-        <v>0.08058653560502813</v>
+        <v>0.08436402946151383</v>
       </c>
       <c r="X12" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y12" t="n">
-        <v>59.27922885572139</v>
+        <v>62.05794270833334</v>
       </c>
       <c r="Z12" t="n">
         <v>1.359439674918279</v>
@@ -1576,7 +1576,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K13" t="n">
-        <v>6.072261461107134</v>
+        <v>5.780325813938521</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1592,7 +1592,7 @@
         <v>0.145035</v>
       </c>
       <c r="Q13" t="n">
-        <v>475.2</v>
+        <v>499.2</v>
       </c>
       <c r="R13" t="n">
         <v>60200.2</v>
@@ -1608,13 +1608,13 @@
         <v>6.17518114688861</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1012043576851189</v>
+        <v>0.09633876356564201</v>
       </c>
       <c r="X13" t="n">
         <v>0.161938569284539</v>
       </c>
       <c r="Y13" t="n">
-        <v>126.6839225589226</v>
+        <v>120.5933493589743</v>
       </c>
       <c r="Z13" t="n">
         <v>0.7988729401558218</v>
@@ -1666,7 +1666,7 @@
         <v>47.6305176437724</v>
       </c>
       <c r="K14" t="n">
-        <v>9.248644202674251</v>
+        <v>9.680999521091952</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1682,7 @@
         <v>0.208445</v>
       </c>
       <c r="Q14" t="n">
-        <v>309</v>
+        <v>295.2</v>
       </c>
       <c r="R14" t="n">
         <v>30999.6</v>
@@ -1698,13 +1698,13 @@
         <v>8.555202665891516</v>
       </c>
       <c r="W14" t="n">
-        <v>0.1541440700445709</v>
+        <v>0.1613499920181992</v>
       </c>
       <c r="X14" t="n">
         <v>0.1168879381416492</v>
       </c>
       <c r="Y14" t="n">
-        <v>100.3223300970874</v>
+        <v>105.0121951219512</v>
       </c>
       <c r="Z14" t="n">
         <v>1.53648813674281</v>
@@ -1756,7 +1756,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>2.564690813375406</v>
+        <v>2.66627730368706</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1772,7 +1772,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>1086.6</v>
+        <v>1045.2</v>
       </c>
       <c r="R15" t="n">
         <v>80561.39999999999</v>
@@ -1788,13 +1788,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.0427448468895901</v>
+        <v>0.04443795506145101</v>
       </c>
       <c r="X15" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>74.1408061844285</v>
+        <v>77.07749712973593</v>
       </c>
       <c r="Z15" t="n">
         <v>0.5765360412086756</v>
@@ -1846,7 +1846,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>2.04521883139242</v>
+        <v>2.18510408165275</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1862,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1359</v>
+        <v>1272</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1878,13 +1878,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.03408698052320699</v>
+        <v>0.03641840136087917</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>47.29632082413539</v>
+        <v>50.53121069182389</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1936,7 +1936,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.237134527323675</v>
+        <v>1.132831341931956</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1952,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2202.6</v>
+        <v>2405.4</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1968,13 +1968,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.02061890878872791</v>
+        <v>0.01888052236553259</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>48.91046944520113</v>
+        <v>44.78681300407416</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -2026,7 +2026,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>3.924398982087117</v>
+        <v>3.57076494303142</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2042,7 +2042,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q18" t="n">
-        <v>684.6</v>
+        <v>752.4</v>
       </c>
       <c r="R18" t="n">
         <v>71127.60000000001</v>
@@ -2058,13 +2058,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W18" t="n">
-        <v>0.06540664970145194</v>
+        <v>0.05951274905052366</v>
       </c>
       <c r="X18" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y18" t="n">
-        <v>103.8965819456617</v>
+        <v>94.53429027113239</v>
       </c>
       <c r="Z18" t="n">
         <v>0.629536106737947</v>
@@ -2116,7 +2116,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>4.283477464658315</v>
+        <v>4.041987515172033</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2132,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q19" t="n">
-        <v>612.6</v>
+        <v>649.2</v>
       </c>
       <c r="R19" t="n">
         <v>64144.3</v>
@@ -2148,13 +2148,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W19" t="n">
-        <v>0.07139129107763859</v>
+        <v>0.06736645858620055</v>
       </c>
       <c r="X19" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y19" t="n">
-        <v>104.7082925236696</v>
+        <v>98.80514479359211</v>
       </c>
       <c r="Z19" t="n">
         <v>0.6818112429968274</v>
@@ -2206,7 +2206,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>2.320054441292081</v>
+        <v>2.329974503039989</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2222,7 +2222,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q20" t="n">
-        <v>1127.4</v>
+        <v>1122.6</v>
       </c>
       <c r="R20" t="n">
         <v>48455.2</v>
@@ -2238,13 +2238,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W20" t="n">
-        <v>0.03866757402153469</v>
+        <v>0.03883290838399982</v>
       </c>
       <c r="X20" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y20" t="n">
-        <v>42.97959907752351</v>
+        <v>43.16337074648138</v>
       </c>
       <c r="Z20" t="n">
         <v>0.8996727482680539</v>
@@ -2296,7 +2296,7 @@
         <v>43.3950199670746</v>
       </c>
       <c r="K21" t="n">
-        <v>6.137909472004893</v>
+        <v>6.172833565728962</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.064523</v>
       </c>
       <c r="Q21" t="n">
-        <v>424.2</v>
+        <v>421.8</v>
       </c>
       <c r="R21" t="n">
         <v>162164.2</v>
@@ -2328,13 +2328,13 @@
         <v>40.74733935074209</v>
       </c>
       <c r="W21" t="n">
-        <v>0.1022984912000816</v>
+        <v>0.102880559428816</v>
       </c>
       <c r="X21" t="n">
         <v>0.02454147966305898</v>
       </c>
       <c r="Y21" t="n">
-        <v>382.2824139556812</v>
+        <v>384.4575628259839</v>
       </c>
       <c r="Z21" t="n">
         <v>0.2675992602995889</v>
@@ -2386,7 +2386,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K22" t="n">
-        <v>2.929745347824457</v>
+        <v>3.110674562013021</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q22" t="n">
-        <v>856.1999999999999</v>
+        <v>806.4</v>
       </c>
       <c r="R22" t="n">
         <v>68673.2</v>
@@ -2418,13 +2418,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W22" t="n">
-        <v>0.04882908913040762</v>
+        <v>0.05184457603355035</v>
       </c>
       <c r="X22" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y22" t="n">
-        <v>80.2069609904228</v>
+        <v>85.16021825396825</v>
       </c>
       <c r="Z22" t="n">
         <v>0.6087886703030441</v>
@@ -2476,7 +2476,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K23" t="n">
-        <v>4.562567689697927</v>
+        <v>4.725892861038153</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2492,7 +2492,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q23" t="n">
-        <v>538.2</v>
+        <v>519.6</v>
       </c>
       <c r="R23" t="n">
         <v>71002.60000000001</v>
@@ -2508,13 +2508,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W23" t="n">
-        <v>0.07604279482829877</v>
+        <v>0.07876488101730254</v>
       </c>
       <c r="X23" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y23" t="n">
-        <v>131.926049795615</v>
+        <v>136.6485758275597</v>
       </c>
       <c r="Z23" t="n">
         <v>0.5764046975264343</v>
@@ -2566,7 +2566,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K24" t="n">
-        <v>8.202945420483784</v>
+        <v>8.652668305378729</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2582,7 +2582,7 @@
         <v>0.07520300000000001</v>
       </c>
       <c r="Q24" t="n">
-        <v>288.6</v>
+        <v>273.6</v>
       </c>
       <c r="R24" t="n">
         <v>88574</v>
@@ -2598,13 +2598,13 @@
         <v>12.61396912906789</v>
       </c>
       <c r="W24" t="n">
-        <v>0.1367157570080631</v>
+        <v>0.1442111384229788</v>
       </c>
       <c r="X24" t="n">
         <v>0.07927718783579227</v>
       </c>
       <c r="Y24" t="n">
-        <v>306.9092169092169</v>
+        <v>323.7353801169591</v>
       </c>
       <c r="Z24" t="n">
         <v>0.4454599258532639</v>
@@ -2828,7 +2828,7 @@
         <v>33.6962858057476</v>
       </c>
       <c r="K27" t="n">
-        <v>1.840321453071961</v>
+        <v>1.897313389963265</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2844,7 +2844,7 @@
         <v>0.143133</v>
       </c>
       <c r="Q27" t="n">
-        <v>1098.6</v>
+        <v>1065.6</v>
       </c>
       <c r="R27" t="n">
         <v>66797.5</v>
@@ -2860,13 +2860,13 @@
         <v>13.44796592290856</v>
       </c>
       <c r="W27" t="n">
-        <v>0.03067202421786601</v>
+        <v>0.03162188983272109</v>
       </c>
       <c r="X27" t="n">
         <v>0.0743606881317645</v>
       </c>
       <c r="Y27" t="n">
-        <v>60.80238485344985</v>
+        <v>62.68534159159158</v>
       </c>
       <c r="Z27" t="n">
         <v>0.504454295531234</v>
@@ -2980,7 +2980,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K29" t="n">
-        <v>3.541853724076558</v>
+        <v>3.770360415952465</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -2996,7 +2996,7 @@
         <v>0.026182</v>
       </c>
       <c r="Q29" t="n">
-        <v>495</v>
+        <v>465</v>
       </c>
       <c r="R29" t="n">
         <v>48192</v>
@@ -3012,13 +3012,13 @@
         <v>15.27539782478406</v>
       </c>
       <c r="W29" t="n">
-        <v>0.05903089540127596</v>
+        <v>0.06283934026587441</v>
       </c>
       <c r="X29" t="n">
         <v>0.06546474346988973</v>
       </c>
       <c r="Y29" t="n">
-        <v>97.35757575757576</v>
+        <v>103.6387096774194</v>
       </c>
       <c r="Z29" t="n">
         <v>0.6063307856829266</v>
@@ -3070,7 +3070,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K30" t="n">
-        <v>8.527229044347576</v>
+        <v>9.253622629606813</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3086,7 +3086,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q30" t="n">
-        <v>175.8</v>
+        <v>162</v>
       </c>
       <c r="R30" t="n">
         <v>34656</v>
@@ -3102,13 +3102,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W30" t="n">
-        <v>0.1421204840724596</v>
+        <v>0.1542270438267802</v>
       </c>
       <c r="X30" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y30" t="n">
-        <v>197.1331058020478</v>
+        <v>213.9259259259259</v>
       </c>
       <c r="Z30" t="n">
         <v>0.7209366660877885</v>
@@ -3160,7 +3160,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K31" t="n">
-        <v>6.885258961647388</v>
+        <v>7.011593988466606</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3176,7 +3176,7 @@
         <v>0.037626</v>
       </c>
       <c r="Q31" t="n">
-        <v>199.8</v>
+        <v>196.2</v>
       </c>
       <c r="R31" t="n">
         <v>28366.1</v>
@@ -3192,13 +3192,13 @@
         <v>31.96610467696488</v>
       </c>
       <c r="W31" t="n">
-        <v>0.1147543160274564</v>
+        <v>0.1168598998077768</v>
       </c>
       <c r="X31" t="n">
         <v>0.0312831360000085</v>
       </c>
       <c r="Y31" t="n">
-        <v>141.9724724724724</v>
+        <v>144.5774719673802</v>
       </c>
       <c r="Z31" t="n">
         <v>0.8082856769977473</v>
@@ -3250,7 +3250,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K32" t="n">
-        <v>8.82596848936692</v>
+        <v>9.054620522770207</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3266,7 +3266,7 @@
         <v>0.01289</v>
       </c>
       <c r="Q32" t="n">
-        <v>118.8</v>
+        <v>115.8</v>
       </c>
       <c r="R32" t="n">
         <v>13925.2</v>
@@ -3282,13 +3282,13 @@
         <v>76.71116733805002</v>
       </c>
       <c r="W32" t="n">
-        <v>0.147099474822782</v>
+        <v>0.1509103420461701</v>
       </c>
       <c r="X32" t="n">
         <v>0.01303591165016704</v>
       </c>
       <c r="Y32" t="n">
-        <v>117.2154882154882</v>
+        <v>120.2521588946459</v>
       </c>
       <c r="Z32" t="n">
         <v>1.254949128841704</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-12)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.505267381571251</v>
+        <v>4.459935743830983</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>767.4</v>
+        <v>775.2</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07508778969285418</v>
+        <v>0.07433226239718305</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>155.285379202502</v>
+        <v>153.7229102167182</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.776138142823965</v>
+        <v>3.708617791925788</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>889.8</v>
+        <v>906</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.06293563571373274</v>
+        <v>0.06181029653209646</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>221.8817711845359</v>
+        <v>217.914348785872</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.802837252006549</v>
+        <v>6.769933565177014</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>493.8</v>
+        <v>496.2</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1133806208667758</v>
+        <v>0.1128322260862836</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>132.983799108951</v>
+        <v>132.3405884723902</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -864,7 +864,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K5" t="n">
-        <v>11.42498848234684</v>
+        <v>11.64852086569711</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -880,7 +880,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q5" t="n">
-        <v>281.4</v>
+        <v>276</v>
       </c>
       <c r="R5" t="n">
         <v>35584.1</v>
@@ -896,13 +896,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1904164747057807</v>
+        <v>0.1941420144282852</v>
       </c>
       <c r="X5" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y5" t="n">
-        <v>126.453802416489</v>
+        <v>128.9278985507246</v>
       </c>
       <c r="Z5" t="n">
         <v>1.505818497087371</v>
@@ -954,7 +954,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>4.427794685670141</v>
+        <v>4.348404723905884</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -970,7 +970,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q6" t="n">
-        <v>723</v>
+        <v>736.1999999999999</v>
       </c>
       <c r="R6" t="n">
         <v>78110.8</v>
@@ -986,13 +986,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07379657809450235</v>
+        <v>0.07247341206509808</v>
       </c>
       <c r="X6" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y6" t="n">
-        <v>108.0370677731674</v>
+        <v>106.0999728334692</v>
       </c>
       <c r="Z6" t="n">
         <v>0.6830672066132366</v>
@@ -1044,7 +1044,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K7" t="n">
-        <v>5.384945218005506</v>
+        <v>5.357830690220988</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1060,7 +1060,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q7" t="n">
-        <v>592.8000000000001</v>
+        <v>595.8</v>
       </c>
       <c r="R7" t="n">
         <v>60537.6</v>
@@ -1076,13 +1076,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W7" t="n">
-        <v>0.08974908696675843</v>
+        <v>0.08929717817034979</v>
       </c>
       <c r="X7" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y7" t="n">
-        <v>102.1214574898785</v>
+        <v>101.607250755287</v>
       </c>
       <c r="Z7" t="n">
         <v>0.8788465144619939</v>
@@ -1134,7 +1134,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K8" t="n">
-        <v>6.849631910989987</v>
+        <v>7.325962363770932</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1150,7 +1150,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q8" t="n">
-        <v>461.4</v>
+        <v>431.4</v>
       </c>
       <c r="R8" t="n">
         <v>27205.5</v>
@@ -1166,13 +1166,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W8" t="n">
-        <v>0.1141605318498331</v>
+        <v>0.1220993727295155</v>
       </c>
       <c r="X8" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y8" t="n">
-        <v>58.96293888166449</v>
+        <v>63.06328233657857</v>
       </c>
       <c r="Z8" t="n">
         <v>1.936140464079432</v>
@@ -1306,7 +1306,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K10" t="n">
-        <v>10.35302919187316</v>
+        <v>11.19365976728167</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1322,7 +1322,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q10" t="n">
-        <v>303.6</v>
+        <v>280.8</v>
       </c>
       <c r="R10" t="n">
         <v>16901.2</v>
@@ -1338,13 +1338,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W10" t="n">
-        <v>0.1725504865312194</v>
+        <v>0.1865609961213612</v>
       </c>
       <c r="X10" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y10" t="n">
-        <v>55.66930171277998</v>
+        <v>60.1894586894587</v>
       </c>
       <c r="Z10" t="n">
         <v>3.099562617499243</v>
@@ -1396,7 +1396,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K11" t="n">
-        <v>7.079884640969836</v>
+        <v>6.975208927192056</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1412,7 +1412,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q11" t="n">
-        <v>439.8</v>
+        <v>446.4</v>
       </c>
       <c r="R11" t="n">
         <v>74809.60000000001</v>
@@ -1428,13 +1428,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1179980773494973</v>
+        <v>0.1162534821198676</v>
       </c>
       <c r="X11" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y11" t="n">
-        <v>170.0991359708959</v>
+        <v>167.584229390681</v>
       </c>
       <c r="Z11" t="n">
         <v>0.6937018032218979</v>
@@ -1486,7 +1486,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K12" t="n">
-        <v>5.061841767690829</v>
+        <v>5.456132600121484</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1502,7 +1502,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q12" t="n">
-        <v>614.4</v>
+        <v>570</v>
       </c>
       <c r="R12" t="n">
         <v>38128.4</v>
@@ -1518,13 +1518,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W12" t="n">
-        <v>0.08436402946151383</v>
+        <v>0.09093554333535807</v>
       </c>
       <c r="X12" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y12" t="n">
-        <v>62.05794270833334</v>
+        <v>66.8919298245614</v>
       </c>
       <c r="Z12" t="n">
         <v>1.359439674918279</v>
@@ -1576,7 +1576,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K13" t="n">
-        <v>6.103085123346256</v>
+        <v>6.072261461107134</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1592,7 +1592,7 @@
         <v>0.145035</v>
       </c>
       <c r="Q13" t="n">
-        <v>472.8</v>
+        <v>475.2</v>
       </c>
       <c r="R13" t="n">
         <v>60200.2</v>
@@ -1608,13 +1608,13 @@
         <v>6.17518114688861</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1017180853891043</v>
+        <v>0.1012043576851189</v>
       </c>
       <c r="X13" t="n">
         <v>0.161938569284539</v>
       </c>
       <c r="Y13" t="n">
-        <v>127.3269881556683</v>
+        <v>126.6839225589226</v>
       </c>
       <c r="Z13" t="n">
         <v>0.7988729401558218</v>
@@ -1666,7 +1666,7 @@
         <v>47.6305176437724</v>
       </c>
       <c r="K14" t="n">
-        <v>9.94374063544309</v>
+        <v>11.02558278791028</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1682,7 +1682,7 @@
         <v>0.208445</v>
       </c>
       <c r="Q14" t="n">
-        <v>287.4</v>
+        <v>259.2</v>
       </c>
       <c r="R14" t="n">
         <v>30999.6</v>
@@ -1698,13 +1698,13 @@
         <v>8.555202665891516</v>
       </c>
       <c r="W14" t="n">
-        <v>0.1657290105907182</v>
+        <v>0.1837597131318379</v>
       </c>
       <c r="X14" t="n">
         <v>0.1168879381416492</v>
       </c>
       <c r="Y14" t="n">
-        <v>107.8622129436326</v>
+        <v>119.5972222222222</v>
       </c>
       <c r="Z14" t="n">
         <v>1.53648813674281</v>
@@ -1756,7 +1756,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>2.906542592630075</v>
+        <v>3.067803872538216</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1772,7 +1772,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>958.8000000000001</v>
+        <v>908.4000000000001</v>
       </c>
       <c r="R15" t="n">
         <v>80561.39999999999</v>
@@ -1788,13 +1788,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.04844237654383458</v>
+        <v>0.05113006454230361</v>
       </c>
       <c r="X15" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>84.02315394242802</v>
+        <v>88.68494055482165</v>
       </c>
       <c r="Z15" t="n">
         <v>0.5765360412086756</v>
@@ -1846,7 +1846,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>2.501307048112219</v>
+        <v>2.105645751410832</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1862,7 +1862,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1111.2</v>
+        <v>1320</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1878,13 +1878,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.04168845080187032</v>
+        <v>0.0350940958568472</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>57.84350251979841</v>
+        <v>48.69371212121212</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1936,7 +1936,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.092499603032285</v>
+        <v>1.094078740015709</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1952,7 +1952,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2494.2</v>
+        <v>2490.6</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1968,13 +1968,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.01820832671720476</v>
+        <v>0.01823464566692849</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>43.19228610376073</v>
+        <v>43.2547177386975</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -2026,7 +2026,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>3.481912316144169</v>
+        <v>3.599468841287299</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2042,7 +2042,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q18" t="n">
-        <v>771.5999999999999</v>
+        <v>746.4</v>
       </c>
       <c r="R18" t="n">
         <v>71127.60000000001</v>
@@ -2058,13 +2058,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W18" t="n">
-        <v>0.05803187193573614</v>
+        <v>0.05999114735478832</v>
       </c>
       <c r="X18" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y18" t="n">
-        <v>92.18195956454123</v>
+        <v>95.29421221864953</v>
       </c>
       <c r="Z18" t="n">
         <v>0.629536106737947</v>
@@ -2116,7 +2116,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>3.950705050963089</v>
+        <v>3.994000448781863</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2132,7 +2132,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q19" t="n">
-        <v>664.2</v>
+        <v>657</v>
       </c>
       <c r="R19" t="n">
         <v>64144.3</v>
@@ -2148,13 +2148,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W19" t="n">
-        <v>0.06584508418271814</v>
+        <v>0.06656667414636439</v>
       </c>
       <c r="X19" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y19" t="n">
-        <v>96.57377295995182</v>
+        <v>97.63211567732117</v>
       </c>
       <c r="Z19" t="n">
         <v>0.6818112429968274</v>
@@ -2206,7 +2206,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>2.333716432113394</v>
+        <v>2.353878129151091</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2222,7 +2222,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q20" t="n">
-        <v>1120.8</v>
+        <v>1111.2</v>
       </c>
       <c r="R20" t="n">
         <v>48455.2</v>
@@ -2238,13 +2238,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W20" t="n">
-        <v>0.03889527386855657</v>
+        <v>0.03923130215251818</v>
       </c>
       <c r="X20" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y20" t="n">
-        <v>43.23269093504639</v>
+        <v>43.60619150467962</v>
       </c>
       <c r="Z20" t="n">
         <v>0.8996727482680539</v>
@@ -2296,7 +2296,7 @@
         <v>43.3950199670746</v>
       </c>
       <c r="K21" t="n">
-        <v>6.172833565728962</v>
+        <v>6.181626775936554</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2312,7 +2312,7 @@
         <v>0.064523</v>
       </c>
       <c r="Q21" t="n">
-        <v>421.8</v>
+        <v>421.2</v>
       </c>
       <c r="R21" t="n">
         <v>162164.2</v>
@@ -2328,13 +2328,13 @@
         <v>40.74733935074209</v>
       </c>
       <c r="W21" t="n">
-        <v>0.102880559428816</v>
+        <v>0.1030271129322759</v>
       </c>
       <c r="X21" t="n">
         <v>0.02454147966305898</v>
       </c>
       <c r="Y21" t="n">
-        <v>384.4575628259839</v>
+        <v>385.0052231718899</v>
       </c>
       <c r="Z21" t="n">
         <v>0.2675992602995889</v>
@@ -2386,7 +2386,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K22" t="n">
-        <v>3.110674562013021</v>
+        <v>3.20363725007318</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2402,7 +2402,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q22" t="n">
-        <v>806.4</v>
+        <v>783</v>
       </c>
       <c r="R22" t="n">
         <v>68673.2</v>
@@ -2418,13 +2418,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W22" t="n">
-        <v>0.05184457603355035</v>
+        <v>0.05339395416788634</v>
       </c>
       <c r="X22" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y22" t="n">
-        <v>85.16021825396825</v>
+        <v>87.7052362707535</v>
       </c>
       <c r="Z22" t="n">
         <v>0.6087886703030441</v>
@@ -2476,7 +2476,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K23" t="n">
-        <v>4.725892861038153</v>
+        <v>4.742321225560881</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2492,7 +2492,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q23" t="n">
-        <v>519.6</v>
+        <v>517.8000000000001</v>
       </c>
       <c r="R23" t="n">
         <v>71002.60000000001</v>
@@ -2508,13 +2508,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W23" t="n">
-        <v>0.07876488101730254</v>
+        <v>0.07903868709268135</v>
       </c>
       <c r="X23" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y23" t="n">
-        <v>136.6485758275597</v>
+        <v>137.1235998455002</v>
       </c>
       <c r="Z23" t="n">
         <v>0.5764046975264343</v>
@@ -2566,7 +2566,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K24" t="n">
-        <v>8.521850426031749</v>
+        <v>7.782281552766665</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2582,7 +2582,7 @@
         <v>0.07520300000000001</v>
       </c>
       <c r="Q24" t="n">
-        <v>277.8</v>
+        <v>304.2</v>
       </c>
       <c r="R24" t="n">
         <v>88574</v>
@@ -2598,13 +2598,13 @@
         <v>12.61396912906789</v>
       </c>
       <c r="W24" t="n">
-        <v>0.1420308404338625</v>
+        <v>0.1297046925461111</v>
       </c>
       <c r="X24" t="n">
         <v>0.07927718783579227</v>
       </c>
       <c r="Y24" t="n">
-        <v>318.8408927285817</v>
+        <v>291.1702827087442</v>
       </c>
       <c r="Z24" t="n">
         <v>0.4454599258532639</v>
@@ -2738,7 +2738,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K26" t="n">
-        <v>6.364694271614992</v>
+        <v>6.354086447828966</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2754,7 +2754,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q26" t="n">
-        <v>359.4</v>
+        <v>360</v>
       </c>
       <c r="R26" t="n">
         <v>50011.7</v>
@@ -2770,13 +2770,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W26" t="n">
-        <v>0.1060782378602498</v>
+        <v>0.1059014407971494</v>
       </c>
       <c r="X26" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y26" t="n">
-        <v>139.1533110740122</v>
+        <v>138.9213888888889</v>
       </c>
       <c r="Z26" t="n">
         <v>0.7623119927331765</v>
@@ -2980,7 +2980,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K29" t="n">
-        <v>4.013776541707637</v>
+        <v>3.643428082747083</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -2996,7 +2996,7 @@
         <v>0.026182</v>
       </c>
       <c r="Q29" t="n">
-        <v>436.8</v>
+        <v>481.2</v>
       </c>
       <c r="R29" t="n">
         <v>48192</v>
@@ -3012,13 +3012,13 @@
         <v>15.27539782478406</v>
       </c>
       <c r="W29" t="n">
-        <v>0.06689627569512729</v>
+        <v>0.06072380137911804</v>
       </c>
       <c r="X29" t="n">
         <v>0.06546474346988973</v>
       </c>
       <c r="Y29" t="n">
-        <v>110.3296703296703</v>
+        <v>100.1496259351621</v>
       </c>
       <c r="Z29" t="n">
         <v>0.6063307856829266</v>
@@ -3160,7 +3160,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K31" t="n">
-        <v>7.054742259164862</v>
+        <v>7.825226055387644</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3176,7 +3176,7 @@
         <v>0.037626</v>
       </c>
       <c r="Q31" t="n">
-        <v>195</v>
+        <v>175.8</v>
       </c>
       <c r="R31" t="n">
         <v>28366.1</v>
@@ -3192,13 +3192,13 @@
         <v>31.96610467696488</v>
       </c>
       <c r="W31" t="n">
-        <v>0.1175790376527477</v>
+        <v>0.1304204342564607</v>
       </c>
       <c r="X31" t="n">
         <v>0.0312831360000085</v>
       </c>
       <c r="Y31" t="n">
-        <v>145.4671794871795</v>
+        <v>161.3543799772469</v>
       </c>
       <c r="Z31" t="n">
         <v>0.8082856769977473</v>
@@ -3250,7 +3250,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K32" t="n">
-        <v>9.007947221106443</v>
+        <v>9.197588215235001</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3266,7 +3266,7 @@
         <v>0.01289</v>
       </c>
       <c r="Q32" t="n">
-        <v>116.4</v>
+        <v>114</v>
       </c>
       <c r="R32" t="n">
         <v>13925.2</v>
@@ -3282,13 +3282,13 @@
         <v>76.71116733805002</v>
       </c>
       <c r="W32" t="n">
-        <v>0.1501324536851074</v>
+        <v>0.1532931369205833</v>
       </c>
       <c r="X32" t="n">
         <v>0.01303591165016704</v>
       </c>
       <c r="Y32" t="n">
-        <v>119.6323024054983</v>
+        <v>122.1508771929825</v>
       </c>
       <c r="Z32" t="n">
         <v>1.254949128841704</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-13)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z32"/>
+  <dimension ref="A1:Z33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.459935743830983</v>
+        <v>4.365331046234568</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>775.2</v>
+        <v>792</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07433226239718305</v>
+        <v>0.0727555174372428</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>153.7229102167182</v>
+        <v>150.4621212121212</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.708617791925788</v>
+        <v>3.608255712505116</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>906</v>
+        <v>931.1999999999999</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.06181029653209646</v>
+        <v>0.0601375952084186</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>217.914348785872</v>
+        <v>212.0171821305842</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.769933565177014</v>
+        <v>6.70507192622921</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>496.2</v>
+        <v>501</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1128322260862836</v>
+        <v>0.1117511987704868</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>132.3405884723902</v>
+        <v>131.0726546906187</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -821,39 +821,35 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>claude-opus-5-5-high</t>
+          <t>muse-wonder-full</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (High, Default Fallback)</t>
+          <t>Muse Wonder Full (Max)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (high with fallback)</t>
+          <t>Muse Wonder Full (max)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>large</t>
-        </is>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="b">
         <v>1</v>
       </c>
@@ -861,67 +857,39 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>53.5831959822067</v>
-      </c>
-      <c r="K5" t="n">
-        <v>11.64852086569711</v>
-      </c>
+        <v>55.8021199855616</v>
+      </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
-      <c r="M5" t="n">
-        <v>13.220816</v>
-      </c>
-      <c r="N5" t="n">
-        <v>12.509134</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0.346949</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0.364732</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>276</v>
-      </c>
-      <c r="R5" t="n">
-        <v>35584.1</v>
-      </c>
-      <c r="S5" t="n">
-        <v>17347.5</v>
-      </c>
-      <c r="T5" t="n">
-        <v>18236.6</v>
-      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
-      <c r="V5" t="n">
-        <v>4.05294166276928</v>
-      </c>
-      <c r="W5" t="n">
-        <v>0.1941420144282852</v>
-      </c>
-      <c r="X5" t="n">
-        <v>0.2467343680729723</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>128.9278985507246</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>1.505818497087371</v>
-      </c>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>claude-fable-5-1</t>
+          <t>claude-opus-5-5-high</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (Max, Default Fallback)</t>
+          <t>Claude Opus 5.5 (High, Default Fallback)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (max with fallback)</t>
+          <t>Claude Opus 5.5 (high with fallback)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -936,7 +904,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -951,67 +919,67 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>53.3549259623252</v>
+        <v>53.5831959822067</v>
       </c>
       <c r="K6" t="n">
-        <v>4.348404723905884</v>
+        <v>11.88097471889284</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
-        <v>69.77964799999999</v>
+        <v>13.220816</v>
       </c>
       <c r="N6" t="n">
-        <v>65.87410800000001</v>
+        <v>12.509134</v>
       </c>
       <c r="O6" t="n">
-        <v>1.54355</v>
+        <v>0.346949</v>
       </c>
       <c r="P6" t="n">
-        <v>2.361991</v>
+        <v>0.364732</v>
       </c>
       <c r="Q6" t="n">
-        <v>736.1999999999999</v>
+        <v>270.6</v>
       </c>
       <c r="R6" t="n">
-        <v>78110.8</v>
+        <v>35584.1</v>
       </c>
       <c r="S6" t="n">
-        <v>30871</v>
+        <v>17347.5</v>
       </c>
       <c r="T6" t="n">
-        <v>47239.8</v>
+        <v>18236.6</v>
       </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="n">
-        <v>0.7646201649272464</v>
+        <v>4.05294166276928</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07247341206509808</v>
+        <v>0.1980162453148807</v>
       </c>
       <c r="X6" t="n">
-        <v>1.307838905994782</v>
+        <v>0.2467343680729723</v>
       </c>
       <c r="Y6" t="n">
-        <v>106.0999728334692</v>
+        <v>131.5007390983001</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.6830672066132366</v>
+        <v>1.505818497087371</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>claude-fable-5-1-xhigh</t>
+          <t>claude-fable-5-1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (Xhigh, Default Fallback)</t>
+          <t>Claude Fable 5.1 (Max, Default Fallback)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (xhigh with fallback)</t>
+          <t>Claude Fable 5.1 (max with fallback)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1041,82 +1009,82 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>53.2032587538944</v>
+        <v>53.3549259623252</v>
       </c>
       <c r="K7" t="n">
-        <v>5.357830690220988</v>
+        <v>4.564151066067168</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
-        <v>51.954237</v>
+        <v>69.77964799999999</v>
       </c>
       <c r="N7" t="n">
-        <v>48.927356</v>
+        <v>65.87410800000001</v>
       </c>
       <c r="O7" t="n">
-        <v>1.32351</v>
+        <v>1.54355</v>
       </c>
       <c r="P7" t="n">
-        <v>1.70337</v>
+        <v>2.361991</v>
       </c>
       <c r="Q7" t="n">
-        <v>595.8</v>
+        <v>701.4</v>
       </c>
       <c r="R7" t="n">
-        <v>60537.6</v>
+        <v>78110.8</v>
       </c>
       <c r="S7" t="n">
-        <v>26470.2</v>
+        <v>30871</v>
       </c>
       <c r="T7" t="n">
-        <v>34067.4</v>
+        <v>47239.8</v>
       </c>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="n">
-        <v>1.024040806409964</v>
+        <v>0.7646201649272464</v>
       </c>
       <c r="W7" t="n">
-        <v>0.08929717817034979</v>
+        <v>0.07606918443445281</v>
       </c>
       <c r="X7" t="n">
-        <v>0.9765235855256145</v>
+        <v>1.307838905994782</v>
       </c>
       <c r="Y7" t="n">
-        <v>101.607250755287</v>
+        <v>111.364128885087</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.8788465144619939</v>
+        <v>0.6830672066132366</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>gpt-6-astra</t>
+          <t>claude-fable-5-1-xhigh</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (Max)</t>
+          <t>Claude Fable 5.1 (Xhigh, Default Fallback)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (max)</t>
+          <t>Claude Fable 5.1 (xhigh with fallback)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1131,82 +1099,82 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>52.673669395513</v>
+        <v>53.2032587538944</v>
       </c>
       <c r="K8" t="n">
-        <v>7.325962363770932</v>
+        <v>5.26243904588471</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
-        <v>11.948927</v>
+        <v>51.954237</v>
       </c>
       <c r="N8" t="n">
-        <v>10.588652</v>
+        <v>48.927356</v>
       </c>
       <c r="O8" t="n">
-        <v>0.525713</v>
+        <v>1.32351</v>
       </c>
       <c r="P8" t="n">
-        <v>0.834562</v>
+        <v>1.70337</v>
       </c>
       <c r="Q8" t="n">
-        <v>431.4</v>
+        <v>606.5999999999999</v>
       </c>
       <c r="R8" t="n">
-        <v>27205.5</v>
+        <v>60537.6</v>
       </c>
       <c r="S8" t="n">
-        <v>10514.3</v>
+        <v>26470.2</v>
       </c>
       <c r="T8" t="n">
-        <v>16691.2</v>
+        <v>34067.4</v>
       </c>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="n">
-        <v>4.408234261998002</v>
+        <v>1.024040806409964</v>
       </c>
       <c r="W8" t="n">
-        <v>0.1220993727295155</v>
+        <v>0.08770731743141182</v>
       </c>
       <c r="X8" t="n">
-        <v>0.2268481982957858</v>
+        <v>0.9765235855256145</v>
       </c>
       <c r="Y8" t="n">
-        <v>63.06328233657857</v>
+        <v>99.79821958456975</v>
       </c>
       <c r="Z8" t="n">
-        <v>1.936140464079432</v>
+        <v>0.8788465144619939</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>gemini-4-argon</t>
+          <t>gpt-6-astra</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Gemini 4 Argon (High)</t>
+          <t>GPT-6 Astra (Max)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Gemini 4 Argon (high)</t>
+          <t>GPT-6 Astra (max)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1221,74 +1189,82 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>52.5605655745982</v>
-      </c>
-      <c r="K9" t="inlineStr"/>
+        <v>52.673669395513</v>
+      </c>
+      <c r="K9" t="n">
+        <v>7.325962363770932</v>
+      </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
-        <v>8.057855999999999</v>
+        <v>11.948927</v>
       </c>
       <c r="N9" t="n">
-        <v>7.44228</v>
+        <v>10.588652</v>
       </c>
       <c r="O9" t="n">
-        <v>0.260112</v>
+        <v>0.525713</v>
       </c>
       <c r="P9" t="n">
-        <v>0.355464</v>
-      </c>
-      <c r="Q9" t="inlineStr"/>
+        <v>0.834562</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>431.4</v>
+      </c>
       <c r="R9" t="n">
-        <v>61557.6</v>
+        <v>27205.5</v>
       </c>
       <c r="S9" t="n">
-        <v>26011.2</v>
+        <v>10514.3</v>
       </c>
       <c r="T9" t="n">
-        <v>35546.4</v>
+        <v>16691.2</v>
       </c>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="n">
-        <v>6.522897104961693</v>
-      </c>
-      <c r="W9" t="inlineStr"/>
+        <v>4.408234261998002</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.1220993727295155</v>
+      </c>
       <c r="X9" t="n">
-        <v>0.1533061128987214</v>
-      </c>
-      <c r="Y9" t="inlineStr"/>
+        <v>0.2268481982957858</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>63.06328233657857</v>
+      </c>
       <c r="Z9" t="n">
-        <v>0.8538436452135594</v>
+        <v>1.936140464079432</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>gpt-6-astra-xhigh</t>
+          <t>gemini-4-argon</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (Xhigh)</t>
+          <t>Gemini 4 Argon (High)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (xhigh)</t>
+          <t>Gemini 4 Argon (high)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1303,82 +1279,74 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>52.3863277108782</v>
-      </c>
-      <c r="K10" t="n">
-        <v>11.19365976728167</v>
-      </c>
+        <v>52.5605655745982</v>
+      </c>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
-        <v>8.717548000000001</v>
+        <v>8.057855999999999</v>
       </c>
       <c r="N10" t="n">
-        <v>7.872489</v>
+        <v>7.44228</v>
       </c>
       <c r="O10" t="n">
-        <v>0.415935</v>
+        <v>0.260112</v>
       </c>
       <c r="P10" t="n">
-        <v>0.429124</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>280.8</v>
-      </c>
+        <v>0.355464</v>
+      </c>
+      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="n">
-        <v>16901.2</v>
+        <v>61557.6</v>
       </c>
       <c r="S10" t="n">
-        <v>8318.700000000001</v>
+        <v>26011.2</v>
       </c>
       <c r="T10" t="n">
-        <v>8582.5</v>
+        <v>35546.4</v>
       </c>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="n">
-        <v>6.009296158837118</v>
-      </c>
-      <c r="W10" t="n">
-        <v>0.1865609961213612</v>
-      </c>
+        <v>6.522897104961693</v>
+      </c>
+      <c r="W10" t="inlineStr"/>
       <c r="X10" t="n">
-        <v>0.1664088394993523</v>
-      </c>
-      <c r="Y10" t="n">
-        <v>60.1894586894587</v>
-      </c>
+        <v>0.1533061128987214</v>
+      </c>
+      <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="n">
-        <v>3.099562617499243</v>
+        <v>0.8538436452135594</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>claude-sonnet-5-5-xhigh</t>
+          <t>muse-wonder</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5.5 (Xhigh, Default Fallback)</t>
+          <t>Muse Wonder (Max)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5.5 (xhigh with fallback)</t>
+          <t>Muse Wonder (max)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1393,67 +1361,67 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>51.8955544183089</v>
+        <v>52.393894697293</v>
       </c>
       <c r="K11" t="n">
-        <v>6.975208927192056</v>
+        <v>6.267212284365192</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
-        <v>15.865464</v>
+        <v>31.838585</v>
       </c>
       <c r="N11" t="n">
-        <v>15.117367</v>
+        <v>30.753951</v>
       </c>
       <c r="O11" t="n">
-        <v>0.268563</v>
+        <v>0.511023</v>
       </c>
       <c r="P11" t="n">
-        <v>0.479533</v>
+        <v>0.573611</v>
       </c>
       <c r="Q11" t="n">
-        <v>446.4</v>
+        <v>501.6</v>
       </c>
       <c r="R11" t="n">
-        <v>74809.60000000001</v>
+        <v>54231.7</v>
       </c>
       <c r="S11" t="n">
-        <v>26856.3</v>
+        <v>25551.1</v>
       </c>
       <c r="T11" t="n">
-        <v>47953.3</v>
+        <v>28680.5</v>
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>3.270976154136362</v>
+        <v>1.645610026239954</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1162534821198676</v>
+        <v>0.1044535380727532</v>
       </c>
       <c r="X11" t="n">
-        <v>0.3057191348629781</v>
+        <v>0.6076773865342173</v>
       </c>
       <c r="Y11" t="n">
-        <v>167.584229390681</v>
+        <v>108.1174242424242</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.6937018032218979</v>
+        <v>0.9661119732055791</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>gpt-6-1-sol</t>
+          <t>gpt-6-astra-xhigh</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>GPT-6.1 Sol (Max)</t>
+          <t>GPT-6 Astra (Xhigh)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GPT-6.1 Sol (max)</t>
+          <t>GPT-6 Astra (xhigh)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1468,7 +1436,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1483,82 +1451,82 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>51.8332597011541</v>
+        <v>52.3863277108782</v>
       </c>
       <c r="K12" t="n">
-        <v>5.456132600121484</v>
+        <v>11.12236257131172</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
-        <v>3.029649</v>
+        <v>8.717548000000001</v>
       </c>
       <c r="N12" t="n">
-        <v>2.648365</v>
+        <v>7.872489</v>
       </c>
       <c r="O12" t="n">
-        <v>0.129384</v>
+        <v>0.415935</v>
       </c>
       <c r="P12" t="n">
-        <v>0.2519</v>
+        <v>0.429124</v>
       </c>
       <c r="Q12" t="n">
-        <v>570</v>
+        <v>282.6</v>
       </c>
       <c r="R12" t="n">
-        <v>38128.4</v>
+        <v>16901.2</v>
       </c>
       <c r="S12" t="n">
-        <v>12938.4</v>
+        <v>8318.700000000001</v>
       </c>
       <c r="T12" t="n">
-        <v>25190</v>
+        <v>8582.5</v>
       </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="n">
-        <v>17.10866826525254</v>
+        <v>6.009296158837118</v>
       </c>
       <c r="W12" t="n">
-        <v>0.09093554333535807</v>
+        <v>0.185372709521862</v>
       </c>
       <c r="X12" t="n">
-        <v>0.05844990296708164</v>
+        <v>0.1664088394993523</v>
       </c>
       <c r="Y12" t="n">
-        <v>66.8919298245614</v>
+        <v>59.80608634111819</v>
       </c>
       <c r="Z12" t="n">
-        <v>1.359439674918279</v>
+        <v>3.099562617499243</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>muse-spark-1-3</t>
+          <t>claude-sonnet-5-5-xhigh</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Muse Spark 1.3 (Max)</t>
+          <t>Claude Sonnet 5.5 (Xhigh, Default Fallback)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Muse Spark 1.3 (max)</t>
+          <t>Claude Sonnet 5.5 (xhigh with fallback)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1573,67 +1541,67 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>48.0923107719685</v>
+        <v>51.8955544183089</v>
       </c>
       <c r="K13" t="n">
-        <v>6.072261461107134</v>
+        <v>6.965846230645489</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
-        <v>7.788</v>
+        <v>15.865464</v>
       </c>
       <c r="N13" t="n">
-        <v>7.532149</v>
+        <v>15.117367</v>
       </c>
       <c r="O13" t="n">
-        <v>0.110815</v>
+        <v>0.268563</v>
       </c>
       <c r="P13" t="n">
-        <v>0.145035</v>
+        <v>0.479533</v>
       </c>
       <c r="Q13" t="n">
-        <v>475.2</v>
+        <v>447</v>
       </c>
       <c r="R13" t="n">
-        <v>60200.2</v>
+        <v>74809.60000000001</v>
       </c>
       <c r="S13" t="n">
-        <v>26074.2</v>
+        <v>26856.3</v>
       </c>
       <c r="T13" t="n">
-        <v>34125.9</v>
+        <v>47953.3</v>
       </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="n">
-        <v>6.17518114688861</v>
+        <v>3.270976154136362</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1012043576851189</v>
+        <v>0.1160974371774248</v>
       </c>
       <c r="X13" t="n">
-        <v>0.161938569284539</v>
+        <v>0.3057191348629781</v>
       </c>
       <c r="Y13" t="n">
-        <v>126.6839225589226</v>
+        <v>167.3592841163311</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.7988729401558218</v>
+        <v>0.6937018032218979</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>gpt-6-sol</t>
+          <t>gpt-6-1-sol</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>GPT-6 Sol (Max)</t>
+          <t>GPT-6.1 Sol (Max)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GPT-6 Sol (max)</t>
+          <t>GPT-6.1 Sol (max)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1648,7 +1616,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1663,82 +1631,82 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>47.6305176437724</v>
+        <v>51.8332597011541</v>
       </c>
       <c r="K14" t="n">
-        <v>11.02558278791028</v>
+        <v>5.321689907716026</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>5.567433</v>
+        <v>3.029649</v>
       </c>
       <c r="N14" t="n">
-        <v>5.257437</v>
+        <v>2.648365</v>
       </c>
       <c r="O14" t="n">
-        <v>0.101551</v>
+        <v>0.129384</v>
       </c>
       <c r="P14" t="n">
-        <v>0.208445</v>
+        <v>0.2519</v>
       </c>
       <c r="Q14" t="n">
-        <v>259.2</v>
+        <v>584.4</v>
       </c>
       <c r="R14" t="n">
-        <v>30999.6</v>
+        <v>38128.4</v>
       </c>
       <c r="S14" t="n">
-        <v>10155.1</v>
+        <v>12938.4</v>
       </c>
       <c r="T14" t="n">
-        <v>20844.5</v>
+        <v>25190</v>
       </c>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="n">
-        <v>8.555202665891516</v>
+        <v>17.10866826525254</v>
       </c>
       <c r="W14" t="n">
-        <v>0.1837597131318379</v>
+        <v>0.08869483179526712</v>
       </c>
       <c r="X14" t="n">
-        <v>0.1168879381416492</v>
+        <v>0.05844990296708164</v>
       </c>
       <c r="Y14" t="n">
-        <v>119.5972222222222</v>
+        <v>65.24366872005476</v>
       </c>
       <c r="Z14" t="n">
-        <v>1.53648813674281</v>
+        <v>1.359439674918279</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>grok-4-7</t>
+          <t>muse-spark-1-3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Grok 4.7 (Xhigh)</t>
+          <t>Muse Spark 1.3 (Max)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Grok 4.7 (xhigh)</t>
+          <t>Muse Spark 1.3 (max)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>SpaceXAI</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>xai</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1753,77 +1721,77 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>46.4465506302286</v>
+        <v>48.0923107719685</v>
       </c>
       <c r="K15" t="n">
-        <v>3.067803872538216</v>
+        <v>6.173595734527407</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>8.336827</v>
+        <v>7.788</v>
       </c>
       <c r="N15" t="n">
-        <v>7.853459</v>
+        <v>7.532149</v>
       </c>
       <c r="O15" t="n">
-        <v>0.132106</v>
+        <v>0.110815</v>
       </c>
       <c r="P15" t="n">
-        <v>0.351262</v>
+        <v>0.145035</v>
       </c>
       <c r="Q15" t="n">
-        <v>908.4000000000001</v>
+        <v>467.4</v>
       </c>
       <c r="R15" t="n">
-        <v>80561.39999999999</v>
+        <v>60200.2</v>
       </c>
       <c r="S15" t="n">
-        <v>22017.7</v>
+        <v>26074.2</v>
       </c>
       <c r="T15" t="n">
-        <v>58543.6</v>
+        <v>34125.9</v>
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="n">
-        <v>5.571250384616186</v>
+        <v>6.17518114688861</v>
       </c>
       <c r="W15" t="n">
-        <v>0.05113006454230361</v>
+        <v>0.1028932622421234</v>
       </c>
       <c r="X15" t="n">
-        <v>0.1794929200743312</v>
+        <v>0.161938569284539</v>
       </c>
       <c r="Y15" t="n">
-        <v>88.68494055482165</v>
+        <v>128.7980316645272</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.5765360412086756</v>
+        <v>0.7988729401558218</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>mimo-v2-6-pro</t>
+          <t>grok-4-7</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Grok 4.7 (Xhigh)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Grok 4.7 (xhigh)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Xiaomi</t>
+          <t>SpaceXAI</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>xiaomi</t>
+          <t>xai</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1840,85 +1808,85 @@
         <v>1</v>
       </c>
       <c r="I16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>46.3242065310383</v>
+        <v>46.4465506302286</v>
       </c>
       <c r="K16" t="n">
-        <v>2.105645751410832</v>
+        <v>3.082053790990617</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
-        <v>2.466319</v>
+        <v>8.336827</v>
       </c>
       <c r="N16" t="n">
-        <v>2.410399</v>
+        <v>7.853459</v>
       </c>
       <c r="O16" t="n">
-        <v>0.023278</v>
+        <v>0.132106</v>
       </c>
       <c r="P16" t="n">
-        <v>0.032642</v>
+        <v>0.351262</v>
       </c>
       <c r="Q16" t="n">
-        <v>1320</v>
+        <v>904.2</v>
       </c>
       <c r="R16" t="n">
-        <v>64275.7</v>
+        <v>80561.39999999999</v>
       </c>
       <c r="S16" t="n">
-        <v>26756</v>
+        <v>22017.7</v>
       </c>
       <c r="T16" t="n">
-        <v>37519.7</v>
+        <v>58543.6</v>
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="n">
-        <v>18.78273107859863</v>
+        <v>5.571250384616186</v>
       </c>
       <c r="W16" t="n">
-        <v>0.0350940958568472</v>
+        <v>0.05136756318317695</v>
       </c>
       <c r="X16" t="n">
-        <v>0.05324039383918014</v>
+        <v>0.1794929200743312</v>
       </c>
       <c r="Y16" t="n">
-        <v>48.69371212121212</v>
+        <v>89.0968812209688</v>
       </c>
       <c r="Z16" t="n">
-        <v>0.7207110390246749</v>
+        <v>0.5765360412086756</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>qwen3-8-max</t>
+          <t>mimo-v2-6-pro</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>Xiaomi</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>xiaomi</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1930,85 +1898,85 @@
         <v>1</v>
       </c>
       <c r="I17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17" t="n">
-        <v>45.4152084980521</v>
+        <v>46.3242065310383</v>
       </c>
       <c r="K17" t="n">
-        <v>1.094078740015709</v>
+        <v>2.105645751410832</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
-        <v>26.154609</v>
+        <v>2.466319</v>
       </c>
       <c r="N17" t="n">
-        <v>25.508227</v>
+        <v>2.410399</v>
       </c>
       <c r="O17" t="n">
-        <v>0.221402</v>
+        <v>0.023278</v>
       </c>
       <c r="P17" t="n">
-        <v>0.424979</v>
+        <v>0.032642</v>
       </c>
       <c r="Q17" t="n">
-        <v>2490.6</v>
+        <v>1320</v>
       </c>
       <c r="R17" t="n">
-        <v>107730.2</v>
+        <v>64275.7</v>
       </c>
       <c r="S17" t="n">
-        <v>36900.3</v>
+        <v>26756</v>
       </c>
       <c r="T17" t="n">
-        <v>70829.89999999999</v>
+        <v>37519.7</v>
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="n">
-        <v>1.736413207249709</v>
+        <v>18.78273107859863</v>
       </c>
       <c r="W17" t="n">
-        <v>0.01823464566692849</v>
+        <v>0.0350940958568472</v>
       </c>
       <c r="X17" t="n">
-        <v>0.5758997891889408</v>
+        <v>0.05324039383918014</v>
       </c>
       <c r="Y17" t="n">
-        <v>43.2547177386975</v>
+        <v>48.69371212121212</v>
       </c>
       <c r="Z17" t="n">
-        <v>0.421564319921917</v>
+        <v>0.7207110390246749</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>glm-5-3</t>
+          <t>qwen3-8-max</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>GLM-5.3 (Max)</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2020,85 +1988,85 @@
         <v>1</v>
       </c>
       <c r="I18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>44.777392385614</v>
+        <v>45.4152084980521</v>
       </c>
       <c r="K18" t="n">
-        <v>3.599468841287299</v>
+        <v>1.261183240712361</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
-        <v>8.678356000000001</v>
+        <v>26.154609</v>
       </c>
       <c r="N18" t="n">
-        <v>8.365394999999999</v>
+        <v>25.508227</v>
       </c>
       <c r="O18" t="n">
-        <v>0.098552</v>
+        <v>0.221402</v>
       </c>
       <c r="P18" t="n">
-        <v>0.21441</v>
+        <v>0.424979</v>
       </c>
       <c r="Q18" t="n">
-        <v>746.4</v>
+        <v>2160.6</v>
       </c>
       <c r="R18" t="n">
-        <v>71127.60000000001</v>
+        <v>107730.2</v>
       </c>
       <c r="S18" t="n">
-        <v>22398.1</v>
+        <v>36900.3</v>
       </c>
       <c r="T18" t="n">
-        <v>48729.5</v>
+        <v>70829.89999999999</v>
       </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="n">
-        <v>5.159663003639629</v>
+        <v>1.736413207249709</v>
       </c>
       <c r="W18" t="n">
-        <v>0.05999114735478832</v>
+        <v>0.02101972067853934</v>
       </c>
       <c r="X18" t="n">
-        <v>0.1938111072941391</v>
+        <v>0.5758997891889408</v>
       </c>
       <c r="Y18" t="n">
-        <v>95.29421221864953</v>
+        <v>49.86124224752383</v>
       </c>
       <c r="Z18" t="n">
-        <v>0.629536106737947</v>
+        <v>0.421564319921917</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>step-5</t>
+          <t>glm-5-3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>GLM-5.3 (Max)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>StepFun</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>stepfun</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2110,85 +2078,85 @@
         <v>1</v>
       </c>
       <c r="I19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>43.7343049141614</v>
+        <v>44.777392385614</v>
       </c>
       <c r="K19" t="n">
-        <v>3.994000448781863</v>
+        <v>3.599468841287299</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
-        <v>6.586908</v>
+        <v>8.678356000000001</v>
       </c>
       <c r="N19" t="n">
-        <v>6.413718</v>
+        <v>8.365394999999999</v>
       </c>
       <c r="O19" t="n">
-        <v>0.055881</v>
+        <v>0.098552</v>
       </c>
       <c r="P19" t="n">
-        <v>0.117309</v>
+        <v>0.21441</v>
       </c>
       <c r="Q19" t="n">
-        <v>657</v>
+        <v>746.4</v>
       </c>
       <c r="R19" t="n">
-        <v>64144.3</v>
+        <v>71127.60000000001</v>
       </c>
       <c r="S19" t="n">
-        <v>20696.6</v>
+        <v>22398.1</v>
       </c>
       <c r="T19" t="n">
-        <v>43447.7</v>
+        <v>48729.5</v>
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="n">
-        <v>6.639580348497565</v>
+        <v>5.159663003639629</v>
       </c>
       <c r="W19" t="n">
-        <v>0.06656667414636439</v>
+        <v>0.05999114735478832</v>
       </c>
       <c r="X19" t="n">
-        <v>0.1506119283918727</v>
+        <v>0.1938111072941391</v>
       </c>
       <c r="Y19" t="n">
-        <v>97.63211567732117</v>
+        <v>95.29421221864953</v>
       </c>
       <c r="Z19" t="n">
-        <v>0.6818112429968274</v>
+        <v>0.629536106737947</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>kimi-k3</t>
+          <t>step-5</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Kimi K3 (Max)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Kimi K3 (max)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Kimi</t>
+          <t>StepFun</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>kimi</t>
+          <t>stepfun</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2200,265 +2168,265 @@
         <v>1</v>
       </c>
       <c r="I20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>43.5938229518782</v>
+        <v>43.7343049141614</v>
       </c>
       <c r="K20" t="n">
-        <v>2.353878129151091</v>
+        <v>4.008643896806728</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
-        <v>9.216749</v>
+        <v>6.586908</v>
       </c>
       <c r="N20" t="n">
-        <v>8.489921000000001</v>
+        <v>6.413718</v>
       </c>
       <c r="O20" t="n">
-        <v>0.240032</v>
+        <v>0.055881</v>
       </c>
       <c r="P20" t="n">
-        <v>0.486797</v>
+        <v>0.117309</v>
       </c>
       <c r="Q20" t="n">
-        <v>1111.2</v>
+        <v>654.6</v>
       </c>
       <c r="R20" t="n">
-        <v>48455.2</v>
+        <v>64144.3</v>
       </c>
       <c r="S20" t="n">
-        <v>16002.1</v>
+        <v>20696.6</v>
       </c>
       <c r="T20" t="n">
-        <v>32453.1</v>
+        <v>43447.7</v>
       </c>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="n">
-        <v>4.72984812235618</v>
+        <v>6.639580348497565</v>
       </c>
       <c r="W20" t="n">
-        <v>0.03923130215251818</v>
+        <v>0.06681073161344546</v>
       </c>
       <c r="X20" t="n">
-        <v>0.2114232791690251</v>
+        <v>0.1506119283918727</v>
       </c>
       <c r="Y20" t="n">
-        <v>43.60619150467962</v>
+        <v>97.99007027192178</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.8996727482680539</v>
+        <v>0.6818112429968274</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>claude-haiku-5-5</t>
+          <t>kimi-k3</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Claude Haiku 5.5 (Max)</t>
+          <t>Kimi K3 (Max)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Claude Haiku 5.5 (max)</t>
+          <t>Kimi K3 (max)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Kimi</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>kimi</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H21" t="b">
         <v>1</v>
       </c>
       <c r="I21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" t="n">
-        <v>43.3950199670746</v>
+        <v>43.5938229518782</v>
       </c>
       <c r="K21" t="n">
-        <v>6.181626775936554</v>
+        <v>2.62771687473648</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
-        <v>1.064978</v>
+        <v>9.216749</v>
       </c>
       <c r="N21" t="n">
-        <v>0.983896</v>
+        <v>8.489921000000001</v>
       </c>
       <c r="O21" t="n">
-        <v>0.016559</v>
+        <v>0.240032</v>
       </c>
       <c r="P21" t="n">
-        <v>0.064523</v>
+        <v>0.486797</v>
       </c>
       <c r="Q21" t="n">
-        <v>421.2</v>
+        <v>995.4</v>
       </c>
       <c r="R21" t="n">
-        <v>162164.2</v>
+        <v>48455.2</v>
       </c>
       <c r="S21" t="n">
-        <v>33117.6</v>
+        <v>16002.1</v>
       </c>
       <c r="T21" t="n">
-        <v>129046.6</v>
+        <v>32453.1</v>
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="n">
-        <v>40.74733935074209</v>
+        <v>4.72984812235618</v>
       </c>
       <c r="W21" t="n">
-        <v>0.1030271129322759</v>
+        <v>0.043795281245608</v>
       </c>
       <c r="X21" t="n">
-        <v>0.02454147966305898</v>
+        <v>0.2114232791690251</v>
       </c>
       <c r="Y21" t="n">
-        <v>385.0052231718899</v>
+        <v>48.67912397026321</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.2675992602995889</v>
+        <v>0.8996727482680539</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>glm-5-3-flash</t>
+          <t>claude-haiku-5-5</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Claude Haiku 5.5 (Max)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Claude Haiku 5.5 (max)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H22" t="b">
         <v>1</v>
       </c>
       <c r="I22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>41.807466113455</v>
+        <v>43.3950199670746</v>
       </c>
       <c r="K22" t="n">
-        <v>3.20363725007318</v>
+        <v>6.181626775936554</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
-        <v>1.193653</v>
+        <v>1.064978</v>
       </c>
       <c r="N22" t="n">
-        <v>1.159316</v>
+        <v>0.983896</v>
       </c>
       <c r="O22" t="n">
-        <v>0.011012</v>
+        <v>0.016559</v>
       </c>
       <c r="P22" t="n">
-        <v>0.023325</v>
+        <v>0.064523</v>
       </c>
       <c r="Q22" t="n">
-        <v>783</v>
+        <v>421.2</v>
       </c>
       <c r="R22" t="n">
-        <v>68673.2</v>
+        <v>162164.2</v>
       </c>
       <c r="S22" t="n">
-        <v>22023.7</v>
+        <v>33117.6</v>
       </c>
       <c r="T22" t="n">
-        <v>46649.5</v>
+        <v>129046.6</v>
       </c>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="n">
-        <v>35.02480713696107</v>
+        <v>40.74733935074209</v>
       </c>
       <c r="W22" t="n">
-        <v>0.05339395416788634</v>
+        <v>0.1030271129322759</v>
       </c>
       <c r="X22" t="n">
-        <v>0.02855119219042658</v>
+        <v>0.02454147966305898</v>
       </c>
       <c r="Y22" t="n">
-        <v>87.7052362707535</v>
+        <v>385.0052231718899</v>
       </c>
       <c r="Z22" t="n">
-        <v>0.6087886703030441</v>
+        <v>0.2675992602995889</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>gemini-3-8-flash</t>
+          <t>glm-5-3-flash</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (High)</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2470,85 +2438,85 @@
         <v>1</v>
       </c>
       <c r="I23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J23" t="n">
-        <v>40.9262321765904</v>
+        <v>41.807466113455</v>
       </c>
       <c r="K23" t="n">
-        <v>4.742321225560881</v>
+        <v>3.201184235333461</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
-        <v>4.90102</v>
+        <v>1.193653</v>
       </c>
       <c r="N23" t="n">
-        <v>4.63476</v>
+        <v>1.159316</v>
       </c>
       <c r="O23" t="n">
-        <v>0.106033</v>
+        <v>0.011012</v>
       </c>
       <c r="P23" t="n">
-        <v>0.160227</v>
+        <v>0.023325</v>
       </c>
       <c r="Q23" t="n">
-        <v>517.8000000000001</v>
+        <v>783.6</v>
       </c>
       <c r="R23" t="n">
-        <v>71002.60000000001</v>
+        <v>68673.2</v>
       </c>
       <c r="S23" t="n">
-        <v>28275.4</v>
+        <v>22023.7</v>
       </c>
       <c r="T23" t="n">
-        <v>42727.1</v>
+        <v>46649.5</v>
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="n">
-        <v>8.350554002348574</v>
+        <v>35.02480713696107</v>
       </c>
       <c r="W23" t="n">
-        <v>0.07903868709268135</v>
+        <v>0.05335307058889101</v>
       </c>
       <c r="X23" t="n">
-        <v>0.119752533750306</v>
+        <v>0.02855119219042658</v>
       </c>
       <c r="Y23" t="n">
-        <v>137.1235998455002</v>
+        <v>87.63808065339458</v>
       </c>
       <c r="Z23" t="n">
-        <v>0.5764046975264343</v>
+        <v>0.6087886703030441</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>deepseek-v4-1-flash</t>
+          <t>gemini-3-8-flash</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (Max)</t>
+          <t>Gemini 3.8 Flash (High)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (max)</t>
+          <t>Gemini 3.8 Flash (high)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>DeepSeek</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>deepseek</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2560,85 +2528,85 @@
         <v>1</v>
       </c>
       <c r="I24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>39.456167472527</v>
+        <v>40.9262321765904</v>
       </c>
       <c r="K24" t="n">
-        <v>7.782281552766665</v>
+        <v>5.122181749260376</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>3.127974</v>
+        <v>4.90102</v>
       </c>
       <c r="N24" t="n">
-        <v>3.021685</v>
+        <v>4.63476</v>
       </c>
       <c r="O24" t="n">
-        <v>0.031085</v>
+        <v>0.106033</v>
       </c>
       <c r="P24" t="n">
-        <v>0.07520300000000001</v>
+        <v>0.160227</v>
       </c>
       <c r="Q24" t="n">
-        <v>304.2</v>
+        <v>479.4</v>
       </c>
       <c r="R24" t="n">
-        <v>88574</v>
+        <v>71002.60000000001</v>
       </c>
       <c r="S24" t="n">
-        <v>25904.4</v>
+        <v>28275.4</v>
       </c>
       <c r="T24" t="n">
-        <v>62669.6</v>
+        <v>42727.1</v>
       </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="n">
-        <v>12.61396912906789</v>
+        <v>8.350554002348574</v>
       </c>
       <c r="W24" t="n">
-        <v>0.1297046925461111</v>
+        <v>0.08536969582100626</v>
       </c>
       <c r="X24" t="n">
-        <v>0.07927718783579227</v>
+        <v>0.119752533750306</v>
       </c>
       <c r="Y24" t="n">
-        <v>291.1702827087442</v>
+        <v>148.1072173550271</v>
       </c>
       <c r="Z24" t="n">
-        <v>0.4454599258532639</v>
+        <v>0.5764046975264343</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>mistral-large-4</t>
+          <t>deepseek-v4-1-flash</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Mistral Large 4 Preview</t>
+          <t>DeepSeek V4.1 Flash (Max)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mistral Large 4 Preview</t>
+          <t>DeepSeek V4.1 Flash (max)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Mistral</t>
+          <t>DeepSeek</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>mistral</t>
+          <t>deepseek</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2650,82 +2618,90 @@
         <v>1</v>
       </c>
       <c r="I25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>38.3770408917494</v>
-      </c>
-      <c r="K25" t="inlineStr"/>
+        <v>39.456167472527</v>
+      </c>
+      <c r="K25" t="n">
+        <v>7.472758991008901</v>
+      </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
-        <v>6.131298</v>
+        <v>3.127974</v>
       </c>
       <c r="N25" t="n">
-        <v>5.841498</v>
+        <v>3.021685</v>
       </c>
       <c r="O25" t="n">
-        <v>0.072395</v>
+        <v>0.031085</v>
       </c>
       <c r="P25" t="n">
-        <v>0.217404</v>
-      </c>
-      <c r="Q25" t="inlineStr"/>
+        <v>0.07520300000000001</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>316.8</v>
+      </c>
       <c r="R25" t="n">
-        <v>69330</v>
+        <v>88574</v>
       </c>
       <c r="S25" t="n">
-        <v>17319.4</v>
+        <v>25904.4</v>
       </c>
       <c r="T25" t="n">
-        <v>52010.6</v>
+        <v>62669.6</v>
       </c>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="n">
-        <v>6.259203335370325</v>
-      </c>
-      <c r="W25" t="inlineStr"/>
+        <v>12.61396912906789</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0.1245459831834817</v>
+      </c>
       <c r="X25" t="n">
-        <v>0.1597647410412551</v>
-      </c>
-      <c r="Y25" t="inlineStr"/>
+        <v>0.07927718783579227</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>279.5896464646465</v>
+      </c>
       <c r="Z25" t="n">
-        <v>0.5535416254399164</v>
+        <v>0.4454599258532639</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>gpt-6-luna</t>
+          <t>mistral-large-4</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (Max)</t>
+          <t>Mistral Large 4 Preview</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (max)</t>
+          <t>Mistral Large 4 Preview</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Mistral</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>mistral</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H26" t="b">
@@ -2735,177 +2711,169 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>38.1245186869738</v>
-      </c>
-      <c r="K26" t="n">
-        <v>6.354086447828966</v>
-      </c>
+        <v>38.3770408917494</v>
+      </c>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
-        <v>0.326276</v>
+        <v>6.144787</v>
       </c>
       <c r="N26" t="n">
-        <v>0.30127</v>
+        <v>5.854427</v>
       </c>
       <c r="O26" t="n">
-        <v>0.005561</v>
+        <v>0.07260800000000001</v>
       </c>
       <c r="P26" t="n">
-        <v>0.019445</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>360</v>
-      </c>
+        <v>0.217751</v>
+      </c>
+      <c r="Q26" t="inlineStr"/>
       <c r="R26" t="n">
-        <v>50011.7</v>
+        <v>69464</v>
       </c>
       <c r="S26" t="n">
-        <v>11122</v>
+        <v>17370.4</v>
       </c>
       <c r="T26" t="n">
-        <v>38889.7</v>
+        <v>52093.6</v>
       </c>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="n">
-        <v>116.8474502782117</v>
-      </c>
-      <c r="W26" t="n">
-        <v>0.1059014407971494</v>
-      </c>
+        <v>6.245463169309107</v>
+      </c>
+      <c r="W26" t="inlineStr"/>
       <c r="X26" t="n">
-        <v>0.008558167059863248</v>
-      </c>
-      <c r="Y26" t="n">
-        <v>138.9213888888889</v>
-      </c>
+        <v>0.1601162272342122</v>
+      </c>
+      <c r="Y26" t="inlineStr"/>
       <c r="Z26" t="n">
-        <v>0.7623119927331765</v>
+        <v>0.5524738122156715</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>qwen3-8-27b</t>
+          <t>gpt-6-luna</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (Xhigh)</t>
+          <t>GPT-6 Luna (Max)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (xhigh)</t>
+          <t>GPT-6 Luna (max)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H27" t="b">
         <v>1</v>
       </c>
       <c r="I27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>33.6962858057476</v>
+        <v>38.1245186869738</v>
       </c>
       <c r="K27" t="n">
-        <v>1.901596264432709</v>
+        <v>6.169015968765988</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
-        <v>2.505679</v>
+        <v>0.326276</v>
       </c>
       <c r="N27" t="n">
-        <v>2.305287</v>
+        <v>0.30127</v>
       </c>
       <c r="O27" t="n">
-        <v>0.05726</v>
+        <v>0.005561</v>
       </c>
       <c r="P27" t="n">
-        <v>0.143133</v>
+        <v>0.019445</v>
       </c>
       <c r="Q27" t="n">
-        <v>1063.2</v>
+        <v>370.8</v>
       </c>
       <c r="R27" t="n">
-        <v>66797.5</v>
+        <v>50011.7</v>
       </c>
       <c r="S27" t="n">
-        <v>19086.6</v>
+        <v>11122</v>
       </c>
       <c r="T27" t="n">
-        <v>47710.9</v>
+        <v>38889.7</v>
       </c>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="n">
-        <v>13.44796592290856</v>
+        <v>116.8474502782117</v>
       </c>
       <c r="W27" t="n">
-        <v>0.03169327107387849</v>
+        <v>0.1028169328127665</v>
       </c>
       <c r="X27" t="n">
-        <v>0.0743606881317645</v>
+        <v>0.008558167059863248</v>
       </c>
       <c r="Y27" t="n">
-        <v>62.82684349134689</v>
+        <v>134.8751348435815</v>
       </c>
       <c r="Z27" t="n">
-        <v>0.504454295531234</v>
+        <v>0.7623119927331765</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>k2-horizon-375b-a23b</t>
+          <t>qwen3-8-27b</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Qwen3.8 27B (Xhigh)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Qwen3.8 27B (xhigh)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Institute of Foundation Models</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ifm</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H28" t="b">
@@ -2915,54 +2883,82 @@
         <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>30.5015302696723</v>
-      </c>
-      <c r="K28" t="inlineStr"/>
+        <v>33.6962858057476</v>
+      </c>
+      <c r="K28" t="n">
+        <v>1.831319880747152</v>
+      </c>
       <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
-      <c r="T28" t="inlineStr"/>
+      <c r="M28" t="n">
+        <v>2.505679</v>
+      </c>
+      <c r="N28" t="n">
+        <v>2.305287</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0.05726</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0.143133</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>1104</v>
+      </c>
+      <c r="R28" t="n">
+        <v>66797.5</v>
+      </c>
+      <c r="S28" t="n">
+        <v>19086.6</v>
+      </c>
+      <c r="T28" t="n">
+        <v>47710.9</v>
+      </c>
       <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
-      <c r="X28" t="inlineStr"/>
-      <c r="Y28" t="inlineStr"/>
-      <c r="Z28" t="inlineStr"/>
+      <c r="V28" t="n">
+        <v>13.44796592290856</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.03052199801245254</v>
+      </c>
+      <c r="X28" t="n">
+        <v>0.0743606881317645</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>60.50498188405797</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>0.504454295531234</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>minimax-m3</t>
+          <t>k2-horizon-375b-a23b</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>Institute of Foundation Models</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>minimax</t>
+          <t>ifm</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2977,82 +2973,54 @@
         <v>1</v>
       </c>
       <c r="J29" t="n">
-        <v>29.2202932236316</v>
-      </c>
-      <c r="K29" t="n">
-        <v>3.643428082747083</v>
-      </c>
+        <v>30.5015302696723</v>
+      </c>
+      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
-      <c r="M29" t="n">
-        <v>1.912899</v>
-      </c>
-      <c r="N29" t="n">
-        <v>1.855069</v>
-      </c>
-      <c r="O29" t="n">
-        <v>0.031649</v>
-      </c>
-      <c r="P29" t="n">
-        <v>0.026182</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>481.2</v>
-      </c>
-      <c r="R29" t="n">
-        <v>48192</v>
-      </c>
-      <c r="S29" t="n">
-        <v>26373.8</v>
-      </c>
-      <c r="T29" t="n">
-        <v>21818.2</v>
-      </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
-      <c r="V29" t="n">
-        <v>15.27539782478406</v>
-      </c>
-      <c r="W29" t="n">
-        <v>0.06072380137911804</v>
-      </c>
-      <c r="X29" t="n">
-        <v>0.06546474346988973</v>
-      </c>
-      <c r="Y29" t="n">
-        <v>100.1496259351621</v>
-      </c>
-      <c r="Z29" t="n">
-        <v>0.6063307856829266</v>
-      </c>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>inkling</t>
+          <t>minimax-m3</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Inkling (Xhigh)</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Inkling (xhigh)</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Thinking Machines</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>thinking-machines</t>
+          <t>minimax</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3067,82 +3035,82 @@
         <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>24.9847810999384</v>
+        <v>29.2202932236316</v>
       </c>
       <c r="K30" t="n">
-        <v>9.646633629319847</v>
+        <v>3.938044908845229</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
-        <v>2.418996</v>
+        <v>1.912899</v>
       </c>
       <c r="N30" t="n">
-        <v>2.278639</v>
+        <v>1.855069</v>
       </c>
       <c r="O30" t="n">
-        <v>0.04559</v>
+        <v>0.031649</v>
       </c>
       <c r="P30" t="n">
-        <v>0.094767</v>
+        <v>0.026182</v>
       </c>
       <c r="Q30" t="n">
-        <v>155.4</v>
+        <v>445.2</v>
       </c>
       <c r="R30" t="n">
-        <v>34656</v>
+        <v>48192</v>
       </c>
       <c r="S30" t="n">
-        <v>11256.8</v>
+        <v>26373.8</v>
       </c>
       <c r="T30" t="n">
-        <v>23399.2</v>
+        <v>21818.2</v>
       </c>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="n">
-        <v>10.32857478885389</v>
+        <v>15.27539782478406</v>
       </c>
       <c r="W30" t="n">
-        <v>0.1607772271553308</v>
+        <v>0.06563408181408716</v>
       </c>
       <c r="X30" t="n">
-        <v>0.09681877901287532</v>
+        <v>0.06546474346988973</v>
       </c>
       <c r="Y30" t="n">
-        <v>223.011583011583</v>
+        <v>108.2479784366577</v>
       </c>
       <c r="Z30" t="n">
-        <v>0.7209366660877885</v>
+        <v>0.6063307856829266</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
+          <t>inkling</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
+          <t>Inkling (Xhigh)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra</t>
+          <t>Inkling (xhigh)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Thinking Machines</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>thinking-machines</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3157,87 +3125,87 @@
         <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>22.9279123422858</v>
+        <v>24.9847810999384</v>
       </c>
       <c r="K31" t="n">
-        <v>7.825226055387644</v>
+        <v>9.646633629319847</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
-        <v>0.717257</v>
+        <v>2.418996</v>
       </c>
       <c r="N31" t="n">
-        <v>0.646342</v>
+        <v>2.278639</v>
       </c>
       <c r="O31" t="n">
-        <v>0.03329</v>
+        <v>0.04559</v>
       </c>
       <c r="P31" t="n">
-        <v>0.037626</v>
+        <v>0.094767</v>
       </c>
       <c r="Q31" t="n">
-        <v>175.8</v>
+        <v>155.4</v>
       </c>
       <c r="R31" t="n">
-        <v>28366.1</v>
+        <v>34656</v>
       </c>
       <c r="S31" t="n">
-        <v>13315.8</v>
+        <v>11256.8</v>
       </c>
       <c r="T31" t="n">
-        <v>15050.3</v>
+        <v>23399.2</v>
       </c>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="n">
-        <v>31.96610467696488</v>
+        <v>10.32857478885389</v>
       </c>
       <c r="W31" t="n">
-        <v>0.1304204342564607</v>
+        <v>0.1607772271553308</v>
       </c>
       <c r="X31" t="n">
-        <v>0.0312831360000085</v>
+        <v>0.09681877901287532</v>
       </c>
       <c r="Y31" t="n">
-        <v>161.3543799772469</v>
+        <v>223.011583011583</v>
       </c>
       <c r="Z31" t="n">
-        <v>0.8082856769977473</v>
+        <v>0.7209366660877885</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>muse-glimmer</t>
+          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Muse Glimmer (High)</t>
+          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Muse Glimmer (high)</t>
+          <t>Nemotron 3 Ultra</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>nvidia</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H32" t="b">
@@ -3247,50 +3215,140 @@
         <v>1</v>
       </c>
       <c r="J32" t="n">
-        <v>17.4754176089465</v>
+        <v>22.9279123422858</v>
       </c>
       <c r="K32" t="n">
-        <v>9.197588215235001</v>
+        <v>8.247450482836619</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
-        <v>0.227808</v>
+        <v>0.717257</v>
       </c>
       <c r="N32" t="n">
-        <v>0.209009</v>
+        <v>0.646342</v>
       </c>
       <c r="O32" t="n">
-        <v>0.005909</v>
+        <v>0.03329</v>
       </c>
       <c r="P32" t="n">
-        <v>0.01289</v>
+        <v>0.037626</v>
       </c>
       <c r="Q32" t="n">
-        <v>114</v>
+        <v>166.8</v>
       </c>
       <c r="R32" t="n">
-        <v>13925.2</v>
+        <v>28366.1</v>
       </c>
       <c r="S32" t="n">
-        <v>4377.3</v>
+        <v>13315.8</v>
       </c>
       <c r="T32" t="n">
-        <v>9547.9</v>
+        <v>15050.3</v>
       </c>
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="n">
+        <v>31.96610467696488</v>
+      </c>
+      <c r="W32" t="n">
+        <v>0.137457508047277</v>
+      </c>
+      <c r="X32" t="n">
+        <v>0.0312831360000085</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>170.060551558753</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>0.8082856769977473</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>muse-glimmer</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Muse Glimmer (High)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Muse Glimmer (high)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>small</t>
+        </is>
+      </c>
+      <c r="H33" t="b">
+        <v>1</v>
+      </c>
+      <c r="I33" t="b">
+        <v>1</v>
+      </c>
+      <c r="J33" t="n">
+        <v>17.4754176089465</v>
+      </c>
+      <c r="K33" t="n">
+        <v>9.817650342104775</v>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="n">
+        <v>0.227808</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0.209009</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0.005909</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0.01289</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>106.8</v>
+      </c>
+      <c r="R33" t="n">
+        <v>13925.2</v>
+      </c>
+      <c r="S33" t="n">
+        <v>4377.3</v>
+      </c>
+      <c r="T33" t="n">
+        <v>9547.9</v>
+      </c>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="n">
         <v>76.71116733805002</v>
       </c>
-      <c r="W32" t="n">
-        <v>0.1532931369205833</v>
-      </c>
-      <c r="X32" t="n">
+      <c r="W33" t="n">
+        <v>0.1636275057017463</v>
+      </c>
+      <c r="X33" t="n">
         <v>0.01303591165016704</v>
       </c>
-      <c r="Y32" t="n">
-        <v>122.1508771929825</v>
-      </c>
-      <c r="Z32" t="n">
+      <c r="Y33" t="n">
+        <v>130.3857677902622</v>
+      </c>
+      <c r="Z33" t="n">
         <v>1.254949128841704</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-14)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.365331046234568</v>
+        <v>4.381929263140403</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.0727555174372428</v>
+        <v>0.07303215438567338</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>150.4621212121212</v>
+        <v>151.0342205323194</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.608255712505116</v>
+        <v>3.657748442722364</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>931.1999999999999</v>
+        <v>918.6</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.0601375952084186</v>
+        <v>0.06096247404537274</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>212.0171821305842</v>
+        <v>214.9253211408665</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.70507192622921</v>
+        <v>6.641441350416834</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>501</v>
+        <v>505.8</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1117511987704868</v>
+        <v>0.1106906891736139</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>131.0726546906187</v>
+        <v>129.8287860814551</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -922,7 +922,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K6" t="n">
-        <v>11.88097471889284</v>
+        <v>11.82852008437234</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -938,7 +938,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q6" t="n">
-        <v>270.6</v>
+        <v>271.8</v>
       </c>
       <c r="R6" t="n">
         <v>35584.1</v>
@@ -954,13 +954,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1980162453148807</v>
+        <v>0.1971420014062057</v>
       </c>
       <c r="X6" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y6" t="n">
-        <v>131.5007390983001</v>
+        <v>130.920161883738</v>
       </c>
       <c r="Z6" t="n">
         <v>1.505818497087371</v>
@@ -1012,7 +1012,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K7" t="n">
-        <v>4.564151066067168</v>
+        <v>4.67615477320992</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1028,7 +1028,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q7" t="n">
-        <v>701.4</v>
+        <v>684.6</v>
       </c>
       <c r="R7" t="n">
         <v>78110.8</v>
@@ -1044,13 +1044,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W7" t="n">
-        <v>0.07606918443445281</v>
+        <v>0.07793591288683201</v>
       </c>
       <c r="X7" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y7" t="n">
-        <v>111.364128885087</v>
+        <v>114.0969909436167</v>
       </c>
       <c r="Z7" t="n">
         <v>0.6830672066132366</v>
@@ -1102,7 +1102,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K8" t="n">
-        <v>5.26243904588471</v>
+        <v>5.368643668405086</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1118,7 +1118,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q8" t="n">
-        <v>606.5999999999999</v>
+        <v>594.6</v>
       </c>
       <c r="R8" t="n">
         <v>60537.6</v>
@@ -1134,13 +1134,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W8" t="n">
-        <v>0.08770731743141182</v>
+        <v>0.0894773944734181</v>
       </c>
       <c r="X8" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y8" t="n">
-        <v>99.79821958456975</v>
+        <v>101.8123107971746</v>
       </c>
       <c r="Z8" t="n">
         <v>0.8788465144619939</v>
@@ -1192,7 +1192,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K9" t="n">
-        <v>7.325962363770932</v>
+        <v>6.718580280039924</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q9" t="n">
-        <v>431.4</v>
+        <v>470.4</v>
       </c>
       <c r="R9" t="n">
         <v>27205.5</v>
@@ -1224,13 +1224,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1220993727295155</v>
+        <v>0.1119763380006654</v>
       </c>
       <c r="X9" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y9" t="n">
-        <v>63.06328233657857</v>
+        <v>57.83482142857143</v>
       </c>
       <c r="Z9" t="n">
         <v>1.936140464079432</v>
@@ -1364,7 +1364,7 @@
         <v>52.393894697293</v>
       </c>
       <c r="K11" t="n">
-        <v>6.267212284365192</v>
+        <v>7.671141244113177</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1380,7 +1380,7 @@
         <v>0.573611</v>
       </c>
       <c r="Q11" t="n">
-        <v>501.6</v>
+        <v>409.8</v>
       </c>
       <c r="R11" t="n">
         <v>54231.7</v>
@@ -1396,13 +1396,13 @@
         <v>1.645610026239954</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1044535380727532</v>
+        <v>0.1278523540685529</v>
       </c>
       <c r="X11" t="n">
         <v>0.6076773865342173</v>
       </c>
       <c r="Y11" t="n">
-        <v>108.1174242424242</v>
+        <v>132.3369936554417</v>
       </c>
       <c r="Z11" t="n">
         <v>0.9661119732055791</v>
@@ -1454,7 +1454,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K12" t="n">
-        <v>11.12236257131172</v>
+        <v>9.921652975545113</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1470,7 +1470,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q12" t="n">
-        <v>282.6</v>
+        <v>316.8</v>
       </c>
       <c r="R12" t="n">
         <v>16901.2</v>
@@ -1486,13 +1486,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W12" t="n">
-        <v>0.185372709521862</v>
+        <v>0.1653608829257519</v>
       </c>
       <c r="X12" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y12" t="n">
-        <v>59.80608634111819</v>
+        <v>53.34974747474747</v>
       </c>
       <c r="Z12" t="n">
         <v>3.099562617499243</v>
@@ -1544,7 +1544,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K13" t="n">
-        <v>6.965846230645489</v>
+        <v>7.022402492328673</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1560,7 +1560,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q13" t="n">
-        <v>447</v>
+        <v>443.4</v>
       </c>
       <c r="R13" t="n">
         <v>74809.60000000001</v>
@@ -1576,13 +1576,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1160974371774248</v>
+        <v>0.1170400415388112</v>
       </c>
       <c r="X13" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y13" t="n">
-        <v>167.3592841163311</v>
+        <v>168.7180875056383</v>
       </c>
       <c r="Z13" t="n">
         <v>0.6937018032218979</v>
@@ -1634,7 +1634,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K14" t="n">
-        <v>5.321689907716026</v>
+        <v>4.472239836165151</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1650,7 +1650,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q14" t="n">
-        <v>584.4</v>
+        <v>695.4</v>
       </c>
       <c r="R14" t="n">
         <v>38128.4</v>
@@ -1666,13 +1666,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W14" t="n">
-        <v>0.08869483179526712</v>
+        <v>0.07453733060275251</v>
       </c>
       <c r="X14" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y14" t="n">
-        <v>65.24366872005476</v>
+        <v>54.82945067587001</v>
       </c>
       <c r="Z14" t="n">
         <v>1.359439674918279</v>
@@ -1724,7 +1724,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K15" t="n">
-        <v>6.173595734527407</v>
+        <v>6.157786270418502</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1740,7 +1740,7 @@
         <v>0.145035</v>
       </c>
       <c r="Q15" t="n">
-        <v>467.4</v>
+        <v>468.6</v>
       </c>
       <c r="R15" t="n">
         <v>60200.2</v>
@@ -1756,13 +1756,13 @@
         <v>6.17518114688861</v>
       </c>
       <c r="W15" t="n">
-        <v>0.1028932622421234</v>
+        <v>0.1026297711736417</v>
       </c>
       <c r="X15" t="n">
         <v>0.161938569284539</v>
       </c>
       <c r="Y15" t="n">
-        <v>128.7980316645272</v>
+        <v>128.468203158344</v>
       </c>
       <c r="Z15" t="n">
         <v>0.7988729401558218</v>
@@ -1814,7 +1814,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K16" t="n">
-        <v>3.082053790990617</v>
+        <v>2.930381743232088</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1830,7 +1830,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q16" t="n">
-        <v>904.2</v>
+        <v>951</v>
       </c>
       <c r="R16" t="n">
         <v>80561.39999999999</v>
@@ -1846,13 +1846,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W16" t="n">
-        <v>0.05136756318317695</v>
+        <v>0.04883969572053481</v>
       </c>
       <c r="X16" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y16" t="n">
-        <v>89.0968812209688</v>
+        <v>84.71230283911672</v>
       </c>
       <c r="Z16" t="n">
         <v>0.5765360412086756</v>
@@ -1904,7 +1904,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K17" t="n">
-        <v>2.105645751410832</v>
+        <v>2.048837086733229</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1920,7 +1920,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q17" t="n">
-        <v>1320</v>
+        <v>1356.6</v>
       </c>
       <c r="R17" t="n">
         <v>64275.7</v>
@@ -1936,13 +1936,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W17" t="n">
-        <v>0.0350940958568472</v>
+        <v>0.03414728477888715</v>
       </c>
       <c r="X17" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y17" t="n">
-        <v>48.69371212121212</v>
+        <v>47.37999410290432</v>
       </c>
       <c r="Z17" t="n">
         <v>0.7207110390246749</v>
@@ -1994,7 +1994,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K18" t="n">
-        <v>1.261183240712361</v>
+        <v>1.379143896084182</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2010,7 +2010,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q18" t="n">
-        <v>2160.6</v>
+        <v>1975.8</v>
       </c>
       <c r="R18" t="n">
         <v>107730.2</v>
@@ -2026,13 +2026,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W18" t="n">
-        <v>0.02101972067853934</v>
+        <v>0.02298573160140303</v>
       </c>
       <c r="X18" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y18" t="n">
-        <v>49.86124224752383</v>
+        <v>54.52485069339002</v>
       </c>
       <c r="Z18" t="n">
         <v>0.421564319921917</v>
@@ -2084,7 +2084,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K19" t="n">
-        <v>3.599468841287299</v>
+        <v>3.242389021405793</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2100,7 +2100,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q19" t="n">
-        <v>746.4</v>
+        <v>828.6</v>
       </c>
       <c r="R19" t="n">
         <v>71127.60000000001</v>
@@ -2116,13 +2116,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W19" t="n">
-        <v>0.05999114735478832</v>
+        <v>0.05403981702342988</v>
       </c>
       <c r="X19" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y19" t="n">
-        <v>95.29421221864953</v>
+        <v>85.84069514844316</v>
       </c>
       <c r="Z19" t="n">
         <v>0.629536106737947</v>
@@ -2174,7 +2174,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K20" t="n">
-        <v>4.008643896806728</v>
+        <v>4.045726634057483</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2190,7 +2190,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q20" t="n">
-        <v>654.6</v>
+        <v>648.6</v>
       </c>
       <c r="R20" t="n">
         <v>64144.3</v>
@@ -2206,13 +2206,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W20" t="n">
-        <v>0.06681073161344546</v>
+        <v>0.06742877723429139</v>
       </c>
       <c r="X20" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y20" t="n">
-        <v>97.99007027192178</v>
+        <v>98.89654640764724</v>
       </c>
       <c r="Z20" t="n">
         <v>0.6818112429968274</v>
@@ -2264,7 +2264,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K21" t="n">
-        <v>2.62771687473648</v>
+        <v>2.722912114420875</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2280,7 +2280,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q21" t="n">
-        <v>995.4</v>
+        <v>960.6000000000001</v>
       </c>
       <c r="R21" t="n">
         <v>48455.2</v>
@@ -2296,13 +2296,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W21" t="n">
-        <v>0.043795281245608</v>
+        <v>0.04538186857368124</v>
       </c>
       <c r="X21" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y21" t="n">
-        <v>48.67912397026321</v>
+        <v>50.44264001665625</v>
       </c>
       <c r="Z21" t="n">
         <v>0.8996727482680539</v>
@@ -2354,7 +2354,7 @@
         <v>43.3950199670746</v>
       </c>
       <c r="K22" t="n">
-        <v>6.181626775936554</v>
+        <v>6.155321981145334</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2370,7 +2370,7 @@
         <v>0.064523</v>
       </c>
       <c r="Q22" t="n">
-        <v>421.2</v>
+        <v>423</v>
       </c>
       <c r="R22" t="n">
         <v>162164.2</v>
@@ -2386,13 +2386,13 @@
         <v>40.74733935074209</v>
       </c>
       <c r="W22" t="n">
-        <v>0.1030271129322759</v>
+        <v>0.1025886996857556</v>
       </c>
       <c r="X22" t="n">
         <v>0.02454147966305898</v>
       </c>
       <c r="Y22" t="n">
-        <v>385.0052231718899</v>
+        <v>383.3669030732861</v>
       </c>
       <c r="Z22" t="n">
         <v>0.2675992602995889</v>
@@ -2444,7 +2444,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K23" t="n">
-        <v>3.201184235333461</v>
+        <v>3.188975294695271</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2460,7 +2460,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q23" t="n">
-        <v>783.6</v>
+        <v>786.5999999999999</v>
       </c>
       <c r="R23" t="n">
         <v>68673.2</v>
@@ -2476,13 +2476,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W23" t="n">
-        <v>0.05335307058889101</v>
+        <v>0.05314958824492119</v>
       </c>
       <c r="X23" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y23" t="n">
-        <v>87.63808065339458</v>
+        <v>87.30383930841597</v>
       </c>
       <c r="Z23" t="n">
         <v>0.6087886703030441</v>
@@ -2534,7 +2534,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K24" t="n">
-        <v>5.122181749260376</v>
+        <v>5.220182675585511</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2550,7 +2550,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q24" t="n">
-        <v>479.4</v>
+        <v>470.4</v>
       </c>
       <c r="R24" t="n">
         <v>71002.60000000001</v>
@@ -2566,13 +2566,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W24" t="n">
-        <v>0.08536969582100626</v>
+        <v>0.08700304459309186</v>
       </c>
       <c r="X24" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y24" t="n">
-        <v>148.1072173550271</v>
+        <v>150.9409013605442</v>
       </c>
       <c r="Z24" t="n">
         <v>0.5764046975264343</v>
@@ -2624,7 +2624,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K25" t="n">
-        <v>7.472758991008901</v>
+        <v>7.134930826858408</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2640,7 +2640,7 @@
         <v>0.07520300000000001</v>
       </c>
       <c r="Q25" t="n">
-        <v>316.8</v>
+        <v>331.8</v>
       </c>
       <c r="R25" t="n">
         <v>88574</v>
@@ -2656,13 +2656,13 @@
         <v>12.61396912906789</v>
       </c>
       <c r="W25" t="n">
-        <v>0.1245459831834817</v>
+        <v>0.1189155137809735</v>
       </c>
       <c r="X25" t="n">
         <v>0.07927718783579227</v>
       </c>
       <c r="Y25" t="n">
-        <v>279.5896464646465</v>
+        <v>266.9499698613623</v>
       </c>
       <c r="Z25" t="n">
         <v>0.4454599258532639</v>
@@ -2796,7 +2796,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K27" t="n">
-        <v>6.169015968765988</v>
+        <v>6.199108729589235</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2812,7 +2812,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q27" t="n">
-        <v>370.8</v>
+        <v>369</v>
       </c>
       <c r="R27" t="n">
         <v>50011.7</v>
@@ -2828,13 +2828,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W27" t="n">
-        <v>0.1028169328127665</v>
+        <v>0.1033184788264873</v>
       </c>
       <c r="X27" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y27" t="n">
-        <v>134.8751348435815</v>
+        <v>135.5330623306233</v>
       </c>
       <c r="Z27" t="n">
         <v>0.7623119927331765</v>
@@ -2883,51 +2883,51 @@
         <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>33.6962858057476</v>
+        <v>33.6762858057476</v>
       </c>
       <c r="K28" t="n">
-        <v>1.831319880747152</v>
+        <v>1.70168195077047</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
-        <v>2.505679</v>
+        <v>2.505854</v>
       </c>
       <c r="N28" t="n">
-        <v>2.305287</v>
+        <v>2.305504</v>
       </c>
       <c r="O28" t="n">
-        <v>0.05726</v>
+        <v>0.057275</v>
       </c>
       <c r="P28" t="n">
-        <v>0.143133</v>
+        <v>0.143075</v>
       </c>
       <c r="Q28" t="n">
-        <v>1104</v>
+        <v>1187.4</v>
       </c>
       <c r="R28" t="n">
-        <v>66797.5</v>
+        <v>66783.2</v>
       </c>
       <c r="S28" t="n">
-        <v>19086.6</v>
+        <v>19091.6</v>
       </c>
       <c r="T28" t="n">
-        <v>47710.9</v>
+        <v>47691.6</v>
       </c>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="n">
-        <v>13.44796592290856</v>
+        <v>13.43904545346521</v>
       </c>
       <c r="W28" t="n">
-        <v>0.03052199801245254</v>
+        <v>0.0283613658461745</v>
       </c>
       <c r="X28" t="n">
-        <v>0.0743606881317645</v>
+        <v>0.07441004671519687</v>
       </c>
       <c r="Y28" t="n">
-        <v>60.50498188405797</v>
+        <v>56.24322048172478</v>
       </c>
       <c r="Z28" t="n">
-        <v>0.504454295531234</v>
+        <v>0.5042628356494987</v>
       </c>
     </row>
     <row r="29">
@@ -3038,7 +3038,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K30" t="n">
-        <v>3.938044908845229</v>
+        <v>3.491074459215245</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3054,7 +3054,7 @@
         <v>0.026182</v>
       </c>
       <c r="Q30" t="n">
-        <v>445.2</v>
+        <v>502.1999999999999</v>
       </c>
       <c r="R30" t="n">
         <v>48192</v>
@@ -3070,13 +3070,13 @@
         <v>15.27539782478406</v>
       </c>
       <c r="W30" t="n">
-        <v>0.06563408181408716</v>
+        <v>0.05818457432025409</v>
       </c>
       <c r="X30" t="n">
         <v>0.06546474346988973</v>
       </c>
       <c r="Y30" t="n">
-        <v>108.2479784366577</v>
+        <v>95.96176821983275</v>
       </c>
       <c r="Z30" t="n">
         <v>0.6063307856829266</v>
@@ -3128,7 +3128,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K31" t="n">
-        <v>9.646633629319847</v>
+        <v>9.499916768037414</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3144,7 +3144,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q31" t="n">
-        <v>155.4</v>
+        <v>157.8</v>
       </c>
       <c r="R31" t="n">
         <v>34656</v>
@@ -3160,13 +3160,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W31" t="n">
-        <v>0.1607772271553308</v>
+        <v>0.1583319461339569</v>
       </c>
       <c r="X31" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y31" t="n">
-        <v>223.011583011583</v>
+        <v>219.6197718631179</v>
       </c>
       <c r="Z31" t="n">
         <v>0.7209366660877885</v>
@@ -3218,7 +3218,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K32" t="n">
-        <v>8.247450482836619</v>
+        <v>8.188540122244929</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3234,7 +3234,7 @@
         <v>0.037626</v>
       </c>
       <c r="Q32" t="n">
-        <v>166.8</v>
+        <v>168</v>
       </c>
       <c r="R32" t="n">
         <v>28366.1</v>
@@ -3250,13 +3250,13 @@
         <v>31.96610467696488</v>
       </c>
       <c r="W32" t="n">
-        <v>0.137457508047277</v>
+        <v>0.1364756687040821</v>
       </c>
       <c r="X32" t="n">
         <v>0.0312831360000085</v>
       </c>
       <c r="Y32" t="n">
-        <v>170.060551558753</v>
+        <v>168.8458333333333</v>
       </c>
       <c r="Z32" t="n">
         <v>0.8082856769977473</v>
@@ -3312,16 +3312,16 @@
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
-        <v>0.227808</v>
+        <v>0.209642</v>
       </c>
       <c r="N33" t="n">
-        <v>0.209009</v>
+        <v>0.192931</v>
       </c>
       <c r="O33" t="n">
-        <v>0.005909</v>
+        <v>0.005253</v>
       </c>
       <c r="P33" t="n">
-        <v>0.01289</v>
+        <v>0.011457</v>
       </c>
       <c r="Q33" t="n">
         <v>106.8</v>
@@ -3337,13 +3337,13 @@
       </c>
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="n">
-        <v>76.71116733805002</v>
+        <v>83.3583805198696</v>
       </c>
       <c r="W33" t="n">
         <v>0.1636275057017463</v>
       </c>
       <c r="X33" t="n">
-        <v>0.01303591165016704</v>
+        <v>0.0119963942888938</v>
       </c>
       <c r="Y33" t="n">
         <v>130.3857677902622</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-15)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.381929263140403</v>
+        <v>4.335768984973386</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>789</v>
+        <v>797.4</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07303215438567338</v>
+        <v>0.07226281641622311</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>151.0342205323194</v>
+        <v>149.4431903686983</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.657748442722364</v>
+        <v>3.580570886066457</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>918.6</v>
+        <v>938.4000000000001</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.06096247404537274</v>
+        <v>0.05967618143444096</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>214.9253211408665</v>
+        <v>210.390451832907</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.641441350416834</v>
+        <v>6.480017428705311</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>505.8</v>
+        <v>518.4000000000001</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1106906891736139</v>
+        <v>0.1080002904784219</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>129.8287860814551</v>
+        <v>126.6732253086419</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -922,7 +922,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K6" t="n">
-        <v>11.82852008437234</v>
+        <v>11.00270964727037</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -938,7 +938,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q6" t="n">
-        <v>271.8</v>
+        <v>292.2</v>
       </c>
       <c r="R6" t="n">
         <v>35584.1</v>
@@ -954,13 +954,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1971420014062057</v>
+        <v>0.1833784941211729</v>
       </c>
       <c r="X6" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y6" t="n">
-        <v>130.920161883738</v>
+        <v>121.7799452429843</v>
       </c>
       <c r="Z6" t="n">
         <v>1.505818497087371</v>
@@ -1012,7 +1012,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K7" t="n">
-        <v>4.67615477320992</v>
+        <v>4.655752701773577</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1028,7 +1028,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q7" t="n">
-        <v>684.6</v>
+        <v>687.6</v>
       </c>
       <c r="R7" t="n">
         <v>78110.8</v>
@@ -1044,13 +1044,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W7" t="n">
-        <v>0.07793591288683201</v>
+        <v>0.07759587836289296</v>
       </c>
       <c r="X7" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y7" t="n">
-        <v>114.0969909436167</v>
+        <v>113.5991855730076</v>
       </c>
       <c r="Z7" t="n">
         <v>0.6830672066132366</v>
@@ -1102,7 +1102,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K8" t="n">
-        <v>5.368643668405086</v>
+        <v>5.028663398288696</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1118,7 +1118,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q8" t="n">
-        <v>594.6</v>
+        <v>634.8</v>
       </c>
       <c r="R8" t="n">
         <v>60537.6</v>
@@ -1134,13 +1134,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W8" t="n">
-        <v>0.0894773944734181</v>
+        <v>0.08381105663814493</v>
       </c>
       <c r="X8" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y8" t="n">
-        <v>101.8123107971746</v>
+        <v>95.3648393194707</v>
       </c>
       <c r="Z8" t="n">
         <v>0.8788465144619939</v>
@@ -1192,7 +1192,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K9" t="n">
-        <v>6.718580280039924</v>
+        <v>5.325952416128715</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q9" t="n">
-        <v>470.4</v>
+        <v>593.4000000000001</v>
       </c>
       <c r="R9" t="n">
         <v>27205.5</v>
@@ -1224,13 +1224,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1119763380006654</v>
+        <v>0.08876587360214526</v>
       </c>
       <c r="X9" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y9" t="n">
-        <v>57.83482142857143</v>
+        <v>45.84681496461071</v>
       </c>
       <c r="Z9" t="n">
         <v>1.936140464079432</v>
@@ -1364,7 +1364,7 @@
         <v>52.393894697293</v>
       </c>
       <c r="K11" t="n">
-        <v>7.671141244113177</v>
+        <v>8.880321135134405</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1380,7 +1380,7 @@
         <v>0.573611</v>
       </c>
       <c r="Q11" t="n">
-        <v>409.8</v>
+        <v>354</v>
       </c>
       <c r="R11" t="n">
         <v>54231.7</v>
@@ -1396,13 +1396,13 @@
         <v>1.645610026239954</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1278523540685529</v>
+        <v>0.1480053522522401</v>
       </c>
       <c r="X11" t="n">
         <v>0.6076773865342173</v>
       </c>
       <c r="Y11" t="n">
-        <v>132.3369936554417</v>
+        <v>153.1968926553672</v>
       </c>
       <c r="Z11" t="n">
         <v>0.9661119732055791</v>
@@ -1454,7 +1454,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K12" t="n">
-        <v>9.921652975545113</v>
+        <v>8.071853268240092</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1470,7 +1470,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q12" t="n">
-        <v>316.8</v>
+        <v>389.4</v>
       </c>
       <c r="R12" t="n">
         <v>16901.2</v>
@@ -1486,13 +1486,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W12" t="n">
-        <v>0.1653608829257519</v>
+        <v>0.1345308878040015</v>
       </c>
       <c r="X12" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y12" t="n">
-        <v>53.34974747474747</v>
+        <v>43.40318438623523</v>
       </c>
       <c r="Z12" t="n">
         <v>3.099562617499243</v>
@@ -1544,7 +1544,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K13" t="n">
-        <v>7.022402492328673</v>
+        <v>6.585730256130571</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1560,7 +1560,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q13" t="n">
-        <v>443.4</v>
+        <v>472.8</v>
       </c>
       <c r="R13" t="n">
         <v>74809.60000000001</v>
@@ -1576,13 +1576,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1170400415388112</v>
+        <v>0.1097621709355095</v>
       </c>
       <c r="X13" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y13" t="n">
-        <v>168.7180875056383</v>
+        <v>158.2267343485618</v>
       </c>
       <c r="Z13" t="n">
         <v>0.6937018032218979</v>
@@ -1634,7 +1634,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K14" t="n">
-        <v>4.472239836165151</v>
+        <v>3.941692752939475</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1650,7 +1650,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q14" t="n">
-        <v>695.4</v>
+        <v>789</v>
       </c>
       <c r="R14" t="n">
         <v>38128.4</v>
@@ -1666,13 +1666,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W14" t="n">
-        <v>0.07453733060275251</v>
+        <v>0.06569487921565792</v>
       </c>
       <c r="X14" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y14" t="n">
-        <v>54.82945067587001</v>
+        <v>48.32496831432193</v>
       </c>
       <c r="Z14" t="n">
         <v>1.359439674918279</v>
@@ -1724,7 +1724,7 @@
         <v>48.0923107719685</v>
       </c>
       <c r="K15" t="n">
-        <v>6.157786270418502</v>
+        <v>6.213476843923578</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1740,7 +1740,7 @@
         <v>0.145035</v>
       </c>
       <c r="Q15" t="n">
-        <v>468.6</v>
+        <v>464.4</v>
       </c>
       <c r="R15" t="n">
         <v>60200.2</v>
@@ -1756,13 +1756,13 @@
         <v>6.17518114688861</v>
       </c>
       <c r="W15" t="n">
-        <v>0.1026297711736417</v>
+        <v>0.1035579473987263</v>
       </c>
       <c r="X15" t="n">
         <v>0.161938569284539</v>
       </c>
       <c r="Y15" t="n">
-        <v>128.468203158344</v>
+        <v>129.630060292851</v>
       </c>
       <c r="Z15" t="n">
         <v>0.7988729401558218</v>
@@ -1814,7 +1814,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K16" t="n">
-        <v>2.930381743232088</v>
+        <v>2.725736539332665</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1830,7 +1830,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q16" t="n">
-        <v>951</v>
+        <v>1022.4</v>
       </c>
       <c r="R16" t="n">
         <v>80561.39999999999</v>
@@ -1846,13 +1846,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W16" t="n">
-        <v>0.04883969572053481</v>
+        <v>0.04542894232221107</v>
       </c>
       <c r="X16" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y16" t="n">
-        <v>84.71230283911672</v>
+        <v>78.79636150234741</v>
       </c>
       <c r="Z16" t="n">
         <v>0.5765360412086756</v>
@@ -1904,7 +1904,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K17" t="n">
-        <v>2.048837086733229</v>
+        <v>2.065278935846558</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1920,7 +1920,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q17" t="n">
-        <v>1356.6</v>
+        <v>1345.8</v>
       </c>
       <c r="R17" t="n">
         <v>64275.7</v>
@@ -1936,13 +1936,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W17" t="n">
-        <v>0.03414728477888715</v>
+        <v>0.03442131559744264</v>
       </c>
       <c r="X17" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y17" t="n">
-        <v>47.37999410290432</v>
+        <v>47.76021697131817</v>
       </c>
       <c r="Z17" t="n">
         <v>0.7207110390246749</v>
@@ -1994,7 +1994,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K18" t="n">
-        <v>1.379143896084182</v>
+        <v>1.275708103877868</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2010,7 +2010,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q18" t="n">
-        <v>1975.8</v>
+        <v>2136</v>
       </c>
       <c r="R18" t="n">
         <v>107730.2</v>
@@ -2026,13 +2026,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W18" t="n">
-        <v>0.02298573160140303</v>
+        <v>0.0212618017312978</v>
       </c>
       <c r="X18" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y18" t="n">
-        <v>54.52485069339002</v>
+        <v>50.43548689138576</v>
       </c>
       <c r="Z18" t="n">
         <v>0.421564319921917</v>
@@ -2084,7 +2084,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K19" t="n">
-        <v>3.242389021405793</v>
+        <v>3.196102240229408</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2100,7 +2100,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q19" t="n">
-        <v>828.6</v>
+        <v>840.6</v>
       </c>
       <c r="R19" t="n">
         <v>71127.60000000001</v>
@@ -2116,13 +2116,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W19" t="n">
-        <v>0.05403981702342988</v>
+        <v>0.05326837067049012</v>
       </c>
       <c r="X19" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y19" t="n">
-        <v>85.84069514844316</v>
+        <v>84.61527480371164</v>
       </c>
       <c r="Z19" t="n">
         <v>0.629536106737947</v>
@@ -2174,7 +2174,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K20" t="n">
-        <v>4.045726634057483</v>
+        <v>4.258452279859922</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2190,7 +2190,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q20" t="n">
-        <v>648.6</v>
+        <v>616.1999999999999</v>
       </c>
       <c r="R20" t="n">
         <v>64144.3</v>
@@ -2206,13 +2206,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W20" t="n">
-        <v>0.06742877723429139</v>
+        <v>0.07097420466433205</v>
       </c>
       <c r="X20" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y20" t="n">
-        <v>98.89654640764724</v>
+        <v>104.0965595585849</v>
       </c>
       <c r="Z20" t="n">
         <v>0.6818112429968274</v>
@@ -2264,7 +2264,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K21" t="n">
-        <v>2.722912114420875</v>
+        <v>2.643652089258836</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2280,7 +2280,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q21" t="n">
-        <v>960.6000000000001</v>
+        <v>989.3999999999999</v>
       </c>
       <c r="R21" t="n">
         <v>48455.2</v>
@@ -2296,13 +2296,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W21" t="n">
-        <v>0.04538186857368124</v>
+        <v>0.04406086815431393</v>
       </c>
       <c r="X21" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y21" t="n">
-        <v>50.44264001665625</v>
+        <v>48.97432787548009</v>
       </c>
       <c r="Z21" t="n">
         <v>0.8996727482680539</v>
@@ -2354,7 +2354,7 @@
         <v>43.3950199670746</v>
       </c>
       <c r="K22" t="n">
-        <v>6.155321981145334</v>
+        <v>6.12924010834387</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2370,7 +2370,7 @@
         <v>0.064523</v>
       </c>
       <c r="Q22" t="n">
-        <v>423</v>
+        <v>424.8</v>
       </c>
       <c r="R22" t="n">
         <v>162164.2</v>
@@ -2386,13 +2386,13 @@
         <v>40.74733935074209</v>
       </c>
       <c r="W22" t="n">
-        <v>0.1025886996857556</v>
+        <v>0.1021540018057312</v>
       </c>
       <c r="X22" t="n">
         <v>0.02454147966305898</v>
       </c>
       <c r="Y22" t="n">
-        <v>383.3669030732861</v>
+        <v>381.7424670433145</v>
       </c>
       <c r="Z22" t="n">
         <v>0.2675992602995889</v>
@@ -2534,7 +2534,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K24" t="n">
-        <v>5.220182675585511</v>
+        <v>4.966775749586214</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2550,7 +2550,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q24" t="n">
-        <v>470.4</v>
+        <v>494.4</v>
       </c>
       <c r="R24" t="n">
         <v>71002.60000000001</v>
@@ -2566,13 +2566,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W24" t="n">
-        <v>0.08700304459309186</v>
+        <v>0.08277959582643689</v>
       </c>
       <c r="X24" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y24" t="n">
-        <v>150.9409013605442</v>
+        <v>143.6136731391586</v>
       </c>
       <c r="Z24" t="n">
         <v>0.5764046975264343</v>
@@ -2624,7 +2624,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K25" t="n">
-        <v>7.134930826858408</v>
+        <v>6.710232563354932</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2640,7 +2640,7 @@
         <v>0.07520300000000001</v>
       </c>
       <c r="Q25" t="n">
-        <v>331.8</v>
+        <v>352.8</v>
       </c>
       <c r="R25" t="n">
         <v>88574</v>
@@ -2656,13 +2656,13 @@
         <v>12.61396912906789</v>
       </c>
       <c r="W25" t="n">
-        <v>0.1189155137809735</v>
+        <v>0.1118372093892489</v>
       </c>
       <c r="X25" t="n">
         <v>0.07927718783579227</v>
       </c>
       <c r="Y25" t="n">
-        <v>266.9499698613623</v>
+        <v>251.0600907029478</v>
       </c>
       <c r="Z25" t="n">
         <v>0.4454599258532639</v>
@@ -2796,7 +2796,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K27" t="n">
-        <v>6.199108729589235</v>
+        <v>5.273100786580055</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2812,7 +2812,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q27" t="n">
-        <v>369</v>
+        <v>433.8</v>
       </c>
       <c r="R27" t="n">
         <v>50011.7</v>
@@ -2828,13 +2828,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W27" t="n">
-        <v>0.1033184788264873</v>
+        <v>0.08788501310966759</v>
       </c>
       <c r="X27" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y27" t="n">
-        <v>135.5330623306233</v>
+        <v>115.287459658829</v>
       </c>
       <c r="Z27" t="n">
         <v>0.7623119927331765</v>
@@ -2886,7 +2886,7 @@
         <v>33.6762858057476</v>
       </c>
       <c r="K28" t="n">
-        <v>1.70168195077047</v>
+        <v>1.559809439821565</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2902,7 +2902,7 @@
         <v>0.143075</v>
       </c>
       <c r="Q28" t="n">
-        <v>1187.4</v>
+        <v>1295.4</v>
       </c>
       <c r="R28" t="n">
         <v>66783.2</v>
@@ -2918,13 +2918,13 @@
         <v>13.43904545346521</v>
       </c>
       <c r="W28" t="n">
-        <v>0.0283613658461745</v>
+        <v>0.02599682399702609</v>
       </c>
       <c r="X28" t="n">
         <v>0.07441004671519687</v>
       </c>
       <c r="Y28" t="n">
-        <v>56.24322048172478</v>
+        <v>51.5541145592095</v>
       </c>
       <c r="Z28" t="n">
         <v>0.5042628356494987</v>
@@ -3128,7 +3128,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K31" t="n">
-        <v>9.499916768037414</v>
+        <v>9.322679514902386</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3144,7 +3144,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q31" t="n">
-        <v>157.8</v>
+        <v>160.8</v>
       </c>
       <c r="R31" t="n">
         <v>34656</v>
@@ -3160,13 +3160,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W31" t="n">
-        <v>0.1583319461339569</v>
+        <v>0.1553779919150398</v>
       </c>
       <c r="X31" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y31" t="n">
-        <v>219.6197718631179</v>
+        <v>215.5223880597015</v>
       </c>
       <c r="Z31" t="n">
         <v>0.7209366660877885</v>
@@ -3218,7 +3218,7 @@
         <v>22.9279123422858</v>
       </c>
       <c r="K32" t="n">
-        <v>8.188540122244929</v>
+        <v>7.879007677761442</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3234,7 +3234,7 @@
         <v>0.037626</v>
       </c>
       <c r="Q32" t="n">
-        <v>168</v>
+        <v>174.6</v>
       </c>
       <c r="R32" t="n">
         <v>28366.1</v>
@@ -3250,13 +3250,13 @@
         <v>31.96610467696488</v>
       </c>
       <c r="W32" t="n">
-        <v>0.1364756687040821</v>
+        <v>0.1313167946293574</v>
       </c>
       <c r="X32" t="n">
         <v>0.0312831360000085</v>
       </c>
       <c r="Y32" t="n">
-        <v>168.8458333333333</v>
+        <v>162.463344788087</v>
       </c>
       <c r="Z32" t="n">
         <v>0.8082856769977473</v>
@@ -3308,7 +3308,7 @@
         <v>17.4754176089465</v>
       </c>
       <c r="K33" t="n">
-        <v>9.817650342104775</v>
+        <v>9.295434898375799</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -3324,7 +3324,7 @@
         <v>0.011457</v>
       </c>
       <c r="Q33" t="n">
-        <v>106.8</v>
+        <v>112.8</v>
       </c>
       <c r="R33" t="n">
         <v>13925.2</v>
@@ -3340,13 +3340,13 @@
         <v>83.3583805198696</v>
       </c>
       <c r="W33" t="n">
-        <v>0.1636275057017463</v>
+        <v>0.15492391497293</v>
       </c>
       <c r="X33" t="n">
         <v>0.0119963942888938</v>
       </c>
       <c r="Y33" t="n">
-        <v>130.3857677902622</v>
+        <v>123.4503546099291</v>
       </c>
       <c r="Z33" t="n">
         <v>1.254949128841704</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-16)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z33"/>
+  <dimension ref="A1:Z32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.335768984973386</v>
+        <v>4.405379954915619</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>797.4</v>
+        <v>784.8</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07226281641622311</v>
+        <v>0.07342299924859366</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>149.4431903686983</v>
+        <v>151.84250764526</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.580570886066457</v>
+        <v>3.660139127979046</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>938.4000000000001</v>
+        <v>918</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.05967618143444096</v>
+        <v>0.06100231879965076</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>210.390451832907</v>
+        <v>215.0657952069717</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.480017428705311</v>
+        <v>6.713111580817015</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>518.4000000000001</v>
+        <v>500.4</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1080002904784219</v>
+        <v>0.1118851930136169</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>126.6732253086419</v>
+        <v>131.2298161470823</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -922,7 +922,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K6" t="n">
-        <v>11.00270964727037</v>
+        <v>12.1228950185988</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -938,7 +938,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q6" t="n">
-        <v>292.2</v>
+        <v>265.2</v>
       </c>
       <c r="R6" t="n">
         <v>35584.1</v>
@@ -954,13 +954,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1833784941211729</v>
+        <v>0.20204825030998</v>
       </c>
       <c r="X6" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y6" t="n">
-        <v>121.7799452429843</v>
+        <v>134.1783559577677</v>
       </c>
       <c r="Z6" t="n">
         <v>1.505818497087371</v>
@@ -1012,7 +1012,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K7" t="n">
-        <v>4.655752701773577</v>
+        <v>4.525439012919865</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1028,7 +1028,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q7" t="n">
-        <v>687.6</v>
+        <v>707.4</v>
       </c>
       <c r="R7" t="n">
         <v>78110.8</v>
@@ -1044,13 +1044,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W7" t="n">
-        <v>0.07759587836289296</v>
+        <v>0.07542398354866441</v>
       </c>
       <c r="X7" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y7" t="n">
-        <v>113.5991855730076</v>
+        <v>110.4195646027707</v>
       </c>
       <c r="Z7" t="n">
         <v>0.6830672066132366</v>
@@ -1102,7 +1102,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K8" t="n">
-        <v>5.028663398288696</v>
+        <v>5.395868027778338</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1118,7 +1118,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q8" t="n">
-        <v>634.8</v>
+        <v>591.5999999999999</v>
       </c>
       <c r="R8" t="n">
         <v>60537.6</v>
@@ -1134,13 +1134,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W8" t="n">
-        <v>0.08381105663814493</v>
+        <v>0.08993113379630563</v>
       </c>
       <c r="X8" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y8" t="n">
-        <v>95.3648393194707</v>
+        <v>102.3286004056795</v>
       </c>
       <c r="Z8" t="n">
         <v>0.8788465144619939</v>
@@ -1192,7 +1192,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K9" t="n">
-        <v>5.325952416128715</v>
+        <v>6.384687199456121</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q9" t="n">
-        <v>593.4000000000001</v>
+        <v>495</v>
       </c>
       <c r="R9" t="n">
         <v>27205.5</v>
@@ -1224,13 +1224,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W9" t="n">
-        <v>0.08876587360214526</v>
+        <v>0.1064114533242687</v>
       </c>
       <c r="X9" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y9" t="n">
-        <v>45.84681496461071</v>
+        <v>54.96060606060606</v>
       </c>
       <c r="Z9" t="n">
         <v>1.936140464079432</v>
@@ -1364,7 +1364,7 @@
         <v>52.393894697293</v>
       </c>
       <c r="K11" t="n">
-        <v>8.880321135134405</v>
+        <v>11.00712073472542</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1380,7 +1380,7 @@
         <v>0.573611</v>
       </c>
       <c r="Q11" t="n">
-        <v>354</v>
+        <v>285.6</v>
       </c>
       <c r="R11" t="n">
         <v>54231.7</v>
@@ -1396,13 +1396,13 @@
         <v>1.645610026239954</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1480053522522401</v>
+        <v>0.1834520122454237</v>
       </c>
       <c r="X11" t="n">
         <v>0.6076773865342173</v>
       </c>
       <c r="Y11" t="n">
-        <v>153.1968926553672</v>
+        <v>189.8869047619048</v>
       </c>
       <c r="Z11" t="n">
         <v>0.9661119732055791</v>
@@ -1454,7 +1454,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K12" t="n">
-        <v>8.071853268240092</v>
+        <v>9.773568602775782</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1470,7 +1470,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q12" t="n">
-        <v>389.4</v>
+        <v>321.6</v>
       </c>
       <c r="R12" t="n">
         <v>16901.2</v>
@@ -1486,13 +1486,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W12" t="n">
-        <v>0.1345308878040015</v>
+        <v>0.162892810046263</v>
       </c>
       <c r="X12" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y12" t="n">
-        <v>43.40318438623523</v>
+        <v>52.55348258706468</v>
       </c>
       <c r="Z12" t="n">
         <v>3.099562617499243</v>
@@ -1544,7 +1544,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K13" t="n">
-        <v>6.585730256130571</v>
+        <v>7.340248149690083</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1560,7 +1560,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q13" t="n">
-        <v>472.8</v>
+        <v>424.2</v>
       </c>
       <c r="R13" t="n">
         <v>74809.60000000001</v>
@@ -1576,13 +1576,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1097621709355095</v>
+        <v>0.1223374691615014</v>
       </c>
       <c r="X13" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y13" t="n">
-        <v>158.2267343485618</v>
+        <v>176.3545497406884</v>
       </c>
       <c r="Z13" t="n">
         <v>0.6937018032218979</v>
@@ -1634,7 +1634,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K14" t="n">
-        <v>3.941692752939475</v>
+        <v>4.657076343320224</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1650,7 +1650,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q14" t="n">
-        <v>789</v>
+        <v>667.8000000000001</v>
       </c>
       <c r="R14" t="n">
         <v>38128.4</v>
@@ -1666,13 +1666,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W14" t="n">
-        <v>0.06569487921565792</v>
+        <v>0.07761793905533707</v>
       </c>
       <c r="X14" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y14" t="n">
-        <v>48.32496831432193</v>
+        <v>57.09553758610362</v>
       </c>
       <c r="Z14" t="n">
         <v>1.359439674918279</v>
@@ -1681,32 +1681,32 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>muse-spark-1-3</t>
+          <t>grok-4-7</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Muse Spark 1.3 (Max)</t>
+          <t>Grok 4.7 (Xhigh)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Muse Spark 1.3 (max)</t>
+          <t>Grok 4.7 (xhigh)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>SpaceXAI</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>xai</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1721,77 +1721,77 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>48.0923107719685</v>
+        <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>6.213476843923578</v>
+        <v>3.395215689344196</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>7.788</v>
+        <v>8.336827</v>
       </c>
       <c r="N15" t="n">
-        <v>7.532149</v>
+        <v>7.853459</v>
       </c>
       <c r="O15" t="n">
-        <v>0.110815</v>
+        <v>0.132106</v>
       </c>
       <c r="P15" t="n">
-        <v>0.145035</v>
+        <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>464.4</v>
+        <v>820.8</v>
       </c>
       <c r="R15" t="n">
-        <v>60200.2</v>
+        <v>80561.39999999999</v>
       </c>
       <c r="S15" t="n">
-        <v>26074.2</v>
+        <v>22017.7</v>
       </c>
       <c r="T15" t="n">
-        <v>34125.9</v>
+        <v>58543.6</v>
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="n">
-        <v>6.17518114688861</v>
+        <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.1035579473987263</v>
+        <v>0.0565869281557366</v>
       </c>
       <c r="X15" t="n">
-        <v>0.161938569284539</v>
+        <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>129.630060292851</v>
+        <v>98.14985380116958</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.7988729401558218</v>
+        <v>0.5765360412086756</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>grok-4-7</t>
+          <t>mimo-v2-6-pro</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Grok 4.7 (Xhigh)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Grok 4.7 (xhigh)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>SpaceXAI</t>
+          <t>Xiaomi</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>xai</t>
+          <t>xiaomi</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1808,85 +1808,85 @@
         <v>1</v>
       </c>
       <c r="I16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" t="n">
-        <v>46.4465506302286</v>
+        <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>2.725736539332665</v>
+        <v>2.34434243578129</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
-        <v>8.336827</v>
+        <v>2.466319</v>
       </c>
       <c r="N16" t="n">
-        <v>7.853459</v>
+        <v>2.410399</v>
       </c>
       <c r="O16" t="n">
-        <v>0.132106</v>
+        <v>0.023278</v>
       </c>
       <c r="P16" t="n">
-        <v>0.351262</v>
+        <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1022.4</v>
+        <v>1185.6</v>
       </c>
       <c r="R16" t="n">
-        <v>80561.39999999999</v>
+        <v>64275.7</v>
       </c>
       <c r="S16" t="n">
-        <v>22017.7</v>
+        <v>26756</v>
       </c>
       <c r="T16" t="n">
-        <v>58543.6</v>
+        <v>37519.7</v>
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="n">
-        <v>5.571250384616186</v>
+        <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.04542894232221107</v>
+        <v>0.03907237392968817</v>
       </c>
       <c r="X16" t="n">
-        <v>0.1794929200743312</v>
+        <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>78.79636150234741</v>
+        <v>54.21364709851551</v>
       </c>
       <c r="Z16" t="n">
-        <v>0.5765360412086756</v>
+        <v>0.7207110390246749</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>mimo-v2-6-pro</t>
+          <t>qwen3-8-max</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Xiaomi</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>xiaomi</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1898,85 +1898,85 @@
         <v>1</v>
       </c>
       <c r="I17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>46.3242065310383</v>
+        <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>2.065278935846558</v>
+        <v>1.273204611663922</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
-        <v>2.466319</v>
+        <v>26.154609</v>
       </c>
       <c r="N17" t="n">
-        <v>2.410399</v>
+        <v>25.508227</v>
       </c>
       <c r="O17" t="n">
-        <v>0.023278</v>
+        <v>0.221402</v>
       </c>
       <c r="P17" t="n">
-        <v>0.032642</v>
+        <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>1345.8</v>
+        <v>2140.2</v>
       </c>
       <c r="R17" t="n">
-        <v>64275.7</v>
+        <v>107730.2</v>
       </c>
       <c r="S17" t="n">
-        <v>26756</v>
+        <v>36900.3</v>
       </c>
       <c r="T17" t="n">
-        <v>37519.7</v>
+        <v>70829.89999999999</v>
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="n">
-        <v>18.78273107859863</v>
+        <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.03442131559744264</v>
+        <v>0.02122007686106537</v>
       </c>
       <c r="X17" t="n">
-        <v>0.05324039383918014</v>
+        <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>47.76021697131817</v>
+        <v>50.33651060648537</v>
       </c>
       <c r="Z17" t="n">
-        <v>0.7207110390246749</v>
+        <v>0.421564319921917</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>qwen3-8-max</t>
+          <t>glm-5-3</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>GLM-5.3 (Max)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1988,85 +1988,85 @@
         <v>1</v>
       </c>
       <c r="I18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" t="n">
-        <v>45.4152084980521</v>
+        <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>1.275708103877868</v>
+        <v>3.144479802360534</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
-        <v>26.154609</v>
+        <v>8.678356000000001</v>
       </c>
       <c r="N18" t="n">
-        <v>25.508227</v>
+        <v>8.365394999999999</v>
       </c>
       <c r="O18" t="n">
-        <v>0.221402</v>
+        <v>0.098552</v>
       </c>
       <c r="P18" t="n">
-        <v>0.424979</v>
+        <v>0.21441</v>
       </c>
       <c r="Q18" t="n">
-        <v>2136</v>
+        <v>854.4</v>
       </c>
       <c r="R18" t="n">
-        <v>107730.2</v>
+        <v>71127.60000000001</v>
       </c>
       <c r="S18" t="n">
-        <v>36900.3</v>
+        <v>22398.1</v>
       </c>
       <c r="T18" t="n">
-        <v>70829.89999999999</v>
+        <v>48729.5</v>
       </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="n">
-        <v>1.736413207249709</v>
+        <v>5.159663003639629</v>
       </c>
       <c r="W18" t="n">
-        <v>0.0212618017312978</v>
+        <v>0.0524079967060089</v>
       </c>
       <c r="X18" t="n">
-        <v>0.5758997891889408</v>
+        <v>0.1938111072941391</v>
       </c>
       <c r="Y18" t="n">
-        <v>50.43548689138576</v>
+        <v>83.24859550561798</v>
       </c>
       <c r="Z18" t="n">
-        <v>0.421564319921917</v>
+        <v>0.629536106737947</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>glm-5-3</t>
+          <t>step-5</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>GLM-5.3 (Max)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>StepFun</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>stepfun</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2081,82 +2081,82 @@
         <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>44.777392385614</v>
+        <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>3.196102240229408</v>
+        <v>4.471810318421412</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
-        <v>8.678356000000001</v>
+        <v>6.586908</v>
       </c>
       <c r="N19" t="n">
-        <v>8.365394999999999</v>
+        <v>6.413718</v>
       </c>
       <c r="O19" t="n">
-        <v>0.098552</v>
+        <v>0.055881</v>
       </c>
       <c r="P19" t="n">
-        <v>0.21441</v>
+        <v>0.117309</v>
       </c>
       <c r="Q19" t="n">
-        <v>840.6</v>
+        <v>586.8</v>
       </c>
       <c r="R19" t="n">
-        <v>71127.60000000001</v>
+        <v>64144.3</v>
       </c>
       <c r="S19" t="n">
-        <v>22398.1</v>
+        <v>20696.6</v>
       </c>
       <c r="T19" t="n">
-        <v>48729.5</v>
+        <v>43447.7</v>
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="n">
-        <v>5.159663003639629</v>
+        <v>6.639580348497565</v>
       </c>
       <c r="W19" t="n">
-        <v>0.05326837067049012</v>
+        <v>0.07453017197369019</v>
       </c>
       <c r="X19" t="n">
-        <v>0.1938111072941391</v>
+        <v>0.1506119283918727</v>
       </c>
       <c r="Y19" t="n">
-        <v>84.61527480371164</v>
+        <v>109.3120313565099</v>
       </c>
       <c r="Z19" t="n">
-        <v>0.629536106737947</v>
+        <v>0.6818112429968274</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>step-5</t>
+          <t>kimi-k3</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>Kimi K3 (Max)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>Kimi K3 (max)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>StepFun</t>
+          <t>Kimi</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>stepfun</t>
+          <t>kimi</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2168,265 +2168,265 @@
         <v>1</v>
       </c>
       <c r="I20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20" t="n">
-        <v>43.7343049141614</v>
+        <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>4.258452279859922</v>
+        <v>2.613538546275672</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
-        <v>6.586908</v>
+        <v>9.216749</v>
       </c>
       <c r="N20" t="n">
-        <v>6.413718</v>
+        <v>8.489921000000001</v>
       </c>
       <c r="O20" t="n">
-        <v>0.055881</v>
+        <v>0.240032</v>
       </c>
       <c r="P20" t="n">
-        <v>0.117309</v>
+        <v>0.486797</v>
       </c>
       <c r="Q20" t="n">
-        <v>616.1999999999999</v>
+        <v>1000.8</v>
       </c>
       <c r="R20" t="n">
-        <v>64144.3</v>
+        <v>48455.2</v>
       </c>
       <c r="S20" t="n">
-        <v>20696.6</v>
+        <v>16002.1</v>
       </c>
       <c r="T20" t="n">
-        <v>43447.7</v>
+        <v>32453.1</v>
       </c>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="n">
-        <v>6.639580348497565</v>
+        <v>4.72984812235618</v>
       </c>
       <c r="W20" t="n">
-        <v>0.07097420466433205</v>
+        <v>0.04355897577126119</v>
       </c>
       <c r="X20" t="n">
-        <v>0.1506119283918727</v>
+        <v>0.2114232791690251</v>
       </c>
       <c r="Y20" t="n">
-        <v>104.0965595585849</v>
+        <v>48.41646682653877</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.6818112429968274</v>
+        <v>0.8996727482680539</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>kimi-k3</t>
+          <t>claude-haiku-5-5</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Kimi K3 (Max)</t>
+          <t>Claude Haiku 5.5 (Max)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Kimi K3 (max)</t>
+          <t>Claude Haiku 5.5 (max)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Kimi</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>kimi</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H21" t="b">
         <v>1</v>
       </c>
       <c r="I21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>43.5938229518782</v>
+        <v>43.3950199670746</v>
       </c>
       <c r="K21" t="n">
-        <v>2.643652089258836</v>
+        <v>6.103378335734824</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
-        <v>9.216749</v>
+        <v>1.064978</v>
       </c>
       <c r="N21" t="n">
-        <v>8.489921000000001</v>
+        <v>0.983896</v>
       </c>
       <c r="O21" t="n">
-        <v>0.240032</v>
+        <v>0.016559</v>
       </c>
       <c r="P21" t="n">
-        <v>0.486797</v>
+        <v>0.064523</v>
       </c>
       <c r="Q21" t="n">
-        <v>989.3999999999999</v>
+        <v>426.6</v>
       </c>
       <c r="R21" t="n">
-        <v>48455.2</v>
+        <v>162164.2</v>
       </c>
       <c r="S21" t="n">
-        <v>16002.1</v>
+        <v>33117.6</v>
       </c>
       <c r="T21" t="n">
-        <v>32453.1</v>
+        <v>129046.6</v>
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="n">
-        <v>4.72984812235618</v>
+        <v>40.74733935074209</v>
       </c>
       <c r="W21" t="n">
-        <v>0.04406086815431393</v>
+        <v>0.1017229722622471</v>
       </c>
       <c r="X21" t="n">
-        <v>0.2114232791690251</v>
+        <v>0.02454147966305898</v>
       </c>
       <c r="Y21" t="n">
-        <v>48.97432787548009</v>
+        <v>380.131739334271</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.8996727482680539</v>
+        <v>0.2675992602995889</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>claude-haiku-5-5</t>
+          <t>glm-5-3-flash</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Claude Haiku 5.5 (Max)</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Claude Haiku 5.5 (max)</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H22" t="b">
         <v>1</v>
       </c>
       <c r="I22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>43.3950199670746</v>
+        <v>41.807466113455</v>
       </c>
       <c r="K22" t="n">
-        <v>6.12924010834387</v>
+        <v>3.543005602835169</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
-        <v>1.064978</v>
+        <v>1.193653</v>
       </c>
       <c r="N22" t="n">
-        <v>0.983896</v>
+        <v>1.159316</v>
       </c>
       <c r="O22" t="n">
-        <v>0.016559</v>
+        <v>0.011012</v>
       </c>
       <c r="P22" t="n">
-        <v>0.064523</v>
+        <v>0.023325</v>
       </c>
       <c r="Q22" t="n">
-        <v>424.8</v>
+        <v>708</v>
       </c>
       <c r="R22" t="n">
-        <v>162164.2</v>
+        <v>68673.2</v>
       </c>
       <c r="S22" t="n">
-        <v>33117.6</v>
+        <v>22023.7</v>
       </c>
       <c r="T22" t="n">
-        <v>129046.6</v>
+        <v>46649.5</v>
       </c>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="n">
-        <v>40.74733935074209</v>
+        <v>35.02480713696107</v>
       </c>
       <c r="W22" t="n">
-        <v>0.1021540018057312</v>
+        <v>0.05905009338058616</v>
       </c>
       <c r="X22" t="n">
-        <v>0.02454147966305898</v>
+        <v>0.02855119219042658</v>
       </c>
       <c r="Y22" t="n">
-        <v>381.7424670433145</v>
+        <v>96.9960451977401</v>
       </c>
       <c r="Z22" t="n">
-        <v>0.2675992602995889</v>
+        <v>0.6087886703030441</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>glm-5-3-flash</t>
+          <t>gemini-3-8-flash</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Gemini 3.8 Flash (High)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Gemini 3.8 Flash (high)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2438,85 +2438,85 @@
         <v>1</v>
       </c>
       <c r="I23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>41.807466113455</v>
+        <v>40.9262321765904</v>
       </c>
       <c r="K23" t="n">
-        <v>3.188975294695271</v>
+        <v>5.180535718555747</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
-        <v>1.193653</v>
+        <v>4.90102</v>
       </c>
       <c r="N23" t="n">
-        <v>1.159316</v>
+        <v>4.63476</v>
       </c>
       <c r="O23" t="n">
-        <v>0.011012</v>
+        <v>0.106033</v>
       </c>
       <c r="P23" t="n">
-        <v>0.023325</v>
+        <v>0.160227</v>
       </c>
       <c r="Q23" t="n">
-        <v>786.5999999999999</v>
+        <v>474</v>
       </c>
       <c r="R23" t="n">
-        <v>68673.2</v>
+        <v>71002.60000000001</v>
       </c>
       <c r="S23" t="n">
-        <v>22023.7</v>
+        <v>28275.4</v>
       </c>
       <c r="T23" t="n">
-        <v>46649.5</v>
+        <v>42727.1</v>
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="n">
-        <v>35.02480713696107</v>
+        <v>8.350554002348574</v>
       </c>
       <c r="W23" t="n">
-        <v>0.05314958824492119</v>
+        <v>0.08634226197592912</v>
       </c>
       <c r="X23" t="n">
-        <v>0.02855119219042658</v>
+        <v>0.119752533750306</v>
       </c>
       <c r="Y23" t="n">
-        <v>87.30383930841597</v>
+        <v>149.7945147679325</v>
       </c>
       <c r="Z23" t="n">
-        <v>0.6087886703030441</v>
+        <v>0.5764046975264343</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>gemini-3-8-flash</t>
+          <t>deepseek-v4-1-flash</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (High)</t>
+          <t>DeepSeek V4.1 Flash (Max)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>DeepSeek V4.1 Flash (max)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>DeepSeek</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>deepseek</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2528,85 +2528,85 @@
         <v>1</v>
       </c>
       <c r="I24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>40.9262321765904</v>
+        <v>39.456167472527</v>
       </c>
       <c r="K24" t="n">
-        <v>4.966775749586214</v>
+        <v>6.698839978357725</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>4.90102</v>
+        <v>3.127974</v>
       </c>
       <c r="N24" t="n">
-        <v>4.63476</v>
+        <v>3.021685</v>
       </c>
       <c r="O24" t="n">
-        <v>0.106033</v>
+        <v>0.031085</v>
       </c>
       <c r="P24" t="n">
-        <v>0.160227</v>
+        <v>0.07520300000000001</v>
       </c>
       <c r="Q24" t="n">
-        <v>494.4</v>
+        <v>353.4</v>
       </c>
       <c r="R24" t="n">
-        <v>71002.60000000001</v>
+        <v>88574</v>
       </c>
       <c r="S24" t="n">
-        <v>28275.4</v>
+        <v>25904.4</v>
       </c>
       <c r="T24" t="n">
-        <v>42727.1</v>
+        <v>62669.6</v>
       </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="n">
-        <v>8.350554002348574</v>
+        <v>12.61396912906789</v>
       </c>
       <c r="W24" t="n">
-        <v>0.08277959582643689</v>
+        <v>0.1116473329726288</v>
       </c>
       <c r="X24" t="n">
-        <v>0.119752533750306</v>
+        <v>0.07927718783579227</v>
       </c>
       <c r="Y24" t="n">
-        <v>143.6136731391586</v>
+        <v>250.6338426711941</v>
       </c>
       <c r="Z24" t="n">
-        <v>0.5764046975264343</v>
+        <v>0.4454599258532639</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>deepseek-v4-1-flash</t>
+          <t>muse-spark-open</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (Max)</t>
+          <t>Muse Spark Open (Xhigh)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (max)</t>
+          <t>Muse Spark Open (xhigh)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>DeepSeek</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>deepseek</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2621,51 +2621,51 @@
         <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>39.456167472527</v>
+        <v>38.8666662997805</v>
       </c>
       <c r="K25" t="n">
-        <v>6.710232563354932</v>
+        <v>5.933842183172596</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
-        <v>3.127974</v>
+        <v>3.765796</v>
       </c>
       <c r="N25" t="n">
-        <v>3.021685</v>
+        <v>3.594372</v>
       </c>
       <c r="O25" t="n">
-        <v>0.031085</v>
+        <v>0.093234</v>
       </c>
       <c r="P25" t="n">
-        <v>0.07520300000000001</v>
+        <v>0.07819</v>
       </c>
       <c r="Q25" t="n">
-        <v>352.8</v>
+        <v>393</v>
       </c>
       <c r="R25" t="n">
-        <v>88574</v>
+        <v>40335.1</v>
       </c>
       <c r="S25" t="n">
-        <v>25904.4</v>
+        <v>21937.3</v>
       </c>
       <c r="T25" t="n">
-        <v>62669.6</v>
+        <v>18397.7</v>
       </c>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="n">
-        <v>12.61396912906789</v>
+        <v>10.3209696700991</v>
       </c>
       <c r="W25" t="n">
-        <v>0.1118372093892489</v>
+        <v>0.09889736971954326</v>
       </c>
       <c r="X25" t="n">
-        <v>0.07927718783579227</v>
+        <v>0.09689012098321557</v>
       </c>
       <c r="Y25" t="n">
-        <v>251.0600907029478</v>
+        <v>102.6338422391858</v>
       </c>
       <c r="Z25" t="n">
-        <v>0.4454599258532639</v>
+        <v>0.9635941475236333</v>
       </c>
     </row>
     <row r="26">
@@ -2796,7 +2796,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K27" t="n">
-        <v>5.273100786580055</v>
+        <v>5.614803930334875</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2812,7 +2812,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q27" t="n">
-        <v>433.8</v>
+        <v>407.4</v>
       </c>
       <c r="R27" t="n">
         <v>50011.7</v>
@@ -2828,13 +2828,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W27" t="n">
-        <v>0.08788501310966759</v>
+        <v>0.09358006550558125</v>
       </c>
       <c r="X27" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y27" t="n">
-        <v>115.287459658829</v>
+        <v>122.7582228767796</v>
       </c>
       <c r="Z27" t="n">
         <v>0.7623119927331765</v>
@@ -2886,7 +2886,7 @@
         <v>33.6762858057476</v>
       </c>
       <c r="K28" t="n">
-        <v>1.559809439821565</v>
+        <v>1.632393882973708</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2902,7 +2902,7 @@
         <v>0.143075</v>
       </c>
       <c r="Q28" t="n">
-        <v>1295.4</v>
+        <v>1237.8</v>
       </c>
       <c r="R28" t="n">
         <v>66783.2</v>
@@ -2918,13 +2918,13 @@
         <v>13.43904545346521</v>
       </c>
       <c r="W28" t="n">
-        <v>0.02599682399702609</v>
+        <v>0.02720656471622847</v>
       </c>
       <c r="X28" t="n">
         <v>0.07441004671519687</v>
       </c>
       <c r="Y28" t="n">
-        <v>51.5541145592095</v>
+        <v>53.95314267248344</v>
       </c>
       <c r="Z28" t="n">
         <v>0.5042628356494987</v>
@@ -3038,7 +3038,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K30" t="n">
-        <v>3.491074459215245</v>
+        <v>3.421580002767167</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3054,7 +3054,7 @@
         <v>0.026182</v>
       </c>
       <c r="Q30" t="n">
-        <v>502.1999999999999</v>
+        <v>512.4</v>
       </c>
       <c r="R30" t="n">
         <v>48192</v>
@@ -3070,13 +3070,13 @@
         <v>15.27539782478406</v>
       </c>
       <c r="W30" t="n">
-        <v>0.05818457432025409</v>
+        <v>0.05702633337945277</v>
       </c>
       <c r="X30" t="n">
         <v>0.06546474346988973</v>
       </c>
       <c r="Y30" t="n">
-        <v>95.96176821983275</v>
+        <v>94.05152224824356</v>
       </c>
       <c r="Z30" t="n">
         <v>0.6063307856829266</v>
@@ -3085,37 +3085,37 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>inkling</t>
+          <t>nemotron-3-5-super-vl</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Inkling (Xhigh)</t>
+          <t>Nemotron 3.5 Super VL</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Inkling (xhigh)</t>
+          <t>Nemotron 3.5 Super VL</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Thinking Machines</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>thinking-machines</t>
+          <t>nvidia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H31" t="b">
@@ -3125,82 +3125,82 @@
         <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>24.9847810999384</v>
+        <v>26.4910658661689</v>
       </c>
       <c r="K31" t="n">
-        <v>9.322679514902386</v>
+        <v>8.330523857285817</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
-        <v>2.418996</v>
+        <v>0.373143</v>
       </c>
       <c r="N31" t="n">
-        <v>2.278639</v>
+        <v>0.344869</v>
       </c>
       <c r="O31" t="n">
-        <v>0.04559</v>
+        <v>0.007806</v>
       </c>
       <c r="P31" t="n">
-        <v>0.094767</v>
+        <v>0.020469</v>
       </c>
       <c r="Q31" t="n">
-        <v>160.8</v>
+        <v>190.8</v>
       </c>
       <c r="R31" t="n">
-        <v>34656</v>
+        <v>49173.8</v>
       </c>
       <c r="S31" t="n">
-        <v>11256.8</v>
+        <v>13575.6</v>
       </c>
       <c r="T31" t="n">
-        <v>23399.2</v>
+        <v>35598.3</v>
       </c>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="n">
-        <v>10.32857478885389</v>
+        <v>70.994406611323</v>
       </c>
       <c r="W31" t="n">
-        <v>0.1553779919150398</v>
+        <v>0.138842064288097</v>
       </c>
       <c r="X31" t="n">
-        <v>0.09681877901287532</v>
+        <v>0.01408561670885927</v>
       </c>
       <c r="Y31" t="n">
-        <v>215.5223880597015</v>
+        <v>257.7243186582809</v>
       </c>
       <c r="Z31" t="n">
-        <v>0.7209366660877885</v>
+        <v>0.5387231791354116</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
+          <t>inkling</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
+          <t>Inkling (Xhigh)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra</t>
+          <t>Inkling (xhigh)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Thinking Machines</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>thinking-machines</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3215,141 +3215,51 @@
         <v>1</v>
       </c>
       <c r="J32" t="n">
-        <v>22.9279123422858</v>
+        <v>24.9847810999384</v>
       </c>
       <c r="K32" t="n">
-        <v>7.879007677761442</v>
+        <v>9.759680117163438</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
-        <v>0.717257</v>
+        <v>2.418996</v>
       </c>
       <c r="N32" t="n">
-        <v>0.646342</v>
+        <v>2.278639</v>
       </c>
       <c r="O32" t="n">
-        <v>0.03329</v>
+        <v>0.04559</v>
       </c>
       <c r="P32" t="n">
-        <v>0.037626</v>
+        <v>0.094767</v>
       </c>
       <c r="Q32" t="n">
-        <v>174.6</v>
+        <v>153.6</v>
       </c>
       <c r="R32" t="n">
-        <v>28366.1</v>
+        <v>34656</v>
       </c>
       <c r="S32" t="n">
-        <v>13315.8</v>
+        <v>11256.8</v>
       </c>
       <c r="T32" t="n">
-        <v>15050.3</v>
+        <v>23399.2</v>
       </c>
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="n">
-        <v>31.96610467696488</v>
+        <v>10.32857478885389</v>
       </c>
       <c r="W32" t="n">
-        <v>0.1313167946293574</v>
+        <v>0.1626613352860573</v>
       </c>
       <c r="X32" t="n">
-        <v>0.0312831360000085</v>
+        <v>0.09681877901287532</v>
       </c>
       <c r="Y32" t="n">
-        <v>162.463344788087</v>
+        <v>225.625</v>
       </c>
       <c r="Z32" t="n">
-        <v>0.8082856769977473</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>muse-glimmer</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Muse Glimmer (High)</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Muse Glimmer (high)</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Meta</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>meta</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>small</t>
-        </is>
-      </c>
-      <c r="H33" t="b">
-        <v>1</v>
-      </c>
-      <c r="I33" t="b">
-        <v>1</v>
-      </c>
-      <c r="J33" t="n">
-        <v>17.4754176089465</v>
-      </c>
-      <c r="K33" t="n">
-        <v>9.295434898375799</v>
-      </c>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="n">
-        <v>0.209642</v>
-      </c>
-      <c r="N33" t="n">
-        <v>0.192931</v>
-      </c>
-      <c r="O33" t="n">
-        <v>0.005253</v>
-      </c>
-      <c r="P33" t="n">
-        <v>0.011457</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>112.8</v>
-      </c>
-      <c r="R33" t="n">
-        <v>13925.2</v>
-      </c>
-      <c r="S33" t="n">
-        <v>4377.3</v>
-      </c>
-      <c r="T33" t="n">
-        <v>9547.9</v>
-      </c>
-      <c r="U33" t="inlineStr"/>
-      <c r="V33" t="n">
-        <v>83.3583805198696</v>
-      </c>
-      <c r="W33" t="n">
-        <v>0.15492391497293</v>
-      </c>
-      <c r="X33" t="n">
-        <v>0.0119963942888938</v>
-      </c>
-      <c r="Y33" t="n">
-        <v>123.4503546099291</v>
-      </c>
-      <c r="Z33" t="n">
-        <v>1.254949128841704</v>
+        <v>0.7209366660877885</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-17)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.415507265156804</v>
+        <v>4.408750559318768</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>783</v>
+        <v>784.2</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07359178775261341</v>
+        <v>0.07347917598864613</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>152.1915708812261</v>
+        <v>151.9586840091813</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.730854674089234</v>
+        <v>3.718468038385086</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>900.6</v>
+        <v>903.6</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.06218091123482056</v>
+        <v>0.0619744673064181</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>219.2209638019098</v>
+        <v>218.4931385568836</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -1012,7 +1012,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K7" t="n">
-        <v>4.525439012919865</v>
+        <v>4.476084392812517</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1028,7 +1028,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q7" t="n">
-        <v>707.4</v>
+        <v>715.2</v>
       </c>
       <c r="R7" t="n">
         <v>78110.8</v>
@@ -1044,13 +1044,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W7" t="n">
-        <v>0.07542398354866441</v>
+        <v>0.07460140654687528</v>
       </c>
       <c r="X7" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y7" t="n">
-        <v>110.4195646027707</v>
+        <v>109.2153243847875</v>
       </c>
       <c r="Z7" t="n">
         <v>0.6830672066132366</v>
@@ -1192,7 +1192,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K9" t="n">
-        <v>6.519018489543688</v>
+        <v>6.692969427638246</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q9" t="n">
-        <v>484.8</v>
+        <v>472.2</v>
       </c>
       <c r="R9" t="n">
         <v>27205.5</v>
@@ -1224,13 +1224,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1086503081590615</v>
+        <v>0.1115494904606374</v>
       </c>
       <c r="X9" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y9" t="n">
-        <v>56.11695544554455</v>
+        <v>57.6143583227446</v>
       </c>
       <c r="Z9" t="n">
         <v>1.936140464079432</v>
@@ -1281,9 +1281,7 @@
       <c r="J10" t="n">
         <v>52.5605655745982</v>
       </c>
-      <c r="K10" t="n">
-        <v>4.977326285473314</v>
-      </c>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
         <v>8.057855999999999</v>
@@ -1297,9 +1295,7 @@
       <c r="P10" t="n">
         <v>0.355464</v>
       </c>
-      <c r="Q10" t="n">
-        <v>633.6</v>
-      </c>
+      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="n">
         <v>61557.6</v>
       </c>
@@ -1313,15 +1309,11 @@
       <c r="V10" t="n">
         <v>6.522897104961693</v>
       </c>
-      <c r="W10" t="n">
-        <v>0.08295543809122191</v>
-      </c>
+      <c r="W10" t="inlineStr"/>
       <c r="X10" t="n">
         <v>0.1533061128987214</v>
       </c>
-      <c r="Y10" t="n">
-        <v>97.15530303030303</v>
-      </c>
+      <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="n">
         <v>0.8538436452135594</v>
       </c>
@@ -1462,7 +1454,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K12" t="n">
-        <v>9.997390784518739</v>
+        <v>10.15238909125546</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1478,7 +1470,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q12" t="n">
-        <v>314.4</v>
+        <v>309.6</v>
       </c>
       <c r="R12" t="n">
         <v>16901.2</v>
@@ -1494,13 +1486,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W12" t="n">
-        <v>0.166623179741979</v>
+        <v>0.1692064848542577</v>
       </c>
       <c r="X12" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y12" t="n">
-        <v>53.75699745547073</v>
+        <v>54.59043927648579</v>
       </c>
       <c r="Z12" t="n">
         <v>3.099562617499243</v>
@@ -1552,7 +1544,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K13" t="n">
-        <v>7.06061964874951</v>
+        <v>7.258119499064181</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1568,7 +1560,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q13" t="n">
-        <v>441</v>
+        <v>429</v>
       </c>
       <c r="R13" t="n">
         <v>74809.60000000001</v>
@@ -1584,13 +1576,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1176769941458252</v>
+        <v>0.1209686583177364</v>
       </c>
       <c r="X13" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y13" t="n">
-        <v>169.6362811791383</v>
+        <v>174.381351981352</v>
       </c>
       <c r="Z13" t="n">
         <v>0.6937018032218979</v>
@@ -1642,7 +1634,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K14" t="n">
-        <v>5.214613652027576</v>
+        <v>5.299924304821483</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1658,7 +1650,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q14" t="n">
-        <v>596.4</v>
+        <v>586.8</v>
       </c>
       <c r="R14" t="n">
         <v>38128.4</v>
@@ -1674,13 +1666,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W14" t="n">
-        <v>0.08691022753379292</v>
+        <v>0.08833207174702472</v>
       </c>
       <c r="X14" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y14" t="n">
-        <v>63.93091884641181</v>
+        <v>64.9768234492161</v>
       </c>
       <c r="Z14" t="n">
         <v>1.359439674918279</v>
@@ -1822,7 +1814,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>2.244389851309995</v>
+        <v>2.266350613064496</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1838,7 +1830,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1238.4</v>
+        <v>1226.4</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1854,13 +1846,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.03740649752183325</v>
+        <v>0.0377725102177416</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>51.90221253229974</v>
+        <v>52.41006196999347</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1912,7 +1904,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.281467508410048</v>
+        <v>1.265047590474989</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1928,7 +1920,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2126.4</v>
+        <v>2154</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1944,13 +1936,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.02135779180683414</v>
+        <v>0.02108412650791648</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>50.66318660647104</v>
+        <v>50.01402042711235</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -2002,7 +1994,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>3.379425840423698</v>
+        <v>3.473808563662839</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2018,7 +2010,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q18" t="n">
-        <v>795</v>
+        <v>773.4000000000001</v>
       </c>
       <c r="R18" t="n">
         <v>71127.60000000001</v>
@@ -2034,13 +2026,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W18" t="n">
-        <v>0.05632376400706163</v>
+        <v>0.05789680939438065</v>
       </c>
       <c r="X18" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y18" t="n">
-        <v>89.46867924528303</v>
+        <v>91.96741660201707</v>
       </c>
       <c r="Z18" t="n">
         <v>0.629536106737947</v>
@@ -2182,7 +2174,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>2.515511999531345</v>
+        <v>2.442230977696258</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2198,7 +2190,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q20" t="n">
-        <v>1039.8</v>
+        <v>1071</v>
       </c>
       <c r="R20" t="n">
         <v>48455.2</v>
@@ -2214,13 +2206,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W20" t="n">
-        <v>0.04192519999218908</v>
+        <v>0.04070384962827096</v>
       </c>
       <c r="X20" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y20" t="n">
-        <v>46.60050009617234</v>
+        <v>45.24295051353874</v>
       </c>
       <c r="Z20" t="n">
         <v>0.8996727482680539</v>
@@ -2272,7 +2264,7 @@
         <v>43.3950199670746</v>
       </c>
       <c r="K21" t="n">
-        <v>6.094806175150928</v>
+        <v>6.069233561828615</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2288,7 +2280,7 @@
         <v>0.064523</v>
       </c>
       <c r="Q21" t="n">
-        <v>427.2</v>
+        <v>429</v>
       </c>
       <c r="R21" t="n">
         <v>162164.2</v>
@@ -2304,13 +2296,13 @@
         <v>40.74733935074209</v>
       </c>
       <c r="W21" t="n">
-        <v>0.1015801029191821</v>
+        <v>0.1011538926971436</v>
       </c>
       <c r="X21" t="n">
         <v>0.02454147966305898</v>
       </c>
       <c r="Y21" t="n">
-        <v>379.5978464419476</v>
+        <v>378.0051282051282</v>
       </c>
       <c r="Z21" t="n">
         <v>0.2675992602995889</v>
@@ -2362,7 +2354,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K22" t="n">
-        <v>3.543005602835169</v>
+        <v>3.44377809830766</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2378,7 +2370,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q22" t="n">
-        <v>708</v>
+        <v>728.4000000000001</v>
       </c>
       <c r="R22" t="n">
         <v>68673.2</v>
@@ -2394,13 +2386,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W22" t="n">
-        <v>0.05905009338058616</v>
+        <v>0.057396301638461</v>
       </c>
       <c r="X22" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y22" t="n">
-        <v>96.9960451977401</v>
+        <v>94.27951674903898</v>
       </c>
       <c r="Z22" t="n">
         <v>0.6087886703030441</v>
@@ -2542,7 +2534,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K24" t="n">
-        <v>6.698839978357725</v>
+        <v>6.543311355311277</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2558,7 +2550,7 @@
         <v>0.07520300000000001</v>
       </c>
       <c r="Q24" t="n">
-        <v>353.4</v>
+        <v>361.8</v>
       </c>
       <c r="R24" t="n">
         <v>88574</v>
@@ -2574,13 +2566,13 @@
         <v>12.61396912906789</v>
       </c>
       <c r="W24" t="n">
-        <v>0.1116473329726288</v>
+        <v>0.109055189255188</v>
       </c>
       <c r="X24" t="n">
         <v>0.07927718783579227</v>
       </c>
       <c r="Y24" t="n">
-        <v>250.6338426711941</v>
+        <v>244.8148148148148</v>
       </c>
       <c r="Z24" t="n">
         <v>0.4454599258532639</v>
@@ -2632,7 +2624,7 @@
         <v>38.8666662997805</v>
       </c>
       <c r="K25" t="n">
-        <v>7.028330253124864</v>
+        <v>7.546925495103009</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2648,7 +2640,7 @@
         <v>0.07819</v>
       </c>
       <c r="Q25" t="n">
-        <v>331.8</v>
+        <v>309</v>
       </c>
       <c r="R25" t="n">
         <v>40335.1</v>
@@ -2664,13 +2656,13 @@
         <v>10.3209696700991</v>
       </c>
       <c r="W25" t="n">
-        <v>0.1171388375520811</v>
+        <v>0.1257820915850502</v>
       </c>
       <c r="X25" t="n">
         <v>0.09689012098321557</v>
       </c>
       <c r="Y25" t="n">
-        <v>121.5644966847498</v>
+        <v>130.5343042071197</v>
       </c>
       <c r="Z25" t="n">
         <v>0.9635941475236333</v>
@@ -2722,7 +2714,7 @@
         <v>38.3770408917494</v>
       </c>
       <c r="K26" t="n">
-        <v>3.195423887739334</v>
+        <v>3.137942836610744</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2738,7 +2730,7 @@
         <v>0.217751</v>
       </c>
       <c r="Q26" t="n">
-        <v>720.6</v>
+        <v>733.8000000000001</v>
       </c>
       <c r="R26" t="n">
         <v>69464</v>
@@ -2754,13 +2746,13 @@
         <v>6.245463169309107</v>
       </c>
       <c r="W26" t="n">
-        <v>0.05325706479565557</v>
+        <v>0.05229904727684574</v>
       </c>
       <c r="X26" t="n">
         <v>0.1601162272342122</v>
       </c>
       <c r="Y26" t="n">
-        <v>96.39744657230085</v>
+        <v>94.66339602071409</v>
       </c>
       <c r="Z26" t="n">
         <v>0.5524738122156715</v>
@@ -2812,7 +2804,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K27" t="n">
-        <v>5.65645677848276</v>
+        <v>5.430843117802536</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2828,7 +2820,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q27" t="n">
-        <v>404.4</v>
+        <v>421.2</v>
       </c>
       <c r="R27" t="n">
         <v>50011.7</v>
@@ -2844,13 +2836,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W27" t="n">
-        <v>0.09427427964137933</v>
+        <v>0.0905140519633756</v>
       </c>
       <c r="X27" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y27" t="n">
-        <v>123.6688921859545</v>
+        <v>118.7362298195631</v>
       </c>
       <c r="Z27" t="n">
         <v>0.7623119927331765</v>
@@ -2902,7 +2894,7 @@
         <v>33.6762858057476</v>
       </c>
       <c r="K28" t="n">
-        <v>1.626873710422589</v>
+        <v>1.599823553717225</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2918,7 +2910,7 @@
         <v>0.143075</v>
       </c>
       <c r="Q28" t="n">
-        <v>1242</v>
+        <v>1263</v>
       </c>
       <c r="R28" t="n">
         <v>66783.2</v>
@@ -2934,13 +2926,13 @@
         <v>13.43904545346521</v>
       </c>
       <c r="W28" t="n">
-        <v>0.02711456184037649</v>
+        <v>0.02666372589528709</v>
       </c>
       <c r="X28" t="n">
         <v>0.07441004671519687</v>
       </c>
       <c r="Y28" t="n">
-        <v>53.770692431562</v>
+        <v>52.87664291369754</v>
       </c>
       <c r="Z28" t="n">
         <v>0.5042628356494987</v>
@@ -3053,22 +3045,50 @@
       <c r="J30" t="n">
         <v>30.3334426348039</v>
       </c>
-      <c r="K30" t="inlineStr"/>
+      <c r="K30" t="n">
+        <v>21.82262060057835</v>
+      </c>
       <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr"/>
+      <c r="M30" t="n">
+        <v>1.326119</v>
+      </c>
+      <c r="N30" t="n">
+        <v>1.270857</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0.014358</v>
+      </c>
+      <c r="P30" t="n">
+        <v>0.040904</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>83.39999999999999</v>
+      </c>
+      <c r="R30" t="n">
+        <v>26315</v>
+      </c>
+      <c r="S30" t="n">
+        <v>6837.1</v>
+      </c>
+      <c r="T30" t="n">
+        <v>19478</v>
+      </c>
       <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
-      <c r="X30" t="inlineStr"/>
-      <c r="Y30" t="inlineStr"/>
-      <c r="Z30" t="inlineStr"/>
+      <c r="V30" t="n">
+        <v>22.87384664182015</v>
+      </c>
+      <c r="W30" t="n">
+        <v>0.3637103433429725</v>
+      </c>
+      <c r="X30" t="n">
+        <v>0.04371805125997935</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>315.5275779376499</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>1.152705401284587</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3116,7 +3136,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K31" t="n">
-        <v>3.381978382364768</v>
+        <v>3.331846433709419</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3132,7 +3152,7 @@
         <v>0.026182</v>
       </c>
       <c r="Q31" t="n">
-        <v>518.4000000000001</v>
+        <v>526.1999999999999</v>
       </c>
       <c r="R31" t="n">
         <v>48192</v>
@@ -3148,13 +3168,13 @@
         <v>15.27539782478406</v>
       </c>
       <c r="W31" t="n">
-        <v>0.05636630637274613</v>
+        <v>0.05553077389515698</v>
       </c>
       <c r="X31" t="n">
         <v>0.06546474346988973</v>
       </c>
       <c r="Y31" t="n">
-        <v>92.96296296296295</v>
+        <v>91.58494868871153</v>
       </c>
       <c r="Z31" t="n">
         <v>0.6063307856829266</v>
@@ -3206,23 +3226,23 @@
         <v>26.4910658661689</v>
       </c>
       <c r="K32" t="n">
-        <v>12.98581660106318</v>
+        <v>13.65518859080871</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
-        <v>0.369455</v>
+        <v>0.416252</v>
       </c>
       <c r="N32" t="n">
-        <v>0.344869</v>
+        <v>0.387977</v>
       </c>
       <c r="O32" t="n">
-        <v>0.006788</v>
+        <v>0.007806</v>
       </c>
       <c r="P32" t="n">
-        <v>0.017799</v>
+        <v>0.020469</v>
       </c>
       <c r="Q32" t="n">
-        <v>122.4</v>
+        <v>116.4</v>
       </c>
       <c r="R32" t="n">
         <v>49173.8</v>
@@ -3235,16 +3255,16 @@
       </c>
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="n">
-        <v>71.70309203060968</v>
+        <v>63.641894492204</v>
       </c>
       <c r="W32" t="n">
-        <v>0.2164302766843864</v>
+        <v>0.2275864765134785</v>
       </c>
       <c r="X32" t="n">
-        <v>0.01394639996240476</v>
+        <v>0.01571292005021155</v>
       </c>
       <c r="Y32" t="n">
-        <v>401.7467320261438</v>
+        <v>422.4553264604812</v>
       </c>
       <c r="Z32" t="n">
         <v>0.5387231791354116</v>
@@ -3296,7 +3316,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K33" t="n">
-        <v>10.19786983670955</v>
+        <v>10.15641508127577</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -3312,7 +3332,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q33" t="n">
-        <v>147</v>
+        <v>147.6</v>
       </c>
       <c r="R33" t="n">
         <v>34656</v>
@@ -3328,13 +3348,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W33" t="n">
-        <v>0.1699644972784925</v>
+        <v>0.1692735846879296</v>
       </c>
       <c r="X33" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y33" t="n">
-        <v>235.7551020408163</v>
+        <v>234.7967479674797</v>
       </c>
       <c r="Z33" t="n">
         <v>0.7209366660877885</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-18)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.408750559318768</v>
+        <v>4.378599529657773</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>784.2</v>
+        <v>789.6</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07347917598864613</v>
+        <v>0.07297665882762956</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>151.9586840091813</v>
+        <v>150.919452887538</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.718468038385086</v>
+        <v>3.781237586636016</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>903.6</v>
+        <v>888.6</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.0619744673064181</v>
+        <v>0.06302062644393359</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>218.4931385568836</v>
+        <v>222.1814089579113</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.721170538296987</v>
+        <v>6.786345525335019</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>499.8</v>
+        <v>495</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1120195089716164</v>
+        <v>0.1131057587555836</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>131.3873549419768</v>
+        <v>132.6614141414141</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -922,7 +922,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K6" t="n">
-        <v>11.77652658949598</v>
+        <v>11.8546893765944</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -938,7 +938,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q6" t="n">
-        <v>273</v>
+        <v>271.2</v>
       </c>
       <c r="R6" t="n">
         <v>35584.1</v>
@@ -954,13 +954,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1962754431582663</v>
+        <v>0.1975781562765734</v>
       </c>
       <c r="X6" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y6" t="n">
-        <v>130.3446886446886</v>
+        <v>131.209808259587</v>
       </c>
       <c r="Z6" t="n">
         <v>1.505818497087371</v>
@@ -1012,7 +1012,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K7" t="n">
-        <v>4.476084392812517</v>
+        <v>4.472332436070847</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1028,7 +1028,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q7" t="n">
-        <v>715.2</v>
+        <v>715.8</v>
       </c>
       <c r="R7" t="n">
         <v>78110.8</v>
@@ -1044,13 +1044,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W7" t="n">
-        <v>0.07460140654687528</v>
+        <v>0.07453887393451411</v>
       </c>
       <c r="X7" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y7" t="n">
-        <v>109.2153243847875</v>
+        <v>109.123777591506</v>
       </c>
       <c r="Z7" t="n">
         <v>0.6830672066132366</v>
@@ -1102,7 +1102,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K8" t="n">
-        <v>5.395868027778338</v>
+        <v>5.401346066385218</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1118,7 +1118,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q8" t="n">
-        <v>591.5999999999999</v>
+        <v>591</v>
       </c>
       <c r="R8" t="n">
         <v>60537.6</v>
@@ -1134,13 +1134,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W8" t="n">
-        <v>0.08993113379630563</v>
+        <v>0.09002243443975365</v>
       </c>
       <c r="X8" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y8" t="n">
-        <v>102.3286004056795</v>
+        <v>102.4324873096447</v>
       </c>
       <c r="Z8" t="n">
         <v>0.8788465144619939</v>
@@ -1192,7 +1192,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K9" t="n">
-        <v>6.692969427638246</v>
+        <v>7.667200785373072</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q9" t="n">
-        <v>472.2</v>
+        <v>412.2</v>
       </c>
       <c r="R9" t="n">
         <v>27205.5</v>
@@ -1224,13 +1224,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1115494904606374</v>
+        <v>0.1277866797562179</v>
       </c>
       <c r="X9" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y9" t="n">
-        <v>57.6143583227446</v>
+        <v>66.00072780203784</v>
       </c>
       <c r="Z9" t="n">
         <v>1.936140464079432</v>
@@ -1364,7 +1364,7 @@
         <v>52.393894697293</v>
       </c>
       <c r="K11" t="n">
-        <v>10.84759724581636</v>
+        <v>10.5420311262159</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1380,7 +1380,7 @@
         <v>0.573611</v>
       </c>
       <c r="Q11" t="n">
-        <v>289.8</v>
+        <v>298.2</v>
       </c>
       <c r="R11" t="n">
         <v>54231.7</v>
@@ -1396,13 +1396,13 @@
         <v>1.645610026239954</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1807932874302726</v>
+        <v>0.1757005187702649</v>
       </c>
       <c r="X11" t="n">
         <v>0.6076773865342173</v>
       </c>
       <c r="Y11" t="n">
-        <v>187.1349206349206</v>
+        <v>181.8635144198524</v>
       </c>
       <c r="Z11" t="n">
         <v>0.9661119732055791</v>
@@ -1454,7 +1454,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K12" t="n">
-        <v>10.15238909125546</v>
+        <v>10.47726554217564</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1470,7 +1470,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q12" t="n">
-        <v>309.6</v>
+        <v>300</v>
       </c>
       <c r="R12" t="n">
         <v>16901.2</v>
@@ -1486,13 +1486,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W12" t="n">
-        <v>0.1692064848542577</v>
+        <v>0.174621092369594</v>
       </c>
       <c r="X12" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y12" t="n">
-        <v>54.59043927648579</v>
+        <v>56.33733333333333</v>
       </c>
       <c r="Z12" t="n">
         <v>3.099562617499243</v>
@@ -1544,7 +1544,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K13" t="n">
-        <v>7.258119499064181</v>
+        <v>7.298952801449915</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1560,7 +1560,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q13" t="n">
-        <v>429</v>
+        <v>426.6</v>
       </c>
       <c r="R13" t="n">
         <v>74809.60000000001</v>
@@ -1576,13 +1576,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1209686583177364</v>
+        <v>0.1216492133574986</v>
       </c>
       <c r="X13" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y13" t="n">
-        <v>174.381351981352</v>
+        <v>175.3624003750586</v>
       </c>
       <c r="Z13" t="n">
         <v>0.6937018032218979</v>
@@ -1634,7 +1634,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K14" t="n">
-        <v>5.299924304821483</v>
+        <v>5.262259868137472</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1650,7 +1650,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q14" t="n">
-        <v>586.8</v>
+        <v>591</v>
       </c>
       <c r="R14" t="n">
         <v>38128.4</v>
@@ -1666,13 +1666,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W14" t="n">
-        <v>0.08833207174702472</v>
+        <v>0.08770433113562454</v>
       </c>
       <c r="X14" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y14" t="n">
-        <v>64.9768234492161</v>
+        <v>64.51505922165821</v>
       </c>
       <c r="Z14" t="n">
         <v>1.359439674918279</v>
@@ -1724,7 +1724,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>3.377930954925716</v>
+        <v>3.422737703038217</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1740,7 +1740,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>825</v>
+        <v>814.2</v>
       </c>
       <c r="R15" t="n">
         <v>80561.39999999999</v>
@@ -1756,13 +1756,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.05629884924876194</v>
+        <v>0.05704562838397027</v>
       </c>
       <c r="X15" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>97.65018181818181</v>
+        <v>98.94546794399409</v>
       </c>
       <c r="Z15" t="n">
         <v>0.5765360412086756</v>
@@ -1994,7 +1994,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K18" t="n">
-        <v>3.473808563662839</v>
+        <v>4.411565752277241</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2010,7 +2010,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q18" t="n">
-        <v>773.4000000000001</v>
+        <v>609</v>
       </c>
       <c r="R18" t="n">
         <v>71127.60000000001</v>
@@ -2026,13 +2026,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W18" t="n">
-        <v>0.05789680939438065</v>
+        <v>0.07352609587128736</v>
       </c>
       <c r="X18" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y18" t="n">
-        <v>91.96741660201707</v>
+        <v>116.7940886699508</v>
       </c>
       <c r="Z18" t="n">
         <v>0.629536106737947</v>
@@ -2084,7 +2084,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K19" t="n">
-        <v>4.399829468225493</v>
+        <v>4.417606556986</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2100,7 +2100,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q19" t="n">
-        <v>596.4</v>
+        <v>594</v>
       </c>
       <c r="R19" t="n">
         <v>64144.3</v>
@@ -2116,13 +2116,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W19" t="n">
-        <v>0.07333049113709154</v>
+        <v>0.07362677594976666</v>
       </c>
       <c r="X19" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y19" t="n">
-        <v>107.5524815560027</v>
+        <v>107.987037037037</v>
       </c>
       <c r="Z19" t="n">
         <v>0.6818112429968274</v>
@@ -2174,7 +2174,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K20" t="n">
-        <v>2.442230977696258</v>
+        <v>2.537475142717008</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2190,7 +2190,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q20" t="n">
-        <v>1071</v>
+        <v>1030.8</v>
       </c>
       <c r="R20" t="n">
         <v>48455.2</v>
@@ -2206,13 +2206,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W20" t="n">
-        <v>0.04070384962827096</v>
+        <v>0.04229125237861681</v>
       </c>
       <c r="X20" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y20" t="n">
-        <v>45.24295051353874</v>
+        <v>47.00737291424137</v>
       </c>
       <c r="Z20" t="n">
         <v>0.8996727482680539</v>
@@ -2264,7 +2264,7 @@
         <v>43.3950199670746</v>
       </c>
       <c r="K21" t="n">
-        <v>6.069233561828615</v>
+        <v>6.12924010834387</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2280,7 +2280,7 @@
         <v>0.064523</v>
       </c>
       <c r="Q21" t="n">
-        <v>429</v>
+        <v>424.8</v>
       </c>
       <c r="R21" t="n">
         <v>162164.2</v>
@@ -2296,13 +2296,13 @@
         <v>40.74733935074209</v>
       </c>
       <c r="W21" t="n">
-        <v>0.1011538926971436</v>
+        <v>0.1021540018057312</v>
       </c>
       <c r="X21" t="n">
         <v>0.02454147966305898</v>
       </c>
       <c r="Y21" t="n">
-        <v>378.0051282051282</v>
+        <v>381.7424670433145</v>
       </c>
       <c r="Z21" t="n">
         <v>0.2675992602995889</v>
@@ -2354,7 +2354,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K22" t="n">
-        <v>3.44377809830766</v>
+        <v>3.786908162450634</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2370,7 +2370,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q22" t="n">
-        <v>728.4000000000001</v>
+        <v>662.4</v>
       </c>
       <c r="R22" t="n">
         <v>68673.2</v>
@@ -2386,13 +2386,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W22" t="n">
-        <v>0.057396301638461</v>
+        <v>0.0631151360408439</v>
       </c>
       <c r="X22" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y22" t="n">
-        <v>94.27951674903898</v>
+        <v>103.673309178744</v>
       </c>
       <c r="Z22" t="n">
         <v>0.6087886703030441</v>
@@ -2444,7 +2444,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K23" t="n">
-        <v>5.180535718555747</v>
+        <v>5.335884247273847</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2460,7 +2460,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q23" t="n">
-        <v>474</v>
+        <v>460.2</v>
       </c>
       <c r="R23" t="n">
         <v>71002.60000000001</v>
@@ -2476,13 +2476,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W23" t="n">
-        <v>0.08634226197592912</v>
+        <v>0.08893140412123078</v>
       </c>
       <c r="X23" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y23" t="n">
-        <v>149.7945147679325</v>
+        <v>154.2863972186006</v>
       </c>
       <c r="Z23" t="n">
         <v>0.5764046975264343</v>
@@ -2534,7 +2534,7 @@
         <v>39.456167472527</v>
       </c>
       <c r="K24" t="n">
-        <v>6.543311355311277</v>
+        <v>8.035879322306924</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2550,7 +2550,7 @@
         <v>0.07520300000000001</v>
       </c>
       <c r="Q24" t="n">
-        <v>361.8</v>
+        <v>294.6</v>
       </c>
       <c r="R24" t="n">
         <v>88574</v>
@@ -2566,13 +2566,13 @@
         <v>12.61396912906789</v>
       </c>
       <c r="W24" t="n">
-        <v>0.109055189255188</v>
+        <v>0.1339313220384487</v>
       </c>
       <c r="X24" t="n">
         <v>0.07927718783579227</v>
       </c>
       <c r="Y24" t="n">
-        <v>244.8148148148148</v>
+        <v>300.6585200271554</v>
       </c>
       <c r="Z24" t="n">
         <v>0.4454599258532639</v>
@@ -2624,7 +2624,7 @@
         <v>38.8666662997805</v>
       </c>
       <c r="K25" t="n">
-        <v>7.546925495103009</v>
+        <v>8.046928840534264</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2640,7 +2640,7 @@
         <v>0.07819</v>
       </c>
       <c r="Q25" t="n">
-        <v>309</v>
+        <v>289.8</v>
       </c>
       <c r="R25" t="n">
         <v>40335.1</v>
@@ -2656,13 +2656,13 @@
         <v>10.3209696700991</v>
       </c>
       <c r="W25" t="n">
-        <v>0.1257820915850502</v>
+        <v>0.1341154806755711</v>
       </c>
       <c r="X25" t="n">
         <v>0.09689012098321557</v>
       </c>
       <c r="Y25" t="n">
-        <v>130.5343042071197</v>
+        <v>139.1825396825397</v>
       </c>
       <c r="Z25" t="n">
         <v>0.9635941475236333</v>
@@ -2804,7 +2804,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K27" t="n">
-        <v>5.430843117802536</v>
+        <v>5.690226669697582</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2820,7 +2820,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q27" t="n">
-        <v>421.2</v>
+        <v>402</v>
       </c>
       <c r="R27" t="n">
         <v>50011.7</v>
@@ -2836,13 +2836,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W27" t="n">
-        <v>0.0905140519633756</v>
+        <v>0.09483711116162637</v>
       </c>
       <c r="X27" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y27" t="n">
-        <v>118.7362298195631</v>
+        <v>124.4072139303482</v>
       </c>
       <c r="Z27" t="n">
         <v>0.7623119927331765</v>
@@ -2894,7 +2894,7 @@
         <v>33.6762858057476</v>
       </c>
       <c r="K28" t="n">
-        <v>1.599823553717225</v>
+        <v>1.5952764474537</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2910,7 +2910,7 @@
         <v>0.143075</v>
       </c>
       <c r="Q28" t="n">
-        <v>1263</v>
+        <v>1266.6</v>
       </c>
       <c r="R28" t="n">
         <v>66783.2</v>
@@ -2926,13 +2926,13 @@
         <v>13.43904545346521</v>
       </c>
       <c r="W28" t="n">
-        <v>0.02666372589528709</v>
+        <v>0.02658794079089499</v>
       </c>
       <c r="X28" t="n">
         <v>0.07441004671519687</v>
       </c>
       <c r="Y28" t="n">
-        <v>52.87664291369754</v>
+        <v>52.72635401863256</v>
       </c>
       <c r="Z28" t="n">
         <v>0.5042628356494987</v>
@@ -3046,7 +3046,7 @@
         <v>30.3334426348039</v>
       </c>
       <c r="K30" t="n">
-        <v>21.82262060057835</v>
+        <v>24.8634775695114</v>
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="n">
@@ -3062,7 +3062,7 @@
         <v>0.040904</v>
       </c>
       <c r="Q30" t="n">
-        <v>83.39999999999999</v>
+        <v>73.2</v>
       </c>
       <c r="R30" t="n">
         <v>26315</v>
@@ -3078,13 +3078,13 @@
         <v>22.87384664182015</v>
       </c>
       <c r="W30" t="n">
-        <v>0.3637103433429725</v>
+        <v>0.4143912928251899</v>
       </c>
       <c r="X30" t="n">
         <v>0.04371805125997935</v>
       </c>
       <c r="Y30" t="n">
-        <v>315.5275779376499</v>
+        <v>359.4945355191257</v>
       </c>
       <c r="Z30" t="n">
         <v>1.152705401284587</v>
@@ -3136,7 +3136,7 @@
         <v>29.2202932236316</v>
       </c>
       <c r="K31" t="n">
-        <v>3.331846433709419</v>
+        <v>4.18029945974701</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3152,7 +3152,7 @@
         <v>0.026182</v>
       </c>
       <c r="Q31" t="n">
-        <v>526.1999999999999</v>
+        <v>419.4</v>
       </c>
       <c r="R31" t="n">
         <v>48192</v>
@@ -3168,13 +3168,13 @@
         <v>15.27539782478406</v>
       </c>
       <c r="W31" t="n">
-        <v>0.05553077389515698</v>
+        <v>0.06967165766245016</v>
       </c>
       <c r="X31" t="n">
         <v>0.06546474346988973</v>
       </c>
       <c r="Y31" t="n">
-        <v>91.58494868871153</v>
+        <v>114.9070100143061</v>
       </c>
       <c r="Z31" t="n">
         <v>0.6063307856829266</v>
@@ -3226,7 +3226,7 @@
         <v>26.4910658661689</v>
       </c>
       <c r="K32" t="n">
-        <v>13.65518859080871</v>
+        <v>15.22475049779822</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3242,7 +3242,7 @@
         <v>0.020469</v>
       </c>
       <c r="Q32" t="n">
-        <v>116.4</v>
+        <v>104.4</v>
       </c>
       <c r="R32" t="n">
         <v>49173.8</v>
@@ -3258,13 +3258,13 @@
         <v>63.641894492204</v>
       </c>
       <c r="W32" t="n">
-        <v>0.2275864765134785</v>
+        <v>0.2537458416299703</v>
       </c>
       <c r="X32" t="n">
         <v>0.01571292005021155</v>
       </c>
       <c r="Y32" t="n">
-        <v>422.4553264604812</v>
+        <v>471.0134099616859</v>
       </c>
       <c r="Z32" t="n">
         <v>0.5387231791354116</v>
@@ -3316,7 +3316,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K33" t="n">
-        <v>10.15641508127577</v>
+        <v>10.72308201714094</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -3332,7 +3332,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q33" t="n">
-        <v>147.6</v>
+        <v>139.8</v>
       </c>
       <c r="R33" t="n">
         <v>34656</v>
@@ -3348,13 +3348,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W33" t="n">
-        <v>0.1692735846879296</v>
+        <v>0.1787180336190157</v>
       </c>
       <c r="X33" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y33" t="n">
-        <v>234.7967479674797</v>
+        <v>247.8969957081545</v>
       </c>
       <c r="Z33" t="n">
         <v>0.7209366660877885</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-19)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.378599529657773</v>
+        <v>4.326003739511734</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>789.6</v>
+        <v>799.2</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07297665882762956</v>
+        <v>0.07210006232519557</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>150.919452887538</v>
+        <v>149.1066066066066</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.781237586636016</v>
+        <v>3.735832465515637</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>888.6</v>
+        <v>899.4</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.06302062644393359</v>
+        <v>0.06226387442526062</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>222.1814089579113</v>
+        <v>219.5134534133867</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.786345525335019</v>
+        <v>6.745463925784807</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>495</v>
+        <v>498.0000000000001</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1131057587555836</v>
+        <v>0.1124243987630801</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>132.6614141414141</v>
+        <v>131.8622489959839</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -922,7 +922,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K6" t="n">
-        <v>11.8546893765944</v>
+        <v>11.54810258237213</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -938,7 +938,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q6" t="n">
-        <v>271.2</v>
+        <v>278.4</v>
       </c>
       <c r="R6" t="n">
         <v>35584.1</v>
@@ -954,13 +954,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1975781562765734</v>
+        <v>0.1924683763728689</v>
       </c>
       <c r="X6" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y6" t="n">
-        <v>131.209808259587</v>
+        <v>127.8164511494253</v>
       </c>
       <c r="Z6" t="n">
         <v>1.505818497087371</v>
@@ -1012,7 +1012,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K7" t="n">
-        <v>4.472332436070847</v>
+        <v>4.337798858725625</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1028,7 +1028,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q7" t="n">
-        <v>715.8</v>
+        <v>738</v>
       </c>
       <c r="R7" t="n">
         <v>78110.8</v>
@@ -1044,13 +1044,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W7" t="n">
-        <v>0.07453887393451411</v>
+        <v>0.07229664764542709</v>
       </c>
       <c r="X7" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y7" t="n">
-        <v>109.123777591506</v>
+        <v>105.8411924119241</v>
       </c>
       <c r="Z7" t="n">
         <v>0.6830672066132366</v>
@@ -1102,7 +1102,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K8" t="n">
-        <v>5.401346066385218</v>
+        <v>5.257239007301819</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1118,7 +1118,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q8" t="n">
-        <v>591</v>
+        <v>607.1999999999999</v>
       </c>
       <c r="R8" t="n">
         <v>60537.6</v>
@@ -1134,13 +1134,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W8" t="n">
-        <v>0.09002243443975365</v>
+        <v>0.08762065012169698</v>
       </c>
       <c r="X8" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y8" t="n">
-        <v>102.4324873096447</v>
+        <v>99.69960474308301</v>
       </c>
       <c r="Z8" t="n">
         <v>0.8788465144619939</v>
@@ -1192,7 +1192,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K9" t="n">
-        <v>7.667200785373072</v>
+        <v>7.920852540678647</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q9" t="n">
-        <v>412.2</v>
+        <v>399</v>
       </c>
       <c r="R9" t="n">
         <v>27205.5</v>
@@ -1224,13 +1224,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1277866797562179</v>
+        <v>0.1320142090113108</v>
       </c>
       <c r="X9" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y9" t="n">
-        <v>66.00072780203784</v>
+        <v>68.18421052631579</v>
       </c>
       <c r="Z9" t="n">
         <v>1.936140464079432</v>
@@ -1364,7 +1364,7 @@
         <v>52.393894697293</v>
       </c>
       <c r="K11" t="n">
-        <v>10.5420311262159</v>
+        <v>8.396457483540544</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1380,7 +1380,7 @@
         <v>0.573611</v>
       </c>
       <c r="Q11" t="n">
-        <v>298.2</v>
+        <v>374.4</v>
       </c>
       <c r="R11" t="n">
         <v>54231.7</v>
@@ -1396,13 +1396,13 @@
         <v>1.645610026239954</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1757005187702649</v>
+        <v>0.1399409580590091</v>
       </c>
       <c r="X11" t="n">
         <v>0.6076773865342173</v>
       </c>
       <c r="Y11" t="n">
-        <v>181.8635144198524</v>
+        <v>144.849626068376</v>
       </c>
       <c r="Z11" t="n">
         <v>0.9661119732055791</v>
@@ -1454,7 +1454,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K12" t="n">
-        <v>10.47726554217564</v>
+        <v>11.33903197205156</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1470,7 +1470,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q12" t="n">
-        <v>300</v>
+        <v>277.2</v>
       </c>
       <c r="R12" t="n">
         <v>16901.2</v>
@@ -1486,13 +1486,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W12" t="n">
-        <v>0.174621092369594</v>
+        <v>0.1889838662008593</v>
       </c>
       <c r="X12" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y12" t="n">
-        <v>56.33733333333333</v>
+        <v>60.97113997113998</v>
       </c>
       <c r="Z12" t="n">
         <v>3.099562617499243</v>
@@ -1544,7 +1544,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K13" t="n">
-        <v>7.298952801449915</v>
+        <v>7.258119499064181</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1560,7 +1560,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q13" t="n">
-        <v>426.6</v>
+        <v>429</v>
       </c>
       <c r="R13" t="n">
         <v>74809.60000000001</v>
@@ -1576,13 +1576,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1216492133574986</v>
+        <v>0.1209686583177364</v>
       </c>
       <c r="X13" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y13" t="n">
-        <v>175.3624003750586</v>
+        <v>174.381351981352</v>
       </c>
       <c r="Z13" t="n">
         <v>0.6937018032218979</v>
@@ -1634,7 +1634,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K14" t="n">
-        <v>5.262259868137472</v>
+        <v>4.74229274484484</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1650,7 +1650,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q14" t="n">
-        <v>591</v>
+        <v>655.8</v>
       </c>
       <c r="R14" t="n">
         <v>38128.4</v>
@@ -1666,13 +1666,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W14" t="n">
-        <v>0.08770433113562454</v>
+        <v>0.07903821241408067</v>
       </c>
       <c r="X14" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y14" t="n">
-        <v>64.51505922165821</v>
+        <v>58.14028667276609</v>
       </c>
       <c r="Z14" t="n">
         <v>1.359439674918279</v>
@@ -1724,7 +1724,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>3.422737703038217</v>
+        <v>3.134045251702335</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1740,7 +1740,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>814.2</v>
+        <v>889.2</v>
       </c>
       <c r="R15" t="n">
         <v>80561.39999999999</v>
@@ -1756,13 +1756,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.05704562838397027</v>
+        <v>0.05223408752837224</v>
       </c>
       <c r="X15" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>98.94546794399409</v>
+        <v>90.59986504723345</v>
       </c>
       <c r="Z15" t="n">
         <v>0.5765360412086756</v>
@@ -1814,7 +1814,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>2.266350613064496</v>
+        <v>2.297827704912614</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1830,7 +1830,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1226.4</v>
+        <v>1209.6</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1846,13 +1846,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.0377725102177416</v>
+        <v>0.03829712841521024</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>52.41006196999347</v>
+        <v>53.1379794973545</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1904,7 +1904,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.265047590474989</v>
+        <v>1.241531123511539</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1920,7 +1920,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2154</v>
+        <v>2194.8</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1936,13 +1936,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.02108412650791648</v>
+        <v>0.02069218539185899</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>50.01402042711235</v>
+        <v>49.0842901403317</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -1951,32 +1951,32 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>glm-5-3</t>
+          <t>deepseek-v4-1-flash-1017</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>GLM-5.3 (Max)</t>
+          <t>DeepSeek V4.1 Flash 1017 (Max)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>DeepSeek V4.1 Flash 1017 (max)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>DeepSeek</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>deepseek</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1991,82 +1991,82 @@
         <v>1</v>
       </c>
       <c r="J18" t="n">
-        <v>44.777392385614</v>
+        <v>45.0965048681912</v>
       </c>
       <c r="K18" t="n">
-        <v>4.411565752277241</v>
+        <v>9.055523065901847</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
-        <v>8.678356000000001</v>
+        <v>3.00199</v>
       </c>
       <c r="N18" t="n">
-        <v>8.365394999999999</v>
+        <v>2.894596</v>
       </c>
       <c r="O18" t="n">
-        <v>0.098552</v>
+        <v>0.036302</v>
       </c>
       <c r="P18" t="n">
-        <v>0.21441</v>
+        <v>0.071092</v>
       </c>
       <c r="Q18" t="n">
-        <v>609</v>
+        <v>298.8</v>
       </c>
       <c r="R18" t="n">
-        <v>71127.60000000001</v>
+        <v>89495.10000000001</v>
       </c>
       <c r="S18" t="n">
-        <v>22398.1</v>
+        <v>30252</v>
       </c>
       <c r="T18" t="n">
-        <v>48729.5</v>
+        <v>59243</v>
       </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="n">
-        <v>5.159663003639629</v>
+        <v>15.02220356103491</v>
       </c>
       <c r="W18" t="n">
-        <v>0.07352609587128736</v>
+        <v>0.1509253844316975</v>
       </c>
       <c r="X18" t="n">
-        <v>0.1938111072941391</v>
+        <v>0.06656813003079209</v>
       </c>
       <c r="Y18" t="n">
-        <v>116.7940886699508</v>
+        <v>299.5150602409639</v>
       </c>
       <c r="Z18" t="n">
-        <v>0.629536106737947</v>
+        <v>0.5038991505478086</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>step-5</t>
+          <t>glm-5-3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>GLM-5.3 (Max)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>StepFun</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>stepfun</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2081,82 +2081,82 @@
         <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>43.7343049141614</v>
+        <v>44.777392385614</v>
       </c>
       <c r="K19" t="n">
-        <v>4.417606556986</v>
+        <v>4.773709209553731</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
-        <v>6.586908</v>
+        <v>8.678356000000001</v>
       </c>
       <c r="N19" t="n">
-        <v>6.413718</v>
+        <v>8.365394999999999</v>
       </c>
       <c r="O19" t="n">
-        <v>0.055881</v>
+        <v>0.098552</v>
       </c>
       <c r="P19" t="n">
-        <v>0.117309</v>
+        <v>0.21441</v>
       </c>
       <c r="Q19" t="n">
-        <v>594</v>
+        <v>562.8000000000001</v>
       </c>
       <c r="R19" t="n">
-        <v>64144.3</v>
+        <v>71127.60000000001</v>
       </c>
       <c r="S19" t="n">
-        <v>20696.6</v>
+        <v>22398.1</v>
       </c>
       <c r="T19" t="n">
-        <v>43447.7</v>
+        <v>48729.5</v>
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="n">
-        <v>6.639580348497565</v>
+        <v>5.159663003639629</v>
       </c>
       <c r="W19" t="n">
-        <v>0.07362677594976666</v>
+        <v>0.07956182015922884</v>
       </c>
       <c r="X19" t="n">
-        <v>0.1506119283918727</v>
+        <v>0.1938111072941391</v>
       </c>
       <c r="Y19" t="n">
-        <v>107.987037037037</v>
+        <v>126.3816631130064</v>
       </c>
       <c r="Z19" t="n">
-        <v>0.6818112429968274</v>
+        <v>0.629536106737947</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>kimi-k3</t>
+          <t>step-5</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Kimi K3 (Max)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Kimi K3 (max)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Kimi</t>
+          <t>StepFun</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>kimi</t>
+          <t>stepfun</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2171,267 +2171,267 @@
         <v>1</v>
       </c>
       <c r="J20" t="n">
-        <v>43.5938229518782</v>
+        <v>43.7343049141614</v>
       </c>
       <c r="K20" t="n">
-        <v>2.537475142717008</v>
+        <v>4.173120697916164</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
-        <v>9.216749</v>
+        <v>6.586908</v>
       </c>
       <c r="N20" t="n">
-        <v>8.489921000000001</v>
+        <v>6.413718</v>
       </c>
       <c r="O20" t="n">
-        <v>0.240032</v>
+        <v>0.055881</v>
       </c>
       <c r="P20" t="n">
-        <v>0.486797</v>
+        <v>0.117309</v>
       </c>
       <c r="Q20" t="n">
-        <v>1030.8</v>
+        <v>628.8000000000001</v>
       </c>
       <c r="R20" t="n">
-        <v>48455.2</v>
+        <v>64144.3</v>
       </c>
       <c r="S20" t="n">
-        <v>16002.1</v>
+        <v>20696.6</v>
       </c>
       <c r="T20" t="n">
-        <v>32453.1</v>
+        <v>43447.7</v>
       </c>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="n">
-        <v>4.72984812235618</v>
+        <v>6.639580348497565</v>
       </c>
       <c r="W20" t="n">
-        <v>0.04229125237861681</v>
+        <v>0.06955201163193606</v>
       </c>
       <c r="X20" t="n">
-        <v>0.2114232791690251</v>
+        <v>0.1506119283918727</v>
       </c>
       <c r="Y20" t="n">
-        <v>47.00737291424137</v>
+        <v>102.010655216285</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.8996727482680539</v>
+        <v>0.6818112429968274</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>claude-haiku-5-5</t>
+          <t>kimi-k3</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Claude Haiku 5.5 (Max)</t>
+          <t>Kimi K3 (Max)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Claude Haiku 5.5 (max)</t>
+          <t>Kimi K3 (max)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Kimi</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>kimi</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H21" t="b">
         <v>1</v>
       </c>
       <c r="I21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" t="n">
-        <v>43.3950199670746</v>
+        <v>43.5938229518782</v>
       </c>
       <c r="K21" t="n">
-        <v>6.12924010834387</v>
+        <v>2.442230977696258</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
-        <v>1.064978</v>
+        <v>9.216749</v>
       </c>
       <c r="N21" t="n">
-        <v>0.983896</v>
+        <v>8.489921000000001</v>
       </c>
       <c r="O21" t="n">
-        <v>0.016559</v>
+        <v>0.240032</v>
       </c>
       <c r="P21" t="n">
-        <v>0.064523</v>
+        <v>0.486797</v>
       </c>
       <c r="Q21" t="n">
-        <v>424.8</v>
+        <v>1071</v>
       </c>
       <c r="R21" t="n">
-        <v>162164.2</v>
+        <v>48455.2</v>
       </c>
       <c r="S21" t="n">
-        <v>33117.6</v>
+        <v>16002.1</v>
       </c>
       <c r="T21" t="n">
-        <v>129046.6</v>
+        <v>32453.1</v>
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="n">
-        <v>40.74733935074209</v>
+        <v>4.72984812235618</v>
       </c>
       <c r="W21" t="n">
-        <v>0.1021540018057312</v>
+        <v>0.04070384962827096</v>
       </c>
       <c r="X21" t="n">
-        <v>0.02454147966305898</v>
+        <v>0.2114232791690251</v>
       </c>
       <c r="Y21" t="n">
-        <v>381.7424670433145</v>
+        <v>45.24295051353874</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.2675992602995889</v>
+        <v>0.8996727482680539</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>glm-5-3-flash</t>
+          <t>claude-haiku-5-5</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Claude Haiku 5.5 (Max)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Claude Haiku 5.5 (max)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H22" t="b">
         <v>1</v>
       </c>
       <c r="I22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>41.807466113455</v>
+        <v>43.3950199670746</v>
       </c>
       <c r="K22" t="n">
-        <v>3.786908162450634</v>
+        <v>6.120595199869479</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
-        <v>1.193653</v>
+        <v>1.064978</v>
       </c>
       <c r="N22" t="n">
-        <v>1.159316</v>
+        <v>0.983896</v>
       </c>
       <c r="O22" t="n">
-        <v>0.011012</v>
+        <v>0.016559</v>
       </c>
       <c r="P22" t="n">
-        <v>0.023325</v>
+        <v>0.064523</v>
       </c>
       <c r="Q22" t="n">
-        <v>662.4</v>
+        <v>425.4</v>
       </c>
       <c r="R22" t="n">
-        <v>68673.2</v>
+        <v>162164.2</v>
       </c>
       <c r="S22" t="n">
-        <v>22023.7</v>
+        <v>33117.6</v>
       </c>
       <c r="T22" t="n">
-        <v>46649.5</v>
+        <v>129046.6</v>
       </c>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="n">
-        <v>35.02480713696107</v>
+        <v>40.74733935074209</v>
       </c>
       <c r="W22" t="n">
-        <v>0.0631151360408439</v>
+        <v>0.1020099199978246</v>
       </c>
       <c r="X22" t="n">
-        <v>0.02855119219042658</v>
+        <v>0.02454147966305898</v>
       </c>
       <c r="Y22" t="n">
-        <v>103.673309178744</v>
+        <v>381.2040432534086</v>
       </c>
       <c r="Z22" t="n">
-        <v>0.6087886703030441</v>
+        <v>0.2675992602995889</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>gemini-3-8-flash</t>
+          <t>minimax-m3-1-flash</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (High)</t>
+          <t>MiniMax-M3.1-Flash</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>MiniMax-M3.1-Flash</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>minimax</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H23" t="b">
@@ -2441,82 +2441,74 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>40.9262321765904</v>
-      </c>
-      <c r="K23" t="n">
-        <v>5.335884247273847</v>
-      </c>
+        <v>42.3811052132362</v>
+      </c>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
-        <v>4.90102</v>
+        <v>1.306119</v>
       </c>
       <c r="N23" t="n">
-        <v>4.63476</v>
+        <v>1.258952</v>
       </c>
       <c r="O23" t="n">
-        <v>0.106033</v>
+        <v>0.014367</v>
       </c>
       <c r="P23" t="n">
-        <v>0.160227</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>460.2</v>
-      </c>
+        <v>0.032801</v>
+      </c>
+      <c r="Q23" t="inlineStr"/>
       <c r="R23" t="n">
-        <v>71002.60000000001</v>
+        <v>78612.3</v>
       </c>
       <c r="S23" t="n">
-        <v>28275.4</v>
+        <v>23944.7</v>
       </c>
       <c r="T23" t="n">
-        <v>42727.1</v>
+        <v>54667.6</v>
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="n">
-        <v>8.350554002348574</v>
-      </c>
-      <c r="W23" t="n">
-        <v>0.08893140412123078</v>
-      </c>
+        <v>32.44811936219915</v>
+      </c>
+      <c r="W23" t="inlineStr"/>
       <c r="X23" t="n">
-        <v>0.119752533750306</v>
-      </c>
-      <c r="Y23" t="n">
-        <v>154.2863972186006</v>
-      </c>
+        <v>0.03081842706622199</v>
+      </c>
+      <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="n">
-        <v>0.5764046975264343</v>
+        <v>0.5391154464789377</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>deepseek-v4-1-flash</t>
+          <t>glm-5-3-flash</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (Max)</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash (max)</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>DeepSeek</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>deepseek</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2531,82 +2523,82 @@
         <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>39.456167472527</v>
+        <v>41.807466113455</v>
       </c>
       <c r="K24" t="n">
-        <v>8.035879322306924</v>
+        <v>3.73948713000492</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>3.127974</v>
+        <v>1.193653</v>
       </c>
       <c r="N24" t="n">
-        <v>3.021685</v>
+        <v>1.159316</v>
       </c>
       <c r="O24" t="n">
-        <v>0.031085</v>
+        <v>0.011012</v>
       </c>
       <c r="P24" t="n">
-        <v>0.07520300000000001</v>
+        <v>0.023325</v>
       </c>
       <c r="Q24" t="n">
-        <v>294.6</v>
+        <v>670.8</v>
       </c>
       <c r="R24" t="n">
-        <v>88574</v>
+        <v>68673.2</v>
       </c>
       <c r="S24" t="n">
-        <v>25904.4</v>
+        <v>22023.7</v>
       </c>
       <c r="T24" t="n">
-        <v>62669.6</v>
+        <v>46649.5</v>
       </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="n">
-        <v>12.61396912906789</v>
+        <v>35.02480713696107</v>
       </c>
       <c r="W24" t="n">
-        <v>0.1339313220384487</v>
+        <v>0.062324785500082</v>
       </c>
       <c r="X24" t="n">
-        <v>0.07927718783579227</v>
+        <v>0.02855119219042658</v>
       </c>
       <c r="Y24" t="n">
-        <v>300.6585200271554</v>
+        <v>102.3750745378652</v>
       </c>
       <c r="Z24" t="n">
-        <v>0.4454599258532639</v>
+        <v>0.6087886703030441</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>muse-spark-open</t>
+          <t>gemini-3-8-flash</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Muse Spark Open (Xhigh)</t>
+          <t>Gemini 3.8 Flash (High)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Muse Spark Open (xhigh)</t>
+          <t>Gemini 3.8 Flash (high)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2618,85 +2610,85 @@
         <v>1</v>
       </c>
       <c r="I25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>38.8666662997805</v>
+        <v>40.9262321765904</v>
       </c>
       <c r="K25" t="n">
-        <v>8.046928840534264</v>
+        <v>5.240234593673548</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
-        <v>3.765796</v>
+        <v>4.90102</v>
       </c>
       <c r="N25" t="n">
-        <v>3.594372</v>
+        <v>4.63476</v>
       </c>
       <c r="O25" t="n">
-        <v>0.093234</v>
+        <v>0.106033</v>
       </c>
       <c r="P25" t="n">
-        <v>0.07819</v>
+        <v>0.160227</v>
       </c>
       <c r="Q25" t="n">
-        <v>289.8</v>
+        <v>468.6</v>
       </c>
       <c r="R25" t="n">
-        <v>40335.1</v>
+        <v>71002.60000000001</v>
       </c>
       <c r="S25" t="n">
-        <v>21937.3</v>
+        <v>28275.4</v>
       </c>
       <c r="T25" t="n">
-        <v>18397.7</v>
+        <v>42727.1</v>
       </c>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="n">
-        <v>10.3209696700991</v>
+        <v>8.350554002348574</v>
       </c>
       <c r="W25" t="n">
-        <v>0.1341154806755711</v>
+        <v>0.08733724322789246</v>
       </c>
       <c r="X25" t="n">
-        <v>0.09689012098321557</v>
+        <v>0.119752533750306</v>
       </c>
       <c r="Y25" t="n">
-        <v>139.1825396825397</v>
+        <v>151.5206999573197</v>
       </c>
       <c r="Z25" t="n">
-        <v>0.9635941475236333</v>
+        <v>0.5764046975264343</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>mistral-large-4</t>
+          <t>muse-spark-open</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Mistral Large 4 Preview</t>
+          <t>Muse Spark Open (Xhigh)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mistral Large 4 Preview</t>
+          <t>Muse Spark Open (xhigh)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Mistral</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>mistral</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2708,90 +2700,90 @@
         <v>1</v>
       </c>
       <c r="I26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>38.3770408917494</v>
+        <v>38.8666662997805</v>
       </c>
       <c r="K26" t="n">
-        <v>3.137942836610744</v>
+        <v>8.08038800411237</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
-        <v>6.144787</v>
+        <v>3.765796</v>
       </c>
       <c r="N26" t="n">
-        <v>5.854427</v>
+        <v>3.594372</v>
       </c>
       <c r="O26" t="n">
-        <v>0.07260800000000001</v>
+        <v>0.093234</v>
       </c>
       <c r="P26" t="n">
-        <v>0.217751</v>
+        <v>0.07819</v>
       </c>
       <c r="Q26" t="n">
-        <v>733.8000000000001</v>
+        <v>288.6</v>
       </c>
       <c r="R26" t="n">
-        <v>69464</v>
+        <v>40335.1</v>
       </c>
       <c r="S26" t="n">
-        <v>17370.4</v>
+        <v>21937.3</v>
       </c>
       <c r="T26" t="n">
-        <v>52093.6</v>
+        <v>18397.7</v>
       </c>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="n">
-        <v>6.245463169309107</v>
+        <v>10.3209696700991</v>
       </c>
       <c r="W26" t="n">
-        <v>0.05229904727684574</v>
+        <v>0.1346731334018728</v>
       </c>
       <c r="X26" t="n">
-        <v>0.1601162272342122</v>
+        <v>0.09689012098321557</v>
       </c>
       <c r="Y26" t="n">
-        <v>94.66339602071409</v>
+        <v>139.7612612612613</v>
       </c>
       <c r="Z26" t="n">
-        <v>0.5524738122156715</v>
+        <v>0.9635941475236333</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>gpt-6-luna</t>
+          <t>mistral-large-4</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (Max)</t>
+          <t>Mistral Large 4 Preview</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (max)</t>
+          <t>Mistral Large 4 Preview</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Mistral</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>mistral</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H27" t="b">
@@ -2801,177 +2793,177 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>38.1245186869738</v>
+        <v>38.3770408917494</v>
       </c>
       <c r="K27" t="n">
-        <v>5.690226669697582</v>
+        <v>3.130264346798483</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
-        <v>0.326276</v>
+        <v>6.144787</v>
       </c>
       <c r="N27" t="n">
-        <v>0.30127</v>
+        <v>5.854427</v>
       </c>
       <c r="O27" t="n">
-        <v>0.005561</v>
+        <v>0.07260800000000001</v>
       </c>
       <c r="P27" t="n">
-        <v>0.019445</v>
+        <v>0.217751</v>
       </c>
       <c r="Q27" t="n">
-        <v>402</v>
+        <v>735.6</v>
       </c>
       <c r="R27" t="n">
-        <v>50011.7</v>
+        <v>69464</v>
       </c>
       <c r="S27" t="n">
-        <v>11122</v>
+        <v>17370.4</v>
       </c>
       <c r="T27" t="n">
-        <v>38889.7</v>
+        <v>52093.6</v>
       </c>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="n">
-        <v>116.8474502782117</v>
+        <v>6.245463169309107</v>
       </c>
       <c r="W27" t="n">
-        <v>0.09483711116162637</v>
+        <v>0.05217107244664138</v>
       </c>
       <c r="X27" t="n">
-        <v>0.008558167059863248</v>
+        <v>0.1601162272342122</v>
       </c>
       <c r="Y27" t="n">
-        <v>124.4072139303482</v>
+        <v>94.43175638934203</v>
       </c>
       <c r="Z27" t="n">
-        <v>0.7623119927331765</v>
+        <v>0.5524738122156715</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>qwen3-8-27b</t>
+          <t>gpt-6-luna</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (Xhigh)</t>
+          <t>GPT-6 Luna (Max)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (xhigh)</t>
+          <t>GPT-6 Luna (max)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H28" t="b">
         <v>1</v>
       </c>
       <c r="I28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>33.6762858057476</v>
+        <v>38.1245186869738</v>
       </c>
       <c r="K28" t="n">
-        <v>1.5952764474537</v>
+        <v>5.785207691498301</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
-        <v>2.505854</v>
+        <v>0.326276</v>
       </c>
       <c r="N28" t="n">
-        <v>2.305504</v>
+        <v>0.30127</v>
       </c>
       <c r="O28" t="n">
-        <v>0.057275</v>
+        <v>0.005561</v>
       </c>
       <c r="P28" t="n">
-        <v>0.143075</v>
+        <v>0.019445</v>
       </c>
       <c r="Q28" t="n">
-        <v>1266.6</v>
+        <v>395.4</v>
       </c>
       <c r="R28" t="n">
-        <v>66783.2</v>
+        <v>50011.7</v>
       </c>
       <c r="S28" t="n">
-        <v>19091.6</v>
+        <v>11122</v>
       </c>
       <c r="T28" t="n">
-        <v>47691.6</v>
+        <v>38889.7</v>
       </c>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="n">
-        <v>13.43904545346521</v>
+        <v>116.8474502782117</v>
       </c>
       <c r="W28" t="n">
-        <v>0.02658794079089499</v>
+        <v>0.09642012819163835</v>
       </c>
       <c r="X28" t="n">
-        <v>0.07441004671519687</v>
+        <v>0.008558167059863248</v>
       </c>
       <c r="Y28" t="n">
-        <v>52.72635401863256</v>
+        <v>126.4838138593829</v>
       </c>
       <c r="Z28" t="n">
-        <v>0.5042628356494987</v>
+        <v>0.7623119927331765</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>k2-horizon-375b-a23b</t>
+          <t>qwen3-8-27b</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Qwen3.8 27B (Xhigh)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Qwen3.8 27B (xhigh)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Institute of Foundation Models</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ifm</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H29" t="b">
@@ -2981,54 +2973,82 @@
         <v>1</v>
       </c>
       <c r="J29" t="n">
-        <v>30.5015302696723</v>
-      </c>
-      <c r="K29" t="inlineStr"/>
+        <v>33.6762858057476</v>
+      </c>
+      <c r="K29" t="n">
+        <v>1.669622499045493</v>
+      </c>
       <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr"/>
+      <c r="M29" t="n">
+        <v>2.505854</v>
+      </c>
+      <c r="N29" t="n">
+        <v>2.305504</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0.057275</v>
+      </c>
+      <c r="P29" t="n">
+        <v>0.143075</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>1210.2</v>
+      </c>
+      <c r="R29" t="n">
+        <v>66783.2</v>
+      </c>
+      <c r="S29" t="n">
+        <v>19091.6</v>
+      </c>
+      <c r="T29" t="n">
+        <v>47691.6</v>
+      </c>
       <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr"/>
-      <c r="X29" t="inlineStr"/>
-      <c r="Y29" t="inlineStr"/>
-      <c r="Z29" t="inlineStr"/>
+      <c r="V29" t="n">
+        <v>13.43904545346521</v>
+      </c>
+      <c r="W29" t="n">
+        <v>0.02782704165075822</v>
+      </c>
+      <c r="X29" t="n">
+        <v>0.07441004671519687</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>55.18360601553461</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>0.5042628356494987</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>reflection-beam</t>
+          <t>k2-horizon-375b-a23b</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Beam 1.0</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Beam 1.0</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Reflection</t>
+          <t>Institute of Foundation Models</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>reflection</t>
+          <t>ifm</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3043,82 +3063,54 @@
         <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>30.3334426348039</v>
-      </c>
-      <c r="K30" t="n">
-        <v>24.8634775695114</v>
-      </c>
+        <v>30.5015302696723</v>
+      </c>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
-      <c r="M30" t="n">
-        <v>1.326119</v>
-      </c>
-      <c r="N30" t="n">
-        <v>1.270857</v>
-      </c>
-      <c r="O30" t="n">
-        <v>0.014358</v>
-      </c>
-      <c r="P30" t="n">
-        <v>0.040904</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>73.2</v>
-      </c>
-      <c r="R30" t="n">
-        <v>26315</v>
-      </c>
-      <c r="S30" t="n">
-        <v>6837.1</v>
-      </c>
-      <c r="T30" t="n">
-        <v>19478</v>
-      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
-      <c r="V30" t="n">
-        <v>22.87384664182015</v>
-      </c>
-      <c r="W30" t="n">
-        <v>0.4143912928251899</v>
-      </c>
-      <c r="X30" t="n">
-        <v>0.04371805125997935</v>
-      </c>
-      <c r="Y30" t="n">
-        <v>359.4945355191257</v>
-      </c>
-      <c r="Z30" t="n">
-        <v>1.152705401284587</v>
-      </c>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>minimax-m3</t>
+          <t>reflection-beam</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>Beam 1.0</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>Beam 1.0</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>Reflection</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>minimax</t>
+          <t>reflection</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3133,51 +3125,51 @@
         <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>29.2202932236316</v>
+        <v>30.3334426348039</v>
       </c>
       <c r="K31" t="n">
-        <v>4.18029945974701</v>
+        <v>28.61645531585274</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
-        <v>1.912899</v>
+        <v>1.326119</v>
       </c>
       <c r="N31" t="n">
-        <v>1.855069</v>
+        <v>1.270857</v>
       </c>
       <c r="O31" t="n">
-        <v>0.031649</v>
+        <v>0.014358</v>
       </c>
       <c r="P31" t="n">
-        <v>0.026182</v>
+        <v>0.040904</v>
       </c>
       <c r="Q31" t="n">
-        <v>419.4</v>
+        <v>63.6</v>
       </c>
       <c r="R31" t="n">
-        <v>48192</v>
+        <v>26315</v>
       </c>
       <c r="S31" t="n">
-        <v>26373.8</v>
+        <v>6837.1</v>
       </c>
       <c r="T31" t="n">
-        <v>21818.2</v>
+        <v>19478</v>
       </c>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="n">
-        <v>15.27539782478406</v>
+        <v>22.87384664182015</v>
       </c>
       <c r="W31" t="n">
-        <v>0.06967165766245016</v>
+        <v>0.4769409219308789</v>
       </c>
       <c r="X31" t="n">
-        <v>0.06546474346988973</v>
+        <v>0.04371805125997935</v>
       </c>
       <c r="Y31" t="n">
-        <v>114.9070100143061</v>
+        <v>413.7578616352201</v>
       </c>
       <c r="Z31" t="n">
-        <v>0.6063307856829266</v>
+        <v>1.152705401284587</v>
       </c>
     </row>
     <row r="32">
@@ -3226,7 +3218,7 @@
         <v>26.4910658661689</v>
       </c>
       <c r="K32" t="n">
-        <v>15.22475049779822</v>
+        <v>16.35250979393142</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3242,7 +3234,7 @@
         <v>0.020469</v>
       </c>
       <c r="Q32" t="n">
-        <v>104.4</v>
+        <v>97.2</v>
       </c>
       <c r="R32" t="n">
         <v>49173.8</v>
@@ -3258,13 +3250,13 @@
         <v>63.641894492204</v>
       </c>
       <c r="W32" t="n">
-        <v>0.2537458416299703</v>
+        <v>0.272541829898857</v>
       </c>
       <c r="X32" t="n">
         <v>0.01571292005021155</v>
       </c>
       <c r="Y32" t="n">
-        <v>471.0134099616859</v>
+        <v>505.90329218107</v>
       </c>
       <c r="Z32" t="n">
         <v>0.5387231791354116</v>
@@ -3316,7 +3308,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K33" t="n">
-        <v>10.72308201714094</v>
+        <v>12.18769809753093</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -3332,7 +3324,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q33" t="n">
-        <v>139.8</v>
+        <v>123</v>
       </c>
       <c r="R33" t="n">
         <v>34656</v>
@@ -3348,13 +3340,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W33" t="n">
-        <v>0.1787180336190157</v>
+        <v>0.2031283016255155</v>
       </c>
       <c r="X33" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y33" t="n">
-        <v>247.8969957081545</v>
+        <v>281.7560975609757</v>
       </c>
       <c r="Z33" t="n">
         <v>0.7209366660877885</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-20)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.326003739511734</v>
+        <v>4.391948918467706</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>799.2</v>
+        <v>787.1999999999999</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07210006232519557</v>
+        <v>0.07319914864112843</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>149.1066066066066</v>
+        <v>151.3795731707317</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.735832465515637</v>
+        <v>3.743324108160387</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>899.4</v>
+        <v>897.6</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.06226387442526062</v>
+        <v>0.06238873513600646</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>219.5134534133867</v>
+        <v>219.9536541889483</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.745463925784807</v>
+        <v>6.827725680977306</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>498.0000000000001</v>
+        <v>491.9999999999999</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1124243987630801</v>
+        <v>0.1137954280162884</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>131.8622489959839</v>
+        <v>133.470325203252</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -922,7 +922,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K6" t="n">
-        <v>11.54810258237213</v>
+        <v>11.8546893765944</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -938,7 +938,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q6" t="n">
-        <v>278.4</v>
+        <v>271.2</v>
       </c>
       <c r="R6" t="n">
         <v>35584.1</v>
@@ -954,13 +954,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1924683763728689</v>
+        <v>0.1975781562765734</v>
       </c>
       <c r="X6" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y6" t="n">
-        <v>127.8164511494253</v>
+        <v>131.209808259587</v>
       </c>
       <c r="Z6" t="n">
         <v>1.505818497087371</v>
@@ -1012,7 +1012,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K7" t="n">
-        <v>4.337798858725625</v>
+        <v>4.398592412392843</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1028,7 +1028,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q7" t="n">
-        <v>738</v>
+        <v>727.8000000000001</v>
       </c>
       <c r="R7" t="n">
         <v>78110.8</v>
@@ -1044,13 +1044,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W7" t="n">
-        <v>0.07229664764542709</v>
+        <v>0.07330987353988072</v>
       </c>
       <c r="X7" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y7" t="n">
-        <v>105.8411924119241</v>
+        <v>107.3245397087112</v>
       </c>
       <c r="Z7" t="n">
         <v>0.6830672066132366</v>
@@ -1102,7 +1102,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K8" t="n">
-        <v>5.257239007301819</v>
+        <v>5.30441263747701</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1118,7 +1118,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q8" t="n">
-        <v>607.1999999999999</v>
+        <v>601.8</v>
       </c>
       <c r="R8" t="n">
         <v>60537.6</v>
@@ -1134,13 +1134,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W8" t="n">
-        <v>0.08762065012169698</v>
+        <v>0.08840687729128349</v>
       </c>
       <c r="X8" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y8" t="n">
-        <v>99.69960474308301</v>
+        <v>100.5942173479561</v>
       </c>
       <c r="Z8" t="n">
         <v>0.8788465144619939</v>
@@ -1192,7 +1192,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K9" t="n">
-        <v>7.920852540678647</v>
+        <v>7.826696789823625</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q9" t="n">
-        <v>399</v>
+        <v>403.8</v>
       </c>
       <c r="R9" t="n">
         <v>27205.5</v>
@@ -1224,13 +1224,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1320142090113108</v>
+        <v>0.1304449464970604</v>
       </c>
       <c r="X9" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y9" t="n">
-        <v>68.18421052631579</v>
+        <v>67.37369985141159</v>
       </c>
       <c r="Z9" t="n">
         <v>1.936140464079432</v>
@@ -1281,7 +1281,9 @@
       <c r="J10" t="n">
         <v>52.5605655745982</v>
       </c>
-      <c r="K10" t="inlineStr"/>
+      <c r="K10" t="n">
+        <v>4.369124320415478</v>
+      </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
         <v>8.057855999999999</v>
@@ -1295,7 +1297,9 @@
       <c r="P10" t="n">
         <v>0.355464</v>
       </c>
-      <c r="Q10" t="inlineStr"/>
+      <c r="Q10" t="n">
+        <v>721.8</v>
+      </c>
       <c r="R10" t="n">
         <v>61557.6</v>
       </c>
@@ -1309,11 +1313,15 @@
       <c r="V10" t="n">
         <v>6.522897104961693</v>
       </c>
-      <c r="W10" t="inlineStr"/>
+      <c r="W10" t="n">
+        <v>0.0728187386735913</v>
+      </c>
       <c r="X10" t="n">
         <v>0.1533061128987214</v>
       </c>
-      <c r="Y10" t="inlineStr"/>
+      <c r="Y10" t="n">
+        <v>85.28345802161265</v>
+      </c>
       <c r="Z10" t="n">
         <v>0.8538436452135594</v>
       </c>
@@ -1364,7 +1372,7 @@
         <v>52.393894697293</v>
       </c>
       <c r="K11" t="n">
-        <v>8.396457483540544</v>
+        <v>9.306197992414388</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1380,7 +1388,7 @@
         <v>0.573611</v>
       </c>
       <c r="Q11" t="n">
-        <v>374.4</v>
+        <v>337.8</v>
       </c>
       <c r="R11" t="n">
         <v>54231.7</v>
@@ -1396,13 +1404,13 @@
         <v>1.645610026239954</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1399409580590091</v>
+        <v>0.1551032998735731</v>
       </c>
       <c r="X11" t="n">
         <v>0.6076773865342173</v>
       </c>
       <c r="Y11" t="n">
-        <v>144.849626068376</v>
+        <v>160.5438129070456</v>
       </c>
       <c r="Z11" t="n">
         <v>0.9661119732055791</v>
@@ -1454,7 +1462,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K12" t="n">
-        <v>11.33903197205156</v>
+        <v>11.82535614241043</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1470,7 +1478,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q12" t="n">
-        <v>277.2</v>
+        <v>265.8</v>
       </c>
       <c r="R12" t="n">
         <v>16901.2</v>
@@ -1486,13 +1494,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W12" t="n">
-        <v>0.1889838662008593</v>
+        <v>0.1970892690401738</v>
       </c>
       <c r="X12" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y12" t="n">
-        <v>60.97113997113998</v>
+        <v>63.58615500376224</v>
       </c>
       <c r="Z12" t="n">
         <v>3.099562617499243</v>
@@ -1544,7 +1552,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K13" t="n">
-        <v>7.258119499064181</v>
+        <v>7.445560174793243</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1560,7 +1568,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q13" t="n">
-        <v>429</v>
+        <v>418.2</v>
       </c>
       <c r="R13" t="n">
         <v>74809.60000000001</v>
@@ -1576,13 +1584,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1209686583177364</v>
+        <v>0.1240926695798874</v>
       </c>
       <c r="X13" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y13" t="n">
-        <v>174.381351981352</v>
+        <v>178.8847441415591</v>
       </c>
       <c r="Z13" t="n">
         <v>0.6937018032218979</v>
@@ -1634,7 +1642,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K14" t="n">
-        <v>4.74229274484484</v>
+        <v>4.519028744651621</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1650,7 +1658,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q14" t="n">
-        <v>655.8</v>
+        <v>688.2</v>
       </c>
       <c r="R14" t="n">
         <v>38128.4</v>
@@ -1666,13 +1674,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W14" t="n">
-        <v>0.07903821241408067</v>
+        <v>0.07531714574419368</v>
       </c>
       <c r="X14" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y14" t="n">
-        <v>58.14028667276609</v>
+        <v>55.40308049985469</v>
       </c>
       <c r="Z14" t="n">
         <v>1.359439674918279</v>
@@ -1724,7 +1732,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>3.134045251702335</v>
+        <v>3.322356983564278</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1740,7 +1748,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>889.2</v>
+        <v>838.8000000000001</v>
       </c>
       <c r="R15" t="n">
         <v>80561.39999999999</v>
@@ -1756,13 +1764,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.05223408752837224</v>
+        <v>0.05537261639273795</v>
       </c>
       <c r="X15" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>90.59986504723345</v>
+        <v>96.04363376251787</v>
       </c>
       <c r="Z15" t="n">
         <v>0.5765360412086756</v>
@@ -1814,7 +1822,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>2.297827704912614</v>
+        <v>2.296688474518508</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1830,7 +1838,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1209.6</v>
+        <v>1210.2</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1846,13 +1854,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.03829712841521024</v>
+        <v>0.03827814124197513</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>53.1379794973545</v>
+        <v>53.11163444058833</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1904,7 +1912,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.241531123511539</v>
+        <v>1.319825879048303</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1920,7 +1928,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2194.8</v>
+        <v>2064.6</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1936,13 +1944,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.02069218539185899</v>
+        <v>0.02199709798413838</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>49.0842901403317</v>
+        <v>52.17969582485711</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -1994,7 +2002,7 @@
         <v>45.0965048681912</v>
       </c>
       <c r="K18" t="n">
-        <v>9.055523065901847</v>
+        <v>9.298248426431176</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2010,7 +2018,7 @@
         <v>0.071092</v>
       </c>
       <c r="Q18" t="n">
-        <v>298.8</v>
+        <v>291</v>
       </c>
       <c r="R18" t="n">
         <v>89495.10000000001</v>
@@ -2026,13 +2034,13 @@
         <v>15.02220356103491</v>
       </c>
       <c r="W18" t="n">
-        <v>0.1509253844316975</v>
+        <v>0.1549708071071862</v>
       </c>
       <c r="X18" t="n">
         <v>0.06656813003079209</v>
       </c>
       <c r="Y18" t="n">
-        <v>299.5150602409639</v>
+        <v>307.5432989690722</v>
       </c>
       <c r="Z18" t="n">
         <v>0.5038991505478086</v>
@@ -2174,7 +2182,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K20" t="n">
-        <v>4.173120697916164</v>
+        <v>4.304557570291476</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2190,7 +2198,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q20" t="n">
-        <v>628.8000000000001</v>
+        <v>609.6</v>
       </c>
       <c r="R20" t="n">
         <v>64144.3</v>
@@ -2206,13 +2214,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W20" t="n">
-        <v>0.06955201163193606</v>
+        <v>0.0717426261715246</v>
       </c>
       <c r="X20" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y20" t="n">
-        <v>102.010655216285</v>
+        <v>105.2235892388452</v>
       </c>
       <c r="Z20" t="n">
         <v>0.6818112429968274</v>
@@ -2264,7 +2272,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K21" t="n">
-        <v>2.442230977696258</v>
+        <v>2.367942582937436</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2280,7 +2288,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q21" t="n">
-        <v>1071</v>
+        <v>1104.6</v>
       </c>
       <c r="R21" t="n">
         <v>48455.2</v>
@@ -2296,13 +2304,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W21" t="n">
-        <v>0.04070384962827096</v>
+        <v>0.03946570971562394</v>
       </c>
       <c r="X21" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y21" t="n">
-        <v>45.24295051353874</v>
+        <v>43.86673909107369</v>
       </c>
       <c r="Z21" t="n">
         <v>0.8996727482680539</v>
@@ -2441,9 +2449,11 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>42.3811052132362</v>
-      </c>
-      <c r="K23" t="inlineStr"/>
+        <v>42.7057475126235</v>
+      </c>
+      <c r="K23" t="n">
+        <v>4.462460555133072</v>
+      </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
         <v>1.306119</v>
@@ -2457,7 +2467,9 @@
       <c r="P23" t="n">
         <v>0.032801</v>
       </c>
-      <c r="Q23" t="inlineStr"/>
+      <c r="Q23" t="n">
+        <v>574.2</v>
+      </c>
       <c r="R23" t="n">
         <v>78612.3</v>
       </c>
@@ -2469,15 +2481,19 @@
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="n">
-        <v>32.44811936219915</v>
-      </c>
-      <c r="W23" t="inlineStr"/>
+        <v>32.69667427900789</v>
+      </c>
+      <c r="W23" t="n">
+        <v>0.0743743425855512</v>
+      </c>
       <c r="X23" t="n">
-        <v>0.03081842706622199</v>
-      </c>
-      <c r="Y23" t="inlineStr"/>
+        <v>0.03058415028595205</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>136.9075235109718</v>
+      </c>
       <c r="Z23" t="n">
-        <v>0.5391154464789377</v>
+        <v>0.5432451093864892</v>
       </c>
     </row>
     <row r="24">
@@ -2526,7 +2542,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K24" t="n">
-        <v>3.73948713000492</v>
+        <v>3.773237013849729</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2542,7 +2558,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q24" t="n">
-        <v>670.8</v>
+        <v>664.8</v>
       </c>
       <c r="R24" t="n">
         <v>68673.2</v>
@@ -2558,13 +2574,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W24" t="n">
-        <v>0.062324785500082</v>
+        <v>0.06288728356416216</v>
       </c>
       <c r="X24" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y24" t="n">
-        <v>102.3750745378652</v>
+        <v>103.2990373044525</v>
       </c>
       <c r="Z24" t="n">
         <v>0.6087886703030441</v>
@@ -2616,7 +2632,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K25" t="n">
-        <v>5.240234593673548</v>
+        <v>5.253688341025725</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2632,7 +2648,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q25" t="n">
-        <v>468.6</v>
+        <v>467.4</v>
       </c>
       <c r="R25" t="n">
         <v>71002.60000000001</v>
@@ -2648,13 +2664,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W25" t="n">
-        <v>0.08733724322789246</v>
+        <v>0.08756147235042877</v>
       </c>
       <c r="X25" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y25" t="n">
-        <v>151.5206999573197</v>
+        <v>151.9097133076594</v>
       </c>
       <c r="Z25" t="n">
         <v>0.5764046975264343</v>
@@ -2706,7 +2722,7 @@
         <v>38.8666662997805</v>
       </c>
       <c r="K26" t="n">
-        <v>8.08038800411237</v>
+        <v>8.013745628820722</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2722,7 +2738,7 @@
         <v>0.07819</v>
       </c>
       <c r="Q26" t="n">
-        <v>288.6</v>
+        <v>291</v>
       </c>
       <c r="R26" t="n">
         <v>40335.1</v>
@@ -2738,13 +2754,13 @@
         <v>10.3209696700991</v>
       </c>
       <c r="W26" t="n">
-        <v>0.1346731334018728</v>
+        <v>0.133562427147012</v>
       </c>
       <c r="X26" t="n">
         <v>0.09689012098321557</v>
       </c>
       <c r="Y26" t="n">
-        <v>139.7612612612613</v>
+        <v>138.6085910652921</v>
       </c>
       <c r="Z26" t="n">
         <v>0.9635941475236333</v>
@@ -2796,7 +2812,7 @@
         <v>38.3770408917494</v>
       </c>
       <c r="K27" t="n">
-        <v>3.130264346798483</v>
+        <v>2.71024300082976</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2812,7 +2828,7 @@
         <v>0.217751</v>
       </c>
       <c r="Q27" t="n">
-        <v>735.6</v>
+        <v>849.6</v>
       </c>
       <c r="R27" t="n">
         <v>69464</v>
@@ -2828,13 +2844,13 @@
         <v>6.245463169309107</v>
       </c>
       <c r="W27" t="n">
-        <v>0.05217107244664138</v>
+        <v>0.045170716680496</v>
       </c>
       <c r="X27" t="n">
         <v>0.1601162272342122</v>
       </c>
       <c r="Y27" t="n">
-        <v>94.43175638934203</v>
+        <v>81.7608286252354</v>
       </c>
       <c r="Z27" t="n">
         <v>0.5524738122156715</v>
@@ -2886,7 +2902,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K28" t="n">
-        <v>5.785207691498301</v>
+        <v>5.664861617678127</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2902,7 +2918,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q28" t="n">
-        <v>395.4</v>
+        <v>403.8</v>
       </c>
       <c r="R28" t="n">
         <v>50011.7</v>
@@ -2918,13 +2934,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W28" t="n">
-        <v>0.09642012819163835</v>
+        <v>0.09441436029463546</v>
       </c>
       <c r="X28" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y28" t="n">
-        <v>126.4838138593829</v>
+        <v>123.8526498266468</v>
       </c>
       <c r="Z28" t="n">
         <v>0.7623119927331765</v>
@@ -2976,7 +2992,7 @@
         <v>33.6762858057476</v>
       </c>
       <c r="K29" t="n">
-        <v>1.669622499045493</v>
+        <v>1.720811742756648</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -2992,7 +3008,7 @@
         <v>0.143075</v>
       </c>
       <c r="Q29" t="n">
-        <v>1210.2</v>
+        <v>1174.2</v>
       </c>
       <c r="R29" t="n">
         <v>66783.2</v>
@@ -3008,13 +3024,13 @@
         <v>13.43904545346521</v>
       </c>
       <c r="W29" t="n">
-        <v>0.02782704165075822</v>
+        <v>0.0286801957126108</v>
       </c>
       <c r="X29" t="n">
         <v>0.07441004671519687</v>
       </c>
       <c r="Y29" t="n">
-        <v>55.18360601553461</v>
+        <v>56.87548969511156</v>
       </c>
       <c r="Z29" t="n">
         <v>0.5042628356494987</v>
@@ -3128,7 +3144,7 @@
         <v>30.3334426348039</v>
       </c>
       <c r="K31" t="n">
-        <v>28.61645531585274</v>
+        <v>31.59733607792074</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3144,7 +3160,7 @@
         <v>0.040904</v>
       </c>
       <c r="Q31" t="n">
-        <v>63.6</v>
+        <v>57.59999999999999</v>
       </c>
       <c r="R31" t="n">
         <v>26315</v>
@@ -3160,13 +3176,13 @@
         <v>22.87384664182015</v>
       </c>
       <c r="W31" t="n">
-        <v>0.4769409219308789</v>
+        <v>0.5266222679653456</v>
       </c>
       <c r="X31" t="n">
         <v>0.04371805125997935</v>
       </c>
       <c r="Y31" t="n">
-        <v>413.7578616352201</v>
+        <v>456.8576388888889</v>
       </c>
       <c r="Z31" t="n">
         <v>1.152705401284587</v>
@@ -3218,7 +3234,7 @@
         <v>26.4910658661689</v>
       </c>
       <c r="K32" t="n">
-        <v>16.35250979393142</v>
+        <v>16.15308894278591</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3234,7 +3250,7 @@
         <v>0.020469</v>
       </c>
       <c r="Q32" t="n">
-        <v>97.2</v>
+        <v>98.39999999999999</v>
       </c>
       <c r="R32" t="n">
         <v>49173.8</v>
@@ -3250,13 +3266,13 @@
         <v>63.641894492204</v>
       </c>
       <c r="W32" t="n">
-        <v>0.272541829898857</v>
+        <v>0.2692181490464319</v>
       </c>
       <c r="X32" t="n">
         <v>0.01571292005021155</v>
       </c>
       <c r="Y32" t="n">
-        <v>505.90329218107</v>
+        <v>499.7337398373984</v>
       </c>
       <c r="Z32" t="n">
         <v>0.5387231791354116</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-21)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.391948918467706</v>
+        <v>4.335768984973386</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>787.1999999999999</v>
+        <v>797.4</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07319914864112843</v>
+        <v>0.07226281641622311</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>151.3795731707317</v>
+        <v>149.4431903686983</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.743324108160387</v>
+        <v>3.589751837056372</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>897.6</v>
+        <v>936</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.06238873513600646</v>
+        <v>0.05982919728427286</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>219.9536541889483</v>
+        <v>210.9299145299145</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.827725680977306</v>
+        <v>6.786345525335019</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>491.9999999999999</v>
+        <v>495</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1137954280162884</v>
+        <v>0.1131057587555836</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>133.470325203252</v>
+        <v>132.6614141414141</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -922,7 +922,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K6" t="n">
-        <v>11.8546893765944</v>
+        <v>11.69938776904077</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -938,7 +938,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q6" t="n">
-        <v>271.2</v>
+        <v>274.8</v>
       </c>
       <c r="R6" t="n">
         <v>35584.1</v>
@@ -954,13 +954,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1975781562765734</v>
+        <v>0.1949897961506794</v>
       </c>
       <c r="X6" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y6" t="n">
-        <v>131.209808259587</v>
+        <v>129.4909024745269</v>
       </c>
       <c r="Z6" t="n">
         <v>1.505818497087371</v>
@@ -1012,7 +1012,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K7" t="n">
-        <v>4.398592412392843</v>
+        <v>4.351951546682316</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1028,7 +1028,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q7" t="n">
-        <v>727.8000000000001</v>
+        <v>735.6</v>
       </c>
       <c r="R7" t="n">
         <v>78110.8</v>
@@ -1044,13 +1044,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W7" t="n">
-        <v>0.07330987353988072</v>
+        <v>0.07253252577803861</v>
       </c>
       <c r="X7" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y7" t="n">
-        <v>107.3245397087112</v>
+        <v>106.1865144100054</v>
       </c>
       <c r="Z7" t="n">
         <v>0.6830672066132366</v>
@@ -1102,7 +1102,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K8" t="n">
-        <v>5.30441263747701</v>
+        <v>5.272870044984579</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1118,7 +1118,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q8" t="n">
-        <v>601.8</v>
+        <v>605.4</v>
       </c>
       <c r="R8" t="n">
         <v>60537.6</v>
@@ -1134,13 +1134,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W8" t="n">
-        <v>0.08840687729128349</v>
+        <v>0.08788116741640965</v>
       </c>
       <c r="X8" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y8" t="n">
-        <v>100.5942173479561</v>
+        <v>99.99603567889</v>
       </c>
       <c r="Z8" t="n">
         <v>0.8788465144619939</v>
@@ -1192,7 +1192,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K9" t="n">
-        <v>7.826696789823625</v>
+        <v>7.12769545270812</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q9" t="n">
-        <v>403.8</v>
+        <v>443.4</v>
       </c>
       <c r="R9" t="n">
         <v>27205.5</v>
@@ -1224,13 +1224,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1304449464970604</v>
+        <v>0.118794924211802</v>
       </c>
       <c r="X9" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y9" t="n">
-        <v>67.37369985141159</v>
+        <v>61.35656292286875</v>
       </c>
       <c r="Z9" t="n">
         <v>1.936140464079432</v>
@@ -1462,7 +1462,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K12" t="n">
-        <v>11.82535614241043</v>
+        <v>10.11319067777572</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1478,7 +1478,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q12" t="n">
-        <v>265.8</v>
+        <v>310.8</v>
       </c>
       <c r="R12" t="n">
         <v>16901.2</v>
@@ -1494,13 +1494,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W12" t="n">
-        <v>0.1970892690401738</v>
+        <v>0.1685531779629286</v>
       </c>
       <c r="X12" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y12" t="n">
-        <v>63.58615500376224</v>
+        <v>54.37966537966539</v>
       </c>
       <c r="Z12" t="n">
         <v>3.099562617499243</v>
@@ -1552,7 +1552,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K13" t="n">
-        <v>7.445560174793243</v>
+        <v>7.19771905940484</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1568,7 +1568,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q13" t="n">
-        <v>418.2</v>
+        <v>432.6</v>
       </c>
       <c r="R13" t="n">
         <v>74809.60000000001</v>
@@ -1584,13 +1584,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1240926695798874</v>
+        <v>0.119961984323414</v>
       </c>
       <c r="X13" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y13" t="n">
-        <v>178.8847441415591</v>
+        <v>172.9301895515488</v>
       </c>
       <c r="Z13" t="n">
         <v>0.6937018032218979</v>
@@ -1642,7 +1642,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K14" t="n">
-        <v>4.519028744651621</v>
+        <v>4.483845994909524</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1658,7 +1658,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q14" t="n">
-        <v>688.2</v>
+        <v>693.6</v>
       </c>
       <c r="R14" t="n">
         <v>38128.4</v>
@@ -1674,13 +1674,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W14" t="n">
-        <v>0.07531714574419368</v>
+        <v>0.0747307665818254</v>
       </c>
       <c r="X14" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y14" t="n">
-        <v>55.40308049985469</v>
+        <v>54.97174163783161</v>
       </c>
       <c r="Z14" t="n">
         <v>1.359439674918279</v>
@@ -1732,7 +1732,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>3.322356983564278</v>
+        <v>3.270883847199197</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1748,7 +1748,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>838.8000000000001</v>
+        <v>852</v>
       </c>
       <c r="R15" t="n">
         <v>80561.39999999999</v>
@@ -1764,13 +1764,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.05537261639273795</v>
+        <v>0.05451473078665329</v>
       </c>
       <c r="X15" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>96.04363376251787</v>
+        <v>94.5556338028169</v>
       </c>
       <c r="Z15" t="n">
         <v>0.5765360412086756</v>
@@ -1822,7 +1822,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>2.296688474518508</v>
+        <v>2.261924147023354</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1838,7 +1838,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1210.2</v>
+        <v>1228.8</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1854,13 +1854,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.03827814124197513</v>
+        <v>0.03769873578372258</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>53.11163444058833</v>
+        <v>52.30769856770834</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1912,7 +1912,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.319825879048303</v>
+        <v>1.326378752863671</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1928,7 +1928,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2064.6</v>
+        <v>2054.4</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1944,13 +1944,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.02199709798413838</v>
+        <v>0.02210631254772785</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>52.17969582485711</v>
+        <v>52.43876557632398</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -2002,7 +2002,7 @@
         <v>45.0965048681912</v>
       </c>
       <c r="K18" t="n">
-        <v>9.298248426431176</v>
+        <v>8.912352740749249</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2018,7 +2018,7 @@
         <v>0.071092</v>
       </c>
       <c r="Q18" t="n">
-        <v>291</v>
+        <v>303.6</v>
       </c>
       <c r="R18" t="n">
         <v>89495.10000000001</v>
@@ -2034,13 +2034,13 @@
         <v>15.02220356103491</v>
       </c>
       <c r="W18" t="n">
-        <v>0.1549708071071862</v>
+        <v>0.1485392123458208</v>
       </c>
       <c r="X18" t="n">
         <v>0.06656813003079209</v>
       </c>
       <c r="Y18" t="n">
-        <v>307.5432989690722</v>
+        <v>294.7796442687747</v>
       </c>
       <c r="Z18" t="n">
         <v>0.5038991505478086</v>
@@ -2092,7 +2092,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K19" t="n">
-        <v>4.773709209553731</v>
+        <v>4.518404882503935</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2108,7 +2108,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q19" t="n">
-        <v>562.8000000000001</v>
+        <v>594.6</v>
       </c>
       <c r="R19" t="n">
         <v>71127.60000000001</v>
@@ -2124,13 +2124,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W19" t="n">
-        <v>0.07956182015922884</v>
+        <v>0.07530674804173225</v>
       </c>
       <c r="X19" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y19" t="n">
-        <v>126.3816631130064</v>
+        <v>119.6226034308779</v>
       </c>
       <c r="Z19" t="n">
         <v>0.629536106737947</v>
@@ -2182,7 +2182,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K20" t="n">
-        <v>4.304557570291476</v>
+        <v>4.157253318836635</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2198,7 +2198,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q20" t="n">
-        <v>609.6</v>
+        <v>631.1999999999999</v>
       </c>
       <c r="R20" t="n">
         <v>64144.3</v>
@@ -2214,13 +2214,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W20" t="n">
-        <v>0.0717426261715246</v>
+        <v>0.06928755531394393</v>
       </c>
       <c r="X20" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y20" t="n">
-        <v>105.2235892388452</v>
+        <v>101.6227820025349</v>
       </c>
       <c r="Z20" t="n">
         <v>0.6818112429968274</v>
@@ -2272,7 +2272,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K21" t="n">
-        <v>2.367942582937436</v>
+        <v>2.298040218865483</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2288,7 +2288,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q21" t="n">
-        <v>1104.6</v>
+        <v>1138.2</v>
       </c>
       <c r="R21" t="n">
         <v>48455.2</v>
@@ -2304,13 +2304,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W21" t="n">
-        <v>0.03946570971562394</v>
+        <v>0.03830067031442471</v>
       </c>
       <c r="X21" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y21" t="n">
-        <v>43.86673909107369</v>
+        <v>42.57178000351433</v>
       </c>
       <c r="Z21" t="n">
         <v>0.8996727482680539</v>
@@ -2362,7 +2362,7 @@
         <v>43.3950199670746</v>
       </c>
       <c r="K22" t="n">
-        <v>6.120595199869479</v>
+        <v>6.035468701957525</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2378,7 +2378,7 @@
         <v>0.064523</v>
       </c>
       <c r="Q22" t="n">
-        <v>425.4</v>
+        <v>431.4</v>
       </c>
       <c r="R22" t="n">
         <v>162164.2</v>
@@ -2394,13 +2394,13 @@
         <v>40.74733935074209</v>
       </c>
       <c r="W22" t="n">
-        <v>0.1020099199978246</v>
+        <v>0.1005911450326254</v>
       </c>
       <c r="X22" t="n">
         <v>0.02454147966305898</v>
       </c>
       <c r="Y22" t="n">
-        <v>381.2040432534086</v>
+        <v>375.9021789522485</v>
       </c>
       <c r="Z22" t="n">
         <v>0.2675992602995889</v>
@@ -2452,7 +2452,7 @@
         <v>42.7057475126235</v>
       </c>
       <c r="K23" t="n">
-        <v>4.462460555133072</v>
+        <v>4.162353558735234</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2468,7 +2468,7 @@
         <v>0.032801</v>
       </c>
       <c r="Q23" t="n">
-        <v>574.2</v>
+        <v>615.6</v>
       </c>
       <c r="R23" t="n">
         <v>78612.3</v>
@@ -2484,13 +2484,13 @@
         <v>32.69667427900789</v>
       </c>
       <c r="W23" t="n">
-        <v>0.0743743425855512</v>
+        <v>0.0693725593122539</v>
       </c>
       <c r="X23" t="n">
         <v>0.03058415028595205</v>
       </c>
       <c r="Y23" t="n">
-        <v>136.9075235109718</v>
+        <v>127.7002923976608</v>
       </c>
       <c r="Z23" t="n">
         <v>0.5432451093864892</v>
@@ -2542,7 +2542,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K24" t="n">
-        <v>3.773237013849729</v>
+        <v>3.498532729159415</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2558,7 +2558,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q24" t="n">
-        <v>664.8</v>
+        <v>717</v>
       </c>
       <c r="R24" t="n">
         <v>68673.2</v>
@@ -2574,13 +2574,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W24" t="n">
-        <v>0.06288728356416216</v>
+        <v>0.05830887881932357</v>
       </c>
       <c r="X24" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y24" t="n">
-        <v>103.2990373044525</v>
+        <v>95.77852161785216</v>
       </c>
       <c r="Z24" t="n">
         <v>0.6087886703030441</v>
@@ -2632,7 +2632,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K25" t="n">
-        <v>5.253688341025725</v>
+        <v>5.027792650686782</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2648,7 +2648,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q25" t="n">
-        <v>467.4</v>
+        <v>488.4</v>
       </c>
       <c r="R25" t="n">
         <v>71002.60000000001</v>
@@ -2664,13 +2664,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W25" t="n">
-        <v>0.08756147235042877</v>
+        <v>0.08379654417811302</v>
       </c>
       <c r="X25" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y25" t="n">
-        <v>151.9097133076594</v>
+        <v>145.3779688779689</v>
       </c>
       <c r="Z25" t="n">
         <v>0.5764046975264343</v>
@@ -2722,7 +2722,7 @@
         <v>38.8666662997805</v>
       </c>
       <c r="K26" t="n">
-        <v>8.013745628820722</v>
+        <v>7.742363804737152</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2738,7 +2738,7 @@
         <v>0.07819</v>
       </c>
       <c r="Q26" t="n">
-        <v>291</v>
+        <v>301.2</v>
       </c>
       <c r="R26" t="n">
         <v>40335.1</v>
@@ -2754,13 +2754,13 @@
         <v>10.3209696700991</v>
       </c>
       <c r="W26" t="n">
-        <v>0.133562427147012</v>
+        <v>0.1290393967456192</v>
       </c>
       <c r="X26" t="n">
         <v>0.09689012098321557</v>
       </c>
       <c r="Y26" t="n">
-        <v>138.6085910652921</v>
+        <v>133.9146746347942</v>
       </c>
       <c r="Z26" t="n">
         <v>0.9635941475236333</v>
@@ -2812,7 +2812,7 @@
         <v>38.3770408917494</v>
       </c>
       <c r="K27" t="n">
-        <v>2.71024300082976</v>
+        <v>2.485559643248018</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2828,7 +2828,7 @@
         <v>0.217751</v>
       </c>
       <c r="Q27" t="n">
-        <v>849.6</v>
+        <v>926.4</v>
       </c>
       <c r="R27" t="n">
         <v>69464</v>
@@ -2844,13 +2844,13 @@
         <v>6.245463169309107</v>
       </c>
       <c r="W27" t="n">
-        <v>0.045170716680496</v>
+        <v>0.04142599405413364</v>
       </c>
       <c r="X27" t="n">
         <v>0.1601162272342122</v>
       </c>
       <c r="Y27" t="n">
-        <v>81.7608286252354</v>
+        <v>74.98272884283247</v>
       </c>
       <c r="Z27" t="n">
         <v>0.5524738122156715</v>
@@ -2902,7 +2902,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K28" t="n">
-        <v>5.664861617678127</v>
+        <v>5.469801820225797</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2918,7 +2918,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q28" t="n">
-        <v>403.8</v>
+        <v>418.2</v>
       </c>
       <c r="R28" t="n">
         <v>50011.7</v>
@@ -2934,13 +2934,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W28" t="n">
-        <v>0.09441436029463546</v>
+        <v>0.09116336367042994</v>
       </c>
       <c r="X28" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y28" t="n">
-        <v>123.8526498266468</v>
+        <v>119.5879961740794</v>
       </c>
       <c r="Z28" t="n">
         <v>0.7623119927331765</v>
@@ -2992,7 +2992,7 @@
         <v>33.6762858057476</v>
       </c>
       <c r="K29" t="n">
-        <v>1.720811742756648</v>
+        <v>1.705992188741013</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -3008,7 +3008,7 @@
         <v>0.143075</v>
       </c>
       <c r="Q29" t="n">
-        <v>1174.2</v>
+        <v>1184.4</v>
       </c>
       <c r="R29" t="n">
         <v>66783.2</v>
@@ -3024,13 +3024,13 @@
         <v>13.43904545346521</v>
       </c>
       <c r="W29" t="n">
-        <v>0.0286801957126108</v>
+        <v>0.02843320314568355</v>
       </c>
       <c r="X29" t="n">
         <v>0.07441004671519687</v>
       </c>
       <c r="Y29" t="n">
-        <v>56.87548969511156</v>
+        <v>56.38568051334009</v>
       </c>
       <c r="Z29" t="n">
         <v>0.5042628356494987</v>
@@ -3144,7 +3144,7 @@
         <v>30.3334426348039</v>
       </c>
       <c r="K31" t="n">
-        <v>31.59733607792074</v>
+        <v>29.44994430563485</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3160,7 +3160,7 @@
         <v>0.040904</v>
       </c>
       <c r="Q31" t="n">
-        <v>57.59999999999999</v>
+        <v>61.8</v>
       </c>
       <c r="R31" t="n">
         <v>26315</v>
@@ -3176,13 +3176,13 @@
         <v>22.87384664182015</v>
       </c>
       <c r="W31" t="n">
-        <v>0.5266222679653456</v>
+        <v>0.4908324050939142</v>
       </c>
       <c r="X31" t="n">
         <v>0.04371805125997935</v>
       </c>
       <c r="Y31" t="n">
-        <v>456.8576388888889</v>
+        <v>425.8090614886731</v>
       </c>
       <c r="Z31" t="n">
         <v>1.152705401284587</v>
@@ -3234,7 +3234,7 @@
         <v>26.4910658661689</v>
       </c>
       <c r="K32" t="n">
-        <v>16.15308894278591</v>
+        <v>15.86291369231671</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3250,7 +3250,7 @@
         <v>0.020469</v>
       </c>
       <c r="Q32" t="n">
-        <v>98.39999999999999</v>
+        <v>100.2</v>
       </c>
       <c r="R32" t="n">
         <v>49173.8</v>
@@ -3266,13 +3266,13 @@
         <v>63.641894492204</v>
       </c>
       <c r="W32" t="n">
-        <v>0.2692181490464319</v>
+        <v>0.2643818948719451</v>
       </c>
       <c r="X32" t="n">
         <v>0.01571292005021155</v>
       </c>
       <c r="Y32" t="n">
-        <v>499.7337398373984</v>
+        <v>490.7564870259482</v>
       </c>
       <c r="Z32" t="n">
         <v>0.5387231791354116</v>
@@ -3324,7 +3324,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K33" t="n">
-        <v>12.18769809753093</v>
+        <v>11.20393771297686</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -3340,7 +3340,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q33" t="n">
-        <v>123</v>
+        <v>133.8</v>
       </c>
       <c r="R33" t="n">
         <v>34656</v>
@@ -3356,13 +3356,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W33" t="n">
-        <v>0.2031283016255155</v>
+        <v>0.186732295216281</v>
       </c>
       <c r="X33" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y33" t="n">
-        <v>281.7560975609757</v>
+        <v>259.0134529147982</v>
       </c>
       <c r="Z33" t="n">
         <v>0.7209366660877885</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-22)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.335768984973386</v>
+        <v>4.339033871257252</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>797.4</v>
+        <v>796.8</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07226281641622311</v>
+        <v>0.07231723118762086</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>149.4431903686983</v>
+        <v>149.5557228915663</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.589751837056372</v>
+        <v>3.573715932232253</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>936</v>
+        <v>940.2</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.05982919728427286</v>
+        <v>0.05956193220387087</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>210.9299145299145</v>
+        <v>209.987662199532</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.786345525335019</v>
+        <v>6.697051505264821</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>495</v>
+        <v>501.6</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1131057587555836</v>
+        <v>0.111617525087747</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>132.6614141414141</v>
+        <v>130.9158692185008</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -922,7 +922,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K6" t="n">
-        <v>11.69938776904077</v>
+        <v>11.3283712435955</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -938,7 +938,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q6" t="n">
-        <v>274.8</v>
+        <v>283.8</v>
       </c>
       <c r="R6" t="n">
         <v>35584.1</v>
@@ -954,13 +954,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1949897961506794</v>
+        <v>0.1888061873932583</v>
       </c>
       <c r="X6" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y6" t="n">
-        <v>129.4909024745269</v>
+        <v>125.3844256518675</v>
       </c>
       <c r="Z6" t="n">
         <v>1.505818497087371</v>
@@ -1012,7 +1012,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K7" t="n">
-        <v>4.351951546682316</v>
+        <v>4.449952123630124</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1028,7 +1028,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q7" t="n">
-        <v>735.6</v>
+        <v>719.4</v>
       </c>
       <c r="R7" t="n">
         <v>78110.8</v>
@@ -1044,13 +1044,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W7" t="n">
-        <v>0.07253252577803861</v>
+        <v>0.07416586872716875</v>
       </c>
       <c r="X7" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y7" t="n">
-        <v>106.1865144100054</v>
+        <v>108.5777036419238</v>
       </c>
       <c r="Z7" t="n">
         <v>0.6830672066132366</v>
@@ -1102,7 +1102,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K8" t="n">
-        <v>5.272870044984579</v>
+        <v>5.26243904588471</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1118,7 +1118,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q8" t="n">
-        <v>605.4</v>
+        <v>606.5999999999999</v>
       </c>
       <c r="R8" t="n">
         <v>60537.6</v>
@@ -1134,13 +1134,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W8" t="n">
-        <v>0.08788116741640965</v>
+        <v>0.08770731743141182</v>
       </c>
       <c r="X8" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y8" t="n">
-        <v>99.99603567889</v>
+        <v>99.79821958456975</v>
       </c>
       <c r="Z8" t="n">
         <v>0.8788465144619939</v>
@@ -1192,7 +1192,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K9" t="n">
-        <v>7.12769545270812</v>
+        <v>6.592449235984105</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q9" t="n">
-        <v>443.4</v>
+        <v>479.4</v>
       </c>
       <c r="R9" t="n">
         <v>27205.5</v>
@@ -1224,13 +1224,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W9" t="n">
-        <v>0.118794924211802</v>
+        <v>0.1098741539330684</v>
       </c>
       <c r="X9" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y9" t="n">
-        <v>61.35656292286875</v>
+        <v>56.74906132665832</v>
       </c>
       <c r="Z9" t="n">
         <v>1.936140464079432</v>
@@ -1372,7 +1372,7 @@
         <v>52.393894697293</v>
       </c>
       <c r="K11" t="n">
-        <v>9.306197992414388</v>
+        <v>8.805696587780336</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1388,7 +1388,7 @@
         <v>0.573611</v>
       </c>
       <c r="Q11" t="n">
-        <v>337.8</v>
+        <v>357</v>
       </c>
       <c r="R11" t="n">
         <v>54231.7</v>
@@ -1404,13 +1404,13 @@
         <v>1.645610026239954</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1551032998735731</v>
+        <v>0.1467616097963389</v>
       </c>
       <c r="X11" t="n">
         <v>0.6076773865342173</v>
       </c>
       <c r="Y11" t="n">
-        <v>160.5438129070456</v>
+        <v>151.9095238095238</v>
       </c>
       <c r="Z11" t="n">
         <v>0.9661119732055791</v>
@@ -1462,7 +1462,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K12" t="n">
-        <v>10.11319067777572</v>
+        <v>9.773568602775782</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1478,7 +1478,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q12" t="n">
-        <v>310.8</v>
+        <v>321.6</v>
       </c>
       <c r="R12" t="n">
         <v>16901.2</v>
@@ -1494,13 +1494,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W12" t="n">
-        <v>0.1685531779629286</v>
+        <v>0.162892810046263</v>
       </c>
       <c r="X12" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y12" t="n">
-        <v>54.37966537966539</v>
+        <v>52.55348258706468</v>
       </c>
       <c r="Z12" t="n">
         <v>3.099562617499243</v>
@@ -1552,7 +1552,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K13" t="n">
-        <v>7.19771905940484</v>
+        <v>7.0510264155311</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1568,7 +1568,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q13" t="n">
-        <v>432.6</v>
+        <v>441.6</v>
       </c>
       <c r="R13" t="n">
         <v>74809.60000000001</v>
@@ -1584,13 +1584,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W13" t="n">
-        <v>0.119961984323414</v>
+        <v>0.1175171069255183</v>
       </c>
       <c r="X13" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y13" t="n">
-        <v>172.9301895515488</v>
+        <v>169.4057971014493</v>
       </c>
       <c r="Z13" t="n">
         <v>0.6937018032218979</v>
@@ -1732,7 +1732,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>3.270883847199197</v>
+        <v>3.11721816310259</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1748,7 +1748,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>852</v>
+        <v>894</v>
       </c>
       <c r="R15" t="n">
         <v>80561.39999999999</v>
@@ -1764,13 +1764,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.05451473078665329</v>
+        <v>0.05195363605170984</v>
       </c>
       <c r="X15" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>94.5556338028169</v>
+        <v>90.11342281879195</v>
       </c>
       <c r="Z15" t="n">
         <v>0.5765360412086756</v>
@@ -1822,7 +1822,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>2.261924147023354</v>
+        <v>2.135740273445749</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1838,7 +1838,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1228.8</v>
+        <v>1301.4</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1854,13 +1854,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.03769873578372258</v>
+        <v>0.03559567122409582</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>52.30769856770834</v>
+        <v>49.38965729214691</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1912,7 +1912,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.326378752863671</v>
+        <v>1.289838355525479</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1928,7 +1928,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2054.4</v>
+        <v>2112.6</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1944,13 +1944,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.02210631254772785</v>
+        <v>0.02149730592542464</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>52.43876557632398</v>
+        <v>50.99413045536306</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -2002,7 +2002,7 @@
         <v>45.0965048681912</v>
       </c>
       <c r="K18" t="n">
-        <v>8.912352740749249</v>
+        <v>8.429253246390878</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2018,7 +2018,7 @@
         <v>0.071092</v>
       </c>
       <c r="Q18" t="n">
-        <v>303.6</v>
+        <v>321</v>
       </c>
       <c r="R18" t="n">
         <v>89495.10000000001</v>
@@ -2034,13 +2034,13 @@
         <v>15.02220356103491</v>
       </c>
       <c r="W18" t="n">
-        <v>0.1485392123458208</v>
+        <v>0.1404875541065146</v>
       </c>
       <c r="X18" t="n">
         <v>0.06656813003079209</v>
       </c>
       <c r="Y18" t="n">
-        <v>294.7796442687747</v>
+        <v>278.8009345794393</v>
       </c>
       <c r="Z18" t="n">
         <v>0.5038991505478086</v>
@@ -2092,7 +2092,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K19" t="n">
-        <v>4.518404882503935</v>
+        <v>4.161467693830297</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2108,7 +2108,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q19" t="n">
-        <v>594.6</v>
+        <v>645.6</v>
       </c>
       <c r="R19" t="n">
         <v>71127.60000000001</v>
@@ -2124,13 +2124,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W19" t="n">
-        <v>0.07530674804173225</v>
+        <v>0.06935779489717162</v>
       </c>
       <c r="X19" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y19" t="n">
-        <v>119.6226034308779</v>
+        <v>110.1728624535316</v>
       </c>
       <c r="Z19" t="n">
         <v>0.629536106737947</v>
@@ -2182,7 +2182,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K20" t="n">
-        <v>4.157253318836635</v>
+        <v>4.536753621800974</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2198,7 +2198,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q20" t="n">
-        <v>631.1999999999999</v>
+        <v>578.4000000000001</v>
       </c>
       <c r="R20" t="n">
         <v>64144.3</v>
@@ -2214,13 +2214,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W20" t="n">
-        <v>0.06928755531394393</v>
+        <v>0.07561256036334957</v>
       </c>
       <c r="X20" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y20" t="n">
-        <v>101.6227820025349</v>
+        <v>110.899550484094</v>
       </c>
       <c r="Z20" t="n">
         <v>0.6818112429968274</v>
@@ -2272,7 +2272,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K21" t="n">
-        <v>2.298040218865483</v>
+        <v>2.227584208067358</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2288,7 +2288,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q21" t="n">
-        <v>1138.2</v>
+        <v>1174.2</v>
       </c>
       <c r="R21" t="n">
         <v>48455.2</v>
@@ -2304,13 +2304,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W21" t="n">
-        <v>0.03830067031442471</v>
+        <v>0.0371264034677893</v>
       </c>
       <c r="X21" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y21" t="n">
-        <v>42.57178000351433</v>
+        <v>41.26656446942599</v>
       </c>
       <c r="Z21" t="n">
         <v>0.8996727482680539</v>
@@ -2362,7 +2362,7 @@
         <v>43.3950199670746</v>
       </c>
       <c r="K22" t="n">
-        <v>6.035468701957525</v>
+        <v>6.052304040038299</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2378,7 +2378,7 @@
         <v>0.064523</v>
       </c>
       <c r="Q22" t="n">
-        <v>431.4</v>
+        <v>430.2</v>
       </c>
       <c r="R22" t="n">
         <v>162164.2</v>
@@ -2394,13 +2394,13 @@
         <v>40.74733935074209</v>
       </c>
       <c r="W22" t="n">
-        <v>0.1005911450326254</v>
+        <v>0.1008717340006383</v>
       </c>
       <c r="X22" t="n">
         <v>0.02454147966305898</v>
       </c>
       <c r="Y22" t="n">
-        <v>375.9021789522485</v>
+        <v>376.9507205950721</v>
       </c>
       <c r="Z22" t="n">
         <v>0.2675992602995889</v>
@@ -2452,7 +2452,7 @@
         <v>42.7057475126235</v>
       </c>
       <c r="K23" t="n">
-        <v>4.162353558735234</v>
+        <v>4.074975907693082</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2468,7 +2468,7 @@
         <v>0.032801</v>
       </c>
       <c r="Q23" t="n">
-        <v>615.6</v>
+        <v>628.8000000000001</v>
       </c>
       <c r="R23" t="n">
         <v>78612.3</v>
@@ -2484,13 +2484,13 @@
         <v>32.69667427900789</v>
       </c>
       <c r="W23" t="n">
-        <v>0.0693725593122539</v>
+        <v>0.06791626512821804</v>
       </c>
       <c r="X23" t="n">
         <v>0.03058415028595205</v>
       </c>
       <c r="Y23" t="n">
-        <v>127.7002923976608</v>
+        <v>125.0195610687023</v>
       </c>
       <c r="Z23" t="n">
         <v>0.5432451093864892</v>
@@ -2542,7 +2542,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K24" t="n">
-        <v>3.498532729159415</v>
+        <v>3.191409626981298</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2558,7 +2558,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q24" t="n">
-        <v>717</v>
+        <v>786</v>
       </c>
       <c r="R24" t="n">
         <v>68673.2</v>
@@ -2574,13 +2574,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W24" t="n">
-        <v>0.05830887881932357</v>
+        <v>0.05319016044968829</v>
       </c>
       <c r="X24" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y24" t="n">
-        <v>95.77852161785216</v>
+        <v>87.3704834605598</v>
       </c>
       <c r="Z24" t="n">
         <v>0.6087886703030441</v>
@@ -2632,7 +2632,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K25" t="n">
-        <v>5.027792650686782</v>
+        <v>4.913113106433422</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2648,7 +2648,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q25" t="n">
-        <v>488.4</v>
+        <v>499.8</v>
       </c>
       <c r="R25" t="n">
         <v>71002.60000000001</v>
@@ -2664,13 +2664,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W25" t="n">
-        <v>0.08379654417811302</v>
+        <v>0.08188521844055703</v>
       </c>
       <c r="X25" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y25" t="n">
-        <v>145.3779688779689</v>
+        <v>142.062024809924</v>
       </c>
       <c r="Z25" t="n">
         <v>0.5764046975264343</v>
@@ -2722,7 +2722,7 @@
         <v>38.8666662997805</v>
       </c>
       <c r="K26" t="n">
-        <v>7.742363804737152</v>
+        <v>7.576348206584893</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2738,7 +2738,7 @@
         <v>0.07819</v>
       </c>
       <c r="Q26" t="n">
-        <v>301.2</v>
+        <v>307.8</v>
       </c>
       <c r="R26" t="n">
         <v>40335.1</v>
@@ -2754,13 +2754,13 @@
         <v>10.3209696700991</v>
       </c>
       <c r="W26" t="n">
-        <v>0.1290393967456192</v>
+        <v>0.1262724701097482</v>
       </c>
       <c r="X26" t="n">
         <v>0.09689012098321557</v>
       </c>
       <c r="Y26" t="n">
-        <v>133.9146746347942</v>
+        <v>131.0432098765432</v>
       </c>
       <c r="Z26" t="n">
         <v>0.9635941475236333</v>
@@ -2812,7 +2812,7 @@
         <v>38.3770408917494</v>
       </c>
       <c r="K27" t="n">
-        <v>2.485559643248018</v>
+        <v>2.780944992155754</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2828,7 +2828,7 @@
         <v>0.217751</v>
       </c>
       <c r="Q27" t="n">
-        <v>926.4</v>
+        <v>828</v>
       </c>
       <c r="R27" t="n">
         <v>69464</v>
@@ -2844,13 +2844,13 @@
         <v>6.245463169309107</v>
       </c>
       <c r="W27" t="n">
-        <v>0.04142599405413364</v>
+        <v>0.0463490832025959</v>
       </c>
       <c r="X27" t="n">
         <v>0.1601162272342122</v>
       </c>
       <c r="Y27" t="n">
-        <v>74.98272884283247</v>
+        <v>83.89371980676329</v>
       </c>
       <c r="Z27" t="n">
         <v>0.5524738122156715</v>
@@ -2902,7 +2902,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K28" t="n">
-        <v>5.469801820225797</v>
+        <v>5.493446496682104</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2918,7 +2918,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q28" t="n">
-        <v>418.2</v>
+        <v>416.4</v>
       </c>
       <c r="R28" t="n">
         <v>50011.7</v>
@@ -2934,13 +2934,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W28" t="n">
-        <v>0.09116336367042994</v>
+        <v>0.09155744161136839</v>
       </c>
       <c r="X28" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y28" t="n">
-        <v>119.5879961740794</v>
+        <v>120.1049471661863</v>
       </c>
       <c r="Z28" t="n">
         <v>0.7623119927331765</v>
@@ -2992,7 +2992,7 @@
         <v>33.6762858057476</v>
       </c>
       <c r="K29" t="n">
-        <v>1.705992188741013</v>
+        <v>1.62923492045223</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -3008,7 +3008,7 @@
         <v>0.143075</v>
       </c>
       <c r="Q29" t="n">
-        <v>1184.4</v>
+        <v>1240.2</v>
       </c>
       <c r="R29" t="n">
         <v>66783.2</v>
@@ -3024,13 +3024,13 @@
         <v>13.43904545346521</v>
       </c>
       <c r="W29" t="n">
-        <v>0.02843320314568355</v>
+        <v>0.0271539153408705</v>
       </c>
       <c r="X29" t="n">
         <v>0.07441004671519687</v>
       </c>
       <c r="Y29" t="n">
-        <v>56.38568051334009</v>
+        <v>53.84873407514917</v>
       </c>
       <c r="Z29" t="n">
         <v>0.5042628356494987</v>
@@ -3144,23 +3144,23 @@
         <v>30.3334426348039</v>
       </c>
       <c r="K31" t="n">
-        <v>29.44994430563485</v>
+        <v>28.08652095815175</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
-        <v>1.326119</v>
+        <v>0.757782</v>
       </c>
       <c r="N31" t="n">
-        <v>1.270857</v>
+        <v>0.726204</v>
       </c>
       <c r="O31" t="n">
-        <v>0.014358</v>
+        <v>0.008203999999999999</v>
       </c>
       <c r="P31" t="n">
-        <v>0.040904</v>
+        <v>0.023374</v>
       </c>
       <c r="Q31" t="n">
-        <v>61.8</v>
+        <v>64.80000000000001</v>
       </c>
       <c r="R31" t="n">
         <v>26315</v>
@@ -3173,16 +3173,16 @@
       </c>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="n">
-        <v>22.87384664182015</v>
+        <v>40.02924671581524</v>
       </c>
       <c r="W31" t="n">
-        <v>0.4908324050939142</v>
+        <v>0.4681086826358626</v>
       </c>
       <c r="X31" t="n">
-        <v>0.04371805125997935</v>
+        <v>0.02498173415801272</v>
       </c>
       <c r="Y31" t="n">
-        <v>425.8090614886731</v>
+        <v>406.0956790123456</v>
       </c>
       <c r="Z31" t="n">
         <v>1.152705401284587</v>
@@ -3324,7 +3324,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K33" t="n">
-        <v>11.20393771297686</v>
+        <v>9.357595917579925</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -3340,7 +3340,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q33" t="n">
-        <v>133.8</v>
+        <v>160.2</v>
       </c>
       <c r="R33" t="n">
         <v>34656</v>
@@ -3356,13 +3356,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W33" t="n">
-        <v>0.186732295216281</v>
+        <v>0.1559599319596654</v>
       </c>
       <c r="X33" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y33" t="n">
-        <v>259.0134529147982</v>
+        <v>216.3295880149813</v>
       </c>
       <c r="Z33" t="n">
         <v>0.7209366660877885</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-23)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.573715932232253</v>
+        <v>3.544311940384772</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>940.2</v>
+        <v>948</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.05956193220387087</v>
+        <v>0.05907186567307953</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>209.987662199532</v>
+        <v>208.2599156118143</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -774,7 +774,7 @@
         <v>55.9873505840139</v>
       </c>
       <c r="K4" t="n">
-        <v>6.697051505264821</v>
+        <v>6.753600794211569</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.806295</v>
       </c>
       <c r="Q4" t="n">
-        <v>501.6</v>
+        <v>497.4</v>
       </c>
       <c r="R4" t="n">
         <v>65667.39999999999</v>
@@ -806,13 +806,13 @@
         <v>1.908085258606485</v>
       </c>
       <c r="W4" t="n">
-        <v>0.111617525087747</v>
+        <v>0.1125600132368595</v>
       </c>
       <c r="X4" t="n">
         <v>0.5240855960127908</v>
       </c>
       <c r="Y4" t="n">
-        <v>130.9158692185008</v>
+        <v>132.0213108162445</v>
       </c>
       <c r="Z4" t="n">
         <v>0.8525897261657063</v>
@@ -922,7 +922,7 @@
         <v>53.5831959822067</v>
       </c>
       <c r="K6" t="n">
-        <v>11.3283712435955</v>
+        <v>11.47391776920914</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -938,7 +938,7 @@
         <v>0.364732</v>
       </c>
       <c r="Q6" t="n">
-        <v>283.8</v>
+        <v>280.2</v>
       </c>
       <c r="R6" t="n">
         <v>35584.1</v>
@@ -954,13 +954,13 @@
         <v>4.05294166276928</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1888061873932583</v>
+        <v>0.1912319628201524</v>
       </c>
       <c r="X6" t="n">
         <v>0.2467343680729723</v>
       </c>
       <c r="Y6" t="n">
-        <v>125.3844256518675</v>
+        <v>126.9953604568166</v>
       </c>
       <c r="Z6" t="n">
         <v>1.505818497087371</v>
@@ -1012,7 +1012,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K7" t="n">
-        <v>4.449952123630124</v>
+        <v>4.337798858725625</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1028,7 +1028,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q7" t="n">
-        <v>719.4</v>
+        <v>738</v>
       </c>
       <c r="R7" t="n">
         <v>78110.8</v>
@@ -1044,13 +1044,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W7" t="n">
-        <v>0.07416586872716875</v>
+        <v>0.07229664764542709</v>
       </c>
       <c r="X7" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y7" t="n">
-        <v>108.5777036419238</v>
+        <v>105.8411924119241</v>
       </c>
       <c r="Z7" t="n">
         <v>0.6830672066132366</v>
@@ -1102,7 +1102,7 @@
         <v>53.2032587538944</v>
       </c>
       <c r="K8" t="n">
-        <v>5.26243904588471</v>
+        <v>5.23139220785589</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1118,7 +1118,7 @@
         <v>1.70337</v>
       </c>
       <c r="Q8" t="n">
-        <v>606.5999999999999</v>
+        <v>610.2</v>
       </c>
       <c r="R8" t="n">
         <v>60537.6</v>
@@ -1134,13 +1134,13 @@
         <v>1.024040806409964</v>
       </c>
       <c r="W8" t="n">
-        <v>0.08770731743141182</v>
+        <v>0.08718987013093149</v>
       </c>
       <c r="X8" t="n">
         <v>0.9765235855256145</v>
       </c>
       <c r="Y8" t="n">
-        <v>99.79821958456975</v>
+        <v>99.20943952802359</v>
       </c>
       <c r="Z8" t="n">
         <v>0.8788465144619939</v>
@@ -1192,7 +1192,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K9" t="n">
-        <v>6.592449235984105</v>
+        <v>6.650715832766793</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q9" t="n">
-        <v>479.4</v>
+        <v>475.2</v>
       </c>
       <c r="R9" t="n">
         <v>27205.5</v>
@@ -1224,13 +1224,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1098741539330684</v>
+        <v>0.1108452638794466</v>
       </c>
       <c r="X9" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y9" t="n">
-        <v>56.74906132665832</v>
+        <v>57.25063131313131</v>
       </c>
       <c r="Z9" t="n">
         <v>1.936140464079432</v>
@@ -1372,48 +1372,48 @@
         <v>52.393894697293</v>
       </c>
       <c r="K11" t="n">
-        <v>8.805696587780336</v>
+        <v>8.925706081310562</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
-        <v>31.838585</v>
+        <v>32.024787</v>
       </c>
       <c r="N11" t="n">
-        <v>30.753951</v>
+        <v>30.935256</v>
       </c>
       <c r="O11" t="n">
-        <v>0.511023</v>
+        <v>0.513532</v>
       </c>
       <c r="P11" t="n">
-        <v>0.573611</v>
+        <v>0.575999</v>
       </c>
       <c r="Q11" t="n">
-        <v>357</v>
+        <v>352.2</v>
       </c>
       <c r="R11" t="n">
-        <v>54231.7</v>
+        <v>54476.5</v>
       </c>
       <c r="S11" t="n">
-        <v>25551.1</v>
+        <v>25676.6</v>
       </c>
       <c r="T11" t="n">
-        <v>28680.5</v>
+        <v>28799.9</v>
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>1.645610026239954</v>
+        <v>1.636041941427838</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1467616097963389</v>
+        <v>0.1487617680218427</v>
       </c>
       <c r="X11" t="n">
-        <v>0.6076773865342173</v>
+        <v>0.6112312738921966</v>
       </c>
       <c r="Y11" t="n">
-        <v>151.9095238095238</v>
+        <v>154.6749006246451</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.9661119732055791</v>
+        <v>0.9617705744181987</v>
       </c>
     </row>
     <row r="12">
@@ -1462,7 +1462,7 @@
         <v>52.3863277108782</v>
       </c>
       <c r="K12" t="n">
-        <v>9.773568602775782</v>
+        <v>9.959377891801939</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1478,7 +1478,7 @@
         <v>0.429124</v>
       </c>
       <c r="Q12" t="n">
-        <v>321.6</v>
+        <v>315.6</v>
       </c>
       <c r="R12" t="n">
         <v>16901.2</v>
@@ -1494,13 +1494,13 @@
         <v>6.009296158837118</v>
       </c>
       <c r="W12" t="n">
-        <v>0.162892810046263</v>
+        <v>0.1659896315300323</v>
       </c>
       <c r="X12" t="n">
         <v>0.1664088394993523</v>
       </c>
       <c r="Y12" t="n">
-        <v>52.55348258706468</v>
+        <v>53.55259822560203</v>
       </c>
       <c r="Z12" t="n">
         <v>3.099562617499243</v>
@@ -1552,7 +1552,7 @@
         <v>51.8955544183089</v>
       </c>
       <c r="K13" t="n">
-        <v>7.0510264155311</v>
+        <v>7.079884640969836</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1568,7 +1568,7 @@
         <v>0.479533</v>
       </c>
       <c r="Q13" t="n">
-        <v>441.6</v>
+        <v>439.8</v>
       </c>
       <c r="R13" t="n">
         <v>74809.60000000001</v>
@@ -1584,13 +1584,13 @@
         <v>3.270976154136362</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1175171069255183</v>
+        <v>0.1179980773494973</v>
       </c>
       <c r="X13" t="n">
         <v>0.3057191348629781</v>
       </c>
       <c r="Y13" t="n">
-        <v>169.4057971014493</v>
+        <v>170.0991359708959</v>
       </c>
       <c r="Z13" t="n">
         <v>0.6937018032218979</v>
@@ -1732,7 +1732,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K15" t="n">
-        <v>3.11721816310259</v>
+        <v>3.261695971223919</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1748,7 +1748,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q15" t="n">
-        <v>894</v>
+        <v>854.4</v>
       </c>
       <c r="R15" t="n">
         <v>80561.39999999999</v>
@@ -1764,13 +1764,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W15" t="n">
-        <v>0.05195363605170984</v>
+        <v>0.05436159952039864</v>
       </c>
       <c r="X15" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y15" t="n">
-        <v>90.11342281879195</v>
+        <v>94.29002808988764</v>
       </c>
       <c r="Z15" t="n">
         <v>0.5765360412086756</v>
@@ -1822,7 +1822,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K16" t="n">
-        <v>2.135740273445749</v>
+        <v>2.541097450962057</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1838,7 +1838,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q16" t="n">
-        <v>1301.4</v>
+        <v>1093.8</v>
       </c>
       <c r="R16" t="n">
         <v>64275.7</v>
@@ -1854,13 +1854,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W16" t="n">
-        <v>0.03559567122409582</v>
+        <v>0.04235162418270095</v>
       </c>
       <c r="X16" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y16" t="n">
-        <v>49.38965729214691</v>
+        <v>58.76366794660815</v>
       </c>
       <c r="Z16" t="n">
         <v>0.7207110390246749</v>
@@ -1912,7 +1912,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K17" t="n">
-        <v>1.289838355525479</v>
+        <v>1.301668343309031</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1928,7 +1928,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q17" t="n">
-        <v>2112.6</v>
+        <v>2093.4</v>
       </c>
       <c r="R17" t="n">
         <v>107730.2</v>
@@ -1944,13 +1944,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W17" t="n">
-        <v>0.02149730592542464</v>
+        <v>0.02169447238848386</v>
       </c>
       <c r="X17" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y17" t="n">
-        <v>50.99413045536306</v>
+        <v>51.46183242571892</v>
       </c>
       <c r="Z17" t="n">
         <v>0.421564319921917</v>
@@ -2002,7 +2002,7 @@
         <v>45.0965048681912</v>
       </c>
       <c r="K18" t="n">
-        <v>8.429253246390878</v>
+        <v>7.656452439421257</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2018,7 +2018,7 @@
         <v>0.071092</v>
       </c>
       <c r="Q18" t="n">
-        <v>321</v>
+        <v>353.4</v>
       </c>
       <c r="R18" t="n">
         <v>89495.10000000001</v>
@@ -2034,13 +2034,13 @@
         <v>15.02220356103491</v>
       </c>
       <c r="W18" t="n">
-        <v>0.1404875541065146</v>
+        <v>0.1276075406570209</v>
       </c>
       <c r="X18" t="n">
         <v>0.06656813003079209</v>
       </c>
       <c r="Y18" t="n">
-        <v>278.8009345794393</v>
+        <v>253.2402376910017</v>
       </c>
       <c r="Z18" t="n">
         <v>0.5038991505478086</v>
@@ -2092,7 +2092,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K19" t="n">
-        <v>4.161467693830297</v>
+        <v>3.820596619932935</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2108,7 +2108,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q19" t="n">
-        <v>645.6</v>
+        <v>703.2</v>
       </c>
       <c r="R19" t="n">
         <v>71127.60000000001</v>
@@ -2124,13 +2124,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W19" t="n">
-        <v>0.06935779489717162</v>
+        <v>0.06367661033221558</v>
       </c>
       <c r="X19" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y19" t="n">
-        <v>110.1728624535316</v>
+        <v>101.1484641638225</v>
       </c>
       <c r="Z19" t="n">
         <v>0.629536106737947</v>
@@ -2182,7 +2182,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K20" t="n">
-        <v>4.536753621800974</v>
+        <v>9.405226863260514</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2198,7 +2198,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q20" t="n">
-        <v>578.4000000000001</v>
+        <v>279</v>
       </c>
       <c r="R20" t="n">
         <v>64144.3</v>
@@ -2214,13 +2214,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W20" t="n">
-        <v>0.07561256036334957</v>
+        <v>0.1567537810543419</v>
       </c>
       <c r="X20" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y20" t="n">
-        <v>110.899550484094</v>
+        <v>229.9078853046595</v>
       </c>
       <c r="Z20" t="n">
         <v>0.6818112429968274</v>
@@ -2272,7 +2272,7 @@
         <v>43.5938229518782</v>
       </c>
       <c r="K21" t="n">
-        <v>2.227584208067358</v>
+        <v>2.124455309545721</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2288,7 +2288,7 @@
         <v>0.486797</v>
       </c>
       <c r="Q21" t="n">
-        <v>1174.2</v>
+        <v>1231.2</v>
       </c>
       <c r="R21" t="n">
         <v>48455.2</v>
@@ -2304,13 +2304,13 @@
         <v>4.72984812235618</v>
       </c>
       <c r="W21" t="n">
-        <v>0.0371264034677893</v>
+        <v>0.03540758849242868</v>
       </c>
       <c r="X21" t="n">
         <v>0.2114232791690251</v>
       </c>
       <c r="Y21" t="n">
-        <v>41.26656446942599</v>
+        <v>39.35607537361923</v>
       </c>
       <c r="Z21" t="n">
         <v>0.8996727482680539</v>
@@ -2362,7 +2362,7 @@
         <v>43.3950199670746</v>
       </c>
       <c r="K22" t="n">
-        <v>6.052304040038299</v>
+        <v>6.018726763810625</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2378,7 +2378,7 @@
         <v>0.064523</v>
       </c>
       <c r="Q22" t="n">
-        <v>430.2</v>
+        <v>432.6</v>
       </c>
       <c r="R22" t="n">
         <v>162164.2</v>
@@ -2394,13 +2394,13 @@
         <v>40.74733935074209</v>
       </c>
       <c r="W22" t="n">
-        <v>0.1008717340006383</v>
+        <v>0.1003121127301771</v>
       </c>
       <c r="X22" t="n">
         <v>0.02454147966305898</v>
       </c>
       <c r="Y22" t="n">
-        <v>376.9507205950721</v>
+        <v>374.8594544613962</v>
       </c>
       <c r="Z22" t="n">
         <v>0.2675992602995889</v>
@@ -2452,7 +2452,7 @@
         <v>42.7057475126235</v>
       </c>
       <c r="K23" t="n">
-        <v>4.074975907693082</v>
+        <v>3.333782007230562</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2468,7 +2468,7 @@
         <v>0.032801</v>
       </c>
       <c r="Q23" t="n">
-        <v>628.8000000000001</v>
+        <v>768.6</v>
       </c>
       <c r="R23" t="n">
         <v>78612.3</v>
@@ -2484,13 +2484,13 @@
         <v>32.69667427900789</v>
       </c>
       <c r="W23" t="n">
-        <v>0.06791626512821804</v>
+        <v>0.0555630334538427</v>
       </c>
       <c r="X23" t="n">
         <v>0.03058415028595205</v>
       </c>
       <c r="Y23" t="n">
-        <v>125.0195610687023</v>
+        <v>102.2798594847775</v>
       </c>
       <c r="Z23" t="n">
         <v>0.5432451093864892</v>
@@ -2542,7 +2542,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K24" t="n">
-        <v>3.191409626981298</v>
+        <v>3.016411696497475</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2558,7 +2558,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q24" t="n">
-        <v>786</v>
+        <v>831.5999999999999</v>
       </c>
       <c r="R24" t="n">
         <v>68673.2</v>
@@ -2574,13 +2574,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W24" t="n">
-        <v>0.05319016044968829</v>
+        <v>0.05027352827495792</v>
       </c>
       <c r="X24" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y24" t="n">
-        <v>87.3704834605598</v>
+        <v>82.57960557960558</v>
       </c>
       <c r="Z24" t="n">
         <v>0.6087886703030441</v>
@@ -2632,7 +2632,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K25" t="n">
-        <v>4.913113106433422</v>
+        <v>5.021623579949742</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2648,7 +2648,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q25" t="n">
-        <v>499.8</v>
+        <v>489</v>
       </c>
       <c r="R25" t="n">
         <v>71002.60000000001</v>
@@ -2664,13 +2664,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W25" t="n">
-        <v>0.08188521844055703</v>
+        <v>0.08369372633249571</v>
       </c>
       <c r="X25" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y25" t="n">
-        <v>142.062024809924</v>
+        <v>145.199591002045</v>
       </c>
       <c r="Z25" t="n">
         <v>0.5764046975264343</v>
@@ -2722,48 +2722,48 @@
         <v>38.8666662997805</v>
       </c>
       <c r="K26" t="n">
-        <v>7.576348206584893</v>
+        <v>8.714499170354372</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
-        <v>3.765796</v>
+        <v>3.768032</v>
       </c>
       <c r="N26" t="n">
-        <v>3.594372</v>
+        <v>3.596336</v>
       </c>
       <c r="O26" t="n">
-        <v>0.093234</v>
+        <v>0.093496</v>
       </c>
       <c r="P26" t="n">
-        <v>0.07819</v>
+        <v>0.078199</v>
       </c>
       <c r="Q26" t="n">
-        <v>307.8</v>
+        <v>267.6</v>
       </c>
       <c r="R26" t="n">
-        <v>40335.1</v>
+        <v>40399</v>
       </c>
       <c r="S26" t="n">
-        <v>21937.3</v>
+        <v>21999.2</v>
       </c>
       <c r="T26" t="n">
-        <v>18397.7</v>
+        <v>18399.8</v>
       </c>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="n">
-        <v>10.3209696700991</v>
+        <v>10.31484507025962</v>
       </c>
       <c r="W26" t="n">
-        <v>0.1262724701097482</v>
+        <v>0.1452416528392395</v>
       </c>
       <c r="X26" t="n">
-        <v>0.09689012098321557</v>
+        <v>0.09694765100091129</v>
       </c>
       <c r="Y26" t="n">
-        <v>131.0432098765432</v>
+        <v>150.9678624813154</v>
       </c>
       <c r="Z26" t="n">
-        <v>0.9635941475236333</v>
+        <v>0.9620700091532092</v>
       </c>
     </row>
     <row r="27">
@@ -2812,48 +2812,48 @@
         <v>38.3770408917494</v>
       </c>
       <c r="K27" t="n">
-        <v>2.780944992155754</v>
+        <v>3.454279108168264</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
-        <v>6.144787</v>
+        <v>6.146153</v>
       </c>
       <c r="N27" t="n">
-        <v>5.854427</v>
+        <v>5.855662</v>
       </c>
       <c r="O27" t="n">
-        <v>0.07260800000000001</v>
+        <v>0.07263600000000001</v>
       </c>
       <c r="P27" t="n">
-        <v>0.217751</v>
+        <v>0.217855</v>
       </c>
       <c r="Q27" t="n">
-        <v>828</v>
+        <v>666.5999999999999</v>
       </c>
       <c r="R27" t="n">
-        <v>69464</v>
+        <v>69495.5</v>
       </c>
       <c r="S27" t="n">
-        <v>17370.4</v>
+        <v>17377.1</v>
       </c>
       <c r="T27" t="n">
-        <v>52093.6</v>
+        <v>52118.5</v>
       </c>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="n">
-        <v>6.245463169309107</v>
+        <v>6.24407509734128</v>
       </c>
       <c r="W27" t="n">
-        <v>0.0463490832025959</v>
+        <v>0.05757131846947106</v>
       </c>
       <c r="X27" t="n">
-        <v>0.1601162272342122</v>
+        <v>0.1601518214324166</v>
       </c>
       <c r="Y27" t="n">
-        <v>83.89371980676329</v>
+        <v>104.2536753675368</v>
       </c>
       <c r="Z27" t="n">
-        <v>0.5524738122156715</v>
+        <v>0.5522233942017742</v>
       </c>
     </row>
     <row r="28">
@@ -2902,7 +2902,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K28" t="n">
-        <v>5.493446496682104</v>
+        <v>6.149115917253838</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2918,7 +2918,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q28" t="n">
-        <v>416.4</v>
+        <v>372</v>
       </c>
       <c r="R28" t="n">
         <v>50011.7</v>
@@ -2934,13 +2934,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W28" t="n">
-        <v>0.09155744161136839</v>
+        <v>0.102485265287564</v>
       </c>
       <c r="X28" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y28" t="n">
-        <v>120.1049471661863</v>
+        <v>134.4400537634409</v>
       </c>
       <c r="Z28" t="n">
         <v>0.7623119927331765</v>
@@ -2992,7 +2992,7 @@
         <v>33.6762858057476</v>
       </c>
       <c r="K29" t="n">
-        <v>1.62923492045223</v>
+        <v>1.708588828297696</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -3008,7 +3008,7 @@
         <v>0.143075</v>
       </c>
       <c r="Q29" t="n">
-        <v>1240.2</v>
+        <v>1182.6</v>
       </c>
       <c r="R29" t="n">
         <v>66783.2</v>
@@ -3024,13 +3024,13 @@
         <v>13.43904545346521</v>
       </c>
       <c r="W29" t="n">
-        <v>0.0271539153408705</v>
+        <v>0.02847648047162827</v>
       </c>
       <c r="X29" t="n">
         <v>0.07441004671519687</v>
       </c>
       <c r="Y29" t="n">
-        <v>53.84873407514917</v>
+        <v>56.47150346693725</v>
       </c>
       <c r="Z29" t="n">
         <v>0.5042628356494987</v>
@@ -3144,7 +3144,7 @@
         <v>30.3334426348039</v>
       </c>
       <c r="K31" t="n">
-        <v>28.08652095815175</v>
+        <v>30.03311151960782</v>
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="n">
@@ -3160,7 +3160,7 @@
         <v>0.023374</v>
       </c>
       <c r="Q31" t="n">
-        <v>64.80000000000001</v>
+        <v>60.6</v>
       </c>
       <c r="R31" t="n">
         <v>26315</v>
@@ -3176,13 +3176,13 @@
         <v>40.02924671581524</v>
       </c>
       <c r="W31" t="n">
-        <v>0.4681086826358626</v>
+        <v>0.5005518586601304</v>
       </c>
       <c r="X31" t="n">
         <v>0.02498173415801272</v>
       </c>
       <c r="Y31" t="n">
-        <v>406.0956790123456</v>
+        <v>434.2409240924092</v>
       </c>
       <c r="Z31" t="n">
         <v>1.152705401284587</v>
@@ -3234,7 +3234,7 @@
         <v>26.4910658661689</v>
       </c>
       <c r="K32" t="n">
-        <v>15.86291369231671</v>
+        <v>16.25218764795638</v>
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="n">
@@ -3250,7 +3250,7 @@
         <v>0.020469</v>
       </c>
       <c r="Q32" t="n">
-        <v>100.2</v>
+        <v>97.8</v>
       </c>
       <c r="R32" t="n">
         <v>49173.8</v>
@@ -3266,13 +3266,13 @@
         <v>63.641894492204</v>
       </c>
       <c r="W32" t="n">
-        <v>0.2643818948719451</v>
+        <v>0.2708697941326063</v>
       </c>
       <c r="X32" t="n">
         <v>0.01571292005021155</v>
       </c>
       <c r="Y32" t="n">
-        <v>490.7564870259482</v>
+        <v>502.799591002045</v>
       </c>
       <c r="Z32" t="n">
         <v>0.5387231791354116</v>
@@ -3324,7 +3324,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K33" t="n">
-        <v>9.357595917579925</v>
+        <v>9.836527992101731</v>
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="n">
@@ -3340,7 +3340,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q33" t="n">
-        <v>160.2</v>
+        <v>152.4</v>
       </c>
       <c r="R33" t="n">
         <v>34656</v>
@@ -3356,13 +3356,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W33" t="n">
-        <v>0.1559599319596654</v>
+        <v>0.1639421332016955</v>
       </c>
       <c r="X33" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y33" t="n">
-        <v>216.3295880149813</v>
+        <v>227.4015748031496</v>
       </c>
       <c r="Z33" t="n">
         <v>0.7209366660877885</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-24)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z33"/>
+  <dimension ref="A1:Z28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.339033871257252</v>
+        <v>4.345578417066086</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>796.8</v>
+        <v>795.6</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07231723118762086</v>
+        <v>0.07242630695110143</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>149.5557228915663</v>
+        <v>149.7812971342383</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.544311940384772</v>
+        <v>3.537594987876147</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>948</v>
+        <v>949.8</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.05907186567307953</v>
+        <v>0.05895991646460244</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>208.2599156118143</v>
+        <v>207.8652347862708</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -731,39 +731,35 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>claude-opus-5-5-xhigh</t>
+          <t>muse-wonder-full</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (Xhigh, Default Fallback)</t>
+          <t>Muse Wonder Full (Max)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (xhigh with fallback)</t>
+          <t>Muse Wonder Full (max)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>large</t>
-        </is>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="b">
         <v>1</v>
       </c>
@@ -771,85 +767,61 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>55.9873505840139</v>
-      </c>
-      <c r="K4" t="n">
-        <v>6.753600794211569</v>
-      </c>
+        <v>55.8021199855616</v>
+      </c>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
-      <c r="M4" t="n">
-        <v>29.342164</v>
-      </c>
-      <c r="N4" t="n">
-        <v>28.028816</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0.507053</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.806295</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>497.4</v>
-      </c>
-      <c r="R4" t="n">
-        <v>65667.39999999999</v>
-      </c>
-      <c r="S4" t="n">
-        <v>25352.7</v>
-      </c>
-      <c r="T4" t="n">
-        <v>40314.7</v>
-      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
-      <c r="V4" t="n">
-        <v>1.908085258606485</v>
-      </c>
-      <c r="W4" t="n">
-        <v>0.1125600132368595</v>
-      </c>
-      <c r="X4" t="n">
-        <v>0.5240855960127908</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>132.0213108162445</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>0.8525897261657063</v>
-      </c>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>muse-wonder-full</t>
+          <t>kimi-k3-1-pro</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Muse Wonder Full (Max)</t>
+          <t>Kimi K3.1 Pro</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Muse Wonder Full (max)</t>
+          <t>Kimi K3.1 Pro</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>Kimi</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>kimi</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
       <c r="H5" t="b">
         <v>1</v>
       </c>
@@ -857,39 +829,67 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>55.8021199855616</v>
-      </c>
-      <c r="K5" t="inlineStr"/>
+        <v>55.0869210959395</v>
+      </c>
+      <c r="K5" t="n">
+        <v>5.34305733229287</v>
+      </c>
       <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
+      <c r="M5" t="n">
+        <v>11.623139</v>
+      </c>
+      <c r="N5" t="n">
+        <v>11.071193</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.203119</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.348827</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>618.6</v>
+      </c>
+      <c r="R5" t="n">
+        <v>55194.6</v>
+      </c>
+      <c r="S5" t="n">
+        <v>20311.9</v>
+      </c>
+      <c r="T5" t="n">
+        <v>34882.7</v>
+      </c>
       <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
+      <c r="V5" t="n">
+        <v>4.739418593887546</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.08905095553821452</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0.2109963448448519</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>89.22502424830262</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0.9980491043678096</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>claude-opus-5-5-high</t>
+          <t>claude-fable-5-1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (High, Default Fallback)</t>
+          <t>Claude Fable 5.1 (Max, Default Fallback)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (high with fallback)</t>
+          <t>Claude Fable 5.1 (max with fallback)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -919,82 +919,82 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>53.5831959822067</v>
+        <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>11.47391776920914</v>
+        <v>4.355504160189812</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
-        <v>13.220816</v>
+        <v>69.77964799999999</v>
       </c>
       <c r="N6" t="n">
-        <v>12.509134</v>
+        <v>65.87410800000001</v>
       </c>
       <c r="O6" t="n">
-        <v>0.346949</v>
+        <v>1.54355</v>
       </c>
       <c r="P6" t="n">
-        <v>0.364732</v>
+        <v>2.361991</v>
       </c>
       <c r="Q6" t="n">
-        <v>280.2</v>
+        <v>735</v>
       </c>
       <c r="R6" t="n">
-        <v>35584.1</v>
+        <v>78110.8</v>
       </c>
       <c r="S6" t="n">
-        <v>17347.5</v>
+        <v>30871</v>
       </c>
       <c r="T6" t="n">
-        <v>18236.6</v>
+        <v>47239.8</v>
       </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="n">
-        <v>4.05294166276928</v>
+        <v>0.7646201649272464</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1912319628201524</v>
+        <v>0.07259173600316353</v>
       </c>
       <c r="X6" t="n">
-        <v>0.2467343680729723</v>
+        <v>1.307838905994782</v>
       </c>
       <c r="Y6" t="n">
-        <v>126.9953604568166</v>
+        <v>106.2731972789116</v>
       </c>
       <c r="Z6" t="n">
-        <v>1.505818497087371</v>
+        <v>0.6830672066132366</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>claude-fable-5-1</t>
+          <t>gpt-6-astra</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (Max, Default Fallback)</t>
+          <t>GPT-6 Astra (Max)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (max with fallback)</t>
+          <t>GPT-6 Astra (max)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1009,82 +1009,82 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>53.3549259623252</v>
+        <v>52.673669395513</v>
       </c>
       <c r="K7" t="n">
-        <v>4.337798858725625</v>
+        <v>6.66755308803962</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
-        <v>69.77964799999999</v>
+        <v>11.948927</v>
       </c>
       <c r="N7" t="n">
-        <v>65.87410800000001</v>
+        <v>10.588652</v>
       </c>
       <c r="O7" t="n">
-        <v>1.54355</v>
+        <v>0.525713</v>
       </c>
       <c r="P7" t="n">
-        <v>2.361991</v>
+        <v>0.834562</v>
       </c>
       <c r="Q7" t="n">
-        <v>738</v>
+        <v>474</v>
       </c>
       <c r="R7" t="n">
-        <v>78110.8</v>
+        <v>27205.5</v>
       </c>
       <c r="S7" t="n">
-        <v>30871</v>
+        <v>10514.3</v>
       </c>
       <c r="T7" t="n">
-        <v>47239.8</v>
+        <v>16691.2</v>
       </c>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="n">
-        <v>0.7646201649272464</v>
+        <v>4.408234261998002</v>
       </c>
       <c r="W7" t="n">
-        <v>0.07229664764542709</v>
+        <v>0.1111258848006603</v>
       </c>
       <c r="X7" t="n">
-        <v>1.307838905994782</v>
+        <v>0.2268481982957858</v>
       </c>
       <c r="Y7" t="n">
-        <v>105.8411924119241</v>
+        <v>57.39556962025316</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.6830672066132366</v>
+        <v>1.936140464079432</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>claude-fable-5-1-xhigh</t>
+          <t>gemini-4-argon</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (Xhigh, Default Fallback)</t>
+          <t>Gemini 4 Argon (High)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (xhigh with fallback)</t>
+          <t>Gemini 4 Argon (high)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1099,82 +1099,82 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>53.2032587538944</v>
+        <v>52.5605655745982</v>
       </c>
       <c r="K8" t="n">
-        <v>5.23139220785589</v>
+        <v>4.361872661792382</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
-        <v>51.954237</v>
+        <v>8.057855999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>48.927356</v>
+        <v>7.44228</v>
       </c>
       <c r="O8" t="n">
-        <v>1.32351</v>
+        <v>0.260112</v>
       </c>
       <c r="P8" t="n">
-        <v>1.70337</v>
+        <v>0.355464</v>
       </c>
       <c r="Q8" t="n">
-        <v>610.2</v>
+        <v>723</v>
       </c>
       <c r="R8" t="n">
-        <v>60537.6</v>
+        <v>61557.6</v>
       </c>
       <c r="S8" t="n">
-        <v>26470.2</v>
+        <v>26011.2</v>
       </c>
       <c r="T8" t="n">
-        <v>34067.4</v>
+        <v>35546.4</v>
       </c>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="n">
-        <v>1.024040806409964</v>
+        <v>6.522897104961693</v>
       </c>
       <c r="W8" t="n">
-        <v>0.08718987013093149</v>
+        <v>0.0726978776965397</v>
       </c>
       <c r="X8" t="n">
-        <v>0.9765235855256145</v>
+        <v>0.1533061128987214</v>
       </c>
       <c r="Y8" t="n">
-        <v>99.20943952802359</v>
+        <v>85.14190871369294</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.8788465144619939</v>
+        <v>0.8538436452135594</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>gpt-6-astra</t>
+          <t>muse-wonder</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (Max)</t>
+          <t>Muse Wonder (Max)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (max)</t>
+          <t>Muse Wonder (max)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1189,82 +1189,82 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>52.673669395513</v>
+        <v>52.393894697293</v>
       </c>
       <c r="K9" t="n">
-        <v>6.650715832766793</v>
+        <v>8.850320050218413</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
-        <v>11.948927</v>
+        <v>32.024787</v>
       </c>
       <c r="N9" t="n">
-        <v>10.588652</v>
+        <v>30.935256</v>
       </c>
       <c r="O9" t="n">
-        <v>0.525713</v>
+        <v>0.513532</v>
       </c>
       <c r="P9" t="n">
-        <v>0.834562</v>
+        <v>0.575999</v>
       </c>
       <c r="Q9" t="n">
-        <v>475.2</v>
+        <v>355.2</v>
       </c>
       <c r="R9" t="n">
-        <v>27205.5</v>
+        <v>54476.5</v>
       </c>
       <c r="S9" t="n">
-        <v>10514.3</v>
+        <v>25676.6</v>
       </c>
       <c r="T9" t="n">
-        <v>16691.2</v>
+        <v>28799.9</v>
       </c>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="n">
-        <v>4.408234261998002</v>
+        <v>1.636041941427838</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1108452638794466</v>
+        <v>0.1475053341703069</v>
       </c>
       <c r="X9" t="n">
-        <v>0.2268481982957858</v>
+        <v>0.6112312738921966</v>
       </c>
       <c r="Y9" t="n">
-        <v>57.25063131313131</v>
+        <v>153.3685247747748</v>
       </c>
       <c r="Z9" t="n">
-        <v>1.936140464079432</v>
+        <v>0.9617705744181987</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>gemini-4-argon</t>
+          <t>gpt-6-1-sol</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Gemini 4 Argon (High)</t>
+          <t>GPT-6.1 Sol (Max)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Gemini 4 Argon (high)</t>
+          <t>GPT-6.1 Sol (max)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1279,82 +1279,82 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>52.5605655745982</v>
+        <v>51.8332597011541</v>
       </c>
       <c r="K10" t="n">
-        <v>4.369124320415478</v>
+        <v>4.574868464356054</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
-        <v>8.057855999999999</v>
+        <v>3.029649</v>
       </c>
       <c r="N10" t="n">
-        <v>7.44228</v>
+        <v>2.648365</v>
       </c>
       <c r="O10" t="n">
-        <v>0.260112</v>
+        <v>0.129384</v>
       </c>
       <c r="P10" t="n">
-        <v>0.355464</v>
+        <v>0.2519</v>
       </c>
       <c r="Q10" t="n">
-        <v>721.8</v>
+        <v>679.8</v>
       </c>
       <c r="R10" t="n">
-        <v>61557.6</v>
+        <v>38128.4</v>
       </c>
       <c r="S10" t="n">
-        <v>26011.2</v>
+        <v>12938.4</v>
       </c>
       <c r="T10" t="n">
-        <v>35546.4</v>
+        <v>25190</v>
       </c>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="n">
-        <v>6.522897104961693</v>
+        <v>17.10866826525254</v>
       </c>
       <c r="W10" t="n">
-        <v>0.0728187386735913</v>
+        <v>0.07624780773926758</v>
       </c>
       <c r="X10" t="n">
-        <v>0.1533061128987214</v>
+        <v>0.05844990296708164</v>
       </c>
       <c r="Y10" t="n">
-        <v>85.28345802161265</v>
+        <v>56.0876728449544</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.8538436452135594</v>
+        <v>1.359439674918279</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>muse-wonder</t>
+          <t>grok-4-7</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Muse Wonder (Max)</t>
+          <t>Grok 4.7 (Xhigh)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Muse Wonder (max)</t>
+          <t>Grok 4.7 (xhigh)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>SpaceXAI</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>xai</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1369,82 +1369,82 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>52.393894697293</v>
+        <v>46.4465506302286</v>
       </c>
       <c r="K11" t="n">
-        <v>8.925706081310562</v>
+        <v>3.270883847199197</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
-        <v>32.024787</v>
+        <v>8.336827</v>
       </c>
       <c r="N11" t="n">
-        <v>30.935256</v>
+        <v>7.853459</v>
       </c>
       <c r="O11" t="n">
-        <v>0.513532</v>
+        <v>0.132106</v>
       </c>
       <c r="P11" t="n">
-        <v>0.575999</v>
+        <v>0.351262</v>
       </c>
       <c r="Q11" t="n">
-        <v>352.2</v>
+        <v>852</v>
       </c>
       <c r="R11" t="n">
-        <v>54476.5</v>
+        <v>80561.39999999999</v>
       </c>
       <c r="S11" t="n">
-        <v>25676.6</v>
+        <v>22017.7</v>
       </c>
       <c r="T11" t="n">
-        <v>28799.9</v>
+        <v>58543.6</v>
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>1.636041941427838</v>
+        <v>5.571250384616186</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1487617680218427</v>
+        <v>0.05451473078665329</v>
       </c>
       <c r="X11" t="n">
-        <v>0.6112312738921966</v>
+        <v>0.1794929200743312</v>
       </c>
       <c r="Y11" t="n">
-        <v>154.6749006246451</v>
+        <v>94.5556338028169</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.9617705744181987</v>
+        <v>0.5765360412086756</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>gpt-6-astra-xhigh</t>
+          <t>mimo-v2-6-pro</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (Xhigh)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (xhigh)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Xiaomi</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>xiaomi</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1456,85 +1456,85 @@
         <v>1</v>
       </c>
       <c r="I12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" t="n">
-        <v>52.3863277108782</v>
+        <v>46.3242065310383</v>
       </c>
       <c r="K12" t="n">
-        <v>9.959377891801939</v>
+        <v>2.549488526749494</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
-        <v>8.717548000000001</v>
+        <v>2.466319</v>
       </c>
       <c r="N12" t="n">
-        <v>7.872489</v>
+        <v>2.410399</v>
       </c>
       <c r="O12" t="n">
-        <v>0.415935</v>
+        <v>0.023278</v>
       </c>
       <c r="P12" t="n">
-        <v>0.429124</v>
+        <v>0.032642</v>
       </c>
       <c r="Q12" t="n">
-        <v>315.6</v>
+        <v>1090.2</v>
       </c>
       <c r="R12" t="n">
-        <v>16901.2</v>
+        <v>64275.7</v>
       </c>
       <c r="S12" t="n">
-        <v>8318.700000000001</v>
+        <v>26756</v>
       </c>
       <c r="T12" t="n">
-        <v>8582.5</v>
+        <v>37519.7</v>
       </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="n">
-        <v>6.009296158837118</v>
+        <v>18.78273107859863</v>
       </c>
       <c r="W12" t="n">
-        <v>0.1659896315300323</v>
+        <v>0.04249147544582489</v>
       </c>
       <c r="X12" t="n">
-        <v>0.1664088394993523</v>
+        <v>0.05324039383918014</v>
       </c>
       <c r="Y12" t="n">
-        <v>53.55259822560203</v>
+        <v>58.95771418088424</v>
       </c>
       <c r="Z12" t="n">
-        <v>3.099562617499243</v>
+        <v>0.7207110390246749</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>claude-sonnet-5-5-xhigh</t>
+          <t>qwen3-8-max</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5.5 (Xhigh, Default Fallback)</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5.5 (xhigh with fallback)</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1549,82 +1549,82 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>51.8955544183089</v>
+        <v>45.4152084980521</v>
       </c>
       <c r="K13" t="n">
-        <v>7.079884640969836</v>
+        <v>1.301668343309031</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
-        <v>15.865464</v>
+        <v>26.154609</v>
       </c>
       <c r="N13" t="n">
-        <v>15.117367</v>
+        <v>25.508227</v>
       </c>
       <c r="O13" t="n">
-        <v>0.268563</v>
+        <v>0.221402</v>
       </c>
       <c r="P13" t="n">
-        <v>0.479533</v>
+        <v>0.424979</v>
       </c>
       <c r="Q13" t="n">
-        <v>439.8</v>
+        <v>2093.4</v>
       </c>
       <c r="R13" t="n">
-        <v>74809.60000000001</v>
+        <v>107730.2</v>
       </c>
       <c r="S13" t="n">
-        <v>26856.3</v>
+        <v>36900.3</v>
       </c>
       <c r="T13" t="n">
-        <v>47953.3</v>
+        <v>70829.89999999999</v>
       </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="n">
-        <v>3.270976154136362</v>
+        <v>1.736413207249709</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1179980773494973</v>
+        <v>0.02169447238848386</v>
       </c>
       <c r="X13" t="n">
-        <v>0.3057191348629781</v>
+        <v>0.5758997891889408</v>
       </c>
       <c r="Y13" t="n">
-        <v>170.0991359708959</v>
+        <v>51.46183242571892</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.6937018032218979</v>
+        <v>0.421564319921917</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>gpt-6-1-sol</t>
+          <t>deepseek-v4-1-flash-1017</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>GPT-6.1 Sol (Max)</t>
+          <t>DeepSeek V4.1 Flash 1017 (Max)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GPT-6.1 Sol (max)</t>
+          <t>DeepSeek V4.1 Flash 1017 (max)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>DeepSeek</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>deepseek</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1636,85 +1636,85 @@
         <v>1</v>
       </c>
       <c r="I14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
-        <v>51.8332597011541</v>
+        <v>45.0965048681912</v>
       </c>
       <c r="K14" t="n">
-        <v>4.483845994909524</v>
+        <v>7.566527662448188</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>3.029649</v>
+        <v>3.00199</v>
       </c>
       <c r="N14" t="n">
-        <v>2.648365</v>
+        <v>2.894596</v>
       </c>
       <c r="O14" t="n">
-        <v>0.129384</v>
+        <v>0.036302</v>
       </c>
       <c r="P14" t="n">
-        <v>0.2519</v>
+        <v>0.071092</v>
       </c>
       <c r="Q14" t="n">
-        <v>693.6</v>
+        <v>357.6</v>
       </c>
       <c r="R14" t="n">
-        <v>38128.4</v>
+        <v>89495.10000000001</v>
       </c>
       <c r="S14" t="n">
-        <v>12938.4</v>
+        <v>30252</v>
       </c>
       <c r="T14" t="n">
-        <v>25190</v>
+        <v>59243</v>
       </c>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="n">
-        <v>17.10866826525254</v>
+        <v>15.02220356103491</v>
       </c>
       <c r="W14" t="n">
-        <v>0.0747307665818254</v>
+        <v>0.1261087943741364</v>
       </c>
       <c r="X14" t="n">
-        <v>0.05844990296708164</v>
+        <v>0.06656813003079209</v>
       </c>
       <c r="Y14" t="n">
-        <v>54.97174163783161</v>
+        <v>250.2659395973154</v>
       </c>
       <c r="Z14" t="n">
-        <v>1.359439674918279</v>
+        <v>0.5038991505478086</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>grok-4-7</t>
+          <t>glm-5-3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Grok 4.7 (Xhigh)</t>
+          <t>GLM-5.3 (Max)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Grok 4.7 (xhigh)</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>SpaceXAI</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>xai</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1726,85 +1726,85 @@
         <v>1</v>
       </c>
       <c r="I15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" t="n">
-        <v>46.4465506302286</v>
+        <v>44.777392385614</v>
       </c>
       <c r="K15" t="n">
-        <v>3.261695971223919</v>
+        <v>4.048588823292405</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>8.336827</v>
+        <v>8.678356000000001</v>
       </c>
       <c r="N15" t="n">
-        <v>7.853459</v>
+        <v>8.365394999999999</v>
       </c>
       <c r="O15" t="n">
-        <v>0.132106</v>
+        <v>0.098552</v>
       </c>
       <c r="P15" t="n">
-        <v>0.351262</v>
+        <v>0.21441</v>
       </c>
       <c r="Q15" t="n">
-        <v>854.4</v>
+        <v>663.6</v>
       </c>
       <c r="R15" t="n">
-        <v>80561.39999999999</v>
+        <v>71127.60000000001</v>
       </c>
       <c r="S15" t="n">
-        <v>22017.7</v>
+        <v>22398.1</v>
       </c>
       <c r="T15" t="n">
-        <v>58543.6</v>
+        <v>48729.5</v>
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="n">
-        <v>5.571250384616186</v>
+        <v>5.159663003639629</v>
       </c>
       <c r="W15" t="n">
-        <v>0.05436159952039864</v>
+        <v>0.06747648038820675</v>
       </c>
       <c r="X15" t="n">
-        <v>0.1794929200743312</v>
+        <v>0.1938111072941391</v>
       </c>
       <c r="Y15" t="n">
-        <v>94.29002808988764</v>
+        <v>107.1844484629295</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.5765360412086756</v>
+        <v>0.629536106737947</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>mimo-v2-6-pro</t>
+          <t>step-5</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Xiaomi</t>
+          <t>StepFun</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>xiaomi</t>
+          <t>stepfun</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1819,87 +1819,87 @@
         <v>1</v>
       </c>
       <c r="J16" t="n">
-        <v>46.3242065310383</v>
+        <v>43.7343049141614</v>
       </c>
       <c r="K16" t="n">
-        <v>2.541097450962057</v>
+        <v>10.24222597521344</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
-        <v>2.466319</v>
+        <v>6.586908</v>
       </c>
       <c r="N16" t="n">
-        <v>2.410399</v>
+        <v>6.413718</v>
       </c>
       <c r="O16" t="n">
-        <v>0.023278</v>
+        <v>0.055881</v>
       </c>
       <c r="P16" t="n">
-        <v>0.032642</v>
+        <v>0.117309</v>
       </c>
       <c r="Q16" t="n">
-        <v>1093.8</v>
+        <v>256.2</v>
       </c>
       <c r="R16" t="n">
-        <v>64275.7</v>
+        <v>64144.3</v>
       </c>
       <c r="S16" t="n">
-        <v>26756</v>
+        <v>20696.6</v>
       </c>
       <c r="T16" t="n">
-        <v>37519.7</v>
+        <v>43447.7</v>
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="n">
-        <v>18.78273107859863</v>
+        <v>6.639580348497565</v>
       </c>
       <c r="W16" t="n">
-        <v>0.04235162418270095</v>
+        <v>0.1707037662535574</v>
       </c>
       <c r="X16" t="n">
-        <v>0.05324039383918014</v>
+        <v>0.1506119283918727</v>
       </c>
       <c r="Y16" t="n">
-        <v>58.76366794660815</v>
+        <v>250.3680718188915</v>
       </c>
       <c r="Z16" t="n">
-        <v>0.7207110390246749</v>
+        <v>0.6818112429968274</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>qwen3-8-max</t>
+          <t>claude-haiku-5-5</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>Claude Haiku 5.5 (Max)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>Claude Haiku 5.5 (max)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H17" t="b">
@@ -1909,157 +1909,157 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>45.4152084980521</v>
+        <v>43.3950199670746</v>
       </c>
       <c r="K17" t="n">
-        <v>1.301668343309031</v>
+        <v>6.052304040038299</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
-        <v>26.154609</v>
+        <v>1.064978</v>
       </c>
       <c r="N17" t="n">
-        <v>25.508227</v>
+        <v>0.983896</v>
       </c>
       <c r="O17" t="n">
-        <v>0.221402</v>
+        <v>0.016559</v>
       </c>
       <c r="P17" t="n">
-        <v>0.424979</v>
+        <v>0.064523</v>
       </c>
       <c r="Q17" t="n">
-        <v>2093.4</v>
+        <v>430.2</v>
       </c>
       <c r="R17" t="n">
-        <v>107730.2</v>
+        <v>162164.2</v>
       </c>
       <c r="S17" t="n">
-        <v>36900.3</v>
+        <v>33117.6</v>
       </c>
       <c r="T17" t="n">
-        <v>70829.89999999999</v>
+        <v>129046.6</v>
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="n">
-        <v>1.736413207249709</v>
+        <v>40.74733935074209</v>
       </c>
       <c r="W17" t="n">
-        <v>0.02169447238848386</v>
+        <v>0.1008717340006383</v>
       </c>
       <c r="X17" t="n">
-        <v>0.5758997891889408</v>
+        <v>0.02454147966305898</v>
       </c>
       <c r="Y17" t="n">
-        <v>51.46183242571892</v>
+        <v>376.9507205950721</v>
       </c>
       <c r="Z17" t="n">
-        <v>0.421564319921917</v>
+        <v>0.2675992602995889</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>deepseek-v4-1-flash-1017</t>
+          <t>minimax-m3-1-flash</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash 1017 (Max)</t>
+          <t>MiniMax-M3.1-Flash</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash 1017 (max)</t>
+          <t>MiniMax-M3.1-Flash</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>DeepSeek</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>deepseek</t>
+          <t>minimax</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H18" t="b">
         <v>1</v>
       </c>
       <c r="I18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>45.0965048681912</v>
+        <v>42.7057475126235</v>
       </c>
       <c r="K18" t="n">
-        <v>7.656452439421257</v>
+        <v>3.333782007230562</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
-        <v>3.00199</v>
+        <v>1.306119</v>
       </c>
       <c r="N18" t="n">
-        <v>2.894596</v>
+        <v>1.258952</v>
       </c>
       <c r="O18" t="n">
-        <v>0.036302</v>
+        <v>0.014367</v>
       </c>
       <c r="P18" t="n">
-        <v>0.071092</v>
+        <v>0.032801</v>
       </c>
       <c r="Q18" t="n">
-        <v>353.4</v>
+        <v>768.6</v>
       </c>
       <c r="R18" t="n">
-        <v>89495.10000000001</v>
+        <v>78612.3</v>
       </c>
       <c r="S18" t="n">
-        <v>30252</v>
+        <v>23944.7</v>
       </c>
       <c r="T18" t="n">
-        <v>59243</v>
+        <v>54667.6</v>
       </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="n">
-        <v>15.02220356103491</v>
+        <v>32.69667427900789</v>
       </c>
       <c r="W18" t="n">
-        <v>0.1276075406570209</v>
+        <v>0.0555630334538427</v>
       </c>
       <c r="X18" t="n">
-        <v>0.06656813003079209</v>
+        <v>0.03058415028595205</v>
       </c>
       <c r="Y18" t="n">
-        <v>253.2402376910017</v>
+        <v>102.2798594847775</v>
       </c>
       <c r="Z18" t="n">
-        <v>0.5038991505478086</v>
+        <v>0.5432451093864892</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>glm-5-3</t>
+          <t>glm-5-3-flash</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>GLM-5.3 (Max)</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2089,82 +2089,82 @@
         <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>44.777392385614</v>
+        <v>41.807466113455</v>
       </c>
       <c r="K19" t="n">
-        <v>3.820596619932935</v>
+        <v>3.016411696497475</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
-        <v>8.678356000000001</v>
+        <v>1.193653</v>
       </c>
       <c r="N19" t="n">
-        <v>8.365394999999999</v>
+        <v>1.159316</v>
       </c>
       <c r="O19" t="n">
-        <v>0.098552</v>
+        <v>0.011012</v>
       </c>
       <c r="P19" t="n">
-        <v>0.21441</v>
+        <v>0.023325</v>
       </c>
       <c r="Q19" t="n">
-        <v>703.2</v>
+        <v>831.5999999999999</v>
       </c>
       <c r="R19" t="n">
-        <v>71127.60000000001</v>
+        <v>68673.2</v>
       </c>
       <c r="S19" t="n">
-        <v>22398.1</v>
+        <v>22023.7</v>
       </c>
       <c r="T19" t="n">
-        <v>48729.5</v>
+        <v>46649.5</v>
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="n">
-        <v>5.159663003639629</v>
+        <v>35.02480713696107</v>
       </c>
       <c r="W19" t="n">
-        <v>0.06367661033221558</v>
+        <v>0.05027352827495792</v>
       </c>
       <c r="X19" t="n">
-        <v>0.1938111072941391</v>
+        <v>0.02855119219042658</v>
       </c>
       <c r="Y19" t="n">
-        <v>101.1484641638225</v>
+        <v>82.57960557960558</v>
       </c>
       <c r="Z19" t="n">
-        <v>0.629536106737947</v>
+        <v>0.6087886703030441</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>step-5</t>
+          <t>gemini-3-8-flash</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>Gemini 3.8 Flash (High)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>Gemini 3.8 Flash (high)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>StepFun</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>stepfun</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2176,85 +2176,85 @@
         <v>1</v>
       </c>
       <c r="I20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>43.7343049141614</v>
+        <v>40.9262321765904</v>
       </c>
       <c r="K20" t="n">
-        <v>9.405226863260514</v>
+        <v>5.021623579949742</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
-        <v>6.586908</v>
+        <v>4.90102</v>
       </c>
       <c r="N20" t="n">
-        <v>6.413718</v>
+        <v>4.63476</v>
       </c>
       <c r="O20" t="n">
-        <v>0.055881</v>
+        <v>0.106033</v>
       </c>
       <c r="P20" t="n">
-        <v>0.117309</v>
+        <v>0.160227</v>
       </c>
       <c r="Q20" t="n">
-        <v>279</v>
+        <v>489</v>
       </c>
       <c r="R20" t="n">
-        <v>64144.3</v>
+        <v>71002.60000000001</v>
       </c>
       <c r="S20" t="n">
-        <v>20696.6</v>
+        <v>28275.4</v>
       </c>
       <c r="T20" t="n">
-        <v>43447.7</v>
+        <v>42727.1</v>
       </c>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="n">
-        <v>6.639580348497565</v>
+        <v>8.350554002348574</v>
       </c>
       <c r="W20" t="n">
-        <v>0.1567537810543419</v>
+        <v>0.08369372633249571</v>
       </c>
       <c r="X20" t="n">
-        <v>0.1506119283918727</v>
+        <v>0.119752533750306</v>
       </c>
       <c r="Y20" t="n">
-        <v>229.9078853046595</v>
+        <v>145.199591002045</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.6818112429968274</v>
+        <v>0.5764046975264343</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>kimi-k3</t>
+          <t>muse-spark-open</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Kimi K3 (Max)</t>
+          <t>Muse Spark Open (Xhigh)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Kimi K3 (max)</t>
+          <t>Muse Spark Open (xhigh)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Kimi</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>kimi</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2269,87 +2269,87 @@
         <v>1</v>
       </c>
       <c r="J21" t="n">
-        <v>43.5938229518782</v>
+        <v>38.8666662997805</v>
       </c>
       <c r="K21" t="n">
-        <v>2.124455309545721</v>
+        <v>8.217054186000105</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
-        <v>9.216749</v>
+        <v>3.768032</v>
       </c>
       <c r="N21" t="n">
-        <v>8.489921000000001</v>
+        <v>3.596336</v>
       </c>
       <c r="O21" t="n">
-        <v>0.240032</v>
+        <v>0.093496</v>
       </c>
       <c r="P21" t="n">
-        <v>0.486797</v>
+        <v>0.078199</v>
       </c>
       <c r="Q21" t="n">
-        <v>1231.2</v>
+        <v>283.8</v>
       </c>
       <c r="R21" t="n">
-        <v>48455.2</v>
+        <v>40399</v>
       </c>
       <c r="S21" t="n">
-        <v>16002.1</v>
+        <v>21999.2</v>
       </c>
       <c r="T21" t="n">
-        <v>32453.1</v>
+        <v>18399.8</v>
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="n">
-        <v>4.72984812235618</v>
+        <v>10.31484507025962</v>
       </c>
       <c r="W21" t="n">
-        <v>0.03540758849242868</v>
+        <v>0.1369509031000017</v>
       </c>
       <c r="X21" t="n">
-        <v>0.2114232791690251</v>
+        <v>0.09694765100091129</v>
       </c>
       <c r="Y21" t="n">
-        <v>39.35607537361923</v>
+        <v>142.3502466525722</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.8996727482680539</v>
+        <v>0.9620700091532092</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>claude-haiku-5-5</t>
+          <t>mistral-large-4</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Claude Haiku 5.5 (Max)</t>
+          <t>Mistral Large 4 Preview</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Claude Haiku 5.5 (max)</t>
+          <t>Mistral Large 4 Preview</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Mistral</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>mistral</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H22" t="b">
@@ -2359,82 +2359,82 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>43.3950199670746</v>
+        <v>38.3770408917494</v>
       </c>
       <c r="K22" t="n">
-        <v>6.018726763810625</v>
+        <v>3.560022346173414</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
-        <v>1.064978</v>
+        <v>6.146153</v>
       </c>
       <c r="N22" t="n">
-        <v>0.983896</v>
+        <v>5.855662</v>
       </c>
       <c r="O22" t="n">
-        <v>0.016559</v>
+        <v>0.07263600000000001</v>
       </c>
       <c r="P22" t="n">
-        <v>0.064523</v>
+        <v>0.217855</v>
       </c>
       <c r="Q22" t="n">
-        <v>432.6</v>
+        <v>646.8</v>
       </c>
       <c r="R22" t="n">
-        <v>162164.2</v>
+        <v>69495.5</v>
       </c>
       <c r="S22" t="n">
-        <v>33117.6</v>
+        <v>17377.1</v>
       </c>
       <c r="T22" t="n">
-        <v>129046.6</v>
+        <v>52118.5</v>
       </c>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="n">
-        <v>40.74733935074209</v>
+        <v>6.24407509734128</v>
       </c>
       <c r="W22" t="n">
-        <v>0.1003121127301771</v>
+        <v>0.0593337057695569</v>
       </c>
       <c r="X22" t="n">
-        <v>0.02454147966305898</v>
+        <v>0.1601518214324166</v>
       </c>
       <c r="Y22" t="n">
-        <v>374.8594544613962</v>
+        <v>107.4451144094001</v>
       </c>
       <c r="Z22" t="n">
-        <v>0.2675992602995889</v>
+        <v>0.5522233942017742</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>minimax-m3-1-flash</t>
+          <t>gpt-6-luna</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MiniMax-M3.1-Flash</t>
+          <t>GPT-6 Luna (Max)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MiniMax-M3.1-Flash</t>
+          <t>GPT-6 Luna (max)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>minimax</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2449,87 +2449,87 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>42.7057475126235</v>
+        <v>38.1245186869738</v>
       </c>
       <c r="K23" t="n">
-        <v>3.333782007230562</v>
+        <v>6.407482132264504</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
-        <v>1.306119</v>
+        <v>0.326276</v>
       </c>
       <c r="N23" t="n">
-        <v>1.258952</v>
+        <v>0.30127</v>
       </c>
       <c r="O23" t="n">
-        <v>0.014367</v>
+        <v>0.005561</v>
       </c>
       <c r="P23" t="n">
-        <v>0.032801</v>
+        <v>0.019445</v>
       </c>
       <c r="Q23" t="n">
-        <v>768.6</v>
+        <v>357</v>
       </c>
       <c r="R23" t="n">
-        <v>78612.3</v>
+        <v>50011.7</v>
       </c>
       <c r="S23" t="n">
-        <v>23944.7</v>
+        <v>11122</v>
       </c>
       <c r="T23" t="n">
-        <v>54667.6</v>
+        <v>38889.7</v>
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="n">
-        <v>32.69667427900789</v>
+        <v>116.8474502782117</v>
       </c>
       <c r="W23" t="n">
-        <v>0.0555630334538427</v>
+        <v>0.1067913688710751</v>
       </c>
       <c r="X23" t="n">
-        <v>0.03058415028595205</v>
+        <v>0.008558167059863248</v>
       </c>
       <c r="Y23" t="n">
-        <v>102.2798594847775</v>
+        <v>140.0887955182073</v>
       </c>
       <c r="Z23" t="n">
-        <v>0.5432451093864892</v>
+        <v>0.7623119927331765</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>glm-5-3-flash</t>
+          <t>qwen3-8-27b</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Qwen3.8 27B (Xhigh)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Qwen3.8 27B (xhigh)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H24" t="b">
@@ -2539,82 +2539,82 @@
         <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>41.807466113455</v>
+        <v>33.6762858057476</v>
       </c>
       <c r="K24" t="n">
-        <v>3.016411696497475</v>
+        <v>1.647567798715636</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>1.193653</v>
+        <v>2.505854</v>
       </c>
       <c r="N24" t="n">
-        <v>1.159316</v>
+        <v>2.305504</v>
       </c>
       <c r="O24" t="n">
-        <v>0.011012</v>
+        <v>0.057275</v>
       </c>
       <c r="P24" t="n">
-        <v>0.023325</v>
+        <v>0.143075</v>
       </c>
       <c r="Q24" t="n">
-        <v>831.5999999999999</v>
+        <v>1226.4</v>
       </c>
       <c r="R24" t="n">
-        <v>68673.2</v>
+        <v>66783.2</v>
       </c>
       <c r="S24" t="n">
-        <v>22023.7</v>
+        <v>19091.6</v>
       </c>
       <c r="T24" t="n">
-        <v>46649.5</v>
+        <v>47691.6</v>
       </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="n">
-        <v>35.02480713696107</v>
+        <v>13.43904545346521</v>
       </c>
       <c r="W24" t="n">
-        <v>0.05027352827495792</v>
+        <v>0.02745946331192726</v>
       </c>
       <c r="X24" t="n">
-        <v>0.02855119219042658</v>
+        <v>0.07441004671519687</v>
       </c>
       <c r="Y24" t="n">
-        <v>82.57960557960558</v>
+        <v>54.45466405740378</v>
       </c>
       <c r="Z24" t="n">
-        <v>0.6087886703030441</v>
+        <v>0.5042628356494987</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>gemini-3-8-flash</t>
+          <t>k2-horizon-375b-a23b</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (High)</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Institute of Foundation Models</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>ifm</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2626,85 +2626,57 @@
         <v>1</v>
       </c>
       <c r="I25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>40.9262321765904</v>
-      </c>
-      <c r="K25" t="n">
-        <v>5.021623579949742</v>
-      </c>
+        <v>30.5015302696723</v>
+      </c>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
-      <c r="M25" t="n">
-        <v>4.90102</v>
-      </c>
-      <c r="N25" t="n">
-        <v>4.63476</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0.106033</v>
-      </c>
-      <c r="P25" t="n">
-        <v>0.160227</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>489</v>
-      </c>
-      <c r="R25" t="n">
-        <v>71002.60000000001</v>
-      </c>
-      <c r="S25" t="n">
-        <v>28275.4</v>
-      </c>
-      <c r="T25" t="n">
-        <v>42727.1</v>
-      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
-      <c r="V25" t="n">
-        <v>8.350554002348574</v>
-      </c>
-      <c r="W25" t="n">
-        <v>0.08369372633249571</v>
-      </c>
-      <c r="X25" t="n">
-        <v>0.119752533750306</v>
-      </c>
-      <c r="Y25" t="n">
-        <v>145.199591002045</v>
-      </c>
-      <c r="Z25" t="n">
-        <v>0.5764046975264343</v>
-      </c>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>muse-spark-open</t>
+          <t>reflection-beam</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Muse Spark Open (Xhigh)</t>
+          <t>Beam 1.0</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Muse Spark Open (xhigh)</t>
+          <t>Beam 1.0</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>Reflection</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>reflection</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2719,652 +2691,230 @@
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>38.8666662997805</v>
+        <v>30.3334426348039</v>
       </c>
       <c r="K26" t="n">
-        <v>8.714499170354372</v>
+        <v>28.88899298552752</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
-        <v>3.768032</v>
+        <v>0.757782</v>
       </c>
       <c r="N26" t="n">
-        <v>3.596336</v>
+        <v>0.726204</v>
       </c>
       <c r="O26" t="n">
-        <v>0.093496</v>
+        <v>0.008203999999999999</v>
       </c>
       <c r="P26" t="n">
-        <v>0.078199</v>
+        <v>0.023374</v>
       </c>
       <c r="Q26" t="n">
-        <v>267.6</v>
+        <v>63</v>
       </c>
       <c r="R26" t="n">
-        <v>40399</v>
+        <v>26315</v>
       </c>
       <c r="S26" t="n">
-        <v>21999.2</v>
+        <v>6837.1</v>
       </c>
       <c r="T26" t="n">
-        <v>18399.8</v>
+        <v>19478</v>
       </c>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="n">
-        <v>10.31484507025962</v>
+        <v>40.02924671581524</v>
       </c>
       <c r="W26" t="n">
-        <v>0.1452416528392395</v>
+        <v>0.4814832164254588</v>
       </c>
       <c r="X26" t="n">
-        <v>0.09694765100091129</v>
+        <v>0.02498173415801272</v>
       </c>
       <c r="Y26" t="n">
-        <v>150.9678624813154</v>
+        <v>417.6984126984127</v>
       </c>
       <c r="Z26" t="n">
-        <v>0.9620700091532092</v>
+        <v>1.152705401284587</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>mistral-large-4</t>
+          <t>nemotron-3-5-super-vl</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Mistral Large 4 Preview</t>
+          <t>Nemotron 3.5 Super VL</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mistral Large 4 Preview</t>
+          <t>Nemotron 3.5 Super VL</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Mistral</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>mistral</t>
+          <t>nvidia</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H27" t="b">
         <v>1</v>
       </c>
       <c r="I27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>38.3770408917494</v>
+        <v>26.4910658661689</v>
       </c>
       <c r="K27" t="n">
-        <v>3.454279108168264</v>
+        <v>16.55691616635556</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
-        <v>6.146153</v>
+        <v>0.416252</v>
       </c>
       <c r="N27" t="n">
-        <v>5.855662</v>
+        <v>0.387977</v>
       </c>
       <c r="O27" t="n">
-        <v>0.07263600000000001</v>
+        <v>0.007806</v>
       </c>
       <c r="P27" t="n">
-        <v>0.217855</v>
+        <v>0.020469</v>
       </c>
       <c r="Q27" t="n">
-        <v>666.5999999999999</v>
+        <v>96</v>
       </c>
       <c r="R27" t="n">
-        <v>69495.5</v>
+        <v>49173.8</v>
       </c>
       <c r="S27" t="n">
-        <v>17377.1</v>
+        <v>13575.6</v>
       </c>
       <c r="T27" t="n">
-        <v>52118.5</v>
+        <v>35598.3</v>
       </c>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="n">
-        <v>6.24407509734128</v>
+        <v>63.641894492204</v>
       </c>
       <c r="W27" t="n">
-        <v>0.05757131846947106</v>
+        <v>0.2759486027725927</v>
       </c>
       <c r="X27" t="n">
-        <v>0.1601518214324166</v>
+        <v>0.01571292005021155</v>
       </c>
       <c r="Y27" t="n">
-        <v>104.2536753675368</v>
+        <v>512.2270833333333</v>
       </c>
       <c r="Z27" t="n">
-        <v>0.5522233942017742</v>
+        <v>0.5387231791354116</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>gpt-6-luna</t>
+          <t>inkling</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (Max)</t>
+          <t>Inkling (Xhigh)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (max)</t>
+          <t>Inkling (xhigh)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Thinking Machines</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>thinking-machines</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H28" t="b">
         <v>1</v>
       </c>
       <c r="I28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>38.1245186869738</v>
+        <v>24.9847810999384</v>
       </c>
       <c r="K28" t="n">
-        <v>6.149115917253838</v>
+        <v>9.836527992101731</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
-        <v>0.326276</v>
+        <v>2.418996</v>
       </c>
       <c r="N28" t="n">
-        <v>0.30127</v>
+        <v>2.278639</v>
       </c>
       <c r="O28" t="n">
-        <v>0.005561</v>
+        <v>0.04559</v>
       </c>
       <c r="P28" t="n">
-        <v>0.019445</v>
+        <v>0.094767</v>
       </c>
       <c r="Q28" t="n">
-        <v>372</v>
+        <v>152.4</v>
       </c>
       <c r="R28" t="n">
-        <v>50011.7</v>
+        <v>34656</v>
       </c>
       <c r="S28" t="n">
-        <v>11122</v>
+        <v>11256.8</v>
       </c>
       <c r="T28" t="n">
-        <v>38889.7</v>
+        <v>23399.2</v>
       </c>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="n">
-        <v>116.8474502782117</v>
+        <v>10.32857478885389</v>
       </c>
       <c r="W28" t="n">
-        <v>0.102485265287564</v>
+        <v>0.1639421332016955</v>
       </c>
       <c r="X28" t="n">
-        <v>0.008558167059863248</v>
+        <v>0.09681877901287532</v>
       </c>
       <c r="Y28" t="n">
-        <v>134.4400537634409</v>
+        <v>227.4015748031496</v>
       </c>
       <c r="Z28" t="n">
-        <v>0.7623119927331765</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>qwen3-8-27b</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Qwen3.8 27B (Xhigh)</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Qwen3.8 27B (xhigh)</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Alibaba</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>alibaba</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>small</t>
-        </is>
-      </c>
-      <c r="H29" t="b">
-        <v>1</v>
-      </c>
-      <c r="I29" t="b">
-        <v>1</v>
-      </c>
-      <c r="J29" t="n">
-        <v>33.6762858057476</v>
-      </c>
-      <c r="K29" t="n">
-        <v>1.708588828297696</v>
-      </c>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="n">
-        <v>2.505854</v>
-      </c>
-      <c r="N29" t="n">
-        <v>2.305504</v>
-      </c>
-      <c r="O29" t="n">
-        <v>0.057275</v>
-      </c>
-      <c r="P29" t="n">
-        <v>0.143075</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>1182.6</v>
-      </c>
-      <c r="R29" t="n">
-        <v>66783.2</v>
-      </c>
-      <c r="S29" t="n">
-        <v>19091.6</v>
-      </c>
-      <c r="T29" t="n">
-        <v>47691.6</v>
-      </c>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="n">
-        <v>13.43904545346521</v>
-      </c>
-      <c r="W29" t="n">
-        <v>0.02847648047162827</v>
-      </c>
-      <c r="X29" t="n">
-        <v>0.07441004671519687</v>
-      </c>
-      <c r="Y29" t="n">
-        <v>56.47150346693725</v>
-      </c>
-      <c r="Z29" t="n">
-        <v>0.5042628356494987</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>k2-horizon-375b-a23b</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>K2 Horizon 375B A23B</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>K2 Horizon 375B A23B</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Institute of Foundation Models</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>ifm</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>2026-09-03</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>large</t>
-        </is>
-      </c>
-      <c r="H30" t="b">
-        <v>1</v>
-      </c>
-      <c r="I30" t="b">
-        <v>1</v>
-      </c>
-      <c r="J30" t="n">
-        <v>30.5015302696723</v>
-      </c>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr"/>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr"/>
-      <c r="W30" t="inlineStr"/>
-      <c r="X30" t="inlineStr"/>
-      <c r="Y30" t="inlineStr"/>
-      <c r="Z30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>reflection-beam</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Beam 1.0</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Beam 1.0</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Reflection</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>reflection</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>large</t>
-        </is>
-      </c>
-      <c r="H31" t="b">
-        <v>1</v>
-      </c>
-      <c r="I31" t="b">
-        <v>1</v>
-      </c>
-      <c r="J31" t="n">
-        <v>30.3334426348039</v>
-      </c>
-      <c r="K31" t="n">
-        <v>30.03311151960782</v>
-      </c>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="n">
-        <v>0.757782</v>
-      </c>
-      <c r="N31" t="n">
-        <v>0.726204</v>
-      </c>
-      <c r="O31" t="n">
-        <v>0.008203999999999999</v>
-      </c>
-      <c r="P31" t="n">
-        <v>0.023374</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>60.6</v>
-      </c>
-      <c r="R31" t="n">
-        <v>26315</v>
-      </c>
-      <c r="S31" t="n">
-        <v>6837.1</v>
-      </c>
-      <c r="T31" t="n">
-        <v>19478</v>
-      </c>
-      <c r="U31" t="inlineStr"/>
-      <c r="V31" t="n">
-        <v>40.02924671581524</v>
-      </c>
-      <c r="W31" t="n">
-        <v>0.5005518586601304</v>
-      </c>
-      <c r="X31" t="n">
-        <v>0.02498173415801272</v>
-      </c>
-      <c r="Y31" t="n">
-        <v>434.2409240924092</v>
-      </c>
-      <c r="Z31" t="n">
-        <v>1.152705401284587</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>nemotron-3-5-super-vl</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Nemotron 3.5 Super VL</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Nemotron 3.5 Super VL</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>NVIDIA</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>nvidia</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="H32" t="b">
-        <v>1</v>
-      </c>
-      <c r="I32" t="b">
-        <v>1</v>
-      </c>
-      <c r="J32" t="n">
-        <v>26.4910658661689</v>
-      </c>
-      <c r="K32" t="n">
-        <v>16.25218764795638</v>
-      </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="n">
-        <v>0.416252</v>
-      </c>
-      <c r="N32" t="n">
-        <v>0.387977</v>
-      </c>
-      <c r="O32" t="n">
-        <v>0.007806</v>
-      </c>
-      <c r="P32" t="n">
-        <v>0.020469</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>97.8</v>
-      </c>
-      <c r="R32" t="n">
-        <v>49173.8</v>
-      </c>
-      <c r="S32" t="n">
-        <v>13575.6</v>
-      </c>
-      <c r="T32" t="n">
-        <v>35598.3</v>
-      </c>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="n">
-        <v>63.641894492204</v>
-      </c>
-      <c r="W32" t="n">
-        <v>0.2708697941326063</v>
-      </c>
-      <c r="X32" t="n">
-        <v>0.01571292005021155</v>
-      </c>
-      <c r="Y32" t="n">
-        <v>502.799591002045</v>
-      </c>
-      <c r="Z32" t="n">
-        <v>0.5387231791354116</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>inkling</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Inkling (Xhigh)</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Inkling (xhigh)</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Thinking Machines</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>thinking-machines</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>large</t>
-        </is>
-      </c>
-      <c r="H33" t="b">
-        <v>1</v>
-      </c>
-      <c r="I33" t="b">
-        <v>1</v>
-      </c>
-      <c r="J33" t="n">
-        <v>24.9847810999384</v>
-      </c>
-      <c r="K33" t="n">
-        <v>9.836527992101731</v>
-      </c>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="n">
-        <v>2.418996</v>
-      </c>
-      <c r="N33" t="n">
-        <v>2.278639</v>
-      </c>
-      <c r="O33" t="n">
-        <v>0.04559</v>
-      </c>
-      <c r="P33" t="n">
-        <v>0.094767</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>152.4</v>
-      </c>
-      <c r="R33" t="n">
-        <v>34656</v>
-      </c>
-      <c r="S33" t="n">
-        <v>11256.8</v>
-      </c>
-      <c r="T33" t="n">
-        <v>23399.2</v>
-      </c>
-      <c r="U33" t="inlineStr"/>
-      <c r="V33" t="n">
-        <v>10.32857478885389</v>
-      </c>
-      <c r="W33" t="n">
-        <v>0.1639421332016955</v>
-      </c>
-      <c r="X33" t="n">
-        <v>0.09681877901287532</v>
-      </c>
-      <c r="Y33" t="n">
-        <v>227.4015748031496</v>
-      </c>
-      <c r="Z33" t="n">
         <v>0.7209366660877885</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-25)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.345578417066086</v>
+        <v>4.362026480718872</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>795.6</v>
+        <v>792.6</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07242630695110143</v>
+        <v>0.07270044134531453</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>149.7812971342383</v>
+        <v>150.3482210446631</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.537594987876147</v>
+        <v>3.573715932232253</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>949.8</v>
+        <v>940.2</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.05895991646460244</v>
+        <v>0.05956193220387087</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>207.8652347862708</v>
+        <v>209.987662199532</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -832,7 +832,7 @@
         <v>55.0869210959395</v>
       </c>
       <c r="K5" t="n">
-        <v>5.34305733229287</v>
+        <v>3.909646635623811</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -848,7 +848,7 @@
         <v>0.348827</v>
       </c>
       <c r="Q5" t="n">
-        <v>618.6</v>
+        <v>845.4</v>
       </c>
       <c r="R5" t="n">
         <v>55194.6</v>
@@ -864,13 +864,13 @@
         <v>4.739418593887546</v>
       </c>
       <c r="W5" t="n">
-        <v>0.08905095553821452</v>
+        <v>0.06516077726039686</v>
       </c>
       <c r="X5" t="n">
         <v>0.2109963448448519</v>
       </c>
       <c r="Y5" t="n">
-        <v>89.22502424830262</v>
+        <v>65.28814762242726</v>
       </c>
       <c r="Z5" t="n">
         <v>0.9980491043678096</v>
@@ -922,7 +922,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>4.355504160189812</v>
+        <v>4.327244603594907</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -938,7 +938,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q6" t="n">
-        <v>735</v>
+        <v>739.8</v>
       </c>
       <c r="R6" t="n">
         <v>78110.8</v>
@@ -954,13 +954,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07259173600316353</v>
+        <v>0.07212074339324845</v>
       </c>
       <c r="X6" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y6" t="n">
-        <v>106.2731972789116</v>
+        <v>105.5836712625034</v>
       </c>
       <c r="Z6" t="n">
         <v>0.6830672066132366</v>
@@ -1012,7 +1012,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K7" t="n">
-        <v>6.66755308803962</v>
+        <v>7.838343660046578</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1028,7 +1028,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q7" t="n">
-        <v>474</v>
+        <v>403.2</v>
       </c>
       <c r="R7" t="n">
         <v>27205.5</v>
@@ -1044,13 +1044,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W7" t="n">
-        <v>0.1111258848006603</v>
+        <v>0.1306390610007763</v>
       </c>
       <c r="X7" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y7" t="n">
-        <v>57.39556962025316</v>
+        <v>67.47395833333333</v>
       </c>
       <c r="Z7" t="n">
         <v>1.936140464079432</v>
@@ -1102,7 +1102,7 @@
         <v>52.5605655745982</v>
       </c>
       <c r="K8" t="n">
-        <v>4.361872661792382</v>
+        <v>4.343848394594893</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1118,7 +1118,7 @@
         <v>0.355464</v>
       </c>
       <c r="Q8" t="n">
-        <v>723</v>
+        <v>726</v>
       </c>
       <c r="R8" t="n">
         <v>61557.6</v>
@@ -1134,13 +1134,13 @@
         <v>6.522897104961693</v>
       </c>
       <c r="W8" t="n">
-        <v>0.0726978776965397</v>
+        <v>0.0723974732432482</v>
       </c>
       <c r="X8" t="n">
         <v>0.1533061128987214</v>
       </c>
       <c r="Y8" t="n">
-        <v>85.14190871369294</v>
+        <v>84.7900826446281</v>
       </c>
       <c r="Z8" t="n">
         <v>0.8538436452135594</v>
@@ -1192,7 +1192,7 @@
         <v>52.393894697293</v>
       </c>
       <c r="K9" t="n">
-        <v>8.850320050218413</v>
+        <v>9.22427723543891</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>0.575999</v>
       </c>
       <c r="Q9" t="n">
-        <v>355.2</v>
+        <v>340.8</v>
       </c>
       <c r="R9" t="n">
         <v>54476.5</v>
@@ -1224,13 +1224,13 @@
         <v>1.636041941427838</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1475053341703069</v>
+        <v>0.1537379539239818</v>
       </c>
       <c r="X9" t="n">
         <v>0.6112312738921966</v>
       </c>
       <c r="Y9" t="n">
-        <v>153.3685247747748</v>
+        <v>159.8488849765259</v>
       </c>
       <c r="Z9" t="n">
         <v>0.9617705744181987</v>
@@ -1282,7 +1282,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K10" t="n">
-        <v>4.574868464356054</v>
+        <v>4.950645625707172</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1298,7 +1298,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q10" t="n">
-        <v>679.8</v>
+        <v>628.2</v>
       </c>
       <c r="R10" t="n">
         <v>38128.4</v>
@@ -1314,13 +1314,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W10" t="n">
-        <v>0.07624780773926758</v>
+        <v>0.08251076042845287</v>
       </c>
       <c r="X10" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y10" t="n">
-        <v>56.0876728449544</v>
+        <v>60.69468322190385</v>
       </c>
       <c r="Z10" t="n">
         <v>1.359439674918279</v>
@@ -1372,7 +1372,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K11" t="n">
-        <v>3.270883847199197</v>
+        <v>3.092313623850107</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1388,7 +1388,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q11" t="n">
-        <v>852</v>
+        <v>901.1999999999999</v>
       </c>
       <c r="R11" t="n">
         <v>80561.39999999999</v>
@@ -1404,13 +1404,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W11" t="n">
-        <v>0.05451473078665329</v>
+        <v>0.05153856039750178</v>
       </c>
       <c r="X11" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y11" t="n">
-        <v>94.5556338028169</v>
+        <v>89.39347536617844</v>
       </c>
       <c r="Z11" t="n">
         <v>0.5765360412086756</v>
@@ -1462,7 +1462,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K12" t="n">
-        <v>2.549488526749494</v>
+        <v>2.742700209060882</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1478,7 +1478,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q12" t="n">
-        <v>1090.2</v>
+        <v>1013.4</v>
       </c>
       <c r="R12" t="n">
         <v>64275.7</v>
@@ -1494,13 +1494,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W12" t="n">
-        <v>0.04249147544582489</v>
+        <v>0.0457116701510147</v>
       </c>
       <c r="X12" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y12" t="n">
-        <v>58.95771418088424</v>
+        <v>63.42579435563449</v>
       </c>
       <c r="Z12" t="n">
         <v>0.7207110390246749</v>
@@ -1552,7 +1552,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K13" t="n">
-        <v>1.301668343309031</v>
+        <v>1.311820002832239</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1568,7 +1568,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q13" t="n">
-        <v>2093.4</v>
+        <v>2077.2</v>
       </c>
       <c r="R13" t="n">
         <v>107730.2</v>
@@ -1584,13 +1584,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W13" t="n">
-        <v>0.02169447238848386</v>
+        <v>0.02186366671387065</v>
       </c>
       <c r="X13" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y13" t="n">
-        <v>51.46183242571892</v>
+        <v>51.8631812054689</v>
       </c>
       <c r="Z13" t="n">
         <v>0.421564319921917</v>
@@ -1642,7 +1642,7 @@
         <v>45.0965048681912</v>
       </c>
       <c r="K14" t="n">
-        <v>7.566527662448188</v>
+        <v>6.822466697154493</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1658,7 +1658,7 @@
         <v>0.071092</v>
       </c>
       <c r="Q14" t="n">
-        <v>357.6</v>
+        <v>396.6</v>
       </c>
       <c r="R14" t="n">
         <v>89495.10000000001</v>
@@ -1674,13 +1674,13 @@
         <v>15.02220356103491</v>
       </c>
       <c r="W14" t="n">
-        <v>0.1261087943741364</v>
+        <v>0.1137077782859082</v>
       </c>
       <c r="X14" t="n">
         <v>0.06656813003079209</v>
       </c>
       <c r="Y14" t="n">
-        <v>250.2659395973154</v>
+        <v>225.6558245083207</v>
       </c>
       <c r="Z14" t="n">
         <v>0.5038991505478086</v>
@@ -1732,7 +1732,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K15" t="n">
-        <v>4.048588823292405</v>
+        <v>4.115569153089522</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1748,7 +1748,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q15" t="n">
-        <v>663.6</v>
+        <v>652.8000000000001</v>
       </c>
       <c r="R15" t="n">
         <v>71127.60000000001</v>
@@ -1764,13 +1764,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W15" t="n">
-        <v>0.06747648038820675</v>
+        <v>0.0685928192181587</v>
       </c>
       <c r="X15" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y15" t="n">
-        <v>107.1844484629295</v>
+        <v>108.9577205882353</v>
       </c>
       <c r="Z15" t="n">
         <v>0.629536106737947</v>
@@ -1822,7 +1822,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K16" t="n">
-        <v>10.24222597521344</v>
+        <v>9.96225624468369</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1838,7 +1838,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q16" t="n">
-        <v>256.2</v>
+        <v>263.4</v>
       </c>
       <c r="R16" t="n">
         <v>64144.3</v>
@@ -1854,13 +1854,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W16" t="n">
-        <v>0.1707037662535574</v>
+        <v>0.1660376040780615</v>
       </c>
       <c r="X16" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y16" t="n">
-        <v>250.3680718188915</v>
+        <v>243.5242976461656</v>
       </c>
       <c r="Z16" t="n">
         <v>0.6818112429968274</v>
@@ -1912,7 +1912,7 @@
         <v>43.3950199670746</v>
       </c>
       <c r="K17" t="n">
-        <v>6.052304040038299</v>
+        <v>6.077733888946023</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1928,7 +1928,7 @@
         <v>0.064523</v>
       </c>
       <c r="Q17" t="n">
-        <v>430.2</v>
+        <v>428.4</v>
       </c>
       <c r="R17" t="n">
         <v>162164.2</v>
@@ -1944,13 +1944,13 @@
         <v>40.74733935074209</v>
       </c>
       <c r="W17" t="n">
-        <v>0.1008717340006383</v>
+        <v>0.1012955648157671</v>
       </c>
       <c r="X17" t="n">
         <v>0.02454147966305898</v>
       </c>
       <c r="Y17" t="n">
-        <v>376.9507205950721</v>
+        <v>378.5345471521942</v>
       </c>
       <c r="Z17" t="n">
         <v>0.2675992602995889</v>
@@ -2002,7 +2002,7 @@
         <v>42.7057475126235</v>
       </c>
       <c r="K18" t="n">
-        <v>3.333782007230562</v>
+        <v>4.548002929991852</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2018,7 +2018,7 @@
         <v>0.032801</v>
       </c>
       <c r="Q18" t="n">
-        <v>768.6</v>
+        <v>563.4000000000001</v>
       </c>
       <c r="R18" t="n">
         <v>78612.3</v>
@@ -2034,13 +2034,13 @@
         <v>32.69667427900789</v>
       </c>
       <c r="W18" t="n">
-        <v>0.0555630334538427</v>
+        <v>0.07580004883319755</v>
       </c>
       <c r="X18" t="n">
         <v>0.03058415028595205</v>
       </c>
       <c r="Y18" t="n">
-        <v>102.2798594847775</v>
+        <v>139.5319488817891</v>
       </c>
       <c r="Z18" t="n">
         <v>0.5432451093864892</v>
@@ -2092,7 +2092,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K19" t="n">
-        <v>3.016411696497475</v>
+        <v>3.003409921943606</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2108,7 +2108,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q19" t="n">
-        <v>831.5999999999999</v>
+        <v>835.2</v>
       </c>
       <c r="R19" t="n">
         <v>68673.2</v>
@@ -2124,13 +2124,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W19" t="n">
-        <v>0.05027352827495792</v>
+        <v>0.05005683203239344</v>
       </c>
       <c r="X19" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y19" t="n">
-        <v>82.57960557960558</v>
+        <v>82.22365900383141</v>
       </c>
       <c r="Z19" t="n">
         <v>0.6087886703030441</v>
@@ -2182,7 +2182,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K20" t="n">
-        <v>5.021623579949742</v>
+        <v>4.930871346577157</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2198,7 +2198,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q20" t="n">
-        <v>489</v>
+        <v>498.0000000000001</v>
       </c>
       <c r="R20" t="n">
         <v>71002.60000000001</v>
@@ -2214,13 +2214,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W20" t="n">
-        <v>0.08369372633249571</v>
+        <v>0.08218118910961927</v>
       </c>
       <c r="X20" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y20" t="n">
-        <v>145.199591002045</v>
+        <v>142.5755020080321</v>
       </c>
       <c r="Z20" t="n">
         <v>0.5764046975264343</v>
@@ -2362,7 +2362,7 @@
         <v>38.3770408917494</v>
       </c>
       <c r="K22" t="n">
-        <v>3.560022346173414</v>
+        <v>3.924032811017322</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2378,7 +2378,7 @@
         <v>0.217855</v>
       </c>
       <c r="Q22" t="n">
-        <v>646.8</v>
+        <v>586.8</v>
       </c>
       <c r="R22" t="n">
         <v>69495.5</v>
@@ -2394,13 +2394,13 @@
         <v>6.24407509734128</v>
       </c>
       <c r="W22" t="n">
-        <v>0.0593337057695569</v>
+        <v>0.06540054685028869</v>
       </c>
       <c r="X22" t="n">
         <v>0.1601518214324166</v>
       </c>
       <c r="Y22" t="n">
-        <v>107.4451144094001</v>
+        <v>118.4313224267212</v>
       </c>
       <c r="Z22" t="n">
         <v>0.5522233942017742</v>
@@ -2452,7 +2452,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K23" t="n">
-        <v>6.407482132264504</v>
+        <v>6.354086447828966</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2468,7 +2468,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q23" t="n">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="R23" t="n">
         <v>50011.7</v>
@@ -2484,13 +2484,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W23" t="n">
-        <v>0.1067913688710751</v>
+        <v>0.1059014407971494</v>
       </c>
       <c r="X23" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y23" t="n">
-        <v>140.0887955182073</v>
+        <v>138.9213888888889</v>
       </c>
       <c r="Z23" t="n">
         <v>0.7623119927331765</v>
@@ -2542,7 +2542,7 @@
         <v>33.6762858057476</v>
       </c>
       <c r="K24" t="n">
-        <v>1.647567798715636</v>
+        <v>1.665493857851019</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2558,7 +2558,7 @@
         <v>0.143075</v>
       </c>
       <c r="Q24" t="n">
-        <v>1226.4</v>
+        <v>1213.2</v>
       </c>
       <c r="R24" t="n">
         <v>66783.2</v>
@@ -2574,13 +2574,13 @@
         <v>13.43904545346521</v>
       </c>
       <c r="W24" t="n">
-        <v>0.02745946331192726</v>
+        <v>0.02775823096418365</v>
       </c>
       <c r="X24" t="n">
         <v>0.07441004671519687</v>
       </c>
       <c r="Y24" t="n">
-        <v>54.45466405740378</v>
+        <v>55.04714803824596</v>
       </c>
       <c r="Z24" t="n">
         <v>0.5042628356494987</v>
@@ -2694,7 +2694,7 @@
         <v>30.3334426348039</v>
       </c>
       <c r="K26" t="n">
-        <v>28.88899298552752</v>
+        <v>31.59733607792074</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2710,7 +2710,7 @@
         <v>0.023374</v>
       </c>
       <c r="Q26" t="n">
-        <v>63</v>
+        <v>57.59999999999999</v>
       </c>
       <c r="R26" t="n">
         <v>26315</v>
@@ -2726,13 +2726,13 @@
         <v>40.02924671581524</v>
       </c>
       <c r="W26" t="n">
-        <v>0.4814832164254588</v>
+        <v>0.5266222679653456</v>
       </c>
       <c r="X26" t="n">
         <v>0.02498173415801272</v>
       </c>
       <c r="Y26" t="n">
-        <v>417.6984126984127</v>
+        <v>456.8576388888889</v>
       </c>
       <c r="Z26" t="n">
         <v>1.152705401284587</v>
@@ -2784,7 +2784,7 @@
         <v>26.4910658661689</v>
       </c>
       <c r="K27" t="n">
-        <v>16.55691616635556</v>
+        <v>16.45407817774466</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2800,7 +2800,7 @@
         <v>0.020469</v>
       </c>
       <c r="Q27" t="n">
-        <v>96</v>
+        <v>96.60000000000001</v>
       </c>
       <c r="R27" t="n">
         <v>49173.8</v>
@@ -2816,13 +2816,13 @@
         <v>63.641894492204</v>
       </c>
       <c r="W27" t="n">
-        <v>0.2759486027725927</v>
+        <v>0.2742346362957443</v>
       </c>
       <c r="X27" t="n">
         <v>0.01571292005021155</v>
       </c>
       <c r="Y27" t="n">
-        <v>512.2270833333333</v>
+        <v>509.0455486542443</v>
       </c>
       <c r="Z27" t="n">
         <v>0.5387231791354116</v>
@@ -2874,7 +2874,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K28" t="n">
-        <v>9.836527992101731</v>
+        <v>9.085374945432145</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2890,7 +2890,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q28" t="n">
-        <v>152.4</v>
+        <v>165</v>
       </c>
       <c r="R28" t="n">
         <v>34656</v>
@@ -2906,13 +2906,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W28" t="n">
-        <v>0.1639421332016955</v>
+        <v>0.1514229157572024</v>
       </c>
       <c r="X28" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y28" t="n">
-        <v>227.4015748031496</v>
+        <v>210.0363636363636</v>
       </c>
       <c r="Z28" t="n">
         <v>0.7209366660877885</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-26)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.362026480718872</v>
+        <v>4.45648645091232</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>792.6</v>
+        <v>775.8</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07270044134531453</v>
+        <v>0.07427477418187201</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>150.3482210446631</v>
+        <v>153.6040216550657</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.573715932232253</v>
+        <v>3.725890130278071</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>940.2</v>
+        <v>901.8</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.05956193220387087</v>
+        <v>0.06209816883796784</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>209.987662199532</v>
+        <v>218.9292526058993</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -832,7 +832,7 @@
         <v>55.0869210959395</v>
       </c>
       <c r="K5" t="n">
-        <v>3.909646635623811</v>
+        <v>3.473324154851167</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -848,7 +848,7 @@
         <v>0.348827</v>
       </c>
       <c r="Q5" t="n">
-        <v>845.4</v>
+        <v>951.5999999999999</v>
       </c>
       <c r="R5" t="n">
         <v>55194.6</v>
@@ -864,13 +864,13 @@
         <v>4.739418593887546</v>
       </c>
       <c r="W5" t="n">
-        <v>0.06516077726039686</v>
+        <v>0.05788873591418611</v>
       </c>
       <c r="X5" t="n">
         <v>0.2109963448448519</v>
       </c>
       <c r="Y5" t="n">
-        <v>65.28814762242726</v>
+        <v>58.00189155107189</v>
       </c>
       <c r="Z5" t="n">
         <v>0.9980491043678096</v>
@@ -922,7 +922,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>4.327244603594907</v>
+        <v>4.502525397664574</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -938,7 +938,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q6" t="n">
-        <v>739.8</v>
+        <v>711</v>
       </c>
       <c r="R6" t="n">
         <v>78110.8</v>
@@ -954,13 +954,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07212074339324845</v>
+        <v>0.07504208996107622</v>
       </c>
       <c r="X6" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y6" t="n">
-        <v>105.5836712625034</v>
+        <v>109.8604781997187</v>
       </c>
       <c r="Z6" t="n">
         <v>0.6830672066132366</v>
@@ -1012,7 +1012,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K7" t="n">
-        <v>7.838343660046578</v>
+        <v>7.712103864643192</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1028,7 +1028,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q7" t="n">
-        <v>403.2</v>
+        <v>409.8</v>
       </c>
       <c r="R7" t="n">
         <v>27205.5</v>
@@ -1044,13 +1044,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W7" t="n">
-        <v>0.1306390610007763</v>
+        <v>0.1285350644107199</v>
       </c>
       <c r="X7" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y7" t="n">
-        <v>67.47395833333333</v>
+        <v>66.38726207906295</v>
       </c>
       <c r="Z7" t="n">
         <v>1.936140464079432</v>
@@ -1102,7 +1102,7 @@
         <v>52.5605655745982</v>
       </c>
       <c r="K8" t="n">
-        <v>4.343848394594893</v>
+        <v>4.361872661792382</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1118,7 +1118,7 @@
         <v>0.355464</v>
       </c>
       <c r="Q8" t="n">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="R8" t="n">
         <v>61557.6</v>
@@ -1134,13 +1134,13 @@
         <v>6.522897104961693</v>
       </c>
       <c r="W8" t="n">
-        <v>0.0723974732432482</v>
+        <v>0.0726978776965397</v>
       </c>
       <c r="X8" t="n">
         <v>0.1533061128987214</v>
       </c>
       <c r="Y8" t="n">
-        <v>84.7900826446281</v>
+        <v>85.14190871369294</v>
       </c>
       <c r="Z8" t="n">
         <v>0.8538436452135594</v>
@@ -1192,7 +1192,7 @@
         <v>52.393894697293</v>
       </c>
       <c r="K9" t="n">
-        <v>9.22427723543891</v>
+        <v>10.33410151820375</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>0.575999</v>
       </c>
       <c r="Q9" t="n">
-        <v>340.8</v>
+        <v>304.2</v>
       </c>
       <c r="R9" t="n">
         <v>54476.5</v>
@@ -1224,13 +1224,13 @@
         <v>1.636041941427838</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1537379539239818</v>
+        <v>0.1722350253033958</v>
       </c>
       <c r="X9" t="n">
         <v>0.6112312738921966</v>
       </c>
       <c r="Y9" t="n">
-        <v>159.8488849765259</v>
+        <v>179.0811965811966</v>
       </c>
       <c r="Z9" t="n">
         <v>0.9617705744181987</v>
@@ -1282,7 +1282,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K10" t="n">
-        <v>4.950645625707172</v>
+        <v>5.162675269039253</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1298,7 +1298,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q10" t="n">
-        <v>628.2</v>
+        <v>602.4</v>
       </c>
       <c r="R10" t="n">
         <v>38128.4</v>
@@ -1314,13 +1314,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W10" t="n">
-        <v>0.08251076042845287</v>
+        <v>0.08604458781732088</v>
       </c>
       <c r="X10" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y10" t="n">
-        <v>60.69468322190385</v>
+        <v>63.29415670650731</v>
       </c>
       <c r="Z10" t="n">
         <v>1.359439674918279</v>
@@ -1372,7 +1372,7 @@
         <v>46.4465506302286</v>
       </c>
       <c r="K11" t="n">
-        <v>3.092313623850107</v>
+        <v>2.973530770181088</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1388,7 +1388,7 @@
         <v>0.351262</v>
       </c>
       <c r="Q11" t="n">
-        <v>901.1999999999999</v>
+        <v>937.1999999999999</v>
       </c>
       <c r="R11" t="n">
         <v>80561.39999999999</v>
@@ -1404,13 +1404,13 @@
         <v>5.571250384616186</v>
       </c>
       <c r="W11" t="n">
-        <v>0.05153856039750178</v>
+        <v>0.04955884616968481</v>
       </c>
       <c r="X11" t="n">
         <v>0.1794929200743312</v>
       </c>
       <c r="Y11" t="n">
-        <v>89.39347536617844</v>
+        <v>85.9596670934699</v>
       </c>
       <c r="Z11" t="n">
         <v>0.5765360412086756</v>
@@ -1462,7 +1462,7 @@
         <v>46.3242065310383</v>
       </c>
       <c r="K12" t="n">
-        <v>2.742700209060882</v>
+        <v>2.593740567247385</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1478,7 +1478,7 @@
         <v>0.032642</v>
       </c>
       <c r="Q12" t="n">
-        <v>1013.4</v>
+        <v>1071.6</v>
       </c>
       <c r="R12" t="n">
         <v>64275.7</v>
@@ -1494,13 +1494,13 @@
         <v>18.78273107859863</v>
       </c>
       <c r="W12" t="n">
-        <v>0.0457116701510147</v>
+        <v>0.04322900945412309</v>
       </c>
       <c r="X12" t="n">
         <v>0.05324039383918014</v>
       </c>
       <c r="Y12" t="n">
-        <v>63.42579435563449</v>
+        <v>59.98105636431504</v>
       </c>
       <c r="Z12" t="n">
         <v>0.7207110390246749</v>
@@ -1552,7 +1552,7 @@
         <v>45.4152084980521</v>
       </c>
       <c r="K13" t="n">
-        <v>1.311820002832239</v>
+        <v>1.336527619130433</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1568,7 +1568,7 @@
         <v>0.424979</v>
       </c>
       <c r="Q13" t="n">
-        <v>2077.2</v>
+        <v>2038.8</v>
       </c>
       <c r="R13" t="n">
         <v>107730.2</v>
@@ -1584,13 +1584,13 @@
         <v>1.736413207249709</v>
       </c>
       <c r="W13" t="n">
-        <v>0.02186366671387065</v>
+        <v>0.02227546031884055</v>
       </c>
       <c r="X13" t="n">
         <v>0.5758997891889408</v>
       </c>
       <c r="Y13" t="n">
-        <v>51.8631812054689</v>
+        <v>52.84000392387679</v>
       </c>
       <c r="Z13" t="n">
         <v>0.421564319921917</v>
@@ -1732,7 +1732,7 @@
         <v>44.777392385614</v>
       </c>
       <c r="K15" t="n">
-        <v>4.115569153089522</v>
+        <v>4.733339575646299</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1748,7 +1748,7 @@
         <v>0.21441</v>
       </c>
       <c r="Q15" t="n">
-        <v>652.8000000000001</v>
+        <v>567.6</v>
       </c>
       <c r="R15" t="n">
         <v>71127.60000000001</v>
@@ -1764,13 +1764,13 @@
         <v>5.159663003639629</v>
       </c>
       <c r="W15" t="n">
-        <v>0.0685928192181587</v>
+        <v>0.07888899292743834</v>
       </c>
       <c r="X15" t="n">
         <v>0.1938111072941391</v>
       </c>
       <c r="Y15" t="n">
-        <v>108.9577205882353</v>
+        <v>125.3128964059197</v>
       </c>
       <c r="Z15" t="n">
         <v>0.629536106737947</v>
@@ -1822,7 +1822,7 @@
         <v>43.7343049141614</v>
       </c>
       <c r="K16" t="n">
-        <v>9.96225624468369</v>
+        <v>9.850068674360674</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1838,7 +1838,7 @@
         <v>0.117309</v>
       </c>
       <c r="Q16" t="n">
-        <v>263.4</v>
+        <v>266.4</v>
       </c>
       <c r="R16" t="n">
         <v>64144.3</v>
@@ -1854,13 +1854,13 @@
         <v>6.639580348497565</v>
       </c>
       <c r="W16" t="n">
-        <v>0.1660376040780615</v>
+        <v>0.1641678112393446</v>
       </c>
       <c r="X16" t="n">
         <v>0.1506119283918727</v>
       </c>
       <c r="Y16" t="n">
-        <v>243.5242976461656</v>
+        <v>240.7819069069069</v>
       </c>
       <c r="Z16" t="n">
         <v>0.6818112429968274</v>
@@ -1912,7 +1912,7 @@
         <v>43.3950199670746</v>
       </c>
       <c r="K17" t="n">
-        <v>6.077733888946023</v>
+        <v>6.103378335734824</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1928,7 +1928,7 @@
         <v>0.064523</v>
       </c>
       <c r="Q17" t="n">
-        <v>428.4</v>
+        <v>426.6</v>
       </c>
       <c r="R17" t="n">
         <v>162164.2</v>
@@ -1944,13 +1944,13 @@
         <v>40.74733935074209</v>
       </c>
       <c r="W17" t="n">
-        <v>0.1012955648157671</v>
+        <v>0.1017229722622471</v>
       </c>
       <c r="X17" t="n">
         <v>0.02454147966305898</v>
       </c>
       <c r="Y17" t="n">
-        <v>378.5345471521942</v>
+        <v>380.131739334271</v>
       </c>
       <c r="Z17" t="n">
         <v>0.2675992602995889</v>
@@ -2002,7 +2002,7 @@
         <v>42.7057475126235</v>
       </c>
       <c r="K18" t="n">
-        <v>4.548002929991852</v>
+        <v>4.44388631765073</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2018,7 +2018,7 @@
         <v>0.032801</v>
       </c>
       <c r="Q18" t="n">
-        <v>563.4000000000001</v>
+        <v>576.5999999999999</v>
       </c>
       <c r="R18" t="n">
         <v>78612.3</v>
@@ -2034,13 +2034,13 @@
         <v>32.69667427900789</v>
       </c>
       <c r="W18" t="n">
-        <v>0.07580004883319755</v>
+        <v>0.07406477196084549</v>
       </c>
       <c r="X18" t="n">
         <v>0.03058415028595205</v>
       </c>
       <c r="Y18" t="n">
-        <v>139.5319488817891</v>
+        <v>136.337669094693</v>
       </c>
       <c r="Z18" t="n">
         <v>0.5432451093864892</v>
@@ -2092,7 +2092,7 @@
         <v>41.807466113455</v>
       </c>
       <c r="K19" t="n">
-        <v>3.003409921943606</v>
+        <v>3.424034898726863</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
@@ -2108,7 +2108,7 @@
         <v>0.023325</v>
       </c>
       <c r="Q19" t="n">
-        <v>835.2</v>
+        <v>732.6</v>
       </c>
       <c r="R19" t="n">
         <v>68673.2</v>
@@ -2124,13 +2124,13 @@
         <v>35.02480713696107</v>
       </c>
       <c r="W19" t="n">
-        <v>0.05005683203239344</v>
+        <v>0.05706724831211438</v>
       </c>
       <c r="X19" t="n">
         <v>0.02855119219042658</v>
       </c>
       <c r="Y19" t="n">
-        <v>82.22365900383141</v>
+        <v>93.73901173901173</v>
       </c>
       <c r="Z19" t="n">
         <v>0.6087886703030441</v>
@@ -2182,7 +2182,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K20" t="n">
-        <v>4.930871346577157</v>
+        <v>4.487525457959475</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2198,7 +2198,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q20" t="n">
-        <v>498.0000000000001</v>
+        <v>547.1999999999999</v>
       </c>
       <c r="R20" t="n">
         <v>71002.60000000001</v>
@@ -2214,13 +2214,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W20" t="n">
-        <v>0.08218118910961927</v>
+        <v>0.07479209096599124</v>
       </c>
       <c r="X20" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y20" t="n">
-        <v>142.5755020080321</v>
+        <v>129.7562134502924</v>
       </c>
       <c r="Z20" t="n">
         <v>0.5764046975264343</v>
@@ -2272,7 +2272,7 @@
         <v>38.8666662997805</v>
       </c>
       <c r="K21" t="n">
-        <v>8.217054186000105</v>
+        <v>9.320543477165588</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2288,7 +2288,7 @@
         <v>0.078199</v>
       </c>
       <c r="Q21" t="n">
-        <v>283.8</v>
+        <v>250.2</v>
       </c>
       <c r="R21" t="n">
         <v>40399</v>
@@ -2304,13 +2304,13 @@
         <v>10.31484507025962</v>
       </c>
       <c r="W21" t="n">
-        <v>0.1369509031000017</v>
+        <v>0.1553423912860931</v>
       </c>
       <c r="X21" t="n">
         <v>0.09694765100091129</v>
       </c>
       <c r="Y21" t="n">
-        <v>142.3502466525722</v>
+        <v>161.466826538769</v>
       </c>
       <c r="Z21" t="n">
         <v>0.9620700091532092</v>
@@ -2362,7 +2362,7 @@
         <v>38.3770408917494</v>
       </c>
       <c r="K22" t="n">
-        <v>3.924032811017322</v>
+        <v>4.574140749910536</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2378,7 +2378,7 @@
         <v>0.217855</v>
       </c>
       <c r="Q22" t="n">
-        <v>586.8</v>
+        <v>503.4</v>
       </c>
       <c r="R22" t="n">
         <v>69495.5</v>
@@ -2394,13 +2394,13 @@
         <v>6.24407509734128</v>
       </c>
       <c r="W22" t="n">
-        <v>0.06540054685028869</v>
+        <v>0.07623567916517561</v>
       </c>
       <c r="X22" t="n">
         <v>0.1601518214324166</v>
       </c>
       <c r="Y22" t="n">
-        <v>118.4313224267212</v>
+        <v>138.0522447357966</v>
       </c>
       <c r="Z22" t="n">
         <v>0.5522233942017742</v>
@@ -2452,7 +2452,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K23" t="n">
-        <v>6.354086447828966</v>
+        <v>6.239692092794402</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2468,7 +2468,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q23" t="n">
-        <v>360</v>
+        <v>366.6</v>
       </c>
       <c r="R23" t="n">
         <v>50011.7</v>
@@ -2484,13 +2484,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W23" t="n">
-        <v>0.1059014407971494</v>
+        <v>0.10399486821324</v>
       </c>
       <c r="X23" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y23" t="n">
-        <v>138.9213888888889</v>
+        <v>136.4203491543917</v>
       </c>
       <c r="Z23" t="n">
         <v>0.7623119927331765</v>
@@ -2542,7 +2542,7 @@
         <v>33.6762858057476</v>
       </c>
       <c r="K24" t="n">
-        <v>1.665493857851019</v>
+        <v>1.68129235175974</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2558,7 +2558,7 @@
         <v>0.143075</v>
       </c>
       <c r="Q24" t="n">
-        <v>1213.2</v>
+        <v>1201.8</v>
       </c>
       <c r="R24" t="n">
         <v>66783.2</v>
@@ -2574,13 +2574,13 @@
         <v>13.43904545346521</v>
       </c>
       <c r="W24" t="n">
-        <v>0.02775823096418365</v>
+        <v>0.02802153919599567</v>
       </c>
       <c r="X24" t="n">
         <v>0.07441004671519687</v>
       </c>
       <c r="Y24" t="n">
-        <v>55.04714803824596</v>
+        <v>55.56931269762023</v>
       </c>
       <c r="Z24" t="n">
         <v>0.5042628356494987</v>
@@ -2694,7 +2694,7 @@
         <v>30.3334426348039</v>
       </c>
       <c r="K26" t="n">
-        <v>31.59733607792074</v>
+        <v>33.70382514978211</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2710,7 +2710,7 @@
         <v>0.023374</v>
       </c>
       <c r="Q26" t="n">
-        <v>57.59999999999999</v>
+        <v>54</v>
       </c>
       <c r="R26" t="n">
         <v>26315</v>
@@ -2726,13 +2726,13 @@
         <v>40.02924671581524</v>
       </c>
       <c r="W26" t="n">
-        <v>0.5266222679653456</v>
+        <v>0.5617304191630352</v>
       </c>
       <c r="X26" t="n">
         <v>0.02498173415801272</v>
       </c>
       <c r="Y26" t="n">
-        <v>456.8576388888889</v>
+        <v>487.3148148148148</v>
       </c>
       <c r="Z26" t="n">
         <v>1.152705401284587</v>
@@ -2784,7 +2784,7 @@
         <v>26.4910658661689</v>
       </c>
       <c r="K27" t="n">
-        <v>16.45407817774466</v>
+        <v>16.66104771457163</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2800,7 +2800,7 @@
         <v>0.020469</v>
       </c>
       <c r="Q27" t="n">
-        <v>96.60000000000001</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="R27" t="n">
         <v>49173.8</v>
@@ -2816,13 +2816,13 @@
         <v>63.641894492204</v>
       </c>
       <c r="W27" t="n">
-        <v>0.2742346362957443</v>
+        <v>0.2776841285761939</v>
       </c>
       <c r="X27" t="n">
         <v>0.01571292005021155</v>
       </c>
       <c r="Y27" t="n">
-        <v>509.0455486542443</v>
+        <v>515.4486373165619</v>
       </c>
       <c r="Z27" t="n">
         <v>0.5387231791354116</v>
@@ -2874,7 +2874,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K28" t="n">
-        <v>9.085374945432145</v>
+        <v>9.759680117163438</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2890,7 +2890,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q28" t="n">
-        <v>165</v>
+        <v>153.6</v>
       </c>
       <c r="R28" t="n">
         <v>34656</v>
@@ -2906,13 +2906,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W28" t="n">
-        <v>0.1514229157572024</v>
+        <v>0.1626613352860573</v>
       </c>
       <c r="X28" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y28" t="n">
-        <v>210.0363636363636</v>
+        <v>225.625</v>
       </c>
       <c r="Z28" t="n">
         <v>0.7209366660877885</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-27)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>57.6223698102963</v>
       </c>
       <c r="K2" t="n">
-        <v>4.45648645091232</v>
+        <v>4.46339038034828</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>1.678582</v>
       </c>
       <c r="Q2" t="n">
-        <v>775.8</v>
+        <v>774.6</v>
       </c>
       <c r="R2" t="n">
         <v>119166</v>
@@ -626,13 +626,13 @@
         <v>1.111797328614408</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07427477418187201</v>
+        <v>0.07438983967247134</v>
       </c>
       <c r="X2" t="n">
         <v>0.8994445068925133</v>
       </c>
       <c r="Y2" t="n">
-        <v>153.6040216550657</v>
+        <v>153.8419829589465</v>
       </c>
       <c r="Z2" t="n">
         <v>0.4835470672028624</v>
@@ -684,7 +684,7 @@
         <v>56.0001286580794</v>
       </c>
       <c r="K3" t="n">
-        <v>3.725890130278071</v>
+        <v>3.664929885999961</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.466335</v>
       </c>
       <c r="Q3" t="n">
-        <v>901.8</v>
+        <v>916.8</v>
       </c>
       <c r="R3" t="n">
         <v>197430.4</v>
@@ -716,13 +716,13 @@
         <v>1.188266410883277</v>
       </c>
       <c r="W3" t="n">
-        <v>0.06209816883796784</v>
+        <v>0.06108216476666601</v>
       </c>
       <c r="X3" t="n">
         <v>0.8415621201113203</v>
       </c>
       <c r="Y3" t="n">
-        <v>218.9292526058993</v>
+        <v>215.347294938918</v>
       </c>
       <c r="Z3" t="n">
         <v>0.2836449131343471</v>
@@ -832,7 +832,7 @@
         <v>55.0869210959395</v>
       </c>
       <c r="K5" t="n">
-        <v>3.473324154851167</v>
+        <v>2.876601623808852</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -848,7 +848,7 @@
         <v>0.348827</v>
       </c>
       <c r="Q5" t="n">
-        <v>951.5999999999999</v>
+        <v>1149</v>
       </c>
       <c r="R5" t="n">
         <v>55194.6</v>
@@ -864,13 +864,13 @@
         <v>4.739418593887546</v>
       </c>
       <c r="W5" t="n">
-        <v>0.05788873591418611</v>
+        <v>0.04794336039681419</v>
       </c>
       <c r="X5" t="n">
         <v>0.2109963448448519</v>
       </c>
       <c r="Y5" t="n">
-        <v>58.00189155107189</v>
+        <v>48.03707571801566</v>
       </c>
       <c r="Z5" t="n">
         <v>0.9980491043678096</v>
@@ -922,7 +922,7 @@
         <v>53.3549259623252</v>
       </c>
       <c r="K6" t="n">
-        <v>4.502525397664574</v>
+        <v>4.316741582712395</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -938,7 +938,7 @@
         <v>2.361991</v>
       </c>
       <c r="Q6" t="n">
-        <v>711</v>
+        <v>741.5999999999999</v>
       </c>
       <c r="R6" t="n">
         <v>78110.8</v>
@@ -954,13 +954,13 @@
         <v>0.7646201649272464</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07504208996107622</v>
+        <v>0.07194569304520658</v>
       </c>
       <c r="X6" t="n">
         <v>1.307838905994782</v>
       </c>
       <c r="Y6" t="n">
-        <v>109.8604781997187</v>
+        <v>105.3274002157497</v>
       </c>
       <c r="Z6" t="n">
         <v>0.6830672066132366</v>
@@ -1012,7 +1012,7 @@
         <v>52.673669395513</v>
       </c>
       <c r="K7" t="n">
-        <v>7.712103864643192</v>
+        <v>7.932781535468826</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1028,7 +1028,7 @@
         <v>0.834562</v>
       </c>
       <c r="Q7" t="n">
-        <v>409.8</v>
+        <v>398.4</v>
       </c>
       <c r="R7" t="n">
         <v>27205.5</v>
@@ -1044,13 +1044,13 @@
         <v>4.408234261998002</v>
       </c>
       <c r="W7" t="n">
-        <v>0.1285350644107199</v>
+        <v>0.1322130255911471</v>
       </c>
       <c r="X7" t="n">
         <v>0.2268481982957858</v>
       </c>
       <c r="Y7" t="n">
-        <v>66.38726207906295</v>
+        <v>68.28689759036145</v>
       </c>
       <c r="Z7" t="n">
         <v>1.936140464079432</v>
@@ -1102,7 +1102,7 @@
         <v>52.5605655745982</v>
       </c>
       <c r="K8" t="n">
-        <v>4.361872661792382</v>
+        <v>4.365495479617791</v>
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="n">
@@ -1118,7 +1118,7 @@
         <v>0.355464</v>
       </c>
       <c r="Q8" t="n">
-        <v>723</v>
+        <v>722.4</v>
       </c>
       <c r="R8" t="n">
         <v>61557.6</v>
@@ -1134,13 +1134,13 @@
         <v>6.522897104961693</v>
       </c>
       <c r="W8" t="n">
-        <v>0.0726978776965397</v>
+        <v>0.07275825799362985</v>
       </c>
       <c r="X8" t="n">
         <v>0.1533061128987214</v>
       </c>
       <c r="Y8" t="n">
-        <v>85.14190871369294</v>
+        <v>85.2126245847176</v>
       </c>
       <c r="Z8" t="n">
         <v>0.8538436452135594</v>
@@ -1192,7 +1192,7 @@
         <v>52.393894697293</v>
       </c>
       <c r="K9" t="n">
-        <v>10.33410151820375</v>
+        <v>12.27023295018572</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>0.575999</v>
       </c>
       <c r="Q9" t="n">
-        <v>304.2</v>
+        <v>256.2</v>
       </c>
       <c r="R9" t="n">
         <v>54476.5</v>
@@ -1224,13 +1224,13 @@
         <v>1.636041941427838</v>
       </c>
       <c r="W9" t="n">
-        <v>0.1722350253033958</v>
+        <v>0.2045038825030953</v>
       </c>
       <c r="X9" t="n">
         <v>0.6112312738921966</v>
       </c>
       <c r="Y9" t="n">
-        <v>179.0811965811966</v>
+        <v>212.6327088212334</v>
       </c>
       <c r="Z9" t="n">
         <v>0.9617705744181987</v>
@@ -1282,7 +1282,7 @@
         <v>51.8332597011541</v>
       </c>
       <c r="K10" t="n">
-        <v>5.162675269039253</v>
+        <v>6.215019148819437</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1298,7 +1298,7 @@
         <v>0.2519</v>
       </c>
       <c r="Q10" t="n">
-        <v>602.4</v>
+        <v>500.4</v>
       </c>
       <c r="R10" t="n">
         <v>38128.4</v>
@@ -1314,13 +1314,13 @@
         <v>17.10866826525254</v>
       </c>
       <c r="W10" t="n">
-        <v>0.08604458781732088</v>
+        <v>0.1035836524803239</v>
       </c>
       <c r="X10" t="n">
         <v>0.05844990296708164</v>
       </c>
       <c r="Y10" t="n">
-        <v>63.29415670650731</v>
+        <v>76.19584332533974</v>
       </c>
       <c r="Z10" t="n">
         <v>1.359439674918279</v>
@@ -1329,32 +1329,32 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>grok-4-7</t>
+          <t>gpt-6-1-terra</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Grok 4.7 (Xhigh)</t>
+          <t>GPT-6.1 Terra (Max)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Grok 4.7 (xhigh)</t>
+          <t>GPT-6.1 Terra (max)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SpaceXAI</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>xai</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1369,77 +1369,77 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>46.4465506302286</v>
+        <v>48.1061836463044</v>
       </c>
       <c r="K11" t="n">
-        <v>2.973530770181088</v>
+        <v>7.504864843417224</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
-        <v>8.336827</v>
+        <v>2.553753</v>
       </c>
       <c r="N11" t="n">
-        <v>7.853459</v>
+        <v>2.378273</v>
       </c>
       <c r="O11" t="n">
-        <v>0.132106</v>
+        <v>0.051021</v>
       </c>
       <c r="P11" t="n">
-        <v>0.351262</v>
+        <v>0.124459</v>
       </c>
       <c r="Q11" t="n">
-        <v>937.1999999999999</v>
+        <v>384.6</v>
       </c>
       <c r="R11" t="n">
-        <v>80561.39999999999</v>
+        <v>35096</v>
       </c>
       <c r="S11" t="n">
-        <v>22017.7</v>
+        <v>10204.2</v>
       </c>
       <c r="T11" t="n">
-        <v>58543.6</v>
+        <v>24891.8</v>
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>5.571250384616186</v>
+        <v>18.83744576954169</v>
       </c>
       <c r="W11" t="n">
-        <v>0.04955884616968481</v>
+        <v>0.1250810807236204</v>
       </c>
       <c r="X11" t="n">
-        <v>0.1794929200743312</v>
+        <v>0.05308575335711927</v>
       </c>
       <c r="Y11" t="n">
-        <v>85.9596670934699</v>
+        <v>91.2532501300052</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.5765360412086756</v>
+        <v>1.370702748071131</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>mimo-v2-6-pro</t>
+          <t>grok-4-7</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Grok 4.7 (Xhigh)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Grok 4.7 (xhigh)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Xiaomi</t>
+          <t>SpaceXAI</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>xiaomi</t>
+          <t>xai</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1456,85 +1456,85 @@
         <v>1</v>
       </c>
       <c r="I12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>46.3242065310383</v>
+        <v>46.4465506302286</v>
       </c>
       <c r="K12" t="n">
-        <v>2.593740567247385</v>
+        <v>3.207634712032362</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
-        <v>2.466319</v>
+        <v>8.336827</v>
       </c>
       <c r="N12" t="n">
-        <v>2.410399</v>
+        <v>7.853459</v>
       </c>
       <c r="O12" t="n">
-        <v>0.023278</v>
+        <v>0.132106</v>
       </c>
       <c r="P12" t="n">
-        <v>0.032642</v>
+        <v>0.351262</v>
       </c>
       <c r="Q12" t="n">
-        <v>1071.6</v>
+        <v>868.8000000000001</v>
       </c>
       <c r="R12" t="n">
-        <v>64275.7</v>
+        <v>80561.39999999999</v>
       </c>
       <c r="S12" t="n">
-        <v>26756</v>
+        <v>22017.7</v>
       </c>
       <c r="T12" t="n">
-        <v>37519.7</v>
+        <v>58543.6</v>
       </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="n">
-        <v>18.78273107859863</v>
+        <v>5.571250384616186</v>
       </c>
       <c r="W12" t="n">
-        <v>0.04322900945412309</v>
+        <v>0.05346057853387269</v>
       </c>
       <c r="X12" t="n">
-        <v>0.05324039383918014</v>
+        <v>0.1794929200743312</v>
       </c>
       <c r="Y12" t="n">
-        <v>59.98105636431504</v>
+        <v>92.72720994475137</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.7207110390246749</v>
+        <v>0.5765360412086756</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>qwen3-8-max</t>
+          <t>mimo-v2-6-pro</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Qwen3.8 Max (0902)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>Xiaomi</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>xiaomi</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1546,85 +1546,85 @@
         <v>1</v>
       </c>
       <c r="I13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" t="n">
-        <v>45.4152084980521</v>
+        <v>46.3242065310383</v>
       </c>
       <c r="K13" t="n">
-        <v>1.336527619130433</v>
+        <v>2.731380102065937</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
-        <v>26.154609</v>
+        <v>2.466319</v>
       </c>
       <c r="N13" t="n">
-        <v>25.508227</v>
+        <v>2.410399</v>
       </c>
       <c r="O13" t="n">
-        <v>0.221402</v>
+        <v>0.023278</v>
       </c>
       <c r="P13" t="n">
-        <v>0.424979</v>
+        <v>0.032642</v>
       </c>
       <c r="Q13" t="n">
-        <v>2038.8</v>
+        <v>1017.6</v>
       </c>
       <c r="R13" t="n">
-        <v>107730.2</v>
+        <v>64275.7</v>
       </c>
       <c r="S13" t="n">
-        <v>36900.3</v>
+        <v>26756</v>
       </c>
       <c r="T13" t="n">
-        <v>70829.89999999999</v>
+        <v>37519.7</v>
       </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="n">
-        <v>1.736413207249709</v>
+        <v>18.78273107859863</v>
       </c>
       <c r="W13" t="n">
-        <v>0.02227546031884055</v>
+        <v>0.04552300170109896</v>
       </c>
       <c r="X13" t="n">
-        <v>0.5758997891889408</v>
+        <v>0.05324039383918014</v>
       </c>
       <c r="Y13" t="n">
-        <v>52.84000392387679</v>
+        <v>63.16401336477987</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.421564319921917</v>
+        <v>0.7207110390246749</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>deepseek-v4-1-flash-1017</t>
+          <t>qwen3-8-max</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash 1017 (Max)</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>DeepSeek V4.1 Flash 1017 (max)</t>
+          <t>Qwen3.8 Max (0902)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>DeepSeek</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>deepseek</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1636,85 +1636,85 @@
         <v>1</v>
       </c>
       <c r="I14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>45.0965048681912</v>
+        <v>45.4152084980521</v>
       </c>
       <c r="K14" t="n">
-        <v>6.822466697154493</v>
+        <v>1.308795633949628</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>3.00199</v>
+        <v>26.154609</v>
       </c>
       <c r="N14" t="n">
-        <v>2.894596</v>
+        <v>25.508227</v>
       </c>
       <c r="O14" t="n">
-        <v>0.036302</v>
+        <v>0.221402</v>
       </c>
       <c r="P14" t="n">
-        <v>0.071092</v>
+        <v>0.424979</v>
       </c>
       <c r="Q14" t="n">
-        <v>396.6</v>
+        <v>2082</v>
       </c>
       <c r="R14" t="n">
-        <v>89495.10000000001</v>
+        <v>107730.2</v>
       </c>
       <c r="S14" t="n">
-        <v>30252</v>
+        <v>36900.3</v>
       </c>
       <c r="T14" t="n">
-        <v>59243</v>
+        <v>70829.89999999999</v>
       </c>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="n">
-        <v>15.02220356103491</v>
+        <v>1.736413207249709</v>
       </c>
       <c r="W14" t="n">
-        <v>0.1137077782859082</v>
+        <v>0.02181326056582714</v>
       </c>
       <c r="X14" t="n">
-        <v>0.06656813003079209</v>
+        <v>0.5758997891889408</v>
       </c>
       <c r="Y14" t="n">
-        <v>225.6558245083207</v>
+        <v>51.74361191162344</v>
       </c>
       <c r="Z14" t="n">
-        <v>0.5038991505478086</v>
+        <v>0.421564319921917</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>glm-5-3</t>
+          <t>deepseek-v4-1-flash-1017</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>GLM-5.3 (Max)</t>
+          <t>DeepSeek V4.1 Flash 1017 (Max)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>DeepSeek V4.1 Flash 1017 (max)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>DeepSeek</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>deepseek</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1729,82 +1729,82 @@
         <v>1</v>
       </c>
       <c r="J15" t="n">
-        <v>44.777392385614</v>
+        <v>45.0965048681912</v>
       </c>
       <c r="K15" t="n">
-        <v>4.733339575646299</v>
+        <v>7.046328885654874</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>8.678356000000001</v>
+        <v>3.00199</v>
       </c>
       <c r="N15" t="n">
-        <v>8.365394999999999</v>
+        <v>2.894596</v>
       </c>
       <c r="O15" t="n">
-        <v>0.098552</v>
+        <v>0.036302</v>
       </c>
       <c r="P15" t="n">
-        <v>0.21441</v>
+        <v>0.071092</v>
       </c>
       <c r="Q15" t="n">
-        <v>567.6</v>
+        <v>384</v>
       </c>
       <c r="R15" t="n">
-        <v>71127.60000000001</v>
+        <v>89495.10000000001</v>
       </c>
       <c r="S15" t="n">
-        <v>22398.1</v>
+        <v>30252</v>
       </c>
       <c r="T15" t="n">
-        <v>48729.5</v>
+        <v>59243</v>
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="n">
-        <v>5.159663003639629</v>
+        <v>15.02220356103491</v>
       </c>
       <c r="W15" t="n">
-        <v>0.07888899292743834</v>
+        <v>0.1174388147609146</v>
       </c>
       <c r="X15" t="n">
-        <v>0.1938111072941391</v>
+        <v>0.06656813003079209</v>
       </c>
       <c r="Y15" t="n">
-        <v>125.3128964059197</v>
+        <v>233.06015625</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.629536106737947</v>
+        <v>0.5038991505478086</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>step-5</t>
+          <t>glm-5-3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>GLM-5.3 (Max)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>StepFun</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>stepfun</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1819,172 +1819,172 @@
         <v>1</v>
       </c>
       <c r="J16" t="n">
-        <v>43.7343049141614</v>
+        <v>44.777392385614</v>
       </c>
       <c r="K16" t="n">
-        <v>9.850068674360674</v>
+        <v>4.119355325263478</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
-        <v>6.586908</v>
+        <v>8.678356000000001</v>
       </c>
       <c r="N16" t="n">
-        <v>6.413718</v>
+        <v>8.365394999999999</v>
       </c>
       <c r="O16" t="n">
-        <v>0.055881</v>
+        <v>0.098552</v>
       </c>
       <c r="P16" t="n">
-        <v>0.117309</v>
+        <v>0.21441</v>
       </c>
       <c r="Q16" t="n">
-        <v>266.4</v>
+        <v>652.1999999999999</v>
       </c>
       <c r="R16" t="n">
-        <v>64144.3</v>
+        <v>71127.60000000001</v>
       </c>
       <c r="S16" t="n">
-        <v>20696.6</v>
+        <v>22398.1</v>
       </c>
       <c r="T16" t="n">
-        <v>43447.7</v>
+        <v>48729.5</v>
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="n">
-        <v>6.639580348497565</v>
+        <v>5.159663003639629</v>
       </c>
       <c r="W16" t="n">
-        <v>0.1641678112393446</v>
+        <v>0.06865592208772463</v>
       </c>
       <c r="X16" t="n">
-        <v>0.1506119283918727</v>
+        <v>0.1938111072941391</v>
       </c>
       <c r="Y16" t="n">
-        <v>240.7819069069069</v>
+        <v>109.0579576816928</v>
       </c>
       <c r="Z16" t="n">
-        <v>0.6818112429968274</v>
+        <v>0.629536106737947</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>claude-haiku-5-5</t>
+          <t>step-5</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Claude Haiku 5.5 (Max)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Claude Haiku 5.5 (max)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>StepFun</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>stepfun</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H17" t="b">
         <v>1</v>
       </c>
       <c r="I17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17" t="n">
-        <v>43.3950199670746</v>
+        <v>43.7343049141614</v>
       </c>
       <c r="K17" t="n">
-        <v>6.103378335734824</v>
+        <v>8.558572390246848</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
-        <v>1.064978</v>
+        <v>6.586908</v>
       </c>
       <c r="N17" t="n">
-        <v>0.983896</v>
+        <v>6.413718</v>
       </c>
       <c r="O17" t="n">
-        <v>0.016559</v>
+        <v>0.055881</v>
       </c>
       <c r="P17" t="n">
-        <v>0.064523</v>
+        <v>0.117309</v>
       </c>
       <c r="Q17" t="n">
-        <v>426.6</v>
+        <v>306.6</v>
       </c>
       <c r="R17" t="n">
-        <v>162164.2</v>
+        <v>64144.3</v>
       </c>
       <c r="S17" t="n">
-        <v>33117.6</v>
+        <v>20696.6</v>
       </c>
       <c r="T17" t="n">
-        <v>129046.6</v>
+        <v>43447.7</v>
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="n">
-        <v>40.74733935074209</v>
+        <v>6.639580348497565</v>
       </c>
       <c r="W17" t="n">
-        <v>0.1017229722622471</v>
+        <v>0.1426428731707808</v>
       </c>
       <c r="X17" t="n">
-        <v>0.02454147966305898</v>
+        <v>0.1506119283918727</v>
       </c>
       <c r="Y17" t="n">
-        <v>380.131739334271</v>
+        <v>209.2116764514025</v>
       </c>
       <c r="Z17" t="n">
-        <v>0.2675992602995889</v>
+        <v>0.6818112429968274</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>minimax-m3-1-flash</t>
+          <t>claude-haiku-5-5</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MiniMax-M3.1-Flash</t>
+          <t>Claude Haiku 5.5 (Max)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MiniMax-M3.1-Flash</t>
+          <t>Claude Haiku 5.5 (max)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>minimax</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1999,141 +1999,141 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>42.7057475126235</v>
+        <v>43.3950199670746</v>
       </c>
       <c r="K18" t="n">
-        <v>4.44388631765073</v>
+        <v>6.111974643249944</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
-        <v>1.306119</v>
+        <v>1.064978</v>
       </c>
       <c r="N18" t="n">
-        <v>1.258952</v>
+        <v>0.983896</v>
       </c>
       <c r="O18" t="n">
-        <v>0.014367</v>
+        <v>0.016559</v>
       </c>
       <c r="P18" t="n">
-        <v>0.032801</v>
+        <v>0.064523</v>
       </c>
       <c r="Q18" t="n">
-        <v>576.5999999999999</v>
+        <v>426</v>
       </c>
       <c r="R18" t="n">
-        <v>78612.3</v>
+        <v>162164.2</v>
       </c>
       <c r="S18" t="n">
-        <v>23944.7</v>
+        <v>33117.6</v>
       </c>
       <c r="T18" t="n">
-        <v>54667.6</v>
+        <v>129046.6</v>
       </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="n">
-        <v>32.69667427900789</v>
+        <v>40.74733935074209</v>
       </c>
       <c r="W18" t="n">
-        <v>0.07406477196084549</v>
+        <v>0.1018662440541657</v>
       </c>
       <c r="X18" t="n">
-        <v>0.03058415028595205</v>
+        <v>0.02454147966305898</v>
       </c>
       <c r="Y18" t="n">
-        <v>136.337669094693</v>
+        <v>380.6671361502348</v>
       </c>
       <c r="Z18" t="n">
-        <v>0.5432451093864892</v>
+        <v>0.2675992602995889</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>glm-5-3-flash</t>
+          <t>minimax-m3-1-flash</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>MiniMax-M3.1-Flash</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>MiniMax-M3.1-Flash</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>minimax</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H19" t="b">
         <v>1</v>
       </c>
       <c r="I19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>41.807466113455</v>
+        <v>42.7057475126235</v>
       </c>
       <c r="K19" t="n">
-        <v>3.424034898726863</v>
+        <v>4.398120238169258</v>
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
-        <v>1.193653</v>
+        <v>1.306119</v>
       </c>
       <c r="N19" t="n">
-        <v>1.159316</v>
+        <v>1.258952</v>
       </c>
       <c r="O19" t="n">
-        <v>0.011012</v>
+        <v>0.014367</v>
       </c>
       <c r="P19" t="n">
-        <v>0.023325</v>
+        <v>0.032801</v>
       </c>
       <c r="Q19" t="n">
-        <v>732.6</v>
+        <v>582.6</v>
       </c>
       <c r="R19" t="n">
-        <v>68673.2</v>
+        <v>78612.3</v>
       </c>
       <c r="S19" t="n">
-        <v>22023.7</v>
+        <v>23944.7</v>
       </c>
       <c r="T19" t="n">
-        <v>46649.5</v>
+        <v>54667.6</v>
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="n">
-        <v>35.02480713696107</v>
+        <v>32.69667427900789</v>
       </c>
       <c r="W19" t="n">
-        <v>0.05706724831211438</v>
+        <v>0.07330200396948765</v>
       </c>
       <c r="X19" t="n">
-        <v>0.02855119219042658</v>
+        <v>0.03058415028595205</v>
       </c>
       <c r="Y19" t="n">
-        <v>93.73901173901173</v>
+        <v>134.9335736354274</v>
       </c>
       <c r="Z19" t="n">
-        <v>0.6087886703030441</v>
+        <v>0.5432451093864892</v>
       </c>
     </row>
     <row r="20">
@@ -2182,7 +2182,7 @@
         <v>40.9262321765904</v>
       </c>
       <c r="K20" t="n">
-        <v>4.487525457959475</v>
+        <v>4.725892861038153</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2198,7 +2198,7 @@
         <v>0.160227</v>
       </c>
       <c r="Q20" t="n">
-        <v>547.1999999999999</v>
+        <v>519.6</v>
       </c>
       <c r="R20" t="n">
         <v>71002.60000000001</v>
@@ -2214,13 +2214,13 @@
         <v>8.350554002348574</v>
       </c>
       <c r="W20" t="n">
-        <v>0.07479209096599124</v>
+        <v>0.07876488101730254</v>
       </c>
       <c r="X20" t="n">
         <v>0.119752533750306</v>
       </c>
       <c r="Y20" t="n">
-        <v>129.7562134502924</v>
+        <v>136.6485758275597</v>
       </c>
       <c r="Z20" t="n">
         <v>0.5764046975264343</v>
@@ -2272,48 +2272,48 @@
         <v>38.8666662997805</v>
       </c>
       <c r="K21" t="n">
-        <v>9.320543477165588</v>
+        <v>11.77777766660015</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
-        <v>3.768032</v>
+        <v>3.768433</v>
       </c>
       <c r="N21" t="n">
-        <v>3.596336</v>
+        <v>3.596656</v>
       </c>
       <c r="O21" t="n">
-        <v>0.093496</v>
+        <v>0.093573</v>
       </c>
       <c r="P21" t="n">
-        <v>0.078199</v>
+        <v>0.078204</v>
       </c>
       <c r="Q21" t="n">
-        <v>250.2</v>
+        <v>198</v>
       </c>
       <c r="R21" t="n">
-        <v>40399</v>
+        <v>40418.1</v>
       </c>
       <c r="S21" t="n">
-        <v>21999.2</v>
+        <v>22017.2</v>
       </c>
       <c r="T21" t="n">
-        <v>18399.8</v>
+        <v>18400.9</v>
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="n">
-        <v>10.31484507025962</v>
+        <v>10.3137474647368</v>
       </c>
       <c r="W21" t="n">
-        <v>0.1553423912860931</v>
+        <v>0.1962962944433359</v>
       </c>
       <c r="X21" t="n">
-        <v>0.09694765100091129</v>
+        <v>0.09695796832519393</v>
       </c>
       <c r="Y21" t="n">
-        <v>161.466826538769</v>
+        <v>204.1318181818182</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.9620700091532092</v>
+        <v>0.9616153728102138</v>
       </c>
     </row>
     <row r="22">
@@ -2362,7 +2362,7 @@
         <v>38.3770408917494</v>
       </c>
       <c r="K22" t="n">
-        <v>4.574140749910536</v>
+        <v>4.346210746517486</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2378,7 +2378,7 @@
         <v>0.217855</v>
       </c>
       <c r="Q22" t="n">
-        <v>503.4</v>
+        <v>529.8</v>
       </c>
       <c r="R22" t="n">
         <v>69495.5</v>
@@ -2394,13 +2394,13 @@
         <v>6.24407509734128</v>
       </c>
       <c r="W22" t="n">
-        <v>0.07623567916517561</v>
+        <v>0.07243684577529144</v>
       </c>
       <c r="X22" t="n">
         <v>0.1601518214324166</v>
       </c>
       <c r="Y22" t="n">
-        <v>138.0522447357966</v>
+        <v>131.1730841827105</v>
       </c>
       <c r="Z22" t="n">
         <v>0.5522233942017742</v>
@@ -2452,7 +2452,7 @@
         <v>38.1245186869738</v>
       </c>
       <c r="K23" t="n">
-        <v>6.239692092794402</v>
+        <v>5.767703280934009</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2468,7 +2468,7 @@
         <v>0.019445</v>
       </c>
       <c r="Q23" t="n">
-        <v>366.6</v>
+        <v>396.6</v>
       </c>
       <c r="R23" t="n">
         <v>50011.7</v>
@@ -2484,13 +2484,13 @@
         <v>116.8474502782117</v>
       </c>
       <c r="W23" t="n">
-        <v>0.10399486821324</v>
+        <v>0.09612838801556682</v>
       </c>
       <c r="X23" t="n">
         <v>0.008558167059863248</v>
       </c>
       <c r="Y23" t="n">
-        <v>136.4203491543917</v>
+        <v>126.1011094301563</v>
       </c>
       <c r="Z23" t="n">
         <v>0.7623119927331765</v>
@@ -2542,7 +2542,7 @@
         <v>33.6762858057476</v>
       </c>
       <c r="K24" t="n">
-        <v>1.68129235175974</v>
+        <v>1.682132158129251</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2558,7 +2558,7 @@
         <v>0.143075</v>
       </c>
       <c r="Q24" t="n">
-        <v>1201.8</v>
+        <v>1201.2</v>
       </c>
       <c r="R24" t="n">
         <v>66783.2</v>
@@ -2574,13 +2574,13 @@
         <v>13.43904545346521</v>
       </c>
       <c r="W24" t="n">
-        <v>0.02802153919599567</v>
+        <v>0.02803553596882084</v>
       </c>
       <c r="X24" t="n">
         <v>0.07441004671519687</v>
       </c>
       <c r="Y24" t="n">
-        <v>55.56931269762023</v>
+        <v>55.59706959706959</v>
       </c>
       <c r="Z24" t="n">
         <v>0.5042628356494987</v>
@@ -2694,7 +2694,7 @@
         <v>30.3334426348039</v>
       </c>
       <c r="K26" t="n">
-        <v>33.70382514978211</v>
+        <v>37.44869461086901</v>
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="n">
@@ -2710,7 +2710,7 @@
         <v>0.023374</v>
       </c>
       <c r="Q26" t="n">
-        <v>54</v>
+        <v>48.6</v>
       </c>
       <c r="R26" t="n">
         <v>26315</v>
@@ -2726,13 +2726,13 @@
         <v>40.02924671581524</v>
       </c>
       <c r="W26" t="n">
-        <v>0.5617304191630352</v>
+        <v>0.6241449101811503</v>
       </c>
       <c r="X26" t="n">
         <v>0.02498173415801272</v>
       </c>
       <c r="Y26" t="n">
-        <v>487.3148148148148</v>
+        <v>541.4609053497942</v>
       </c>
       <c r="Z26" t="n">
         <v>1.152705401284587</v>
@@ -2874,7 +2874,7 @@
         <v>24.9847810999384</v>
       </c>
       <c r="K28" t="n">
-        <v>9.759680117163438</v>
+        <v>10.32428971071835</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2890,7 +2890,7 @@
         <v>0.094767</v>
       </c>
       <c r="Q28" t="n">
-        <v>153.6</v>
+        <v>145.2</v>
       </c>
       <c r="R28" t="n">
         <v>34656</v>
@@ -2906,13 +2906,13 @@
         <v>10.32857478885389</v>
       </c>
       <c r="W28" t="n">
-        <v>0.1626613352860573</v>
+        <v>0.1720714951786391</v>
       </c>
       <c r="X28" t="n">
         <v>0.09681877901287532</v>
       </c>
       <c r="Y28" t="n">
-        <v>225.625</v>
+        <v>238.6776859504132</v>
       </c>
       <c r="Z28" t="n">
         <v>0.7209366660877885</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-28)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z28"/>
+  <dimension ref="A1:Z29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -591,82 +591,82 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>57.6223698102963</v>
+        <v>58.4060336078904</v>
       </c>
       <c r="K2" t="n">
-        <v>4.46339038034828</v>
+        <v>4.520590836524025</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
-        <v>51.828124</v>
+        <v>51.818032</v>
       </c>
       <c r="N2" t="n">
-        <v>49.444803</v>
+        <v>49.444751</v>
       </c>
       <c r="O2" t="n">
-        <v>0.704739</v>
+        <v>0.704638</v>
       </c>
       <c r="P2" t="n">
-        <v>1.678582</v>
+        <v>1.668643</v>
       </c>
       <c r="Q2" t="n">
-        <v>774.6</v>
+        <v>775.2</v>
       </c>
       <c r="R2" t="n">
-        <v>119166</v>
+        <v>118664.1</v>
       </c>
       <c r="S2" t="n">
-        <v>35236.9</v>
+        <v>35231.9</v>
       </c>
       <c r="T2" t="n">
-        <v>83929.10000000001</v>
+        <v>83432.10000000001</v>
       </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="n">
-        <v>1.111797328614408</v>
+        <v>1.127137240717486</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07438983967247134</v>
+        <v>0.07534318060873374</v>
       </c>
       <c r="X2" t="n">
-        <v>0.8994445068925133</v>
+        <v>0.8872034068925305</v>
       </c>
       <c r="Y2" t="n">
-        <v>153.8419829589465</v>
+        <v>153.0754643962848</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.4835470672028624</v>
+        <v>0.492196322290317</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>claude-sonnet-5-5</t>
+          <t>gpt-6-astra</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5.5 (Max, Default Fallback)</t>
+          <t>GPT-6 Astra (Max)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5.5 (max with fallback)</t>
+          <t>GPT-6 Astra (max)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -681,85 +681,89 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>56.0001286580794</v>
+        <v>56.8538559596797</v>
       </c>
       <c r="K3" t="n">
-        <v>3.664929885999961</v>
+        <v>9.214563364615834</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
-        <v>47.127587</v>
+        <v>11.94179</v>
       </c>
       <c r="N3" t="n">
-        <v>45.153283</v>
+        <v>10.588558</v>
       </c>
       <c r="O3" t="n">
-        <v>0.507969</v>
+        <v>0.52565</v>
       </c>
       <c r="P3" t="n">
-        <v>1.466335</v>
+        <v>0.827582</v>
       </c>
       <c r="Q3" t="n">
-        <v>916.8</v>
+        <v>370.2</v>
       </c>
       <c r="R3" t="n">
-        <v>197430.4</v>
+        <v>27064.6</v>
       </c>
       <c r="S3" t="n">
-        <v>50796.9</v>
+        <v>10513</v>
       </c>
       <c r="T3" t="n">
-        <v>146633.5</v>
+        <v>16551.6</v>
       </c>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="n">
-        <v>1.188266410883277</v>
+        <v>4.76091573873596</v>
       </c>
       <c r="W3" t="n">
-        <v>0.06108216476666601</v>
+        <v>0.1535760560769306</v>
       </c>
       <c r="X3" t="n">
-        <v>0.8415621201113203</v>
+        <v>0.210043624982429</v>
       </c>
       <c r="Y3" t="n">
-        <v>215.347294938918</v>
+        <v>73.10804970286331</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.2836449131343471</v>
+        <v>2.100672315854648</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>muse-wonder-full</t>
+          <t>gpt-6-1-sol</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Muse Wonder Full (Max)</t>
+          <t>GPT-6.1 Sol (Max)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Muse Wonder Full (max)</t>
+          <t>GPT-6.1 Sol (max)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
       <c r="H4" t="b">
         <v>1</v>
       </c>
@@ -767,54 +771,82 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>55.8021199855616</v>
-      </c>
-      <c r="K4" t="inlineStr"/>
+        <v>54.5087338138148</v>
+      </c>
+      <c r="K4" t="n">
+        <v>6.796600226161447</v>
+      </c>
       <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
+      <c r="M4" t="n">
+        <v>3.028512</v>
+      </c>
+      <c r="N4" t="n">
+        <v>2.648346</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.129372</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.250794</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>481.2</v>
+      </c>
+      <c r="R4" t="n">
+        <v>38016.6</v>
+      </c>
+      <c r="S4" t="n">
+        <v>12937.2</v>
+      </c>
+      <c r="T4" t="n">
+        <v>25079.4</v>
+      </c>
       <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
+      <c r="V4" t="n">
+        <v>17.99852000382194</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.1132766704360241</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0.05556012382060594</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>79.00374064837905</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>1.433814013189365</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>kimi-k3-1-pro</t>
+          <t>claude-sonnet-5-5</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Kimi K3.1 Pro</t>
+          <t>Claude Sonnet 5.5 (Max, Default Fallback)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Kimi K3.1 Pro</t>
+          <t>Claude Sonnet 5.5 (max with fallback)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Kimi</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>kimi</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -829,82 +861,82 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>55.0869210959395</v>
+        <v>54.24133407109</v>
       </c>
       <c r="K5" t="n">
-        <v>2.876601623808852</v>
+        <v>3.568508820466448</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
-        <v>11.623139</v>
+        <v>47.116982</v>
       </c>
       <c r="N5" t="n">
-        <v>11.071193</v>
+        <v>45.153257</v>
       </c>
       <c r="O5" t="n">
-        <v>0.203119</v>
+        <v>0.507917</v>
       </c>
       <c r="P5" t="n">
-        <v>0.348827</v>
+        <v>1.455808</v>
       </c>
       <c r="Q5" t="n">
-        <v>1149</v>
+        <v>912</v>
       </c>
       <c r="R5" t="n">
-        <v>55194.6</v>
+        <v>196372.5</v>
       </c>
       <c r="S5" t="n">
-        <v>20311.9</v>
+        <v>50791.7</v>
       </c>
       <c r="T5" t="n">
-        <v>34882.7</v>
+        <v>145580.8</v>
       </c>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="n">
-        <v>4.739418593887546</v>
+        <v>1.151205611409704</v>
       </c>
       <c r="W5" t="n">
-        <v>0.04794336039681419</v>
+        <v>0.05947514700777413</v>
       </c>
       <c r="X5" t="n">
-        <v>0.2109963448448519</v>
+        <v>0.8686545566568725</v>
       </c>
       <c r="Y5" t="n">
-        <v>48.03707571801566</v>
+        <v>215.3207236842105</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.9980491043678096</v>
+        <v>0.276216547994704</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>claude-fable-5-1</t>
+          <t>gpt-6-1-terra</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (Max, Default Fallback)</t>
+          <t>GPT-6.1 Terra (Max)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (max with fallback)</t>
+          <t>GPT-6.1 Terra (max)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -919,82 +951,82 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>53.3549259623252</v>
+        <v>50.9765188577015</v>
       </c>
       <c r="K6" t="n">
-        <v>4.316741582712395</v>
+        <v>8.065904882547704</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
-        <v>69.77964799999999</v>
+        <v>2.551231</v>
       </c>
       <c r="N6" t="n">
-        <v>65.87410800000001</v>
+        <v>2.378263</v>
       </c>
       <c r="O6" t="n">
-        <v>1.54355</v>
+        <v>0.051016</v>
       </c>
       <c r="P6" t="n">
-        <v>2.361991</v>
+        <v>0.121952</v>
       </c>
       <c r="Q6" t="n">
-        <v>741.5999999999999</v>
+        <v>379.2</v>
       </c>
       <c r="R6" t="n">
-        <v>78110.8</v>
+        <v>34593.4</v>
       </c>
       <c r="S6" t="n">
-        <v>30871</v>
+        <v>10203.1</v>
       </c>
       <c r="T6" t="n">
-        <v>47239.8</v>
+        <v>24390.3</v>
       </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="n">
-        <v>0.7646201649272464</v>
+        <v>19.98114590866194</v>
       </c>
       <c r="W6" t="n">
-        <v>0.07194569304520658</v>
+        <v>0.1344317480424617</v>
       </c>
       <c r="X6" t="n">
-        <v>1.307838905994782</v>
+        <v>0.0500471797048684</v>
       </c>
       <c r="Y6" t="n">
-        <v>105.3274002157497</v>
+        <v>91.22732067510547</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.6830672066132366</v>
+        <v>1.473590883165618</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>gpt-6-astra</t>
+          <t>gemini-4-argon</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (Max)</t>
+          <t>Gemini 4 Argon (High)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (max)</t>
+          <t>Gemini 4 Argon (high)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1009,89 +1041,85 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>52.673669395513</v>
+        <v>50.4121935905389</v>
       </c>
       <c r="K7" t="n">
-        <v>7.932781535468826</v>
+        <v>4.187059268317184</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
-        <v>11.948927</v>
+        <v>8.057097000000001</v>
       </c>
       <c r="N7" t="n">
-        <v>10.588652</v>
+        <v>7.442264</v>
       </c>
       <c r="O7" t="n">
-        <v>0.525713</v>
+        <v>0.260092</v>
       </c>
       <c r="P7" t="n">
-        <v>0.834562</v>
+        <v>0.35474</v>
       </c>
       <c r="Q7" t="n">
-        <v>398.4</v>
+        <v>722.4</v>
       </c>
       <c r="R7" t="n">
-        <v>27205.5</v>
+        <v>61483.3</v>
       </c>
       <c r="S7" t="n">
-        <v>10514.3</v>
+        <v>26009.2</v>
       </c>
       <c r="T7" t="n">
-        <v>16691.2</v>
+        <v>35474</v>
       </c>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="n">
-        <v>4.408234261998002</v>
+        <v>6.256868148731347</v>
       </c>
       <c r="W7" t="n">
-        <v>0.1322130255911471</v>
+        <v>0.06978432113861974</v>
       </c>
       <c r="X7" t="n">
-        <v>0.2268481982957858</v>
+        <v>0.1598243683947154</v>
       </c>
       <c r="Y7" t="n">
-        <v>68.28689759036145</v>
+        <v>85.10977297895903</v>
       </c>
       <c r="Z7" t="n">
-        <v>1.936140464079432</v>
+        <v>0.8199331133907728</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>gemini-4-argon</t>
+          <t>muse-wonder-full</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Gemini 4 Argon (High)</t>
+          <t>Muse Wonder Full (Max)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Gemini 4 Argon (high)</t>
+          <t>Muse Wonder Full (max)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>large</t>
-        </is>
-      </c>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="b">
         <v>1</v>
       </c>
@@ -1099,82 +1127,54 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>52.5605655745982</v>
-      </c>
-      <c r="K8" t="n">
-        <v>4.365495479617791</v>
-      </c>
+        <v>49.7272123627021</v>
+      </c>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
-      <c r="M8" t="n">
-        <v>8.057855999999999</v>
-      </c>
-      <c r="N8" t="n">
-        <v>7.44228</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0.260112</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0.355464</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>722.4</v>
-      </c>
-      <c r="R8" t="n">
-        <v>61557.6</v>
-      </c>
-      <c r="S8" t="n">
-        <v>26011.2</v>
-      </c>
-      <c r="T8" t="n">
-        <v>35546.4</v>
-      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
-      <c r="V8" t="n">
-        <v>6.522897104961693</v>
-      </c>
-      <c r="W8" t="n">
-        <v>0.07275825799362985</v>
-      </c>
-      <c r="X8" t="n">
-        <v>0.1533061128987214</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>85.2126245847176</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>0.8538436452135594</v>
-      </c>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>muse-wonder</t>
+          <t>claude-fable-5-1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Muse Wonder (Max)</t>
+          <t>Claude Fable 5.1 (Max, Default Fallback)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Muse Wonder (max)</t>
+          <t>Claude Fable 5.1 (max with fallback)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1189,82 +1189,82 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>52.393894697293</v>
+        <v>49.0102124158081</v>
       </c>
       <c r="K9" t="n">
-        <v>12.27023295018572</v>
+        <v>3.784572387321089</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
-        <v>32.024787</v>
+        <v>69.76362399999999</v>
       </c>
       <c r="N9" t="n">
-        <v>30.935256</v>
+        <v>65.87397799999999</v>
       </c>
       <c r="O9" t="n">
-        <v>0.513532</v>
+        <v>1.543315</v>
       </c>
       <c r="P9" t="n">
-        <v>0.575999</v>
+        <v>2.346331</v>
       </c>
       <c r="Q9" t="n">
-        <v>256.2</v>
+        <v>777</v>
       </c>
       <c r="R9" t="n">
-        <v>54476.5</v>
+        <v>77792.89999999999</v>
       </c>
       <c r="S9" t="n">
-        <v>25676.6</v>
+        <v>30866.3</v>
       </c>
       <c r="T9" t="n">
-        <v>28799.9</v>
+        <v>46926.6</v>
       </c>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="n">
-        <v>1.636041941427838</v>
+        <v>0.7025181549600706</v>
       </c>
       <c r="W9" t="n">
-        <v>0.2045038825030953</v>
+        <v>0.06307620645535147</v>
       </c>
       <c r="X9" t="n">
-        <v>0.6112312738921966</v>
+        <v>1.423450757734279</v>
       </c>
       <c r="Y9" t="n">
-        <v>212.6327088212334</v>
+        <v>100.1195624195624</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.9617705744181987</v>
+        <v>0.6300088107758948</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>gpt-6-1-sol</t>
+          <t>kimi-k3-1-pro</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GPT-6.1 Sol (Max)</t>
+          <t>Kimi K3.1 Pro</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GPT-6.1 Sol (max)</t>
+          <t>Kimi K3.1 Pro</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Kimi</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>kimi</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1279,82 +1279,82 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>51.8332597011541</v>
+        <v>46.0026236744189</v>
       </c>
       <c r="K10" t="n">
-        <v>6.215019148819437</v>
+        <v>2.413568923106973</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
-        <v>3.029649</v>
+        <v>11.62043</v>
       </c>
       <c r="N10" t="n">
-        <v>2.648365</v>
+        <v>11.071161</v>
       </c>
       <c r="O10" t="n">
-        <v>0.129384</v>
+        <v>0.203099</v>
       </c>
       <c r="P10" t="n">
-        <v>0.2519</v>
+        <v>0.346169</v>
       </c>
       <c r="Q10" t="n">
-        <v>500.4</v>
+        <v>1143.6</v>
       </c>
       <c r="R10" t="n">
-        <v>38128.4</v>
+        <v>54926.9</v>
       </c>
       <c r="S10" t="n">
-        <v>12938.4</v>
+        <v>20309.9</v>
       </c>
       <c r="T10" t="n">
-        <v>25190</v>
+        <v>34616.9</v>
       </c>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="n">
-        <v>17.10866826525254</v>
+        <v>3.958771205060303</v>
       </c>
       <c r="W10" t="n">
-        <v>0.1035836524803239</v>
+        <v>0.04022614871844955</v>
       </c>
       <c r="X10" t="n">
-        <v>0.05844990296708164</v>
+        <v>0.2526036358761398</v>
       </c>
       <c r="Y10" t="n">
-        <v>76.19584332533974</v>
+        <v>48.02981811822316</v>
       </c>
       <c r="Z10" t="n">
-        <v>1.359439674918279</v>
+        <v>0.8375244857149938</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>gpt-6-1-terra</t>
+          <t>muse-wonder</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>GPT-6.1 Terra (Max)</t>
+          <t>Muse Wonder (Max)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GPT-6.1 Terra (max)</t>
+          <t>Muse Wonder (max)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1369,87 +1369,87 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>48.1061836463044</v>
+        <v>43.3248225998431</v>
       </c>
       <c r="K11" t="n">
-        <v>7.504864843417224</v>
+        <v>9.824222811755805</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
-        <v>2.553753</v>
+        <v>32.020831</v>
       </c>
       <c r="N11" t="n">
-        <v>2.378273</v>
+        <v>30.935219</v>
       </c>
       <c r="O11" t="n">
-        <v>0.051021</v>
+        <v>0.5135110000000001</v>
       </c>
       <c r="P11" t="n">
-        <v>0.124459</v>
+        <v>0.572101</v>
       </c>
       <c r="Q11" t="n">
-        <v>384.6</v>
+        <v>264.6</v>
       </c>
       <c r="R11" t="n">
-        <v>35096</v>
+        <v>54280.6</v>
       </c>
       <c r="S11" t="n">
-        <v>10204.2</v>
+        <v>25675.6</v>
       </c>
       <c r="T11" t="n">
-        <v>24891.8</v>
+        <v>28605</v>
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>18.83744576954169</v>
+        <v>1.353019932550879</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1250810807236204</v>
+        <v>0.1637370468625967</v>
       </c>
       <c r="X11" t="n">
-        <v>0.05308575335711927</v>
+        <v>0.7390874117535559</v>
       </c>
       <c r="Y11" t="n">
-        <v>91.2532501300052</v>
+        <v>205.1421012849584</v>
       </c>
       <c r="Z11" t="n">
-        <v>1.370702748071131</v>
+        <v>0.798164032819149</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>grok-4-7</t>
+          <t>claude-haiku-5-5</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Grok 4.7 (Xhigh)</t>
+          <t>Claude Haiku 5.5 (Max)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Grok 4.7 (xhigh)</t>
+          <t>Claude Haiku 5.5 (max)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>SpaceXAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>xai</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H12" t="b">
@@ -1459,77 +1459,77 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>46.4465506302286</v>
+        <v>36.2345435880142</v>
       </c>
       <c r="K12" t="n">
-        <v>3.207634712032362</v>
+        <v>5.132371613033173</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
-        <v>8.336827</v>
+        <v>1.06449</v>
       </c>
       <c r="N12" t="n">
-        <v>7.853459</v>
+        <v>0.983895</v>
       </c>
       <c r="O12" t="n">
-        <v>0.132106</v>
+        <v>0.016557</v>
       </c>
       <c r="P12" t="n">
-        <v>0.351262</v>
+        <v>0.064039</v>
       </c>
       <c r="Q12" t="n">
-        <v>868.8000000000001</v>
+        <v>423.6</v>
       </c>
       <c r="R12" t="n">
-        <v>80561.39999999999</v>
+        <v>161190.3</v>
       </c>
       <c r="S12" t="n">
-        <v>22017.7</v>
+        <v>33113.2</v>
       </c>
       <c r="T12" t="n">
-        <v>58543.6</v>
+        <v>128077.1</v>
       </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="n">
-        <v>5.571250384616186</v>
+        <v>34.03934615450986</v>
       </c>
       <c r="W12" t="n">
-        <v>0.05346057853387269</v>
+        <v>0.08553952688388622</v>
       </c>
       <c r="X12" t="n">
-        <v>0.1794929200743312</v>
+        <v>0.02937776758286852</v>
       </c>
       <c r="Y12" t="n">
-        <v>92.72720994475137</v>
+        <v>380.5247875354108</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.5765360412086756</v>
+        <v>0.2247935737325025</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>mimo-v2-6-pro</t>
+          <t>grok-4-7</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Grok 4.7 (Xhigh)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MiMo-V2.6-Pro</t>
+          <t>Grok 4.7 (xhigh)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Xiaomi</t>
+          <t>SpaceXAI</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>xiaomi</t>
+          <t>xai</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1546,54 +1546,54 @@
         <v>1</v>
       </c>
       <c r="I13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>46.3242065310383</v>
+        <v>34.3350117067196</v>
       </c>
       <c r="K13" t="n">
-        <v>2.731380102065937</v>
+        <v>2.414557785282672</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
-        <v>2.466319</v>
+        <v>8.333793</v>
       </c>
       <c r="N13" t="n">
-        <v>2.410399</v>
+        <v>7.853533</v>
       </c>
       <c r="O13" t="n">
-        <v>0.023278</v>
+        <v>0.132105</v>
       </c>
       <c r="P13" t="n">
-        <v>0.032642</v>
+        <v>0.348155</v>
       </c>
       <c r="Q13" t="n">
-        <v>1017.6</v>
+        <v>853.2</v>
       </c>
       <c r="R13" t="n">
-        <v>64275.7</v>
+        <v>80043.3</v>
       </c>
       <c r="S13" t="n">
-        <v>26756</v>
+        <v>22017.4</v>
       </c>
       <c r="T13" t="n">
-        <v>37519.7</v>
+        <v>58025.9</v>
       </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="n">
-        <v>18.78273107859863</v>
+        <v>4.119974147032401</v>
       </c>
       <c r="W13" t="n">
-        <v>0.04552300170109896</v>
+        <v>0.0402426297547112</v>
       </c>
       <c r="X13" t="n">
-        <v>0.05324039383918014</v>
+        <v>0.2427199696678426</v>
       </c>
       <c r="Y13" t="n">
-        <v>63.16401336477987</v>
+        <v>93.81540084388186</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.7207110390246749</v>
+        <v>0.4289554741835931</v>
       </c>
     </row>
     <row r="14">
@@ -1639,51 +1639,51 @@
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>45.4152084980521</v>
+        <v>33.5545627367888</v>
       </c>
       <c r="K14" t="n">
-        <v>1.308795633949628</v>
+        <v>1.018038917985097</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
-        <v>26.154609</v>
+        <v>26.153879</v>
       </c>
       <c r="N14" t="n">
-        <v>25.508227</v>
+        <v>25.508207</v>
       </c>
       <c r="O14" t="n">
-        <v>0.221402</v>
+        <v>0.221396</v>
       </c>
       <c r="P14" t="n">
-        <v>0.424979</v>
+        <v>0.424275</v>
       </c>
       <c r="Q14" t="n">
-        <v>2082</v>
+        <v>1977.6</v>
       </c>
       <c r="R14" t="n">
-        <v>107730.2</v>
+        <v>107612</v>
       </c>
       <c r="S14" t="n">
-        <v>36900.3</v>
+        <v>36899.4</v>
       </c>
       <c r="T14" t="n">
-        <v>70829.89999999999</v>
+        <v>70712.60000000001</v>
       </c>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="n">
-        <v>1.736413207249709</v>
+        <v>1.282966963974591</v>
       </c>
       <c r="W14" t="n">
-        <v>0.02181326056582714</v>
+        <v>0.01696731529975162</v>
       </c>
       <c r="X14" t="n">
-        <v>0.5758997891889408</v>
+        <v>0.7794432967330912</v>
       </c>
       <c r="Y14" t="n">
-        <v>51.74361191162344</v>
+        <v>54.41545307443365</v>
       </c>
       <c r="Z14" t="n">
-        <v>0.421564319921917</v>
+        <v>0.3118106041778687</v>
       </c>
     </row>
     <row r="15">
@@ -1729,51 +1729,51 @@
         <v>1</v>
       </c>
       <c r="J15" t="n">
-        <v>45.0965048681912</v>
+        <v>32.4896393532027</v>
       </c>
       <c r="K15" t="n">
-        <v>7.046328885654874</v>
+        <v>5.791379563850747</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>3.00199</v>
+        <v>3.001861</v>
       </c>
       <c r="N15" t="n">
-        <v>2.894596</v>
+        <v>2.894593</v>
       </c>
       <c r="O15" t="n">
-        <v>0.036302</v>
+        <v>0.036299</v>
       </c>
       <c r="P15" t="n">
-        <v>0.071092</v>
+        <v>0.070968</v>
       </c>
       <c r="Q15" t="n">
-        <v>384</v>
+        <v>336.6</v>
       </c>
       <c r="R15" t="n">
-        <v>89495.10000000001</v>
+        <v>89389.5</v>
       </c>
       <c r="S15" t="n">
-        <v>30252</v>
+        <v>30249.3</v>
       </c>
       <c r="T15" t="n">
-        <v>59243</v>
+        <v>59140.2</v>
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="n">
-        <v>15.02220356103491</v>
+        <v>10.82316581387436</v>
       </c>
       <c r="W15" t="n">
-        <v>0.1174388147609146</v>
+        <v>0.0965229927308458</v>
       </c>
       <c r="X15" t="n">
-        <v>0.06656813003079209</v>
+        <v>0.09239440817935976</v>
       </c>
       <c r="Y15" t="n">
-        <v>233.06015625</v>
+        <v>265.5659536541889</v>
       </c>
       <c r="Z15" t="n">
-        <v>0.5038991505478086</v>
+        <v>0.3634614731394929</v>
       </c>
     </row>
     <row r="16">
@@ -1819,82 +1819,82 @@
         <v>1</v>
       </c>
       <c r="J16" t="n">
-        <v>44.777392385614</v>
+        <v>31.653381843882</v>
       </c>
       <c r="K16" t="n">
-        <v>4.119355325263478</v>
+        <v>2.997479341276704</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
-        <v>8.678356000000001</v>
+        <v>8.678190000000001</v>
       </c>
       <c r="N16" t="n">
-        <v>8.365394999999999</v>
+        <v>8.365380999999999</v>
       </c>
       <c r="O16" t="n">
-        <v>0.098552</v>
+        <v>0.098528</v>
       </c>
       <c r="P16" t="n">
-        <v>0.21441</v>
+        <v>0.214281</v>
       </c>
       <c r="Q16" t="n">
-        <v>652.1999999999999</v>
+        <v>633.6</v>
       </c>
       <c r="R16" t="n">
-        <v>71127.60000000001</v>
+        <v>71092.89999999999</v>
       </c>
       <c r="S16" t="n">
-        <v>22398.1</v>
+        <v>22392.6</v>
       </c>
       <c r="T16" t="n">
-        <v>48729.5</v>
+        <v>48700.3</v>
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="n">
-        <v>5.159663003639629</v>
+        <v>3.647463566006505</v>
       </c>
       <c r="W16" t="n">
-        <v>0.06865592208772463</v>
+        <v>0.0499579890212784</v>
       </c>
       <c r="X16" t="n">
-        <v>0.1938111072941391</v>
+        <v>0.2741631223735208</v>
       </c>
       <c r="Y16" t="n">
-        <v>109.0579576816928</v>
+        <v>112.2047032828283</v>
       </c>
       <c r="Z16" t="n">
-        <v>0.629536106737947</v>
+        <v>0.445239705285366</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>step-5</t>
+          <t>gemini-3-8-flash</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>Gemini 3.8 Flash (High)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Step 5 Preview</t>
+          <t>Gemini 3.8 Flash (high)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>StepFun</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>stepfun</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1906,270 +1906,262 @@
         <v>1</v>
       </c>
       <c r="I17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>43.7343049141614</v>
+        <v>30.5468119957291</v>
       </c>
       <c r="K17" t="n">
-        <v>8.558572390246848</v>
+        <v>3.53960741549584</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
-        <v>6.586908</v>
+        <v>4.900073</v>
       </c>
       <c r="N17" t="n">
-        <v>6.413718</v>
+        <v>4.634753</v>
       </c>
       <c r="O17" t="n">
-        <v>0.055881</v>
+        <v>0.106031</v>
       </c>
       <c r="P17" t="n">
-        <v>0.117309</v>
+        <v>0.159289</v>
       </c>
       <c r="Q17" t="n">
-        <v>306.6</v>
+        <v>517.8000000000001</v>
       </c>
       <c r="R17" t="n">
-        <v>64144.3</v>
+        <v>70751.8</v>
       </c>
       <c r="S17" t="n">
-        <v>20696.6</v>
+        <v>28274.8</v>
       </c>
       <c r="T17" t="n">
-        <v>43447.7</v>
+        <v>42477</v>
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="n">
-        <v>6.639580348497565</v>
+        <v>6.233950391296028</v>
       </c>
       <c r="W17" t="n">
-        <v>0.1426428731707808</v>
+        <v>0.05899345692493066</v>
       </c>
       <c r="X17" t="n">
-        <v>0.1506119283918727</v>
+        <v>0.1604119277875905</v>
       </c>
       <c r="Y17" t="n">
-        <v>209.2116764514025</v>
+        <v>136.6392429509463</v>
       </c>
       <c r="Z17" t="n">
-        <v>0.6818112429968274</v>
+        <v>0.4317460756578504</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>claude-haiku-5-5</t>
+          <t>mimo-v2-6-pro</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Claude Haiku 5.5 (Max)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Claude Haiku 5.5 (max)</t>
+          <t>MiMo-V2.6-Pro</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Xiaomi</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>xiaomi</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H18" t="b">
         <v>1</v>
       </c>
       <c r="I18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" t="n">
-        <v>43.3950199670746</v>
+        <v>29.8897833093321</v>
       </c>
       <c r="K18" t="n">
-        <v>6.111974643249944</v>
+        <v>1.853055381855679</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
-        <v>1.064978</v>
+        <v>2.466142</v>
       </c>
       <c r="N18" t="n">
-        <v>0.983896</v>
+        <v>2.410395</v>
       </c>
       <c r="O18" t="n">
-        <v>0.016559</v>
+        <v>0.023228</v>
       </c>
       <c r="P18" t="n">
-        <v>0.064523</v>
+        <v>0.032518</v>
       </c>
       <c r="Q18" t="n">
-        <v>426</v>
+        <v>967.8</v>
       </c>
       <c r="R18" t="n">
-        <v>162164.2</v>
+        <v>64076.5</v>
       </c>
       <c r="S18" t="n">
-        <v>33117.6</v>
+        <v>26699.2</v>
       </c>
       <c r="T18" t="n">
-        <v>129046.6</v>
+        <v>37377.3</v>
       </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="n">
-        <v>40.74733935074209</v>
+        <v>12.12005768902687</v>
       </c>
       <c r="W18" t="n">
-        <v>0.1018662440541657</v>
+        <v>0.03088425636426131</v>
       </c>
       <c r="X18" t="n">
-        <v>0.02454147966305898</v>
+        <v>0.08250785810247172</v>
       </c>
       <c r="Y18" t="n">
-        <v>380.6671361502348</v>
+        <v>66.20841082868361</v>
       </c>
       <c r="Z18" t="n">
-        <v>0.2675992602995889</v>
+        <v>0.4664702864440489</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>minimax-m3-1-flash</t>
+          <t>ling-3-1-flash-1019</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MiniMax-M3.1-Flash</t>
+          <t>Ling 3.1 Flash 1019</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MiniMax-M3.1-Flash</t>
+          <t>Ling 3.1 Flash 1019</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>InclusionAI</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>minimax</t>
+          <t>inclusionai</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H19" t="b">
         <v>1</v>
       </c>
       <c r="I19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>42.7057475126235</v>
-      </c>
-      <c r="K19" t="n">
-        <v>4.398120238169258</v>
-      </c>
+        <v>29.470119369837</v>
+      </c>
+      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
-        <v>1.306119</v>
+        <v>4.832016</v>
       </c>
       <c r="N19" t="n">
-        <v>1.258952</v>
+        <v>4.70269</v>
       </c>
       <c r="O19" t="n">
-        <v>0.014367</v>
+        <v>0.046295</v>
       </c>
       <c r="P19" t="n">
-        <v>0.032801</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>582.6</v>
-      </c>
+        <v>0.08303000000000001</v>
+      </c>
+      <c r="Q19" t="inlineStr"/>
       <c r="R19" t="n">
-        <v>78612.3</v>
+        <v>143695.3</v>
       </c>
       <c r="S19" t="n">
-        <v>23944.7</v>
+        <v>51439.2</v>
       </c>
       <c r="T19" t="n">
-        <v>54667.6</v>
+        <v>92256.10000000001</v>
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="n">
-        <v>32.69667427900789</v>
-      </c>
-      <c r="W19" t="n">
-        <v>0.07330200396948765</v>
-      </c>
+        <v>6.098928349955174</v>
+      </c>
+      <c r="W19" t="inlineStr"/>
       <c r="X19" t="n">
-        <v>0.03058415028595205</v>
-      </c>
-      <c r="Y19" t="n">
-        <v>134.9335736354274</v>
-      </c>
+        <v>0.1639632313449542</v>
+      </c>
+      <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="n">
-        <v>0.5432451093864892</v>
+        <v>0.2050875663284534</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>gemini-3-8-flash</t>
+          <t>minimax-m3-1-flash</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (High)</t>
+          <t>MiniMax-M3.1-Flash</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>MiniMax-M3.1-Flash</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>minimax</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H20" t="b">
@@ -2179,82 +2171,82 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>40.9262321765904</v>
+        <v>28.9095214290458</v>
       </c>
       <c r="K20" t="n">
-        <v>4.725892861038153</v>
+        <v>3.014548637022503</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
-        <v>4.90102</v>
+        <v>1.305936</v>
       </c>
       <c r="N20" t="n">
-        <v>4.63476</v>
+        <v>1.258948</v>
       </c>
       <c r="O20" t="n">
-        <v>0.106033</v>
+        <v>0.014367</v>
       </c>
       <c r="P20" t="n">
-        <v>0.160227</v>
+        <v>0.032621</v>
       </c>
       <c r="Q20" t="n">
-        <v>519.6</v>
+        <v>575.4</v>
       </c>
       <c r="R20" t="n">
-        <v>71002.60000000001</v>
+        <v>78313</v>
       </c>
       <c r="S20" t="n">
-        <v>28275.4</v>
+        <v>23944.2</v>
       </c>
       <c r="T20" t="n">
-        <v>42727.1</v>
+        <v>54368.8</v>
       </c>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="n">
-        <v>8.350554002348574</v>
+        <v>22.13701240263367</v>
       </c>
       <c r="W20" t="n">
-        <v>0.07876488101730254</v>
+        <v>0.05024247728370838</v>
       </c>
       <c r="X20" t="n">
-        <v>0.119752533750306</v>
+        <v>0.04517321406392801</v>
       </c>
       <c r="Y20" t="n">
-        <v>136.6485758275597</v>
+        <v>136.1018421967327</v>
       </c>
       <c r="Z20" t="n">
-        <v>0.5764046975264343</v>
+        <v>0.3691535432054167</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>muse-spark-open</t>
+          <t>step-5</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Muse Spark Open (Xhigh)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Muse Spark Open (xhigh)</t>
+          <t>Step 5 Preview</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>StepFun</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>stepfun</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2269,87 +2261,87 @@
         <v>1</v>
       </c>
       <c r="J21" t="n">
-        <v>38.8666662997805</v>
+        <v>28.5283090216016</v>
       </c>
       <c r="K21" t="n">
-        <v>11.77777766660015</v>
+        <v>5.372562904256422</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
-        <v>3.768433</v>
+        <v>6.585749</v>
       </c>
       <c r="N21" t="n">
-        <v>3.596656</v>
+        <v>6.413708</v>
       </c>
       <c r="O21" t="n">
-        <v>0.093573</v>
+        <v>0.055862</v>
       </c>
       <c r="P21" t="n">
-        <v>0.078204</v>
+        <v>0.116179</v>
       </c>
       <c r="Q21" t="n">
-        <v>198</v>
+        <v>318.6</v>
       </c>
       <c r="R21" t="n">
-        <v>40418.1</v>
+        <v>63718.6</v>
       </c>
       <c r="S21" t="n">
-        <v>22017.2</v>
+        <v>20689.5</v>
       </c>
       <c r="T21" t="n">
-        <v>18400.9</v>
+        <v>43029.2</v>
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="n">
-        <v>10.3137474647368</v>
+        <v>4.33182452316382</v>
       </c>
       <c r="W21" t="n">
-        <v>0.1962962944433359</v>
+        <v>0.08954271507094037</v>
       </c>
       <c r="X21" t="n">
-        <v>0.09695796832519393</v>
+        <v>0.2308496095935192</v>
       </c>
       <c r="Y21" t="n">
-        <v>204.1318181818182</v>
+        <v>199.9956057752668</v>
       </c>
       <c r="Z21" t="n">
-        <v>0.9616153728102138</v>
+        <v>0.4477234123411626</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>mistral-large-4</t>
+          <t>gpt-6-luna</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Mistral Large 4 Preview</t>
+          <t>GPT-6 Luna (Max)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mistral Large 4 Preview</t>
+          <t>GPT-6 Luna (max)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Mistral</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>mistral</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H22" t="b">
@@ -2359,87 +2351,87 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>38.3770408917494</v>
+        <v>27.7552004938153</v>
       </c>
       <c r="K22" t="n">
-        <v>4.346210746517486</v>
+        <v>4.23097568503282</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
-        <v>6.146153</v>
+        <v>0.326073</v>
       </c>
       <c r="N22" t="n">
-        <v>5.855662</v>
+        <v>0.301269</v>
       </c>
       <c r="O22" t="n">
-        <v>0.07263600000000001</v>
+        <v>0.00556</v>
       </c>
       <c r="P22" t="n">
-        <v>0.217855</v>
+        <v>0.019244</v>
       </c>
       <c r="Q22" t="n">
-        <v>529.8</v>
+        <v>393.6</v>
       </c>
       <c r="R22" t="n">
-        <v>69495.5</v>
+        <v>49608.1</v>
       </c>
       <c r="S22" t="n">
-        <v>17377.1</v>
+        <v>11120.9</v>
       </c>
       <c r="T22" t="n">
-        <v>52118.5</v>
+        <v>38487.2</v>
       </c>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="n">
-        <v>6.24407509734128</v>
+        <v>85.1195912995412</v>
       </c>
       <c r="W22" t="n">
-        <v>0.07243684577529144</v>
+        <v>0.07051626141721368</v>
       </c>
       <c r="X22" t="n">
-        <v>0.1601518214324166</v>
+        <v>0.01174817670917776</v>
       </c>
       <c r="Y22" t="n">
-        <v>131.1730841827105</v>
+        <v>126.0368394308943</v>
       </c>
       <c r="Z22" t="n">
-        <v>0.5522233942017742</v>
+        <v>0.5594892869070837</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>gpt-6-luna</t>
+          <t>mistral-large-4</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (Max)</t>
+          <t>Mistral Large 4 Preview</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GPT-6 Luna (max)</t>
+          <t>Mistral Large 4 Preview</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Mistral</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>mistral</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H23" t="b">
@@ -2449,87 +2441,87 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>38.1245186869738</v>
+        <v>25.286451488165</v>
       </c>
       <c r="K23" t="n">
-        <v>5.767703280934009</v>
+        <v>2.787921884031422</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
-        <v>0.326276</v>
+        <v>6.144715</v>
       </c>
       <c r="N23" t="n">
-        <v>0.30127</v>
+        <v>5.855647</v>
       </c>
       <c r="O23" t="n">
-        <v>0.005561</v>
+        <v>0.072592</v>
       </c>
       <c r="P23" t="n">
-        <v>0.019445</v>
+        <v>0.216476</v>
       </c>
       <c r="Q23" t="n">
-        <v>396.6</v>
+        <v>544.2</v>
       </c>
       <c r="R23" t="n">
-        <v>50011.7</v>
+        <v>69155</v>
       </c>
       <c r="S23" t="n">
-        <v>11122</v>
+        <v>17366.6</v>
       </c>
       <c r="T23" t="n">
-        <v>38889.7</v>
+        <v>51788.4</v>
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="n">
-        <v>116.8474502782117</v>
+        <v>4.11515448449033</v>
       </c>
       <c r="W23" t="n">
-        <v>0.09612838801556682</v>
+        <v>0.04646536473385703</v>
       </c>
       <c r="X23" t="n">
-        <v>0.008558167059863248</v>
+        <v>0.243004242919413</v>
       </c>
       <c r="Y23" t="n">
-        <v>126.1011094301563</v>
+        <v>127.0764424843807</v>
       </c>
       <c r="Z23" t="n">
-        <v>0.7623119927331765</v>
+        <v>0.365648926153785</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>qwen3-8-27b</t>
+          <t>muse-spark-open</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (Xhigh)</t>
+          <t>Muse Spark Open (Xhigh)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (xhigh)</t>
+          <t>Muse Spark Open (xhigh)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H24" t="b">
@@ -2539,87 +2531,87 @@
         <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>33.6762858057476</v>
+        <v>24.6815868992913</v>
       </c>
       <c r="K24" t="n">
-        <v>1.682132158129251</v>
+        <v>7.031791139399231</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
-        <v>2.505854</v>
+        <v>3.767941</v>
       </c>
       <c r="N24" t="n">
-        <v>2.305504</v>
+        <v>3.596657</v>
       </c>
       <c r="O24" t="n">
-        <v>0.057275</v>
+        <v>0.093567</v>
       </c>
       <c r="P24" t="n">
-        <v>0.143075</v>
+        <v>0.07771699999999999</v>
       </c>
       <c r="Q24" t="n">
-        <v>1201.2</v>
+        <v>210.6</v>
       </c>
       <c r="R24" t="n">
-        <v>66783.2</v>
+        <v>40302</v>
       </c>
       <c r="S24" t="n">
-        <v>19091.6</v>
+        <v>22015.7</v>
       </c>
       <c r="T24" t="n">
-        <v>47691.6</v>
+        <v>18286.4</v>
       </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="n">
-        <v>13.43904545346521</v>
+        <v>6.55041756208266</v>
       </c>
       <c r="W24" t="n">
-        <v>0.02803553596882084</v>
+        <v>0.1171965189899872</v>
       </c>
       <c r="X24" t="n">
-        <v>0.07441004671519687</v>
+        <v>0.1526620235309178</v>
       </c>
       <c r="Y24" t="n">
-        <v>55.59706959706959</v>
+        <v>191.3675213675214</v>
       </c>
       <c r="Z24" t="n">
-        <v>0.5042628356494987</v>
+        <v>0.6124159321942162</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>k2-horizon-375b-a23b</t>
+          <t>qwen3-8-27b</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Qwen3.8 27B (Xhigh)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>Qwen3.8 27B (xhigh)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Institute of Foundation Models</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ifm</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H25" t="b">
@@ -2629,54 +2621,82 @@
         <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>30.5015302696723</v>
-      </c>
-      <c r="K25" t="inlineStr"/>
+        <v>20.1068756031705</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0.9732272799211278</v>
+      </c>
       <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
+      <c r="M25" t="n">
+        <v>2.504963</v>
+      </c>
+      <c r="N25" t="n">
+        <v>2.305498</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0.057272</v>
+      </c>
+      <c r="P25" t="n">
+        <v>0.142193</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>1239.6</v>
+      </c>
+      <c r="R25" t="n">
+        <v>66488.39999999999</v>
+      </c>
+      <c r="S25" t="n">
+        <v>19090.7</v>
+      </c>
+      <c r="T25" t="n">
+        <v>47397.7</v>
+      </c>
       <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
-      <c r="Z25" t="inlineStr"/>
+      <c r="V25" t="n">
+        <v>8.026815407321585</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0.01622045466535213</v>
+      </c>
+      <c r="X25" t="n">
+        <v>0.1245824089947128</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>53.63697967086157</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>0.3024117831557159</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>reflection-beam</t>
+          <t>k2-horizon-375b-a23b</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Beam 1.0</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Beam 1.0</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Reflection</t>
+          <t>Institute of Foundation Models</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>reflection</t>
+          <t>ifm</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2691,87 +2711,59 @@
         <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>30.3334426348039</v>
-      </c>
-      <c r="K26" t="n">
-        <v>37.44869461086901</v>
-      </c>
+        <v>17.7702731734027</v>
+      </c>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
-      <c r="M26" t="n">
-        <v>0.757782</v>
-      </c>
-      <c r="N26" t="n">
-        <v>0.726204</v>
-      </c>
-      <c r="O26" t="n">
-        <v>0.008203999999999999</v>
-      </c>
-      <c r="P26" t="n">
-        <v>0.023374</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>48.6</v>
-      </c>
-      <c r="R26" t="n">
-        <v>26315</v>
-      </c>
-      <c r="S26" t="n">
-        <v>6837.1</v>
-      </c>
-      <c r="T26" t="n">
-        <v>19478</v>
-      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
-      <c r="V26" t="n">
-        <v>40.02924671581524</v>
-      </c>
-      <c r="W26" t="n">
-        <v>0.6241449101811503</v>
-      </c>
-      <c r="X26" t="n">
-        <v>0.02498173415801272</v>
-      </c>
-      <c r="Y26" t="n">
-        <v>541.4609053497942</v>
-      </c>
-      <c r="Z26" t="n">
-        <v>1.152705401284587</v>
-      </c>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>nemotron-3-5-super-vl</t>
+          <t>reflection-beam</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Nemotron 3.5 Super VL</t>
+          <t>Beam 1.0</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Nemotron 3.5 Super VL</t>
+          <t>Beam 1.0</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Reflection</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>reflection</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H27" t="b">
@@ -2781,87 +2773,87 @@
         <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>26.4910658661689</v>
+        <v>17.7307282547205</v>
       </c>
       <c r="K27" t="n">
-        <v>16.66104771457163</v>
+        <v>23.02691981132532</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
-        <v>0.416252</v>
+        <v>0.757616</v>
       </c>
       <c r="N27" t="n">
-        <v>0.387977</v>
+        <v>0.726199</v>
       </c>
       <c r="O27" t="n">
-        <v>0.007806</v>
+        <v>0.008203</v>
       </c>
       <c r="P27" t="n">
-        <v>0.020469</v>
+        <v>0.023214</v>
       </c>
       <c r="Q27" t="n">
-        <v>95.40000000000001</v>
+        <v>46.2</v>
       </c>
       <c r="R27" t="n">
-        <v>49173.8</v>
+        <v>26180.8</v>
       </c>
       <c r="S27" t="n">
-        <v>13575.6</v>
+        <v>6835.5</v>
       </c>
       <c r="T27" t="n">
-        <v>35598.3</v>
+        <v>19345.2</v>
       </c>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="n">
-        <v>63.641894492204</v>
+        <v>23.40331811197295</v>
       </c>
       <c r="W27" t="n">
-        <v>0.2776841285761939</v>
+        <v>0.383781996855422</v>
       </c>
       <c r="X27" t="n">
-        <v>0.01571292005021155</v>
+        <v>0.04272898377980035</v>
       </c>
       <c r="Y27" t="n">
-        <v>515.4486373165619</v>
+        <v>566.6839826839827</v>
       </c>
       <c r="Z27" t="n">
-        <v>0.5387231791354116</v>
+        <v>0.677241652459837</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>inkling</t>
+          <t>nemotron-3-5-super-vl</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Inkling (Xhigh)</t>
+          <t>Nemotron 3.5 Super VL</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Inkling (xhigh)</t>
+          <t>Nemotron 3.5 Super VL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Thinking Machines</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>thinking-machines</t>
+          <t>nvidia</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H28" t="b">
@@ -2871,51 +2863,141 @@
         <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>24.9847810999384</v>
+        <v>13.6203422723141</v>
       </c>
       <c r="K28" t="n">
-        <v>10.32428971071835</v>
+        <v>8.620469792603858</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
-        <v>2.418996</v>
+        <v>0.415919</v>
       </c>
       <c r="N28" t="n">
-        <v>2.278639</v>
+        <v>0.387975</v>
       </c>
       <c r="O28" t="n">
-        <v>0.04559</v>
+        <v>0.007805</v>
       </c>
       <c r="P28" t="n">
-        <v>0.094767</v>
+        <v>0.020139</v>
       </c>
       <c r="Q28" t="n">
-        <v>145.2</v>
+        <v>94.80000000000001</v>
       </c>
       <c r="R28" t="n">
-        <v>34656</v>
+        <v>48599.1</v>
       </c>
       <c r="S28" t="n">
-        <v>11256.8</v>
+        <v>13574</v>
       </c>
       <c r="T28" t="n">
-        <v>23399.2</v>
+        <v>35025.1</v>
       </c>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="n">
-        <v>10.32857478885389</v>
+        <v>32.74758371777702</v>
       </c>
       <c r="W28" t="n">
-        <v>0.1720714951786391</v>
+        <v>0.1436744965433976</v>
       </c>
       <c r="X28" t="n">
-        <v>0.09681877901287532</v>
+        <v>0.03053660412377693</v>
       </c>
       <c r="Y28" t="n">
-        <v>238.6776859504132</v>
+        <v>512.6487341772151</v>
       </c>
       <c r="Z28" t="n">
-        <v>0.7209366660877885</v>
+        <v>0.2802591462046437</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>inkling</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Inkling (Xhigh)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Inkling (xhigh)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Thinking Machines</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>thinking-machines</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+      <c r="H29" t="b">
+        <v>1</v>
+      </c>
+      <c r="I29" t="b">
+        <v>1</v>
+      </c>
+      <c r="J29" t="n">
+        <v>12.4781698715401</v>
+      </c>
+      <c r="K29" t="n">
+        <v>5.425291248495696</v>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="n">
+        <v>2.417186</v>
+      </c>
+      <c r="N29" t="n">
+        <v>2.278629</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0.045585</v>
+      </c>
+      <c r="P29" t="n">
+        <v>0.092972</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>138</v>
+      </c>
+      <c r="R29" t="n">
+        <v>34211.6</v>
+      </c>
+      <c r="S29" t="n">
+        <v>11255.6</v>
+      </c>
+      <c r="T29" t="n">
+        <v>22956</v>
+      </c>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="n">
+        <v>5.162271282201742</v>
+      </c>
+      <c r="W29" t="n">
+        <v>0.09042152080826159</v>
+      </c>
+      <c r="X29" t="n">
+        <v>0.1937131826930052</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>247.9101449275362</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>0.364735056867849</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-29)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -551,32 +551,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>claude-opus-5-5</t>
+          <t>gemini-4-carbon</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (Max, Default Fallback)</t>
+          <t>Gemini 4 Carbon (High)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5 (max with fallback)</t>
+          <t>Gemini 4 Carbon (high)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -591,82 +591,82 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>58.4060336078904</v>
+        <v>59.425738829526</v>
       </c>
       <c r="K2" t="n">
-        <v>4.520590836524025</v>
+        <v>4.588860141276139</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
-        <v>51.818032</v>
+        <v>14.870251</v>
       </c>
       <c r="N2" t="n">
-        <v>49.444751</v>
+        <v>13.342112</v>
       </c>
       <c r="O2" t="n">
-        <v>0.704638</v>
+        <v>0.507506</v>
       </c>
       <c r="P2" t="n">
-        <v>1.668643</v>
+        <v>1.020633</v>
       </c>
       <c r="Q2" t="n">
-        <v>775.2</v>
+        <v>777</v>
       </c>
       <c r="R2" t="n">
-        <v>118664.1</v>
+        <v>76406.89999999999</v>
       </c>
       <c r="S2" t="n">
-        <v>35231.9</v>
+        <v>25375.3</v>
       </c>
       <c r="T2" t="n">
-        <v>83432.10000000001</v>
+        <v>51031.6</v>
       </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="n">
-        <v>1.127137240717486</v>
+        <v>3.996283507892772</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07534318060873374</v>
+        <v>0.07648100235460231</v>
       </c>
       <c r="X2" t="n">
-        <v>0.8872034068925305</v>
+        <v>0.2502324967748089</v>
       </c>
       <c r="Y2" t="n">
-        <v>153.0754643962848</v>
+        <v>98.33577863577862</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.492196322290317</v>
+        <v>0.7777535645278896</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>gpt-6-astra</t>
+          <t>claude-opus-5-5</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (Max)</t>
+          <t>Claude Opus 5.5 (Max, Default Fallback)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (max)</t>
+          <t>Claude Opus 5.5 (max with fallback)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -681,67 +681,67 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>56.8538559596797</v>
+        <v>58.4060336078904</v>
       </c>
       <c r="K3" t="n">
-        <v>9.214563364615834</v>
+        <v>4.455075027299039</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
-        <v>11.94179</v>
+        <v>51.818032</v>
       </c>
       <c r="N3" t="n">
-        <v>10.588558</v>
+        <v>49.444751</v>
       </c>
       <c r="O3" t="n">
-        <v>0.52565</v>
+        <v>0.704638</v>
       </c>
       <c r="P3" t="n">
-        <v>0.827582</v>
+        <v>1.668643</v>
       </c>
       <c r="Q3" t="n">
-        <v>370.2</v>
+        <v>786.5999999999999</v>
       </c>
       <c r="R3" t="n">
-        <v>27064.6</v>
+        <v>118664.1</v>
       </c>
       <c r="S3" t="n">
-        <v>10513</v>
+        <v>35231.9</v>
       </c>
       <c r="T3" t="n">
-        <v>16551.6</v>
+        <v>83432.10000000001</v>
       </c>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="n">
-        <v>4.76091573873596</v>
+        <v>1.127137240717486</v>
       </c>
       <c r="W3" t="n">
-        <v>0.1535760560769306</v>
+        <v>0.07425125045498399</v>
       </c>
       <c r="X3" t="n">
-        <v>0.210043624982429</v>
+        <v>0.8872034068925305</v>
       </c>
       <c r="Y3" t="n">
-        <v>73.10804970286331</v>
+        <v>150.8569794050343</v>
       </c>
       <c r="Z3" t="n">
-        <v>2.100672315854648</v>
+        <v>0.492196322290317</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>gpt-6-1-sol</t>
+          <t>gpt-6-astra</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>GPT-6.1 Sol (Max)</t>
+          <t>GPT-6 Astra (Max)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GPT-6.1 Sol (max)</t>
+          <t>GPT-6 Astra (max)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -771,82 +771,82 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>54.5087338138148</v>
+        <v>56.8538559596797</v>
       </c>
       <c r="K4" t="n">
-        <v>6.796600226161447</v>
+        <v>9.444162119548123</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
-        <v>3.028512</v>
+        <v>11.94179</v>
       </c>
       <c r="N4" t="n">
-        <v>2.648346</v>
+        <v>10.588558</v>
       </c>
       <c r="O4" t="n">
-        <v>0.129372</v>
+        <v>0.52565</v>
       </c>
       <c r="P4" t="n">
-        <v>0.250794</v>
+        <v>0.827582</v>
       </c>
       <c r="Q4" t="n">
-        <v>481.2</v>
+        <v>361.2</v>
       </c>
       <c r="R4" t="n">
-        <v>38016.6</v>
+        <v>27064.6</v>
       </c>
       <c r="S4" t="n">
-        <v>12937.2</v>
+        <v>10513</v>
       </c>
       <c r="T4" t="n">
-        <v>25079.4</v>
+        <v>16551.6</v>
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="n">
-        <v>17.99852000382194</v>
+        <v>4.76091573873596</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1132766704360241</v>
+        <v>0.1574027019924687</v>
       </c>
       <c r="X4" t="n">
-        <v>0.05556012382060594</v>
+        <v>0.210043624982429</v>
       </c>
       <c r="Y4" t="n">
-        <v>79.00374064837905</v>
+        <v>74.9296788482835</v>
       </c>
       <c r="Z4" t="n">
-        <v>1.433814013189365</v>
+        <v>2.100672315854648</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>claude-sonnet-5-5</t>
+          <t>gpt-6-1-sol</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5.5 (Max, Default Fallback)</t>
+          <t>GPT-6.1 Sol (Max)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5.5 (max with fallback)</t>
+          <t>GPT-6.1 Sol (max)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -861,82 +861,82 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>54.24133407109</v>
+        <v>54.5087338138148</v>
       </c>
       <c r="K5" t="n">
-        <v>3.568508820466448</v>
+        <v>6.779693260424727</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
-        <v>47.116982</v>
+        <v>3.028512</v>
       </c>
       <c r="N5" t="n">
-        <v>45.153257</v>
+        <v>2.648346</v>
       </c>
       <c r="O5" t="n">
-        <v>0.507917</v>
+        <v>0.129372</v>
       </c>
       <c r="P5" t="n">
-        <v>1.455808</v>
+        <v>0.250794</v>
       </c>
       <c r="Q5" t="n">
-        <v>912</v>
+        <v>482.4</v>
       </c>
       <c r="R5" t="n">
-        <v>196372.5</v>
+        <v>38016.6</v>
       </c>
       <c r="S5" t="n">
-        <v>50791.7</v>
+        <v>12937.2</v>
       </c>
       <c r="T5" t="n">
-        <v>145580.8</v>
+        <v>25079.4</v>
       </c>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="n">
-        <v>1.151205611409704</v>
+        <v>17.99852000382194</v>
       </c>
       <c r="W5" t="n">
-        <v>0.05947514700777413</v>
+        <v>0.1129948876737455</v>
       </c>
       <c r="X5" t="n">
-        <v>0.8686545566568725</v>
+        <v>0.05556012382060594</v>
       </c>
       <c r="Y5" t="n">
-        <v>215.3207236842105</v>
+        <v>78.80721393034825</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.276216547994704</v>
+        <v>1.433814013189365</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>gpt-6-1-terra</t>
+          <t>claude-sonnet-5-5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GPT-6.1 Terra (Max)</t>
+          <t>Claude Sonnet 5.5 (Max, Default Fallback)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>GPT-6.1 Terra (max)</t>
+          <t>Claude Sonnet 5.5 (max with fallback)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -951,82 +951,82 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>50.9765188577015</v>
+        <v>54.24133407109</v>
       </c>
       <c r="K6" t="n">
-        <v>8.065904882547704</v>
+        <v>3.524453156016244</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
-        <v>2.551231</v>
+        <v>47.116982</v>
       </c>
       <c r="N6" t="n">
-        <v>2.378263</v>
+        <v>45.153257</v>
       </c>
       <c r="O6" t="n">
-        <v>0.051016</v>
+        <v>0.507917</v>
       </c>
       <c r="P6" t="n">
-        <v>0.121952</v>
+        <v>1.455808</v>
       </c>
       <c r="Q6" t="n">
-        <v>379.2</v>
+        <v>923.4000000000001</v>
       </c>
       <c r="R6" t="n">
-        <v>34593.4</v>
+        <v>196372.5</v>
       </c>
       <c r="S6" t="n">
-        <v>10203.1</v>
+        <v>50791.7</v>
       </c>
       <c r="T6" t="n">
-        <v>24390.3</v>
+        <v>145580.8</v>
       </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="n">
-        <v>19.98114590866194</v>
+        <v>1.151205611409704</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1344317480424617</v>
+        <v>0.05874088593360407</v>
       </c>
       <c r="X6" t="n">
-        <v>0.0500471797048684</v>
+        <v>0.8686545566568725</v>
       </c>
       <c r="Y6" t="n">
-        <v>91.22732067510547</v>
+        <v>212.6624431448993</v>
       </c>
       <c r="Z6" t="n">
-        <v>1.473590883165618</v>
+        <v>0.276216547994704</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>gemini-4-argon</t>
+          <t>gpt-6-1-terra</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Gemini 4 Argon (High)</t>
+          <t>GPT-6.1 Terra (Max)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Gemini 4 Argon (high)</t>
+          <t>GPT-6.1 Terra (max)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1041,51 +1041,51 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>50.4121935905389</v>
+        <v>50.9765188577015</v>
       </c>
       <c r="K7" t="n">
-        <v>4.187059268317184</v>
+        <v>8.078687616117513</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
-        <v>8.057097000000001</v>
+        <v>2.551231</v>
       </c>
       <c r="N7" t="n">
-        <v>7.442264</v>
+        <v>2.378263</v>
       </c>
       <c r="O7" t="n">
-        <v>0.260092</v>
+        <v>0.051016</v>
       </c>
       <c r="P7" t="n">
-        <v>0.35474</v>
+        <v>0.121952</v>
       </c>
       <c r="Q7" t="n">
-        <v>722.4</v>
+        <v>378.6</v>
       </c>
       <c r="R7" t="n">
-        <v>61483.3</v>
+        <v>34593.4</v>
       </c>
       <c r="S7" t="n">
-        <v>26009.2</v>
+        <v>10203.1</v>
       </c>
       <c r="T7" t="n">
-        <v>35474</v>
+        <v>24390.3</v>
       </c>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="n">
-        <v>6.256868148731347</v>
+        <v>19.98114590866194</v>
       </c>
       <c r="W7" t="n">
-        <v>0.06978432113861974</v>
+        <v>0.1346447936019586</v>
       </c>
       <c r="X7" t="n">
-        <v>0.1598243683947154</v>
+        <v>0.0500471797048684</v>
       </c>
       <c r="Y7" t="n">
-        <v>85.10977297895903</v>
+        <v>91.37189646064449</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.8199331133907728</v>
+        <v>1.473590883165618</v>
       </c>
     </row>
     <row r="8">
@@ -1192,7 +1192,7 @@
         <v>49.0102124158081</v>
       </c>
       <c r="K9" t="n">
-        <v>3.784572387321089</v>
+        <v>3.744095677296264</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>2.346331</v>
       </c>
       <c r="Q9" t="n">
-        <v>777</v>
+        <v>785.4</v>
       </c>
       <c r="R9" t="n">
         <v>77792.89999999999</v>
@@ -1224,13 +1224,13 @@
         <v>0.7025181549600706</v>
       </c>
       <c r="W9" t="n">
-        <v>0.06307620645535147</v>
+        <v>0.0624015946216044</v>
       </c>
       <c r="X9" t="n">
         <v>1.423450757734279</v>
       </c>
       <c r="Y9" t="n">
-        <v>100.1195624195624</v>
+        <v>99.04876496052967</v>
       </c>
       <c r="Z9" t="n">
         <v>0.6300088107758948</v>
@@ -1282,7 +1282,7 @@
         <v>46.0026236744189</v>
       </c>
       <c r="K10" t="n">
-        <v>2.413568923106973</v>
+        <v>2.228809286551303</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1298,7 +1298,7 @@
         <v>0.346169</v>
       </c>
       <c r="Q10" t="n">
-        <v>1143.6</v>
+        <v>1238.4</v>
       </c>
       <c r="R10" t="n">
         <v>54926.9</v>
@@ -1314,13 +1314,13 @@
         <v>3.958771205060303</v>
       </c>
       <c r="W10" t="n">
-        <v>0.04022614871844955</v>
+        <v>0.03714682144252172</v>
       </c>
       <c r="X10" t="n">
         <v>0.2526036358761398</v>
       </c>
       <c r="Y10" t="n">
-        <v>48.02981811822316</v>
+        <v>44.3531169250646</v>
       </c>
       <c r="Z10" t="n">
         <v>0.8375244857149938</v>
@@ -1372,7 +1372,7 @@
         <v>43.3248225998431</v>
       </c>
       <c r="K11" t="n">
-        <v>9.824222811755805</v>
+        <v>10.09902624704967</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1388,7 +1388,7 @@
         <v>0.572101</v>
       </c>
       <c r="Q11" t="n">
-        <v>264.6</v>
+        <v>257.4</v>
       </c>
       <c r="R11" t="n">
         <v>54280.6</v>
@@ -1404,13 +1404,13 @@
         <v>1.353019932550879</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1637370468625967</v>
+        <v>0.1683171041174946</v>
       </c>
       <c r="X11" t="n">
         <v>0.7390874117535559</v>
       </c>
       <c r="Y11" t="n">
-        <v>205.1421012849584</v>
+        <v>210.8803418803419</v>
       </c>
       <c r="Z11" t="n">
         <v>0.798164032819149</v>
@@ -1462,7 +1462,7 @@
         <v>36.2345435880142</v>
       </c>
       <c r="K12" t="n">
-        <v>5.132371613033173</v>
+        <v>5.117873388137599</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1478,7 +1478,7 @@
         <v>0.064039</v>
       </c>
       <c r="Q12" t="n">
-        <v>423.6</v>
+        <v>424.8</v>
       </c>
       <c r="R12" t="n">
         <v>161190.3</v>
@@ -1494,13 +1494,13 @@
         <v>34.03934615450986</v>
       </c>
       <c r="W12" t="n">
-        <v>0.08553952688388622</v>
+        <v>0.0852978898022933</v>
       </c>
       <c r="X12" t="n">
         <v>0.02937776758286852</v>
       </c>
       <c r="Y12" t="n">
-        <v>380.5247875354108</v>
+        <v>379.4498587570621</v>
       </c>
       <c r="Z12" t="n">
         <v>0.2247935737325025</v>
@@ -1552,7 +1552,7 @@
         <v>34.3350117067196</v>
       </c>
       <c r="K13" t="n">
-        <v>2.414557785282672</v>
+        <v>2.589367398696802</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1568,7 +1568,7 @@
         <v>0.348155</v>
       </c>
       <c r="Q13" t="n">
-        <v>853.2</v>
+        <v>795.6</v>
       </c>
       <c r="R13" t="n">
         <v>80043.3</v>
@@ -1584,13 +1584,13 @@
         <v>4.119974147032401</v>
       </c>
       <c r="W13" t="n">
-        <v>0.0402426297547112</v>
+        <v>0.04315612331161337</v>
       </c>
       <c r="X13" t="n">
         <v>0.2427199696678426</v>
       </c>
       <c r="Y13" t="n">
-        <v>93.81540084388186</v>
+        <v>100.6074660633484</v>
       </c>
       <c r="Z13" t="n">
         <v>0.4289554741835931</v>
@@ -1642,7 +1642,7 @@
         <v>33.5545627367888</v>
       </c>
       <c r="K14" t="n">
-        <v>1.018038917985097</v>
+        <v>1.002526523357897</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1658,7 +1658,7 @@
         <v>0.424275</v>
       </c>
       <c r="Q14" t="n">
-        <v>1977.6</v>
+        <v>2008.2</v>
       </c>
       <c r="R14" t="n">
         <v>107612</v>
@@ -1674,13 +1674,13 @@
         <v>1.282966963974591</v>
       </c>
       <c r="W14" t="n">
-        <v>0.01696731529975162</v>
+        <v>0.01670877538929828</v>
       </c>
       <c r="X14" t="n">
         <v>0.7794432967330912</v>
       </c>
       <c r="Y14" t="n">
-        <v>54.41545307443365</v>
+        <v>53.58629618563889</v>
       </c>
       <c r="Z14" t="n">
         <v>0.3118106041778687</v>
@@ -1732,7 +1732,7 @@
         <v>32.4896393532027</v>
       </c>
       <c r="K15" t="n">
-        <v>5.791379563850747</v>
+        <v>5.885804230652663</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1748,7 +1748,7 @@
         <v>0.070968</v>
       </c>
       <c r="Q15" t="n">
-        <v>336.6</v>
+        <v>331.2</v>
       </c>
       <c r="R15" t="n">
         <v>89389.5</v>
@@ -1764,13 +1764,13 @@
         <v>10.82316581387436</v>
       </c>
       <c r="W15" t="n">
-        <v>0.0965229927308458</v>
+        <v>0.09809673717754439</v>
       </c>
       <c r="X15" t="n">
         <v>0.09239440817935976</v>
       </c>
       <c r="Y15" t="n">
-        <v>265.5659536541889</v>
+        <v>269.8958333333333</v>
       </c>
       <c r="Z15" t="n">
         <v>0.3634614731394929</v>
@@ -1822,7 +1822,7 @@
         <v>31.653381843882</v>
       </c>
       <c r="K16" t="n">
-        <v>2.997479341276704</v>
+        <v>2.687044299141087</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1838,7 +1838,7 @@
         <v>0.214281</v>
       </c>
       <c r="Q16" t="n">
-        <v>633.6</v>
+        <v>706.8</v>
       </c>
       <c r="R16" t="n">
         <v>71092.89999999999</v>
@@ -1854,13 +1854,13 @@
         <v>3.647463566006505</v>
       </c>
       <c r="W16" t="n">
-        <v>0.0499579890212784</v>
+        <v>0.04478407165235145</v>
       </c>
       <c r="X16" t="n">
         <v>0.2741631223735208</v>
       </c>
       <c r="Y16" t="n">
-        <v>112.2047032828283</v>
+        <v>100.584182229768</v>
       </c>
       <c r="Z16" t="n">
         <v>0.445239705285366</v>
@@ -1912,7 +1912,7 @@
         <v>30.5468119957291</v>
       </c>
       <c r="K17" t="n">
-        <v>3.53960741549584</v>
+        <v>3.757295448429163</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1928,7 +1928,7 @@
         <v>0.159289</v>
       </c>
       <c r="Q17" t="n">
-        <v>517.8000000000001</v>
+        <v>487.8000000000001</v>
       </c>
       <c r="R17" t="n">
         <v>70751.8</v>
@@ -1944,13 +1944,13 @@
         <v>6.233950391296028</v>
       </c>
       <c r="W17" t="n">
-        <v>0.05899345692493066</v>
+        <v>0.06262159080715272</v>
       </c>
       <c r="X17" t="n">
         <v>0.1604119277875905</v>
       </c>
       <c r="Y17" t="n">
-        <v>136.6392429509463</v>
+        <v>145.0426404264043</v>
       </c>
       <c r="Z17" t="n">
         <v>0.4317460756578504</v>
@@ -2002,7 +2002,7 @@
         <v>29.8897833093321</v>
       </c>
       <c r="K18" t="n">
-        <v>1.853055381855679</v>
+        <v>1.774927749960338</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2018,7 +2018,7 @@
         <v>0.032518</v>
       </c>
       <c r="Q18" t="n">
-        <v>967.8</v>
+        <v>1010.4</v>
       </c>
       <c r="R18" t="n">
         <v>64076.5</v>
@@ -2034,13 +2034,13 @@
         <v>12.12005768902687</v>
       </c>
       <c r="W18" t="n">
-        <v>0.03088425636426131</v>
+        <v>0.02958212916600564</v>
       </c>
       <c r="X18" t="n">
         <v>0.08250785810247172</v>
       </c>
       <c r="Y18" t="n">
-        <v>66.20841082868361</v>
+        <v>63.41696357878068</v>
       </c>
       <c r="Z18" t="n">
         <v>0.4664702864440489</v>
@@ -2094,38 +2094,38 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
-        <v>4.832016</v>
+        <v>4.86007</v>
       </c>
       <c r="N19" t="n">
-        <v>4.70269</v>
+        <v>4.729953</v>
       </c>
       <c r="O19" t="n">
-        <v>0.046295</v>
+        <v>0.046641</v>
       </c>
       <c r="P19" t="n">
-        <v>0.08303000000000001</v>
+        <v>0.08347599999999999</v>
       </c>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="n">
-        <v>143695.3</v>
+        <v>144574.6</v>
       </c>
       <c r="S19" t="n">
-        <v>51439.2</v>
+        <v>51823.1</v>
       </c>
       <c r="T19" t="n">
-        <v>92256.10000000001</v>
+        <v>92751.5</v>
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="n">
-        <v>6.098928349955174</v>
+        <v>6.063723232347888</v>
       </c>
       <c r="W19" t="inlineStr"/>
       <c r="X19" t="n">
-        <v>0.1639632313449542</v>
+        <v>0.1649151786257892</v>
       </c>
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="n">
-        <v>0.2050875663284534</v>
+        <v>0.2038402276045516</v>
       </c>
     </row>
     <row r="20">
@@ -2161,20 +2161,20 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H20" t="b">
         <v>1</v>
       </c>
       <c r="I20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20" t="n">
         <v>28.9095214290458</v>
       </c>
       <c r="K20" t="n">
-        <v>3.014548637022503</v>
+        <v>3.219323099002873</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2190,7 +2190,7 @@
         <v>0.032621</v>
       </c>
       <c r="Q20" t="n">
-        <v>575.4</v>
+        <v>538.8000000000001</v>
       </c>
       <c r="R20" t="n">
         <v>78313</v>
@@ -2206,13 +2206,13 @@
         <v>22.13701240263367</v>
       </c>
       <c r="W20" t="n">
-        <v>0.05024247728370838</v>
+        <v>0.05365538498338121</v>
       </c>
       <c r="X20" t="n">
         <v>0.04517321406392801</v>
       </c>
       <c r="Y20" t="n">
-        <v>136.1018421967327</v>
+        <v>145.3470675575352</v>
       </c>
       <c r="Z20" t="n">
         <v>0.3691535432054167</v>
@@ -2264,7 +2264,7 @@
         <v>28.5283090216016</v>
       </c>
       <c r="K21" t="n">
-        <v>5.372562904256422</v>
+        <v>5.168171924203189</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2280,7 +2280,7 @@
         <v>0.116179</v>
       </c>
       <c r="Q21" t="n">
-        <v>318.6</v>
+        <v>331.2</v>
       </c>
       <c r="R21" t="n">
         <v>63718.6</v>
@@ -2296,13 +2296,13 @@
         <v>4.33182452316382</v>
       </c>
       <c r="W21" t="n">
-        <v>0.08954271507094037</v>
+        <v>0.08613619873671981</v>
       </c>
       <c r="X21" t="n">
         <v>0.2308496095935192</v>
       </c>
       <c r="Y21" t="n">
-        <v>199.9956057752668</v>
+        <v>192.387077294686</v>
       </c>
       <c r="Z21" t="n">
         <v>0.4477234123411626</v>
@@ -2354,7 +2354,7 @@
         <v>27.7552004938153</v>
       </c>
       <c r="K22" t="n">
-        <v>4.23097568503282</v>
+        <v>4.075653523320896</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2370,7 +2370,7 @@
         <v>0.019244</v>
       </c>
       <c r="Q22" t="n">
-        <v>393.6</v>
+        <v>408.6</v>
       </c>
       <c r="R22" t="n">
         <v>49608.1</v>
@@ -2386,13 +2386,13 @@
         <v>85.1195912995412</v>
       </c>
       <c r="W22" t="n">
-        <v>0.07051626141721368</v>
+        <v>0.06792755872201493</v>
       </c>
       <c r="X22" t="n">
         <v>0.01174817670917776</v>
       </c>
       <c r="Y22" t="n">
-        <v>126.0368394308943</v>
+        <v>121.4099363680862</v>
       </c>
       <c r="Z22" t="n">
         <v>0.5594892869070837</v>
@@ -2401,7 +2401,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>mistral-large-4</t>
+          <t>mistral-large-4-preview</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2444,7 +2444,7 @@
         <v>25.286451488165</v>
       </c>
       <c r="K23" t="n">
-        <v>2.787921884031422</v>
+        <v>2.471793889361193</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
@@ -2460,7 +2460,7 @@
         <v>0.216476</v>
       </c>
       <c r="Q23" t="n">
-        <v>544.2</v>
+        <v>613.8000000000001</v>
       </c>
       <c r="R23" t="n">
         <v>69155</v>
@@ -2476,13 +2476,13 @@
         <v>4.11515448449033</v>
       </c>
       <c r="W23" t="n">
-        <v>0.04646536473385703</v>
+        <v>0.04119656482268653</v>
       </c>
       <c r="X23" t="n">
         <v>0.243004242919413</v>
       </c>
       <c r="Y23" t="n">
-        <v>127.0764424843807</v>
+        <v>112.6669925057022</v>
       </c>
       <c r="Z23" t="n">
         <v>0.365648926153785</v>
@@ -2534,7 +2534,7 @@
         <v>24.6815868992913</v>
       </c>
       <c r="K24" t="n">
-        <v>7.031791139399231</v>
+        <v>5.229149766799004</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2550,7 +2550,7 @@
         <v>0.07771699999999999</v>
       </c>
       <c r="Q24" t="n">
-        <v>210.6</v>
+        <v>283.2</v>
       </c>
       <c r="R24" t="n">
         <v>40302</v>
@@ -2566,13 +2566,13 @@
         <v>6.55041756208266</v>
       </c>
       <c r="W24" t="n">
-        <v>0.1171965189899872</v>
+        <v>0.08715249611331674</v>
       </c>
       <c r="X24" t="n">
         <v>0.1526620235309178</v>
       </c>
       <c r="Y24" t="n">
-        <v>191.3675213675214</v>
+        <v>142.3093220338983</v>
       </c>
       <c r="Z24" t="n">
         <v>0.6124159321942162</v>
@@ -2624,7 +2624,7 @@
         <v>20.1068756031705</v>
       </c>
       <c r="K25" t="n">
-        <v>0.9732272799211278</v>
+        <v>0.9118764445882312</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2640,7 +2640,7 @@
         <v>0.142193</v>
       </c>
       <c r="Q25" t="n">
-        <v>1239.6</v>
+        <v>1323</v>
       </c>
       <c r="R25" t="n">
         <v>66488.39999999999</v>
@@ -2656,13 +2656,13 @@
         <v>8.026815407321585</v>
       </c>
       <c r="W25" t="n">
-        <v>0.01622045466535213</v>
+        <v>0.01519794074313719</v>
       </c>
       <c r="X25" t="n">
         <v>0.1245824089947128</v>
       </c>
       <c r="Y25" t="n">
-        <v>53.63697967086157</v>
+        <v>50.25578231292516</v>
       </c>
       <c r="Z25" t="n">
         <v>0.3024117831557159</v>
@@ -2776,7 +2776,7 @@
         <v>17.7307282547205</v>
       </c>
       <c r="K27" t="n">
-        <v>23.02691981132532</v>
+        <v>16.57077406983224</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2792,7 +2792,7 @@
         <v>0.023214</v>
       </c>
       <c r="Q27" t="n">
-        <v>46.2</v>
+        <v>64.2</v>
       </c>
       <c r="R27" t="n">
         <v>26180.8</v>
@@ -2808,13 +2808,13 @@
         <v>23.40331811197295</v>
       </c>
       <c r="W27" t="n">
-        <v>0.383781996855422</v>
+        <v>0.2761795678305374</v>
       </c>
       <c r="X27" t="n">
         <v>0.04272898377980035</v>
       </c>
       <c r="Y27" t="n">
-        <v>566.6839826839827</v>
+        <v>407.8006230529595</v>
       </c>
       <c r="Z27" t="n">
         <v>0.677241652459837</v>
@@ -2866,7 +2866,7 @@
         <v>13.6203422723141</v>
       </c>
       <c r="K28" t="n">
-        <v>8.620469792603858</v>
+        <v>8.512713920196312</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2882,7 +2882,7 @@
         <v>0.020139</v>
       </c>
       <c r="Q28" t="n">
-        <v>94.80000000000001</v>
+        <v>96</v>
       </c>
       <c r="R28" t="n">
         <v>48599.1</v>
@@ -2898,13 +2898,13 @@
         <v>32.74758371777702</v>
       </c>
       <c r="W28" t="n">
-        <v>0.1436744965433976</v>
+        <v>0.1418785653366052</v>
       </c>
       <c r="X28" t="n">
         <v>0.03053660412377693</v>
       </c>
       <c r="Y28" t="n">
-        <v>512.6487341772151</v>
+        <v>506.240625</v>
       </c>
       <c r="Z28" t="n">
         <v>0.2802591462046437</v>
@@ -2956,7 +2956,7 @@
         <v>12.4781698715401</v>
       </c>
       <c r="K29" t="n">
-        <v>5.425291248495696</v>
+        <v>5.378521496353492</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -2972,7 +2972,7 @@
         <v>0.092972</v>
       </c>
       <c r="Q29" t="n">
-        <v>138</v>
+        <v>139.2</v>
       </c>
       <c r="R29" t="n">
         <v>34211.6</v>
@@ -2988,13 +2988,13 @@
         <v>5.162271282201742</v>
       </c>
       <c r="W29" t="n">
-        <v>0.09042152080826159</v>
+        <v>0.08964202493922487</v>
       </c>
       <c r="X29" t="n">
         <v>0.1937131826930052</v>
       </c>
       <c r="Y29" t="n">
-        <v>247.9101449275362</v>
+        <v>245.7729885057471</v>
       </c>
       <c r="Z29" t="n">
         <v>0.364735056867849</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-30)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,48 +594,48 @@
         <v>59.425738829526</v>
       </c>
       <c r="K2" t="n">
-        <v>4.588860141276139</v>
+        <v>5.820346604263075</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
-        <v>14.870251</v>
+        <v>14.217524</v>
       </c>
       <c r="N2" t="n">
-        <v>13.342112</v>
+        <v>13.197352</v>
       </c>
       <c r="O2" t="n">
-        <v>0.507506</v>
+        <v>0.492342</v>
       </c>
       <c r="P2" t="n">
-        <v>1.020633</v>
+        <v>0.52783</v>
       </c>
       <c r="Q2" t="n">
-        <v>777</v>
+        <v>612.6</v>
       </c>
       <c r="R2" t="n">
-        <v>76406.89999999999</v>
+        <v>51008.6</v>
       </c>
       <c r="S2" t="n">
-        <v>25375.3</v>
+        <v>24617.1</v>
       </c>
       <c r="T2" t="n">
-        <v>51031.6</v>
+        <v>26391.5</v>
       </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="n">
-        <v>3.996283507892772</v>
+        <v>4.17975301673667</v>
       </c>
       <c r="W2" t="n">
-        <v>0.07648100235460231</v>
+        <v>0.09700577673771792</v>
       </c>
       <c r="X2" t="n">
-        <v>0.2502324967748089</v>
+        <v>0.2392485862192755</v>
       </c>
       <c r="Y2" t="n">
-        <v>98.33577863577862</v>
+        <v>83.26575253019915</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.7777535645278896</v>
+        <v>1.165014111924773</v>
       </c>
     </row>
     <row r="3">
@@ -684,7 +684,7 @@
         <v>58.4060336078904</v>
       </c>
       <c r="K3" t="n">
-        <v>4.455075027299039</v>
+        <v>4.444903623127122</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.668643</v>
       </c>
       <c r="Q3" t="n">
-        <v>786.5999999999999</v>
+        <v>788.4000000000001</v>
       </c>
       <c r="R3" t="n">
         <v>118664.1</v>
@@ -716,13 +716,13 @@
         <v>1.127137240717486</v>
       </c>
       <c r="W3" t="n">
-        <v>0.07425125045498399</v>
+        <v>0.07408172705211871</v>
       </c>
       <c r="X3" t="n">
         <v>0.8872034068925305</v>
       </c>
       <c r="Y3" t="n">
-        <v>150.8569794050343</v>
+        <v>150.5125570776256</v>
       </c>
       <c r="Z3" t="n">
         <v>0.492196322290317</v>
@@ -774,7 +774,7 @@
         <v>56.8538559596797</v>
       </c>
       <c r="K4" t="n">
-        <v>9.444162119548123</v>
+        <v>10.06262937339464</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.827582</v>
       </c>
       <c r="Q4" t="n">
-        <v>361.2</v>
+        <v>339</v>
       </c>
       <c r="R4" t="n">
         <v>27064.6</v>
@@ -806,13 +806,13 @@
         <v>4.76091573873596</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1574027019924687</v>
+        <v>0.1677104895565773</v>
       </c>
       <c r="X4" t="n">
         <v>0.210043624982429</v>
       </c>
       <c r="Y4" t="n">
-        <v>74.9296788482835</v>
+        <v>79.83657817109145</v>
       </c>
       <c r="Z4" t="n">
         <v>2.100672315854648</v>
@@ -954,7 +954,7 @@
         <v>54.24133407109</v>
       </c>
       <c r="K6" t="n">
-        <v>3.524453156016244</v>
+        <v>3.635478154898794</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -970,7 +970,7 @@
         <v>1.455808</v>
       </c>
       <c r="Q6" t="n">
-        <v>923.4000000000001</v>
+        <v>895.2</v>
       </c>
       <c r="R6" t="n">
         <v>196372.5</v>
@@ -986,13 +986,13 @@
         <v>1.151205611409704</v>
       </c>
       <c r="W6" t="n">
-        <v>0.05874088593360407</v>
+        <v>0.06059130258164656</v>
       </c>
       <c r="X6" t="n">
         <v>0.8686545566568725</v>
       </c>
       <c r="Y6" t="n">
-        <v>212.6624431448993</v>
+        <v>219.3615951742627</v>
       </c>
       <c r="Z6" t="n">
         <v>0.276216547994704</v>
@@ -1192,7 +1192,7 @@
         <v>49.0102124158081</v>
       </c>
       <c r="K9" t="n">
-        <v>3.744095677296264</v>
+        <v>3.877390222769627</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>2.346331</v>
       </c>
       <c r="Q9" t="n">
-        <v>785.4</v>
+        <v>758.4000000000001</v>
       </c>
       <c r="R9" t="n">
         <v>77792.89999999999</v>
@@ -1224,13 +1224,13 @@
         <v>0.7025181549600706</v>
       </c>
       <c r="W9" t="n">
-        <v>0.0624015946216044</v>
+        <v>0.06462317037949379</v>
       </c>
       <c r="X9" t="n">
         <v>1.423450757734279</v>
       </c>
       <c r="Y9" t="n">
-        <v>99.04876496052967</v>
+        <v>102.575026371308</v>
       </c>
       <c r="Z9" t="n">
         <v>0.6300088107758948</v>
@@ -1282,7 +1282,7 @@
         <v>46.0026236744189</v>
       </c>
       <c r="K10" t="n">
-        <v>2.228809286551303</v>
+        <v>2.044561052196396</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1298,7 +1298,7 @@
         <v>0.346169</v>
       </c>
       <c r="Q10" t="n">
-        <v>1238.4</v>
+        <v>1350</v>
       </c>
       <c r="R10" t="n">
         <v>54926.9</v>
@@ -1314,13 +1314,13 @@
         <v>3.958771205060303</v>
       </c>
       <c r="W10" t="n">
-        <v>0.03714682144252172</v>
+        <v>0.03407601753660659</v>
       </c>
       <c r="X10" t="n">
         <v>0.2526036358761398</v>
       </c>
       <c r="Y10" t="n">
-        <v>44.3531169250646</v>
+        <v>40.6865925925926</v>
       </c>
       <c r="Z10" t="n">
         <v>0.8375244857149938</v>
@@ -1372,7 +1372,7 @@
         <v>43.3248225998431</v>
       </c>
       <c r="K11" t="n">
-        <v>10.09902624704967</v>
+        <v>6.866057464317449</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1388,7 +1388,7 @@
         <v>0.572101</v>
       </c>
       <c r="Q11" t="n">
-        <v>257.4</v>
+        <v>378.6</v>
       </c>
       <c r="R11" t="n">
         <v>54280.6</v>
@@ -1404,13 +1404,13 @@
         <v>1.353019932550879</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1683171041174946</v>
+        <v>0.1144342910719575</v>
       </c>
       <c r="X11" t="n">
         <v>0.7390874117535559</v>
       </c>
       <c r="Y11" t="n">
-        <v>210.8803418803419</v>
+        <v>143.3718964606445</v>
       </c>
       <c r="Z11" t="n">
         <v>0.798164032819149</v>
@@ -1462,7 +1462,7 @@
         <v>36.2345435880142</v>
       </c>
       <c r="K12" t="n">
-        <v>5.117873388137599</v>
+        <v>5.096278985656005</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1478,7 +1478,7 @@
         <v>0.064039</v>
       </c>
       <c r="Q12" t="n">
-        <v>424.8</v>
+        <v>426.6</v>
       </c>
       <c r="R12" t="n">
         <v>161190.3</v>
@@ -1494,13 +1494,13 @@
         <v>34.03934615450986</v>
       </c>
       <c r="W12" t="n">
-        <v>0.0852978898022933</v>
+        <v>0.08493798309426676</v>
       </c>
       <c r="X12" t="n">
         <v>0.02937776758286852</v>
       </c>
       <c r="Y12" t="n">
-        <v>379.4498587570621</v>
+        <v>377.8488045007032</v>
       </c>
       <c r="Z12" t="n">
         <v>0.2247935737325025</v>
@@ -1552,7 +1552,7 @@
         <v>34.3350117067196</v>
       </c>
       <c r="K13" t="n">
-        <v>2.589367398696802</v>
+        <v>2.319933223427</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1568,7 +1568,7 @@
         <v>0.348155</v>
       </c>
       <c r="Q13" t="n">
-        <v>795.6</v>
+        <v>888</v>
       </c>
       <c r="R13" t="n">
         <v>80043.3</v>
@@ -1584,13 +1584,13 @@
         <v>4.119974147032401</v>
       </c>
       <c r="W13" t="n">
-        <v>0.04315612331161337</v>
+        <v>0.03866555372378333</v>
       </c>
       <c r="X13" t="n">
         <v>0.2427199696678426</v>
       </c>
       <c r="Y13" t="n">
-        <v>100.6074660633484</v>
+        <v>90.13885135135135</v>
       </c>
       <c r="Z13" t="n">
         <v>0.4289554741835931</v>
@@ -1642,7 +1642,7 @@
         <v>33.5545627367888</v>
       </c>
       <c r="K14" t="n">
-        <v>1.002526523357897</v>
+        <v>0.9745734166944178</v>
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
@@ -1658,7 +1658,7 @@
         <v>0.424275</v>
       </c>
       <c r="Q14" t="n">
-        <v>2008.2</v>
+        <v>2065.8</v>
       </c>
       <c r="R14" t="n">
         <v>107612</v>
@@ -1674,13 +1674,13 @@
         <v>1.282966963974591</v>
       </c>
       <c r="W14" t="n">
-        <v>0.01670877538929828</v>
+        <v>0.01624289027824029</v>
       </c>
       <c r="X14" t="n">
         <v>0.7794432967330912</v>
       </c>
       <c r="Y14" t="n">
-        <v>53.58629618563889</v>
+        <v>52.09216768322199</v>
       </c>
       <c r="Z14" t="n">
         <v>0.3118106041778687</v>
@@ -1732,7 +1732,7 @@
         <v>32.4896393532027</v>
       </c>
       <c r="K15" t="n">
-        <v>5.885804230652663</v>
+        <v>5.853989072649135</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1748,7 +1748,7 @@
         <v>0.070968</v>
       </c>
       <c r="Q15" t="n">
-        <v>331.2</v>
+        <v>333</v>
       </c>
       <c r="R15" t="n">
         <v>89389.5</v>
@@ -1764,13 +1764,13 @@
         <v>10.82316581387436</v>
       </c>
       <c r="W15" t="n">
-        <v>0.09809673717754439</v>
+        <v>0.09756648454415225</v>
       </c>
       <c r="X15" t="n">
         <v>0.09239440817935976</v>
       </c>
       <c r="Y15" t="n">
-        <v>269.8958333333333</v>
+        <v>268.4369369369369</v>
       </c>
       <c r="Z15" t="n">
         <v>0.3634614731394929</v>
@@ -1822,7 +1822,7 @@
         <v>31.653381843882</v>
       </c>
       <c r="K16" t="n">
-        <v>2.687044299141087</v>
+        <v>2.607362590105601</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1838,7 +1838,7 @@
         <v>0.214281</v>
       </c>
       <c r="Q16" t="n">
-        <v>706.8</v>
+        <v>728.4000000000001</v>
       </c>
       <c r="R16" t="n">
         <v>71092.89999999999</v>
@@ -1854,13 +1854,13 @@
         <v>3.647463566006505</v>
       </c>
       <c r="W16" t="n">
-        <v>0.04478407165235145</v>
+        <v>0.04345604316842668</v>
       </c>
       <c r="X16" t="n">
         <v>0.2741631223735208</v>
       </c>
       <c r="Y16" t="n">
-        <v>100.584182229768</v>
+        <v>97.60145524437121</v>
       </c>
       <c r="Z16" t="n">
         <v>0.445239705285366</v>
@@ -1912,7 +1912,7 @@
         <v>30.5468119957291</v>
       </c>
       <c r="K17" t="n">
-        <v>3.757295448429163</v>
+        <v>3.379072123421361</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1928,7 +1928,7 @@
         <v>0.159289</v>
       </c>
       <c r="Q17" t="n">
-        <v>487.8000000000001</v>
+        <v>542.4</v>
       </c>
       <c r="R17" t="n">
         <v>70751.8</v>
@@ -1944,13 +1944,13 @@
         <v>6.233950391296028</v>
       </c>
       <c r="W17" t="n">
-        <v>0.06262159080715272</v>
+        <v>0.05631786872368934</v>
       </c>
       <c r="X17" t="n">
         <v>0.1604119277875905</v>
       </c>
       <c r="Y17" t="n">
-        <v>145.0426404264043</v>
+        <v>130.4421091445428</v>
       </c>
       <c r="Z17" t="n">
         <v>0.4317460756578504</v>
@@ -2002,7 +2002,7 @@
         <v>29.8897833093321</v>
       </c>
       <c r="K18" t="n">
-        <v>1.774927749960338</v>
+        <v>1.605251520372293</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2018,7 +2018,7 @@
         <v>0.032518</v>
       </c>
       <c r="Q18" t="n">
-        <v>1010.4</v>
+        <v>1117.2</v>
       </c>
       <c r="R18" t="n">
         <v>64076.5</v>
@@ -2034,13 +2034,13 @@
         <v>12.12005768902687</v>
       </c>
       <c r="W18" t="n">
-        <v>0.02958212916600564</v>
+        <v>0.02675419200620489</v>
       </c>
       <c r="X18" t="n">
         <v>0.08250785810247172</v>
       </c>
       <c r="Y18" t="n">
-        <v>63.41696357878068</v>
+        <v>57.35454708199069</v>
       </c>
       <c r="Z18" t="n">
         <v>0.4664702864440489</v>
@@ -2174,7 +2174,7 @@
         <v>28.9095214290458</v>
       </c>
       <c r="K20" t="n">
-        <v>3.219323099002873</v>
+        <v>3.197955910292677</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2190,7 +2190,7 @@
         <v>0.032621</v>
       </c>
       <c r="Q20" t="n">
-        <v>538.8000000000001</v>
+        <v>542.4</v>
       </c>
       <c r="R20" t="n">
         <v>78313</v>
@@ -2206,13 +2206,13 @@
         <v>22.13701240263367</v>
       </c>
       <c r="W20" t="n">
-        <v>0.05365538498338121</v>
+        <v>0.05329926517154462</v>
       </c>
       <c r="X20" t="n">
         <v>0.04517321406392801</v>
       </c>
       <c r="Y20" t="n">
-        <v>145.3470675575352</v>
+        <v>144.3823746312684</v>
       </c>
       <c r="Z20" t="n">
         <v>0.3691535432054167</v>
@@ -2354,7 +2354,7 @@
         <v>27.7552004938153</v>
       </c>
       <c r="K22" t="n">
-        <v>4.075653523320896</v>
+        <v>4.136393516216885</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2370,7 +2370,7 @@
         <v>0.019244</v>
       </c>
       <c r="Q22" t="n">
-        <v>408.6</v>
+        <v>402.6</v>
       </c>
       <c r="R22" t="n">
         <v>49608.1</v>
@@ -2386,13 +2386,13 @@
         <v>85.1195912995412</v>
       </c>
       <c r="W22" t="n">
-        <v>0.06792755872201493</v>
+        <v>0.06893989193694808</v>
       </c>
       <c r="X22" t="n">
         <v>0.01174817670917776</v>
       </c>
       <c r="Y22" t="n">
-        <v>121.4099363680862</v>
+        <v>123.2193243914555</v>
       </c>
       <c r="Z22" t="n">
         <v>0.5594892869070837</v>
@@ -2401,17 +2401,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>mistral-large-4-preview</t>
+          <t>mistral-large-4</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Mistral Large 4 Preview</t>
+          <t>Mistral Large 4 (High)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mistral Large 4 Preview</t>
+          <t>Mistral Large 4 (high)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2438,54 +2438,54 @@
         <v>1</v>
       </c>
       <c r="I23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J23" t="n">
-        <v>25.286451488165</v>
+        <v>26.0249946754784</v>
       </c>
       <c r="K23" t="n">
-        <v>2.471793889361193</v>
+        <v>7.699702566709586</v>
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
-        <v>6.144715</v>
+        <v>2.758198</v>
       </c>
       <c r="N23" t="n">
-        <v>5.855647</v>
+        <v>2.666781</v>
       </c>
       <c r="O23" t="n">
-        <v>0.072592</v>
+        <v>0.027</v>
       </c>
       <c r="P23" t="n">
-        <v>0.216476</v>
+        <v>0.064417</v>
       </c>
       <c r="Q23" t="n">
-        <v>613.8000000000001</v>
+        <v>202.8</v>
       </c>
       <c r="R23" t="n">
-        <v>69155</v>
+        <v>43531.9</v>
       </c>
       <c r="S23" t="n">
-        <v>17366.6</v>
+        <v>12857.2</v>
       </c>
       <c r="T23" t="n">
-        <v>51788.4</v>
+        <v>30674.7</v>
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="n">
-        <v>4.11515448449033</v>
+        <v>9.435506325317617</v>
       </c>
       <c r="W23" t="n">
-        <v>0.04119656482268653</v>
+        <v>0.1283283761118264</v>
       </c>
       <c r="X23" t="n">
-        <v>0.243004242919413</v>
+        <v>0.1059826537677975</v>
       </c>
       <c r="Y23" t="n">
-        <v>112.6669925057022</v>
+        <v>214.6543392504931</v>
       </c>
       <c r="Z23" t="n">
-        <v>0.365648926153785</v>
+        <v>0.5978373256273767</v>
       </c>
     </row>
     <row r="24">
@@ -2534,7 +2534,7 @@
         <v>24.6815868992913</v>
       </c>
       <c r="K24" t="n">
-        <v>5.229149766799004</v>
+        <v>5.099501425473409</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2550,7 +2550,7 @@
         <v>0.07771699999999999</v>
       </c>
       <c r="Q24" t="n">
-        <v>283.2</v>
+        <v>290.4</v>
       </c>
       <c r="R24" t="n">
         <v>40302</v>
@@ -2566,13 +2566,13 @@
         <v>6.55041756208266</v>
       </c>
       <c r="W24" t="n">
-        <v>0.08715249611331674</v>
+        <v>0.08499169042455683</v>
       </c>
       <c r="X24" t="n">
         <v>0.1526620235309178</v>
       </c>
       <c r="Y24" t="n">
-        <v>142.3093220338983</v>
+        <v>138.7809917355372</v>
       </c>
       <c r="Z24" t="n">
         <v>0.6124159321942162</v>
@@ -2624,7 +2624,7 @@
         <v>20.1068756031705</v>
       </c>
       <c r="K25" t="n">
-        <v>0.9118764445882312</v>
+        <v>0.8730731916270298</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2640,7 +2640,7 @@
         <v>0.142193</v>
       </c>
       <c r="Q25" t="n">
-        <v>1323</v>
+        <v>1381.8</v>
       </c>
       <c r="R25" t="n">
         <v>66488.39999999999</v>
@@ -2656,13 +2656,13 @@
         <v>8.026815407321585</v>
       </c>
       <c r="W25" t="n">
-        <v>0.01519794074313719</v>
+        <v>0.0145512198604505</v>
       </c>
       <c r="X25" t="n">
         <v>0.1245824089947128</v>
       </c>
       <c r="Y25" t="n">
-        <v>50.25578231292516</v>
+        <v>48.11723838471558</v>
       </c>
       <c r="Z25" t="n">
         <v>0.3024117831557159</v>
@@ -2776,7 +2776,7 @@
         <v>17.7307282547205</v>
       </c>
       <c r="K27" t="n">
-        <v>16.57077406983224</v>
+        <v>15.15446859377821</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2792,7 +2792,7 @@
         <v>0.023214</v>
       </c>
       <c r="Q27" t="n">
-        <v>64.2</v>
+        <v>70.19999999999999</v>
       </c>
       <c r="R27" t="n">
         <v>26180.8</v>
@@ -2808,13 +2808,13 @@
         <v>23.40331811197295</v>
       </c>
       <c r="W27" t="n">
-        <v>0.2761795678305374</v>
+        <v>0.2525744765629701</v>
       </c>
       <c r="X27" t="n">
         <v>0.04272898377980035</v>
       </c>
       <c r="Y27" t="n">
-        <v>407.8006230529595</v>
+        <v>372.945868945869</v>
       </c>
       <c r="Z27" t="n">
         <v>0.677241652459837</v>
@@ -2866,7 +2866,7 @@
         <v>13.6203422723141</v>
       </c>
       <c r="K28" t="n">
-        <v>8.512713920196312</v>
+        <v>8.675377243512164</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
@@ -2882,7 +2882,7 @@
         <v>0.020139</v>
       </c>
       <c r="Q28" t="n">
-        <v>96</v>
+        <v>94.2</v>
       </c>
       <c r="R28" t="n">
         <v>48599.1</v>
@@ -2898,13 +2898,13 @@
         <v>32.74758371777702</v>
       </c>
       <c r="W28" t="n">
-        <v>0.1418785653366052</v>
+        <v>0.1445896207252028</v>
       </c>
       <c r="X28" t="n">
         <v>0.03053660412377693</v>
       </c>
       <c r="Y28" t="n">
-        <v>506.240625</v>
+        <v>515.9140127388534</v>
       </c>
       <c r="Z28" t="n">
         <v>0.2802591462046437</v>
@@ -2956,7 +2956,7 @@
         <v>12.4781698715401</v>
       </c>
       <c r="K29" t="n">
-        <v>5.378521496353492</v>
+        <v>5.570611549794687</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -2972,7 +2972,7 @@
         <v>0.092972</v>
       </c>
       <c r="Q29" t="n">
-        <v>139.2</v>
+        <v>134.4</v>
       </c>
       <c r="R29" t="n">
         <v>34211.6</v>
@@ -2988,13 +2988,13 @@
         <v>5.162271282201742</v>
       </c>
       <c r="W29" t="n">
-        <v>0.08964202493922487</v>
+        <v>0.09284352582991146</v>
       </c>
       <c r="X29" t="n">
         <v>0.1937131826930052</v>
       </c>
       <c r="Y29" t="n">
-        <v>245.7729885057471</v>
+        <v>254.5505952380952</v>
       </c>
       <c r="Z29" t="n">
         <v>0.364735056867849</v>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-10-31)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -594,7 +594,7 @@
         <v>59.425738829526</v>
       </c>
       <c r="K2" t="n">
-        <v>5.820346604263075</v>
+        <v>6.045344743593692</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
@@ -610,7 +610,7 @@
         <v>0.52783</v>
       </c>
       <c r="Q2" t="n">
-        <v>612.6</v>
+        <v>589.8</v>
       </c>
       <c r="R2" t="n">
         <v>51008.6</v>
@@ -626,13 +626,13 @@
         <v>4.17975301673667</v>
       </c>
       <c r="W2" t="n">
-        <v>0.09700577673771792</v>
+        <v>0.1007557457265616</v>
       </c>
       <c r="X2" t="n">
         <v>0.2392485862192755</v>
       </c>
       <c r="Y2" t="n">
-        <v>83.26575253019915</v>
+        <v>86.48457104103086</v>
       </c>
       <c r="Z2" t="n">
         <v>1.165014111924773</v>
@@ -684,7 +684,7 @@
         <v>58.4060336078904</v>
       </c>
       <c r="K3" t="n">
-        <v>4.444903623127122</v>
+        <v>4.485870476796498</v>
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
@@ -700,7 +700,7 @@
         <v>1.668643</v>
       </c>
       <c r="Q3" t="n">
-        <v>788.4000000000001</v>
+        <v>781.1999999999999</v>
       </c>
       <c r="R3" t="n">
         <v>118664.1</v>
@@ -716,13 +716,13 @@
         <v>1.127137240717486</v>
       </c>
       <c r="W3" t="n">
-        <v>0.07408172705211871</v>
+        <v>0.0747645079466083</v>
       </c>
       <c r="X3" t="n">
         <v>0.8872034068925305</v>
       </c>
       <c r="Y3" t="n">
-        <v>150.5125570776256</v>
+        <v>151.8997695852535</v>
       </c>
       <c r="Z3" t="n">
         <v>0.492196322290317</v>
@@ -774,7 +774,7 @@
         <v>56.8538559596797</v>
       </c>
       <c r="K4" t="n">
-        <v>10.06262937339464</v>
+        <v>9.956892462290666</v>
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
@@ -790,7 +790,7 @@
         <v>0.827582</v>
       </c>
       <c r="Q4" t="n">
-        <v>339</v>
+        <v>342.6</v>
       </c>
       <c r="R4" t="n">
         <v>27064.6</v>
@@ -806,13 +806,13 @@
         <v>4.76091573873596</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1677104895565773</v>
+        <v>0.1659482077048444</v>
       </c>
       <c r="X4" t="n">
         <v>0.210043624982429</v>
       </c>
       <c r="Y4" t="n">
-        <v>79.83657817109145</v>
+        <v>78.99766491535317</v>
       </c>
       <c r="Z4" t="n">
         <v>2.100672315854648</v>
@@ -864,7 +864,7 @@
         <v>54.5087338138148</v>
       </c>
       <c r="K5" t="n">
-        <v>6.779693260424727</v>
+        <v>6.287051189598016</v>
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="n">
@@ -880,7 +880,7 @@
         <v>0.250794</v>
       </c>
       <c r="Q5" t="n">
-        <v>482.4</v>
+        <v>520.2</v>
       </c>
       <c r="R5" t="n">
         <v>38016.6</v>
@@ -896,13 +896,13 @@
         <v>17.99852000382194</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1129948876737455</v>
+        <v>0.1047841864933003</v>
       </c>
       <c r="X5" t="n">
         <v>0.05556012382060594</v>
       </c>
       <c r="Y5" t="n">
-        <v>78.80721393034825</v>
+        <v>73.08073817762399</v>
       </c>
       <c r="Z5" t="n">
         <v>1.433814013189365</v>
@@ -954,7 +954,7 @@
         <v>54.24133407109</v>
       </c>
       <c r="K6" t="n">
-        <v>3.635478154898794</v>
+        <v>3.642802825459368</v>
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="n">
@@ -970,7 +970,7 @@
         <v>1.455808</v>
       </c>
       <c r="Q6" t="n">
-        <v>895.2</v>
+        <v>893.4000000000001</v>
       </c>
       <c r="R6" t="n">
         <v>196372.5</v>
@@ -986,13 +986,13 @@
         <v>1.151205611409704</v>
       </c>
       <c r="W6" t="n">
-        <v>0.06059130258164656</v>
+        <v>0.06071338042432281</v>
       </c>
       <c r="X6" t="n">
         <v>0.8686545566568725</v>
       </c>
       <c r="Y6" t="n">
-        <v>219.3615951742627</v>
+        <v>219.803559435863</v>
       </c>
       <c r="Z6" t="n">
         <v>0.276216547994704</v>
@@ -1044,7 +1044,7 @@
         <v>50.9765188577015</v>
       </c>
       <c r="K7" t="n">
-        <v>8.078687616117513</v>
+        <v>8.684245120562435</v>
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="n">
@@ -1060,7 +1060,7 @@
         <v>0.121952</v>
       </c>
       <c r="Q7" t="n">
-        <v>378.6</v>
+        <v>352.2</v>
       </c>
       <c r="R7" t="n">
         <v>34593.4</v>
@@ -1076,13 +1076,13 @@
         <v>19.98114590866194</v>
       </c>
       <c r="W7" t="n">
-        <v>0.1346447936019586</v>
+        <v>0.1447374186760406</v>
       </c>
       <c r="X7" t="n">
         <v>0.0500471797048684</v>
       </c>
       <c r="Y7" t="n">
-        <v>91.37189646064449</v>
+        <v>98.22089721749008</v>
       </c>
       <c r="Z7" t="n">
         <v>1.473590883165618</v>
@@ -1192,7 +1192,7 @@
         <v>49.0102124158081</v>
       </c>
       <c r="K9" t="n">
-        <v>3.877390222769627</v>
+        <v>4.149890975089593</v>
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="n">
@@ -1208,7 +1208,7 @@
         <v>2.346331</v>
       </c>
       <c r="Q9" t="n">
-        <v>758.4000000000001</v>
+        <v>708.6</v>
       </c>
       <c r="R9" t="n">
         <v>77792.89999999999</v>
@@ -1224,13 +1224,13 @@
         <v>0.7025181549600706</v>
       </c>
       <c r="W9" t="n">
-        <v>0.06462317037949379</v>
+        <v>0.06916484958482655</v>
       </c>
       <c r="X9" t="n">
         <v>1.423450757734279</v>
       </c>
       <c r="Y9" t="n">
-        <v>102.575026371308</v>
+        <v>109.7839401637031</v>
       </c>
       <c r="Z9" t="n">
         <v>0.6300088107758948</v>
@@ -1282,7 +1282,7 @@
         <v>46.0026236744189</v>
       </c>
       <c r="K10" t="n">
-        <v>2.044561052196396</v>
+        <v>1.919174955128031</v>
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="n">
@@ -1298,7 +1298,7 @@
         <v>0.346169</v>
       </c>
       <c r="Q10" t="n">
-        <v>1350</v>
+        <v>1438.2</v>
       </c>
       <c r="R10" t="n">
         <v>54926.9</v>
@@ -1314,13 +1314,13 @@
         <v>3.958771205060303</v>
       </c>
       <c r="W10" t="n">
-        <v>0.03407601753660659</v>
+        <v>0.03198624925213385</v>
       </c>
       <c r="X10" t="n">
         <v>0.2526036358761398</v>
       </c>
       <c r="Y10" t="n">
-        <v>40.6865925925926</v>
+        <v>38.19141983034349</v>
       </c>
       <c r="Z10" t="n">
         <v>0.8375244857149938</v>
@@ -1372,7 +1372,7 @@
         <v>43.3248225998431</v>
       </c>
       <c r="K11" t="n">
-        <v>6.866057464317449</v>
+        <v>6.748414735178053</v>
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
@@ -1388,7 +1388,7 @@
         <v>0.572101</v>
       </c>
       <c r="Q11" t="n">
-        <v>378.6</v>
+        <v>385.2</v>
       </c>
       <c r="R11" t="n">
         <v>54280.6</v>
@@ -1404,13 +1404,13 @@
         <v>1.353019932550879</v>
       </c>
       <c r="W11" t="n">
-        <v>0.1144342910719575</v>
+        <v>0.1124735789196342</v>
       </c>
       <c r="X11" t="n">
         <v>0.7390874117535559</v>
       </c>
       <c r="Y11" t="n">
-        <v>143.3718964606445</v>
+        <v>140.9153686396677</v>
       </c>
       <c r="Z11" t="n">
         <v>0.798164032819149</v>
@@ -1462,7 +1462,7 @@
         <v>36.2345435880142</v>
       </c>
       <c r="K12" t="n">
-        <v>5.096278985656005</v>
+        <v>5.146952214206562</v>
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
@@ -1478,7 +1478,7 @@
         <v>0.064039</v>
       </c>
       <c r="Q12" t="n">
-        <v>426.6</v>
+        <v>422.4</v>
       </c>
       <c r="R12" t="n">
         <v>161190.3</v>
@@ -1494,13 +1494,13 @@
         <v>34.03934615450986</v>
       </c>
       <c r="W12" t="n">
-        <v>0.08493798309426676</v>
+        <v>0.0857825369034427</v>
       </c>
       <c r="X12" t="n">
         <v>0.02937776758286852</v>
       </c>
       <c r="Y12" t="n">
-        <v>377.8488045007032</v>
+        <v>381.6058238636364</v>
       </c>
       <c r="Z12" t="n">
         <v>0.2247935737325025</v>
@@ -1552,7 +1552,7 @@
         <v>34.3350117067196</v>
       </c>
       <c r="K13" t="n">
-        <v>2.319933223427</v>
+        <v>2.195333229329897</v>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
@@ -1568,7 +1568,7 @@
         <v>0.348155</v>
       </c>
       <c r="Q13" t="n">
-        <v>888</v>
+        <v>938.4000000000001</v>
       </c>
       <c r="R13" t="n">
         <v>80043.3</v>
@@ -1584,13 +1584,13 @@
         <v>4.119974147032401</v>
       </c>
       <c r="W13" t="n">
-        <v>0.03866555372378333</v>
+        <v>0.03658888715549829</v>
       </c>
       <c r="X13" t="n">
         <v>0.2427199696678426</v>
       </c>
       <c r="Y13" t="n">
-        <v>90.13885135135135</v>
+        <v>85.29763427109974</v>
       </c>
       <c r="Z13" t="n">
         <v>0.4289554741835931</v>
@@ -1732,7 +1732,7 @@
         <v>32.4896393532027</v>
       </c>
       <c r="K15" t="n">
-        <v>5.853989072649135</v>
+        <v>5.132644447583364</v>
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
@@ -1748,7 +1748,7 @@
         <v>0.070968</v>
       </c>
       <c r="Q15" t="n">
-        <v>333</v>
+        <v>379.8</v>
       </c>
       <c r="R15" t="n">
         <v>89389.5</v>
@@ -1764,13 +1764,13 @@
         <v>10.82316581387436</v>
       </c>
       <c r="W15" t="n">
-        <v>0.09756648454415225</v>
+        <v>0.08554407412638941</v>
       </c>
       <c r="X15" t="n">
         <v>0.09239440817935976</v>
       </c>
       <c r="Y15" t="n">
-        <v>268.4369369369369</v>
+        <v>235.3593996840442</v>
       </c>
       <c r="Z15" t="n">
         <v>0.3634614731394929</v>
@@ -1822,7 +1822,7 @@
         <v>31.653381843882</v>
       </c>
       <c r="K16" t="n">
-        <v>2.607362590105601</v>
+        <v>2.613821787273493</v>
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="n">
@@ -1838,7 +1838,7 @@
         <v>0.214281</v>
       </c>
       <c r="Q16" t="n">
-        <v>728.4000000000001</v>
+        <v>726.5999999999999</v>
       </c>
       <c r="R16" t="n">
         <v>71092.89999999999</v>
@@ -1854,13 +1854,13 @@
         <v>3.647463566006505</v>
       </c>
       <c r="W16" t="n">
-        <v>0.04345604316842668</v>
+        <v>0.04356369645455822</v>
       </c>
       <c r="X16" t="n">
         <v>0.2741631223735208</v>
       </c>
       <c r="Y16" t="n">
-        <v>97.60145524437121</v>
+        <v>97.84324249931187</v>
       </c>
       <c r="Z16" t="n">
         <v>0.445239705285366</v>
@@ -1912,7 +1912,7 @@
         <v>30.5468119957291</v>
       </c>
       <c r="K17" t="n">
-        <v>3.379072123421361</v>
+        <v>3.260065314378773</v>
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="n">
@@ -1928,7 +1928,7 @@
         <v>0.159289</v>
       </c>
       <c r="Q17" t="n">
-        <v>542.4</v>
+        <v>562.1999999999999</v>
       </c>
       <c r="R17" t="n">
         <v>70751.8</v>
@@ -1944,13 +1944,13 @@
         <v>6.233950391296028</v>
       </c>
       <c r="W17" t="n">
-        <v>0.05631786872368934</v>
+        <v>0.05433442190631289</v>
       </c>
       <c r="X17" t="n">
         <v>0.1604119277875905</v>
       </c>
       <c r="Y17" t="n">
-        <v>130.4421091445428</v>
+        <v>125.8480967627179</v>
       </c>
       <c r="Z17" t="n">
         <v>0.4317460756578504</v>
@@ -2002,7 +2002,7 @@
         <v>29.8897833093321</v>
       </c>
       <c r="K18" t="n">
-        <v>1.605251520372293</v>
+        <v>1.550299964176976</v>
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
@@ -2018,7 +2018,7 @@
         <v>0.032518</v>
       </c>
       <c r="Q18" t="n">
-        <v>1117.2</v>
+        <v>1156.8</v>
       </c>
       <c r="R18" t="n">
         <v>64076.5</v>
@@ -2034,13 +2034,13 @@
         <v>12.12005768902687</v>
       </c>
       <c r="W18" t="n">
-        <v>0.02675419200620489</v>
+        <v>0.02583833273628293</v>
       </c>
       <c r="X18" t="n">
         <v>0.08250785810247172</v>
       </c>
       <c r="Y18" t="n">
-        <v>57.35454708199069</v>
+        <v>55.39116528354079</v>
       </c>
       <c r="Z18" t="n">
         <v>0.4664702864440489</v>
@@ -2174,7 +2174,7 @@
         <v>28.9095214290458</v>
       </c>
       <c r="K20" t="n">
-        <v>3.197955910292677</v>
+        <v>3.17687048670833</v>
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
@@ -2190,7 +2190,7 @@
         <v>0.032621</v>
       </c>
       <c r="Q20" t="n">
-        <v>542.4</v>
+        <v>546</v>
       </c>
       <c r="R20" t="n">
         <v>78313</v>
@@ -2206,13 +2206,13 @@
         <v>22.13701240263367</v>
       </c>
       <c r="W20" t="n">
-        <v>0.05329926517154462</v>
+        <v>0.05294784144513882</v>
       </c>
       <c r="X20" t="n">
         <v>0.04517321406392801</v>
       </c>
       <c r="Y20" t="n">
-        <v>144.3823746312684</v>
+        <v>143.4304029304029</v>
       </c>
       <c r="Z20" t="n">
         <v>0.3691535432054167</v>
@@ -2264,7 +2264,7 @@
         <v>28.5283090216016</v>
       </c>
       <c r="K21" t="n">
-        <v>5.168171924203189</v>
+        <v>4.944247664055737</v>
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
@@ -2280,7 +2280,7 @@
         <v>0.116179</v>
       </c>
       <c r="Q21" t="n">
-        <v>331.2</v>
+        <v>346.2</v>
       </c>
       <c r="R21" t="n">
         <v>63718.6</v>
@@ -2296,13 +2296,13 @@
         <v>4.33182452316382</v>
       </c>
       <c r="W21" t="n">
-        <v>0.08613619873671981</v>
+        <v>0.08240412773426228</v>
       </c>
       <c r="X21" t="n">
         <v>0.2308496095935192</v>
       </c>
       <c r="Y21" t="n">
-        <v>192.387077294686</v>
+        <v>184.05141536684</v>
       </c>
       <c r="Z21" t="n">
         <v>0.4477234123411626</v>
@@ -2354,7 +2354,7 @@
         <v>27.7552004938153</v>
       </c>
       <c r="K22" t="n">
-        <v>4.136393516216885</v>
+        <v>4.005079436336985</v>
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
@@ -2370,7 +2370,7 @@
         <v>0.019244</v>
       </c>
       <c r="Q22" t="n">
-        <v>402.6</v>
+        <v>415.8</v>
       </c>
       <c r="R22" t="n">
         <v>49608.1</v>
@@ -2386,13 +2386,13 @@
         <v>85.1195912995412</v>
       </c>
       <c r="W22" t="n">
-        <v>0.06893989193694808</v>
+        <v>0.06675132393894974</v>
       </c>
       <c r="X22" t="n">
         <v>0.01174817670917776</v>
       </c>
       <c r="Y22" t="n">
-        <v>123.2193243914555</v>
+        <v>119.3075998075998</v>
       </c>
       <c r="Z22" t="n">
         <v>0.5594892869070837</v>
@@ -2534,7 +2534,7 @@
         <v>24.6815868992913</v>
       </c>
       <c r="K24" t="n">
-        <v>5.099501425473409</v>
+        <v>5.088986989544598</v>
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="n">
@@ -2550,7 +2550,7 @@
         <v>0.07771699999999999</v>
       </c>
       <c r="Q24" t="n">
-        <v>290.4</v>
+        <v>291</v>
       </c>
       <c r="R24" t="n">
         <v>40302</v>
@@ -2566,13 +2566,13 @@
         <v>6.55041756208266</v>
       </c>
       <c r="W24" t="n">
-        <v>0.08499169042455683</v>
+        <v>0.0848164498257433</v>
       </c>
       <c r="X24" t="n">
         <v>0.1526620235309178</v>
       </c>
       <c r="Y24" t="n">
-        <v>138.7809917355372</v>
+        <v>138.4948453608247</v>
       </c>
       <c r="Z24" t="n">
         <v>0.6124159321942162</v>
@@ -2624,7 +2624,7 @@
         <v>20.1068756031705</v>
       </c>
       <c r="K25" t="n">
-        <v>0.8730731916270298</v>
+        <v>0.9122901816320554</v>
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="n">
@@ -2640,7 +2640,7 @@
         <v>0.142193</v>
       </c>
       <c r="Q25" t="n">
-        <v>1381.8</v>
+        <v>1322.4</v>
       </c>
       <c r="R25" t="n">
         <v>66488.39999999999</v>
@@ -2656,13 +2656,13 @@
         <v>8.026815407321585</v>
       </c>
       <c r="W25" t="n">
-        <v>0.0145512198604505</v>
+        <v>0.01520483636053426</v>
       </c>
       <c r="X25" t="n">
         <v>0.1245824089947128</v>
       </c>
       <c r="Y25" t="n">
-        <v>48.11723838471558</v>
+        <v>50.27858439201452</v>
       </c>
       <c r="Z25" t="n">
         <v>0.3024117831557159</v>
@@ -2776,7 +2776,7 @@
         <v>17.7307282547205</v>
       </c>
       <c r="K27" t="n">
-        <v>15.15446859377821</v>
+        <v>15.97362905830676</v>
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="n">
@@ -2792,7 +2792,7 @@
         <v>0.023214</v>
       </c>
       <c r="Q27" t="n">
-        <v>70.19999999999999</v>
+        <v>66.60000000000001</v>
       </c>
       <c r="R27" t="n">
         <v>26180.8</v>
@@ -2808,13 +2808,13 @@
         <v>23.40331811197295</v>
       </c>
       <c r="W27" t="n">
-        <v>0.2525744765629701</v>
+        <v>0.2662271509717792</v>
       </c>
       <c r="X27" t="n">
         <v>0.04272898377980035</v>
       </c>
       <c r="Y27" t="n">
-        <v>372.945868945869</v>
+        <v>393.1051051051051</v>
       </c>
       <c r="Z27" t="n">
         <v>0.677241652459837</v>
@@ -2866,23 +2866,23 @@
         <v>13.6203422723141</v>
       </c>
       <c r="K28" t="n">
-        <v>8.675377243512164</v>
+        <v>8.84437809890526</v>
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="n">
-        <v>0.415919</v>
+        <v>0.369166</v>
       </c>
       <c r="N28" t="n">
-        <v>0.387975</v>
+        <v>0.344867</v>
       </c>
       <c r="O28" t="n">
-        <v>0.007805</v>
+        <v>0.006787</v>
       </c>
       <c r="P28" t="n">
-        <v>0.020139</v>
+        <v>0.017513</v>
       </c>
       <c r="Q28" t="n">
-        <v>94.2</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="R28" t="n">
         <v>48599.1</v>
@@ -2895,16 +2895,16 @@
       </c>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="n">
-        <v>32.74758371777702</v>
+        <v>36.89489896771127</v>
       </c>
       <c r="W28" t="n">
-        <v>0.1445896207252028</v>
+        <v>0.147406301648421</v>
       </c>
       <c r="X28" t="n">
-        <v>0.03053660412377693</v>
+        <v>0.02710401784472033</v>
       </c>
       <c r="Y28" t="n">
-        <v>515.9140127388534</v>
+        <v>525.9642857142857</v>
       </c>
       <c r="Z28" t="n">
         <v>0.2802591462046437</v>
@@ -2956,7 +2956,7 @@
         <v>12.4781698715401</v>
       </c>
       <c r="K29" t="n">
-        <v>5.570611549794687</v>
+        <v>4.912665303755944</v>
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="n">
@@ -2972,7 +2972,7 @@
         <v>0.092972</v>
       </c>
       <c r="Q29" t="n">
-        <v>134.4</v>
+        <v>152.4</v>
       </c>
       <c r="R29" t="n">
         <v>34211.6</v>
@@ -2988,13 +2988,13 @@
         <v>5.162271282201742</v>
       </c>
       <c r="W29" t="n">
-        <v>0.09284352582991146</v>
+        <v>0.08187775506259908</v>
       </c>
       <c r="X29" t="n">
         <v>0.1937131826930052</v>
       </c>
       <c r="Y29" t="n">
-        <v>254.5505952380952</v>
+        <v>224.4855643044619</v>
       </c>
       <c r="Z29" t="n">
         <v>0.364735056867849</v>

</xml_diff>